<commit_message>
Floor Cleanup and Official Timeout
Floor Cleanup takes the sizes first, then shuffles, then deals — dealing as it
went would have the first man drawing out of a deck the others had not gone
into yet.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -2549,7 +2549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J113"/>
+  <dimension ref="A1:J115"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="22.25" customHeight="1"/>
   <cols>
     <col width="15.5" customWidth="1" style="8" min="1" max="1"/>
@@ -2626,39 +2626,40 @@
         </is>
       </c>
       <c r="B2" s="12">
-        <f>COUNTIF($B$5:$B$113,"Pass")</f>
+        <f>COUNTIF($B$5:$B$115,"Pass")</f>
         <v/>
       </c>
       <c r="C2" s="13">
-        <f>COUNTIF($B$5:$B$113,"Move")+COUNTIF($B$5:$B$113,"Special Move")</f>
+        <f>COUNTIF($B$5:$B$115,"Move")+COUNTIF($B$5:$B$115,"Special Move")</f>
         <v/>
       </c>
       <c r="D2" s="14">
-        <f>COUNTIF($B$5:$B$113,"Clamp")</f>
+        <f>COUNTIF($B$5:$B$115,"Clamp")</f>
         <v/>
       </c>
       <c r="E2" s="15">
-        <f>COUNTIF($B$5:$B$113,"Whistle")</f>
+        <f>COUNTIF($B$5:$B$115,"Whistle")</f>
         <v/>
       </c>
       <c r="F2" s="16">
-        <f>COUNTIF($B$5:$B$113,"Game Break")</f>
+        <f>COUNTIF($B$5:$B$115,"Game Break")</f>
         <v/>
       </c>
       <c r="G2" s="18">
-        <f>COUNTIF($B$5:$B$113,"Injury GB")</f>
+        <f>COUNTIF($B$5:$B$115,"Injury GB")</f>
         <v/>
       </c>
       <c r="H2" s="19">
-        <f>COUNTIF($B$5:$B$113,"Devastating Injury GB")</f>
+        <f>COUNTIF($B$5:$B$115,"Devastating Injury GB")</f>
         <v/>
       </c>
       <c r="I2" s="17">
-        <f>COUNTIF($B$5:$B$113,"Intangible")</f>
+        <f>COUNTIF($B$5:$B$115,"Intangible")</f>
         <v/>
       </c>
       <c r="J2" s="19" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4" ht="20.75" customHeight="1" s="132" thickBot="1">
       <c r="A4" s="123" t="inlineStr">
         <is>
@@ -2702,7 +2703,7 @@
         </is>
       </c>
       <c r="B5" s="22">
-        <f>COUNTIF($B$5:$B$113,"Pass")</f>
+        <f>COUNTIF($B$5:$B$115,"Pass")</f>
         <v/>
       </c>
       <c r="C5" s="23" t="n"/>
@@ -2959,7 +2960,7 @@
         </is>
       </c>
       <c r="B15" s="40">
-        <f>COUNTIF($B$5:$B$113,"Move")+COUNTIF($B$5:$B$113,"Special Move")</f>
+        <f>COUNTIF($B$5:$B$115,"Move")+COUNTIF($B$5:$B$115,"Special Move")</f>
         <v/>
       </c>
       <c r="C15" s="41" t="n"/>
@@ -3333,7 +3334,7 @@
         </is>
       </c>
       <c r="B28" s="43">
-        <f>COUNTIF($B$5:$B$113,"Special Move")</f>
+        <f>COUNTIF($B$5:$B$115,"Special Move")</f>
         <v/>
       </c>
       <c r="C28" s="44" t="n"/>
@@ -3718,7 +3719,7 @@
         </is>
       </c>
       <c r="B41" s="59">
-        <f>COUNTIF($B$5:$B$113,"Clamp")</f>
+        <f>COUNTIF($B$5:$B$115,"Clamp")</f>
         <v/>
       </c>
       <c r="C41" s="60" t="n"/>
@@ -3887,7 +3888,7 @@
         </is>
       </c>
       <c r="B47" s="59">
-        <f>COUNTIF($B$5:$B$113,"Whistle")</f>
+        <f>COUNTIF($B$5:$B$115,"Whistle")</f>
         <v/>
       </c>
       <c r="C47" s="60" t="n"/>
@@ -4346,7 +4347,7 @@
         </is>
       </c>
       <c r="B65" s="59">
-        <f>COUNTIF($B$5:$B$113,"Game Break")</f>
+        <f>COUNTIF($B$5:$B$115,"Game Break")</f>
         <v/>
       </c>
       <c r="C65" s="60" t="n"/>
@@ -4859,20 +4860,27 @@
       <c r="J83" s="102" t="n"/>
     </row>
     <row r="84" ht="28" customHeight="1" s="132">
-      <c r="A84" s="55" t="inlineStr">
-        <is>
-          <t>Injury GB</t>
-        </is>
-      </c>
-      <c r="B84" s="56">
-        <f>COUNTIF($B$5:$B$113,"Injury GB")</f>
-        <v/>
-      </c>
-      <c r="C84" s="57" t="n"/>
-      <c r="D84" s="57" t="n"/>
-      <c r="E84" s="57" t="n"/>
-      <c r="F84" s="88" t="n"/>
-      <c r="G84" s="108" t="n"/>
+      <c r="A84" s="29" t="n"/>
+      <c r="B84" s="30" t="inlineStr">
+        <is>
+          <t>Game Break</t>
+        </is>
+      </c>
+      <c r="C84" s="134" t="inlineStr">
+        <is>
+          <t>Floor Cleanup</t>
+        </is>
+      </c>
+      <c r="D84" s="91" t="inlineStr">
+        <is>
+          <t>All players shuffle their hands into the deck and draw the same number of cards</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="n"/>
+      <c r="F84" s="76" t="n">
+        <v>3</v>
+      </c>
+      <c r="G84" s="111" t="n"/>
       <c r="H84" s="102" t="n"/>
       <c r="I84" s="102" t="n"/>
       <c r="J84" s="102" t="n"/>
@@ -4881,144 +4889,141 @@
       <c r="A85" s="29" t="n"/>
       <c r="B85" s="30" t="inlineStr">
         <is>
-          <t>Injury GB</t>
-        </is>
-      </c>
-      <c r="C85" s="31" t="inlineStr">
-        <is>
-          <t>Bone Bruise</t>
+          <t>Game Break</t>
+        </is>
+      </c>
+      <c r="C85" s="134" t="inlineStr">
+        <is>
+          <t>Official Timeout</t>
         </is>
       </c>
       <c r="D85" s="91" t="inlineStr">
         <is>
-          <t>Discard 1 card at the start of each turn after drawing (your choice)</t>
+          <t>Discard all Injuries on all players</t>
         </is>
       </c>
       <c r="E85" s="7" t="n"/>
       <c r="F85" s="76" t="n">
-        <v>3</v>
-      </c>
-      <c r="G85" s="101" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="G85" s="111" t="n"/>
       <c r="H85" s="102" t="n"/>
       <c r="I85" s="102" t="n"/>
       <c r="J85" s="102" t="n"/>
     </row>
     <row r="86" ht="56" customHeight="1" s="132">
-      <c r="A86" s="58" t="inlineStr">
+      <c r="A86" s="55" t="inlineStr">
+        <is>
+          <t>Injury GB</t>
+        </is>
+      </c>
+      <c r="B86" s="56">
+        <f>COUNTIF($B$5:$B$115,"Injury GB")</f>
+        <v/>
+      </c>
+      <c r="C86" s="57" t="n"/>
+      <c r="D86" s="57" t="n"/>
+      <c r="E86" s="57" t="n"/>
+      <c r="F86" s="88" t="n"/>
+      <c r="G86" s="108" t="n"/>
+      <c r="H86" s="102" t="n"/>
+      <c r="I86" s="102" t="n"/>
+      <c r="J86" s="102" t="n"/>
+    </row>
+    <row r="87" ht="56" customHeight="1" s="132">
+      <c r="A87" s="29" t="n"/>
+      <c r="B87" s="30" t="inlineStr">
+        <is>
+          <t>Injury GB</t>
+        </is>
+      </c>
+      <c r="C87" s="31" t="inlineStr">
+        <is>
+          <t>Bone Bruise</t>
+        </is>
+      </c>
+      <c r="D87" s="91" t="inlineStr">
+        <is>
+          <t>Discard 1 card at the start of each turn after drawing (your choice)</t>
+        </is>
+      </c>
+      <c r="E87" s="7" t="n"/>
+      <c r="F87" s="76" t="n">
+        <v>3</v>
+      </c>
+      <c r="G87" s="101" t="n"/>
+      <c r="H87" s="102" t="n"/>
+      <c r="I87" s="102" t="n"/>
+      <c r="J87" s="102" t="n"/>
+    </row>
+    <row r="88" ht="28" customHeight="1" s="132">
+      <c r="A88" s="58" t="inlineStr">
         <is>
           <t>Devastating Injury GB</t>
         </is>
       </c>
-      <c r="B86" s="59">
-        <f>COUNTIF($B$5:$B$113,"Devastating Injury GB")</f>
+      <c r="B88" s="59">
+        <f>COUNTIF($B$5:$B$115,"Devastating Injury GB")</f>
         <v/>
       </c>
-      <c r="C86" s="60" t="n"/>
-      <c r="D86" s="60" t="n"/>
-      <c r="E86" s="60" t="n"/>
-      <c r="F86" s="86" t="n"/>
-      <c r="G86" s="109" t="n"/>
-      <c r="H86" s="110" t="n"/>
-      <c r="I86" s="110" t="n"/>
-      <c r="J86" s="110" t="n"/>
-    </row>
-    <row r="87" ht="56" customHeight="1" s="132">
-      <c r="A87" s="50" t="n"/>
-      <c r="B87" s="51" t="inlineStr">
+      <c r="C88" s="60" t="n"/>
+      <c r="D88" s="60" t="n"/>
+      <c r="E88" s="60" t="n"/>
+      <c r="F88" s="86" t="n"/>
+      <c r="G88" s="109" t="n"/>
+      <c r="H88" s="110" t="n"/>
+      <c r="I88" s="110" t="n"/>
+      <c r="J88" s="110" t="n"/>
+    </row>
+    <row r="89" ht="42" customHeight="1" s="132">
+      <c r="A89" s="50" t="n"/>
+      <c r="B89" s="51" t="inlineStr">
         <is>
           <t>Devastating Injury GB</t>
         </is>
       </c>
-      <c r="C87" s="136" t="inlineStr">
+      <c r="C89" s="136" t="inlineStr">
         <is>
           <t>Torn Achilles</t>
         </is>
       </c>
-      <c r="D87" s="137" t="inlineStr">
+      <c r="D89" s="137" t="inlineStr">
         <is>
           <t>Hand is locked every turn except 1 card (randomly)</t>
         </is>
       </c>
-      <c r="E87" s="54" t="n"/>
-      <c r="F87" s="141" t="n"/>
-      <c r="G87" s="114" t="n"/>
-      <c r="H87" s="115" t="n"/>
-      <c r="I87" s="115" t="n"/>
-      <c r="J87" s="115" t="n"/>
-    </row>
-    <row r="88" ht="28" customHeight="1" s="132">
-      <c r="A88" s="55" t="inlineStr">
+      <c r="E89" s="54" t="n"/>
+      <c r="F89" s="141" t="n"/>
+      <c r="G89" s="114" t="n"/>
+      <c r="H89" s="115" t="n"/>
+      <c r="I89" s="115" t="n"/>
+      <c r="J89" s="115" t="n"/>
+    </row>
+    <row r="90" ht="28" customHeight="1" s="132">
+      <c r="A90" s="55" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="B88" s="56">
-        <f>COUNTIF($B$5:$B$113,"Intangible")</f>
+      <c r="B90" s="56">
+        <f>COUNTIF($B$5:$B$115,"Intangible")</f>
         <v/>
       </c>
-      <c r="C88" s="57" t="n"/>
-      <c r="D88" s="57" t="n"/>
-      <c r="E88" s="57" t="n"/>
-      <c r="F88" s="88" t="n"/>
-      <c r="G88" s="108" t="n"/>
-      <c r="H88" s="102" t="n"/>
-      <c r="I88" s="102" t="n"/>
-      <c r="J88" s="102" t="n"/>
-    </row>
-    <row r="89" ht="42" customHeight="1" s="132">
-      <c r="A89" s="96" t="inlineStr">
-        <is>
-          <t>All intangibles are limited to 1</t>
-        </is>
-      </c>
-      <c r="B89" s="30" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C89" s="31" t="inlineStr">
-        <is>
-          <t>Board-Crasher</t>
-        </is>
-      </c>
-      <c r="D89" s="6" t="inlineStr">
-        <is>
-          <t>SHOT +10% upon Rebounding your own missed shot</t>
-        </is>
-      </c>
-      <c r="E89" s="7" t="n"/>
-      <c r="F89" s="138" t="n"/>
-      <c r="G89" s="101" t="n"/>
-      <c r="H89" s="102" t="n"/>
-      <c r="I89" s="102" t="n"/>
-      <c r="J89" s="102" t="n"/>
-    </row>
-    <row r="90" ht="28" customHeight="1" s="132">
-      <c r="A90" s="29" t="n"/>
-      <c r="B90" s="30" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C90" s="32" t="inlineStr">
-        <is>
-          <t>Catch &amp; Shoot Specialist</t>
-        </is>
-      </c>
-      <c r="D90" s="33" t="inlineStr">
-        <is>
-          <t>Additional SHOT +10% on all received passes</t>
-        </is>
-      </c>
-      <c r="E90" s="34" t="n"/>
-      <c r="F90" s="138" t="n"/>
-      <c r="G90" s="107" t="n"/>
+      <c r="C90" s="57" t="n"/>
+      <c r="D90" s="57" t="n"/>
+      <c r="E90" s="57" t="n"/>
+      <c r="F90" s="88" t="n"/>
+      <c r="G90" s="108" t="n"/>
       <c r="H90" s="102" t="n"/>
       <c r="I90" s="102" t="n"/>
       <c r="J90" s="102" t="n"/>
     </row>
     <row r="91" ht="42" customHeight="1" s="132">
-      <c r="A91" s="29" t="n"/>
+      <c r="A91" s="96" t="inlineStr">
+        <is>
+          <t>All intangibles are limited to 1</t>
+        </is>
+      </c>
       <c r="B91" s="30" t="inlineStr">
         <is>
           <t>Intangible</t>
@@ -5026,12 +5031,12 @@
       </c>
       <c r="C91" s="31" t="inlineStr">
         <is>
-          <t>Clutch Gene</t>
+          <t>Board-Crasher</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>SHOT x2 if attempting a shot with 1 or fewer cards in hand or Shot Clock 3 or less</t>
+          <t>SHOT +10% upon Rebounding your own missed shot</t>
         </is>
       </c>
       <c r="E91" s="7" t="n"/>
@@ -5050,12 +5055,12 @@
       </c>
       <c r="C92" s="32" t="inlineStr">
         <is>
-          <t>Floor General</t>
+          <t>Catch &amp; Shoot Specialist</t>
         </is>
       </c>
       <c r="D92" s="33" t="inlineStr">
         <is>
-          <t>You decide all targets for direct targeting passes</t>
+          <t>Additional SHOT +10% on all received passes</t>
         </is>
       </c>
       <c r="E92" s="34" t="n"/>
@@ -5074,20 +5079,16 @@
       </c>
       <c r="C93" s="31" t="inlineStr">
         <is>
-          <t>Fox-Like First Step</t>
+          <t>Clutch Gene</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>All Move cards that reduce SHOT increase it by that amount instead.</t>
-        </is>
-      </c>
-      <c r="E93" s="6" t="inlineStr">
-        <is>
-          <t>Your Move cards are unaffected by opponents</t>
-        </is>
-      </c>
-      <c r="F93" s="139" t="n"/>
+          <t>SHOT x2 if attempting a shot with 1 or fewer cards in hand or Shot Clock 3 or less</t>
+        </is>
+      </c>
+      <c r="E93" s="7" t="n"/>
+      <c r="F93" s="138" t="n"/>
       <c r="G93" s="101" t="n"/>
       <c r="H93" s="102" t="n"/>
       <c r="I93" s="102" t="n"/>
@@ -5100,19 +5101,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C94" s="90" t="inlineStr">
-        <is>
-          <t>Freethrow Merchant</t>
-        </is>
-      </c>
-      <c r="D94" s="94" t="inlineStr">
-        <is>
-          <t>All Clamps on you grant 1 FT instead</t>
+      <c r="C94" s="32" t="inlineStr">
+        <is>
+          <t>Floor General</t>
+        </is>
+      </c>
+      <c r="D94" s="33" t="inlineStr">
+        <is>
+          <t>You decide all targets for direct targeting passes</t>
         </is>
       </c>
       <c r="E94" s="34" t="n"/>
       <c r="F94" s="138" t="n"/>
-      <c r="G94" s="125" t="n"/>
+      <c r="G94" s="107" t="n"/>
       <c r="H94" s="102" t="n"/>
       <c r="I94" s="102" t="n"/>
       <c r="J94" s="102" t="n"/>
@@ -5124,18 +5125,22 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C95" s="90" t="inlineStr">
-        <is>
-          <t>Generational Whistle</t>
-        </is>
-      </c>
-      <c r="D95" s="91" t="inlineStr">
-        <is>
-          <t>Take 1 additional FT</t>
-        </is>
-      </c>
-      <c r="E95" s="7" t="n"/>
-      <c r="F95" s="138" t="n"/>
+      <c r="C95" s="31" t="inlineStr">
+        <is>
+          <t>Fox-Like First Step</t>
+        </is>
+      </c>
+      <c r="D95" s="6" t="inlineStr">
+        <is>
+          <t>All Move cards that reduce SHOT increase it by that amount instead.</t>
+        </is>
+      </c>
+      <c r="E95" s="6" t="inlineStr">
+        <is>
+          <t>Your Move cards are unaffected by opponents</t>
+        </is>
+      </c>
+      <c r="F95" s="139" t="n"/>
       <c r="G95" s="101" t="n"/>
       <c r="H95" s="102" t="n"/>
       <c r="I95" s="102" t="n"/>
@@ -5148,19 +5153,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C96" s="32" t="inlineStr">
-        <is>
-          <t>Gravity</t>
-        </is>
-      </c>
-      <c r="D96" s="33" t="inlineStr">
-        <is>
-          <t>All Clamps automatically apply to you. +1 AST whenever another player attempts a shot</t>
+      <c r="C96" s="90" t="inlineStr">
+        <is>
+          <t>Freethrow Merchant</t>
+        </is>
+      </c>
+      <c r="D96" s="94" t="inlineStr">
+        <is>
+          <t>All Clamps on you grant 1 FT instead</t>
         </is>
       </c>
       <c r="E96" s="34" t="n"/>
       <c r="F96" s="138" t="n"/>
-      <c r="G96" s="107" t="n"/>
+      <c r="G96" s="125" t="n"/>
       <c r="H96" s="102" t="n"/>
       <c r="I96" s="102" t="n"/>
       <c r="J96" s="102" t="n"/>
@@ -5172,14 +5177,14 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C97" s="31" t="inlineStr">
-        <is>
-          <t>Great Conditioning</t>
-        </is>
-      </c>
-      <c r="D97" s="6" t="inlineStr">
-        <is>
-          <t>Immediately discard all Injury Game Breaks you draw and draw a new card for each</t>
+      <c r="C97" s="90" t="inlineStr">
+        <is>
+          <t>Generational Whistle</t>
+        </is>
+      </c>
+      <c r="D97" s="91" t="inlineStr">
+        <is>
+          <t>Take 1 additional FT</t>
         </is>
       </c>
       <c r="E97" s="7" t="n"/>
@@ -5198,12 +5203,12 @@
       </c>
       <c r="C98" s="32" t="inlineStr">
         <is>
-          <t>Hot Hand</t>
+          <t>Gravity</t>
         </is>
       </c>
       <c r="D98" s="33" t="inlineStr">
         <is>
-          <t>SHOT +20% if you scored last round.</t>
+          <t>All Clamps automatically apply to you. +1 AST whenever another player attempts a shot</t>
         </is>
       </c>
       <c r="E98" s="34" t="n"/>
@@ -5222,12 +5227,12 @@
       </c>
       <c r="C99" s="31" t="inlineStr">
         <is>
-          <t>Like That</t>
-        </is>
-      </c>
-      <c r="D99" s="91" t="inlineStr">
-        <is>
-          <t>Your SHOT % cannot be reduced</t>
+          <t>Great Conditioning</t>
+        </is>
+      </c>
+      <c r="D99" s="6" t="inlineStr">
+        <is>
+          <t>Immediately discard all Injury Game Breaks you draw and draw a new card for each</t>
         </is>
       </c>
       <c r="E99" s="7" t="n"/>
@@ -5246,21 +5251,17 @@
       </c>
       <c r="C100" s="32" t="inlineStr">
         <is>
-          <t>No Bag</t>
+          <t>Hot Hand</t>
         </is>
       </c>
       <c r="D100" s="33" t="inlineStr">
         <is>
-          <t>Cannot activate Move cards this round</t>
+          <t>SHOT +20% if you scored last round.</t>
         </is>
       </c>
       <c r="E100" s="34" t="n"/>
       <c r="F100" s="138" t="n"/>
-      <c r="G100" s="113" t="inlineStr">
-        <is>
-          <t>Bad card to draw</t>
-        </is>
-      </c>
+      <c r="G100" s="107" t="n"/>
       <c r="H100" s="102" t="n"/>
       <c r="I100" s="102" t="n"/>
       <c r="J100" s="102" t="n"/>
@@ -5274,12 +5275,12 @@
       </c>
       <c r="C101" s="31" t="inlineStr">
         <is>
-          <t>Point God</t>
-        </is>
-      </c>
-      <c r="D101" s="6" t="inlineStr">
-        <is>
-          <t>Draw 1 card following each of your passes</t>
+          <t>Like That</t>
+        </is>
+      </c>
+      <c r="D101" s="91" t="inlineStr">
+        <is>
+          <t>Your SHOT % cannot be reduced</t>
         </is>
       </c>
       <c r="E101" s="7" t="n"/>
@@ -5298,12 +5299,12 @@
       </c>
       <c r="C102" s="32" t="inlineStr">
         <is>
-          <t>Shooting Slump</t>
+          <t>No Bag</t>
         </is>
       </c>
       <c r="D102" s="33" t="inlineStr">
         <is>
-          <t>SHOT -20% this round</t>
+          <t>Cannot activate Move cards this round</t>
         </is>
       </c>
       <c r="E102" s="34" t="n"/>
@@ -5326,12 +5327,12 @@
       </c>
       <c r="C103" s="31" t="inlineStr">
         <is>
-          <t>Shot Creator</t>
+          <t>Point God</t>
         </is>
       </c>
       <c r="D103" s="6" t="inlineStr">
         <is>
-          <t>Draw 1 additional card after every draw effect</t>
+          <t>Draw 1 card following each of your passes</t>
         </is>
       </c>
       <c r="E103" s="7" t="n"/>
@@ -5350,17 +5351,21 @@
       </c>
       <c r="C104" s="32" t="inlineStr">
         <is>
-          <t>Sixth Man</t>
+          <t>Shooting Slump</t>
         </is>
       </c>
       <c r="D104" s="33" t="inlineStr">
         <is>
-          <t>SHOT = 100% if taking 6th shot of the round</t>
+          <t>SHOT -20% this round</t>
         </is>
       </c>
       <c r="E104" s="34" t="n"/>
       <c r="F104" s="138" t="n"/>
-      <c r="G104" s="107" t="n"/>
+      <c r="G104" s="113" t="inlineStr">
+        <is>
+          <t>Bad card to draw</t>
+        </is>
+      </c>
       <c r="H104" s="102" t="n"/>
       <c r="I104" s="102" t="n"/>
       <c r="J104" s="102" t="n"/>
@@ -5374,12 +5379,12 @@
       </c>
       <c r="C105" s="31" t="inlineStr">
         <is>
-          <t>Sniper</t>
+          <t>Shot Creator</t>
         </is>
       </c>
       <c r="D105" s="6" t="inlineStr">
         <is>
-          <t>SHOT +10% on all Three-Point Line Shots</t>
+          <t>Draw 1 additional card after every draw effect</t>
         </is>
       </c>
       <c r="E105" s="7" t="n"/>
@@ -5398,12 +5403,12 @@
       </c>
       <c r="C106" s="32" t="inlineStr">
         <is>
-          <t>Splash Cousin</t>
+          <t>Sixth Man</t>
         </is>
       </c>
       <c r="D106" s="33" t="inlineStr">
         <is>
-          <t>All Three-Point Line Shots: SHOT = 100%</t>
+          <t>SHOT = 100% if taking 6th shot of the round</t>
         </is>
       </c>
       <c r="E106" s="34" t="n"/>
@@ -5422,12 +5427,12 @@
       </c>
       <c r="C107" s="31" t="inlineStr">
         <is>
-          <t>Unguardable</t>
-        </is>
-      </c>
-      <c r="D107" s="91" t="inlineStr">
-        <is>
-          <t>All Clamps on you have no effect on SHOT %</t>
+          <t>Sniper</t>
+        </is>
+      </c>
+      <c r="D107" s="6" t="inlineStr">
+        <is>
+          <t>SHOT +10% on all Three-Point Line Shots</t>
         </is>
       </c>
       <c r="E107" s="7" t="n"/>
@@ -5446,72 +5451,72 @@
       </c>
       <c r="C108" s="32" t="inlineStr">
         <is>
-          <t>Lethal Shooter</t>
+          <t>Splash Cousin</t>
         </is>
       </c>
       <c r="D108" s="33" t="inlineStr">
         <is>
-          <t>SHOT = 100% on next shot attempt after rebounding your own miss.</t>
+          <t>All Three-Point Line Shots: SHOT = 100%</t>
         </is>
       </c>
       <c r="E108" s="34" t="n"/>
       <c r="F108" s="138" t="n"/>
-      <c r="G108" s="113" t="inlineStr">
-        <is>
-          <t>Special text: “I understand it now”</t>
-        </is>
-      </c>
+      <c r="G108" s="107" t="n"/>
       <c r="H108" s="102" t="n"/>
       <c r="I108" s="102" t="n"/>
       <c r="J108" s="102" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="61" t="n"/>
-      <c r="B109" s="62" t="inlineStr">
+      <c r="A109" s="29" t="n"/>
+      <c r="B109" s="30" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C109" s="66" t="inlineStr">
-        <is>
-          <t>Ball Pounder</t>
-        </is>
-      </c>
-      <c r="D109" s="95" t="inlineStr">
-        <is>
-          <t>All Dribble cards you play draw an additional card but lower SHOT by an additional 10%</t>
-        </is>
-      </c>
-      <c r="E109" s="68" t="n"/>
-      <c r="F109" s="140" t="n"/>
-      <c r="G109" s="126" t="n"/>
-      <c r="H109" s="117" t="n"/>
-      <c r="I109" s="117" t="n"/>
-      <c r="J109" s="117" t="n"/>
+      <c r="C109" s="31" t="inlineStr">
+        <is>
+          <t>Unguardable</t>
+        </is>
+      </c>
+      <c r="D109" s="91" t="inlineStr">
+        <is>
+          <t>All Clamps on you have no effect on SHOT %</t>
+        </is>
+      </c>
+      <c r="E109" s="7" t="n"/>
+      <c r="F109" s="138" t="n"/>
+      <c r="G109" s="101" t="n"/>
+      <c r="H109" s="102" t="n"/>
+      <c r="I109" s="102" t="n"/>
+      <c r="J109" s="102" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="61" t="n"/>
-      <c r="B110" s="62" t="inlineStr">
+      <c r="A110" s="29" t="n"/>
+      <c r="B110" s="30" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C110" s="66" t="inlineStr">
-        <is>
-          <t>Unselfish</t>
-        </is>
-      </c>
-      <c r="D110" s="95" t="inlineStr">
-        <is>
-          <t>Draw 1 card whenever you pass the ball at 50% SHOT or higher</t>
-        </is>
-      </c>
-      <c r="E110" s="68" t="n"/>
-      <c r="F110" s="140" t="n"/>
-      <c r="G110" s="126" t="n"/>
-      <c r="H110" s="117" t="n"/>
-      <c r="I110" s="117" t="n"/>
-      <c r="J110" s="117" t="n"/>
+      <c r="C110" s="32" t="inlineStr">
+        <is>
+          <t>Lethal Shooter</t>
+        </is>
+      </c>
+      <c r="D110" s="33" t="inlineStr">
+        <is>
+          <t>SHOT = 100% on next shot attempt after rebounding your own miss.</t>
+        </is>
+      </c>
+      <c r="E110" s="34" t="n"/>
+      <c r="F110" s="138" t="n"/>
+      <c r="G110" s="113" t="inlineStr">
+        <is>
+          <t>Special text: “I understand it now”</t>
+        </is>
+      </c>
+      <c r="H110" s="102" t="n"/>
+      <c r="I110" s="102" t="n"/>
+      <c r="J110" s="102" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="61" t="n"/>
@@ -5522,12 +5527,12 @@
       </c>
       <c r="C111" s="66" t="inlineStr">
         <is>
-          <t>Dirty Player</t>
+          <t>Ball Pounder</t>
         </is>
       </c>
       <c r="D111" s="95" t="inlineStr">
         <is>
-          <t>When sending Clamps, the clamped player discards 1 if they have any Injuries</t>
+          <t>All Dribble cards you play draw an additional card but lower SHOT by an additional 10%</t>
         </is>
       </c>
       <c r="E111" s="68" t="n"/>
@@ -5546,21 +5551,20 @@
       </c>
       <c r="C112" s="66" t="inlineStr">
         <is>
-          <t>Villainous Reputation</t>
+          <t>Unselfish</t>
         </is>
       </c>
       <c r="D112" s="95" t="inlineStr">
         <is>
-          <t>Discard 1 whenever any Whistle triggers</t>
+          <t>Draw 1 card whenever you pass the ball at 50% SHOT or higher</t>
         </is>
       </c>
       <c r="E112" s="68" t="n"/>
       <c r="F112" s="140" t="n"/>
-      <c r="G112" s="126" t="inlineStr">
-        <is>
-          <t>Discarded during play, it attaches to a random player — possibly you again</t>
-        </is>
-      </c>
+      <c r="G112" s="126" t="n"/>
+      <c r="H112" s="117" t="n"/>
+      <c r="I112" s="117" t="n"/>
+      <c r="J112" s="117" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="61" t="n"/>
@@ -5571,24 +5575,73 @@
       </c>
       <c r="C113" s="66" t="inlineStr">
         <is>
-          <t>Free Agent</t>
+          <t>Dirty Player</t>
         </is>
       </c>
       <c r="D113" s="95" t="inlineStr">
         <is>
-          <t>Discard your hand. Play a card at random from a player of your choosing (they keep it)</t>
+          <t>When sending Clamps, the clamped player discards 1 if they have any Injuries</t>
         </is>
       </c>
       <c r="E113" s="68" t="n"/>
       <c r="F113" s="140" t="n"/>
-      <c r="G113" s="126" t="inlineStr">
+      <c r="G113" s="126" t="n"/>
+      <c r="H113" s="117" t="n"/>
+      <c r="I113" s="117" t="n"/>
+      <c r="J113" s="117" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="61" t="n"/>
+      <c r="B114" s="62" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C114" s="66" t="inlineStr">
+        <is>
+          <t>Villainous Reputation</t>
+        </is>
+      </c>
+      <c r="D114" s="95" t="inlineStr">
+        <is>
+          <t>Discard 1 whenever any Whistle triggers</t>
+        </is>
+      </c>
+      <c r="E114" s="68" t="n"/>
+      <c r="F114" s="140" t="n"/>
+      <c r="G114" s="126" t="inlineStr">
+        <is>
+          <t>Discarded during play, it attaches to a random player — possibly you again</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="61" t="n"/>
+      <c r="B115" s="62" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C115" s="66" t="inlineStr">
+        <is>
+          <t>Free Agent</t>
+        </is>
+      </c>
+      <c r="D115" s="95" t="inlineStr">
+        <is>
+          <t>Discard your hand. Play a card at random from a player of your choosing (they keep it)</t>
+        </is>
+      </c>
+      <c r="E115" s="68" t="n"/>
+      <c r="F115" s="140" t="n"/>
+      <c r="G115" s="126" t="inlineStr">
         <is>
           <t>The discard waits for the draw chain to finish. Target is shuffled first and is affected by Floor General. Your own draws are kept. All-0 rebounds are yours; otherwise you cannot bid</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="100">
+  <mergeCells count="102">
     <mergeCell ref="G55:J55"/>
     <mergeCell ref="G4:J4"/>
     <mergeCell ref="G109:J109"/>
@@ -5600,6 +5653,7 @@
     <mergeCell ref="G72:J72"/>
     <mergeCell ref="G81:J81"/>
     <mergeCell ref="G96:J96"/>
+    <mergeCell ref="G5:J5"/>
     <mergeCell ref="G71:J71"/>
     <mergeCell ref="G8:J8"/>
     <mergeCell ref="G57:J57"/>
@@ -5613,22 +5667,22 @@
     <mergeCell ref="G108:J108"/>
     <mergeCell ref="G58:J58"/>
     <mergeCell ref="G110:J110"/>
+    <mergeCell ref="G113:J113"/>
     <mergeCell ref="G20:J20"/>
+    <mergeCell ref="G29:J29"/>
     <mergeCell ref="G91:J91"/>
-    <mergeCell ref="G29:J29"/>
-    <mergeCell ref="G85:J85"/>
     <mergeCell ref="G100:J100"/>
     <mergeCell ref="G94:J94"/>
-    <mergeCell ref="G84:J84"/>
+    <mergeCell ref="G85:J85"/>
     <mergeCell ref="G75:J75"/>
     <mergeCell ref="G44:J44"/>
     <mergeCell ref="G22:J22"/>
+    <mergeCell ref="G102:J102"/>
     <mergeCell ref="G31:J31"/>
-    <mergeCell ref="G102:J102"/>
     <mergeCell ref="G12:J12"/>
     <mergeCell ref="G77:J77"/>
+    <mergeCell ref="G86:J86"/>
     <mergeCell ref="G21:J21"/>
-    <mergeCell ref="G86:J86"/>
     <mergeCell ref="G67:J67"/>
     <mergeCell ref="G61:J61"/>
     <mergeCell ref="G70:J70"/>
@@ -5636,6 +5690,8 @@
     <mergeCell ref="G97:J97"/>
     <mergeCell ref="G7:J7"/>
     <mergeCell ref="G38:J38"/>
+    <mergeCell ref="G84:J84"/>
+    <mergeCell ref="G112:J112"/>
     <mergeCell ref="G45:J45"/>
     <mergeCell ref="G62:J62"/>
     <mergeCell ref="G49:J49"/>
@@ -5668,27 +5724,26 @@
     <mergeCell ref="G54:J54"/>
     <mergeCell ref="G63:J63"/>
     <mergeCell ref="G41:J41"/>
+    <mergeCell ref="G106:J106"/>
     <mergeCell ref="G50:J50"/>
-    <mergeCell ref="G106:J106"/>
     <mergeCell ref="G56:J56"/>
+    <mergeCell ref="G14:J14"/>
     <mergeCell ref="G105:J105"/>
     <mergeCell ref="G43:J43"/>
     <mergeCell ref="G52:J52"/>
     <mergeCell ref="G27:J27"/>
     <mergeCell ref="G98:J98"/>
+    <mergeCell ref="G107:J107"/>
     <mergeCell ref="G36:J36"/>
     <mergeCell ref="G42:J42"/>
-    <mergeCell ref="G107:J107"/>
     <mergeCell ref="G17:J17"/>
     <mergeCell ref="G19:J19"/>
+    <mergeCell ref="G93:J93"/>
     <mergeCell ref="G28:J28"/>
-    <mergeCell ref="G93:J93"/>
     <mergeCell ref="G6:J6"/>
     <mergeCell ref="G69:J69"/>
     <mergeCell ref="G92:J92"/>
     <mergeCell ref="G30:J30"/>
-    <mergeCell ref="G5:J5"/>
-    <mergeCell ref="G14:J14"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
Franchise Player, and Floor General names everything
Floor General was aiming passes only. It names every target on the floor now —
who a pass finds, which card comes out of a hand, which branch a card takes —
asked through one `asker(instead:in:)` so a prompt added later cannot forget it.
Choices about your own board are not targets and stay yours.

Franchise Player is the first question over two kinds of card at once: his
passives are face up and his hand is not, so the answer says which. `CardPick`
is named-or-position, and the picker draws the backs after the faces.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -2549,7 +2549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J115"/>
+  <dimension ref="A1:J116"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="22.25" customHeight="1"/>
   <cols>
     <col width="15.5" customWidth="1" style="8" min="1" max="1"/>
@@ -2626,39 +2626,40 @@
         </is>
       </c>
       <c r="B2" s="12">
-        <f>COUNTIF($B$5:$B$115,"Pass")</f>
+        <f>COUNTIF($B$5:$B$116,"Pass")</f>
         <v/>
       </c>
       <c r="C2" s="13">
-        <f>COUNTIF($B$5:$B$115,"Move")+COUNTIF($B$5:$B$115,"Special Move")</f>
+        <f>COUNTIF($B$5:$B$116,"Move")+COUNTIF($B$5:$B$116,"Special Move")</f>
         <v/>
       </c>
       <c r="D2" s="14">
-        <f>COUNTIF($B$5:$B$115,"Clamp")</f>
+        <f>COUNTIF($B$5:$B$116,"Clamp")</f>
         <v/>
       </c>
       <c r="E2" s="15">
-        <f>COUNTIF($B$5:$B$115,"Whistle")</f>
+        <f>COUNTIF($B$5:$B$116,"Whistle")</f>
         <v/>
       </c>
       <c r="F2" s="16">
-        <f>COUNTIF($B$5:$B$115,"Game Break")</f>
+        <f>COUNTIF($B$5:$B$116,"Game Break")</f>
         <v/>
       </c>
       <c r="G2" s="18">
-        <f>COUNTIF($B$5:$B$115,"Injury GB")</f>
+        <f>COUNTIF($B$5:$B$116,"Injury GB")</f>
         <v/>
       </c>
       <c r="H2" s="19">
-        <f>COUNTIF($B$5:$B$115,"Devastating Injury GB")</f>
+        <f>COUNTIF($B$5:$B$116,"Devastating Injury GB")</f>
         <v/>
       </c>
       <c r="I2" s="17">
-        <f>COUNTIF($B$5:$B$115,"Intangible")</f>
+        <f>COUNTIF($B$5:$B$116,"Intangible")</f>
         <v/>
       </c>
       <c r="J2" s="19" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4" ht="20.75" customHeight="1" s="132" thickBot="1">
       <c r="A4" s="123" t="inlineStr">
         <is>
@@ -2702,7 +2703,7 @@
         </is>
       </c>
       <c r="B5" s="22">
-        <f>COUNTIF($B$5:$B$115,"Pass")</f>
+        <f>COUNTIF($B$5:$B$116,"Pass")</f>
         <v/>
       </c>
       <c r="C5" s="23" t="n"/>
@@ -2959,7 +2960,7 @@
         </is>
       </c>
       <c r="B15" s="40">
-        <f>COUNTIF($B$5:$B$115,"Move")+COUNTIF($B$5:$B$115,"Special Move")</f>
+        <f>COUNTIF($B$5:$B$116,"Move")+COUNTIF($B$5:$B$116,"Special Move")</f>
         <v/>
       </c>
       <c r="C15" s="41" t="n"/>
@@ -3333,7 +3334,7 @@
         </is>
       </c>
       <c r="B28" s="43">
-        <f>COUNTIF($B$5:$B$115,"Special Move")</f>
+        <f>COUNTIF($B$5:$B$116,"Special Move")</f>
         <v/>
       </c>
       <c r="C28" s="44" t="n"/>
@@ -3718,7 +3719,7 @@
         </is>
       </c>
       <c r="B41" s="59">
-        <f>COUNTIF($B$5:$B$115,"Clamp")</f>
+        <f>COUNTIF($B$5:$B$116,"Clamp")</f>
         <v/>
       </c>
       <c r="C41" s="60" t="n"/>
@@ -3887,7 +3888,7 @@
         </is>
       </c>
       <c r="B47" s="59">
-        <f>COUNTIF($B$5:$B$115,"Whistle")</f>
+        <f>COUNTIF($B$5:$B$116,"Whistle")</f>
         <v/>
       </c>
       <c r="C47" s="60" t="n"/>
@@ -4346,7 +4347,7 @@
         </is>
       </c>
       <c r="B65" s="59">
-        <f>COUNTIF($B$5:$B$115,"Game Break")</f>
+        <f>COUNTIF($B$5:$B$116,"Game Break")</f>
         <v/>
       </c>
       <c r="C65" s="60" t="n"/>
@@ -4917,7 +4918,7 @@
         </is>
       </c>
       <c r="B86" s="56">
-        <f>COUNTIF($B$5:$B$115,"Injury GB")</f>
+        <f>COUNTIF($B$5:$B$116,"Injury GB")</f>
         <v/>
       </c>
       <c r="C86" s="57" t="n"/>
@@ -4962,7 +4963,7 @@
         </is>
       </c>
       <c r="B88" s="59">
-        <f>COUNTIF($B$5:$B$115,"Devastating Injury GB")</f>
+        <f>COUNTIF($B$5:$B$116,"Devastating Injury GB")</f>
         <v/>
       </c>
       <c r="C88" s="60" t="n"/>
@@ -5005,7 +5006,7 @@
         </is>
       </c>
       <c r="B90" s="56">
-        <f>COUNTIF($B$5:$B$115,"Intangible")</f>
+        <f>COUNTIF($B$5:$B$116,"Intangible")</f>
         <v/>
       </c>
       <c r="C90" s="57" t="n"/>
@@ -5107,7 +5108,7 @@
       </c>
       <c r="D94" s="33" t="inlineStr">
         <is>
-          <t>You decide all targets for direct targeting passes</t>
+          <t>You choose all targets of all kinds — card declarations, non auto-pass targets, and the rest</t>
         </is>
       </c>
       <c r="E94" s="34" t="n"/>
@@ -5639,8 +5640,32 @@
         </is>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" s="61" t="n"/>
+      <c r="B116" s="62" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C116" s="66" t="inlineStr">
+        <is>
+          <t>Franchise Player</t>
+        </is>
+      </c>
+      <c r="D116" s="95" t="inlineStr">
+        <is>
+          <t>When passing, choose 1 of the new player's Intangibles or a card in their hand for them to discard</t>
+        </is>
+      </c>
+      <c r="E116" s="68" t="n"/>
+      <c r="F116" s="140" t="n"/>
+      <c r="G116" s="126" t="n"/>
+      <c r="H116" s="117" t="n"/>
+      <c r="I116" s="117" t="n"/>
+      <c r="J116" s="117" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="102">
+  <mergeCells count="103">
     <mergeCell ref="G55:J55"/>
     <mergeCell ref="G4:J4"/>
     <mergeCell ref="G109:J109"/>
@@ -5652,6 +5677,7 @@
     <mergeCell ref="G72:J72"/>
     <mergeCell ref="G81:J81"/>
     <mergeCell ref="G96:J96"/>
+    <mergeCell ref="G5:J5"/>
     <mergeCell ref="G71:J71"/>
     <mergeCell ref="G8:J8"/>
     <mergeCell ref="G57:J57"/>
@@ -5708,6 +5734,7 @@
     <mergeCell ref="G11:J11"/>
     <mergeCell ref="G39:J39"/>
     <mergeCell ref="G101:J101"/>
+    <mergeCell ref="G116:J116"/>
     <mergeCell ref="G103:J103"/>
     <mergeCell ref="G37:J37"/>
     <mergeCell ref="A4:B4"/>
@@ -5725,6 +5752,7 @@
     <mergeCell ref="G50:J50"/>
     <mergeCell ref="G106:J106"/>
     <mergeCell ref="G56:J56"/>
+    <mergeCell ref="G14:J14"/>
     <mergeCell ref="G105:J105"/>
     <mergeCell ref="G43:J43"/>
     <mergeCell ref="G52:J52"/>
@@ -5741,8 +5769,6 @@
     <mergeCell ref="G69:J69"/>
     <mergeCell ref="G92:J92"/>
     <mergeCell ref="G30:J30"/>
-    <mergeCell ref="G5:J5"/>
-    <mergeCell ref="G14:J14"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
Team Doctor, and Unselfish means what it says
Unselfish was a pass at 50% or better. It is what the card actually says now:
one place — Rules.credit — decides what "positively affects another player"
means, and every route that hands somebody the ball, a card, a point, a trip to
the line, or takes something off them calls it. Passing, inbounding, a Nutmeg's
card travelling on, a Whistle that draws for the man it caught, a Clear Path
paying him, a Timeout dealing the table in. Never for helping yourself, and
never for a Game Break — a Break is an event, not a thing anybody did.

The SHOT it pays is owed to the player rather than to the board, so passing the
ball away does not hand the bonus to whoever ends up shooting.

Team Doctor only offers the hurt as choices, and only pays for looking after
somebody else.

Franchise Player can wave it off — the card says "can", so declining is an
answer rather than a missing button.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -2549,7 +2549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J116"/>
+  <dimension ref="A1:J117"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="22.25" customHeight="1"/>
   <cols>
     <col width="15.5" customWidth="1" style="8" min="1" max="1"/>
@@ -2626,35 +2626,35 @@
         </is>
       </c>
       <c r="B2" s="12">
-        <f>COUNTIF($B$5:$B$116,"Pass")</f>
+        <f>COUNTIF($B$5:$B$117,"Pass")</f>
         <v/>
       </c>
       <c r="C2" s="13">
-        <f>COUNTIF($B$5:$B$116,"Move")+COUNTIF($B$5:$B$116,"Special Move")</f>
+        <f>COUNTIF($B$5:$B$117,"Move")+COUNTIF($B$5:$B$117,"Special Move")</f>
         <v/>
       </c>
       <c r="D2" s="14">
-        <f>COUNTIF($B$5:$B$116,"Clamp")</f>
+        <f>COUNTIF($B$5:$B$117,"Clamp")</f>
         <v/>
       </c>
       <c r="E2" s="15">
-        <f>COUNTIF($B$5:$B$116,"Whistle")</f>
+        <f>COUNTIF($B$5:$B$117,"Whistle")</f>
         <v/>
       </c>
       <c r="F2" s="16">
-        <f>COUNTIF($B$5:$B$116,"Game Break")</f>
+        <f>COUNTIF($B$5:$B$117,"Game Break")</f>
         <v/>
       </c>
       <c r="G2" s="18">
-        <f>COUNTIF($B$5:$B$116,"Injury GB")</f>
+        <f>COUNTIF($B$5:$B$117,"Injury GB")</f>
         <v/>
       </c>
       <c r="H2" s="19">
-        <f>COUNTIF($B$5:$B$116,"Devastating Injury GB")</f>
+        <f>COUNTIF($B$5:$B$117,"Devastating Injury GB")</f>
         <v/>
       </c>
       <c r="I2" s="17">
-        <f>COUNTIF($B$5:$B$116,"Intangible")</f>
+        <f>COUNTIF($B$5:$B$117,"Intangible")</f>
         <v/>
       </c>
       <c r="J2" s="19" t="n"/>
@@ -2703,7 +2703,7 @@
         </is>
       </c>
       <c r="B5" s="22">
-        <f>COUNTIF($B$5:$B$116,"Pass")</f>
+        <f>COUNTIF($B$5:$B$117,"Pass")</f>
         <v/>
       </c>
       <c r="C5" s="23" t="n"/>
@@ -2960,7 +2960,7 @@
         </is>
       </c>
       <c r="B15" s="40">
-        <f>COUNTIF($B$5:$B$116,"Move")+COUNTIF($B$5:$B$116,"Special Move")</f>
+        <f>COUNTIF($B$5:$B$117,"Move")+COUNTIF($B$5:$B$117,"Special Move")</f>
         <v/>
       </c>
       <c r="C15" s="41" t="n"/>
@@ -3334,7 +3334,7 @@
         </is>
       </c>
       <c r="B28" s="43">
-        <f>COUNTIF($B$5:$B$116,"Special Move")</f>
+        <f>COUNTIF($B$5:$B$117,"Special Move")</f>
         <v/>
       </c>
       <c r="C28" s="44" t="n"/>
@@ -3719,7 +3719,7 @@
         </is>
       </c>
       <c r="B41" s="59">
-        <f>COUNTIF($B$5:$B$116,"Clamp")</f>
+        <f>COUNTIF($B$5:$B$117,"Clamp")</f>
         <v/>
       </c>
       <c r="C41" s="60" t="n"/>
@@ -3888,7 +3888,7 @@
         </is>
       </c>
       <c r="B47" s="59">
-        <f>COUNTIF($B$5:$B$116,"Whistle")</f>
+        <f>COUNTIF($B$5:$B$117,"Whistle")</f>
         <v/>
       </c>
       <c r="C47" s="60" t="n"/>
@@ -4347,7 +4347,7 @@
         </is>
       </c>
       <c r="B65" s="59">
-        <f>COUNTIF($B$5:$B$116,"Game Break")</f>
+        <f>COUNTIF($B$5:$B$117,"Game Break")</f>
         <v/>
       </c>
       <c r="C65" s="60" t="n"/>
@@ -4912,160 +4912,162 @@
       <c r="J85" s="102" t="n"/>
     </row>
     <row r="86" ht="56" customHeight="1" s="132">
-      <c r="A86" s="55" t="inlineStr">
-        <is>
-          <t>Injury GB</t>
-        </is>
-      </c>
-      <c r="B86" s="56">
-        <f>COUNTIF($B$5:$B$116,"Injury GB")</f>
-        <v/>
-      </c>
-      <c r="C86" s="57" t="n"/>
-      <c r="D86" s="57" t="n"/>
-      <c r="E86" s="57" t="n"/>
-      <c r="F86" s="88" t="n"/>
-      <c r="G86" s="108" t="n"/>
+      <c r="A86" s="29" t="n"/>
+      <c r="B86" s="30" t="inlineStr">
+        <is>
+          <t>Game Break</t>
+        </is>
+      </c>
+      <c r="C86" s="134" t="inlineStr">
+        <is>
+          <t>Team Doctor</t>
+        </is>
+      </c>
+      <c r="D86" s="91" t="inlineStr">
+        <is>
+          <t>Discard 1 Injury from a player of choice. Draw 2 cards if not choosing yourself</t>
+        </is>
+      </c>
+      <c r="E86" s="7" t="n"/>
+      <c r="F86" s="76" t="n">
+        <v>3</v>
+      </c>
+      <c r="G86" s="111" t="n"/>
       <c r="H86" s="102" t="n"/>
       <c r="I86" s="102" t="n"/>
       <c r="J86" s="102" t="n"/>
     </row>
     <row r="87" ht="56" customHeight="1" s="132">
-      <c r="A87" s="29" t="n"/>
-      <c r="B87" s="30" t="inlineStr">
+      <c r="A87" s="55" t="inlineStr">
         <is>
           <t>Injury GB</t>
         </is>
       </c>
-      <c r="C87" s="31" t="inlineStr">
-        <is>
-          <t>Bone Bruise</t>
-        </is>
-      </c>
-      <c r="D87" s="91" t="inlineStr">
-        <is>
-          <t>Discard 1 card at the start of each turn after drawing (your choice)</t>
-        </is>
-      </c>
-      <c r="E87" s="7" t="n"/>
-      <c r="F87" s="76" t="n">
-        <v>3</v>
-      </c>
-      <c r="G87" s="101" t="n"/>
+      <c r="B87" s="56">
+        <f>COUNTIF($B$5:$B$117,"Injury GB")</f>
+        <v/>
+      </c>
+      <c r="C87" s="57" t="n"/>
+      <c r="D87" s="57" t="n"/>
+      <c r="E87" s="57" t="n"/>
+      <c r="F87" s="88" t="n"/>
+      <c r="G87" s="108" t="n"/>
       <c r="H87" s="102" t="n"/>
       <c r="I87" s="102" t="n"/>
       <c r="J87" s="102" t="n"/>
     </row>
     <row r="88" ht="28" customHeight="1" s="132">
-      <c r="A88" s="58" t="inlineStr">
+      <c r="A88" s="29" t="n"/>
+      <c r="B88" s="30" t="inlineStr">
+        <is>
+          <t>Injury GB</t>
+        </is>
+      </c>
+      <c r="C88" s="31" t="inlineStr">
+        <is>
+          <t>Bone Bruise</t>
+        </is>
+      </c>
+      <c r="D88" s="91" t="inlineStr">
+        <is>
+          <t>Discard 1 card at the start of each turn after drawing (your choice)</t>
+        </is>
+      </c>
+      <c r="E88" s="7" t="n"/>
+      <c r="F88" s="76" t="n">
+        <v>3</v>
+      </c>
+      <c r="G88" s="101" t="n"/>
+      <c r="H88" s="102" t="n"/>
+      <c r="I88" s="102" t="n"/>
+      <c r="J88" s="102" t="n"/>
+    </row>
+    <row r="89" ht="42" customHeight="1" s="132">
+      <c r="A89" s="58" t="inlineStr">
         <is>
           <t>Devastating Injury GB</t>
         </is>
       </c>
-      <c r="B88" s="59">
-        <f>COUNTIF($B$5:$B$116,"Devastating Injury GB")</f>
+      <c r="B89" s="59">
+        <f>COUNTIF($B$5:$B$117,"Devastating Injury GB")</f>
         <v/>
       </c>
-      <c r="C88" s="60" t="n"/>
-      <c r="D88" s="60" t="n"/>
-      <c r="E88" s="60" t="n"/>
-      <c r="F88" s="86" t="n"/>
-      <c r="G88" s="109" t="n"/>
-      <c r="H88" s="110" t="n"/>
-      <c r="I88" s="110" t="n"/>
-      <c r="J88" s="110" t="n"/>
-    </row>
-    <row r="89" ht="42" customHeight="1" s="132">
-      <c r="A89" s="50" t="n"/>
-      <c r="B89" s="51" t="inlineStr">
+      <c r="C89" s="60" t="n"/>
+      <c r="D89" s="60" t="n"/>
+      <c r="E89" s="60" t="n"/>
+      <c r="F89" s="86" t="n"/>
+      <c r="G89" s="109" t="n"/>
+      <c r="H89" s="110" t="n"/>
+      <c r="I89" s="110" t="n"/>
+      <c r="J89" s="110" t="n"/>
+    </row>
+    <row r="90" ht="28" customHeight="1" s="132">
+      <c r="A90" s="50" t="n"/>
+      <c r="B90" s="51" t="inlineStr">
         <is>
           <t>Devastating Injury GB</t>
         </is>
       </c>
-      <c r="C89" s="136" t="inlineStr">
+      <c r="C90" s="136" t="inlineStr">
         <is>
           <t>Torn Achilles</t>
         </is>
       </c>
-      <c r="D89" s="137" t="inlineStr">
+      <c r="D90" s="137" t="inlineStr">
         <is>
           <t>Hand is locked every turn except 1 card (randomly)</t>
         </is>
       </c>
-      <c r="E89" s="54" t="n"/>
-      <c r="F89" s="141" t="n"/>
-      <c r="G89" s="114" t="n"/>
-      <c r="H89" s="115" t="n"/>
-      <c r="I89" s="115" t="n"/>
-      <c r="J89" s="115" t="n"/>
-    </row>
-    <row r="90" ht="28" customHeight="1" s="132">
-      <c r="A90" s="55" t="inlineStr">
+      <c r="E90" s="54" t="n"/>
+      <c r="F90" s="141" t="n"/>
+      <c r="G90" s="114" t="n"/>
+      <c r="H90" s="115" t="n"/>
+      <c r="I90" s="115" t="n"/>
+      <c r="J90" s="115" t="n"/>
+    </row>
+    <row r="91" ht="42" customHeight="1" s="132">
+      <c r="A91" s="55" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="B90" s="56">
-        <f>COUNTIF($B$5:$B$116,"Intangible")</f>
+      <c r="B91" s="56">
+        <f>COUNTIF($B$5:$B$117,"Intangible")</f>
         <v/>
       </c>
-      <c r="C90" s="57" t="n"/>
-      <c r="D90" s="57" t="n"/>
-      <c r="E90" s="57" t="n"/>
-      <c r="F90" s="88" t="n"/>
-      <c r="G90" s="108" t="n"/>
-      <c r="H90" s="102" t="n"/>
-      <c r="I90" s="102" t="n"/>
-      <c r="J90" s="102" t="n"/>
-    </row>
-    <row r="91" ht="42" customHeight="1" s="132">
-      <c r="A91" s="96" t="inlineStr">
-        <is>
-          <t>All intangibles are limited to 1</t>
-        </is>
-      </c>
-      <c r="B91" s="30" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C91" s="31" t="inlineStr">
-        <is>
-          <t>Board-Crasher</t>
-        </is>
-      </c>
-      <c r="D91" s="6" t="inlineStr">
-        <is>
-          <t>SHOT +10% upon Rebounding your own missed shot</t>
-        </is>
-      </c>
-      <c r="E91" s="7" t="n"/>
-      <c r="F91" s="138" t="n"/>
-      <c r="G91" s="101" t="n"/>
+      <c r="C91" s="57" t="n"/>
+      <c r="D91" s="57" t="n"/>
+      <c r="E91" s="57" t="n"/>
+      <c r="F91" s="88" t="n"/>
+      <c r="G91" s="108" t="n"/>
       <c r="H91" s="102" t="n"/>
       <c r="I91" s="102" t="n"/>
       <c r="J91" s="102" t="n"/>
     </row>
     <row r="92" ht="14" customHeight="1" s="132">
-      <c r="A92" s="29" t="n"/>
+      <c r="A92" s="96" t="inlineStr">
+        <is>
+          <t>All intangibles are limited to 1</t>
+        </is>
+      </c>
       <c r="B92" s="30" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C92" s="32" t="inlineStr">
-        <is>
-          <t>Catch &amp; Shoot Specialist</t>
-        </is>
-      </c>
-      <c r="D92" s="33" t="inlineStr">
-        <is>
-          <t>Additional SHOT +10% on all received passes</t>
-        </is>
-      </c>
-      <c r="E92" s="34" t="n"/>
+      <c r="C92" s="31" t="inlineStr">
+        <is>
+          <t>Board-Crasher</t>
+        </is>
+      </c>
+      <c r="D92" s="6" t="inlineStr">
+        <is>
+          <t>SHOT +10% upon Rebounding your own missed shot</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="n"/>
       <c r="F92" s="138" t="n"/>
-      <c r="G92" s="107" t="n"/>
+      <c r="G92" s="101" t="n"/>
       <c r="H92" s="102" t="n"/>
       <c r="I92" s="102" t="n"/>
       <c r="J92" s="102" t="n"/>
@@ -5077,19 +5079,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C93" s="31" t="inlineStr">
-        <is>
-          <t>Clutch Gene</t>
-        </is>
-      </c>
-      <c r="D93" s="6" t="inlineStr">
-        <is>
-          <t>SHOT x2 if attempting a shot with 1 or fewer cards in hand or Shot Clock 3 or less</t>
-        </is>
-      </c>
-      <c r="E93" s="7" t="n"/>
+      <c r="C93" s="32" t="inlineStr">
+        <is>
+          <t>Catch &amp; Shoot Specialist</t>
+        </is>
+      </c>
+      <c r="D93" s="33" t="inlineStr">
+        <is>
+          <t>Additional SHOT +10% on all received passes</t>
+        </is>
+      </c>
+      <c r="E93" s="34" t="n"/>
       <c r="F93" s="138" t="n"/>
-      <c r="G93" s="101" t="n"/>
+      <c r="G93" s="107" t="n"/>
       <c r="H93" s="102" t="n"/>
       <c r="I93" s="102" t="n"/>
       <c r="J93" s="102" t="n"/>
@@ -5101,19 +5103,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C94" s="32" t="inlineStr">
-        <is>
-          <t>Floor General</t>
-        </is>
-      </c>
-      <c r="D94" s="33" t="inlineStr">
-        <is>
-          <t>You choose all targets of all kinds — card declarations, non auto-pass targets, and the rest</t>
-        </is>
-      </c>
-      <c r="E94" s="34" t="n"/>
+      <c r="C94" s="31" t="inlineStr">
+        <is>
+          <t>Clutch Gene</t>
+        </is>
+      </c>
+      <c r="D94" s="6" t="inlineStr">
+        <is>
+          <t>SHOT x2 if attempting a shot with 1 or fewer cards in hand or Shot Clock 3 or less</t>
+        </is>
+      </c>
+      <c r="E94" s="7" t="n"/>
       <c r="F94" s="138" t="n"/>
-      <c r="G94" s="107" t="n"/>
+      <c r="G94" s="101" t="n"/>
       <c r="H94" s="102" t="n"/>
       <c r="I94" s="102" t="n"/>
       <c r="J94" s="102" t="n"/>
@@ -5125,23 +5127,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C95" s="31" t="inlineStr">
-        <is>
-          <t>Fox-Like First Step</t>
-        </is>
-      </c>
-      <c r="D95" s="6" t="inlineStr">
-        <is>
-          <t>All Move cards that reduce SHOT increase it by that amount instead.</t>
-        </is>
-      </c>
-      <c r="E95" s="6" t="inlineStr">
-        <is>
-          <t>Your Move cards are unaffected by opponents</t>
-        </is>
-      </c>
-      <c r="F95" s="139" t="n"/>
-      <c r="G95" s="101" t="n"/>
+      <c r="C95" s="32" t="inlineStr">
+        <is>
+          <t>Floor General</t>
+        </is>
+      </c>
+      <c r="D95" s="33" t="inlineStr">
+        <is>
+          <t>You choose all targets of all kinds — card declarations, non auto-pass targets, and the rest</t>
+        </is>
+      </c>
+      <c r="E95" s="34" t="n"/>
+      <c r="F95" s="138" t="n"/>
+      <c r="G95" s="107" t="n"/>
       <c r="H95" s="102" t="n"/>
       <c r="I95" s="102" t="n"/>
       <c r="J95" s="102" t="n"/>
@@ -5153,19 +5151,23 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C96" s="90" t="inlineStr">
-        <is>
-          <t>Freethrow Merchant</t>
-        </is>
-      </c>
-      <c r="D96" s="94" t="inlineStr">
-        <is>
-          <t>All Clamps on you grant 1 FT instead</t>
-        </is>
-      </c>
-      <c r="E96" s="34" t="n"/>
-      <c r="F96" s="138" t="n"/>
-      <c r="G96" s="125" t="n"/>
+      <c r="C96" s="31" t="inlineStr">
+        <is>
+          <t>Fox-Like First Step</t>
+        </is>
+      </c>
+      <c r="D96" s="6" t="inlineStr">
+        <is>
+          <t>All Move cards that reduce SHOT increase it by that amount instead.</t>
+        </is>
+      </c>
+      <c r="E96" s="6" t="inlineStr">
+        <is>
+          <t>Your Move cards are unaffected by opponents</t>
+        </is>
+      </c>
+      <c r="F96" s="139" t="n"/>
+      <c r="G96" s="101" t="n"/>
       <c r="H96" s="102" t="n"/>
       <c r="I96" s="102" t="n"/>
       <c r="J96" s="102" t="n"/>
@@ -5179,17 +5181,17 @@
       </c>
       <c r="C97" s="90" t="inlineStr">
         <is>
-          <t>Generational Whistle</t>
-        </is>
-      </c>
-      <c r="D97" s="91" t="inlineStr">
-        <is>
-          <t>Take 1 additional FT</t>
-        </is>
-      </c>
-      <c r="E97" s="7" t="n"/>
+          <t>Freethrow Merchant</t>
+        </is>
+      </c>
+      <c r="D97" s="94" t="inlineStr">
+        <is>
+          <t>All Clamps on you grant 1 FT instead</t>
+        </is>
+      </c>
+      <c r="E97" s="34" t="n"/>
       <c r="F97" s="138" t="n"/>
-      <c r="G97" s="101" t="n"/>
+      <c r="G97" s="125" t="n"/>
       <c r="H97" s="102" t="n"/>
       <c r="I97" s="102" t="n"/>
       <c r="J97" s="102" t="n"/>
@@ -5201,19 +5203,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C98" s="32" t="inlineStr">
-        <is>
-          <t>Gravity</t>
-        </is>
-      </c>
-      <c r="D98" s="33" t="inlineStr">
-        <is>
-          <t>All Clamps automatically apply to you. +1 AST whenever another player attempts a shot</t>
-        </is>
-      </c>
-      <c r="E98" s="34" t="n"/>
+      <c r="C98" s="90" t="inlineStr">
+        <is>
+          <t>Generational Whistle</t>
+        </is>
+      </c>
+      <c r="D98" s="91" t="inlineStr">
+        <is>
+          <t>Take 1 additional FT</t>
+        </is>
+      </c>
+      <c r="E98" s="7" t="n"/>
       <c r="F98" s="138" t="n"/>
-      <c r="G98" s="107" t="n"/>
+      <c r="G98" s="101" t="n"/>
       <c r="H98" s="102" t="n"/>
       <c r="I98" s="102" t="n"/>
       <c r="J98" s="102" t="n"/>
@@ -5225,19 +5227,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C99" s="31" t="inlineStr">
-        <is>
-          <t>Great Conditioning</t>
-        </is>
-      </c>
-      <c r="D99" s="6" t="inlineStr">
-        <is>
-          <t>Immediately discard all Injury Game Breaks you draw and draw a new card for each</t>
-        </is>
-      </c>
-      <c r="E99" s="7" t="n"/>
+      <c r="C99" s="32" t="inlineStr">
+        <is>
+          <t>Gravity</t>
+        </is>
+      </c>
+      <c r="D99" s="33" t="inlineStr">
+        <is>
+          <t>All Clamps automatically apply to you. +1 AST whenever another player attempts a shot</t>
+        </is>
+      </c>
+      <c r="E99" s="34" t="n"/>
       <c r="F99" s="138" t="n"/>
-      <c r="G99" s="101" t="n"/>
+      <c r="G99" s="107" t="n"/>
       <c r="H99" s="102" t="n"/>
       <c r="I99" s="102" t="n"/>
       <c r="J99" s="102" t="n"/>
@@ -5249,19 +5251,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C100" s="32" t="inlineStr">
-        <is>
-          <t>Hot Hand</t>
-        </is>
-      </c>
-      <c r="D100" s="33" t="inlineStr">
-        <is>
-          <t>SHOT +20% if you scored last round.</t>
-        </is>
-      </c>
-      <c r="E100" s="34" t="n"/>
+      <c r="C100" s="31" t="inlineStr">
+        <is>
+          <t>Great Conditioning</t>
+        </is>
+      </c>
+      <c r="D100" s="6" t="inlineStr">
+        <is>
+          <t>Immediately discard all Injury Game Breaks you draw and draw a new card for each</t>
+        </is>
+      </c>
+      <c r="E100" s="7" t="n"/>
       <c r="F100" s="138" t="n"/>
-      <c r="G100" s="107" t="n"/>
+      <c r="G100" s="101" t="n"/>
       <c r="H100" s="102" t="n"/>
       <c r="I100" s="102" t="n"/>
       <c r="J100" s="102" t="n"/>
@@ -5273,19 +5275,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C101" s="31" t="inlineStr">
-        <is>
-          <t>Like That</t>
-        </is>
-      </c>
-      <c r="D101" s="91" t="inlineStr">
-        <is>
-          <t>Your SHOT % cannot be reduced</t>
-        </is>
-      </c>
-      <c r="E101" s="7" t="n"/>
+      <c r="C101" s="32" t="inlineStr">
+        <is>
+          <t>Hot Hand</t>
+        </is>
+      </c>
+      <c r="D101" s="33" t="inlineStr">
+        <is>
+          <t>SHOT +20% if you scored last round.</t>
+        </is>
+      </c>
+      <c r="E101" s="34" t="n"/>
       <c r="F101" s="138" t="n"/>
-      <c r="G101" s="101" t="n"/>
+      <c r="G101" s="107" t="n"/>
       <c r="H101" s="102" t="n"/>
       <c r="I101" s="102" t="n"/>
       <c r="J101" s="102" t="n"/>
@@ -5297,23 +5299,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C102" s="32" t="inlineStr">
-        <is>
-          <t>No Bag</t>
-        </is>
-      </c>
-      <c r="D102" s="33" t="inlineStr">
-        <is>
-          <t>Cannot activate Move cards this round</t>
-        </is>
-      </c>
-      <c r="E102" s="34" t="n"/>
+      <c r="C102" s="31" t="inlineStr">
+        <is>
+          <t>Like That</t>
+        </is>
+      </c>
+      <c r="D102" s="91" t="inlineStr">
+        <is>
+          <t>Your SHOT % cannot be reduced</t>
+        </is>
+      </c>
+      <c r="E102" s="7" t="n"/>
       <c r="F102" s="138" t="n"/>
-      <c r="G102" s="113" t="inlineStr">
-        <is>
-          <t>Bad card to draw</t>
-        </is>
-      </c>
+      <c r="G102" s="101" t="n"/>
       <c r="H102" s="102" t="n"/>
       <c r="I102" s="102" t="n"/>
       <c r="J102" s="102" t="n"/>
@@ -5325,19 +5323,23 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C103" s="31" t="inlineStr">
-        <is>
-          <t>Point God</t>
-        </is>
-      </c>
-      <c r="D103" s="6" t="inlineStr">
-        <is>
-          <t>Draw 1 card following each of your passes</t>
-        </is>
-      </c>
-      <c r="E103" s="7" t="n"/>
+      <c r="C103" s="32" t="inlineStr">
+        <is>
+          <t>No Bag</t>
+        </is>
+      </c>
+      <c r="D103" s="33" t="inlineStr">
+        <is>
+          <t>Cannot activate Move cards this round</t>
+        </is>
+      </c>
+      <c r="E103" s="34" t="n"/>
       <c r="F103" s="138" t="n"/>
-      <c r="G103" s="101" t="n"/>
+      <c r="G103" s="113" t="inlineStr">
+        <is>
+          <t>Bad card to draw</t>
+        </is>
+      </c>
       <c r="H103" s="102" t="n"/>
       <c r="I103" s="102" t="n"/>
       <c r="J103" s="102" t="n"/>
@@ -5349,23 +5351,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C104" s="32" t="inlineStr">
-        <is>
-          <t>Shooting Slump</t>
-        </is>
-      </c>
-      <c r="D104" s="33" t="inlineStr">
-        <is>
-          <t>SHOT -20% this round</t>
-        </is>
-      </c>
-      <c r="E104" s="34" t="n"/>
+      <c r="C104" s="31" t="inlineStr">
+        <is>
+          <t>Point God</t>
+        </is>
+      </c>
+      <c r="D104" s="6" t="inlineStr">
+        <is>
+          <t>Draw 1 card following each of your passes</t>
+        </is>
+      </c>
+      <c r="E104" s="7" t="n"/>
       <c r="F104" s="138" t="n"/>
-      <c r="G104" s="113" t="inlineStr">
-        <is>
-          <t>Bad card to draw</t>
-        </is>
-      </c>
+      <c r="G104" s="101" t="n"/>
       <c r="H104" s="102" t="n"/>
       <c r="I104" s="102" t="n"/>
       <c r="J104" s="102" t="n"/>
@@ -5377,19 +5375,23 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C105" s="31" t="inlineStr">
-        <is>
-          <t>Shot Creator</t>
-        </is>
-      </c>
-      <c r="D105" s="6" t="inlineStr">
-        <is>
-          <t>Draw 1 additional card after every draw effect</t>
-        </is>
-      </c>
-      <c r="E105" s="7" t="n"/>
+      <c r="C105" s="32" t="inlineStr">
+        <is>
+          <t>Shooting Slump</t>
+        </is>
+      </c>
+      <c r="D105" s="33" t="inlineStr">
+        <is>
+          <t>SHOT -20% this round</t>
+        </is>
+      </c>
+      <c r="E105" s="34" t="n"/>
       <c r="F105" s="138" t="n"/>
-      <c r="G105" s="101" t="n"/>
+      <c r="G105" s="113" t="inlineStr">
+        <is>
+          <t>Bad card to draw</t>
+        </is>
+      </c>
       <c r="H105" s="102" t="n"/>
       <c r="I105" s="102" t="n"/>
       <c r="J105" s="102" t="n"/>
@@ -5401,19 +5403,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C106" s="32" t="inlineStr">
-        <is>
-          <t>Sixth Man</t>
-        </is>
-      </c>
-      <c r="D106" s="33" t="inlineStr">
-        <is>
-          <t>SHOT = 100% if taking 6th shot of the round</t>
-        </is>
-      </c>
-      <c r="E106" s="34" t="n"/>
+      <c r="C106" s="31" t="inlineStr">
+        <is>
+          <t>Shot Creator</t>
+        </is>
+      </c>
+      <c r="D106" s="6" t="inlineStr">
+        <is>
+          <t>Draw 1 additional card after every draw effect</t>
+        </is>
+      </c>
+      <c r="E106" s="7" t="n"/>
       <c r="F106" s="138" t="n"/>
-      <c r="G106" s="107" t="n"/>
+      <c r="G106" s="101" t="n"/>
       <c r="H106" s="102" t="n"/>
       <c r="I106" s="102" t="n"/>
       <c r="J106" s="102" t="n"/>
@@ -5425,19 +5427,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C107" s="31" t="inlineStr">
-        <is>
-          <t>Sniper</t>
-        </is>
-      </c>
-      <c r="D107" s="6" t="inlineStr">
-        <is>
-          <t>SHOT +10% on all Three-Point Line Shots</t>
-        </is>
-      </c>
-      <c r="E107" s="7" t="n"/>
+      <c r="C107" s="32" t="inlineStr">
+        <is>
+          <t>Sixth Man</t>
+        </is>
+      </c>
+      <c r="D107" s="33" t="inlineStr">
+        <is>
+          <t>SHOT = 100% if taking 6th shot of the round</t>
+        </is>
+      </c>
+      <c r="E107" s="34" t="n"/>
       <c r="F107" s="138" t="n"/>
-      <c r="G107" s="101" t="n"/>
+      <c r="G107" s="107" t="n"/>
       <c r="H107" s="102" t="n"/>
       <c r="I107" s="102" t="n"/>
       <c r="J107" s="102" t="n"/>
@@ -5449,19 +5451,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C108" s="32" t="inlineStr">
-        <is>
-          <t>Splash Cousin</t>
-        </is>
-      </c>
-      <c r="D108" s="33" t="inlineStr">
-        <is>
-          <t>All Three-Point Line Shots: SHOT = 100%</t>
-        </is>
-      </c>
-      <c r="E108" s="34" t="n"/>
+      <c r="C108" s="31" t="inlineStr">
+        <is>
+          <t>Sniper</t>
+        </is>
+      </c>
+      <c r="D108" s="6" t="inlineStr">
+        <is>
+          <t>SHOT +10% on all Three-Point Line Shots</t>
+        </is>
+      </c>
+      <c r="E108" s="7" t="n"/>
       <c r="F108" s="138" t="n"/>
-      <c r="G108" s="107" t="n"/>
+      <c r="G108" s="101" t="n"/>
       <c r="H108" s="102" t="n"/>
       <c r="I108" s="102" t="n"/>
       <c r="J108" s="102" t="n"/>
@@ -5473,19 +5475,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C109" s="31" t="inlineStr">
-        <is>
-          <t>Unguardable</t>
-        </is>
-      </c>
-      <c r="D109" s="91" t="inlineStr">
-        <is>
-          <t>All Clamps on you have no effect on SHOT %</t>
-        </is>
-      </c>
-      <c r="E109" s="7" t="n"/>
+      <c r="C109" s="32" t="inlineStr">
+        <is>
+          <t>Splash Cousin</t>
+        </is>
+      </c>
+      <c r="D109" s="33" t="inlineStr">
+        <is>
+          <t>All Three-Point Line Shots: SHOT = 100%</t>
+        </is>
+      </c>
+      <c r="E109" s="34" t="n"/>
       <c r="F109" s="138" t="n"/>
-      <c r="G109" s="101" t="n"/>
+      <c r="G109" s="107" t="n"/>
       <c r="H109" s="102" t="n"/>
       <c r="I109" s="102" t="n"/>
       <c r="J109" s="102" t="n"/>
@@ -5497,50 +5499,50 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C110" s="32" t="inlineStr">
-        <is>
-          <t>Lethal Shooter</t>
-        </is>
-      </c>
-      <c r="D110" s="33" t="inlineStr">
-        <is>
-          <t>SHOT = 100% on next shot attempt after rebounding your own miss.</t>
-        </is>
-      </c>
-      <c r="E110" s="34" t="n"/>
+      <c r="C110" s="31" t="inlineStr">
+        <is>
+          <t>Unguardable</t>
+        </is>
+      </c>
+      <c r="D110" s="91" t="inlineStr">
+        <is>
+          <t>All Clamps on you have no effect on SHOT %</t>
+        </is>
+      </c>
+      <c r="E110" s="7" t="n"/>
       <c r="F110" s="138" t="n"/>
-      <c r="G110" s="113" t="inlineStr">
-        <is>
-          <t>Special text: “I understand it now”</t>
-        </is>
-      </c>
+      <c r="G110" s="101" t="n"/>
       <c r="H110" s="102" t="n"/>
       <c r="I110" s="102" t="n"/>
       <c r="J110" s="102" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="61" t="n"/>
-      <c r="B111" s="62" t="inlineStr">
+      <c r="A111" s="29" t="n"/>
+      <c r="B111" s="30" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C111" s="66" t="inlineStr">
-        <is>
-          <t>Ball Pounder</t>
-        </is>
-      </c>
-      <c r="D111" s="95" t="inlineStr">
-        <is>
-          <t>All Dribble cards you play draw an additional card but lower SHOT by an additional 10%</t>
-        </is>
-      </c>
-      <c r="E111" s="68" t="n"/>
-      <c r="F111" s="140" t="n"/>
-      <c r="G111" s="126" t="n"/>
-      <c r="H111" s="117" t="n"/>
-      <c r="I111" s="117" t="n"/>
-      <c r="J111" s="117" t="n"/>
+      <c r="C111" s="32" t="inlineStr">
+        <is>
+          <t>Lethal Shooter</t>
+        </is>
+      </c>
+      <c r="D111" s="33" t="inlineStr">
+        <is>
+          <t>SHOT = 100% on next shot attempt after rebounding your own miss.</t>
+        </is>
+      </c>
+      <c r="E111" s="34" t="n"/>
+      <c r="F111" s="138" t="n"/>
+      <c r="G111" s="113" t="inlineStr">
+        <is>
+          <t>Special text: “I understand it now”</t>
+        </is>
+      </c>
+      <c r="H111" s="102" t="n"/>
+      <c r="I111" s="102" t="n"/>
+      <c r="J111" s="102" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="61" t="n"/>
@@ -5551,12 +5553,12 @@
       </c>
       <c r="C112" s="66" t="inlineStr">
         <is>
-          <t>Unselfish</t>
+          <t>Ball Pounder</t>
         </is>
       </c>
       <c r="D112" s="95" t="inlineStr">
         <is>
-          <t>Draw 1 card whenever you pass the ball at 50% SHOT or higher</t>
+          <t>All Dribble cards you play draw an additional card but lower SHOT by an additional 10%</t>
         </is>
       </c>
       <c r="E112" s="68" t="n"/>
@@ -5575,12 +5577,12 @@
       </c>
       <c r="C113" s="66" t="inlineStr">
         <is>
-          <t>Dirty Player</t>
+          <t>Unselfish</t>
         </is>
       </c>
       <c r="D113" s="95" t="inlineStr">
         <is>
-          <t>When sending Clamps, the clamped player discards 1 if they have any Injuries</t>
+          <t>Draw 1 card and increase next SHOT +5% whenever you positively affect another player</t>
         </is>
       </c>
       <c r="E113" s="68" t="n"/>
@@ -5599,21 +5601,20 @@
       </c>
       <c r="C114" s="66" t="inlineStr">
         <is>
-          <t>Villainous Reputation</t>
+          <t>Dirty Player</t>
         </is>
       </c>
       <c r="D114" s="95" t="inlineStr">
         <is>
-          <t>Discard 1 whenever any Whistle triggers</t>
+          <t>When sending Clamps, the clamped player discards 1 if they have any Injuries</t>
         </is>
       </c>
       <c r="E114" s="68" t="n"/>
       <c r="F114" s="140" t="n"/>
-      <c r="G114" s="126" t="inlineStr">
-        <is>
-          <t>Discarded during play, it attaches to a random player — possibly you again</t>
-        </is>
-      </c>
+      <c r="G114" s="126" t="n"/>
+      <c r="H114" s="117" t="n"/>
+      <c r="I114" s="117" t="n"/>
+      <c r="J114" s="117" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="61" t="n"/>
@@ -5624,19 +5625,19 @@
       </c>
       <c r="C115" s="66" t="inlineStr">
         <is>
-          <t>Free Agent</t>
+          <t>Villainous Reputation</t>
         </is>
       </c>
       <c r="D115" s="95" t="inlineStr">
         <is>
-          <t>Discard your hand. Play a card at random from a player of your choosing (they keep it)</t>
+          <t>Discard 1 whenever any Whistle triggers</t>
         </is>
       </c>
       <c r="E115" s="68" t="n"/>
       <c r="F115" s="140" t="n"/>
       <c r="G115" s="126" t="inlineStr">
         <is>
-          <t>The discard waits for the draw chain to finish. Target is shuffled first and is affected by Floor General. Your own draws are kept. All-0 rebounds are yours; otherwise you cannot bid</t>
+          <t>Discarded during play, it attaches to a random player — possibly you again</t>
         </is>
       </c>
     </row>
@@ -5649,23 +5650,48 @@
       </c>
       <c r="C116" s="66" t="inlineStr">
         <is>
-          <t>Franchise Player</t>
+          <t>Free Agent</t>
         </is>
       </c>
       <c r="D116" s="95" t="inlineStr">
         <is>
-          <t>When passing, choose 1 of the new player's Intangibles or a card in their hand for them to discard</t>
+          <t>Discard your hand. Play a card at random from a player of your choosing (they keep it)</t>
         </is>
       </c>
       <c r="E116" s="68" t="n"/>
       <c r="F116" s="140" t="n"/>
-      <c r="G116" s="126" t="n"/>
-      <c r="H116" s="117" t="n"/>
-      <c r="I116" s="117" t="n"/>
-      <c r="J116" s="117" t="n"/>
+      <c r="G116" s="126" t="inlineStr">
+        <is>
+          <t>The discard waits for the draw chain to finish. Target is shuffled first and is affected by Floor General. Your own draws are kept. All-0 rebounds are yours; otherwise you cannot bid</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="61" t="n"/>
+      <c r="B117" s="62" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C117" s="66" t="inlineStr">
+        <is>
+          <t>Franchise Player</t>
+        </is>
+      </c>
+      <c r="D117" s="95" t="inlineStr">
+        <is>
+          <t>When passing, choose 1 of the new player's Intangibles or a card in their hand for them to discard</t>
+        </is>
+      </c>
+      <c r="E117" s="68" t="n"/>
+      <c r="F117" s="140" t="n"/>
+      <c r="G117" s="126" t="n"/>
+      <c r="H117" s="117" t="n"/>
+      <c r="I117" s="117" t="n"/>
+      <c r="J117" s="117" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="103">
+  <mergeCells count="104">
     <mergeCell ref="G55:J55"/>
     <mergeCell ref="G4:J4"/>
     <mergeCell ref="G109:J109"/>
@@ -5690,12 +5716,12 @@
     <mergeCell ref="G68:J68"/>
     <mergeCell ref="G108:J108"/>
     <mergeCell ref="G58:J58"/>
+    <mergeCell ref="G114:J114"/>
     <mergeCell ref="G110:J110"/>
-    <mergeCell ref="G113:J113"/>
     <mergeCell ref="G20:J20"/>
-    <mergeCell ref="G91:J91"/>
     <mergeCell ref="G29:J29"/>
     <mergeCell ref="G85:J85"/>
+    <mergeCell ref="G91:J91"/>
     <mergeCell ref="G100:J100"/>
     <mergeCell ref="G94:J94"/>
     <mergeCell ref="G75:J75"/>
@@ -5732,10 +5758,11 @@
     <mergeCell ref="G9:J9"/>
     <mergeCell ref="G59:J59"/>
     <mergeCell ref="G11:J11"/>
+    <mergeCell ref="G117:J117"/>
     <mergeCell ref="G39:J39"/>
     <mergeCell ref="G101:J101"/>
-    <mergeCell ref="G116:J116"/>
     <mergeCell ref="G103:J103"/>
+    <mergeCell ref="G113:J113"/>
     <mergeCell ref="G37:J37"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G13:J13"/>
@@ -5758,14 +5785,14 @@
     <mergeCell ref="G52:J52"/>
     <mergeCell ref="G27:J27"/>
     <mergeCell ref="G98:J98"/>
+    <mergeCell ref="G107:J107"/>
     <mergeCell ref="G36:J36"/>
     <mergeCell ref="G42:J42"/>
-    <mergeCell ref="G107:J107"/>
     <mergeCell ref="G17:J17"/>
     <mergeCell ref="G19:J19"/>
     <mergeCell ref="G28:J28"/>
+    <mergeCell ref="G6:J6"/>
     <mergeCell ref="G93:J93"/>
-    <mergeCell ref="G6:J6"/>
     <mergeCell ref="G69:J69"/>
     <mergeCell ref="G92:J92"/>
     <mergeCell ref="G30:J30"/>

</xml_diff>

<commit_message>
The board after a basket, and Wide-Open Three
Every make puts the score up on the scorer's own card — his colour, his points
— with an assist badge hanging off its south-east corner for each man credited.
A radial star, his face and his name in his own colour, drawn as a badge rather
than a line of text because Wide-Open Three can owe three of them at once.

Wide-Open Three names as many of the others as it likes, one tap each on the
floor, and closes with a button that says what the naming came to. Naming
nobody rolls off the current SHOT and is still a three.

The two halves of the card are the same list read twice: once for what the shot
is worth, and once if it drops.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -2549,7 +2549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J117"/>
+  <dimension ref="A1:J118"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="22.25" customHeight="1"/>
   <cols>
     <col width="15.5" customWidth="1" style="8" min="1" max="1"/>
@@ -2626,35 +2626,35 @@
         </is>
       </c>
       <c r="B2" s="12">
-        <f>COUNTIF($B$5:$B$117,"Pass")</f>
+        <f>COUNTIF($B$5:$B$118,"Pass")</f>
         <v/>
       </c>
       <c r="C2" s="13">
-        <f>COUNTIF($B$5:$B$117,"Move")+COUNTIF($B$5:$B$117,"Special Move")</f>
+        <f>COUNTIF($B$5:$B$118,"Move")+COUNTIF($B$5:$B$118,"Special Move")</f>
         <v/>
       </c>
       <c r="D2" s="14">
-        <f>COUNTIF($B$5:$B$117,"Clamp")</f>
+        <f>COUNTIF($B$5:$B$118,"Clamp")</f>
         <v/>
       </c>
       <c r="E2" s="15">
-        <f>COUNTIF($B$5:$B$117,"Whistle")</f>
+        <f>COUNTIF($B$5:$B$118,"Whistle")</f>
         <v/>
       </c>
       <c r="F2" s="16">
-        <f>COUNTIF($B$5:$B$117,"Game Break")</f>
+        <f>COUNTIF($B$5:$B$118,"Game Break")</f>
         <v/>
       </c>
       <c r="G2" s="18">
-        <f>COUNTIF($B$5:$B$117,"Injury GB")</f>
+        <f>COUNTIF($B$5:$B$118,"Injury GB")</f>
         <v/>
       </c>
       <c r="H2" s="19">
-        <f>COUNTIF($B$5:$B$117,"Devastating Injury GB")</f>
+        <f>COUNTIF($B$5:$B$118,"Devastating Injury GB")</f>
         <v/>
       </c>
       <c r="I2" s="17">
-        <f>COUNTIF($B$5:$B$117,"Intangible")</f>
+        <f>COUNTIF($B$5:$B$118,"Intangible")</f>
         <v/>
       </c>
       <c r="J2" s="19" t="n"/>
@@ -2703,7 +2703,7 @@
         </is>
       </c>
       <c r="B5" s="22">
-        <f>COUNTIF($B$5:$B$117,"Pass")</f>
+        <f>COUNTIF($B$5:$B$118,"Pass")</f>
         <v/>
       </c>
       <c r="C5" s="23" t="n"/>
@@ -2960,7 +2960,7 @@
         </is>
       </c>
       <c r="B15" s="40">
-        <f>COUNTIF($B$5:$B$117,"Move")+COUNTIF($B$5:$B$117,"Special Move")</f>
+        <f>COUNTIF($B$5:$B$118,"Move")+COUNTIF($B$5:$B$118,"Special Move")</f>
         <v/>
       </c>
       <c r="C15" s="41" t="n"/>
@@ -3334,7 +3334,7 @@
         </is>
       </c>
       <c r="B28" s="43">
-        <f>COUNTIF($B$5:$B$117,"Special Move")</f>
+        <f>COUNTIF($B$5:$B$118,"Special Move")</f>
         <v/>
       </c>
       <c r="C28" s="44" t="n"/>
@@ -3713,53 +3713,57 @@
       <c r="J40" s="104" t="n"/>
     </row>
     <row r="41" ht="20" customHeight="1" s="132">
-      <c r="A41" s="58" t="inlineStr">
+      <c r="A41" s="61" t="n"/>
+      <c r="B41" s="62" t="inlineStr">
+        <is>
+          <t>Special Move</t>
+        </is>
+      </c>
+      <c r="C41" s="66" t="inlineStr">
+        <is>
+          <t>Wide-Open Three</t>
+        </is>
+      </c>
+      <c r="D41" s="67" t="inlineStr">
+        <is>
+          <t>Select any number of other players. SHOT +10% for each</t>
+        </is>
+      </c>
+      <c r="E41" s="68" t="inlineStr">
+        <is>
+          <t>Shoot the ball. +1 Point on make. Selected players receive +1 AST on a make</t>
+        </is>
+      </c>
+      <c r="F41" s="85" t="n">
+        <v>2</v>
+      </c>
+      <c r="G41" s="122" t="inlineStr">
+        <is>
+          <t>Selecting none rolls off current SHOT and is still a three</t>
+        </is>
+      </c>
+      <c r="H41" s="104" t="n"/>
+      <c r="I41" s="104" t="n"/>
+      <c r="J41" s="104" t="n"/>
+    </row>
+    <row r="42" ht="28" customHeight="1" s="132">
+      <c r="A42" s="58" t="inlineStr">
         <is>
           <t>Clamp</t>
         </is>
       </c>
-      <c r="B41" s="59">
-        <f>COUNTIF($B$5:$B$117,"Clamp")</f>
+      <c r="B42" s="59">
+        <f>COUNTIF($B$5:$B$118,"Clamp")</f>
         <v/>
       </c>
-      <c r="C41" s="60" t="n"/>
-      <c r="D41" s="60" t="n"/>
-      <c r="E41" s="60" t="n"/>
-      <c r="F41" s="86" t="n"/>
-      <c r="G41" s="109" t="n"/>
-      <c r="H41" s="110" t="n"/>
-      <c r="I41" s="110" t="n"/>
-      <c r="J41" s="110" t="n"/>
-    </row>
-    <row r="42" ht="28" customHeight="1" s="132">
-      <c r="A42" s="29" t="n"/>
-      <c r="B42" s="30" t="inlineStr">
-        <is>
-          <t>Clamp</t>
-        </is>
-      </c>
-      <c r="C42" s="31" t="inlineStr">
-        <is>
-          <t>Contest</t>
-        </is>
-      </c>
-      <c r="D42" s="6" t="inlineStr">
-        <is>
-          <t>Next player SHOT -25% if they shoot</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="n"/>
-      <c r="F42" s="76" t="n">
-        <v>10</v>
-      </c>
-      <c r="G42" s="130" t="inlineStr">
-        <is>
-          <t>1 def</t>
-        </is>
-      </c>
-      <c r="H42" s="102" t="n"/>
-      <c r="I42" s="102" t="n"/>
-      <c r="J42" s="102" t="n"/>
+      <c r="C42" s="60" t="n"/>
+      <c r="D42" s="60" t="n"/>
+      <c r="E42" s="60" t="n"/>
+      <c r="F42" s="86" t="n"/>
+      <c r="G42" s="109" t="n"/>
+      <c r="H42" s="110" t="n"/>
+      <c r="I42" s="110" t="n"/>
+      <c r="J42" s="110" t="n"/>
     </row>
     <row r="43" ht="28" customHeight="1" s="132">
       <c r="A43" s="29" t="n"/>
@@ -3768,23 +3772,23 @@
           <t>Clamp</t>
         </is>
       </c>
-      <c r="C43" s="32" t="inlineStr">
-        <is>
-          <t>Double-Team</t>
-        </is>
-      </c>
-      <c r="D43" s="33" t="inlineStr">
-        <is>
-          <t>Next Player cannot play 2 random cards from hand.</t>
-        </is>
-      </c>
-      <c r="E43" s="34" t="n"/>
-      <c r="F43" s="75" t="n">
-        <v>4</v>
-      </c>
-      <c r="G43" s="125" t="inlineStr">
-        <is>
-          <t>2 def</t>
+      <c r="C43" s="31" t="inlineStr">
+        <is>
+          <t>Contest</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>Next player SHOT -25% if they shoot</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="n"/>
+      <c r="F43" s="76" t="n">
+        <v>10</v>
+      </c>
+      <c r="G43" s="130" t="inlineStr">
+        <is>
+          <t>1 def</t>
         </is>
       </c>
       <c r="H43" s="102" t="n"/>
@@ -3798,23 +3802,23 @@
           <t>Clamp</t>
         </is>
       </c>
-      <c r="C44" s="31" t="inlineStr">
-        <is>
-          <t>Full-Court Press</t>
-        </is>
-      </c>
-      <c r="D44" s="6" t="inlineStr">
-        <is>
-          <t>Next player discards 2 cards at the start of their turn</t>
-        </is>
-      </c>
-      <c r="E44" s="7" t="n"/>
-      <c r="F44" s="76" t="n">
-        <v>3</v>
-      </c>
-      <c r="G44" s="130" t="inlineStr">
-        <is>
-          <t>1 def</t>
+      <c r="C44" s="32" t="inlineStr">
+        <is>
+          <t>Double-Team</t>
+        </is>
+      </c>
+      <c r="D44" s="33" t="inlineStr">
+        <is>
+          <t>Next Player cannot play 2 random cards from hand.</t>
+        </is>
+      </c>
+      <c r="E44" s="34" t="n"/>
+      <c r="F44" s="75" t="n">
+        <v>4</v>
+      </c>
+      <c r="G44" s="125" t="inlineStr">
+        <is>
+          <t>2 def</t>
         </is>
       </c>
       <c r="H44" s="102" t="n"/>
@@ -3828,23 +3832,23 @@
           <t>Clamp</t>
         </is>
       </c>
-      <c r="C45" s="32" t="inlineStr">
-        <is>
-          <t>Trap</t>
-        </is>
-      </c>
-      <c r="D45" s="94" t="inlineStr">
-        <is>
-          <t>Next player can only play Pass cards during their turn</t>
-        </is>
-      </c>
-      <c r="E45" s="34" t="n"/>
-      <c r="F45" s="75" t="n">
-        <v>5</v>
-      </c>
-      <c r="G45" s="125" t="inlineStr">
-        <is>
-          <t>They can still shoot as another option; 3 def</t>
+      <c r="C45" s="31" t="inlineStr">
+        <is>
+          <t>Full-Court Press</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>Next player discards 2 cards at the start of their turn</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="n"/>
+      <c r="F45" s="76" t="n">
+        <v>3</v>
+      </c>
+      <c r="G45" s="130" t="inlineStr">
+        <is>
+          <t>1 def</t>
         </is>
       </c>
       <c r="H45" s="102" t="n"/>
@@ -3852,106 +3856,112 @@
       <c r="J45" s="102" t="n"/>
     </row>
     <row r="46" ht="29" customHeight="1" s="132" thickBot="1">
-      <c r="A46" s="61" t="n"/>
-      <c r="B46" s="62" t="inlineStr">
+      <c r="A46" s="29" t="n"/>
+      <c r="B46" s="30" t="inlineStr">
         <is>
           <t>Clamp</t>
         </is>
       </c>
-      <c r="C46" s="66" t="inlineStr">
+      <c r="C46" s="32" t="inlineStr">
+        <is>
+          <t>Trap</t>
+        </is>
+      </c>
+      <c r="D46" s="94" t="inlineStr">
+        <is>
+          <t>Next player can only play Pass cards during their turn</t>
+        </is>
+      </c>
+      <c r="E46" s="34" t="n"/>
+      <c r="F46" s="75" t="n">
+        <v>5</v>
+      </c>
+      <c r="G46" s="125" t="inlineStr">
+        <is>
+          <t>They can still shoot as another option; 3 def</t>
+        </is>
+      </c>
+      <c r="H46" s="102" t="n"/>
+      <c r="I46" s="102" t="n"/>
+      <c r="J46" s="102" t="n"/>
+    </row>
+    <row r="47" ht="20" customHeight="1" s="132">
+      <c r="A47" s="61" t="n"/>
+      <c r="B47" s="62" t="inlineStr">
+        <is>
+          <t>Clamp</t>
+        </is>
+      </c>
+      <c r="C47" s="66" t="inlineStr">
         <is>
           <t>Triple-Team</t>
         </is>
       </c>
-      <c r="D46" s="67" t="inlineStr">
+      <c r="D47" s="67" t="inlineStr">
         <is>
           <t>Next player cannot play 3 random cards from hand.</t>
         </is>
       </c>
-      <c r="E46" s="68" t="n"/>
-      <c r="F46" s="85" t="n">
+      <c r="E47" s="68" t="n"/>
+      <c r="F47" s="85" t="n">
         <v>2</v>
       </c>
-      <c r="G46" s="135" t="inlineStr">
+      <c r="G47" s="135" t="inlineStr">
         <is>
           <t>3 def</t>
         </is>
       </c>
-      <c r="H46" s="117" t="n"/>
-      <c r="I46" s="117" t="n"/>
-      <c r="J46" s="117" t="n"/>
-    </row>
-    <row r="47" ht="20" customHeight="1" s="132">
-      <c r="A47" s="58" t="inlineStr">
+      <c r="H47" s="117" t="n"/>
+      <c r="I47" s="117" t="n"/>
+      <c r="J47" s="117" t="n"/>
+    </row>
+    <row r="48" ht="56" customHeight="1" s="132">
+      <c r="A48" s="58" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="B47" s="59">
-        <f>COUNTIF($B$5:$B$117,"Whistle")</f>
+      <c r="B48" s="59">
+        <f>COUNTIF($B$5:$B$118,"Whistle")</f>
         <v/>
       </c>
-      <c r="C47" s="60" t="n"/>
-      <c r="D47" s="60" t="n"/>
-      <c r="E47" s="60" t="n"/>
-      <c r="F47" s="86" t="n"/>
-      <c r="G47" s="109" t="n"/>
-      <c r="H47" s="110" t="n"/>
-      <c r="I47" s="110" t="n"/>
-      <c r="J47" s="110" t="n"/>
-    </row>
-    <row r="48" ht="56" customHeight="1" s="132">
-      <c r="A48" s="29" t="inlineStr">
+      <c r="C48" s="60" t="n"/>
+      <c r="D48" s="60" t="n"/>
+      <c r="E48" s="60" t="n"/>
+      <c r="F48" s="86" t="n"/>
+      <c r="G48" s="109" t="n"/>
+      <c r="H48" s="110" t="n"/>
+      <c r="I48" s="110" t="n"/>
+      <c r="J48" s="110" t="n"/>
+    </row>
+    <row r="49" ht="47" customHeight="1" s="132">
+      <c r="A49" s="29" t="inlineStr">
         <is>
           <t>All whistles are limited to 1</t>
         </is>
       </c>
-      <c r="B48" s="30" t="inlineStr">
+      <c r="B49" s="30" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C48" s="31" t="inlineStr">
+      <c r="C49" s="31" t="inlineStr">
         <is>
           <t>Back Court Violation</t>
         </is>
       </c>
-      <c r="D48" s="6" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>Pass Card Played: Cancel that card. That player TOV +1. Move ball to player of choice</t>
         </is>
       </c>
-      <c r="E48" s="7" t="n"/>
-      <c r="F48" s="138" t="n"/>
-      <c r="G48" s="101" t="inlineStr">
+      <c r="E49" s="7" t="n"/>
+      <c r="F49" s="138" t="n"/>
+      <c r="G49" s="101" t="inlineStr">
         <is>
           <t>The player who played this whistle chooses, excluding the player who played the pass but including themselves.</t>
         </is>
       </c>
-      <c r="H48" s="102" t="n"/>
-      <c r="I48" s="102" t="n"/>
-      <c r="J48" s="102" t="n"/>
-    </row>
-    <row r="49" ht="47" customHeight="1" s="132">
-      <c r="A49" s="29" t="n"/>
-      <c r="B49" s="30" t="inlineStr">
-        <is>
-          <t>Whistle</t>
-        </is>
-      </c>
-      <c r="C49" s="90" t="inlineStr">
-        <is>
-          <t>Blocking Foul</t>
-        </is>
-      </c>
-      <c r="D49" s="93" t="inlineStr">
-        <is>
-          <t>Clamp Card Played: Cancel card. Clamped player +1 FT</t>
-        </is>
-      </c>
-      <c r="E49" s="34" t="n"/>
-      <c r="F49" s="138" t="n"/>
-      <c r="G49" s="107" t="n"/>
       <c r="H49" s="102" t="n"/>
       <c r="I49" s="102" t="n"/>
       <c r="J49" s="102" t="n"/>
@@ -3963,19 +3973,19 @@
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C50" s="31" t="inlineStr">
-        <is>
-          <t>Charge</t>
-        </is>
-      </c>
-      <c r="D50" s="92" t="inlineStr">
-        <is>
-          <t>Shot Attempt: Cancel. Shooter Inbounds</t>
-        </is>
-      </c>
-      <c r="E50" s="7" t="n"/>
+      <c r="C50" s="90" t="inlineStr">
+        <is>
+          <t>Blocking Foul</t>
+        </is>
+      </c>
+      <c r="D50" s="93" t="inlineStr">
+        <is>
+          <t>Clamp Card Played: Cancel card. Clamped player +1 FT</t>
+        </is>
+      </c>
+      <c r="E50" s="34" t="n"/>
       <c r="F50" s="138" t="n"/>
-      <c r="G50" s="101" t="n"/>
+      <c r="G50" s="107" t="n"/>
       <c r="H50" s="102" t="n"/>
       <c r="I50" s="102" t="n"/>
       <c r="J50" s="102" t="n"/>
@@ -3987,19 +3997,19 @@
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C51" s="32" t="inlineStr">
-        <is>
-          <t>Cleared to Play</t>
-        </is>
-      </c>
-      <c r="D51" s="33" t="inlineStr">
-        <is>
-          <t>Injury Card Played: Cancel card.</t>
-        </is>
-      </c>
-      <c r="E51" s="34" t="n"/>
+      <c r="C51" s="31" t="inlineStr">
+        <is>
+          <t>Charge</t>
+        </is>
+      </c>
+      <c r="D51" s="92" t="inlineStr">
+        <is>
+          <t>Shot Attempt: Cancel. Shooter Inbounds</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="n"/>
       <c r="F51" s="138" t="n"/>
-      <c r="G51" s="107" t="n"/>
+      <c r="G51" s="101" t="n"/>
       <c r="H51" s="102" t="n"/>
       <c r="I51" s="102" t="n"/>
       <c r="J51" s="102" t="n"/>
@@ -4011,23 +4021,19 @@
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C52" s="31" t="inlineStr">
-        <is>
-          <t>Coach’s Challenge</t>
-        </is>
-      </c>
-      <c r="D52" s="6" t="inlineStr">
-        <is>
-          <t>Any Whistle Card Played: Cancel card.</t>
-        </is>
-      </c>
-      <c r="E52" s="7" t="inlineStr">
-        <is>
-          <t>Pull a Timeout from the discards, if one is there, and take it</t>
-        </is>
-      </c>
+      <c r="C52" s="32" t="inlineStr">
+        <is>
+          <t>Cleared to Play</t>
+        </is>
+      </c>
+      <c r="D52" s="33" t="inlineStr">
+        <is>
+          <t>Injury Card Played: Cancel card.</t>
+        </is>
+      </c>
+      <c r="E52" s="34" t="n"/>
       <c r="F52" s="138" t="n"/>
-      <c r="G52" s="101" t="n"/>
+      <c r="G52" s="107" t="n"/>
       <c r="H52" s="102" t="n"/>
       <c r="I52" s="102" t="n"/>
       <c r="J52" s="102" t="n"/>
@@ -4039,27 +4045,23 @@
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C53" s="90" t="inlineStr">
-        <is>
-          <t>Delay-of-Game Warning</t>
-        </is>
-      </c>
-      <c r="D53" s="94" t="inlineStr">
-        <is>
-          <t>Lower Shot Clock with a card: Cancel that card's effects</t>
-        </is>
-      </c>
-      <c r="E53" s="33" t="inlineStr">
-        <is>
-          <t>If 2nd time activated this round: Whistle player takes 1 FT in addition</t>
-        </is>
-      </c>
-      <c r="F53" s="139" t="n"/>
-      <c r="G53" s="113" t="inlineStr">
-        <is>
-          <t>The Shot Clock reduction still applies. Game Breaks do not count — those are game events, not cards the player activates.</t>
-        </is>
-      </c>
+      <c r="C53" s="31" t="inlineStr">
+        <is>
+          <t>Coach’s Challenge</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>Any Whistle Card Played: Cancel card.</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>Pull a Timeout from the discards, if one is there, and take it</t>
+        </is>
+      </c>
+      <c r="F53" s="138" t="n"/>
+      <c r="G53" s="101" t="n"/>
       <c r="H53" s="102" t="n"/>
       <c r="I53" s="102" t="n"/>
       <c r="J53" s="102" t="n"/>
@@ -4071,21 +4073,25 @@
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C54" s="31" t="inlineStr">
-        <is>
-          <t>Double Dribble</t>
-        </is>
-      </c>
-      <c r="D54" s="6" t="inlineStr">
-        <is>
-          <t>Dribble Move Card Played (Dribble, Rhythm Dribble, etc.): Cancel card. Discard 1 card. TOV +1</t>
-        </is>
-      </c>
-      <c r="E54" s="7" t="n"/>
-      <c r="F54" s="138" t="n"/>
-      <c r="G54" s="101" t="inlineStr">
-        <is>
-          <t>The dribbling player inbounds. The round is NOT incremented.</t>
+      <c r="C54" s="90" t="inlineStr">
+        <is>
+          <t>Delay-of-Game Warning</t>
+        </is>
+      </c>
+      <c r="D54" s="94" t="inlineStr">
+        <is>
+          <t>Lower Shot Clock with a card: Cancel that card's effects</t>
+        </is>
+      </c>
+      <c r="E54" s="33" t="inlineStr">
+        <is>
+          <t>If 2nd time activated this round: Whistle player takes 1 FT in addition</t>
+        </is>
+      </c>
+      <c r="F54" s="139" t="n"/>
+      <c r="G54" s="113" t="inlineStr">
+        <is>
+          <t>The Shot Clock reduction still applies. Game Breaks do not count — those are game events, not cards the player activates.</t>
         </is>
       </c>
       <c r="H54" s="102" t="n"/>
@@ -4099,19 +4105,23 @@
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C55" s="90" t="inlineStr">
-        <is>
-          <t>Flagrant Foul</t>
-        </is>
-      </c>
-      <c r="D55" s="94" t="inlineStr">
-        <is>
-          <t>Clamp Card Played: Cancel card. Clamper discard 1. Clamped player +1 FT then gets ball</t>
-        </is>
-      </c>
-      <c r="E55" s="34" t="n"/>
+      <c r="C55" s="31" t="inlineStr">
+        <is>
+          <t>Double Dribble</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>Dribble Move Card Played (Dribble, Rhythm Dribble, etc.): Cancel card. Discard 1 card. TOV +1</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="n"/>
       <c r="F55" s="138" t="n"/>
-      <c r="G55" s="107" t="n"/>
+      <c r="G55" s="101" t="inlineStr">
+        <is>
+          <t>The dribbling player inbounds. The round is NOT incremented.</t>
+        </is>
+      </c>
       <c r="H55" s="102" t="n"/>
       <c r="I55" s="102" t="n"/>
       <c r="J55" s="102" t="n"/>
@@ -4125,17 +4135,17 @@
       </c>
       <c r="C56" s="90" t="inlineStr">
         <is>
-          <t>Flagrant Foul II</t>
-        </is>
-      </c>
-      <c r="D56" s="91" t="inlineStr">
-        <is>
-          <t>Clamp Card Played: Cancel card. Clamper discards Bag. Clamped player +1 FT then gets ball</t>
-        </is>
-      </c>
-      <c r="E56" s="7" t="n"/>
+          <t>Flagrant Foul</t>
+        </is>
+      </c>
+      <c r="D56" s="94" t="inlineStr">
+        <is>
+          <t>Clamp Card Played: Cancel card. Clamper discard 1. Clamped player +1 FT then gets ball</t>
+        </is>
+      </c>
+      <c r="E56" s="34" t="n"/>
       <c r="F56" s="138" t="n"/>
-      <c r="G56" s="101" t="n"/>
+      <c r="G56" s="107" t="n"/>
       <c r="H56" s="102" t="n"/>
       <c r="I56" s="102" t="n"/>
       <c r="J56" s="102" t="n"/>
@@ -4147,19 +4157,19 @@
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C57" s="32" t="inlineStr">
-        <is>
-          <t>Goaltending</t>
-        </is>
-      </c>
-      <c r="D57" s="33" t="inlineStr">
-        <is>
-          <t>Clamp Card Played: Cancel card. Clamped player +2 points. End round.</t>
-        </is>
-      </c>
-      <c r="E57" s="34" t="n"/>
+      <c r="C57" s="90" t="inlineStr">
+        <is>
+          <t>Flagrant Foul II</t>
+        </is>
+      </c>
+      <c r="D57" s="91" t="inlineStr">
+        <is>
+          <t>Clamp Card Played: Cancel card. Clamper discards Bag. Clamped player +1 FT then gets ball</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="n"/>
       <c r="F57" s="138" t="n"/>
-      <c r="G57" s="107" t="n"/>
+      <c r="G57" s="101" t="n"/>
       <c r="H57" s="102" t="n"/>
       <c r="I57" s="102" t="n"/>
       <c r="J57" s="102" t="n"/>
@@ -4171,19 +4181,19 @@
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C58" s="31" t="inlineStr">
-        <is>
-          <t>Inadvertent Whistle</t>
-        </is>
-      </c>
-      <c r="D58" s="91" t="inlineStr">
-        <is>
-          <t>Any other whistle triggers: Cancel that card. Turn player draws 1 card.</t>
-        </is>
-      </c>
-      <c r="E58" s="7" t="n"/>
+      <c r="C58" s="32" t="inlineStr">
+        <is>
+          <t>Goaltending</t>
+        </is>
+      </c>
+      <c r="D58" s="33" t="inlineStr">
+        <is>
+          <t>Clamp Card Played: Cancel card. Clamped player +2 points. End round.</t>
+        </is>
+      </c>
+      <c r="E58" s="34" t="n"/>
       <c r="F58" s="138" t="n"/>
-      <c r="G58" s="101" t="n"/>
+      <c r="G58" s="107" t="n"/>
       <c r="H58" s="102" t="n"/>
       <c r="I58" s="102" t="n"/>
       <c r="J58" s="102" t="n"/>
@@ -4195,19 +4205,19 @@
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C59" s="32" t="inlineStr">
-        <is>
-          <t>Official Review</t>
-        </is>
-      </c>
-      <c r="D59" s="94" t="inlineStr">
-        <is>
-          <t>Intangible Played: Discard all Intangibles from player.</t>
-        </is>
-      </c>
-      <c r="E59" s="34" t="n"/>
+      <c r="C59" s="31" t="inlineStr">
+        <is>
+          <t>Inadvertent Whistle</t>
+        </is>
+      </c>
+      <c r="D59" s="91" t="inlineStr">
+        <is>
+          <t>Any other whistle triggers: Cancel that card. Turn player draws 1 card.</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="n"/>
       <c r="F59" s="138" t="n"/>
-      <c r="G59" s="107" t="n"/>
+      <c r="G59" s="101" t="n"/>
       <c r="H59" s="102" t="n"/>
       <c r="I59" s="102" t="n"/>
       <c r="J59" s="102" t="n"/>
@@ -4219,23 +4229,19 @@
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C60" s="31" t="inlineStr">
-        <is>
-          <t>Shot Clock Violation</t>
-        </is>
-      </c>
-      <c r="D60" s="91" t="inlineStr">
-        <is>
-          <t>Shot Clock is changed: TOV +1. Ball OOB</t>
-        </is>
-      </c>
-      <c r="E60" s="7" t="n"/>
+      <c r="C60" s="32" t="inlineStr">
+        <is>
+          <t>Official Review</t>
+        </is>
+      </c>
+      <c r="D60" s="94" t="inlineStr">
+        <is>
+          <t>Intangible Played: Discard all Intangibles from player.</t>
+        </is>
+      </c>
+      <c r="E60" s="34" t="n"/>
       <c r="F60" s="138" t="n"/>
-      <c r="G60" s="101" t="inlineStr">
-        <is>
-          <t>This inbound does NOT increment the round.</t>
-        </is>
-      </c>
+      <c r="G60" s="107" t="n"/>
       <c r="H60" s="102" t="n"/>
       <c r="I60" s="102" t="n"/>
       <c r="J60" s="102" t="n"/>
@@ -4247,19 +4253,23 @@
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C61" s="32" t="inlineStr">
-        <is>
-          <t>Technical Foul</t>
-        </is>
-      </c>
-      <c r="D61" s="94" t="inlineStr">
-        <is>
-          <t>Any Non-Whistle Card Played: Cancel card. Take 1 FT</t>
-        </is>
-      </c>
-      <c r="E61" s="34" t="n"/>
+      <c r="C61" s="31" t="inlineStr">
+        <is>
+          <t>Shot Clock Violation</t>
+        </is>
+      </c>
+      <c r="D61" s="91" t="inlineStr">
+        <is>
+          <t>Shot Clock is changed: TOV +1. Ball OOB</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="n"/>
       <c r="F61" s="138" t="n"/>
-      <c r="G61" s="107" t="n"/>
+      <c r="G61" s="101" t="inlineStr">
+        <is>
+          <t>This inbound does NOT increment the round.</t>
+        </is>
+      </c>
       <c r="H61" s="102" t="n"/>
       <c r="I61" s="102" t="n"/>
       <c r="J61" s="102" t="n"/>
@@ -4271,46 +4281,46 @@
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C62" s="31" t="inlineStr">
-        <is>
-          <t>Timeout</t>
-        </is>
-      </c>
-      <c r="D62" s="91" t="inlineStr">
-        <is>
-          <t>Immediate: Reset Shot Clock. You inbound. All players draw 1 card</t>
-        </is>
-      </c>
-      <c r="E62" s="7" t="n"/>
+      <c r="C62" s="32" t="inlineStr">
+        <is>
+          <t>Technical Foul</t>
+        </is>
+      </c>
+      <c r="D62" s="94" t="inlineStr">
+        <is>
+          <t>Any Non-Whistle Card Played: Cancel card. Take 1 FT</t>
+        </is>
+      </c>
+      <c r="E62" s="34" t="n"/>
       <c r="F62" s="138" t="n"/>
-      <c r="G62" s="101" t="n"/>
+      <c r="G62" s="107" t="n"/>
       <c r="H62" s="102" t="n"/>
       <c r="I62" s="102" t="n"/>
       <c r="J62" s="102" t="n"/>
     </row>
     <row r="63" ht="29" customHeight="1" s="132" thickBot="1">
-      <c r="A63" s="61" t="n"/>
-      <c r="B63" s="62" t="inlineStr">
+      <c r="A63" s="29" t="n"/>
+      <c r="B63" s="30" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C63" s="63" t="inlineStr">
-        <is>
-          <t>Travel</t>
-        </is>
-      </c>
-      <c r="D63" s="64" t="inlineStr">
-        <is>
-          <t>Move card played: Cancel card. TOV +1</t>
-        </is>
-      </c>
-      <c r="E63" s="65" t="n"/>
-      <c r="F63" s="140" t="n"/>
-      <c r="G63" s="116" t="n"/>
-      <c r="H63" s="117" t="n"/>
-      <c r="I63" s="117" t="n"/>
-      <c r="J63" s="117" t="n"/>
+      <c r="C63" s="31" t="inlineStr">
+        <is>
+          <t>Timeout</t>
+        </is>
+      </c>
+      <c r="D63" s="91" t="inlineStr">
+        <is>
+          <t>Immediate: Reset Shot Clock. You inbound. All players draw 1 card</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="n"/>
+      <c r="F63" s="138" t="n"/>
+      <c r="G63" s="101" t="n"/>
+      <c r="H63" s="102" t="n"/>
+      <c r="I63" s="102" t="n"/>
+      <c r="J63" s="102" t="n"/>
     </row>
     <row r="64" ht="20" customHeight="1" s="132">
       <c r="A64" s="61" t="n"/>
@@ -4321,69 +4331,67 @@
       </c>
       <c r="C64" s="63" t="inlineStr">
         <is>
-          <t>Clear Path Foul</t>
+          <t>Travel</t>
         </is>
       </c>
       <c r="D64" s="64" t="inlineStr">
         <is>
-          <t>On Shot, when Clamped by SHOT-reducing Clamps: Cancel those Clamps. Award the points the shot was worth. Take 1 FT</t>
+          <t>Move card played: Cancel card. TOV +1</t>
         </is>
       </c>
       <c r="E64" s="65" t="n"/>
       <c r="F64" s="140" t="n"/>
-      <c r="G64" s="116" t="inlineStr">
-        <is>
-          <t>Fires as the shot starts, before the cutscene. This DOES count as a completed round.</t>
-        </is>
-      </c>
+      <c r="G64" s="116" t="n"/>
       <c r="H64" s="117" t="n"/>
       <c r="I64" s="117" t="n"/>
       <c r="J64" s="117" t="n"/>
     </row>
     <row r="65" ht="28" customHeight="1" s="132">
-      <c r="A65" s="58" t="inlineStr">
+      <c r="A65" s="61" t="n"/>
+      <c r="B65" s="62" t="inlineStr">
+        <is>
+          <t>Whistle</t>
+        </is>
+      </c>
+      <c r="C65" s="63" t="inlineStr">
+        <is>
+          <t>Clear Path Foul</t>
+        </is>
+      </c>
+      <c r="D65" s="64" t="inlineStr">
+        <is>
+          <t>On Shot, when Clamped by SHOT-reducing Clamps: Cancel those Clamps. Award the points the shot was worth. Take 1 FT</t>
+        </is>
+      </c>
+      <c r="E65" s="65" t="n"/>
+      <c r="F65" s="140" t="n"/>
+      <c r="G65" s="116" t="inlineStr">
+        <is>
+          <t>Fires as the shot starts, before the cutscene. This DOES count as a completed round.</t>
+        </is>
+      </c>
+      <c r="H65" s="117" t="n"/>
+      <c r="I65" s="117" t="n"/>
+      <c r="J65" s="117" t="n"/>
+    </row>
+    <row r="66" ht="28" customHeight="1" s="132">
+      <c r="A66" s="58" t="inlineStr">
         <is>
           <t>Game Break</t>
         </is>
       </c>
-      <c r="B65" s="59">
-        <f>COUNTIF($B$5:$B$117,"Game Break")</f>
+      <c r="B66" s="59">
+        <f>COUNTIF($B$5:$B$118,"Game Break")</f>
         <v/>
       </c>
-      <c r="C65" s="60" t="n"/>
-      <c r="D65" s="60" t="n"/>
-      <c r="E65" s="60" t="n"/>
-      <c r="F65" s="86" t="n"/>
-      <c r="G65" s="109" t="n"/>
-      <c r="H65" s="110" t="n"/>
-      <c r="I65" s="110" t="n"/>
-      <c r="J65" s="110" t="n"/>
-    </row>
-    <row r="66" ht="28" customHeight="1" s="132">
-      <c r="A66" s="29" t="n"/>
-      <c r="B66" s="30" t="inlineStr">
-        <is>
-          <t>Game Break</t>
-        </is>
-      </c>
-      <c r="C66" s="32" t="inlineStr">
-        <is>
-          <t>2-Minute Warning</t>
-        </is>
-      </c>
-      <c r="D66" s="33" t="inlineStr">
-        <is>
-          <t>All players discard down to 2 or fewer cards</t>
-        </is>
-      </c>
-      <c r="E66" s="34" t="n"/>
-      <c r="F66" s="75" t="n">
-        <v>2</v>
-      </c>
-      <c r="G66" s="107" t="n"/>
-      <c r="H66" s="102" t="n"/>
-      <c r="I66" s="102" t="n"/>
-      <c r="J66" s="102" t="n"/>
+      <c r="C66" s="60" t="n"/>
+      <c r="D66" s="60" t="n"/>
+      <c r="E66" s="60" t="n"/>
+      <c r="F66" s="86" t="n"/>
+      <c r="G66" s="109" t="n"/>
+      <c r="H66" s="110" t="n"/>
+      <c r="I66" s="110" t="n"/>
+      <c r="J66" s="110" t="n"/>
     </row>
     <row r="67" ht="14" customHeight="1" s="132">
       <c r="A67" s="29" t="n"/>
@@ -4392,25 +4400,21 @@
           <t>Game Break</t>
         </is>
       </c>
-      <c r="C67" s="31" t="inlineStr">
-        <is>
-          <t>Benched</t>
-        </is>
-      </c>
-      <c r="D67" s="6" t="inlineStr">
-        <is>
-          <t>Immediately give ball to any other player.</t>
-        </is>
-      </c>
-      <c r="E67" s="7" t="n"/>
-      <c r="F67" s="76" t="n">
-        <v>5</v>
-      </c>
-      <c r="G67" s="111" t="inlineStr">
-        <is>
-          <t>This is not a pass</t>
-        </is>
-      </c>
+      <c r="C67" s="32" t="inlineStr">
+        <is>
+          <t>2-Minute Warning</t>
+        </is>
+      </c>
+      <c r="D67" s="33" t="inlineStr">
+        <is>
+          <t>All players discard down to 2 or fewer cards</t>
+        </is>
+      </c>
+      <c r="E67" s="34" t="n"/>
+      <c r="F67" s="75" t="n">
+        <v>2</v>
+      </c>
+      <c r="G67" s="107" t="n"/>
       <c r="H67" s="102" t="n"/>
       <c r="I67" s="102" t="n"/>
       <c r="J67" s="102" t="n"/>
@@ -4422,21 +4426,25 @@
           <t>Game Break</t>
         </is>
       </c>
-      <c r="C68" s="32" t="inlineStr">
-        <is>
-          <t>Crowd Noise</t>
-        </is>
-      </c>
-      <c r="D68" s="33" t="inlineStr">
-        <is>
-          <t>Discard 1 card.</t>
-        </is>
-      </c>
-      <c r="E68" s="34" t="n"/>
-      <c r="F68" s="75" t="n">
-        <v>14</v>
-      </c>
-      <c r="G68" s="107" t="n"/>
+      <c r="C68" s="31" t="inlineStr">
+        <is>
+          <t>Benched</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>Immediately give ball to any other player.</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="n"/>
+      <c r="F68" s="76" t="n">
+        <v>5</v>
+      </c>
+      <c r="G68" s="111" t="inlineStr">
+        <is>
+          <t>This is not a pass</t>
+        </is>
+      </c>
       <c r="H68" s="102" t="n"/>
       <c r="I68" s="102" t="n"/>
       <c r="J68" s="102" t="n"/>
@@ -4448,21 +4456,21 @@
           <t>Game Break</t>
         </is>
       </c>
-      <c r="C69" s="31" t="inlineStr">
-        <is>
-          <t>Designed Play</t>
-        </is>
-      </c>
-      <c r="D69" s="6" t="inlineStr">
-        <is>
-          <t>Draw up to a hand of 5</t>
-        </is>
-      </c>
-      <c r="E69" s="7" t="n"/>
-      <c r="F69" s="76" t="n">
-        <v>10</v>
-      </c>
-      <c r="G69" s="101" t="n"/>
+      <c r="C69" s="32" t="inlineStr">
+        <is>
+          <t>Crowd Noise</t>
+        </is>
+      </c>
+      <c r="D69" s="33" t="inlineStr">
+        <is>
+          <t>Discard 1 card.</t>
+        </is>
+      </c>
+      <c r="E69" s="34" t="n"/>
+      <c r="F69" s="75" t="n">
+        <v>14</v>
+      </c>
+      <c r="G69" s="107" t="n"/>
       <c r="H69" s="102" t="n"/>
       <c r="I69" s="102" t="n"/>
       <c r="J69" s="102" t="n"/>
@@ -4474,21 +4482,21 @@
           <t>Game Break</t>
         </is>
       </c>
-      <c r="C70" s="90" t="inlineStr">
-        <is>
-          <t>Foul</t>
-        </is>
-      </c>
-      <c r="D70" s="33" t="inlineStr">
-        <is>
-          <t>Take 1 FT</t>
-        </is>
-      </c>
-      <c r="E70" s="34" t="n"/>
-      <c r="F70" s="75" t="n">
-        <v>5</v>
-      </c>
-      <c r="G70" s="107" t="n"/>
+      <c r="C70" s="31" t="inlineStr">
+        <is>
+          <t>Designed Play</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>Draw up to a hand of 5</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="n"/>
+      <c r="F70" s="76" t="n">
+        <v>10</v>
+      </c>
+      <c r="G70" s="101" t="n"/>
       <c r="H70" s="102" t="n"/>
       <c r="I70" s="102" t="n"/>
       <c r="J70" s="102" t="n"/>
@@ -4500,21 +4508,21 @@
           <t>Game Break</t>
         </is>
       </c>
-      <c r="C71" s="31" t="inlineStr">
-        <is>
-          <t>MVP Vote</t>
-        </is>
-      </c>
-      <c r="D71" s="6" t="inlineStr">
-        <is>
-          <t>Draw 3 cards up to a hand of 7</t>
-        </is>
-      </c>
-      <c r="E71" s="7" t="n"/>
-      <c r="F71" s="76" t="n">
-        <v>1</v>
-      </c>
-      <c r="G71" s="101" t="n"/>
+      <c r="C71" s="90" t="inlineStr">
+        <is>
+          <t>Foul</t>
+        </is>
+      </c>
+      <c r="D71" s="33" t="inlineStr">
+        <is>
+          <t>Take 1 FT</t>
+        </is>
+      </c>
+      <c r="E71" s="34" t="n"/>
+      <c r="F71" s="75" t="n">
+        <v>5</v>
+      </c>
+      <c r="G71" s="107" t="n"/>
       <c r="H71" s="102" t="n"/>
       <c r="I71" s="102" t="n"/>
       <c r="J71" s="102" t="n"/>
@@ -4526,21 +4534,21 @@
           <t>Game Break</t>
         </is>
       </c>
-      <c r="C72" s="32" t="inlineStr">
-        <is>
-          <t>Off Night</t>
-        </is>
-      </c>
-      <c r="D72" s="33" t="inlineStr">
-        <is>
-          <t>SHOT -20% this possession</t>
-        </is>
-      </c>
-      <c r="E72" s="34" t="n"/>
-      <c r="F72" s="75" t="n">
-        <v>3</v>
-      </c>
-      <c r="G72" s="107" t="n"/>
+      <c r="C72" s="31" t="inlineStr">
+        <is>
+          <t>MVP Vote</t>
+        </is>
+      </c>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>Draw 3 cards up to a hand of 7</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="n"/>
+      <c r="F72" s="76" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" s="101" t="n"/>
       <c r="H72" s="102" t="n"/>
       <c r="I72" s="102" t="n"/>
       <c r="J72" s="102" t="n"/>
@@ -4552,25 +4560,21 @@
           <t>Game Break</t>
         </is>
       </c>
-      <c r="C73" s="31" t="inlineStr">
-        <is>
-          <t>Swallowed Whistle</t>
-        </is>
-      </c>
-      <c r="D73" s="6" t="inlineStr">
-        <is>
-          <t>Whistle cards cannot activate this turn.</t>
-        </is>
-      </c>
-      <c r="E73" s="6" t="inlineStr">
-        <is>
-          <t>Remains for remainder of round</t>
-        </is>
-      </c>
-      <c r="F73" s="74" t="n">
-        <v>5</v>
-      </c>
-      <c r="G73" s="101" t="n"/>
+      <c r="C73" s="32" t="inlineStr">
+        <is>
+          <t>Off Night</t>
+        </is>
+      </c>
+      <c r="D73" s="33" t="inlineStr">
+        <is>
+          <t>SHOT -20% this possession</t>
+        </is>
+      </c>
+      <c r="E73" s="34" t="n"/>
+      <c r="F73" s="75" t="n">
+        <v>3</v>
+      </c>
+      <c r="G73" s="107" t="n"/>
       <c r="H73" s="102" t="n"/>
       <c r="I73" s="102" t="n"/>
       <c r="J73" s="102" t="n"/>
@@ -4582,23 +4586,25 @@
           <t>Game Break</t>
         </is>
       </c>
-      <c r="C74" s="32" t="inlineStr">
-        <is>
-          <t>Rock Fight</t>
-        </is>
-      </c>
-      <c r="D74" s="33" t="inlineStr">
-        <is>
-          <t>Players cannot shoot when SHOT is 50% or higher</t>
-        </is>
-      </c>
-      <c r="E74" s="33" t="inlineStr">
+      <c r="C74" s="31" t="inlineStr">
+        <is>
+          <t>Swallowed Whistle</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>Whistle cards cannot activate this turn.</t>
+        </is>
+      </c>
+      <c r="E74" s="6" t="inlineStr">
         <is>
           <t>Remains for remainder of round</t>
         </is>
       </c>
-      <c r="F74" s="80" t="n"/>
-      <c r="G74" s="107" t="n"/>
+      <c r="F74" s="74" t="n">
+        <v>5</v>
+      </c>
+      <c r="G74" s="101" t="n"/>
       <c r="H74" s="102" t="n"/>
       <c r="I74" s="102" t="n"/>
       <c r="J74" s="102" t="n"/>
@@ -4610,23 +4616,23 @@
           <t>Game Break</t>
         </is>
       </c>
-      <c r="C75" s="31" t="inlineStr">
-        <is>
-          <t>Traded Mid-Game</t>
-        </is>
-      </c>
-      <c r="D75" s="6" t="inlineStr">
-        <is>
-          <t>Swap positions with random other player</t>
-        </is>
-      </c>
-      <c r="E75" s="7" t="n"/>
-      <c r="F75" s="76" t="n"/>
-      <c r="G75" s="111" t="inlineStr">
-        <is>
-          <t>Applies to rest of game</t>
-        </is>
-      </c>
+      <c r="C75" s="32" t="inlineStr">
+        <is>
+          <t>Rock Fight</t>
+        </is>
+      </c>
+      <c r="D75" s="33" t="inlineStr">
+        <is>
+          <t>Players cannot shoot when SHOT is 50% or higher</t>
+        </is>
+      </c>
+      <c r="E75" s="33" t="inlineStr">
+        <is>
+          <t>Remains for remainder of round</t>
+        </is>
+      </c>
+      <c r="F75" s="80" t="n"/>
+      <c r="G75" s="107" t="n"/>
       <c r="H75" s="102" t="n"/>
       <c r="I75" s="102" t="n"/>
       <c r="J75" s="102" t="n"/>
@@ -4638,21 +4644,23 @@
           <t>Game Break</t>
         </is>
       </c>
-      <c r="C76" s="134" t="inlineStr">
-        <is>
-          <t>Salary Cap Increase</t>
-        </is>
-      </c>
-      <c r="D76" s="91" t="inlineStr">
-        <is>
-          <t>All players draw 2 cards</t>
+      <c r="C76" s="31" t="inlineStr">
+        <is>
+          <t>Traded Mid-Game</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>Swap positions with random other player</t>
         </is>
       </c>
       <c r="E76" s="7" t="n"/>
-      <c r="F76" s="76" t="n">
-        <v>4</v>
-      </c>
-      <c r="G76" s="111" t="n"/>
+      <c r="F76" s="76" t="n"/>
+      <c r="G76" s="111" t="inlineStr">
+        <is>
+          <t>Applies to rest of game</t>
+        </is>
+      </c>
       <c r="H76" s="102" t="n"/>
       <c r="I76" s="102" t="n"/>
       <c r="J76" s="102" t="n"/>
@@ -4666,23 +4674,19 @@
       </c>
       <c r="C77" s="134" t="inlineStr">
         <is>
-          <t>All-Swissh Selection</t>
+          <t>Salary Cap Increase</t>
         </is>
       </c>
       <c r="D77" s="91" t="inlineStr">
         <is>
-          <t>Draw 3 cards after your next make</t>
+          <t>All players draw 2 cards</t>
         </is>
       </c>
       <c r="E77" s="7" t="n"/>
       <c r="F77" s="76" t="n">
-        <v>3</v>
-      </c>
-      <c r="G77" s="111" t="inlineStr">
-        <is>
-          <t>Arms an icon in the HUD tracking the pending draws</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="G77" s="111" t="n"/>
       <c r="H77" s="102" t="n"/>
       <c r="I77" s="102" t="n"/>
       <c r="J77" s="102" t="n"/>
@@ -4696,19 +4700,23 @@
       </c>
       <c r="C78" s="134" t="inlineStr">
         <is>
-          <t>All Star Selection</t>
+          <t>All-Swissh Selection</t>
         </is>
       </c>
       <c r="D78" s="91" t="inlineStr">
         <is>
-          <t>Draw 2 cards</t>
+          <t>Draw 3 cards after your next make</t>
         </is>
       </c>
       <c r="E78" s="7" t="n"/>
       <c r="F78" s="76" t="n">
-        <v>5</v>
-      </c>
-      <c r="G78" s="111" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="G78" s="111" t="inlineStr">
+        <is>
+          <t>Arms an icon in the HUD tracking the pending draws</t>
+        </is>
+      </c>
       <c r="H78" s="102" t="n"/>
       <c r="I78" s="102" t="n"/>
       <c r="J78" s="102" t="n"/>
@@ -4722,23 +4730,19 @@
       </c>
       <c r="C79" s="134" t="inlineStr">
         <is>
-          <t>Hit the Bike</t>
+          <t>All Star Selection</t>
         </is>
       </c>
       <c r="D79" s="91" t="inlineStr">
         <is>
-          <t>Discard all Injuries. Draw 1 card. Give possession to another player</t>
+          <t>Draw 2 cards</t>
         </is>
       </c>
       <c r="E79" s="7" t="n"/>
       <c r="F79" s="76" t="n">
         <v>5</v>
       </c>
-      <c r="G79" s="111" t="inlineStr">
-        <is>
-          <t>This is not a pass</t>
-        </is>
-      </c>
+      <c r="G79" s="111" t="n"/>
       <c r="H79" s="102" t="n"/>
       <c r="I79" s="102" t="n"/>
       <c r="J79" s="102" t="n"/>
@@ -4752,19 +4756,23 @@
       </c>
       <c r="C80" s="134" t="inlineStr">
         <is>
-          <t>Ice Wrap</t>
+          <t>Hit the Bike</t>
         </is>
       </c>
       <c r="D80" s="91" t="inlineStr">
         <is>
-          <t>Draw 1 card. Discard all Injuries. If none, draw 1 additional card</t>
+          <t>Discard all Injuries. Draw 1 card. Give possession to another player</t>
         </is>
       </c>
       <c r="E80" s="7" t="n"/>
       <c r="F80" s="76" t="n">
         <v>5</v>
       </c>
-      <c r="G80" s="111" t="n"/>
+      <c r="G80" s="111" t="inlineStr">
+        <is>
+          <t>This is not a pass</t>
+        </is>
+      </c>
       <c r="H80" s="102" t="n"/>
       <c r="I80" s="102" t="n"/>
       <c r="J80" s="102" t="n"/>
@@ -4778,23 +4786,19 @@
       </c>
       <c r="C81" s="134" t="inlineStr">
         <is>
-          <t>Wet Spot</t>
+          <t>Ice Wrap</t>
         </is>
       </c>
       <c r="D81" s="91" t="inlineStr">
         <is>
-          <t>All Injuries in the discards and deck are displayed. Take one</t>
+          <t>Draw 1 card. Discard all Injuries. If none, draw 1 additional card</t>
         </is>
       </c>
       <c r="E81" s="7" t="n"/>
       <c r="F81" s="76" t="n">
-        <v>2</v>
-      </c>
-      <c r="G81" s="111" t="inlineStr">
-        <is>
-          <t>Deck ones are shown face down</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="G81" s="111" t="n"/>
       <c r="H81" s="102" t="n"/>
       <c r="I81" s="102" t="n"/>
       <c r="J81" s="102" t="n"/>
@@ -4808,21 +4812,21 @@
       </c>
       <c r="C82" s="134" t="inlineStr">
         <is>
-          <t>Fresh Ball</t>
+          <t>Wet Spot</t>
         </is>
       </c>
       <c r="D82" s="91" t="inlineStr">
         <is>
-          <t>Next player does not draw at the start of their possession</t>
+          <t>All Injuries in the discards and deck are displayed. Take one</t>
         </is>
       </c>
       <c r="E82" s="7" t="n"/>
       <c r="F82" s="76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G82" s="111" t="inlineStr">
         <is>
-          <t>This is a bad thing in the NBA</t>
+          <t>Deck ones are shown face down</t>
         </is>
       </c>
       <c r="H82" s="102" t="n"/>
@@ -4838,12 +4842,12 @@
       </c>
       <c r="C83" s="134" t="inlineStr">
         <is>
-          <t>Trade Deadline</t>
+          <t>Fresh Ball</t>
         </is>
       </c>
       <c r="D83" s="91" t="inlineStr">
         <is>
-          <t>Declare Left or Right: every player passes their hand that way. The ball goes with it</t>
+          <t>Next player does not draw at the start of their possession</t>
         </is>
       </c>
       <c r="E83" s="7" t="n"/>
@@ -4852,7 +4856,7 @@
       </c>
       <c r="G83" s="111" t="inlineStr">
         <is>
-          <t>The hex travels in the declared direction too</t>
+          <t>This is a bad thing in the NBA</t>
         </is>
       </c>
       <c r="H83" s="102" t="n"/>
@@ -4868,19 +4872,23 @@
       </c>
       <c r="C84" s="134" t="inlineStr">
         <is>
-          <t>Floor Cleanup</t>
+          <t>Trade Deadline</t>
         </is>
       </c>
       <c r="D84" s="91" t="inlineStr">
         <is>
-          <t>All players shuffle their hands into the deck and draw the same number of cards</t>
+          <t>Declare Left or Right: every player passes their hand that way. The ball goes with it</t>
         </is>
       </c>
       <c r="E84" s="7" t="n"/>
       <c r="F84" s="76" t="n">
         <v>3</v>
       </c>
-      <c r="G84" s="111" t="n"/>
+      <c r="G84" s="111" t="inlineStr">
+        <is>
+          <t>The hex travels in the declared direction too</t>
+        </is>
+      </c>
       <c r="H84" s="102" t="n"/>
       <c r="I84" s="102" t="n"/>
       <c r="J84" s="102" t="n"/>
@@ -4894,17 +4902,17 @@
       </c>
       <c r="C85" s="134" t="inlineStr">
         <is>
-          <t>Official Timeout</t>
+          <t>Floor Cleanup</t>
         </is>
       </c>
       <c r="D85" s="91" t="inlineStr">
         <is>
-          <t>At least 1 referee must be armed: discard all Injuries on all players and clear all referees. If none, all players draw 1 card</t>
+          <t>All players shuffle their hands into the deck and draw the same number of cards</t>
         </is>
       </c>
       <c r="E85" s="7" t="n"/>
       <c r="F85" s="76" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G85" s="111" t="n"/>
       <c r="H85" s="102" t="n"/>
@@ -4920,17 +4928,17 @@
       </c>
       <c r="C86" s="134" t="inlineStr">
         <is>
-          <t>Team Doctor</t>
+          <t>Official Timeout</t>
         </is>
       </c>
       <c r="D86" s="91" t="inlineStr">
         <is>
-          <t>Discard 1 Injury from a player of choice. Draw 2 cards if not choosing yourself</t>
+          <t>At least 1 referee must be armed: discard all Injuries on all players and clear all referees. If none, all players draw 1 card</t>
         </is>
       </c>
       <c r="E86" s="7" t="n"/>
       <c r="F86" s="76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G86" s="111" t="n"/>
       <c r="H86" s="102" t="n"/>
@@ -4938,160 +4946,162 @@
       <c r="J86" s="102" t="n"/>
     </row>
     <row r="87" ht="56" customHeight="1" s="132">
-      <c r="A87" s="55" t="inlineStr">
-        <is>
-          <t>Injury GB</t>
-        </is>
-      </c>
-      <c r="B87" s="56">
-        <f>COUNTIF($B$5:$B$117,"Injury GB")</f>
-        <v/>
-      </c>
-      <c r="C87" s="57" t="n"/>
-      <c r="D87" s="57" t="n"/>
-      <c r="E87" s="57" t="n"/>
-      <c r="F87" s="88" t="n"/>
-      <c r="G87" s="108" t="n"/>
+      <c r="A87" s="29" t="n"/>
+      <c r="B87" s="30" t="inlineStr">
+        <is>
+          <t>Game Break</t>
+        </is>
+      </c>
+      <c r="C87" s="134" t="inlineStr">
+        <is>
+          <t>Team Doctor</t>
+        </is>
+      </c>
+      <c r="D87" s="91" t="inlineStr">
+        <is>
+          <t>Discard 1 Injury from a player of choice. Draw 2 cards if not choosing yourself</t>
+        </is>
+      </c>
+      <c r="E87" s="7" t="n"/>
+      <c r="F87" s="76" t="n">
+        <v>3</v>
+      </c>
+      <c r="G87" s="111" t="n"/>
       <c r="H87" s="102" t="n"/>
       <c r="I87" s="102" t="n"/>
       <c r="J87" s="102" t="n"/>
     </row>
     <row r="88" ht="28" customHeight="1" s="132">
-      <c r="A88" s="29" t="n"/>
-      <c r="B88" s="30" t="inlineStr">
+      <c r="A88" s="55" t="inlineStr">
         <is>
           <t>Injury GB</t>
         </is>
       </c>
-      <c r="C88" s="31" t="inlineStr">
-        <is>
-          <t>Bone Bruise</t>
-        </is>
-      </c>
-      <c r="D88" s="91" t="inlineStr">
-        <is>
-          <t>Discard 1 card at the start of each turn after drawing (your choice)</t>
-        </is>
-      </c>
-      <c r="E88" s="7" t="n"/>
-      <c r="F88" s="76" t="n">
-        <v>3</v>
-      </c>
-      <c r="G88" s="101" t="n"/>
+      <c r="B88" s="56">
+        <f>COUNTIF($B$5:$B$118,"Injury GB")</f>
+        <v/>
+      </c>
+      <c r="C88" s="57" t="n"/>
+      <c r="D88" s="57" t="n"/>
+      <c r="E88" s="57" t="n"/>
+      <c r="F88" s="88" t="n"/>
+      <c r="G88" s="108" t="n"/>
       <c r="H88" s="102" t="n"/>
       <c r="I88" s="102" t="n"/>
       <c r="J88" s="102" t="n"/>
     </row>
     <row r="89" ht="42" customHeight="1" s="132">
-      <c r="A89" s="58" t="inlineStr">
+      <c r="A89" s="29" t="n"/>
+      <c r="B89" s="30" t="inlineStr">
+        <is>
+          <t>Injury GB</t>
+        </is>
+      </c>
+      <c r="C89" s="31" t="inlineStr">
+        <is>
+          <t>Bone Bruise</t>
+        </is>
+      </c>
+      <c r="D89" s="91" t="inlineStr">
+        <is>
+          <t>Discard 1 card at the start of each turn after drawing (your choice)</t>
+        </is>
+      </c>
+      <c r="E89" s="7" t="n"/>
+      <c r="F89" s="76" t="n">
+        <v>3</v>
+      </c>
+      <c r="G89" s="101" t="n"/>
+      <c r="H89" s="102" t="n"/>
+      <c r="I89" s="102" t="n"/>
+      <c r="J89" s="102" t="n"/>
+    </row>
+    <row r="90" ht="28" customHeight="1" s="132">
+      <c r="A90" s="58" t="inlineStr">
         <is>
           <t>Devastating Injury GB</t>
         </is>
       </c>
-      <c r="B89" s="59">
-        <f>COUNTIF($B$5:$B$117,"Devastating Injury GB")</f>
+      <c r="B90" s="59">
+        <f>COUNTIF($B$5:$B$118,"Devastating Injury GB")</f>
         <v/>
       </c>
-      <c r="C89" s="60" t="n"/>
-      <c r="D89" s="60" t="n"/>
-      <c r="E89" s="60" t="n"/>
-      <c r="F89" s="86" t="n"/>
-      <c r="G89" s="109" t="n"/>
-      <c r="H89" s="110" t="n"/>
-      <c r="I89" s="110" t="n"/>
-      <c r="J89" s="110" t="n"/>
-    </row>
-    <row r="90" ht="28" customHeight="1" s="132">
-      <c r="A90" s="50" t="n"/>
-      <c r="B90" s="51" t="inlineStr">
+      <c r="C90" s="60" t="n"/>
+      <c r="D90" s="60" t="n"/>
+      <c r="E90" s="60" t="n"/>
+      <c r="F90" s="86" t="n"/>
+      <c r="G90" s="109" t="n"/>
+      <c r="H90" s="110" t="n"/>
+      <c r="I90" s="110" t="n"/>
+      <c r="J90" s="110" t="n"/>
+    </row>
+    <row r="91" ht="42" customHeight="1" s="132">
+      <c r="A91" s="50" t="n"/>
+      <c r="B91" s="51" t="inlineStr">
         <is>
           <t>Devastating Injury GB</t>
         </is>
       </c>
-      <c r="C90" s="136" t="inlineStr">
+      <c r="C91" s="136" t="inlineStr">
         <is>
           <t>Torn Achilles</t>
         </is>
       </c>
-      <c r="D90" s="137" t="inlineStr">
+      <c r="D91" s="137" t="inlineStr">
         <is>
           <t>Hand is locked every turn except 1 card (randomly)</t>
         </is>
       </c>
-      <c r="E90" s="54" t="n"/>
-      <c r="F90" s="141" t="n"/>
-      <c r="G90" s="114" t="n"/>
-      <c r="H90" s="115" t="n"/>
-      <c r="I90" s="115" t="n"/>
-      <c r="J90" s="115" t="n"/>
-    </row>
-    <row r="91" ht="42" customHeight="1" s="132">
-      <c r="A91" s="55" t="inlineStr">
+      <c r="E91" s="54" t="n"/>
+      <c r="F91" s="141" t="n"/>
+      <c r="G91" s="114" t="n"/>
+      <c r="H91" s="115" t="n"/>
+      <c r="I91" s="115" t="n"/>
+      <c r="J91" s="115" t="n"/>
+    </row>
+    <row r="92" ht="14" customHeight="1" s="132">
+      <c r="A92" s="55" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="B91" s="56">
-        <f>COUNTIF($B$5:$B$117,"Intangible")</f>
+      <c r="B92" s="56">
+        <f>COUNTIF($B$5:$B$118,"Intangible")</f>
         <v/>
       </c>
-      <c r="C91" s="57" t="n"/>
-      <c r="D91" s="57" t="n"/>
-      <c r="E91" s="57" t="n"/>
-      <c r="F91" s="88" t="n"/>
-      <c r="G91" s="108" t="n"/>
-      <c r="H91" s="102" t="n"/>
-      <c r="I91" s="102" t="n"/>
-      <c r="J91" s="102" t="n"/>
-    </row>
-    <row r="92" ht="14" customHeight="1" s="132">
-      <c r="A92" s="96" t="inlineStr">
-        <is>
-          <t>All intangibles are limited to 1</t>
-        </is>
-      </c>
-      <c r="B92" s="30" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C92" s="31" t="inlineStr">
-        <is>
-          <t>Board-Crasher</t>
-        </is>
-      </c>
-      <c r="D92" s="6" t="inlineStr">
-        <is>
-          <t>SHOT +10% upon Rebounding your own missed shot</t>
-        </is>
-      </c>
-      <c r="E92" s="7" t="n"/>
-      <c r="F92" s="138" t="n"/>
-      <c r="G92" s="101" t="n"/>
+      <c r="C92" s="57" t="n"/>
+      <c r="D92" s="57" t="n"/>
+      <c r="E92" s="57" t="n"/>
+      <c r="F92" s="88" t="n"/>
+      <c r="G92" s="108" t="n"/>
       <c r="H92" s="102" t="n"/>
       <c r="I92" s="102" t="n"/>
       <c r="J92" s="102" t="n"/>
     </row>
     <row r="93" ht="28" customHeight="1" s="132">
-      <c r="A93" s="29" t="n"/>
+      <c r="A93" s="96" t="inlineStr">
+        <is>
+          <t>All intangibles are limited to 1</t>
+        </is>
+      </c>
       <c r="B93" s="30" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C93" s="32" t="inlineStr">
-        <is>
-          <t>Catch &amp; Shoot Specialist</t>
-        </is>
-      </c>
-      <c r="D93" s="33" t="inlineStr">
-        <is>
-          <t>Additional SHOT +10% on all received passes</t>
-        </is>
-      </c>
-      <c r="E93" s="34" t="n"/>
+      <c r="C93" s="31" t="inlineStr">
+        <is>
+          <t>Board-Crasher</t>
+        </is>
+      </c>
+      <c r="D93" s="6" t="inlineStr">
+        <is>
+          <t>SHOT +10% upon Rebounding your own missed shot</t>
+        </is>
+      </c>
+      <c r="E93" s="7" t="n"/>
       <c r="F93" s="138" t="n"/>
-      <c r="G93" s="107" t="n"/>
+      <c r="G93" s="101" t="n"/>
       <c r="H93" s="102" t="n"/>
       <c r="I93" s="102" t="n"/>
       <c r="J93" s="102" t="n"/>
@@ -5103,19 +5113,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C94" s="31" t="inlineStr">
-        <is>
-          <t>Clutch Gene</t>
-        </is>
-      </c>
-      <c r="D94" s="6" t="inlineStr">
-        <is>
-          <t>SHOT x2 if attempting a shot with 1 or fewer cards in hand or Shot Clock 3 or less</t>
-        </is>
-      </c>
-      <c r="E94" s="7" t="n"/>
+      <c r="C94" s="32" t="inlineStr">
+        <is>
+          <t>Catch &amp; Shoot Specialist</t>
+        </is>
+      </c>
+      <c r="D94" s="33" t="inlineStr">
+        <is>
+          <t>Additional SHOT +10% on all received passes</t>
+        </is>
+      </c>
+      <c r="E94" s="34" t="n"/>
       <c r="F94" s="138" t="n"/>
-      <c r="G94" s="101" t="n"/>
+      <c r="G94" s="107" t="n"/>
       <c r="H94" s="102" t="n"/>
       <c r="I94" s="102" t="n"/>
       <c r="J94" s="102" t="n"/>
@@ -5127,19 +5137,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C95" s="32" t="inlineStr">
-        <is>
-          <t>Floor General</t>
-        </is>
-      </c>
-      <c r="D95" s="33" t="inlineStr">
-        <is>
-          <t>You choose all targets of all kinds — card declarations, non auto-pass targets, and the rest</t>
-        </is>
-      </c>
-      <c r="E95" s="34" t="n"/>
+      <c r="C95" s="31" t="inlineStr">
+        <is>
+          <t>Clutch Gene</t>
+        </is>
+      </c>
+      <c r="D95" s="6" t="inlineStr">
+        <is>
+          <t>SHOT x2 if attempting a shot with 1 or fewer cards in hand or Shot Clock 3 or less</t>
+        </is>
+      </c>
+      <c r="E95" s="7" t="n"/>
       <c r="F95" s="138" t="n"/>
-      <c r="G95" s="107" t="n"/>
+      <c r="G95" s="101" t="n"/>
       <c r="H95" s="102" t="n"/>
       <c r="I95" s="102" t="n"/>
       <c r="J95" s="102" t="n"/>
@@ -5151,23 +5161,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C96" s="31" t="inlineStr">
-        <is>
-          <t>Fox-Like First Step</t>
-        </is>
-      </c>
-      <c r="D96" s="6" t="inlineStr">
-        <is>
-          <t>All Move cards that reduce SHOT increase it by that amount instead.</t>
-        </is>
-      </c>
-      <c r="E96" s="6" t="inlineStr">
-        <is>
-          <t>Your Move cards are unaffected by opponents</t>
-        </is>
-      </c>
-      <c r="F96" s="139" t="n"/>
-      <c r="G96" s="101" t="n"/>
+      <c r="C96" s="32" t="inlineStr">
+        <is>
+          <t>Floor General</t>
+        </is>
+      </c>
+      <c r="D96" s="33" t="inlineStr">
+        <is>
+          <t>You choose all targets of all kinds — card declarations, non auto-pass targets, and the rest</t>
+        </is>
+      </c>
+      <c r="E96" s="34" t="n"/>
+      <c r="F96" s="138" t="n"/>
+      <c r="G96" s="107" t="n"/>
       <c r="H96" s="102" t="n"/>
       <c r="I96" s="102" t="n"/>
       <c r="J96" s="102" t="n"/>
@@ -5179,19 +5185,23 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C97" s="90" t="inlineStr">
-        <is>
-          <t>Freethrow Merchant</t>
-        </is>
-      </c>
-      <c r="D97" s="94" t="inlineStr">
-        <is>
-          <t>All Clamps on you grant 1 FT instead</t>
-        </is>
-      </c>
-      <c r="E97" s="34" t="n"/>
-      <c r="F97" s="138" t="n"/>
-      <c r="G97" s="125" t="n"/>
+      <c r="C97" s="31" t="inlineStr">
+        <is>
+          <t>Fox-Like First Step</t>
+        </is>
+      </c>
+      <c r="D97" s="6" t="inlineStr">
+        <is>
+          <t>All Move cards that reduce SHOT increase it by that amount instead.</t>
+        </is>
+      </c>
+      <c r="E97" s="6" t="inlineStr">
+        <is>
+          <t>Your Move cards are unaffected by opponents</t>
+        </is>
+      </c>
+      <c r="F97" s="139" t="n"/>
+      <c r="G97" s="101" t="n"/>
       <c r="H97" s="102" t="n"/>
       <c r="I97" s="102" t="n"/>
       <c r="J97" s="102" t="n"/>
@@ -5205,17 +5215,17 @@
       </c>
       <c r="C98" s="90" t="inlineStr">
         <is>
-          <t>Generational Whistle</t>
-        </is>
-      </c>
-      <c r="D98" s="91" t="inlineStr">
-        <is>
-          <t>Take 1 additional FT</t>
-        </is>
-      </c>
-      <c r="E98" s="7" t="n"/>
+          <t>Freethrow Merchant</t>
+        </is>
+      </c>
+      <c r="D98" s="94" t="inlineStr">
+        <is>
+          <t>All Clamps on you grant 1 FT instead</t>
+        </is>
+      </c>
+      <c r="E98" s="34" t="n"/>
       <c r="F98" s="138" t="n"/>
-      <c r="G98" s="101" t="n"/>
+      <c r="G98" s="125" t="n"/>
       <c r="H98" s="102" t="n"/>
       <c r="I98" s="102" t="n"/>
       <c r="J98" s="102" t="n"/>
@@ -5227,19 +5237,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C99" s="32" t="inlineStr">
-        <is>
-          <t>Gravity</t>
-        </is>
-      </c>
-      <c r="D99" s="33" t="inlineStr">
-        <is>
-          <t>All Clamps automatically apply to you. +1 AST whenever another player attempts a shot</t>
-        </is>
-      </c>
-      <c r="E99" s="34" t="n"/>
+      <c r="C99" s="90" t="inlineStr">
+        <is>
+          <t>Generational Whistle</t>
+        </is>
+      </c>
+      <c r="D99" s="91" t="inlineStr">
+        <is>
+          <t>Take 1 additional FT</t>
+        </is>
+      </c>
+      <c r="E99" s="7" t="n"/>
       <c r="F99" s="138" t="n"/>
-      <c r="G99" s="107" t="n"/>
+      <c r="G99" s="101" t="n"/>
       <c r="H99" s="102" t="n"/>
       <c r="I99" s="102" t="n"/>
       <c r="J99" s="102" t="n"/>
@@ -5251,19 +5261,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C100" s="31" t="inlineStr">
-        <is>
-          <t>Great Conditioning</t>
-        </is>
-      </c>
-      <c r="D100" s="6" t="inlineStr">
-        <is>
-          <t>Immediately discard all Injury Game Breaks you draw and draw a new card for each</t>
-        </is>
-      </c>
-      <c r="E100" s="7" t="n"/>
+      <c r="C100" s="32" t="inlineStr">
+        <is>
+          <t>Gravity</t>
+        </is>
+      </c>
+      <c r="D100" s="33" t="inlineStr">
+        <is>
+          <t>All Clamps automatically apply to you. +1 AST whenever another player attempts a shot</t>
+        </is>
+      </c>
+      <c r="E100" s="34" t="n"/>
       <c r="F100" s="138" t="n"/>
-      <c r="G100" s="101" t="n"/>
+      <c r="G100" s="107" t="n"/>
       <c r="H100" s="102" t="n"/>
       <c r="I100" s="102" t="n"/>
       <c r="J100" s="102" t="n"/>
@@ -5275,19 +5285,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C101" s="32" t="inlineStr">
-        <is>
-          <t>Hot Hand</t>
-        </is>
-      </c>
-      <c r="D101" s="33" t="inlineStr">
-        <is>
-          <t>SHOT +20% if you scored last round.</t>
-        </is>
-      </c>
-      <c r="E101" s="34" t="n"/>
+      <c r="C101" s="31" t="inlineStr">
+        <is>
+          <t>Great Conditioning</t>
+        </is>
+      </c>
+      <c r="D101" s="6" t="inlineStr">
+        <is>
+          <t>Immediately discard all Injury Game Breaks you draw and draw a new card for each</t>
+        </is>
+      </c>
+      <c r="E101" s="7" t="n"/>
       <c r="F101" s="138" t="n"/>
-      <c r="G101" s="107" t="n"/>
+      <c r="G101" s="101" t="n"/>
       <c r="H101" s="102" t="n"/>
       <c r="I101" s="102" t="n"/>
       <c r="J101" s="102" t="n"/>
@@ -5299,19 +5309,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C102" s="31" t="inlineStr">
-        <is>
-          <t>Like That</t>
-        </is>
-      </c>
-      <c r="D102" s="91" t="inlineStr">
-        <is>
-          <t>Your SHOT % cannot be reduced</t>
-        </is>
-      </c>
-      <c r="E102" s="7" t="n"/>
+      <c r="C102" s="32" t="inlineStr">
+        <is>
+          <t>Hot Hand</t>
+        </is>
+      </c>
+      <c r="D102" s="33" t="inlineStr">
+        <is>
+          <t>SHOT +20% if you scored last round.</t>
+        </is>
+      </c>
+      <c r="E102" s="34" t="n"/>
       <c r="F102" s="138" t="n"/>
-      <c r="G102" s="101" t="n"/>
+      <c r="G102" s="107" t="n"/>
       <c r="H102" s="102" t="n"/>
       <c r="I102" s="102" t="n"/>
       <c r="J102" s="102" t="n"/>
@@ -5323,23 +5333,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C103" s="32" t="inlineStr">
-        <is>
-          <t>No Bag</t>
-        </is>
-      </c>
-      <c r="D103" s="33" t="inlineStr">
-        <is>
-          <t>Cannot activate Move cards this round</t>
-        </is>
-      </c>
-      <c r="E103" s="34" t="n"/>
+      <c r="C103" s="31" t="inlineStr">
+        <is>
+          <t>Like That</t>
+        </is>
+      </c>
+      <c r="D103" s="91" t="inlineStr">
+        <is>
+          <t>Your SHOT % cannot be reduced</t>
+        </is>
+      </c>
+      <c r="E103" s="7" t="n"/>
       <c r="F103" s="138" t="n"/>
-      <c r="G103" s="113" t="inlineStr">
-        <is>
-          <t>Bad card to draw</t>
-        </is>
-      </c>
+      <c r="G103" s="101" t="n"/>
       <c r="H103" s="102" t="n"/>
       <c r="I103" s="102" t="n"/>
       <c r="J103" s="102" t="n"/>
@@ -5351,19 +5357,23 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C104" s="31" t="inlineStr">
-        <is>
-          <t>Point God</t>
-        </is>
-      </c>
-      <c r="D104" s="6" t="inlineStr">
-        <is>
-          <t>Draw 1 card following each of your passes</t>
-        </is>
-      </c>
-      <c r="E104" s="7" t="n"/>
+      <c r="C104" s="32" t="inlineStr">
+        <is>
+          <t>No Bag</t>
+        </is>
+      </c>
+      <c r="D104" s="33" t="inlineStr">
+        <is>
+          <t>Cannot activate Move cards this round</t>
+        </is>
+      </c>
+      <c r="E104" s="34" t="n"/>
       <c r="F104" s="138" t="n"/>
-      <c r="G104" s="101" t="n"/>
+      <c r="G104" s="113" t="inlineStr">
+        <is>
+          <t>Bad card to draw</t>
+        </is>
+      </c>
       <c r="H104" s="102" t="n"/>
       <c r="I104" s="102" t="n"/>
       <c r="J104" s="102" t="n"/>
@@ -5375,23 +5385,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C105" s="32" t="inlineStr">
-        <is>
-          <t>Shooting Slump</t>
-        </is>
-      </c>
-      <c r="D105" s="33" t="inlineStr">
-        <is>
-          <t>SHOT -20% this round</t>
-        </is>
-      </c>
-      <c r="E105" s="34" t="n"/>
+      <c r="C105" s="31" t="inlineStr">
+        <is>
+          <t>Point God</t>
+        </is>
+      </c>
+      <c r="D105" s="6" t="inlineStr">
+        <is>
+          <t>Draw 1 card following each of your passes</t>
+        </is>
+      </c>
+      <c r="E105" s="7" t="n"/>
       <c r="F105" s="138" t="n"/>
-      <c r="G105" s="113" t="inlineStr">
-        <is>
-          <t>Bad card to draw</t>
-        </is>
-      </c>
+      <c r="G105" s="101" t="n"/>
       <c r="H105" s="102" t="n"/>
       <c r="I105" s="102" t="n"/>
       <c r="J105" s="102" t="n"/>
@@ -5403,19 +5409,23 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C106" s="31" t="inlineStr">
-        <is>
-          <t>Shot Creator</t>
-        </is>
-      </c>
-      <c r="D106" s="6" t="inlineStr">
-        <is>
-          <t>Draw 1 additional card after every draw effect</t>
-        </is>
-      </c>
-      <c r="E106" s="7" t="n"/>
+      <c r="C106" s="32" t="inlineStr">
+        <is>
+          <t>Shooting Slump</t>
+        </is>
+      </c>
+      <c r="D106" s="33" t="inlineStr">
+        <is>
+          <t>SHOT -20% this round</t>
+        </is>
+      </c>
+      <c r="E106" s="34" t="n"/>
       <c r="F106" s="138" t="n"/>
-      <c r="G106" s="101" t="n"/>
+      <c r="G106" s="113" t="inlineStr">
+        <is>
+          <t>Bad card to draw</t>
+        </is>
+      </c>
       <c r="H106" s="102" t="n"/>
       <c r="I106" s="102" t="n"/>
       <c r="J106" s="102" t="n"/>
@@ -5427,19 +5437,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C107" s="32" t="inlineStr">
-        <is>
-          <t>Sixth Man</t>
-        </is>
-      </c>
-      <c r="D107" s="33" t="inlineStr">
-        <is>
-          <t>SHOT = 100% if taking 6th shot of the round</t>
-        </is>
-      </c>
-      <c r="E107" s="34" t="n"/>
+      <c r="C107" s="31" t="inlineStr">
+        <is>
+          <t>Shot Creator</t>
+        </is>
+      </c>
+      <c r="D107" s="6" t="inlineStr">
+        <is>
+          <t>Draw 1 additional card after every draw effect</t>
+        </is>
+      </c>
+      <c r="E107" s="7" t="n"/>
       <c r="F107" s="138" t="n"/>
-      <c r="G107" s="107" t="n"/>
+      <c r="G107" s="101" t="n"/>
       <c r="H107" s="102" t="n"/>
       <c r="I107" s="102" t="n"/>
       <c r="J107" s="102" t="n"/>
@@ -5451,19 +5461,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C108" s="31" t="inlineStr">
-        <is>
-          <t>Sniper</t>
-        </is>
-      </c>
-      <c r="D108" s="6" t="inlineStr">
-        <is>
-          <t>SHOT +10% on all Three-Point Line Shots</t>
-        </is>
-      </c>
-      <c r="E108" s="7" t="n"/>
+      <c r="C108" s="32" t="inlineStr">
+        <is>
+          <t>Sixth Man</t>
+        </is>
+      </c>
+      <c r="D108" s="33" t="inlineStr">
+        <is>
+          <t>SHOT = 100% if taking 6th shot of the round</t>
+        </is>
+      </c>
+      <c r="E108" s="34" t="n"/>
       <c r="F108" s="138" t="n"/>
-      <c r="G108" s="101" t="n"/>
+      <c r="G108" s="107" t="n"/>
       <c r="H108" s="102" t="n"/>
       <c r="I108" s="102" t="n"/>
       <c r="J108" s="102" t="n"/>
@@ -5475,19 +5485,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C109" s="32" t="inlineStr">
-        <is>
-          <t>Splash Cousin</t>
-        </is>
-      </c>
-      <c r="D109" s="33" t="inlineStr">
-        <is>
-          <t>All Three-Point Line Shots: SHOT = 100%</t>
-        </is>
-      </c>
-      <c r="E109" s="34" t="n"/>
+      <c r="C109" s="31" t="inlineStr">
+        <is>
+          <t>Sniper</t>
+        </is>
+      </c>
+      <c r="D109" s="6" t="inlineStr">
+        <is>
+          <t>SHOT +10% on all Three-Point Line Shots</t>
+        </is>
+      </c>
+      <c r="E109" s="7" t="n"/>
       <c r="F109" s="138" t="n"/>
-      <c r="G109" s="107" t="n"/>
+      <c r="G109" s="101" t="n"/>
       <c r="H109" s="102" t="n"/>
       <c r="I109" s="102" t="n"/>
       <c r="J109" s="102" t="n"/>
@@ -5499,19 +5509,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C110" s="31" t="inlineStr">
-        <is>
-          <t>Unguardable</t>
-        </is>
-      </c>
-      <c r="D110" s="91" t="inlineStr">
-        <is>
-          <t>All Clamps on you have no effect on SHOT %</t>
-        </is>
-      </c>
-      <c r="E110" s="7" t="n"/>
+      <c r="C110" s="32" t="inlineStr">
+        <is>
+          <t>Splash Cousin</t>
+        </is>
+      </c>
+      <c r="D110" s="33" t="inlineStr">
+        <is>
+          <t>All Three-Point Line Shots: SHOT = 100%</t>
+        </is>
+      </c>
+      <c r="E110" s="34" t="n"/>
       <c r="F110" s="138" t="n"/>
-      <c r="G110" s="101" t="n"/>
+      <c r="G110" s="107" t="n"/>
       <c r="H110" s="102" t="n"/>
       <c r="I110" s="102" t="n"/>
       <c r="J110" s="102" t="n"/>
@@ -5523,50 +5533,50 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C111" s="32" t="inlineStr">
-        <is>
-          <t>Lethal Shooter</t>
-        </is>
-      </c>
-      <c r="D111" s="33" t="inlineStr">
-        <is>
-          <t>SHOT = 100% on next shot attempt after rebounding your own miss.</t>
-        </is>
-      </c>
-      <c r="E111" s="34" t="n"/>
+      <c r="C111" s="31" t="inlineStr">
+        <is>
+          <t>Unguardable</t>
+        </is>
+      </c>
+      <c r="D111" s="91" t="inlineStr">
+        <is>
+          <t>All Clamps on you have no effect on SHOT %</t>
+        </is>
+      </c>
+      <c r="E111" s="7" t="n"/>
       <c r="F111" s="138" t="n"/>
-      <c r="G111" s="113" t="inlineStr">
-        <is>
-          <t>Special text: “I understand it now”</t>
-        </is>
-      </c>
+      <c r="G111" s="101" t="n"/>
       <c r="H111" s="102" t="n"/>
       <c r="I111" s="102" t="n"/>
       <c r="J111" s="102" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="61" t="n"/>
-      <c r="B112" s="62" t="inlineStr">
+      <c r="A112" s="29" t="n"/>
+      <c r="B112" s="30" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C112" s="66" t="inlineStr">
-        <is>
-          <t>Ball Pounder</t>
-        </is>
-      </c>
-      <c r="D112" s="95" t="inlineStr">
-        <is>
-          <t>All Dribble cards you play draw an additional card but lower SHOT by an additional 10%</t>
-        </is>
-      </c>
-      <c r="E112" s="68" t="n"/>
-      <c r="F112" s="140" t="n"/>
-      <c r="G112" s="126" t="n"/>
-      <c r="H112" s="117" t="n"/>
-      <c r="I112" s="117" t="n"/>
-      <c r="J112" s="117" t="n"/>
+      <c r="C112" s="32" t="inlineStr">
+        <is>
+          <t>Lethal Shooter</t>
+        </is>
+      </c>
+      <c r="D112" s="33" t="inlineStr">
+        <is>
+          <t>SHOT = 100% on next shot attempt after rebounding your own miss.</t>
+        </is>
+      </c>
+      <c r="E112" s="34" t="n"/>
+      <c r="F112" s="138" t="n"/>
+      <c r="G112" s="113" t="inlineStr">
+        <is>
+          <t>Special text: “I understand it now”</t>
+        </is>
+      </c>
+      <c r="H112" s="102" t="n"/>
+      <c r="I112" s="102" t="n"/>
+      <c r="J112" s="102" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="61" t="n"/>
@@ -5577,12 +5587,12 @@
       </c>
       <c r="C113" s="66" t="inlineStr">
         <is>
-          <t>Unselfish</t>
+          <t>Ball Pounder</t>
         </is>
       </c>
       <c r="D113" s="95" t="inlineStr">
         <is>
-          <t>Draw 1 card and increase next SHOT +5% whenever you positively affect another player</t>
+          <t>All Dribble cards you play draw an additional card but lower SHOT by an additional 10%</t>
         </is>
       </c>
       <c r="E113" s="68" t="n"/>
@@ -5601,12 +5611,12 @@
       </c>
       <c r="C114" s="66" t="inlineStr">
         <is>
-          <t>Dirty Player</t>
+          <t>Unselfish</t>
         </is>
       </c>
       <c r="D114" s="95" t="inlineStr">
         <is>
-          <t>When sending Clamps, the clamped player discards 1 if they have any Injuries</t>
+          <t>Draw 1 card and increase next SHOT +5% whenever you positively affect another player</t>
         </is>
       </c>
       <c r="E114" s="68" t="n"/>
@@ -5625,21 +5635,20 @@
       </c>
       <c r="C115" s="66" t="inlineStr">
         <is>
-          <t>Villainous Reputation</t>
+          <t>Dirty Player</t>
         </is>
       </c>
       <c r="D115" s="95" t="inlineStr">
         <is>
-          <t>Discard 1 whenever any Whistle triggers</t>
+          <t>When sending Clamps, the clamped player discards 1 if they have any Injuries</t>
         </is>
       </c>
       <c r="E115" s="68" t="n"/>
       <c r="F115" s="140" t="n"/>
-      <c r="G115" s="126" t="inlineStr">
-        <is>
-          <t>Discarded during play, it attaches to a random player — possibly you again</t>
-        </is>
-      </c>
+      <c r="G115" s="126" t="n"/>
+      <c r="H115" s="117" t="n"/>
+      <c r="I115" s="117" t="n"/>
+      <c r="J115" s="117" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="61" t="n"/>
@@ -5650,19 +5659,19 @@
       </c>
       <c r="C116" s="66" t="inlineStr">
         <is>
-          <t>Free Agent</t>
+          <t>Villainous Reputation</t>
         </is>
       </c>
       <c r="D116" s="95" t="inlineStr">
         <is>
-          <t>Discard your hand. Play a card at random from a player of your choosing (they keep it)</t>
+          <t>Discard 1 whenever any Whistle triggers</t>
         </is>
       </c>
       <c r="E116" s="68" t="n"/>
       <c r="F116" s="140" t="n"/>
       <c r="G116" s="126" t="inlineStr">
         <is>
-          <t>The discard waits for the draw chain to finish. Target is shuffled first and is affected by Floor General. Your own draws are kept. All-0 rebounds are yours; otherwise you cannot bid</t>
+          <t>Discarded during play, it attaches to a random player — possibly you again</t>
         </is>
       </c>
     </row>
@@ -5675,23 +5684,48 @@
       </c>
       <c r="C117" s="66" t="inlineStr">
         <is>
-          <t>Franchise Player</t>
+          <t>Free Agent</t>
         </is>
       </c>
       <c r="D117" s="95" t="inlineStr">
         <is>
-          <t>When passing, choose 1 of the new player's Intangibles or a card in their hand for them to discard</t>
+          <t>Discard your hand. Play a card at random from a player of your choosing (they keep it)</t>
         </is>
       </c>
       <c r="E117" s="68" t="n"/>
       <c r="F117" s="140" t="n"/>
-      <c r="G117" s="126" t="n"/>
-      <c r="H117" s="117" t="n"/>
-      <c r="I117" s="117" t="n"/>
-      <c r="J117" s="117" t="n"/>
+      <c r="G117" s="126" t="inlineStr">
+        <is>
+          <t>The discard waits for the draw chain to finish. Target is shuffled first and is affected by Floor General. Your own draws are kept. All-0 rebounds are yours; otherwise you cannot bid</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="61" t="n"/>
+      <c r="B118" s="62" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C118" s="66" t="inlineStr">
+        <is>
+          <t>Franchise Player</t>
+        </is>
+      </c>
+      <c r="D118" s="95" t="inlineStr">
+        <is>
+          <t>When passing, choose 1 of the new player's Intangibles or a card in their hand for them to discard</t>
+        </is>
+      </c>
+      <c r="E118" s="68" t="n"/>
+      <c r="F118" s="140" t="n"/>
+      <c r="G118" s="126" t="n"/>
+      <c r="H118" s="117" t="n"/>
+      <c r="I118" s="117" t="n"/>
+      <c r="J118" s="117" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="104">
+  <mergeCells count="105">
     <mergeCell ref="G55:J55"/>
     <mergeCell ref="G4:J4"/>
     <mergeCell ref="G109:J109"/>
@@ -5701,11 +5735,11 @@
     <mergeCell ref="G40:J40"/>
     <mergeCell ref="G111:J111"/>
     <mergeCell ref="G72:J72"/>
-    <mergeCell ref="G81:J81"/>
     <mergeCell ref="G96:J96"/>
     <mergeCell ref="G5:J5"/>
     <mergeCell ref="G71:J71"/>
     <mergeCell ref="G8:J8"/>
+    <mergeCell ref="G82:J82"/>
     <mergeCell ref="G57:J57"/>
     <mergeCell ref="G10:J10"/>
     <mergeCell ref="G66:J66"/>
@@ -5725,15 +5759,12 @@
     <mergeCell ref="G100:J100"/>
     <mergeCell ref="G94:J94"/>
     <mergeCell ref="G75:J75"/>
-    <mergeCell ref="G44:J44"/>
     <mergeCell ref="G22:J22"/>
-    <mergeCell ref="G84:J84"/>
     <mergeCell ref="G31:J31"/>
     <mergeCell ref="G102:J102"/>
     <mergeCell ref="G12:J12"/>
-    <mergeCell ref="G77:J77"/>
+    <mergeCell ref="G86:J86"/>
     <mergeCell ref="G21:J21"/>
-    <mergeCell ref="G86:J86"/>
     <mergeCell ref="G67:J67"/>
     <mergeCell ref="G61:J61"/>
     <mergeCell ref="G70:J70"/>
@@ -5752,13 +5783,14 @@
     <mergeCell ref="G26:J26"/>
     <mergeCell ref="G35:J35"/>
     <mergeCell ref="G16:J16"/>
+    <mergeCell ref="G76:J76"/>
     <mergeCell ref="G90:J90"/>
     <mergeCell ref="G99:J99"/>
     <mergeCell ref="G60:J60"/>
     <mergeCell ref="G9:J9"/>
     <mergeCell ref="G59:J59"/>
+    <mergeCell ref="G115:J115"/>
     <mergeCell ref="G11:J11"/>
-    <mergeCell ref="G117:J117"/>
     <mergeCell ref="G39:J39"/>
     <mergeCell ref="G101:J101"/>
     <mergeCell ref="G103:J103"/>
@@ -5766,8 +5798,11 @@
     <mergeCell ref="G37:J37"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G13:J13"/>
+    <mergeCell ref="G78:J78"/>
+    <mergeCell ref="G118:J118"/>
     <mergeCell ref="G87:J87"/>
     <mergeCell ref="G15:J15"/>
+    <mergeCell ref="G44:J44"/>
     <mergeCell ref="G95:J95"/>
     <mergeCell ref="G89:J89"/>
     <mergeCell ref="G64:J64"/>
@@ -5785,9 +5820,9 @@
     <mergeCell ref="G52:J52"/>
     <mergeCell ref="G27:J27"/>
     <mergeCell ref="G98:J98"/>
+    <mergeCell ref="G42:J42"/>
     <mergeCell ref="G107:J107"/>
     <mergeCell ref="G36:J36"/>
-    <mergeCell ref="G42:J42"/>
     <mergeCell ref="G17:J17"/>
     <mergeCell ref="G19:J19"/>
     <mergeCell ref="G28:J28"/>

</xml_diff>

<commit_message>
Clear Out, Touch Pass and six Game Breaks
Clear Out is playable as your first action only, the way Touch Pass only
pays as one. A pass thrown to a side goes past the man who cleared out; one
that named him is a turnover and the end of the round.

Ending a round now drops the orders still in flight with it. Alley-Oop's
forced shot was surviving the round it was ordered in and going up inside
halftime's deal, which ran the round counter twice.

New Game Breaks: Altercation and Huge Altercation, Home Court Advantage and
Away Game, Mic'd Up and In The Zone. Mic'd Up is SHOT the holder carries
himself rather than SHOT on the ball, so a pass leaves it behind.

Sheet rows for all eight, and the cuts suite is on the TODO.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -2549,7 +2549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J123"/>
+  <dimension ref="A1:J131"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="22.25" customHeight="1"/>
   <cols>
     <col width="15.5" customWidth="1" style="8" min="1" max="1"/>
@@ -2626,41 +2626,40 @@
         </is>
       </c>
       <c r="B2" s="12">
-        <f>COUNTIF($B$5:$B$123,"Pass")</f>
+        <f>COUNTIF($B$5:$B$131,"Pass")</f>
         <v/>
       </c>
       <c r="C2" s="13">
-        <f>COUNTIF($B$5:$B$123,"Move")+COUNTIF($B$5:$B$123,"Special Move")</f>
+        <f>COUNTIF($B$5:$B$131,"Move")+COUNTIF($B$5:$B$131,"Special Move")</f>
         <v/>
       </c>
       <c r="D2" s="14">
-        <f>COUNTIF($B$5:$B$123,"Clamp")</f>
+        <f>COUNTIF($B$5:$B$131,"Clamp")</f>
         <v/>
       </c>
       <c r="E2" s="15">
-        <f>COUNTIF($B$5:$B$123,"Whistle")</f>
+        <f>COUNTIF($B$5:$B$131,"Whistle")</f>
         <v/>
       </c>
       <c r="F2" s="16">
-        <f>COUNTIF($B$5:$B$123,"Game Break")</f>
+        <f>COUNTIF($B$5:$B$131,"Game Break")</f>
         <v/>
       </c>
       <c r="G2" s="18">
-        <f>COUNTIF($B$5:$B$123,"Injury GB")</f>
+        <f>COUNTIF($B$5:$B$131,"Injury GB")</f>
         <v/>
       </c>
       <c r="H2" s="19">
-        <f>COUNTIF($B$5:$B$123,"Devastating Injury GB")</f>
+        <f>COUNTIF($B$5:$B$131,"Devastating Injury GB")</f>
         <v/>
       </c>
       <c r="I2" s="17">
-        <f>COUNTIF($B$5:$B$123,"Intangible")</f>
+        <f>COUNTIF($B$5:$B$131,"Intangible")</f>
         <v/>
       </c>
       <c r="J2" s="19" t="n"/>
     </row>
-    <row r="3"/>
-    <row r="4" ht="20.75" customHeight="1" s="132" thickBot="1">
+    <row r="4" ht="20.75" customHeight="1" s="132">
       <c r="A4" s="123" t="inlineStr">
         <is>
           <t>Type</t>
@@ -2703,7 +2702,7 @@
         </is>
       </c>
       <c r="B5" s="22">
-        <f>COUNTIF($B$5:$B$123,"Pass")</f>
+        <f>COUNTIF($B$5:$B$131,"Pass")</f>
         <v/>
       </c>
       <c r="C5" s="23" t="n"/>
@@ -2923,7 +2922,7 @@
       <c r="I13" s="106" t="n"/>
       <c r="J13" s="106" t="n"/>
     </row>
-    <row r="14" ht="29" customHeight="1" s="132" thickBot="1">
+    <row r="14" ht="29" customHeight="1" s="132">
       <c r="A14" s="35" t="n"/>
       <c r="B14" s="36" t="inlineStr">
         <is>
@@ -3111,80 +3110,76 @@
       <c r="I19" s="104" t="n"/>
       <c r="J19" s="104" t="n"/>
     </row>
-    <row r="20" ht="14" customHeight="1" s="132">
-      <c r="A20" s="39" t="inlineStr">
+    <row r="20" ht="56" customHeight="1" s="132">
+      <c r="A20" s="35" t="n"/>
+      <c r="B20" s="36" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="C20" s="37" t="inlineStr">
+        <is>
+          <t>Touch Pass</t>
+        </is>
+      </c>
+      <c r="D20" s="38" t="inlineStr">
+        <is>
+          <t>SHOT +5%. Pass to player of choice. If played as first action, draw 2 cards</t>
+        </is>
+      </c>
+      <c r="E20" s="38" t="n"/>
+      <c r="F20" s="77" t="n">
+        <v>5</v>
+      </c>
+      <c r="G20" s="127" t="n"/>
+      <c r="H20" s="104" t="n"/>
+      <c r="I20" s="104" t="n"/>
+      <c r="J20" s="104" t="n"/>
+    </row>
+    <row r="21" ht="14" customHeight="1" s="132">
+      <c r="A21" s="39" t="inlineStr">
         <is>
           <t>Move</t>
         </is>
       </c>
-      <c r="B20" s="40">
-        <f>COUNTIF($B$5:$B$123,"Move")+COUNTIF($B$5:$B$123,"Special Move")</f>
+      <c r="B21" s="40">
+        <f>COUNTIF($B$5:$B$131,"Move")+COUNTIF($B$5:$B$131,"Special Move")</f>
         <v/>
       </c>
-      <c r="C20" s="41" t="n"/>
-      <c r="D20" s="41" t="n"/>
-      <c r="E20" s="41" t="n"/>
-      <c r="F20" s="78" t="n"/>
-      <c r="G20" s="120" t="n"/>
-      <c r="H20" s="121" t="n"/>
-      <c r="I20" s="121" t="n"/>
-      <c r="J20" s="121" t="n"/>
-    </row>
-    <row r="21" ht="28" customHeight="1" s="132">
-      <c r="A21" s="45" t="n"/>
-      <c r="B21" s="46" t="inlineStr">
+      <c r="C21" s="41" t="n"/>
+      <c r="D21" s="41" t="n"/>
+      <c r="E21" s="41" t="n"/>
+      <c r="F21" s="78" t="n"/>
+      <c r="G21" s="120" t="n"/>
+      <c r="H21" s="121" t="n"/>
+      <c r="I21" s="121" t="n"/>
+      <c r="J21" s="121" t="n"/>
+    </row>
+    <row r="22" ht="28" customHeight="1" s="132">
+      <c r="A22" s="45" t="n"/>
+      <c r="B22" s="46" t="inlineStr">
         <is>
           <t>Move</t>
         </is>
       </c>
-      <c r="C21" s="47" t="inlineStr">
+      <c r="C22" s="47" t="inlineStr">
         <is>
           <t>Dribble</t>
         </is>
       </c>
-      <c r="D21" s="48" t="inlineStr">
+      <c r="D22" s="48" t="inlineStr">
         <is>
           <t>Draw 1 card. SHOT -10%</t>
         </is>
       </c>
-      <c r="E21" s="49" t="n"/>
-      <c r="F21" s="79" t="n">
+      <c r="E22" s="49" t="n"/>
+      <c r="F22" s="79" t="n">
         <v>15</v>
       </c>
-      <c r="G21" s="118" t="n"/>
-      <c r="H21" s="119" t="n"/>
-      <c r="I21" s="119" t="n"/>
-      <c r="J21" s="119" t="n"/>
-    </row>
-    <row r="22" ht="28" customHeight="1" s="132">
-      <c r="A22" s="29" t="n"/>
-      <c r="B22" s="30" t="inlineStr">
-        <is>
-          <t>Move</t>
-        </is>
-      </c>
-      <c r="C22" s="31" t="inlineStr">
-        <is>
-          <t>Drive</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>SHOT +10%</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>Following Dribble: SHOT +10%</t>
-        </is>
-      </c>
-      <c r="F22" s="74" t="n">
-        <v>7</v>
-      </c>
-      <c r="G22" s="101" t="n"/>
-      <c r="H22" s="102" t="n"/>
-      <c r="I22" s="102" t="n"/>
-      <c r="J22" s="102" t="n"/>
+      <c r="G22" s="118" t="n"/>
+      <c r="H22" s="119" t="n"/>
+      <c r="I22" s="119" t="n"/>
+      <c r="J22" s="119" t="n"/>
     </row>
     <row r="23" ht="28" customHeight="1" s="132">
       <c r="A23" s="29" t="n"/>
@@ -3193,21 +3188,25 @@
           <t>Move</t>
         </is>
       </c>
-      <c r="C23" s="32" t="inlineStr">
-        <is>
-          <t>Ankle Breaker</t>
-        </is>
-      </c>
-      <c r="D23" s="33" t="inlineStr">
-        <is>
-          <t>Target player discards 1 card. SHOT +10%</t>
-        </is>
-      </c>
-      <c r="E23" s="34" t="n"/>
-      <c r="F23" s="75" t="n">
-        <v>10</v>
-      </c>
-      <c r="G23" s="107" t="n"/>
+      <c r="C23" s="31" t="inlineStr">
+        <is>
+          <t>Drive</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>SHOT +10%</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Following Dribble: SHOT +10%</t>
+        </is>
+      </c>
+      <c r="F23" s="74" t="n">
+        <v>7</v>
+      </c>
+      <c r="G23" s="101" t="n"/>
       <c r="H23" s="102" t="n"/>
       <c r="I23" s="102" t="n"/>
       <c r="J23" s="102" t="n"/>
@@ -3219,25 +3218,21 @@
           <t>Move</t>
         </is>
       </c>
-      <c r="C24" s="90" t="inlineStr">
-        <is>
-          <t>Flop</t>
-        </is>
-      </c>
-      <c r="D24" s="91" t="inlineStr">
-        <is>
-          <t>Cancel Clamps. Take 1 FT for each. If no Clamps on you, TOV +1</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="n"/>
-      <c r="F24" s="76" t="n">
-        <v>5</v>
-      </c>
-      <c r="G24" s="130" t="inlineStr">
-        <is>
-          <t>Take 1 FT attempt for each Clamp on you and cancel it. If no Clamps on you, TOV +1</t>
-        </is>
-      </c>
+      <c r="C24" s="32" t="inlineStr">
+        <is>
+          <t>Ankle Breaker</t>
+        </is>
+      </c>
+      <c r="D24" s="33" t="inlineStr">
+        <is>
+          <t>Target player discards 1 card. SHOT +10%</t>
+        </is>
+      </c>
+      <c r="E24" s="34" t="n"/>
+      <c r="F24" s="75" t="n">
+        <v>10</v>
+      </c>
+      <c r="G24" s="107" t="n"/>
       <c r="H24" s="102" t="n"/>
       <c r="I24" s="102" t="n"/>
       <c r="J24" s="102" t="n"/>
@@ -3249,100 +3244,104 @@
           <t>Move</t>
         </is>
       </c>
-      <c r="C25" s="32" t="inlineStr">
-        <is>
-          <t>Hesi</t>
-        </is>
-      </c>
-      <c r="D25" s="33" t="inlineStr">
-        <is>
-          <t>SHOT +10%</t>
-        </is>
-      </c>
-      <c r="E25" s="33" t="inlineStr">
-        <is>
-          <t>Shot Clock -1</t>
-        </is>
-      </c>
-      <c r="F25" s="80" t="n">
-        <v>15</v>
-      </c>
-      <c r="G25" s="107" t="n"/>
+      <c r="C25" s="90" t="inlineStr">
+        <is>
+          <t>Flop</t>
+        </is>
+      </c>
+      <c r="D25" s="91" t="inlineStr">
+        <is>
+          <t>Cancel Clamps. Take 1 FT for each. If no Clamps on you, TOV +1</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="n"/>
+      <c r="F25" s="76" t="n">
+        <v>5</v>
+      </c>
+      <c r="G25" s="130" t="inlineStr">
+        <is>
+          <t>Take 1 FT attempt for each Clamp on you and cancel it. If no Clamps on you, TOV +1</t>
+        </is>
+      </c>
       <c r="H25" s="102" t="n"/>
       <c r="I25" s="102" t="n"/>
       <c r="J25" s="102" t="n"/>
     </row>
-    <row r="26" ht="14" customHeight="1" s="132">
+    <row r="26" ht="28" customHeight="1" s="132">
       <c r="A26" s="29" t="n"/>
       <c r="B26" s="30" t="inlineStr">
         <is>
           <t>Move</t>
         </is>
       </c>
-      <c r="C26" s="31" t="inlineStr">
-        <is>
-          <t>Pump Fake</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="C26" s="32" t="inlineStr">
+        <is>
+          <t>Hesi</t>
+        </is>
+      </c>
+      <c r="D26" s="33" t="inlineStr">
         <is>
           <t>SHOT +10%</t>
         </is>
       </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>Cancel all Clamps on you</t>
-        </is>
-      </c>
-      <c r="F26" s="74" t="n">
-        <v>12</v>
-      </c>
-      <c r="G26" s="101" t="n"/>
+      <c r="E26" s="33" t="inlineStr">
+        <is>
+          <t>Shot Clock -1</t>
+        </is>
+      </c>
+      <c r="F26" s="80" t="n">
+        <v>15</v>
+      </c>
+      <c r="G26" s="107" t="n"/>
       <c r="H26" s="102" t="n"/>
       <c r="I26" s="102" t="n"/>
       <c r="J26" s="102" t="n"/>
     </row>
-    <row r="27" ht="71" customHeight="1" s="132" thickBot="1">
+    <row r="27" ht="14" customHeight="1" s="132">
       <c r="A27" s="29" t="n"/>
       <c r="B27" s="30" t="inlineStr">
         <is>
           <t>Move</t>
         </is>
       </c>
-      <c r="C27" s="32" t="inlineStr">
-        <is>
-          <t>Rhythm Dribble</t>
-        </is>
-      </c>
-      <c r="D27" s="33" t="inlineStr">
-        <is>
-          <t>Draw 1 card. SHOT +10%. Shot Clock -1</t>
-        </is>
-      </c>
-      <c r="E27" s="34" t="n"/>
-      <c r="F27" s="75" t="n">
-        <v>5</v>
-      </c>
-      <c r="G27" s="107" t="n"/>
+      <c r="C27" s="31" t="inlineStr">
+        <is>
+          <t>Pump Fake</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>SHOT +10%</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>Cancel all Clamps on you</t>
+        </is>
+      </c>
+      <c r="F27" s="74" t="n">
+        <v>12</v>
+      </c>
+      <c r="G27" s="101" t="n"/>
       <c r="H27" s="102" t="n"/>
       <c r="I27" s="102" t="n"/>
       <c r="J27" s="102" t="n"/>
     </row>
-    <row r="28" ht="20" customHeight="1" s="132">
+    <row r="28" ht="71" customHeight="1" s="132">
       <c r="A28" s="29" t="n"/>
       <c r="B28" s="30" t="inlineStr">
         <is>
           <t>Move</t>
         </is>
       </c>
-      <c r="C28" s="133" t="inlineStr">
-        <is>
-          <t>Pound Dribble</t>
-        </is>
-      </c>
-      <c r="D28" s="94" t="inlineStr">
-        <is>
-          <t>Draw 2 cards then Discard 1. SHOT +10% Shot Clock -1</t>
+      <c r="C28" s="32" t="inlineStr">
+        <is>
+          <t>Rhythm Dribble</t>
+        </is>
+      </c>
+      <c r="D28" s="33" t="inlineStr">
+        <is>
+          <t>Draw 1 card. SHOT +10%. Shot Clock -1</t>
         </is>
       </c>
       <c r="E28" s="34" t="n"/>
@@ -3354,7 +3353,7 @@
       <c r="I28" s="102" t="n"/>
       <c r="J28" s="102" t="n"/>
     </row>
-    <row r="29" ht="42" customHeight="1" s="132">
+    <row r="29" ht="20" customHeight="1" s="132">
       <c r="A29" s="29" t="n"/>
       <c r="B29" s="30" t="inlineStr">
         <is>
@@ -3363,28 +3362,24 @@
       </c>
       <c r="C29" s="133" t="inlineStr">
         <is>
-          <t>Spin Move</t>
+          <t>Pound Dribble</t>
         </is>
       </c>
       <c r="D29" s="94" t="inlineStr">
         <is>
-          <t>SHOT + 10%. If being Clamped, discard all Clamps and gain additional SHOT +10% for each</t>
+          <t>Draw 2 cards then Discard 1. SHOT +10% Shot Clock -1</t>
         </is>
       </c>
       <c r="E29" s="34" t="n"/>
       <c r="F29" s="75" t="n">
-        <v>10</v>
-      </c>
-      <c r="G29" s="125" t="inlineStr">
-        <is>
-          <t>isDribble = true</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="G29" s="107" t="n"/>
       <c r="H29" s="102" t="n"/>
       <c r="I29" s="102" t="n"/>
       <c r="J29" s="102" t="n"/>
     </row>
-    <row r="30" ht="14" customHeight="1" s="132">
+    <row r="30" ht="42" customHeight="1" s="132">
       <c r="A30" s="29" t="n"/>
       <c r="B30" s="30" t="inlineStr">
         <is>
@@ -3393,17 +3388,17 @@
       </c>
       <c r="C30" s="133" t="inlineStr">
         <is>
-          <t>Crossover</t>
+          <t>Spin Move</t>
         </is>
       </c>
       <c r="D30" s="94" t="inlineStr">
         <is>
-          <t>Draw 1 Card. SHOT +10%. If being Clamped, discard all clamps and Draw 1 card and Clamp-sender discards 1card for each</t>
+          <t>SHOT + 10%. If being Clamped, discard all Clamps and gain additional SHOT +10% for each</t>
         </is>
       </c>
       <c r="E30" s="34" t="n"/>
       <c r="F30" s="75" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G30" s="125" t="inlineStr">
         <is>
@@ -3414,53 +3409,83 @@
       <c r="I30" s="102" t="n"/>
       <c r="J30" s="102" t="n"/>
     </row>
-    <row r="31" ht="28" customHeight="1" s="132">
+    <row r="31" ht="14" customHeight="1" s="132">
       <c r="A31" s="29" t="n"/>
       <c r="B31" s="30" t="inlineStr">
         <is>
           <t>Move</t>
         </is>
       </c>
-      <c r="C31" s="31" t="inlineStr">
-        <is>
-          <t>Stepback</t>
-        </is>
-      </c>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>SHOT +10%</t>
-        </is>
-      </c>
-      <c r="E31" s="6" t="inlineStr">
-        <is>
-          <t>Discard 1: SHOT +10%</t>
-        </is>
-      </c>
-      <c r="F31" s="74" t="n">
-        <v>12</v>
-      </c>
-      <c r="G31" s="101" t="inlineStr">
-        <is>
-          <t>The discard is an optional prompt.</t>
+      <c r="C31" s="133" t="inlineStr">
+        <is>
+          <t>Crossover</t>
+        </is>
+      </c>
+      <c r="D31" s="94" t="inlineStr">
+        <is>
+          <t>Draw 1 Card. SHOT +10%. If being Clamped, discard all clamps and Draw 1 card and Clamp-sender discards 1card for each</t>
+        </is>
+      </c>
+      <c r="E31" s="34" t="n"/>
+      <c r="F31" s="75" t="n">
+        <v>5</v>
+      </c>
+      <c r="G31" s="125" t="inlineStr">
+        <is>
+          <t>isDribble = true</t>
         </is>
       </c>
       <c r="H31" s="102" t="n"/>
       <c r="I31" s="102" t="n"/>
       <c r="J31" s="102" t="n"/>
     </row>
-    <row r="32" ht="14" customHeight="1" s="132">
-      <c r="A32" s="61" t="n"/>
-      <c r="B32" s="62" t="inlineStr">
+    <row r="32" ht="28" customHeight="1" s="132">
+      <c r="A32" s="29" t="n"/>
+      <c r="B32" s="30" t="inlineStr">
         <is>
           <t>Move</t>
         </is>
       </c>
-      <c r="C32" s="63" t="inlineStr">
+      <c r="C32" s="31" t="inlineStr">
+        <is>
+          <t>Stepback</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>SHOT +10%</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>Discard 1: SHOT +10%</t>
+        </is>
+      </c>
+      <c r="F32" s="74" t="n">
+        <v>12</v>
+      </c>
+      <c r="G32" s="101" t="inlineStr">
+        <is>
+          <t>The discard is an optional prompt.</t>
+        </is>
+      </c>
+      <c r="H32" s="102" t="n"/>
+      <c r="I32" s="102" t="n"/>
+      <c r="J32" s="102" t="n"/>
+    </row>
+    <row r="33" ht="14" customHeight="1" s="132">
+      <c r="A33" s="61" t="n"/>
+      <c r="B33" s="62" t="inlineStr">
+        <is>
+          <t>Move</t>
+        </is>
+      </c>
+      <c r="C33" s="63" t="inlineStr">
         <is>
           <t>Triple Threat</t>
         </is>
       </c>
-      <c r="D32" s="64" t="inlineStr">
+      <c r="D33" s="64" t="inlineStr">
         <is>
           <t>Choose 1:
 Draw 1 card
@@ -3468,131 +3493,93 @@
 SHOT +10%</t>
         </is>
       </c>
-      <c r="E32" s="64" t="inlineStr">
+      <c r="E33" s="64" t="inlineStr">
         <is>
           <t>Cannot use further Move cards</t>
         </is>
       </c>
-      <c r="F32" s="81" t="n">
+      <c r="F33" s="81" t="n">
         <v>15</v>
       </c>
-      <c r="G32" s="116" t="inlineStr">
+      <c r="G33" s="116" t="inlineStr">
         <is>
           <t>Cannot use further Move cards applies to that possession only.</t>
         </is>
       </c>
-      <c r="H32" s="117" t="n"/>
-      <c r="I32" s="117" t="n"/>
-      <c r="J32" s="117" t="n"/>
-    </row>
-    <row r="33" ht="28" customHeight="1" s="132">
-      <c r="A33" s="42" t="inlineStr">
+      <c r="H33" s="117" t="n"/>
+      <c r="I33" s="117" t="n"/>
+      <c r="J33" s="117" t="n"/>
+    </row>
+    <row r="34" ht="14" customHeight="1" s="132">
+      <c r="A34" s="61" t="n"/>
+      <c r="B34" s="62" t="inlineStr">
+        <is>
+          <t>Move</t>
+        </is>
+      </c>
+      <c r="C34" s="63" t="inlineStr">
+        <is>
+          <t>Clear Out</t>
+        </is>
+      </c>
+      <c r="D34" s="64" t="inlineStr">
+        <is>
+          <t>First action only. The next pass to a side goes past you. One that named you is a TOV and ends the round</t>
+        </is>
+      </c>
+      <c r="E34" s="64" t="n"/>
+      <c r="F34" s="81" t="n">
+        <v>8</v>
+      </c>
+      <c r="G34" s="116" t="n"/>
+      <c r="H34" s="117" t="n"/>
+      <c r="I34" s="117" t="n"/>
+      <c r="J34" s="117" t="n"/>
+    </row>
+    <row r="35" ht="28" customHeight="1" s="132">
+      <c r="A35" s="42" t="inlineStr">
         <is>
           <t>Special Move</t>
         </is>
       </c>
-      <c r="B33" s="43">
-        <f>COUNTIF($B$5:$B$123,"Special Move")</f>
+      <c r="B35" s="43">
+        <f>COUNTIF($B$5:$B$131,"Special Move")</f>
         <v/>
       </c>
-      <c r="C33" s="44" t="n"/>
-      <c r="D33" s="44" t="n"/>
-      <c r="E33" s="44" t="n"/>
-      <c r="F33" s="82" t="n"/>
-      <c r="G33" s="120" t="n"/>
-      <c r="H33" s="121" t="n"/>
-      <c r="I33" s="121" t="n"/>
-      <c r="J33" s="121" t="n"/>
-    </row>
-    <row r="34" ht="28" customHeight="1" s="132">
-      <c r="A34" s="24" t="n"/>
-      <c r="B34" s="25" t="inlineStr">
+      <c r="C35" s="44" t="n"/>
+      <c r="D35" s="44" t="n"/>
+      <c r="E35" s="44" t="n"/>
+      <c r="F35" s="82" t="n"/>
+      <c r="G35" s="120" t="n"/>
+      <c r="H35" s="121" t="n"/>
+      <c r="I35" s="121" t="n"/>
+      <c r="J35" s="121" t="n"/>
+    </row>
+    <row r="36" ht="28" customHeight="1" s="132">
+      <c r="A36" s="24" t="n"/>
+      <c r="B36" s="25" t="inlineStr">
         <is>
           <t>Special Move</t>
         </is>
       </c>
-      <c r="C34" s="26" t="inlineStr">
+      <c r="C36" s="26" t="inlineStr">
         <is>
           <t>Bankshot</t>
         </is>
       </c>
-      <c r="D34" s="27" t="inlineStr">
+      <c r="D36" s="27" t="inlineStr">
         <is>
           <t>Flip a coin:
 Heads: SHOT +10%
 Tails: SHOT -10%</t>
         </is>
       </c>
-      <c r="E34" s="27" t="inlineStr">
+      <c r="E36" s="27" t="inlineStr">
         <is>
           <t>Shoot the ball</t>
         </is>
       </c>
-      <c r="F34" s="83" t="n">
-        <v>4</v>
-      </c>
-      <c r="G34" s="105" t="n"/>
-      <c r="H34" s="106" t="n"/>
-      <c r="I34" s="106" t="n"/>
-      <c r="J34" s="106" t="n"/>
-    </row>
-    <row r="35" ht="28" customHeight="1" s="132">
-      <c r="A35" s="29" t="n"/>
-      <c r="B35" s="30" t="inlineStr">
-        <is>
-          <t>Special Move</t>
-        </is>
-      </c>
-      <c r="C35" s="31" t="inlineStr">
-        <is>
-          <t>Buzzer Beater</t>
-        </is>
-      </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>SHOT = 100%</t>
-        </is>
-      </c>
-      <c r="E35" s="6" t="inlineStr">
-        <is>
-          <t>Shoot the ball</t>
-        </is>
-      </c>
-      <c r="F35" s="74" t="n">
-        <v>4</v>
-      </c>
-      <c r="G35" s="128" t="inlineStr">
-        <is>
-          <t>Can only play with Shot Clock at 1</t>
-        </is>
-      </c>
-      <c r="H35" s="106" t="n"/>
-      <c r="I35" s="106" t="n"/>
-      <c r="J35" s="106" t="n"/>
-    </row>
-    <row r="36" ht="42" customHeight="1" s="132">
-      <c r="A36" s="29" t="n"/>
-      <c r="B36" s="30" t="inlineStr">
-        <is>
-          <t>Special Move</t>
-        </is>
-      </c>
-      <c r="C36" s="32" t="inlineStr">
-        <is>
-          <t>Dagger Three</t>
-        </is>
-      </c>
-      <c r="D36" s="94" t="inlineStr">
-        <is>
-          <t>[SHOT + 30% at 01 Shot Clock, +20% at 02, +10% at 03, +0% at 04, -10% at 05, etc.]</t>
-        </is>
-      </c>
-      <c r="E36" s="33" t="inlineStr">
-        <is>
-          <t>Shoot the ball. +1 Point on make</t>
-        </is>
-      </c>
-      <c r="F36" s="80" t="n">
+      <c r="F36" s="83" t="n">
         <v>4</v>
       </c>
       <c r="G36" s="105" t="n"/>
@@ -3609,28 +3596,32 @@
       </c>
       <c r="C37" s="31" t="inlineStr">
         <is>
-          <t>Fadeaway</t>
+          <t>Buzzer Beater</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>SHOT -10%. Draw 1 card</t>
+          <t>SHOT = 100%</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Shoot the ball.</t>
+          <t>Shoot the ball</t>
         </is>
       </c>
       <c r="F37" s="74" t="n">
-        <v>10</v>
-      </c>
-      <c r="G37" s="112" t="n"/>
+        <v>4</v>
+      </c>
+      <c r="G37" s="128" t="inlineStr">
+        <is>
+          <t>Can only play with Shot Clock at 1</t>
+        </is>
+      </c>
       <c r="H37" s="106" t="n"/>
       <c r="I37" s="106" t="n"/>
       <c r="J37" s="106" t="n"/>
     </row>
-    <row r="38" ht="28" customHeight="1" s="132">
+    <row r="38" ht="42" customHeight="1" s="132">
       <c r="A38" s="29" t="n"/>
       <c r="B38" s="30" t="inlineStr">
         <is>
@@ -3639,12 +3630,12 @@
       </c>
       <c r="C38" s="32" t="inlineStr">
         <is>
-          <t>From the Hash</t>
+          <t>Dagger Three</t>
         </is>
       </c>
       <c r="D38" s="94" t="inlineStr">
         <is>
-          <t>SHOT -20%</t>
+          <t>[SHOT + 30% at 01 Shot Clock, +20% at 02, +10% at 03, +0% at 04, -10% at 05, etc.]</t>
         </is>
       </c>
       <c r="E38" s="33" t="inlineStr">
@@ -3653,14 +3644,14 @@
         </is>
       </c>
       <c r="F38" s="80" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G38" s="105" t="n"/>
       <c r="H38" s="106" t="n"/>
       <c r="I38" s="106" t="n"/>
       <c r="J38" s="106" t="n"/>
     </row>
-    <row r="39" ht="42" customHeight="1" s="132">
+    <row r="39" ht="28" customHeight="1" s="132">
       <c r="A39" s="29" t="n"/>
       <c r="B39" s="30" t="inlineStr">
         <is>
@@ -3669,28 +3660,28 @@
       </c>
       <c r="C39" s="31" t="inlineStr">
         <is>
-          <t>From the Logo</t>
-        </is>
-      </c>
-      <c r="D39" s="91" t="inlineStr">
-        <is>
-          <t>SHOT -30%</t>
+          <t>Fadeaway</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>SHOT -10%. Draw 1 card</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>Shoot the ball. +1 Point on make</t>
+          <t>Shoot the ball.</t>
         </is>
       </c>
       <c r="F39" s="74" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G39" s="112" t="n"/>
       <c r="H39" s="106" t="n"/>
       <c r="I39" s="106" t="n"/>
       <c r="J39" s="106" t="n"/>
     </row>
-    <row r="40" ht="57" customHeight="1" s="132" thickBot="1">
+    <row r="40" ht="28" customHeight="1" s="132">
       <c r="A40" s="29" t="n"/>
       <c r="B40" s="30" t="inlineStr">
         <is>
@@ -3699,12 +3690,12 @@
       </c>
       <c r="C40" s="32" t="inlineStr">
         <is>
-          <t>Full-Court Heave</t>
-        </is>
-      </c>
-      <c r="D40" s="33" t="inlineStr">
-        <is>
-          <t>SHOT = 10%</t>
+          <t>From the Hash</t>
+        </is>
+      </c>
+      <c r="D40" s="94" t="inlineStr">
+        <is>
+          <t>SHOT -20%</t>
         </is>
       </c>
       <c r="E40" s="33" t="inlineStr">
@@ -3720,7 +3711,7 @@
       <c r="I40" s="106" t="n"/>
       <c r="J40" s="106" t="n"/>
     </row>
-    <row r="41" ht="20" customHeight="1" s="132">
+    <row r="41" ht="42" customHeight="1" s="132">
       <c r="A41" s="29" t="n"/>
       <c r="B41" s="30" t="inlineStr">
         <is>
@@ -3729,17 +3720,17 @@
       </c>
       <c r="C41" s="31" t="inlineStr">
         <is>
-          <t>Putback Tip</t>
-        </is>
-      </c>
-      <c r="D41" s="6" t="inlineStr">
-        <is>
-          <t>SHOT +10%</t>
+          <t>From the Logo</t>
+        </is>
+      </c>
+      <c r="D41" s="91" t="inlineStr">
+        <is>
+          <t>SHOT -30%</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>Shoot the ball. After a missed shot: SHOT = 100%</t>
+          <t>Shoot the ball. +1 Point on make</t>
         </is>
       </c>
       <c r="F41" s="74" t="n">
@@ -3750,7 +3741,7 @@
       <c r="I41" s="106" t="n"/>
       <c r="J41" s="106" t="n"/>
     </row>
-    <row r="42" ht="28" customHeight="1" s="132">
+    <row r="42" ht="57" customHeight="1" s="132">
       <c r="A42" s="29" t="n"/>
       <c r="B42" s="30" t="inlineStr">
         <is>
@@ -3759,28 +3750,28 @@
       </c>
       <c r="C42" s="32" t="inlineStr">
         <is>
-          <t>Skyhook</t>
+          <t>Full-Court Heave</t>
         </is>
       </c>
       <c r="D42" s="33" t="inlineStr">
         <is>
-          <t>SHOT +10%</t>
-        </is>
-      </c>
-      <c r="E42" s="94" t="inlineStr">
-        <is>
-          <t>Shoot the ball. Shot is unaffected by Clamps</t>
+          <t>SHOT = 10%</t>
+        </is>
+      </c>
+      <c r="E42" s="33" t="inlineStr">
+        <is>
+          <t>Shoot the ball. +1 Point on make</t>
         </is>
       </c>
       <c r="F42" s="80" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G42" s="105" t="n"/>
       <c r="H42" s="106" t="n"/>
       <c r="I42" s="106" t="n"/>
       <c r="J42" s="106" t="n"/>
     </row>
-    <row r="43" ht="28" customHeight="1" s="132">
+    <row r="43" ht="20" customHeight="1" s="132">
       <c r="A43" s="29" t="n"/>
       <c r="B43" s="30" t="inlineStr">
         <is>
@@ -3789,201 +3780,201 @@
       </c>
       <c r="C43" s="31" t="inlineStr">
         <is>
-          <t>Slam Dunk</t>
+          <t>Putback Tip</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>SHOT +10%. SHOT = 100% if SHOT &gt;= 70%</t>
+          <t>SHOT +10%</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>Shoot the ball</t>
+          <t>Shoot the ball. After a missed shot: SHOT = 100%</t>
         </is>
       </c>
       <c r="F43" s="74" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G43" s="112" t="n"/>
       <c r="H43" s="106" t="n"/>
       <c r="I43" s="106" t="n"/>
       <c r="J43" s="106" t="n"/>
     </row>
-    <row r="44" ht="42" customHeight="1" s="132">
-      <c r="A44" s="52" t="n"/>
-      <c r="B44" s="53" t="inlineStr">
+    <row r="44" ht="28" customHeight="1" s="132">
+      <c r="A44" s="29" t="n"/>
+      <c r="B44" s="30" t="inlineStr">
         <is>
           <t>Special Move</t>
         </is>
       </c>
-      <c r="C44" s="69" t="inlineStr">
-        <is>
-          <t>Turnaround Three</t>
-        </is>
-      </c>
-      <c r="D44" s="70" t="inlineStr">
-        <is>
-          <t>Discard any number of cards. SHOT +10% for each</t>
-        </is>
-      </c>
-      <c r="E44" s="70" t="inlineStr">
-        <is>
-          <t>Shoot the ball. +1 Point on make</t>
-        </is>
-      </c>
-      <c r="F44" s="84" t="n">
-        <v>1</v>
-      </c>
-      <c r="G44" s="129" t="inlineStr">
-        <is>
-          <t>Only 1 in deck</t>
-        </is>
-      </c>
+      <c r="C44" s="32" t="inlineStr">
+        <is>
+          <t>Skyhook</t>
+        </is>
+      </c>
+      <c r="D44" s="33" t="inlineStr">
+        <is>
+          <t>SHOT +10%</t>
+        </is>
+      </c>
+      <c r="E44" s="94" t="inlineStr">
+        <is>
+          <t>Shoot the ball. Shot is unaffected by Clamps</t>
+        </is>
+      </c>
+      <c r="F44" s="80" t="n">
+        <v>4</v>
+      </c>
+      <c r="G44" s="105" t="n"/>
       <c r="H44" s="106" t="n"/>
       <c r="I44" s="106" t="n"/>
       <c r="J44" s="106" t="n"/>
     </row>
-    <row r="45" ht="42" customHeight="1" s="132">
-      <c r="A45" s="61" t="n"/>
-      <c r="B45" s="62" t="inlineStr">
+    <row r="45" ht="28" customHeight="1" s="132">
+      <c r="A45" s="29" t="n"/>
+      <c r="B45" s="30" t="inlineStr">
         <is>
           <t>Special Move</t>
         </is>
       </c>
-      <c r="C45" s="66" t="inlineStr">
+      <c r="C45" s="31" t="inlineStr">
+        <is>
+          <t>Slam Dunk</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>SHOT +10%. SHOT = 100% if SHOT &gt;= 70%</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>Shoot the ball</t>
+        </is>
+      </c>
+      <c r="F45" s="74" t="n">
+        <v>4</v>
+      </c>
+      <c r="G45" s="112" t="n"/>
+      <c r="H45" s="106" t="n"/>
+      <c r="I45" s="106" t="n"/>
+      <c r="J45" s="106" t="n"/>
+    </row>
+    <row r="46" ht="42" customHeight="1" s="132">
+      <c r="A46" s="52" t="n"/>
+      <c r="B46" s="53" t="inlineStr">
+        <is>
+          <t>Special Move</t>
+        </is>
+      </c>
+      <c r="C46" s="69" t="inlineStr">
+        <is>
+          <t>Turnaround Three</t>
+        </is>
+      </c>
+      <c r="D46" s="70" t="inlineStr">
+        <is>
+          <t>Discard any number of cards. SHOT +10% for each</t>
+        </is>
+      </c>
+      <c r="E46" s="70" t="inlineStr">
+        <is>
+          <t>Shoot the ball. +1 Point on make</t>
+        </is>
+      </c>
+      <c r="F46" s="84" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" s="129" t="inlineStr">
+        <is>
+          <t>Only 1 in deck</t>
+        </is>
+      </c>
+      <c r="H46" s="106" t="n"/>
+      <c r="I46" s="106" t="n"/>
+      <c r="J46" s="106" t="n"/>
+    </row>
+    <row r="47" ht="42" customHeight="1" s="132">
+      <c r="A47" s="61" t="n"/>
+      <c r="B47" s="62" t="inlineStr">
+        <is>
+          <t>Special Move</t>
+        </is>
+      </c>
+      <c r="C47" s="66" t="inlineStr">
         <is>
           <t>Euro Step</t>
         </is>
       </c>
-      <c r="D45" s="67" t="inlineStr">
+      <c r="D47" s="67" t="inlineStr">
         <is>
           <t>Flip a coin until you get Tails. For each Heads, SHOT +5% and Draw 1 card</t>
         </is>
       </c>
-      <c r="E45" s="68" t="n"/>
-      <c r="F45" s="85" t="n">
+      <c r="E47" s="68" t="n"/>
+      <c r="F47" s="85" t="n">
         <v>5</v>
       </c>
-      <c r="G45" s="122" t="n"/>
-      <c r="H45" s="104" t="n"/>
-      <c r="I45" s="104" t="n"/>
-      <c r="J45" s="104" t="n"/>
-    </row>
-    <row r="46" ht="29" customHeight="1" s="132" thickBot="1">
-      <c r="A46" s="61" t="n"/>
-      <c r="B46" s="62" t="inlineStr">
+      <c r="G47" s="122" t="n"/>
+      <c r="H47" s="104" t="n"/>
+      <c r="I47" s="104" t="n"/>
+      <c r="J47" s="104" t="n"/>
+    </row>
+    <row r="48" ht="29" customHeight="1" s="132">
+      <c r="A48" s="61" t="n"/>
+      <c r="B48" s="62" t="inlineStr">
         <is>
           <t>Special Move</t>
         </is>
       </c>
-      <c r="C46" s="66" t="inlineStr">
+      <c r="C48" s="66" t="inlineStr">
         <is>
           <t>Wide-Open Three</t>
         </is>
       </c>
-      <c r="D46" s="67" t="inlineStr">
+      <c r="D48" s="67" t="inlineStr">
         <is>
           <t>Select any number of other players. SHOT +10% for each</t>
         </is>
       </c>
-      <c r="E46" s="68" t="inlineStr">
+      <c r="E48" s="68" t="inlineStr">
         <is>
           <t>Shoot the ball. +1 Point on make. Selected players receive +1 AST on a make</t>
         </is>
       </c>
-      <c r="F46" s="85" t="n">
+      <c r="F48" s="85" t="n">
         <v>2</v>
       </c>
-      <c r="G46" s="122" t="inlineStr">
+      <c r="G48" s="122" t="inlineStr">
         <is>
           <t>Selecting none rolls off current SHOT and is still a three</t>
         </is>
       </c>
-      <c r="H46" s="104" t="n"/>
-      <c r="I46" s="104" t="n"/>
-      <c r="J46" s="104" t="n"/>
-    </row>
-    <row r="47" ht="20" customHeight="1" s="132">
-      <c r="A47" s="58" t="inlineStr">
+      <c r="H48" s="104" t="n"/>
+      <c r="I48" s="104" t="n"/>
+      <c r="J48" s="104" t="n"/>
+    </row>
+    <row r="49" ht="20" customHeight="1" s="132">
+      <c r="A49" s="58" t="inlineStr">
         <is>
           <t>Clamp</t>
         </is>
       </c>
-      <c r="B47" s="59">
-        <f>COUNTIF($B$5:$B$123,"Clamp")</f>
+      <c r="B49" s="59">
+        <f>COUNTIF($B$5:$B$131,"Clamp")</f>
         <v/>
       </c>
-      <c r="C47" s="60" t="n"/>
-      <c r="D47" s="60" t="n"/>
-      <c r="E47" s="60" t="n"/>
-      <c r="F47" s="86" t="n"/>
-      <c r="G47" s="109" t="n"/>
-      <c r="H47" s="110" t="n"/>
-      <c r="I47" s="110" t="n"/>
-      <c r="J47" s="110" t="n"/>
-    </row>
-    <row r="48" ht="56" customHeight="1" s="132">
-      <c r="A48" s="29" t="n"/>
-      <c r="B48" s="30" t="inlineStr">
-        <is>
-          <t>Clamp</t>
-        </is>
-      </c>
-      <c r="C48" s="31" t="inlineStr">
-        <is>
-          <t>Contest</t>
-        </is>
-      </c>
-      <c r="D48" s="6" t="inlineStr">
-        <is>
-          <t>Next player SHOT -25% if they shoot</t>
-        </is>
-      </c>
-      <c r="E48" s="7" t="n"/>
-      <c r="F48" s="76" t="n">
-        <v>10</v>
-      </c>
-      <c r="G48" s="130" t="inlineStr">
-        <is>
-          <t>1 def</t>
-        </is>
-      </c>
-      <c r="H48" s="102" t="n"/>
-      <c r="I48" s="102" t="n"/>
-      <c r="J48" s="102" t="n"/>
-    </row>
-    <row r="49" ht="47" customHeight="1" s="132">
-      <c r="A49" s="29" t="n"/>
-      <c r="B49" s="30" t="inlineStr">
-        <is>
-          <t>Clamp</t>
-        </is>
-      </c>
-      <c r="C49" s="32" t="inlineStr">
-        <is>
-          <t>Double-Team</t>
-        </is>
-      </c>
-      <c r="D49" s="33" t="inlineStr">
-        <is>
-          <t>Next Player cannot play 2 random cards from hand.</t>
-        </is>
-      </c>
-      <c r="E49" s="34" t="n"/>
-      <c r="F49" s="75" t="n">
-        <v>4</v>
-      </c>
-      <c r="G49" s="125" t="inlineStr">
-        <is>
-          <t>2 def</t>
-        </is>
-      </c>
-      <c r="H49" s="102" t="n"/>
-      <c r="I49" s="102" t="n"/>
-      <c r="J49" s="102" t="n"/>
-    </row>
-    <row r="50" ht="54" customHeight="1" s="132">
+      <c r="C49" s="60" t="n"/>
+      <c r="D49" s="60" t="n"/>
+      <c r="E49" s="60" t="n"/>
+      <c r="F49" s="86" t="n"/>
+      <c r="G49" s="109" t="n"/>
+      <c r="H49" s="110" t="n"/>
+      <c r="I49" s="110" t="n"/>
+      <c r="J49" s="110" t="n"/>
+    </row>
+    <row r="50" ht="56" customHeight="1" s="132">
       <c r="A50" s="29" t="n"/>
       <c r="B50" s="30" t="inlineStr">
         <is>
@@ -3992,17 +3983,17 @@
       </c>
       <c r="C50" s="31" t="inlineStr">
         <is>
-          <t>Full-Court Press</t>
+          <t>Contest</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>Next player discards 2 cards at the start of their turn</t>
+          <t>Next player SHOT -25% if they shoot</t>
         </is>
       </c>
       <c r="E50" s="7" t="n"/>
       <c r="F50" s="76" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G50" s="130" t="inlineStr">
         <is>
@@ -4013,7 +4004,7 @@
       <c r="I50" s="102" t="n"/>
       <c r="J50" s="102" t="n"/>
     </row>
-    <row r="51" ht="28" customHeight="1" s="132">
+    <row r="51" ht="47" customHeight="1" s="132">
       <c r="A51" s="29" t="n"/>
       <c r="B51" s="30" t="inlineStr">
         <is>
@@ -4022,171 +4013,183 @@
       </c>
       <c r="C51" s="32" t="inlineStr">
         <is>
-          <t>Trap</t>
-        </is>
-      </c>
-      <c r="D51" s="94" t="inlineStr">
-        <is>
-          <t>Next player can only play Pass cards during their turn</t>
+          <t>Double-Team</t>
+        </is>
+      </c>
+      <c r="D51" s="33" t="inlineStr">
+        <is>
+          <t>Next Player cannot play 2 random cards from hand.</t>
         </is>
       </c>
       <c r="E51" s="34" t="n"/>
       <c r="F51" s="75" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G51" s="125" t="inlineStr">
         <is>
-          <t>They can still shoot as another option; 3 def</t>
+          <t>2 def</t>
         </is>
       </c>
       <c r="H51" s="102" t="n"/>
       <c r="I51" s="102" t="n"/>
       <c r="J51" s="102" t="n"/>
     </row>
-    <row r="52" ht="28" customHeight="1" s="132">
-      <c r="A52" s="61" t="n"/>
-      <c r="B52" s="62" t="inlineStr">
+    <row r="52" ht="54" customHeight="1" s="132">
+      <c r="A52" s="29" t="n"/>
+      <c r="B52" s="30" t="inlineStr">
         <is>
           <t>Clamp</t>
         </is>
       </c>
-      <c r="C52" s="66" t="inlineStr">
+      <c r="C52" s="31" t="inlineStr">
+        <is>
+          <t>Full-Court Press</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>Next player discards 2 cards at the start of their turn</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="n"/>
+      <c r="F52" s="76" t="n">
+        <v>3</v>
+      </c>
+      <c r="G52" s="130" t="inlineStr">
+        <is>
+          <t>1 def</t>
+        </is>
+      </c>
+      <c r="H52" s="102" t="n"/>
+      <c r="I52" s="102" t="n"/>
+      <c r="J52" s="102" t="n"/>
+    </row>
+    <row r="53" ht="28" customHeight="1" s="132">
+      <c r="A53" s="29" t="n"/>
+      <c r="B53" s="30" t="inlineStr">
+        <is>
+          <t>Clamp</t>
+        </is>
+      </c>
+      <c r="C53" s="32" t="inlineStr">
+        <is>
+          <t>Trap</t>
+        </is>
+      </c>
+      <c r="D53" s="94" t="inlineStr">
+        <is>
+          <t>Next player can only play Pass cards during their turn</t>
+        </is>
+      </c>
+      <c r="E53" s="34" t="n"/>
+      <c r="F53" s="75" t="n">
+        <v>5</v>
+      </c>
+      <c r="G53" s="125" t="inlineStr">
+        <is>
+          <t>They can still shoot as another option; 3 def</t>
+        </is>
+      </c>
+      <c r="H53" s="102" t="n"/>
+      <c r="I53" s="102" t="n"/>
+      <c r="J53" s="102" t="n"/>
+    </row>
+    <row r="54" ht="28" customHeight="1" s="132">
+      <c r="A54" s="61" t="n"/>
+      <c r="B54" s="62" t="inlineStr">
+        <is>
+          <t>Clamp</t>
+        </is>
+      </c>
+      <c r="C54" s="66" t="inlineStr">
         <is>
           <t>Triple-Team</t>
         </is>
       </c>
-      <c r="D52" s="67" t="inlineStr">
+      <c r="D54" s="67" t="inlineStr">
         <is>
           <t>Next player cannot play 3 random cards from hand.</t>
         </is>
       </c>
-      <c r="E52" s="68" t="n"/>
-      <c r="F52" s="85" t="n">
+      <c r="E54" s="68" t="n"/>
+      <c r="F54" s="85" t="n">
         <v>2</v>
       </c>
-      <c r="G52" s="135" t="inlineStr">
+      <c r="G54" s="135" t="inlineStr">
         <is>
           <t>3 def</t>
         </is>
       </c>
-      <c r="H52" s="117" t="n"/>
-      <c r="I52" s="117" t="n"/>
-      <c r="J52" s="117" t="n"/>
-    </row>
-    <row r="53" ht="28" customHeight="1" s="132">
-      <c r="A53" s="58" t="inlineStr">
+      <c r="H54" s="117" t="n"/>
+      <c r="I54" s="117" t="n"/>
+      <c r="J54" s="117" t="n"/>
+    </row>
+    <row r="55" ht="28" customHeight="1" s="132">
+      <c r="A55" s="58" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="B53" s="59">
-        <f>COUNTIF($B$5:$B$123,"Whistle")</f>
+      <c r="B55" s="59">
+        <f>COUNTIF($B$5:$B$131,"Whistle")</f>
         <v/>
       </c>
-      <c r="C53" s="60" t="n"/>
-      <c r="D53" s="60" t="n"/>
-      <c r="E53" s="60" t="n"/>
-      <c r="F53" s="86" t="n"/>
-      <c r="G53" s="109" t="n"/>
-      <c r="H53" s="110" t="n"/>
-      <c r="I53" s="110" t="n"/>
-      <c r="J53" s="110" t="n"/>
-    </row>
-    <row r="54" ht="42" customHeight="1" s="132">
-      <c r="A54" s="29" t="inlineStr">
+      <c r="C55" s="60" t="n"/>
+      <c r="D55" s="60" t="n"/>
+      <c r="E55" s="60" t="n"/>
+      <c r="F55" s="86" t="n"/>
+      <c r="G55" s="109" t="n"/>
+      <c r="H55" s="110" t="n"/>
+      <c r="I55" s="110" t="n"/>
+      <c r="J55" s="110" t="n"/>
+    </row>
+    <row r="56" ht="42" customHeight="1" s="132">
+      <c r="A56" s="29" t="inlineStr">
         <is>
           <t>All whistles are limited to 1</t>
         </is>
       </c>
-      <c r="B54" s="30" t="inlineStr">
+      <c r="B56" s="30" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C54" s="31" t="inlineStr">
+      <c r="C56" s="31" t="inlineStr">
         <is>
           <t>Back Court Violation</t>
         </is>
       </c>
-      <c r="D54" s="6" t="inlineStr">
+      <c r="D56" s="6" t="inlineStr">
         <is>
           <t>Pass Card Played: Cancel that card. That player TOV +1. Move ball to player of choice</t>
-        </is>
-      </c>
-      <c r="E54" s="7" t="n"/>
-      <c r="F54" s="138" t="n"/>
-      <c r="G54" s="101" t="inlineStr">
-        <is>
-          <t>The player who played this whistle chooses, excluding the player who played the pass but including themselves.</t>
-        </is>
-      </c>
-      <c r="H54" s="102" t="n"/>
-      <c r="I54" s="102" t="n"/>
-      <c r="J54" s="102" t="n"/>
-    </row>
-    <row r="55" ht="40" customHeight="1" s="132">
-      <c r="A55" s="29" t="n"/>
-      <c r="B55" s="30" t="inlineStr">
-        <is>
-          <t>Whistle</t>
-        </is>
-      </c>
-      <c r="C55" s="90" t="inlineStr">
-        <is>
-          <t>Blocking Foul</t>
-        </is>
-      </c>
-      <c r="D55" s="93" t="inlineStr">
-        <is>
-          <t>Clamp Card Played: Cancel card. Clamped player +1 FT</t>
-        </is>
-      </c>
-      <c r="E55" s="34" t="n"/>
-      <c r="F55" s="138" t="n"/>
-      <c r="G55" s="107" t="n"/>
-      <c r="H55" s="102" t="n"/>
-      <c r="I55" s="102" t="n"/>
-      <c r="J55" s="102" t="n"/>
-    </row>
-    <row r="56" ht="30" customHeight="1" s="132">
-      <c r="A56" s="29" t="n"/>
-      <c r="B56" s="30" t="inlineStr">
-        <is>
-          <t>Whistle</t>
-        </is>
-      </c>
-      <c r="C56" s="31" t="inlineStr">
-        <is>
-          <t>Charge</t>
-        </is>
-      </c>
-      <c r="D56" s="92" t="inlineStr">
-        <is>
-          <t>Shot Attempt: Cancel. Shooter Inbounds</t>
         </is>
       </c>
       <c r="E56" s="7" t="n"/>
       <c r="F56" s="138" t="n"/>
-      <c r="G56" s="101" t="n"/>
+      <c r="G56" s="101" t="inlineStr">
+        <is>
+          <t>The player who played this whistle chooses, excluding the player who played the pass but including themselves.</t>
+        </is>
+      </c>
       <c r="H56" s="102" t="n"/>
       <c r="I56" s="102" t="n"/>
       <c r="J56" s="102" t="n"/>
     </row>
-    <row r="57" ht="56" customHeight="1" s="132">
+    <row r="57" ht="40" customHeight="1" s="132">
       <c r="A57" s="29" t="n"/>
       <c r="B57" s="30" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C57" s="32" t="inlineStr">
-        <is>
-          <t>Cleared to Play</t>
-        </is>
-      </c>
-      <c r="D57" s="33" t="inlineStr">
-        <is>
-          <t>Injury Card Played: Cancel card.</t>
+      <c r="C57" s="90" t="inlineStr">
+        <is>
+          <t>Blocking Foul</t>
+        </is>
+      </c>
+      <c r="D57" s="93" t="inlineStr">
+        <is>
+          <t>Clamp Card Played: Cancel card. Clamped player +1 FT</t>
         </is>
       </c>
       <c r="E57" s="34" t="n"/>
@@ -4196,7 +4199,7 @@
       <c r="I57" s="102" t="n"/>
       <c r="J57" s="102" t="n"/>
     </row>
-    <row r="58" ht="42" customHeight="1" s="132">
+    <row r="58" ht="30" customHeight="1" s="132">
       <c r="A58" s="29" t="n"/>
       <c r="B58" s="30" t="inlineStr">
         <is>
@@ -4205,53 +4208,41 @@
       </c>
       <c r="C58" s="31" t="inlineStr">
         <is>
-          <t>Coach’s Challenge</t>
-        </is>
-      </c>
-      <c r="D58" s="6" t="inlineStr">
-        <is>
-          <t>Any Whistle Card Played: Cancel card.</t>
-        </is>
-      </c>
-      <c r="E58" s="7" t="inlineStr">
-        <is>
-          <t>Pull a Timeout from the discards, if one is there, and take it</t>
-        </is>
-      </c>
+          <t>Charge</t>
+        </is>
+      </c>
+      <c r="D58" s="92" t="inlineStr">
+        <is>
+          <t>Shot Attempt: Cancel. Shooter Inbounds</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="n"/>
       <c r="F58" s="138" t="n"/>
       <c r="G58" s="101" t="n"/>
       <c r="H58" s="102" t="n"/>
       <c r="I58" s="102" t="n"/>
       <c r="J58" s="102" t="n"/>
     </row>
-    <row r="59" ht="42" customHeight="1" s="132">
+    <row r="59" ht="56" customHeight="1" s="132">
       <c r="A59" s="29" t="n"/>
       <c r="B59" s="30" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C59" s="90" t="inlineStr">
-        <is>
-          <t>Delay-of-Game Warning</t>
-        </is>
-      </c>
-      <c r="D59" s="94" t="inlineStr">
-        <is>
-          <t>Lower Shot Clock with a card: Cancel that card's effects</t>
-        </is>
-      </c>
-      <c r="E59" s="33" t="inlineStr">
-        <is>
-          <t>If 2nd time activated this round: Whistle player takes 1 FT in addition</t>
-        </is>
-      </c>
-      <c r="F59" s="139" t="n"/>
-      <c r="G59" s="113" t="inlineStr">
-        <is>
-          <t>The Shot Clock reduction still applies. Game Breaks do not count — those are game events, not cards the player activates.</t>
-        </is>
-      </c>
+      <c r="C59" s="32" t="inlineStr">
+        <is>
+          <t>Cleared to Play</t>
+        </is>
+      </c>
+      <c r="D59" s="33" t="inlineStr">
+        <is>
+          <t>Injury Card Played: Cancel card.</t>
+        </is>
+      </c>
+      <c r="E59" s="34" t="n"/>
+      <c r="F59" s="138" t="n"/>
+      <c r="G59" s="107" t="n"/>
       <c r="H59" s="102" t="n"/>
       <c r="I59" s="102" t="n"/>
       <c r="J59" s="102" t="n"/>
@@ -4265,26 +4256,26 @@
       </c>
       <c r="C60" s="31" t="inlineStr">
         <is>
-          <t>Double Dribble</t>
+          <t>Coach’s Challenge</t>
         </is>
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>Dribble Move Card Played (Dribble, Rhythm Dribble, etc.): Cancel card. Discard 1 card. TOV +1</t>
-        </is>
-      </c>
-      <c r="E60" s="7" t="n"/>
+          <t>Any Whistle Card Played: Cancel card.</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>Pull a Timeout from the discards, if one is there, and take it</t>
+        </is>
+      </c>
       <c r="F60" s="138" t="n"/>
-      <c r="G60" s="101" t="inlineStr">
-        <is>
-          <t>The dribbling player inbounds. The round is NOT incremented.</t>
-        </is>
-      </c>
+      <c r="G60" s="101" t="n"/>
       <c r="H60" s="102" t="n"/>
       <c r="I60" s="102" t="n"/>
       <c r="J60" s="102" t="n"/>
     </row>
-    <row r="61" ht="28" customHeight="1" s="132">
+    <row r="61" ht="42" customHeight="1" s="132">
       <c r="A61" s="29" t="n"/>
       <c r="B61" s="30" t="inlineStr">
         <is>
@@ -4293,17 +4284,25 @@
       </c>
       <c r="C61" s="90" t="inlineStr">
         <is>
-          <t>Flagrant Foul</t>
+          <t>Delay-of-Game Warning</t>
         </is>
       </c>
       <c r="D61" s="94" t="inlineStr">
         <is>
-          <t>Clamp Card Played: Cancel card. Clamper discard 1. Clamped player +1 FT then gets ball</t>
-        </is>
-      </c>
-      <c r="E61" s="34" t="n"/>
-      <c r="F61" s="138" t="n"/>
-      <c r="G61" s="107" t="n"/>
+          <t>Lower Shot Clock with a card: Cancel that card's effects</t>
+        </is>
+      </c>
+      <c r="E61" s="33" t="inlineStr">
+        <is>
+          <t>If 2nd time activated this round: Whistle player takes 1 FT in addition</t>
+        </is>
+      </c>
+      <c r="F61" s="139" t="n"/>
+      <c r="G61" s="113" t="inlineStr">
+        <is>
+          <t>The Shot Clock reduction still applies. Game Breaks do not count — those are game events, not cards the player activates.</t>
+        </is>
+      </c>
       <c r="H61" s="102" t="n"/>
       <c r="I61" s="102" t="n"/>
       <c r="J61" s="102" t="n"/>
@@ -4315,38 +4314,42 @@
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C62" s="90" t="inlineStr">
-        <is>
-          <t>Flagrant Foul II</t>
-        </is>
-      </c>
-      <c r="D62" s="91" t="inlineStr">
-        <is>
-          <t>Clamp Card Played: Cancel card. Clamper discards Bag. Clamped player +1 FT then gets ball</t>
+      <c r="C62" s="31" t="inlineStr">
+        <is>
+          <t>Double Dribble</t>
+        </is>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>Dribble Move Card Played (Dribble, Rhythm Dribble, etc.): Cancel card. Discard 1 card. TOV +1</t>
         </is>
       </c>
       <c r="E62" s="7" t="n"/>
       <c r="F62" s="138" t="n"/>
-      <c r="G62" s="101" t="n"/>
+      <c r="G62" s="101" t="inlineStr">
+        <is>
+          <t>The dribbling player inbounds. The round is NOT incremented.</t>
+        </is>
+      </c>
       <c r="H62" s="102" t="n"/>
       <c r="I62" s="102" t="n"/>
       <c r="J62" s="102" t="n"/>
     </row>
-    <row r="63" ht="29" customHeight="1" s="132" thickBot="1">
+    <row r="63" ht="28" customHeight="1" s="132">
       <c r="A63" s="29" t="n"/>
       <c r="B63" s="30" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C63" s="32" t="inlineStr">
-        <is>
-          <t>Goaltending</t>
-        </is>
-      </c>
-      <c r="D63" s="33" t="inlineStr">
-        <is>
-          <t>Clamp Card Played: Cancel card. Clamped player +2 points. End round.</t>
+      <c r="C63" s="90" t="inlineStr">
+        <is>
+          <t>Flagrant Foul</t>
+        </is>
+      </c>
+      <c r="D63" s="94" t="inlineStr">
+        <is>
+          <t>Clamp Card Played: Cancel card. Clamper discard 1. Clamped player +1 FT then gets ball</t>
         </is>
       </c>
       <c r="E63" s="34" t="n"/>
@@ -4356,21 +4359,21 @@
       <c r="I63" s="102" t="n"/>
       <c r="J63" s="102" t="n"/>
     </row>
-    <row r="64" ht="20" customHeight="1" s="132">
+    <row r="64" ht="42" customHeight="1" s="132">
       <c r="A64" s="29" t="n"/>
       <c r="B64" s="30" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C64" s="31" t="inlineStr">
-        <is>
-          <t>Inadvertent Whistle</t>
+      <c r="C64" s="90" t="inlineStr">
+        <is>
+          <t>Flagrant Foul II</t>
         </is>
       </c>
       <c r="D64" s="91" t="inlineStr">
         <is>
-          <t>Any other whistle triggers: Cancel that card. Turn player draws 1 card.</t>
+          <t>Clamp Card Played: Cancel card. Clamper discards Bag. Clamped player +1 FT then gets ball</t>
         </is>
       </c>
       <c r="E64" s="7" t="n"/>
@@ -4380,7 +4383,7 @@
       <c r="I64" s="102" t="n"/>
       <c r="J64" s="102" t="n"/>
     </row>
-    <row r="65" ht="28" customHeight="1" s="132">
+    <row r="65" ht="29" customHeight="1" s="132">
       <c r="A65" s="29" t="n"/>
       <c r="B65" s="30" t="inlineStr">
         <is>
@@ -4389,12 +4392,12 @@
       </c>
       <c r="C65" s="32" t="inlineStr">
         <is>
-          <t>Official Review</t>
-        </is>
-      </c>
-      <c r="D65" s="94" t="inlineStr">
-        <is>
-          <t>Intangible Played: Discard all Intangibles from player.</t>
+          <t>Goaltending</t>
+        </is>
+      </c>
+      <c r="D65" s="33" t="inlineStr">
+        <is>
+          <t>Clamp Card Played: Cancel card. Clamped player +2 points. End round.</t>
         </is>
       </c>
       <c r="E65" s="34" t="n"/>
@@ -4404,7 +4407,7 @@
       <c r="I65" s="102" t="n"/>
       <c r="J65" s="102" t="n"/>
     </row>
-    <row r="66" ht="28" customHeight="1" s="132">
+    <row r="66" ht="20" customHeight="1" s="132">
       <c r="A66" s="29" t="n"/>
       <c r="B66" s="30" t="inlineStr">
         <is>
@@ -4413,26 +4416,22 @@
       </c>
       <c r="C66" s="31" t="inlineStr">
         <is>
-          <t>Shot Clock Violation</t>
+          <t>Inadvertent Whistle</t>
         </is>
       </c>
       <c r="D66" s="91" t="inlineStr">
         <is>
-          <t>Shot Clock is changed: TOV +1. Ball OOB</t>
+          <t>Any other whistle triggers: Cancel that card. Turn player draws 1 card.</t>
         </is>
       </c>
       <c r="E66" s="7" t="n"/>
       <c r="F66" s="138" t="n"/>
-      <c r="G66" s="101" t="inlineStr">
-        <is>
-          <t>This inbound does NOT increment the round.</t>
-        </is>
-      </c>
+      <c r="G66" s="101" t="n"/>
       <c r="H66" s="102" t="n"/>
       <c r="I66" s="102" t="n"/>
       <c r="J66" s="102" t="n"/>
     </row>
-    <row r="67" ht="14" customHeight="1" s="132">
+    <row r="67" ht="28" customHeight="1" s="132">
       <c r="A67" s="29" t="n"/>
       <c r="B67" s="30" t="inlineStr">
         <is>
@@ -4441,12 +4440,12 @@
       </c>
       <c r="C67" s="32" t="inlineStr">
         <is>
-          <t>Technical Foul</t>
+          <t>Official Review</t>
         </is>
       </c>
       <c r="D67" s="94" t="inlineStr">
         <is>
-          <t>Any Non-Whistle Card Played: Cancel card. Take 1 FT</t>
+          <t>Intangible Played: Discard all Intangibles from player.</t>
         </is>
       </c>
       <c r="E67" s="34" t="n"/>
@@ -4456,7 +4455,7 @@
       <c r="I67" s="102" t="n"/>
       <c r="J67" s="102" t="n"/>
     </row>
-    <row r="68" ht="14" customHeight="1" s="132">
+    <row r="68" ht="28" customHeight="1" s="132">
       <c r="A68" s="29" t="n"/>
       <c r="B68" s="30" t="inlineStr">
         <is>
@@ -4465,147 +4464,143 @@
       </c>
       <c r="C68" s="31" t="inlineStr">
         <is>
-          <t>Timeout</t>
+          <t>Shot Clock Violation</t>
         </is>
       </c>
       <c r="D68" s="91" t="inlineStr">
         <is>
-          <t>Immediate: Reset Shot Clock. You inbound. All players draw 1 card</t>
+          <t>Shot Clock is changed: TOV +1. Ball OOB</t>
         </is>
       </c>
       <c r="E68" s="7" t="n"/>
       <c r="F68" s="138" t="n"/>
-      <c r="G68" s="101" t="n"/>
+      <c r="G68" s="101" t="inlineStr">
+        <is>
+          <t>This inbound does NOT increment the round.</t>
+        </is>
+      </c>
       <c r="H68" s="102" t="n"/>
       <c r="I68" s="102" t="n"/>
       <c r="J68" s="102" t="n"/>
     </row>
     <row r="69" ht="14" customHeight="1" s="132">
-      <c r="A69" s="61" t="n"/>
-      <c r="B69" s="62" t="inlineStr">
+      <c r="A69" s="29" t="n"/>
+      <c r="B69" s="30" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C69" s="63" t="inlineStr">
+      <c r="C69" s="32" t="inlineStr">
+        <is>
+          <t>Technical Foul</t>
+        </is>
+      </c>
+      <c r="D69" s="94" t="inlineStr">
+        <is>
+          <t>Any Non-Whistle Card Played: Cancel card. Take 1 FT</t>
+        </is>
+      </c>
+      <c r="E69" s="34" t="n"/>
+      <c r="F69" s="138" t="n"/>
+      <c r="G69" s="107" t="n"/>
+      <c r="H69" s="102" t="n"/>
+      <c r="I69" s="102" t="n"/>
+      <c r="J69" s="102" t="n"/>
+    </row>
+    <row r="70" ht="14" customHeight="1" s="132">
+      <c r="A70" s="29" t="n"/>
+      <c r="B70" s="30" t="inlineStr">
+        <is>
+          <t>Whistle</t>
+        </is>
+      </c>
+      <c r="C70" s="31" t="inlineStr">
+        <is>
+          <t>Timeout</t>
+        </is>
+      </c>
+      <c r="D70" s="91" t="inlineStr">
+        <is>
+          <t>Immediate: Reset Shot Clock. You inbound. All players draw 1 card</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="n"/>
+      <c r="F70" s="138" t="n"/>
+      <c r="G70" s="101" t="n"/>
+      <c r="H70" s="102" t="n"/>
+      <c r="I70" s="102" t="n"/>
+      <c r="J70" s="102" t="n"/>
+    </row>
+    <row r="71" ht="14" customHeight="1" s="132">
+      <c r="A71" s="61" t="n"/>
+      <c r="B71" s="62" t="inlineStr">
+        <is>
+          <t>Whistle</t>
+        </is>
+      </c>
+      <c r="C71" s="63" t="inlineStr">
         <is>
           <t>Travel</t>
         </is>
       </c>
-      <c r="D69" s="64" t="inlineStr">
+      <c r="D71" s="64" t="inlineStr">
         <is>
           <t>Move card played: Cancel card. TOV +1</t>
         </is>
       </c>
-      <c r="E69" s="65" t="n"/>
-      <c r="F69" s="140" t="n"/>
-      <c r="G69" s="116" t="n"/>
-      <c r="H69" s="117" t="n"/>
-      <c r="I69" s="117" t="n"/>
-      <c r="J69" s="117" t="n"/>
-    </row>
-    <row r="70" ht="28" customHeight="1" s="132">
-      <c r="A70" s="61" t="n"/>
-      <c r="B70" s="62" t="inlineStr">
+      <c r="E71" s="65" t="n"/>
+      <c r="F71" s="140" t="n"/>
+      <c r="G71" s="116" t="n"/>
+      <c r="H71" s="117" t="n"/>
+      <c r="I71" s="117" t="n"/>
+      <c r="J71" s="117" t="n"/>
+    </row>
+    <row r="72" ht="28" customHeight="1" s="132">
+      <c r="A72" s="61" t="n"/>
+      <c r="B72" s="62" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C70" s="63" t="inlineStr">
+      <c r="C72" s="63" t="inlineStr">
         <is>
           <t>Clear Path Foul</t>
         </is>
       </c>
-      <c r="D70" s="64" t="inlineStr">
+      <c r="D72" s="64" t="inlineStr">
         <is>
           <t>On Shot, when Clamped by SHOT-reducing Clamps: Cancel those Clamps. Award the points the shot was worth. Take 1 FT</t>
         </is>
       </c>
-      <c r="E70" s="65" t="n"/>
-      <c r="F70" s="140" t="n"/>
-      <c r="G70" s="116" t="inlineStr">
+      <c r="E72" s="65" t="n"/>
+      <c r="F72" s="140" t="n"/>
+      <c r="G72" s="116" t="inlineStr">
         <is>
           <t>Fires as the shot starts, before the cutscene. This DOES count as a completed round.</t>
         </is>
       </c>
-      <c r="H70" s="117" t="n"/>
-      <c r="I70" s="117" t="n"/>
-      <c r="J70" s="117" t="n"/>
-    </row>
-    <row r="71" ht="28" customHeight="1" s="132">
-      <c r="A71" s="58" t="inlineStr">
+      <c r="H72" s="117" t="n"/>
+      <c r="I72" s="117" t="n"/>
+      <c r="J72" s="117" t="n"/>
+    </row>
+    <row r="73" ht="28" customHeight="1" s="132">
+      <c r="A73" s="58" t="inlineStr">
         <is>
           <t>Game Break</t>
         </is>
       </c>
-      <c r="B71" s="59">
-        <f>COUNTIF($B$5:$B$123,"Game Break")</f>
+      <c r="B73" s="59">
+        <f>COUNTIF($B$5:$B$131,"Game Break")</f>
         <v/>
       </c>
-      <c r="C71" s="60" t="n"/>
-      <c r="D71" s="60" t="n"/>
-      <c r="E71" s="60" t="n"/>
-      <c r="F71" s="86" t="n"/>
-      <c r="G71" s="109" t="n"/>
-      <c r="H71" s="110" t="n"/>
-      <c r="I71" s="110" t="n"/>
-      <c r="J71" s="110" t="n"/>
-    </row>
-    <row r="72" ht="28" customHeight="1" s="132">
-      <c r="A72" s="29" t="n"/>
-      <c r="B72" s="30" t="inlineStr">
-        <is>
-          <t>Game Break</t>
-        </is>
-      </c>
-      <c r="C72" s="32" t="inlineStr">
-        <is>
-          <t>2-Minute Warning</t>
-        </is>
-      </c>
-      <c r="D72" s="33" t="inlineStr">
-        <is>
-          <t>All players discard down to 2 or fewer cards</t>
-        </is>
-      </c>
-      <c r="E72" s="34" t="n"/>
-      <c r="F72" s="75" t="n">
-        <v>2</v>
-      </c>
-      <c r="G72" s="107" t="n"/>
-      <c r="H72" s="102" t="n"/>
-      <c r="I72" s="102" t="n"/>
-      <c r="J72" s="102" t="n"/>
-    </row>
-    <row r="73" ht="42" customHeight="1" s="132">
-      <c r="A73" s="29" t="n"/>
-      <c r="B73" s="30" t="inlineStr">
-        <is>
-          <t>Game Break</t>
-        </is>
-      </c>
-      <c r="C73" s="31" t="inlineStr">
-        <is>
-          <t>Benched</t>
-        </is>
-      </c>
-      <c r="D73" s="6" t="inlineStr">
-        <is>
-          <t>Immediately give ball to any other player.</t>
-        </is>
-      </c>
-      <c r="E73" s="7" t="n"/>
-      <c r="F73" s="76" t="n">
-        <v>5</v>
-      </c>
-      <c r="G73" s="111" t="inlineStr">
-        <is>
-          <t>This is not a pass</t>
-        </is>
-      </c>
-      <c r="H73" s="102" t="n"/>
-      <c r="I73" s="102" t="n"/>
-      <c r="J73" s="102" t="n"/>
+      <c r="C73" s="60" t="n"/>
+      <c r="D73" s="60" t="n"/>
+      <c r="E73" s="60" t="n"/>
+      <c r="F73" s="86" t="n"/>
+      <c r="G73" s="109" t="n"/>
+      <c r="H73" s="110" t="n"/>
+      <c r="I73" s="110" t="n"/>
+      <c r="J73" s="110" t="n"/>
     </row>
     <row r="74" ht="28" customHeight="1" s="132">
       <c r="A74" s="29" t="n"/>
@@ -4616,24 +4611,24 @@
       </c>
       <c r="C74" s="32" t="inlineStr">
         <is>
-          <t>Crowd Noise</t>
+          <t>2-Minute Warning</t>
         </is>
       </c>
       <c r="D74" s="33" t="inlineStr">
         <is>
-          <t>Discard 1 card.</t>
+          <t>All players discard down to 2 or fewer cards</t>
         </is>
       </c>
       <c r="E74" s="34" t="n"/>
       <c r="F74" s="75" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="G74" s="107" t="n"/>
       <c r="H74" s="102" t="n"/>
       <c r="I74" s="102" t="n"/>
       <c r="J74" s="102" t="n"/>
     </row>
-    <row r="75" ht="28" customHeight="1" s="132">
+    <row r="75" ht="42" customHeight="1" s="132">
       <c r="A75" s="29" t="n"/>
       <c r="B75" s="30" t="inlineStr">
         <is>
@@ -4642,43 +4637,47 @@
       </c>
       <c r="C75" s="31" t="inlineStr">
         <is>
-          <t>Designed Play</t>
+          <t>Benched</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>Draw up to a hand of 5</t>
+          <t>Immediately give ball to any other player.</t>
         </is>
       </c>
       <c r="E75" s="7" t="n"/>
       <c r="F75" s="76" t="n">
-        <v>10</v>
-      </c>
-      <c r="G75" s="101" t="n"/>
+        <v>5</v>
+      </c>
+      <c r="G75" s="111" t="inlineStr">
+        <is>
+          <t>This is not a pass</t>
+        </is>
+      </c>
       <c r="H75" s="102" t="n"/>
       <c r="I75" s="102" t="n"/>
       <c r="J75" s="102" t="n"/>
     </row>
-    <row r="76" ht="20" customHeight="1" s="132">
+    <row r="76" ht="28" customHeight="1" s="132">
       <c r="A76" s="29" t="n"/>
       <c r="B76" s="30" t="inlineStr">
         <is>
           <t>Game Break</t>
         </is>
       </c>
-      <c r="C76" s="90" t="inlineStr">
-        <is>
-          <t>Foul</t>
+      <c r="C76" s="32" t="inlineStr">
+        <is>
+          <t>Crowd Noise</t>
         </is>
       </c>
       <c r="D76" s="33" t="inlineStr">
         <is>
-          <t>Take 1 FT</t>
+          <t>Discard 1 card.</t>
         </is>
       </c>
       <c r="E76" s="34" t="n"/>
       <c r="F76" s="75" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="G76" s="107" t="n"/>
       <c r="H76" s="102" t="n"/>
@@ -4694,17 +4693,17 @@
       </c>
       <c r="C77" s="31" t="inlineStr">
         <is>
-          <t>MVP Vote</t>
+          <t>Designed Play</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>Draw 3 cards up to a hand of 7</t>
+          <t>Draw up to a hand of 5</t>
         </is>
       </c>
       <c r="E77" s="7" t="n"/>
       <c r="F77" s="76" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G77" s="101" t="n"/>
       <c r="H77" s="102" t="n"/>
@@ -4718,26 +4717,26 @@
           <t>Game Break</t>
         </is>
       </c>
-      <c r="C78" s="32" t="inlineStr">
-        <is>
-          <t>Off Night</t>
+      <c r="C78" s="90" t="inlineStr">
+        <is>
+          <t>Foul</t>
         </is>
       </c>
       <c r="D78" s="33" t="inlineStr">
         <is>
-          <t>SHOT -20% this possession</t>
+          <t>Take 1 FT</t>
         </is>
       </c>
       <c r="E78" s="34" t="n"/>
       <c r="F78" s="75" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G78" s="107" t="n"/>
       <c r="H78" s="102" t="n"/>
       <c r="I78" s="102" t="n"/>
       <c r="J78" s="102" t="n"/>
     </row>
-    <row r="79" ht="42" customHeight="1" s="132">
+    <row r="79" ht="28" customHeight="1" s="132">
       <c r="A79" s="29" t="n"/>
       <c r="B79" s="30" t="inlineStr">
         <is>
@@ -4746,28 +4745,24 @@
       </c>
       <c r="C79" s="31" t="inlineStr">
         <is>
-          <t>Swallowed Whistle</t>
+          <t>MVP Vote</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>Whistle cards cannot activate this turn.</t>
-        </is>
-      </c>
-      <c r="E79" s="6" t="inlineStr">
-        <is>
-          <t>Remains for remainder of round</t>
-        </is>
-      </c>
-      <c r="F79" s="74" t="n">
-        <v>5</v>
+          <t>Draw 3 cards up to a hand of 7</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="n"/>
+      <c r="F79" s="76" t="n">
+        <v>1</v>
       </c>
       <c r="G79" s="101" t="n"/>
       <c r="H79" s="102" t="n"/>
       <c r="I79" s="102" t="n"/>
       <c r="J79" s="102" t="n"/>
     </row>
-    <row r="80" ht="28" customHeight="1" s="132">
+    <row r="80" ht="20" customHeight="1" s="132">
       <c r="A80" s="29" t="n"/>
       <c r="B80" s="30" t="inlineStr">
         <is>
@@ -4776,26 +4771,24 @@
       </c>
       <c r="C80" s="32" t="inlineStr">
         <is>
-          <t>Rock Fight</t>
+          <t>Off Night</t>
         </is>
       </c>
       <c r="D80" s="33" t="inlineStr">
         <is>
-          <t>Players cannot shoot when SHOT is 50% or higher</t>
-        </is>
-      </c>
-      <c r="E80" s="33" t="inlineStr">
-        <is>
-          <t>Remains for remainder of round</t>
-        </is>
-      </c>
-      <c r="F80" s="80" t="n"/>
+          <t>SHOT -20% this possession</t>
+        </is>
+      </c>
+      <c r="E80" s="34" t="n"/>
+      <c r="F80" s="75" t="n">
+        <v>3</v>
+      </c>
       <c r="G80" s="107" t="n"/>
       <c r="H80" s="102" t="n"/>
       <c r="I80" s="102" t="n"/>
       <c r="J80" s="102" t="n"/>
     </row>
-    <row r="81" ht="56" customHeight="1" s="132">
+    <row r="81" ht="42" customHeight="1" s="132">
       <c r="A81" s="29" t="n"/>
       <c r="B81" s="30" t="inlineStr">
         <is>
@@ -4804,82 +4797,84 @@
       </c>
       <c r="C81" s="31" t="inlineStr">
         <is>
-          <t>Traded Mid-Game</t>
+          <t>Swallowed Whistle</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>Swap positions with random other player</t>
-        </is>
-      </c>
-      <c r="E81" s="7" t="n"/>
-      <c r="F81" s="76" t="n"/>
-      <c r="G81" s="111" t="inlineStr">
-        <is>
-          <t>Applies to rest of game</t>
-        </is>
-      </c>
+          <t>Whistle cards cannot activate this turn.</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="inlineStr">
+        <is>
+          <t>Remains for remainder of round</t>
+        </is>
+      </c>
+      <c r="F81" s="74" t="n">
+        <v>5</v>
+      </c>
+      <c r="G81" s="101" t="n"/>
       <c r="H81" s="102" t="n"/>
       <c r="I81" s="102" t="n"/>
       <c r="J81" s="102" t="n"/>
     </row>
-    <row r="82" ht="42" customHeight="1" s="132">
+    <row r="82" ht="28" customHeight="1" s="132">
       <c r="A82" s="29" t="n"/>
       <c r="B82" s="30" t="inlineStr">
         <is>
           <t>Game Break</t>
         </is>
       </c>
-      <c r="C82" s="134" t="inlineStr">
-        <is>
-          <t>Salary Cap Increase</t>
-        </is>
-      </c>
-      <c r="D82" s="91" t="inlineStr">
-        <is>
-          <t>All players draw 2 cards</t>
-        </is>
-      </c>
-      <c r="E82" s="7" t="n"/>
-      <c r="F82" s="76" t="n">
-        <v>4</v>
-      </c>
-      <c r="G82" s="111" t="n"/>
+      <c r="C82" s="32" t="inlineStr">
+        <is>
+          <t>Rock Fight</t>
+        </is>
+      </c>
+      <c r="D82" s="33" t="inlineStr">
+        <is>
+          <t>Players cannot shoot when SHOT is 50% or higher</t>
+        </is>
+      </c>
+      <c r="E82" s="33" t="inlineStr">
+        <is>
+          <t>Remains for remainder of round</t>
+        </is>
+      </c>
+      <c r="F82" s="80" t="n"/>
+      <c r="G82" s="107" t="n"/>
       <c r="H82" s="102" t="n"/>
       <c r="I82" s="102" t="n"/>
       <c r="J82" s="102" t="n"/>
     </row>
-    <row r="83" ht="42" customHeight="1" s="132">
+    <row r="83" ht="56" customHeight="1" s="132">
       <c r="A83" s="29" t="n"/>
       <c r="B83" s="30" t="inlineStr">
         <is>
           <t>Game Break</t>
         </is>
       </c>
-      <c r="C83" s="134" t="inlineStr">
-        <is>
-          <t>All-Swissh Selection</t>
-        </is>
-      </c>
-      <c r="D83" s="91" t="inlineStr">
-        <is>
-          <t>Draw 3 cards after your next make</t>
+      <c r="C83" s="31" t="inlineStr">
+        <is>
+          <t>Traded Mid-Game</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>Swap positions with random other player</t>
         </is>
       </c>
       <c r="E83" s="7" t="n"/>
-      <c r="F83" s="76" t="n">
-        <v>3</v>
-      </c>
+      <c r="F83" s="76" t="n"/>
       <c r="G83" s="111" t="inlineStr">
         <is>
-          <t>Arms an icon in the HUD tracking the pending draws</t>
+          <t>Applies to rest of game</t>
         </is>
       </c>
       <c r="H83" s="102" t="n"/>
       <c r="I83" s="102" t="n"/>
       <c r="J83" s="102" t="n"/>
     </row>
-    <row r="84" ht="28" customHeight="1" s="132">
+    <row r="84" ht="42" customHeight="1" s="132">
       <c r="A84" s="29" t="n"/>
       <c r="B84" s="30" t="inlineStr">
         <is>
@@ -4888,24 +4883,24 @@
       </c>
       <c r="C84" s="134" t="inlineStr">
         <is>
-          <t>All Star Selection</t>
+          <t>Salary Cap Increase</t>
         </is>
       </c>
       <c r="D84" s="91" t="inlineStr">
         <is>
-          <t>Draw 2 cards</t>
+          <t>All players draw 2 cards</t>
         </is>
       </c>
       <c r="E84" s="7" t="n"/>
       <c r="F84" s="76" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G84" s="111" t="n"/>
       <c r="H84" s="102" t="n"/>
       <c r="I84" s="102" t="n"/>
       <c r="J84" s="102" t="n"/>
     </row>
-    <row r="85" ht="28" customHeight="1" s="132">
+    <row r="85" ht="42" customHeight="1" s="132">
       <c r="A85" s="29" t="n"/>
       <c r="B85" s="30" t="inlineStr">
         <is>
@@ -4914,28 +4909,28 @@
       </c>
       <c r="C85" s="134" t="inlineStr">
         <is>
-          <t>Hit the Bike</t>
+          <t>All-Swissh Selection</t>
         </is>
       </c>
       <c r="D85" s="91" t="inlineStr">
         <is>
-          <t>Discard all Injuries. Draw 1 card. Give possession to another player</t>
+          <t>Draw 3 cards after your next make</t>
         </is>
       </c>
       <c r="E85" s="7" t="n"/>
       <c r="F85" s="76" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G85" s="111" t="inlineStr">
         <is>
-          <t>This is not a pass</t>
+          <t>Arms an icon in the HUD tracking the pending draws</t>
         </is>
       </c>
       <c r="H85" s="102" t="n"/>
       <c r="I85" s="102" t="n"/>
       <c r="J85" s="102" t="n"/>
     </row>
-    <row r="86" ht="56" customHeight="1" s="132">
+    <row r="86" ht="28" customHeight="1" s="132">
       <c r="A86" s="29" t="n"/>
       <c r="B86" s="30" t="inlineStr">
         <is>
@@ -4944,12 +4939,12 @@
       </c>
       <c r="C86" s="134" t="inlineStr">
         <is>
-          <t>Ice Wrap</t>
+          <t>All Star Selection</t>
         </is>
       </c>
       <c r="D86" s="91" t="inlineStr">
         <is>
-          <t>Draw 1 card. Discard all Injuries. If none, draw 1 additional card</t>
+          <t>Draw 2 cards</t>
         </is>
       </c>
       <c r="E86" s="7" t="n"/>
@@ -4961,7 +4956,7 @@
       <c r="I86" s="102" t="n"/>
       <c r="J86" s="102" t="n"/>
     </row>
-    <row r="87" ht="56" customHeight="1" s="132">
+    <row r="87" ht="28" customHeight="1" s="132">
       <c r="A87" s="29" t="n"/>
       <c r="B87" s="30" t="inlineStr">
         <is>
@@ -4970,28 +4965,28 @@
       </c>
       <c r="C87" s="134" t="inlineStr">
         <is>
-          <t>Wet Spot</t>
+          <t>Hit the Bike</t>
         </is>
       </c>
       <c r="D87" s="91" t="inlineStr">
         <is>
-          <t>All Injuries in the discards and deck are displayed. Take one</t>
+          <t>Discard all Injuries. Draw 1 card. Give possession to another player</t>
         </is>
       </c>
       <c r="E87" s="7" t="n"/>
       <c r="F87" s="76" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G87" s="111" t="inlineStr">
         <is>
-          <t>Deck ones are shown face down</t>
+          <t>This is not a pass</t>
         </is>
       </c>
       <c r="H87" s="102" t="n"/>
       <c r="I87" s="102" t="n"/>
       <c r="J87" s="102" t="n"/>
     </row>
-    <row r="88" ht="28" customHeight="1" s="132">
+    <row r="88" ht="56" customHeight="1" s="132">
       <c r="A88" s="29" t="n"/>
       <c r="B88" s="30" t="inlineStr">
         <is>
@@ -5000,28 +4995,24 @@
       </c>
       <c r="C88" s="134" t="inlineStr">
         <is>
-          <t>Fresh Ball</t>
+          <t>Ice Wrap</t>
         </is>
       </c>
       <c r="D88" s="91" t="inlineStr">
         <is>
-          <t>Next player does not draw at the start of their possession</t>
+          <t>Draw 1 card. Discard all Injuries. If none, draw 1 additional card</t>
         </is>
       </c>
       <c r="E88" s="7" t="n"/>
       <c r="F88" s="76" t="n">
-        <v>3</v>
-      </c>
-      <c r="G88" s="111" t="inlineStr">
-        <is>
-          <t>This is a bad thing in the NBA</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="G88" s="111" t="n"/>
       <c r="H88" s="102" t="n"/>
       <c r="I88" s="102" t="n"/>
       <c r="J88" s="102" t="n"/>
     </row>
-    <row r="89" ht="42" customHeight="1" s="132">
+    <row r="89" ht="56" customHeight="1" s="132">
       <c r="A89" s="29" t="n"/>
       <c r="B89" s="30" t="inlineStr">
         <is>
@@ -5030,21 +5021,21 @@
       </c>
       <c r="C89" s="134" t="inlineStr">
         <is>
-          <t>Trade Deadline</t>
+          <t>Wet Spot</t>
         </is>
       </c>
       <c r="D89" s="91" t="inlineStr">
         <is>
-          <t>Declare Left or Right: every player passes their hand that way. The ball goes with it</t>
+          <t>All Injuries in the discards and deck are displayed. Take one</t>
         </is>
       </c>
       <c r="E89" s="7" t="n"/>
       <c r="F89" s="76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G89" s="111" t="inlineStr">
         <is>
-          <t>The hex travels in the declared direction too</t>
+          <t>Deck ones are shown face down</t>
         </is>
       </c>
       <c r="H89" s="102" t="n"/>
@@ -5060,19 +5051,23 @@
       </c>
       <c r="C90" s="134" t="inlineStr">
         <is>
-          <t>Floor Cleanup</t>
+          <t>Fresh Ball</t>
         </is>
       </c>
       <c r="D90" s="91" t="inlineStr">
         <is>
-          <t>All players shuffle their hands into the deck and draw the same number of cards</t>
+          <t>Next player does not draw at the start of their possession</t>
         </is>
       </c>
       <c r="E90" s="7" t="n"/>
       <c r="F90" s="76" t="n">
         <v>3</v>
       </c>
-      <c r="G90" s="111" t="n"/>
+      <c r="G90" s="111" t="inlineStr">
+        <is>
+          <t>This is a bad thing in the NBA</t>
+        </is>
+      </c>
       <c r="H90" s="102" t="n"/>
       <c r="I90" s="102" t="n"/>
       <c r="J90" s="102" t="n"/>
@@ -5086,24 +5081,28 @@
       </c>
       <c r="C91" s="134" t="inlineStr">
         <is>
-          <t>Official Timeout</t>
+          <t>Trade Deadline</t>
         </is>
       </c>
       <c r="D91" s="91" t="inlineStr">
         <is>
-          <t>At least 1 referee must be armed: discard all Injuries on all players and clear all referees. If none, all players draw 1 card</t>
+          <t>Declare Left or Right: every player passes their hand that way. The ball goes with it</t>
         </is>
       </c>
       <c r="E91" s="7" t="n"/>
       <c r="F91" s="76" t="n">
-        <v>2</v>
-      </c>
-      <c r="G91" s="111" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="G91" s="111" t="inlineStr">
+        <is>
+          <t>The hex travels in the declared direction too</t>
+        </is>
+      </c>
       <c r="H91" s="102" t="n"/>
       <c r="I91" s="102" t="n"/>
       <c r="J91" s="102" t="n"/>
     </row>
-    <row r="92" ht="14" customHeight="1" s="132">
+    <row r="92" ht="28" customHeight="1" s="132">
       <c r="A92" s="29" t="n"/>
       <c r="B92" s="30" t="inlineStr">
         <is>
@@ -5112,12 +5111,12 @@
       </c>
       <c r="C92" s="134" t="inlineStr">
         <is>
-          <t>Team Doctor</t>
+          <t>Floor Cleanup</t>
         </is>
       </c>
       <c r="D92" s="91" t="inlineStr">
         <is>
-          <t>Discard 1 Injury from a player of choice. Draw 2 cards if not choosing yourself</t>
+          <t>All players shuffle their hands into the deck and draw the same number of cards</t>
         </is>
       </c>
       <c r="E92" s="7" t="n"/>
@@ -5129,315 +5128,331 @@
       <c r="I92" s="102" t="n"/>
       <c r="J92" s="102" t="n"/>
     </row>
-    <row r="93" ht="28" customHeight="1" s="132">
-      <c r="A93" s="55" t="inlineStr">
-        <is>
-          <t>Injury GB</t>
-        </is>
-      </c>
-      <c r="B93" s="56">
-        <f>COUNTIF($B$5:$B$123,"Injury GB")</f>
-        <v/>
-      </c>
-      <c r="C93" s="57" t="n"/>
-      <c r="D93" s="57" t="n"/>
-      <c r="E93" s="57" t="n"/>
-      <c r="F93" s="88" t="n"/>
-      <c r="G93" s="108" t="n"/>
+    <row r="93" ht="42" customHeight="1" s="132">
+      <c r="A93" s="29" t="n"/>
+      <c r="B93" s="30" t="inlineStr">
+        <is>
+          <t>Game Break</t>
+        </is>
+      </c>
+      <c r="C93" s="134" t="inlineStr">
+        <is>
+          <t>Official Timeout</t>
+        </is>
+      </c>
+      <c r="D93" s="91" t="inlineStr">
+        <is>
+          <t>At least 1 referee must be armed: discard all Injuries on all players and clear all referees. If none, all players draw 1 card</t>
+        </is>
+      </c>
+      <c r="E93" s="7" t="n"/>
+      <c r="F93" s="76" t="n">
+        <v>2</v>
+      </c>
+      <c r="G93" s="111" t="n"/>
       <c r="H93" s="102" t="n"/>
       <c r="I93" s="102" t="n"/>
       <c r="J93" s="102" t="n"/>
     </row>
-    <row r="94" ht="28" customHeight="1" s="132">
+    <row r="94" ht="14" customHeight="1" s="132">
       <c r="A94" s="29" t="n"/>
       <c r="B94" s="30" t="inlineStr">
         <is>
-          <t>Injury GB</t>
-        </is>
-      </c>
-      <c r="C94" s="31" t="inlineStr">
-        <is>
-          <t>Bone Bruise</t>
+          <t>Game Break</t>
+        </is>
+      </c>
+      <c r="C94" s="134" t="inlineStr">
+        <is>
+          <t>Team Doctor</t>
         </is>
       </c>
       <c r="D94" s="91" t="inlineStr">
         <is>
-          <t>Discard 1 card at the start of each turn after drawing (your choice)</t>
+          <t>Discard 1 Injury from a player of choice. Draw 2 cards if not choosing yourself</t>
         </is>
       </c>
       <c r="E94" s="7" t="n"/>
       <c r="F94" s="76" t="n">
         <v>3</v>
       </c>
-      <c r="G94" s="101" t="n"/>
+      <c r="G94" s="111" t="n"/>
       <c r="H94" s="102" t="n"/>
       <c r="I94" s="102" t="n"/>
       <c r="J94" s="102" t="n"/>
     </row>
-    <row r="95" ht="28" customHeight="1" s="132">
-      <c r="A95" s="58" t="inlineStr">
-        <is>
-          <t>Devastating Injury GB</t>
-        </is>
-      </c>
-      <c r="B95" s="59">
-        <f>COUNTIF($B$5:$B$123,"Devastating Injury GB")</f>
-        <v/>
-      </c>
-      <c r="C95" s="60" t="n"/>
-      <c r="D95" s="60" t="n"/>
-      <c r="E95" s="60" t="n"/>
-      <c r="F95" s="86" t="n"/>
-      <c r="G95" s="109" t="n"/>
-      <c r="H95" s="110" t="n"/>
-      <c r="I95" s="110" t="n"/>
-      <c r="J95" s="110" t="n"/>
-    </row>
-    <row r="96" ht="28" customHeight="1" s="132">
-      <c r="A96" s="50" t="n"/>
-      <c r="B96" s="51" t="inlineStr">
-        <is>
-          <t>Devastating Injury GB</t>
-        </is>
-      </c>
-      <c r="C96" s="136" t="inlineStr">
-        <is>
-          <t>Torn Achilles</t>
-        </is>
-      </c>
-      <c r="D96" s="137" t="inlineStr">
-        <is>
-          <t>Hand is locked every turn except 1 card (randomly)</t>
-        </is>
-      </c>
-      <c r="E96" s="54" t="n"/>
-      <c r="F96" s="141" t="n"/>
-      <c r="G96" s="114" t="n"/>
-      <c r="H96" s="115" t="n"/>
-      <c r="I96" s="115" t="n"/>
-      <c r="J96" s="115" t="n"/>
-    </row>
-    <row r="97" ht="42" customHeight="1" s="132">
-      <c r="A97" s="55" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="B97" s="56">
-        <f>COUNTIF($B$5:$B$123,"Intangible")</f>
-        <v/>
-      </c>
-      <c r="C97" s="57" t="n"/>
-      <c r="D97" s="57" t="n"/>
-      <c r="E97" s="57" t="n"/>
-      <c r="F97" s="88" t="n"/>
-      <c r="G97" s="108" t="n"/>
+    <row r="95" ht="14" customHeight="1" s="132">
+      <c r="A95" s="29" t="n"/>
+      <c r="B95" s="30" t="inlineStr">
+        <is>
+          <t>Game Break</t>
+        </is>
+      </c>
+      <c r="C95" s="134" t="inlineStr">
+        <is>
+          <t>Altercation</t>
+        </is>
+      </c>
+      <c r="D95" s="91" t="inlineStr">
+        <is>
+          <t>Select another player: you and that player each discard 1 card at random. Inbound the ball to a player other than that target</t>
+        </is>
+      </c>
+      <c r="E95" s="7" t="n"/>
+      <c r="F95" s="76" t="n">
+        <v>2</v>
+      </c>
+      <c r="G95" s="111" t="n"/>
+      <c r="H95" s="102" t="n"/>
+      <c r="I95" s="102" t="n"/>
+      <c r="J95" s="102" t="n"/>
+    </row>
+    <row r="96" ht="14" customHeight="1" s="132">
+      <c r="A96" s="29" t="n"/>
+      <c r="B96" s="30" t="inlineStr">
+        <is>
+          <t>Game Break</t>
+        </is>
+      </c>
+      <c r="C96" s="134" t="inlineStr">
+        <is>
+          <t>Huge Altercation</t>
+        </is>
+      </c>
+      <c r="D96" s="91" t="inlineStr">
+        <is>
+          <t>All players discard their hands. If a ref is armed, all players receive 1 TOV. Inbound the ball</t>
+        </is>
+      </c>
+      <c r="E96" s="7" t="n"/>
+      <c r="F96" s="76" t="n">
+        <v>1</v>
+      </c>
+      <c r="G96" s="111" t="n"/>
+      <c r="H96" s="102" t="n"/>
+      <c r="I96" s="102" t="n"/>
+      <c r="J96" s="102" t="n"/>
+    </row>
+    <row r="97" ht="14" customHeight="1" s="132">
+      <c r="A97" s="29" t="n"/>
+      <c r="B97" s="30" t="inlineStr">
+        <is>
+          <t>Game Break</t>
+        </is>
+      </c>
+      <c r="C97" s="134" t="inlineStr">
+        <is>
+          <t>Home Court Advantage</t>
+        </is>
+      </c>
+      <c r="D97" s="91" t="inlineStr">
+        <is>
+          <t>SHOT + 10%</t>
+        </is>
+      </c>
+      <c r="E97" s="7" t="n"/>
+      <c r="F97" s="76" t="n">
+        <v>5</v>
+      </c>
+      <c r="G97" s="111" t="n"/>
       <c r="H97" s="102" t="n"/>
       <c r="I97" s="102" t="n"/>
       <c r="J97" s="102" t="n"/>
     </row>
-    <row r="98" ht="56" customHeight="1" s="132">
-      <c r="A98" s="96" t="inlineStr">
-        <is>
-          <t>All intangibles are limited to 1</t>
-        </is>
-      </c>
+    <row r="98" ht="14" customHeight="1" s="132">
+      <c r="A98" s="29" t="n"/>
       <c r="B98" s="30" t="inlineStr">
         <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C98" s="31" t="inlineStr">
-        <is>
-          <t>Board-Crasher</t>
-        </is>
-      </c>
-      <c r="D98" s="6" t="inlineStr">
-        <is>
-          <t>SHOT +10% upon Rebounding your own missed shot</t>
+          <t>Game Break</t>
+        </is>
+      </c>
+      <c r="C98" s="134" t="inlineStr">
+        <is>
+          <t>Away Game</t>
+        </is>
+      </c>
+      <c r="D98" s="91" t="inlineStr">
+        <is>
+          <t>SHOT - 10%</t>
         </is>
       </c>
       <c r="E98" s="7" t="n"/>
-      <c r="F98" s="138" t="n"/>
-      <c r="G98" s="101" t="n"/>
+      <c r="F98" s="76" t="n">
+        <v>5</v>
+      </c>
+      <c r="G98" s="111" t="n"/>
       <c r="H98" s="102" t="n"/>
       <c r="I98" s="102" t="n"/>
       <c r="J98" s="102" t="n"/>
     </row>
-    <row r="99" ht="57" customHeight="1" s="132" thickBot="1">
+    <row r="99" ht="14" customHeight="1" s="132">
       <c r="A99" s="29" t="n"/>
       <c r="B99" s="30" t="inlineStr">
         <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C99" s="32" t="inlineStr">
-        <is>
-          <t>Catch &amp; Shoot Specialist</t>
-        </is>
-      </c>
-      <c r="D99" s="33" t="inlineStr">
-        <is>
-          <t>Additional SHOT +10% on all received passes</t>
-        </is>
-      </c>
-      <c r="E99" s="34" t="n"/>
-      <c r="F99" s="138" t="n"/>
-      <c r="G99" s="107" t="n"/>
+          <t>Game Break</t>
+        </is>
+      </c>
+      <c r="C99" s="134" t="inlineStr">
+        <is>
+          <t>Mic'd Up</t>
+        </is>
+      </c>
+      <c r="D99" s="91" t="inlineStr">
+        <is>
+          <t>SHOT + 10% until passed or shot</t>
+        </is>
+      </c>
+      <c r="E99" s="7" t="n"/>
+      <c r="F99" s="76" t="n">
+        <v>7</v>
+      </c>
+      <c r="G99" s="111" t="inlineStr">
+        <is>
+          <t>The boost is the holder's alone and does not travel with a pass</t>
+        </is>
+      </c>
       <c r="H99" s="102" t="n"/>
       <c r="I99" s="102" t="n"/>
       <c r="J99" s="102" t="n"/>
     </row>
-    <row r="100" ht="20" customHeight="1" s="132">
+    <row r="100" ht="14" customHeight="1" s="132">
       <c r="A100" s="29" t="n"/>
       <c r="B100" s="30" t="inlineStr">
         <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C100" s="31" t="inlineStr">
-        <is>
-          <t>Clutch Gene</t>
-        </is>
-      </c>
-      <c r="D100" s="6" t="inlineStr">
-        <is>
-          <t>SHOT x2 if attempting a shot with 1 or fewer cards in hand or Shot Clock 3 or less</t>
+          <t>Game Break</t>
+        </is>
+      </c>
+      <c r="C100" s="134" t="inlineStr">
+        <is>
+          <t>In The Zone</t>
+        </is>
+      </c>
+      <c r="D100" s="91" t="inlineStr">
+        <is>
+          <t>Draw 1 card for each 10% SHOT the ball has, rounded down. Minimum 1</t>
         </is>
       </c>
       <c r="E100" s="7" t="n"/>
-      <c r="F100" s="138" t="n"/>
-      <c r="G100" s="101" t="n"/>
+      <c r="F100" s="76" t="n">
+        <v>4</v>
+      </c>
+      <c r="G100" s="111" t="n"/>
       <c r="H100" s="102" t="n"/>
       <c r="I100" s="102" t="n"/>
       <c r="J100" s="102" t="n"/>
     </row>
     <row r="101" ht="28" customHeight="1" s="132">
-      <c r="A101" s="29" t="n"/>
-      <c r="B101" s="30" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C101" s="32" t="inlineStr">
-        <is>
-          <t>Floor General</t>
-        </is>
-      </c>
-      <c r="D101" s="33" t="inlineStr">
-        <is>
-          <t>You choose all targets of all kinds — card declarations, non auto-pass targets, and the rest</t>
-        </is>
-      </c>
-      <c r="E101" s="34" t="n"/>
-      <c r="F101" s="138" t="n"/>
-      <c r="G101" s="107" t="n"/>
+      <c r="A101" s="55" t="inlineStr">
+        <is>
+          <t>Injury GB</t>
+        </is>
+      </c>
+      <c r="B101" s="56">
+        <f>COUNTIF($B$5:$B$131,"Injury GB")</f>
+        <v/>
+      </c>
+      <c r="C101" s="57" t="n"/>
+      <c r="D101" s="57" t="n"/>
+      <c r="E101" s="57" t="n"/>
+      <c r="F101" s="88" t="n"/>
+      <c r="G101" s="108" t="n"/>
       <c r="H101" s="102" t="n"/>
       <c r="I101" s="102" t="n"/>
       <c r="J101" s="102" t="n"/>
     </row>
-    <row r="102">
+    <row r="102" ht="28" customHeight="1" s="132">
       <c r="A102" s="29" t="n"/>
       <c r="B102" s="30" t="inlineStr">
         <is>
-          <t>Intangible</t>
+          <t>Injury GB</t>
         </is>
       </c>
       <c r="C102" s="31" t="inlineStr">
         <is>
-          <t>Fox-Like First Step</t>
-        </is>
-      </c>
-      <c r="D102" s="6" t="inlineStr">
-        <is>
-          <t>All Move cards that reduce SHOT increase it by that amount instead.</t>
-        </is>
-      </c>
-      <c r="E102" s="6" t="inlineStr">
-        <is>
-          <t>Your Move cards are unaffected by opponents</t>
-        </is>
-      </c>
-      <c r="F102" s="139" t="n"/>
+          <t>Bone Bruise</t>
+        </is>
+      </c>
+      <c r="D102" s="91" t="inlineStr">
+        <is>
+          <t>Discard 1 card at the start of each turn after drawing (your choice)</t>
+        </is>
+      </c>
+      <c r="E102" s="7" t="n"/>
+      <c r="F102" s="76" t="n">
+        <v>3</v>
+      </c>
       <c r="G102" s="101" t="n"/>
       <c r="H102" s="102" t="n"/>
       <c r="I102" s="102" t="n"/>
       <c r="J102" s="102" t="n"/>
     </row>
-    <row r="103">
-      <c r="A103" s="29" t="n"/>
-      <c r="B103" s="30" t="inlineStr">
+    <row r="103" ht="28" customHeight="1" s="132">
+      <c r="A103" s="58" t="inlineStr">
+        <is>
+          <t>Devastating Injury GB</t>
+        </is>
+      </c>
+      <c r="B103" s="59">
+        <f>COUNTIF($B$5:$B$131,"Devastating Injury GB")</f>
+        <v/>
+      </c>
+      <c r="C103" s="60" t="n"/>
+      <c r="D103" s="60" t="n"/>
+      <c r="E103" s="60" t="n"/>
+      <c r="F103" s="86" t="n"/>
+      <c r="G103" s="109" t="n"/>
+      <c r="H103" s="110" t="n"/>
+      <c r="I103" s="110" t="n"/>
+      <c r="J103" s="110" t="n"/>
+    </row>
+    <row r="104" ht="28" customHeight="1" s="132">
+      <c r="A104" s="50" t="n"/>
+      <c r="B104" s="51" t="inlineStr">
+        <is>
+          <t>Devastating Injury GB</t>
+        </is>
+      </c>
+      <c r="C104" s="136" t="inlineStr">
+        <is>
+          <t>Torn Achilles</t>
+        </is>
+      </c>
+      <c r="D104" s="137" t="inlineStr">
+        <is>
+          <t>Hand is locked every turn except 1 card (randomly)</t>
+        </is>
+      </c>
+      <c r="E104" s="54" t="n"/>
+      <c r="F104" s="141" t="n"/>
+      <c r="G104" s="114" t="n"/>
+      <c r="H104" s="115" t="n"/>
+      <c r="I104" s="115" t="n"/>
+      <c r="J104" s="115" t="n"/>
+    </row>
+    <row r="105" ht="42" customHeight="1" s="132">
+      <c r="A105" s="55" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C103" s="90" t="inlineStr">
-        <is>
-          <t>Freethrow Merchant</t>
-        </is>
-      </c>
-      <c r="D103" s="94" t="inlineStr">
-        <is>
-          <t>All Clamps on you grant 1 FT instead</t>
-        </is>
-      </c>
-      <c r="E103" s="34" t="n"/>
-      <c r="F103" s="138" t="n"/>
-      <c r="G103" s="125" t="n"/>
-      <c r="H103" s="102" t="n"/>
-      <c r="I103" s="102" t="n"/>
-      <c r="J103" s="102" t="n"/>
-    </row>
-    <row r="104">
-      <c r="A104" s="29" t="n"/>
-      <c r="B104" s="30" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C104" s="90" t="inlineStr">
-        <is>
-          <t>Generational Whistle</t>
-        </is>
-      </c>
-      <c r="D104" s="91" t="inlineStr">
-        <is>
-          <t>Take 1 additional FT</t>
-        </is>
-      </c>
-      <c r="E104" s="7" t="n"/>
-      <c r="F104" s="138" t="n"/>
-      <c r="G104" s="101" t="n"/>
-      <c r="H104" s="102" t="n"/>
-      <c r="I104" s="102" t="n"/>
-      <c r="J104" s="102" t="n"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="29" t="n"/>
-      <c r="B105" s="30" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C105" s="32" t="inlineStr">
-        <is>
-          <t>Gravity</t>
-        </is>
-      </c>
-      <c r="D105" s="33" t="inlineStr">
-        <is>
-          <t>All Clamps automatically apply to you. +1 AST whenever another player attempts a shot</t>
-        </is>
-      </c>
-      <c r="E105" s="34" t="n"/>
-      <c r="F105" s="138" t="n"/>
-      <c r="G105" s="107" t="n"/>
+      <c r="B105" s="56">
+        <f>COUNTIF($B$5:$B$131,"Intangible")</f>
+        <v/>
+      </c>
+      <c r="C105" s="57" t="n"/>
+      <c r="D105" s="57" t="n"/>
+      <c r="E105" s="57" t="n"/>
+      <c r="F105" s="88" t="n"/>
+      <c r="G105" s="108" t="n"/>
       <c r="H105" s="102" t="n"/>
       <c r="I105" s="102" t="n"/>
       <c r="J105" s="102" t="n"/>
     </row>
-    <row r="106">
-      <c r="A106" s="29" t="n"/>
+    <row r="106" ht="56" customHeight="1" s="132">
+      <c r="A106" s="96" t="inlineStr">
+        <is>
+          <t>All intangibles are limited to 1</t>
+        </is>
+      </c>
       <c r="B106" s="30" t="inlineStr">
         <is>
           <t>Intangible</t>
@@ -5445,12 +5460,12 @@
       </c>
       <c r="C106" s="31" t="inlineStr">
         <is>
-          <t>Great Conditioning</t>
+          <t>Board-Crasher</t>
         </is>
       </c>
       <c r="D106" s="6" t="inlineStr">
         <is>
-          <t>Immediately discard all Injury Game Breaks you draw and draw a new card for each</t>
+          <t>SHOT +10% upon Rebounding your own missed shot</t>
         </is>
       </c>
       <c r="E106" s="7" t="n"/>
@@ -5460,7 +5475,7 @@
       <c r="I106" s="102" t="n"/>
       <c r="J106" s="102" t="n"/>
     </row>
-    <row r="107">
+    <row r="107" ht="57" customHeight="1" s="132">
       <c r="A107" s="29" t="n"/>
       <c r="B107" s="30" t="inlineStr">
         <is>
@@ -5469,12 +5484,12 @@
       </c>
       <c r="C107" s="32" t="inlineStr">
         <is>
-          <t>Hot Hand</t>
+          <t>Catch &amp; Shoot Specialist</t>
         </is>
       </c>
       <c r="D107" s="33" t="inlineStr">
         <is>
-          <t>SHOT +20% if you scored last round.</t>
+          <t>Additional SHOT +10% on all received passes</t>
         </is>
       </c>
       <c r="E107" s="34" t="n"/>
@@ -5484,7 +5499,7 @@
       <c r="I107" s="102" t="n"/>
       <c r="J107" s="102" t="n"/>
     </row>
-    <row r="108">
+    <row r="108" ht="20" customHeight="1" s="132">
       <c r="A108" s="29" t="n"/>
       <c r="B108" s="30" t="inlineStr">
         <is>
@@ -5493,12 +5508,12 @@
       </c>
       <c r="C108" s="31" t="inlineStr">
         <is>
-          <t>Like That</t>
-        </is>
-      </c>
-      <c r="D108" s="91" t="inlineStr">
-        <is>
-          <t>Your SHOT % cannot be reduced</t>
+          <t>Clutch Gene</t>
+        </is>
+      </c>
+      <c r="D108" s="6" t="inlineStr">
+        <is>
+          <t>SHOT x2 if attempting a shot with 1 or fewer cards in hand or Shot Clock 3 or less</t>
         </is>
       </c>
       <c r="E108" s="7" t="n"/>
@@ -5508,7 +5523,7 @@
       <c r="I108" s="102" t="n"/>
       <c r="J108" s="102" t="n"/>
     </row>
-    <row r="109">
+    <row r="109" ht="28" customHeight="1" s="132">
       <c r="A109" s="29" t="n"/>
       <c r="B109" s="30" t="inlineStr">
         <is>
@@ -5517,21 +5532,17 @@
       </c>
       <c r="C109" s="32" t="inlineStr">
         <is>
-          <t>No Bag</t>
+          <t>Floor General</t>
         </is>
       </c>
       <c r="D109" s="33" t="inlineStr">
         <is>
-          <t>Cannot activate Move cards this round</t>
+          <t>You choose all targets of all kinds — card declarations, non auto-pass targets, and the rest</t>
         </is>
       </c>
       <c r="E109" s="34" t="n"/>
       <c r="F109" s="138" t="n"/>
-      <c r="G109" s="113" t="inlineStr">
-        <is>
-          <t>Bad card to draw</t>
-        </is>
-      </c>
+      <c r="G109" s="107" t="n"/>
       <c r="H109" s="102" t="n"/>
       <c r="I109" s="102" t="n"/>
       <c r="J109" s="102" t="n"/>
@@ -5545,16 +5556,20 @@
       </c>
       <c r="C110" s="31" t="inlineStr">
         <is>
-          <t>Point God</t>
+          <t>Fox-Like First Step</t>
         </is>
       </c>
       <c r="D110" s="6" t="inlineStr">
         <is>
-          <t>Draw 1 card following each of your passes</t>
-        </is>
-      </c>
-      <c r="E110" s="7" t="n"/>
-      <c r="F110" s="138" t="n"/>
+          <t>All Move cards that reduce SHOT increase it by that amount instead.</t>
+        </is>
+      </c>
+      <c r="E110" s="6" t="inlineStr">
+        <is>
+          <t>Your Move cards are unaffected by opponents</t>
+        </is>
+      </c>
+      <c r="F110" s="139" t="n"/>
       <c r="G110" s="101" t="n"/>
       <c r="H110" s="102" t="n"/>
       <c r="I110" s="102" t="n"/>
@@ -5567,23 +5582,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C111" s="32" t="inlineStr">
-        <is>
-          <t>Shooting Slump</t>
-        </is>
-      </c>
-      <c r="D111" s="33" t="inlineStr">
-        <is>
-          <t>SHOT -20% this round</t>
+      <c r="C111" s="90" t="inlineStr">
+        <is>
+          <t>Freethrow Merchant</t>
+        </is>
+      </c>
+      <c r="D111" s="94" t="inlineStr">
+        <is>
+          <t>All Clamps on you grant 1 FT instead</t>
         </is>
       </c>
       <c r="E111" s="34" t="n"/>
       <c r="F111" s="138" t="n"/>
-      <c r="G111" s="113" t="inlineStr">
-        <is>
-          <t>Bad card to draw</t>
-        </is>
-      </c>
+      <c r="G111" s="125" t="n"/>
       <c r="H111" s="102" t="n"/>
       <c r="I111" s="102" t="n"/>
       <c r="J111" s="102" t="n"/>
@@ -5595,14 +5606,14 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C112" s="31" t="inlineStr">
-        <is>
-          <t>Shot Creator</t>
-        </is>
-      </c>
-      <c r="D112" s="6" t="inlineStr">
-        <is>
-          <t>Draw 1 additional card after every draw effect</t>
+      <c r="C112" s="90" t="inlineStr">
+        <is>
+          <t>Generational Whistle</t>
+        </is>
+      </c>
+      <c r="D112" s="91" t="inlineStr">
+        <is>
+          <t>Take 1 additional FT</t>
         </is>
       </c>
       <c r="E112" s="7" t="n"/>
@@ -5621,12 +5632,12 @@
       </c>
       <c r="C113" s="32" t="inlineStr">
         <is>
-          <t>Sixth Man</t>
+          <t>Gravity</t>
         </is>
       </c>
       <c r="D113" s="33" t="inlineStr">
         <is>
-          <t>SHOT = 100% if taking 6th shot of the round</t>
+          <t>All Clamps automatically apply to you. +1 AST whenever another player attempts a shot</t>
         </is>
       </c>
       <c r="E113" s="34" t="n"/>
@@ -5645,12 +5656,12 @@
       </c>
       <c r="C114" s="31" t="inlineStr">
         <is>
-          <t>Sniper</t>
+          <t>Great Conditioning</t>
         </is>
       </c>
       <c r="D114" s="6" t="inlineStr">
         <is>
-          <t>SHOT +10% on all Three-Point Line Shots</t>
+          <t>Immediately discard all Injury Game Breaks you draw and draw a new card for each</t>
         </is>
       </c>
       <c r="E114" s="7" t="n"/>
@@ -5669,12 +5680,12 @@
       </c>
       <c r="C115" s="32" t="inlineStr">
         <is>
-          <t>Splash Cousin</t>
+          <t>Hot Hand</t>
         </is>
       </c>
       <c r="D115" s="33" t="inlineStr">
         <is>
-          <t>All Three-Point Line Shots: SHOT = 100%</t>
+          <t>SHOT +20% if you scored last round.</t>
         </is>
       </c>
       <c r="E115" s="34" t="n"/>
@@ -5693,12 +5704,12 @@
       </c>
       <c r="C116" s="31" t="inlineStr">
         <is>
-          <t>Unguardable</t>
+          <t>Like That</t>
         </is>
       </c>
       <c r="D116" s="91" t="inlineStr">
         <is>
-          <t>All Clamps on you have no effect on SHOT %</t>
+          <t>Your SHOT % cannot be reduced</t>
         </is>
       </c>
       <c r="E116" s="7" t="n"/>
@@ -5717,19 +5728,19 @@
       </c>
       <c r="C117" s="32" t="inlineStr">
         <is>
-          <t>Lethal Shooter</t>
+          <t>No Bag</t>
         </is>
       </c>
       <c r="D117" s="33" t="inlineStr">
         <is>
-          <t>SHOT = 100% on next shot attempt after rebounding your own miss.</t>
+          <t>Cannot activate Move cards this round</t>
         </is>
       </c>
       <c r="E117" s="34" t="n"/>
       <c r="F117" s="138" t="n"/>
       <c r="G117" s="113" t="inlineStr">
         <is>
-          <t>Special text: “I understand it now”</t>
+          <t>Bad card to draw</t>
         </is>
       </c>
       <c r="H117" s="102" t="n"/>
@@ -5737,173 +5748,375 @@
       <c r="J117" s="102" t="n"/>
     </row>
     <row r="118">
-      <c r="A118" s="61" t="n"/>
-      <c r="B118" s="62" t="inlineStr">
+      <c r="A118" s="29" t="n"/>
+      <c r="B118" s="30" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C118" s="66" t="inlineStr">
+      <c r="C118" s="31" t="inlineStr">
+        <is>
+          <t>Point God</t>
+        </is>
+      </c>
+      <c r="D118" s="6" t="inlineStr">
+        <is>
+          <t>Draw 1 card following each of your passes</t>
+        </is>
+      </c>
+      <c r="E118" s="7" t="n"/>
+      <c r="F118" s="138" t="n"/>
+      <c r="G118" s="101" t="n"/>
+      <c r="H118" s="102" t="n"/>
+      <c r="I118" s="102" t="n"/>
+      <c r="J118" s="102" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="29" t="n"/>
+      <c r="B119" s="30" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C119" s="32" t="inlineStr">
+        <is>
+          <t>Shooting Slump</t>
+        </is>
+      </c>
+      <c r="D119" s="33" t="inlineStr">
+        <is>
+          <t>SHOT -20% this round</t>
+        </is>
+      </c>
+      <c r="E119" s="34" t="n"/>
+      <c r="F119" s="138" t="n"/>
+      <c r="G119" s="113" t="inlineStr">
+        <is>
+          <t>Bad card to draw</t>
+        </is>
+      </c>
+      <c r="H119" s="102" t="n"/>
+      <c r="I119" s="102" t="n"/>
+      <c r="J119" s="102" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="29" t="n"/>
+      <c r="B120" s="30" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C120" s="31" t="inlineStr">
+        <is>
+          <t>Shot Creator</t>
+        </is>
+      </c>
+      <c r="D120" s="6" t="inlineStr">
+        <is>
+          <t>Draw 1 additional card after every draw effect</t>
+        </is>
+      </c>
+      <c r="E120" s="7" t="n"/>
+      <c r="F120" s="138" t="n"/>
+      <c r="G120" s="101" t="n"/>
+      <c r="H120" s="102" t="n"/>
+      <c r="I120" s="102" t="n"/>
+      <c r="J120" s="102" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="29" t="n"/>
+      <c r="B121" s="30" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C121" s="32" t="inlineStr">
+        <is>
+          <t>Sixth Man</t>
+        </is>
+      </c>
+      <c r="D121" s="33" t="inlineStr">
+        <is>
+          <t>SHOT = 100% if taking 6th shot of the round</t>
+        </is>
+      </c>
+      <c r="E121" s="34" t="n"/>
+      <c r="F121" s="138" t="n"/>
+      <c r="G121" s="107" t="n"/>
+      <c r="H121" s="102" t="n"/>
+      <c r="I121" s="102" t="n"/>
+      <c r="J121" s="102" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="29" t="n"/>
+      <c r="B122" s="30" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C122" s="31" t="inlineStr">
+        <is>
+          <t>Sniper</t>
+        </is>
+      </c>
+      <c r="D122" s="6" t="inlineStr">
+        <is>
+          <t>SHOT +10% on all Three-Point Line Shots</t>
+        </is>
+      </c>
+      <c r="E122" s="7" t="n"/>
+      <c r="F122" s="138" t="n"/>
+      <c r="G122" s="101" t="n"/>
+      <c r="H122" s="102" t="n"/>
+      <c r="I122" s="102" t="n"/>
+      <c r="J122" s="102" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="29" t="n"/>
+      <c r="B123" s="30" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C123" s="32" t="inlineStr">
+        <is>
+          <t>Splash Cousin</t>
+        </is>
+      </c>
+      <c r="D123" s="33" t="inlineStr">
+        <is>
+          <t>All Three-Point Line Shots: SHOT = 100%</t>
+        </is>
+      </c>
+      <c r="E123" s="34" t="n"/>
+      <c r="F123" s="138" t="n"/>
+      <c r="G123" s="107" t="n"/>
+      <c r="H123" s="102" t="n"/>
+      <c r="I123" s="102" t="n"/>
+      <c r="J123" s="102" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="29" t="n"/>
+      <c r="B124" s="30" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C124" s="31" t="inlineStr">
+        <is>
+          <t>Unguardable</t>
+        </is>
+      </c>
+      <c r="D124" s="91" t="inlineStr">
+        <is>
+          <t>All Clamps on you have no effect on SHOT %</t>
+        </is>
+      </c>
+      <c r="E124" s="7" t="n"/>
+      <c r="F124" s="138" t="n"/>
+      <c r="G124" s="101" t="n"/>
+      <c r="H124" s="102" t="n"/>
+      <c r="I124" s="102" t="n"/>
+      <c r="J124" s="102" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="29" t="n"/>
+      <c r="B125" s="30" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C125" s="32" t="inlineStr">
+        <is>
+          <t>Lethal Shooter</t>
+        </is>
+      </c>
+      <c r="D125" s="33" t="inlineStr">
+        <is>
+          <t>SHOT = 100% on next shot attempt after rebounding your own miss.</t>
+        </is>
+      </c>
+      <c r="E125" s="34" t="n"/>
+      <c r="F125" s="138" t="n"/>
+      <c r="G125" s="113" t="inlineStr">
+        <is>
+          <t>Special text: “I understand it now”</t>
+        </is>
+      </c>
+      <c r="H125" s="102" t="n"/>
+      <c r="I125" s="102" t="n"/>
+      <c r="J125" s="102" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="61" t="n"/>
+      <c r="B126" s="62" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C126" s="66" t="inlineStr">
         <is>
           <t>Ball Pounder</t>
         </is>
       </c>
-      <c r="D118" s="95" t="inlineStr">
+      <c r="D126" s="95" t="inlineStr">
         <is>
           <t>All Dribble cards you play draw an additional card but lower SHOT by an additional 10%</t>
         </is>
       </c>
-      <c r="E118" s="68" t="n"/>
-      <c r="F118" s="140" t="n"/>
-      <c r="G118" s="126" t="n"/>
-      <c r="H118" s="117" t="n"/>
-      <c r="I118" s="117" t="n"/>
-      <c r="J118" s="117" t="n"/>
-    </row>
-    <row r="119">
-      <c r="A119" s="61" t="n"/>
-      <c r="B119" s="62" t="inlineStr">
+      <c r="E126" s="68" t="n"/>
+      <c r="F126" s="140" t="n"/>
+      <c r="G126" s="126" t="n"/>
+      <c r="H126" s="117" t="n"/>
+      <c r="I126" s="117" t="n"/>
+      <c r="J126" s="117" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="61" t="n"/>
+      <c r="B127" s="62" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C119" s="66" t="inlineStr">
+      <c r="C127" s="66" t="inlineStr">
         <is>
           <t>Unselfish</t>
         </is>
       </c>
-      <c r="D119" s="95" t="inlineStr">
+      <c r="D127" s="95" t="inlineStr">
         <is>
           <t>Draw 1 card and increase next SHOT +5% whenever you positively affect another player</t>
         </is>
       </c>
-      <c r="E119" s="68" t="n"/>
-      <c r="F119" s="140" t="n"/>
-      <c r="G119" s="126" t="n"/>
-      <c r="H119" s="117" t="n"/>
-      <c r="I119" s="117" t="n"/>
-      <c r="J119" s="117" t="n"/>
-    </row>
-    <row r="120">
-      <c r="A120" s="61" t="n"/>
-      <c r="B120" s="62" t="inlineStr">
+      <c r="E127" s="68" t="n"/>
+      <c r="F127" s="140" t="n"/>
+      <c r="G127" s="126" t="n"/>
+      <c r="H127" s="117" t="n"/>
+      <c r="I127" s="117" t="n"/>
+      <c r="J127" s="117" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="61" t="n"/>
+      <c r="B128" s="62" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C120" s="66" t="inlineStr">
+      <c r="C128" s="66" t="inlineStr">
         <is>
           <t>Dirty Player</t>
         </is>
       </c>
-      <c r="D120" s="95" t="inlineStr">
+      <c r="D128" s="95" t="inlineStr">
         <is>
           <t>When sending Clamps, the clamped player discards 1 if they have any Injuries</t>
         </is>
       </c>
-      <c r="E120" s="68" t="n"/>
-      <c r="F120" s="140" t="n"/>
-      <c r="G120" s="126" t="n"/>
-      <c r="H120" s="117" t="n"/>
-      <c r="I120" s="117" t="n"/>
-      <c r="J120" s="117" t="n"/>
-    </row>
-    <row r="121">
-      <c r="A121" s="61" t="n"/>
-      <c r="B121" s="62" t="inlineStr">
+      <c r="E128" s="68" t="n"/>
+      <c r="F128" s="140" t="n"/>
+      <c r="G128" s="126" t="n"/>
+      <c r="H128" s="117" t="n"/>
+      <c r="I128" s="117" t="n"/>
+      <c r="J128" s="117" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="61" t="n"/>
+      <c r="B129" s="62" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C121" s="66" t="inlineStr">
+      <c r="C129" s="66" t="inlineStr">
         <is>
           <t>Villainous Reputation</t>
         </is>
       </c>
-      <c r="D121" s="95" t="inlineStr">
+      <c r="D129" s="95" t="inlineStr">
         <is>
           <t>Discard 1 whenever any Whistle triggers</t>
         </is>
       </c>
-      <c r="E121" s="68" t="n"/>
-      <c r="F121" s="140" t="n"/>
-      <c r="G121" s="126" t="inlineStr">
+      <c r="E129" s="68" t="n"/>
+      <c r="F129" s="140" t="n"/>
+      <c r="G129" s="126" t="inlineStr">
         <is>
           <t>Discarded during play, it attaches to a random player — possibly you again</t>
         </is>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" s="61" t="n"/>
-      <c r="B122" s="62" t="inlineStr">
+    <row r="130">
+      <c r="A130" s="61" t="n"/>
+      <c r="B130" s="62" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C122" s="66" t="inlineStr">
+      <c r="C130" s="66" t="inlineStr">
         <is>
           <t>Free Agent</t>
         </is>
       </c>
-      <c r="D122" s="95" t="inlineStr">
+      <c r="D130" s="95" t="inlineStr">
         <is>
           <t>Discard your hand. Play a card at random from a player of your choosing (they keep it)</t>
         </is>
       </c>
-      <c r="E122" s="68" t="n"/>
-      <c r="F122" s="140" t="n"/>
-      <c r="G122" s="126" t="inlineStr">
+      <c r="E130" s="68" t="n"/>
+      <c r="F130" s="140" t="n"/>
+      <c r="G130" s="126" t="inlineStr">
         <is>
           <t>The discard waits for the draw chain to finish. Target is shuffled first and is affected by Floor General. Your own draws are kept. All-0 rebounds are yours; otherwise you cannot bid</t>
         </is>
       </c>
     </row>
-    <row r="123">
-      <c r="A123" s="61" t="n"/>
-      <c r="B123" s="62" t="inlineStr">
+    <row r="131">
+      <c r="A131" s="61" t="n"/>
+      <c r="B131" s="62" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C123" s="66" t="inlineStr">
+      <c r="C131" s="66" t="inlineStr">
         <is>
           <t>Franchise Player</t>
         </is>
       </c>
-      <c r="D123" s="95" t="inlineStr">
+      <c r="D131" s="95" t="inlineStr">
         <is>
           <t>When passing, choose 1 of the new player's Intangibles or a card in their hand for them to discard</t>
         </is>
       </c>
-      <c r="E123" s="68" t="n"/>
-      <c r="F123" s="140" t="n"/>
-      <c r="G123" s="126" t="n"/>
-      <c r="H123" s="117" t="n"/>
-      <c r="I123" s="117" t="n"/>
-      <c r="J123" s="117" t="n"/>
+      <c r="E131" s="68" t="n"/>
+      <c r="F131" s="140" t="n"/>
+      <c r="G131" s="126" t="n"/>
+      <c r="H131" s="117" t="n"/>
+      <c r="I131" s="117" t="n"/>
+      <c r="J131" s="117" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="110">
+  <mergeCells count="118">
     <mergeCell ref="G55:J55"/>
     <mergeCell ref="G4:J4"/>
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
+    <mergeCell ref="G119:J119"/>
     <mergeCell ref="G32:J32"/>
-    <mergeCell ref="G119:J119"/>
     <mergeCell ref="G46:J46"/>
     <mergeCell ref="G40:J40"/>
     <mergeCell ref="G111:J111"/>
     <mergeCell ref="G72:J72"/>
     <mergeCell ref="G81:J81"/>
     <mergeCell ref="G96:J96"/>
-    <mergeCell ref="G5:J5"/>
     <mergeCell ref="G71:J71"/>
     <mergeCell ref="G8:J8"/>
+    <mergeCell ref="G82:J82"/>
     <mergeCell ref="G57:J57"/>
+    <mergeCell ref="G128:J128"/>
     <mergeCell ref="G10:J10"/>
     <mergeCell ref="G66:J66"/>
     <mergeCell ref="G18:J18"/>
     <mergeCell ref="G53:J53"/>
+    <mergeCell ref="G121:J121"/>
     <mergeCell ref="G34:J34"/>
     <mergeCell ref="G74:J74"/>
     <mergeCell ref="G68:J68"/>
@@ -5913,14 +6126,13 @@
     <mergeCell ref="G123:J123"/>
     <mergeCell ref="G110:J110"/>
     <mergeCell ref="G113:J113"/>
-    <mergeCell ref="G91:J91"/>
     <mergeCell ref="G20:J20"/>
+    <mergeCell ref="G85:J85"/>
     <mergeCell ref="G100:J100"/>
     <mergeCell ref="G94:J94"/>
     <mergeCell ref="G75:J75"/>
+    <mergeCell ref="G44:J44"/>
     <mergeCell ref="G22:J22"/>
-    <mergeCell ref="G44:J44"/>
-    <mergeCell ref="G31:J31"/>
     <mergeCell ref="G102:J102"/>
     <mergeCell ref="G12:J12"/>
     <mergeCell ref="G77:J77"/>
@@ -5931,11 +6143,13 @@
     <mergeCell ref="G48:J48"/>
     <mergeCell ref="G23:J23"/>
     <mergeCell ref="G97:J97"/>
+    <mergeCell ref="G125:J125"/>
     <mergeCell ref="G7:J7"/>
     <mergeCell ref="G38:J38"/>
     <mergeCell ref="G112:J112"/>
     <mergeCell ref="G45:J45"/>
     <mergeCell ref="G62:J62"/>
+    <mergeCell ref="G127:J127"/>
     <mergeCell ref="G49:J49"/>
     <mergeCell ref="G24:J24"/>
     <mergeCell ref="G33:J33"/>
@@ -5946,15 +6160,17 @@
     <mergeCell ref="G16:J16"/>
     <mergeCell ref="G76:J76"/>
     <mergeCell ref="G25:J25"/>
-    <mergeCell ref="G90:J90"/>
     <mergeCell ref="G99:J99"/>
     <mergeCell ref="G60:J60"/>
+    <mergeCell ref="G131:J131"/>
     <mergeCell ref="G9:J9"/>
     <mergeCell ref="G59:J59"/>
     <mergeCell ref="G115:J115"/>
     <mergeCell ref="G11:J11"/>
     <mergeCell ref="G117:J117"/>
+    <mergeCell ref="G126:J126"/>
     <mergeCell ref="G39:J39"/>
+    <mergeCell ref="G122:J122"/>
     <mergeCell ref="G101:J101"/>
     <mergeCell ref="G116:J116"/>
     <mergeCell ref="G103:J103"/>
@@ -5963,12 +6179,12 @@
     <mergeCell ref="G13:J13"/>
     <mergeCell ref="G78:J78"/>
     <mergeCell ref="G118:J118"/>
-    <mergeCell ref="G87:J87"/>
     <mergeCell ref="G15:J15"/>
+    <mergeCell ref="G80:J80"/>
     <mergeCell ref="G95:J95"/>
-    <mergeCell ref="G80:J80"/>
+    <mergeCell ref="G89:J89"/>
+    <mergeCell ref="G64:J64"/>
     <mergeCell ref="G79:J79"/>
-    <mergeCell ref="G64:J64"/>
     <mergeCell ref="G73:J73"/>
     <mergeCell ref="G51:J51"/>
     <mergeCell ref="G54:J54"/>
@@ -5977,7 +6193,6 @@
     <mergeCell ref="G50:J50"/>
     <mergeCell ref="G106:J106"/>
     <mergeCell ref="G56:J56"/>
-    <mergeCell ref="G14:J14"/>
     <mergeCell ref="G105:J105"/>
     <mergeCell ref="G43:J43"/>
     <mergeCell ref="G52:J52"/>
@@ -5989,11 +6204,15 @@
     <mergeCell ref="G107:J107"/>
     <mergeCell ref="G17:J17"/>
     <mergeCell ref="G19:J19"/>
+    <mergeCell ref="G28:J28"/>
+    <mergeCell ref="G93:J93"/>
     <mergeCell ref="G6:J6"/>
-    <mergeCell ref="G93:J93"/>
     <mergeCell ref="G69:J69"/>
     <mergeCell ref="G83:J83"/>
     <mergeCell ref="G92:J92"/>
+    <mergeCell ref="G124:J124"/>
+    <mergeCell ref="G5:J5"/>
+    <mergeCell ref="G14:J14"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
The sheet's rules, and the counts that counted themselves
**Circular references.** Every section header's COUNTIF ran from `$B$5`, and the
headers sit in column B — so each one was inside the range it counted. Each now
starts on the row below itself, which loses nothing: a section's rows are all
under its header. The Totals row keeps the full range, since it sits above it.

**Borders.** Inserting a row copies the style of the row above it, so every card
added under a section's last row inherited that section's closing rule and drew
one of its own — seven of them through the passes, six through the Intangibles.
Moving the Devastating rows left their old boundary behind the same way. Redrawn
from the rule rather than patched: a medium line between sections, thin
everywhere else, and the table closed at the bottom.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -176,7 +176,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="50">
+  <borders count="58">
     <border>
       <left/>
       <right/>
@@ -829,13 +829,109 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="10"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="10"/>
+      </left>
+      <right style="thin">
+        <color indexed="10"/>
+      </right>
+      <top style="medium">
+        <color indexed="8"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="10"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="10"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="8"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="10"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="8"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="10"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="10"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="10"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="10"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="142">
+  <cellXfs count="165">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1237,6 +1333,69 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="14" fillId="4" borderId="52" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="52" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="52" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="52" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="53" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="55" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="55" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="55" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2659,7 +2818,6 @@
       </c>
       <c r="J2" s="19" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="20.75" customHeight="1" s="132">
       <c r="A4" s="123" t="inlineStr">
         <is>
@@ -2687,59 +2845,59 @@
           <t>Number in Deck</t>
         </is>
       </c>
-      <c r="G4" s="103" t="inlineStr">
+      <c r="G4" s="142" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="H4" s="104" t="n"/>
-      <c r="I4" s="104" t="n"/>
-      <c r="J4" s="104" t="n"/>
+      <c r="H4" s="143" t="n"/>
+      <c r="I4" s="143" t="n"/>
+      <c r="J4" s="143" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1" s="132">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="144" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="B5" s="22">
-        <f>COUNTIF($B$5:$B$135,"Pass")</f>
+      <c r="B5" s="145">
+        <f>COUNTIF($B$6:$B$135,"Pass")</f>
         <v/>
       </c>
-      <c r="C5" s="23" t="n"/>
-      <c r="D5" s="23" t="n"/>
-      <c r="E5" s="23" t="n"/>
-      <c r="F5" s="72" t="n"/>
-      <c r="G5" s="120" t="n"/>
-      <c r="H5" s="121" t="n"/>
-      <c r="I5" s="121" t="n"/>
-      <c r="J5" s="121" t="n"/>
+      <c r="C5" s="146" t="n"/>
+      <c r="D5" s="146" t="n"/>
+      <c r="E5" s="146" t="n"/>
+      <c r="F5" s="147" t="n"/>
+      <c r="G5" s="148" t="n"/>
+      <c r="H5" s="149" t="n"/>
+      <c r="I5" s="149" t="n"/>
+      <c r="J5" s="149" t="n"/>
     </row>
     <row r="6" ht="56" customHeight="1" s="132">
-      <c r="A6" s="24" t="n"/>
-      <c r="B6" s="25" t="inlineStr">
+      <c r="A6" s="29" t="n"/>
+      <c r="B6" s="30" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="C6" s="26" t="inlineStr">
+      <c r="C6" s="32" t="inlineStr">
         <is>
           <t>Behind-the-Back</t>
         </is>
       </c>
-      <c r="D6" s="27" t="inlineStr">
+      <c r="D6" s="33" t="inlineStr">
         <is>
           <t>Pass back to player who passed to you. If ball not received from a player, TOV +1</t>
         </is>
       </c>
-      <c r="E6" s="28" t="n"/>
-      <c r="F6" s="73" t="n">
+      <c r="E6" s="34" t="n"/>
+      <c r="F6" s="75" t="n">
         <v>5</v>
       </c>
-      <c r="G6" s="105" t="n"/>
-      <c r="H6" s="106" t="n"/>
-      <c r="I6" s="106" t="n"/>
-      <c r="J6" s="106" t="n"/>
+      <c r="G6" s="107" t="n"/>
+      <c r="H6" s="102" t="n"/>
+      <c r="I6" s="102" t="n"/>
+      <c r="J6" s="102" t="n"/>
     </row>
     <row r="7" ht="28" customHeight="1" s="132">
       <c r="A7" s="29" t="n"/>
@@ -2766,10 +2924,10 @@
       <c r="F7" s="74" t="n">
         <v>10</v>
       </c>
-      <c r="G7" s="112" t="n"/>
-      <c r="H7" s="106" t="n"/>
-      <c r="I7" s="106" t="n"/>
-      <c r="J7" s="106" t="n"/>
+      <c r="G7" s="101" t="n"/>
+      <c r="H7" s="102" t="n"/>
+      <c r="I7" s="102" t="n"/>
+      <c r="J7" s="102" t="n"/>
     </row>
     <row r="8" ht="56" customHeight="1" s="132">
       <c r="A8" s="29" t="n"/>
@@ -2792,10 +2950,10 @@
       <c r="F8" s="75" t="n">
         <v>6</v>
       </c>
-      <c r="G8" s="105" t="n"/>
-      <c r="H8" s="106" t="n"/>
-      <c r="I8" s="106" t="n"/>
-      <c r="J8" s="106" t="n"/>
+      <c r="G8" s="107" t="n"/>
+      <c r="H8" s="102" t="n"/>
+      <c r="I8" s="102" t="n"/>
+      <c r="J8" s="102" t="n"/>
     </row>
     <row r="9" ht="56" customHeight="1" s="132">
       <c r="A9" s="29" t="n"/>
@@ -2818,10 +2976,10 @@
       <c r="F9" s="76" t="n">
         <v>6</v>
       </c>
-      <c r="G9" s="112" t="n"/>
-      <c r="H9" s="106" t="n"/>
-      <c r="I9" s="106" t="n"/>
-      <c r="J9" s="106" t="n"/>
+      <c r="G9" s="101" t="n"/>
+      <c r="H9" s="102" t="n"/>
+      <c r="I9" s="102" t="n"/>
+      <c r="J9" s="102" t="n"/>
     </row>
     <row r="10" ht="14" customHeight="1" s="132">
       <c r="A10" s="29" t="n"/>
@@ -2844,10 +3002,10 @@
       <c r="F10" s="75" t="n">
         <v>20</v>
       </c>
-      <c r="G10" s="105" t="n"/>
-      <c r="H10" s="106" t="n"/>
-      <c r="I10" s="106" t="n"/>
-      <c r="J10" s="106" t="n"/>
+      <c r="G10" s="107" t="n"/>
+      <c r="H10" s="102" t="n"/>
+      <c r="I10" s="102" t="n"/>
+      <c r="J10" s="102" t="n"/>
     </row>
     <row r="11" ht="14" customHeight="1" s="132">
       <c r="A11" s="29" t="n"/>
@@ -2870,10 +3028,10 @@
       <c r="F11" s="76" t="n">
         <v>31</v>
       </c>
-      <c r="G11" s="112" t="n"/>
-      <c r="H11" s="106" t="n"/>
-      <c r="I11" s="106" t="n"/>
-      <c r="J11" s="106" t="n"/>
+      <c r="G11" s="101" t="n"/>
+      <c r="H11" s="102" t="n"/>
+      <c r="I11" s="102" t="n"/>
+      <c r="J11" s="102" t="n"/>
     </row>
     <row r="12" ht="14" customHeight="1" s="132">
       <c r="A12" s="29" t="n"/>
@@ -2896,10 +3054,10 @@
       <c r="F12" s="75" t="n">
         <v>31</v>
       </c>
-      <c r="G12" s="105" t="n"/>
-      <c r="H12" s="106" t="n"/>
-      <c r="I12" s="106" t="n"/>
-      <c r="J12" s="106" t="n"/>
+      <c r="G12" s="107" t="n"/>
+      <c r="H12" s="102" t="n"/>
+      <c r="I12" s="102" t="n"/>
+      <c r="J12" s="102" t="n"/>
     </row>
     <row r="13" ht="28" customHeight="1" s="132">
       <c r="A13" s="29" t="n"/>
@@ -2922,198 +3080,198 @@
       <c r="F13" s="76" t="n">
         <v>15</v>
       </c>
-      <c r="G13" s="112" t="n"/>
-      <c r="H13" s="106" t="n"/>
-      <c r="I13" s="106" t="n"/>
-      <c r="J13" s="106" t="n"/>
+      <c r="G13" s="101" t="n"/>
+      <c r="H13" s="102" t="n"/>
+      <c r="I13" s="102" t="n"/>
+      <c r="J13" s="102" t="n"/>
     </row>
     <row r="14" ht="29" customHeight="1" s="132">
-      <c r="A14" s="35" t="n"/>
-      <c r="B14" s="36" t="inlineStr">
+      <c r="A14" s="29" t="n"/>
+      <c r="B14" s="30" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="C14" s="37" t="inlineStr">
+      <c r="C14" s="32" t="inlineStr">
         <is>
           <t>Bullet Pass</t>
         </is>
       </c>
-      <c r="D14" s="38" t="inlineStr">
+      <c r="D14" s="33" t="inlineStr">
         <is>
           <t>Pass to player of choice. SHOT +5%</t>
         </is>
       </c>
-      <c r="E14" s="38" t="inlineStr">
+      <c r="E14" s="33" t="inlineStr">
         <is>
           <t>New players discards 1 card at random</t>
         </is>
       </c>
-      <c r="F14" s="77" t="n">
+      <c r="F14" s="80" t="n">
         <v>12</v>
       </c>
-      <c r="G14" s="127" t="n"/>
-      <c r="H14" s="104" t="n"/>
-      <c r="I14" s="104" t="n"/>
-      <c r="J14" s="104" t="n"/>
+      <c r="G14" s="107" t="n"/>
+      <c r="H14" s="102" t="n"/>
+      <c r="I14" s="102" t="n"/>
+      <c r="J14" s="102" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1" s="132">
-      <c r="A15" s="35" t="n"/>
-      <c r="B15" s="36" t="inlineStr">
+      <c r="A15" s="29" t="n"/>
+      <c r="B15" s="30" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="C15" s="37" t="inlineStr">
+      <c r="C15" s="32" t="inlineStr">
         <is>
           <t>Alley-Oop</t>
         </is>
       </c>
-      <c r="D15" s="38" t="inlineStr">
+      <c r="D15" s="33" t="inlineStr">
         <is>
           <t>SHOT +20%. Pass to player of choice</t>
         </is>
       </c>
-      <c r="E15" s="38" t="inlineStr">
+      <c r="E15" s="33" t="inlineStr">
         <is>
           <t>Receiving player shoots immediately after drawing for turn</t>
         </is>
       </c>
-      <c r="F15" s="77" t="n">
+      <c r="F15" s="80" t="n">
         <v>5</v>
       </c>
-      <c r="G15" s="127" t="n"/>
-      <c r="H15" s="104" t="n"/>
-      <c r="I15" s="104" t="n"/>
-      <c r="J15" s="104" t="n"/>
+      <c r="G15" s="107" t="n"/>
+      <c r="H15" s="102" t="n"/>
+      <c r="I15" s="102" t="n"/>
+      <c r="J15" s="102" t="n"/>
     </row>
     <row r="16" ht="14" customHeight="1" s="132">
-      <c r="A16" s="35" t="n"/>
-      <c r="B16" s="36" t="inlineStr">
+      <c r="A16" s="29" t="n"/>
+      <c r="B16" s="30" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="C16" s="37" t="inlineStr">
+      <c r="C16" s="32" t="inlineStr">
         <is>
           <t>Hand-Off</t>
         </is>
       </c>
-      <c r="D16" s="38" t="inlineStr">
+      <c r="D16" s="33" t="inlineStr">
         <is>
           <t>SHOT +5%. Pass to player to Left or Right. Draw 1 card</t>
         </is>
       </c>
-      <c r="E16" s="38" t="inlineStr">
+      <c r="E16" s="33" t="inlineStr">
         <is>
           <t>If played following a Dribble: draw 1 additional and SHOT +5% more</t>
         </is>
       </c>
-      <c r="F16" s="77" t="n">
+      <c r="F16" s="80" t="n">
         <v>10</v>
       </c>
-      <c r="G16" s="127" t="inlineStr">
+      <c r="G16" s="107" t="inlineStr">
         <is>
           <t>This is the Dribble Hand-Off</t>
         </is>
       </c>
-      <c r="H16" s="104" t="n"/>
-      <c r="I16" s="104" t="n"/>
-      <c r="J16" s="104" t="n"/>
+      <c r="H16" s="102" t="n"/>
+      <c r="I16" s="102" t="n"/>
+      <c r="J16" s="102" t="n"/>
     </row>
     <row r="17" ht="28" customHeight="1" s="132">
-      <c r="A17" s="35" t="n"/>
-      <c r="B17" s="36" t="inlineStr">
+      <c r="A17" s="29" t="n"/>
+      <c r="B17" s="30" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="C17" s="37" t="inlineStr">
+      <c r="C17" s="32" t="inlineStr">
         <is>
           <t>Outlet Pass</t>
         </is>
       </c>
-      <c r="D17" s="38" t="inlineStr">
+      <c r="D17" s="33" t="inlineStr">
         <is>
           <t>SHOT +10%. Shot Clock +01. Pass to player of choice</t>
         </is>
       </c>
-      <c r="E17" s="38" t="n"/>
-      <c r="F17" s="77" t="n">
+      <c r="E17" s="33" t="n"/>
+      <c r="F17" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="G17" s="127" t="inlineStr">
+      <c r="G17" s="107" t="inlineStr">
         <is>
           <t>The clock increments instead of decrementing — it does not break even</t>
         </is>
       </c>
-      <c r="H17" s="104" t="n"/>
-      <c r="I17" s="104" t="n"/>
-      <c r="J17" s="104" t="n"/>
+      <c r="H17" s="102" t="n"/>
+      <c r="I17" s="102" t="n"/>
+      <c r="J17" s="102" t="n"/>
     </row>
     <row r="18" ht="28" customHeight="1" s="132">
-      <c r="A18" s="35" t="n"/>
-      <c r="B18" s="36" t="inlineStr">
+      <c r="A18" s="29" t="n"/>
+      <c r="B18" s="30" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="C18" s="37" t="inlineStr">
+      <c r="C18" s="32" t="inlineStr">
         <is>
           <t>Kick-Out</t>
         </is>
       </c>
-      <c r="D18" s="38" t="inlineStr">
+      <c r="D18" s="33" t="inlineStr">
         <is>
           <t>SHOT +10%. Upgraded to 3pt. Pass to player of choice</t>
         </is>
       </c>
-      <c r="E18" s="38" t="inlineStr">
+      <c r="E18" s="33" t="inlineStr">
         <is>
           <t>Following Drive: draw 1. Following a Dribble Drive: gain 1 AST also</t>
         </is>
       </c>
-      <c r="F18" s="77" t="n">
+      <c r="F18" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="G18" s="127" t="inlineStr">
+      <c r="G18" s="107" t="inlineStr">
         <is>
           <t>The most it grants is a draw and 1 AST</t>
         </is>
       </c>
-      <c r="H18" s="104" t="n"/>
-      <c r="I18" s="104" t="n"/>
-      <c r="J18" s="104" t="n"/>
+      <c r="H18" s="102" t="n"/>
+      <c r="I18" s="102" t="n"/>
+      <c r="J18" s="102" t="n"/>
     </row>
     <row r="19" ht="56" customHeight="1" s="132">
-      <c r="A19" s="35" t="n"/>
-      <c r="B19" s="36" t="inlineStr">
+      <c r="A19" s="29" t="n"/>
+      <c r="B19" s="30" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="C19" s="37" t="inlineStr">
+      <c r="C19" s="32" t="inlineStr">
         <is>
           <t>Right Back</t>
         </is>
       </c>
-      <c r="D19" s="38" t="inlineStr">
+      <c r="D19" s="33" t="inlineStr">
         <is>
           <t>SHOT +5%. Pass to player of choice. They immediately pass it back</t>
         </is>
       </c>
-      <c r="E19" s="38" t="n"/>
-      <c r="F19" s="77" t="n">
+      <c r="E19" s="33" t="n"/>
+      <c r="F19" s="80" t="n">
         <v>7</v>
       </c>
-      <c r="G19" s="127" t="inlineStr">
+      <c r="G19" s="107" t="inlineStr">
         <is>
           <t>Results in a draw for each player and SHOT +10% overall. Whatever the trip costs them happens in between</t>
         </is>
       </c>
-      <c r="H19" s="104" t="n"/>
-      <c r="I19" s="104" t="n"/>
-      <c r="J19" s="104" t="n"/>
+      <c r="H19" s="102" t="n"/>
+      <c r="I19" s="102" t="n"/>
+      <c r="J19" s="102" t="n"/>
     </row>
     <row r="20" ht="56" customHeight="1" s="132">
       <c r="A20" s="35" t="n"/>
@@ -3136,55 +3294,55 @@
       <c r="F20" s="77" t="n">
         <v>5</v>
       </c>
-      <c r="G20" s="127" t="n"/>
-      <c r="H20" s="104" t="n"/>
-      <c r="I20" s="104" t="n"/>
-      <c r="J20" s="104" t="n"/>
+      <c r="G20" s="150" t="n"/>
+      <c r="H20" s="151" t="n"/>
+      <c r="I20" s="151" t="n"/>
+      <c r="J20" s="151" t="n"/>
     </row>
     <row r="21" ht="14" customHeight="1" s="132">
-      <c r="A21" s="39" t="inlineStr">
+      <c r="A21" s="144" t="inlineStr">
         <is>
           <t>Move</t>
         </is>
       </c>
-      <c r="B21" s="40">
-        <f>COUNTIF($B$5:$B$135,"Move")+COUNTIF($B$5:$B$135,"Special Move")</f>
+      <c r="B21" s="145">
+        <f>COUNTIF($B$22:$B$135,"Move")+COUNTIF($B$22:$B$135,"Special Move")</f>
         <v/>
       </c>
-      <c r="C21" s="41" t="n"/>
-      <c r="D21" s="41" t="n"/>
-      <c r="E21" s="41" t="n"/>
-      <c r="F21" s="78" t="n"/>
-      <c r="G21" s="120" t="n"/>
-      <c r="H21" s="121" t="n"/>
-      <c r="I21" s="121" t="n"/>
-      <c r="J21" s="121" t="n"/>
+      <c r="C21" s="146" t="n"/>
+      <c r="D21" s="146" t="n"/>
+      <c r="E21" s="146" t="n"/>
+      <c r="F21" s="147" t="n"/>
+      <c r="G21" s="148" t="n"/>
+      <c r="H21" s="149" t="n"/>
+      <c r="I21" s="149" t="n"/>
+      <c r="J21" s="149" t="n"/>
     </row>
     <row r="22" ht="28" customHeight="1" s="132">
-      <c r="A22" s="45" t="n"/>
-      <c r="B22" s="46" t="inlineStr">
+      <c r="A22" s="29" t="n"/>
+      <c r="B22" s="30" t="inlineStr">
         <is>
           <t>Move</t>
         </is>
       </c>
-      <c r="C22" s="47" t="inlineStr">
+      <c r="C22" s="32" t="inlineStr">
         <is>
           <t>Dribble</t>
         </is>
       </c>
-      <c r="D22" s="48" t="inlineStr">
+      <c r="D22" s="33" t="inlineStr">
         <is>
           <t>Draw 1 card. SHOT -10%</t>
         </is>
       </c>
-      <c r="E22" s="49" t="n"/>
-      <c r="F22" s="79" t="n">
+      <c r="E22" s="34" t="n"/>
+      <c r="F22" s="75" t="n">
         <v>15</v>
       </c>
-      <c r="G22" s="118" t="n"/>
-      <c r="H22" s="119" t="n"/>
-      <c r="I22" s="119" t="n"/>
-      <c r="J22" s="119" t="n"/>
+      <c r="G22" s="107" t="n"/>
+      <c r="H22" s="102" t="n"/>
+      <c r="I22" s="102" t="n"/>
+      <c r="J22" s="102" t="n"/>
     </row>
     <row r="23" ht="28" customHeight="1" s="132">
       <c r="A23" s="29" t="n"/>
@@ -3479,18 +3637,18 @@
       <c r="J32" s="102" t="n"/>
     </row>
     <row r="33" ht="14" customHeight="1" s="132">
-      <c r="A33" s="61" t="n"/>
-      <c r="B33" s="62" t="inlineStr">
+      <c r="A33" s="29" t="n"/>
+      <c r="B33" s="30" t="inlineStr">
         <is>
           <t>Move</t>
         </is>
       </c>
-      <c r="C33" s="63" t="inlineStr">
+      <c r="C33" s="32" t="inlineStr">
         <is>
           <t>Triple Threat</t>
         </is>
       </c>
-      <c r="D33" s="64" t="inlineStr">
+      <c r="D33" s="33" t="inlineStr">
         <is>
           <t>Choose 1:
 Draw 1 card
@@ -3498,99 +3656,99 @@
 SHOT +10%</t>
         </is>
       </c>
-      <c r="E33" s="64" t="inlineStr">
+      <c r="E33" s="33" t="inlineStr">
         <is>
           <t>Cannot use further Move cards</t>
         </is>
       </c>
-      <c r="F33" s="81" t="n">
+      <c r="F33" s="80" t="n">
         <v>15</v>
       </c>
-      <c r="G33" s="116" t="inlineStr">
+      <c r="G33" s="107" t="inlineStr">
         <is>
           <t>Cannot use further Move cards applies to that possession only.</t>
         </is>
       </c>
-      <c r="H33" s="117" t="n"/>
-      <c r="I33" s="117" t="n"/>
-      <c r="J33" s="117" t="n"/>
+      <c r="H33" s="102" t="n"/>
+      <c r="I33" s="102" t="n"/>
+      <c r="J33" s="102" t="n"/>
     </row>
     <row r="34" ht="14" customHeight="1" s="132">
-      <c r="A34" s="61" t="n"/>
-      <c r="B34" s="62" t="inlineStr">
+      <c r="A34" s="35" t="n"/>
+      <c r="B34" s="36" t="inlineStr">
         <is>
           <t>Move</t>
         </is>
       </c>
-      <c r="C34" s="63" t="inlineStr">
+      <c r="C34" s="37" t="inlineStr">
         <is>
           <t>Clear Out</t>
         </is>
       </c>
-      <c r="D34" s="64" t="inlineStr">
+      <c r="D34" s="38" t="inlineStr">
         <is>
           <t>First action only. The next pass to a side goes past you. One that named you is a TOV and ends the round</t>
         </is>
       </c>
-      <c r="E34" s="64" t="n"/>
-      <c r="F34" s="81" t="n">
+      <c r="E34" s="38" t="n"/>
+      <c r="F34" s="77" t="n">
         <v>8</v>
       </c>
-      <c r="G34" s="116" t="n"/>
-      <c r="H34" s="117" t="n"/>
-      <c r="I34" s="117" t="n"/>
-      <c r="J34" s="117" t="n"/>
+      <c r="G34" s="150" t="n"/>
+      <c r="H34" s="151" t="n"/>
+      <c r="I34" s="151" t="n"/>
+      <c r="J34" s="151" t="n"/>
     </row>
     <row r="35" ht="28" customHeight="1" s="132">
-      <c r="A35" s="42" t="inlineStr">
+      <c r="A35" s="144" t="inlineStr">
         <is>
           <t>Special Move</t>
         </is>
       </c>
-      <c r="B35" s="43">
-        <f>COUNTIF($B$5:$B$135,"Special Move")</f>
+      <c r="B35" s="145">
+        <f>COUNTIF($B$36:$B$135,"Special Move")</f>
         <v/>
       </c>
-      <c r="C35" s="44" t="n"/>
-      <c r="D35" s="44" t="n"/>
-      <c r="E35" s="44" t="n"/>
-      <c r="F35" s="82" t="n"/>
-      <c r="G35" s="120" t="n"/>
-      <c r="H35" s="121" t="n"/>
-      <c r="I35" s="121" t="n"/>
-      <c r="J35" s="121" t="n"/>
+      <c r="C35" s="146" t="n"/>
+      <c r="D35" s="146" t="n"/>
+      <c r="E35" s="146" t="n"/>
+      <c r="F35" s="147" t="n"/>
+      <c r="G35" s="148" t="n"/>
+      <c r="H35" s="149" t="n"/>
+      <c r="I35" s="149" t="n"/>
+      <c r="J35" s="149" t="n"/>
     </row>
     <row r="36" ht="28" customHeight="1" s="132">
-      <c r="A36" s="24" t="n"/>
-      <c r="B36" s="25" t="inlineStr">
+      <c r="A36" s="29" t="n"/>
+      <c r="B36" s="30" t="inlineStr">
         <is>
           <t>Special Move</t>
         </is>
       </c>
-      <c r="C36" s="26" t="inlineStr">
+      <c r="C36" s="32" t="inlineStr">
         <is>
           <t>Bankshot</t>
         </is>
       </c>
-      <c r="D36" s="27" t="inlineStr">
+      <c r="D36" s="33" t="inlineStr">
         <is>
           <t>Flip a coin:
 Heads: SHOT +10%
 Tails: SHOT -10%</t>
         </is>
       </c>
-      <c r="E36" s="27" t="inlineStr">
+      <c r="E36" s="33" t="inlineStr">
         <is>
           <t>Shoot the ball</t>
         </is>
       </c>
-      <c r="F36" s="83" t="n">
+      <c r="F36" s="80" t="n">
         <v>4</v>
       </c>
-      <c r="G36" s="105" t="n"/>
-      <c r="H36" s="106" t="n"/>
-      <c r="I36" s="106" t="n"/>
-      <c r="J36" s="106" t="n"/>
+      <c r="G36" s="107" t="n"/>
+      <c r="H36" s="102" t="n"/>
+      <c r="I36" s="102" t="n"/>
+      <c r="J36" s="102" t="n"/>
     </row>
     <row r="37" ht="28" customHeight="1" s="132">
       <c r="A37" s="29" t="n"/>
@@ -3617,14 +3775,14 @@
       <c r="F37" s="74" t="n">
         <v>4</v>
       </c>
-      <c r="G37" s="128" t="inlineStr">
+      <c r="G37" s="111" t="inlineStr">
         <is>
           <t>Can only play with Shot Clock at 1</t>
         </is>
       </c>
-      <c r="H37" s="106" t="n"/>
-      <c r="I37" s="106" t="n"/>
-      <c r="J37" s="106" t="n"/>
+      <c r="H37" s="102" t="n"/>
+      <c r="I37" s="102" t="n"/>
+      <c r="J37" s="102" t="n"/>
     </row>
     <row r="38" ht="42" customHeight="1" s="132">
       <c r="A38" s="29" t="n"/>
@@ -3651,10 +3809,10 @@
       <c r="F38" s="80" t="n">
         <v>4</v>
       </c>
-      <c r="G38" s="105" t="n"/>
-      <c r="H38" s="106" t="n"/>
-      <c r="I38" s="106" t="n"/>
-      <c r="J38" s="106" t="n"/>
+      <c r="G38" s="107" t="n"/>
+      <c r="H38" s="102" t="n"/>
+      <c r="I38" s="102" t="n"/>
+      <c r="J38" s="102" t="n"/>
     </row>
     <row r="39" ht="28" customHeight="1" s="132">
       <c r="A39" s="29" t="n"/>
@@ -3681,10 +3839,10 @@
       <c r="F39" s="74" t="n">
         <v>10</v>
       </c>
-      <c r="G39" s="112" t="n"/>
-      <c r="H39" s="106" t="n"/>
-      <c r="I39" s="106" t="n"/>
-      <c r="J39" s="106" t="n"/>
+      <c r="G39" s="101" t="n"/>
+      <c r="H39" s="102" t="n"/>
+      <c r="I39" s="102" t="n"/>
+      <c r="J39" s="102" t="n"/>
     </row>
     <row r="40" ht="28" customHeight="1" s="132">
       <c r="A40" s="29" t="n"/>
@@ -3711,10 +3869,10 @@
       <c r="F40" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="G40" s="105" t="n"/>
-      <c r="H40" s="106" t="n"/>
-      <c r="I40" s="106" t="n"/>
-      <c r="J40" s="106" t="n"/>
+      <c r="G40" s="107" t="n"/>
+      <c r="H40" s="102" t="n"/>
+      <c r="I40" s="102" t="n"/>
+      <c r="J40" s="102" t="n"/>
     </row>
     <row r="41" ht="42" customHeight="1" s="132">
       <c r="A41" s="29" t="n"/>
@@ -3741,10 +3899,10 @@
       <c r="F41" s="74" t="n">
         <v>3</v>
       </c>
-      <c r="G41" s="112" t="n"/>
-      <c r="H41" s="106" t="n"/>
-      <c r="I41" s="106" t="n"/>
-      <c r="J41" s="106" t="n"/>
+      <c r="G41" s="101" t="n"/>
+      <c r="H41" s="102" t="n"/>
+      <c r="I41" s="102" t="n"/>
+      <c r="J41" s="102" t="n"/>
     </row>
     <row r="42" ht="57" customHeight="1" s="132">
       <c r="A42" s="29" t="n"/>
@@ -3771,10 +3929,10 @@
       <c r="F42" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="G42" s="105" t="n"/>
-      <c r="H42" s="106" t="n"/>
-      <c r="I42" s="106" t="n"/>
-      <c r="J42" s="106" t="n"/>
+      <c r="G42" s="107" t="n"/>
+      <c r="H42" s="102" t="n"/>
+      <c r="I42" s="102" t="n"/>
+      <c r="J42" s="102" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1" s="132">
       <c r="A43" s="29" t="n"/>
@@ -3801,10 +3959,10 @@
       <c r="F43" s="74" t="n">
         <v>3</v>
       </c>
-      <c r="G43" s="112" t="n"/>
-      <c r="H43" s="106" t="n"/>
-      <c r="I43" s="106" t="n"/>
-      <c r="J43" s="106" t="n"/>
+      <c r="G43" s="101" t="n"/>
+      <c r="H43" s="102" t="n"/>
+      <c r="I43" s="102" t="n"/>
+      <c r="J43" s="102" t="n"/>
     </row>
     <row r="44" ht="28" customHeight="1" s="132">
       <c r="A44" s="29" t="n"/>
@@ -3831,10 +3989,10 @@
       <c r="F44" s="80" t="n">
         <v>4</v>
       </c>
-      <c r="G44" s="105" t="n"/>
-      <c r="H44" s="106" t="n"/>
-      <c r="I44" s="106" t="n"/>
-      <c r="J44" s="106" t="n"/>
+      <c r="G44" s="107" t="n"/>
+      <c r="H44" s="102" t="n"/>
+      <c r="I44" s="102" t="n"/>
+      <c r="J44" s="102" t="n"/>
     </row>
     <row r="45" ht="28" customHeight="1" s="132">
       <c r="A45" s="29" t="n"/>
@@ -3861,123 +4019,123 @@
       <c r="F45" s="74" t="n">
         <v>4</v>
       </c>
-      <c r="G45" s="112" t="n"/>
-      <c r="H45" s="106" t="n"/>
-      <c r="I45" s="106" t="n"/>
-      <c r="J45" s="106" t="n"/>
+      <c r="G45" s="101" t="n"/>
+      <c r="H45" s="102" t="n"/>
+      <c r="I45" s="102" t="n"/>
+      <c r="J45" s="102" t="n"/>
     </row>
     <row r="46" ht="42" customHeight="1" s="132">
-      <c r="A46" s="52" t="n"/>
-      <c r="B46" s="53" t="inlineStr">
+      <c r="A46" s="29" t="n"/>
+      <c r="B46" s="30" t="inlineStr">
         <is>
           <t>Special Move</t>
         </is>
       </c>
-      <c r="C46" s="69" t="inlineStr">
+      <c r="C46" s="32" t="inlineStr">
         <is>
           <t>Turnaround Three</t>
         </is>
       </c>
-      <c r="D46" s="70" t="inlineStr">
+      <c r="D46" s="33" t="inlineStr">
         <is>
           <t>Discard any number of cards. SHOT +10% for each</t>
         </is>
       </c>
-      <c r="E46" s="70" t="inlineStr">
+      <c r="E46" s="33" t="inlineStr">
         <is>
           <t>Shoot the ball. +1 Point on make</t>
         </is>
       </c>
-      <c r="F46" s="84" t="n">
+      <c r="F46" s="80" t="n">
         <v>1</v>
       </c>
-      <c r="G46" s="129" t="inlineStr">
+      <c r="G46" s="113" t="inlineStr">
         <is>
           <t>Only 1 in deck</t>
         </is>
       </c>
-      <c r="H46" s="106" t="n"/>
-      <c r="I46" s="106" t="n"/>
-      <c r="J46" s="106" t="n"/>
+      <c r="H46" s="102" t="n"/>
+      <c r="I46" s="102" t="n"/>
+      <c r="J46" s="102" t="n"/>
     </row>
     <row r="47" ht="42" customHeight="1" s="132">
-      <c r="A47" s="61" t="n"/>
-      <c r="B47" s="62" t="inlineStr">
+      <c r="A47" s="29" t="n"/>
+      <c r="B47" s="30" t="inlineStr">
         <is>
           <t>Special Move</t>
         </is>
       </c>
-      <c r="C47" s="66" t="inlineStr">
+      <c r="C47" s="31" t="inlineStr">
         <is>
           <t>Euro Step</t>
         </is>
       </c>
-      <c r="D47" s="67" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>Flip a coin until you get Tails. For each Heads, SHOT +5% and Draw 1 card</t>
         </is>
       </c>
-      <c r="E47" s="68" t="n"/>
-      <c r="F47" s="85" t="n">
+      <c r="E47" s="7" t="n"/>
+      <c r="F47" s="76" t="n">
         <v>5</v>
       </c>
-      <c r="G47" s="122" t="n"/>
-      <c r="H47" s="104" t="n"/>
-      <c r="I47" s="104" t="n"/>
-      <c r="J47" s="104" t="n"/>
+      <c r="G47" s="101" t="n"/>
+      <c r="H47" s="102" t="n"/>
+      <c r="I47" s="102" t="n"/>
+      <c r="J47" s="102" t="n"/>
     </row>
     <row r="48" ht="29" customHeight="1" s="132">
-      <c r="A48" s="61" t="n"/>
-      <c r="B48" s="62" t="inlineStr">
+      <c r="A48" s="35" t="n"/>
+      <c r="B48" s="36" t="inlineStr">
         <is>
           <t>Special Move</t>
         </is>
       </c>
-      <c r="C48" s="66" t="inlineStr">
+      <c r="C48" s="152" t="inlineStr">
         <is>
           <t>Wide-Open Three</t>
         </is>
       </c>
-      <c r="D48" s="67" t="inlineStr">
+      <c r="D48" s="153" t="inlineStr">
         <is>
           <t>Select any number of other players. SHOT +10% for each</t>
         </is>
       </c>
-      <c r="E48" s="68" t="inlineStr">
+      <c r="E48" s="154" t="inlineStr">
         <is>
           <t>Shoot the ball. +1 Point on make. Selected players receive +1 AST on a make</t>
         </is>
       </c>
-      <c r="F48" s="85" t="n">
+      <c r="F48" s="155" t="n">
         <v>2</v>
       </c>
-      <c r="G48" s="122" t="inlineStr">
+      <c r="G48" s="156" t="inlineStr">
         <is>
           <t>Selecting none rolls off current SHOT and is still a three</t>
         </is>
       </c>
-      <c r="H48" s="104" t="n"/>
-      <c r="I48" s="104" t="n"/>
-      <c r="J48" s="104" t="n"/>
+      <c r="H48" s="151" t="n"/>
+      <c r="I48" s="151" t="n"/>
+      <c r="J48" s="151" t="n"/>
     </row>
     <row r="49" ht="20" customHeight="1" s="132">
-      <c r="A49" s="58" t="inlineStr">
+      <c r="A49" s="144" t="inlineStr">
         <is>
           <t>Clamp</t>
         </is>
       </c>
-      <c r="B49" s="59">
-        <f>COUNTIF($B$5:$B$135,"Clamp")</f>
+      <c r="B49" s="145">
+        <f>COUNTIF($B$50:$B$135,"Clamp")</f>
         <v/>
       </c>
-      <c r="C49" s="60" t="n"/>
-      <c r="D49" s="60" t="n"/>
-      <c r="E49" s="60" t="n"/>
-      <c r="F49" s="86" t="n"/>
-      <c r="G49" s="109" t="n"/>
-      <c r="H49" s="110" t="n"/>
-      <c r="I49" s="110" t="n"/>
-      <c r="J49" s="110" t="n"/>
+      <c r="C49" s="146" t="n"/>
+      <c r="D49" s="146" t="n"/>
+      <c r="E49" s="146" t="n"/>
+      <c r="F49" s="147" t="n"/>
+      <c r="G49" s="148" t="n"/>
+      <c r="H49" s="149" t="n"/>
+      <c r="I49" s="149" t="n"/>
+      <c r="J49" s="149" t="n"/>
     </row>
     <row r="50" ht="56" customHeight="1" s="132">
       <c r="A50" s="29" t="n"/>
@@ -4100,53 +4258,53 @@
       <c r="J53" s="102" t="n"/>
     </row>
     <row r="54" ht="28" customHeight="1" s="132">
-      <c r="A54" s="61" t="n"/>
-      <c r="B54" s="62" t="inlineStr">
+      <c r="A54" s="35" t="n"/>
+      <c r="B54" s="36" t="inlineStr">
         <is>
           <t>Clamp</t>
         </is>
       </c>
-      <c r="C54" s="66" t="inlineStr">
+      <c r="C54" s="152" t="inlineStr">
         <is>
           <t>Triple-Team</t>
         </is>
       </c>
-      <c r="D54" s="67" t="inlineStr">
+      <c r="D54" s="153" t="inlineStr">
         <is>
           <t>Next player cannot play 3 random cards from hand.</t>
         </is>
       </c>
-      <c r="E54" s="68" t="n"/>
-      <c r="F54" s="85" t="n">
+      <c r="E54" s="154" t="n"/>
+      <c r="F54" s="155" t="n">
         <v>2</v>
       </c>
-      <c r="G54" s="135" t="inlineStr">
+      <c r="G54" s="157" t="inlineStr">
         <is>
           <t>3 def</t>
         </is>
       </c>
-      <c r="H54" s="117" t="n"/>
-      <c r="I54" s="117" t="n"/>
-      <c r="J54" s="117" t="n"/>
+      <c r="H54" s="151" t="n"/>
+      <c r="I54" s="151" t="n"/>
+      <c r="J54" s="151" t="n"/>
     </row>
     <row r="55" ht="28" customHeight="1" s="132">
-      <c r="A55" s="58" t="inlineStr">
+      <c r="A55" s="144" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="B55" s="59">
-        <f>COUNTIF($B$5:$B$135,"Whistle")</f>
+      <c r="B55" s="145">
+        <f>COUNTIF($B$56:$B$135,"Whistle")</f>
         <v/>
       </c>
-      <c r="C55" s="60" t="n"/>
-      <c r="D55" s="60" t="n"/>
-      <c r="E55" s="60" t="n"/>
-      <c r="F55" s="86" t="n"/>
-      <c r="G55" s="109" t="n"/>
-      <c r="H55" s="110" t="n"/>
-      <c r="I55" s="110" t="n"/>
-      <c r="J55" s="110" t="n"/>
+      <c r="C55" s="146" t="n"/>
+      <c r="D55" s="146" t="n"/>
+      <c r="E55" s="146" t="n"/>
+      <c r="F55" s="147" t="n"/>
+      <c r="G55" s="148" t="n"/>
+      <c r="H55" s="149" t="n"/>
+      <c r="I55" s="149" t="n"/>
+      <c r="J55" s="149" t="n"/>
     </row>
     <row r="56" ht="42" customHeight="1" s="132">
       <c r="A56" s="29" t="inlineStr">
@@ -4537,103 +4695,103 @@
       <c r="J70" s="102" t="n"/>
     </row>
     <row r="71" ht="14" customHeight="1" s="132">
-      <c r="A71" s="61" t="n"/>
-      <c r="B71" s="62" t="inlineStr">
+      <c r="A71" s="29" t="n"/>
+      <c r="B71" s="30" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C71" s="63" t="inlineStr">
+      <c r="C71" s="32" t="inlineStr">
         <is>
           <t>Travel</t>
         </is>
       </c>
-      <c r="D71" s="64" t="inlineStr">
+      <c r="D71" s="33" t="inlineStr">
         <is>
           <t>Move card played: Cancel card. TOV +1</t>
         </is>
       </c>
-      <c r="E71" s="65" t="n"/>
-      <c r="F71" s="140" t="n"/>
-      <c r="G71" s="116" t="n"/>
-      <c r="H71" s="117" t="n"/>
-      <c r="I71" s="117" t="n"/>
-      <c r="J71" s="117" t="n"/>
+      <c r="E71" s="34" t="n"/>
+      <c r="F71" s="138" t="n"/>
+      <c r="G71" s="107" t="n"/>
+      <c r="H71" s="102" t="n"/>
+      <c r="I71" s="102" t="n"/>
+      <c r="J71" s="102" t="n"/>
     </row>
     <row r="72" ht="28" customHeight="1" s="132">
-      <c r="A72" s="61" t="n"/>
-      <c r="B72" s="62" t="inlineStr">
+      <c r="A72" s="29" t="n"/>
+      <c r="B72" s="30" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C72" s="63" t="inlineStr">
+      <c r="C72" s="32" t="inlineStr">
         <is>
           <t>Clear Path Foul</t>
         </is>
       </c>
-      <c r="D72" s="64" t="inlineStr">
+      <c r="D72" s="33" t="inlineStr">
         <is>
           <t>On Shot, when Clamped by SHOT-reducing Clamps: Cancel those Clamps. Award the points the shot was worth. Take 1 FT</t>
         </is>
       </c>
-      <c r="E72" s="65" t="n"/>
-      <c r="F72" s="140" t="n"/>
-      <c r="G72" s="116" t="inlineStr">
+      <c r="E72" s="34" t="n"/>
+      <c r="F72" s="138" t="n"/>
+      <c r="G72" s="107" t="inlineStr">
         <is>
           <t>Fires as the shot starts, before the cutscene. This DOES count as a completed round.</t>
         </is>
       </c>
-      <c r="H72" s="117" t="n"/>
-      <c r="I72" s="117" t="n"/>
-      <c r="J72" s="117" t="n"/>
+      <c r="H72" s="102" t="n"/>
+      <c r="I72" s="102" t="n"/>
+      <c r="J72" s="102" t="n"/>
     </row>
     <row r="73" ht="28" customHeight="1" s="132">
-      <c r="A73" s="61" t="n"/>
-      <c r="B73" s="62" t="inlineStr">
+      <c r="A73" s="35" t="n"/>
+      <c r="B73" s="36" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C73" s="63" t="inlineStr">
+      <c r="C73" s="37" t="inlineStr">
         <is>
           <t>Play-On</t>
         </is>
       </c>
-      <c r="D73" s="64" t="inlineStr">
+      <c r="D73" s="38" t="inlineStr">
         <is>
           <t>Discard each Game Break drawn and draw again, until a card is not one</t>
         </is>
       </c>
-      <c r="E73" s="65" t="n"/>
-      <c r="F73" s="140" t="n"/>
-      <c r="G73" s="116" t="inlineStr">
+      <c r="E73" s="158" t="n"/>
+      <c r="F73" s="159" t="n"/>
+      <c r="G73" s="150" t="inlineStr">
         <is>
           <t>Raised where the Break lands, like Cleared to Play — nobody plays a Break</t>
         </is>
       </c>
-      <c r="H73" s="117" t="n"/>
-      <c r="I73" s="117" t="n"/>
-      <c r="J73" s="117" t="n"/>
+      <c r="H73" s="151" t="n"/>
+      <c r="I73" s="151" t="n"/>
+      <c r="J73" s="151" t="n"/>
     </row>
     <row r="74" ht="28" customHeight="1" s="132">
-      <c r="A74" s="58" t="inlineStr">
+      <c r="A74" s="144" t="inlineStr">
         <is>
           <t>Game Break</t>
         </is>
       </c>
-      <c r="B74" s="59">
-        <f>COUNTIF($B$5:$B$135,"Game Break")</f>
+      <c r="B74" s="145">
+        <f>COUNTIF($B$75:$B$135,"Game Break")</f>
         <v/>
       </c>
-      <c r="C74" s="60" t="n"/>
-      <c r="D74" s="60" t="n"/>
-      <c r="E74" s="60" t="n"/>
-      <c r="F74" s="86" t="n"/>
-      <c r="G74" s="109" t="n"/>
-      <c r="H74" s="110" t="n"/>
-      <c r="I74" s="110" t="n"/>
-      <c r="J74" s="110" t="n"/>
+      <c r="C74" s="146" t="n"/>
+      <c r="D74" s="146" t="n"/>
+      <c r="E74" s="146" t="n"/>
+      <c r="F74" s="147" t="n"/>
+      <c r="G74" s="148" t="n"/>
+      <c r="H74" s="149" t="n"/>
+      <c r="I74" s="149" t="n"/>
+      <c r="J74" s="149" t="n"/>
     </row>
     <row r="75" ht="28" customHeight="1" s="132">
       <c r="A75" s="29" t="n"/>
@@ -5402,137 +5560,137 @@
       <c r="J102" s="102" t="n"/>
     </row>
     <row r="103" ht="14" customHeight="1" s="132">
-      <c r="A103" s="29" t="n"/>
-      <c r="B103" s="30" t="inlineStr">
+      <c r="A103" s="35" t="n"/>
+      <c r="B103" s="36" t="inlineStr">
         <is>
           <t>Game Break</t>
         </is>
       </c>
-      <c r="C103" s="134" t="inlineStr">
+      <c r="C103" s="160" t="inlineStr">
         <is>
           <t>Back-and-Forth Game</t>
         </is>
       </c>
-      <c r="D103" s="91" t="inlineStr">
+      <c r="D103" s="161" t="inlineStr">
         <is>
           <t>Discard the next 3 Game Breaks. Whoever draws one draws again</t>
         </is>
       </c>
-      <c r="E103" s="7" t="n"/>
-      <c r="F103" s="76" t="n">
+      <c r="E103" s="154" t="n"/>
+      <c r="F103" s="155" t="n">
         <v>3</v>
       </c>
-      <c r="G103" s="111" t="n"/>
-      <c r="H103" s="102" t="n"/>
-      <c r="I103" s="102" t="n"/>
-      <c r="J103" s="102" t="n"/>
+      <c r="G103" s="162" t="n"/>
+      <c r="H103" s="151" t="n"/>
+      <c r="I103" s="151" t="n"/>
+      <c r="J103" s="151" t="n"/>
     </row>
     <row r="104" ht="28" customHeight="1" s="132">
-      <c r="A104" s="55" t="inlineStr">
+      <c r="A104" s="144" t="inlineStr">
         <is>
           <t>Injury GB</t>
         </is>
       </c>
-      <c r="B104" s="56">
-        <f>COUNTIF($B$5:$B$135,"Injury GB")</f>
+      <c r="B104" s="145">
+        <f>COUNTIF($B$105:$B$135,"Injury GB")</f>
         <v/>
       </c>
-      <c r="C104" s="57" t="n"/>
-      <c r="D104" s="57" t="n"/>
-      <c r="E104" s="57" t="n"/>
-      <c r="F104" s="88" t="n"/>
-      <c r="G104" s="108" t="n"/>
-      <c r="H104" s="102" t="n"/>
-      <c r="I104" s="102" t="n"/>
-      <c r="J104" s="102" t="n"/>
+      <c r="C104" s="146" t="n"/>
+      <c r="D104" s="146" t="n"/>
+      <c r="E104" s="146" t="n"/>
+      <c r="F104" s="147" t="n"/>
+      <c r="G104" s="148" t="n"/>
+      <c r="H104" s="149" t="n"/>
+      <c r="I104" s="149" t="n"/>
+      <c r="J104" s="149" t="n"/>
     </row>
     <row r="105" ht="28" customHeight="1" s="132">
-      <c r="A105" s="29" t="n"/>
-      <c r="B105" s="30" t="inlineStr">
+      <c r="A105" s="35" t="n"/>
+      <c r="B105" s="36" t="inlineStr">
         <is>
           <t>Injury GB</t>
         </is>
       </c>
-      <c r="C105" s="31" t="inlineStr">
+      <c r="C105" s="152" t="inlineStr">
         <is>
           <t>Bone Bruise</t>
         </is>
       </c>
-      <c r="D105" s="91" t="inlineStr">
+      <c r="D105" s="161" t="inlineStr">
         <is>
           <t>Discard 1 card at the start of each turn after drawing (your choice)</t>
         </is>
       </c>
-      <c r="E105" s="7" t="n"/>
-      <c r="F105" s="76" t="n">
+      <c r="E105" s="154" t="n"/>
+      <c r="F105" s="155" t="n">
         <v>3</v>
       </c>
-      <c r="G105" s="101" t="n"/>
-      <c r="H105" s="102" t="n"/>
-      <c r="I105" s="102" t="n"/>
-      <c r="J105" s="102" t="n"/>
+      <c r="G105" s="156" t="n"/>
+      <c r="H105" s="151" t="n"/>
+      <c r="I105" s="151" t="n"/>
+      <c r="J105" s="151" t="n"/>
     </row>
     <row r="106" ht="28" customHeight="1" s="132">
-      <c r="A106" s="58" t="inlineStr">
+      <c r="A106" s="144" t="inlineStr">
         <is>
           <t>Devastating Injury GB</t>
         </is>
       </c>
-      <c r="B106" s="59">
-        <f>COUNTIF($B$5:$B$135,"Devastating Injury GB")</f>
+      <c r="B106" s="145">
+        <f>COUNTIF($B$107:$B$135,"Devastating Injury GB")</f>
         <v/>
       </c>
-      <c r="C106" s="60" t="n"/>
-      <c r="D106" s="60" t="n"/>
-      <c r="E106" s="60" t="n"/>
-      <c r="F106" s="86" t="n"/>
-      <c r="G106" s="109" t="n"/>
-      <c r="H106" s="110" t="n"/>
-      <c r="I106" s="110" t="n"/>
-      <c r="J106" s="110" t="n"/>
+      <c r="C106" s="146" t="n"/>
+      <c r="D106" s="146" t="n"/>
+      <c r="E106" s="146" t="n"/>
+      <c r="F106" s="147" t="n"/>
+      <c r="G106" s="148" t="n"/>
+      <c r="H106" s="149" t="n"/>
+      <c r="I106" s="149" t="n"/>
+      <c r="J106" s="149" t="n"/>
     </row>
     <row r="107" ht="28" customHeight="1" s="132">
-      <c r="A107" s="50" t="n"/>
-      <c r="B107" s="51" t="inlineStr">
+      <c r="A107" s="35" t="n"/>
+      <c r="B107" s="36" t="inlineStr">
         <is>
           <t>Devastating Injury GB</t>
         </is>
       </c>
-      <c r="C107" s="136" t="inlineStr">
+      <c r="C107" s="163" t="inlineStr">
         <is>
           <t>Torn Achilles</t>
         </is>
       </c>
-      <c r="D107" s="137" t="inlineStr">
+      <c r="D107" s="164" t="inlineStr">
         <is>
           <t>Hand is locked every turn except 1 card (randomly)</t>
         </is>
       </c>
-      <c r="E107" s="54" t="n"/>
-      <c r="F107" s="141" t="n"/>
-      <c r="G107" s="114" t="n"/>
-      <c r="H107" s="115" t="n"/>
-      <c r="I107" s="115" t="n"/>
-      <c r="J107" s="115" t="n"/>
+      <c r="E107" s="154" t="n"/>
+      <c r="F107" s="159" t="n"/>
+      <c r="G107" s="156" t="n"/>
+      <c r="H107" s="151" t="n"/>
+      <c r="I107" s="151" t="n"/>
+      <c r="J107" s="151" t="n"/>
     </row>
     <row r="108" ht="42" customHeight="1" s="132">
-      <c r="A108" s="55" t="inlineStr">
+      <c r="A108" s="144" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="B108" s="56">
-        <f>COUNTIF($B$5:$B$135,"Intangible")</f>
+      <c r="B108" s="145">
+        <f>COUNTIF($B$109:$B$135,"Intangible")</f>
         <v/>
       </c>
-      <c r="C108" s="57" t="n"/>
-      <c r="D108" s="57" t="n"/>
-      <c r="E108" s="57" t="n"/>
-      <c r="F108" s="88" t="n"/>
-      <c r="G108" s="108" t="n"/>
-      <c r="H108" s="102" t="n"/>
-      <c r="I108" s="102" t="n"/>
-      <c r="J108" s="102" t="n"/>
+      <c r="C108" s="146" t="n"/>
+      <c r="D108" s="146" t="n"/>
+      <c r="E108" s="146" t="n"/>
+      <c r="F108" s="147" t="n"/>
+      <c r="G108" s="148" t="n"/>
+      <c r="H108" s="149" t="n"/>
+      <c r="I108" s="149" t="n"/>
+      <c r="J108" s="149" t="n"/>
     </row>
     <row r="109" ht="56" customHeight="1" s="132">
       <c r="A109" s="96" t="inlineStr">
@@ -6035,174 +6193,180 @@
       <c r="J128" s="102" t="n"/>
     </row>
     <row r="129">
-      <c r="A129" s="61" t="n"/>
-      <c r="B129" s="62" t="inlineStr">
+      <c r="A129" s="29" t="n"/>
+      <c r="B129" s="30" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C129" s="66" t="inlineStr">
+      <c r="C129" s="31" t="inlineStr">
         <is>
           <t>Ball Pounder</t>
         </is>
       </c>
-      <c r="D129" s="95" t="inlineStr">
+      <c r="D129" s="91" t="inlineStr">
         <is>
           <t>All Dribble cards you play draw an additional card but lower SHOT by an additional 10%</t>
         </is>
       </c>
-      <c r="E129" s="68" t="n"/>
-      <c r="F129" s="140" t="n"/>
-      <c r="G129" s="126" t="n"/>
-      <c r="H129" s="117" t="n"/>
-      <c r="I129" s="117" t="n"/>
-      <c r="J129" s="117" t="n"/>
+      <c r="E129" s="7" t="n"/>
+      <c r="F129" s="138" t="n"/>
+      <c r="G129" s="101" t="n"/>
+      <c r="H129" s="102" t="n"/>
+      <c r="I129" s="102" t="n"/>
+      <c r="J129" s="102" t="n"/>
     </row>
     <row r="130">
-      <c r="A130" s="61" t="n"/>
-      <c r="B130" s="62" t="inlineStr">
+      <c r="A130" s="29" t="n"/>
+      <c r="B130" s="30" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C130" s="66" t="inlineStr">
+      <c r="C130" s="31" t="inlineStr">
         <is>
           <t>Unselfish</t>
         </is>
       </c>
-      <c r="D130" s="95" t="inlineStr">
+      <c r="D130" s="91" t="inlineStr">
         <is>
           <t>Draw 1 card and increase next SHOT +5% whenever you positively affect another player</t>
         </is>
       </c>
-      <c r="E130" s="68" t="n"/>
-      <c r="F130" s="140" t="n"/>
-      <c r="G130" s="126" t="n"/>
-      <c r="H130" s="117" t="n"/>
-      <c r="I130" s="117" t="n"/>
-      <c r="J130" s="117" t="n"/>
+      <c r="E130" s="7" t="n"/>
+      <c r="F130" s="138" t="n"/>
+      <c r="G130" s="101" t="n"/>
+      <c r="H130" s="102" t="n"/>
+      <c r="I130" s="102" t="n"/>
+      <c r="J130" s="102" t="n"/>
     </row>
     <row r="131">
-      <c r="A131" s="61" t="n"/>
-      <c r="B131" s="62" t="inlineStr">
+      <c r="A131" s="29" t="n"/>
+      <c r="B131" s="30" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C131" s="66" t="inlineStr">
+      <c r="C131" s="31" t="inlineStr">
         <is>
           <t>Dirty Player</t>
         </is>
       </c>
-      <c r="D131" s="95" t="inlineStr">
+      <c r="D131" s="91" t="inlineStr">
         <is>
           <t>When sending Clamps, the clamped player discards 1 if they have any Injuries</t>
         </is>
       </c>
-      <c r="E131" s="68" t="n"/>
-      <c r="F131" s="140" t="n"/>
-      <c r="G131" s="126" t="n"/>
-      <c r="H131" s="117" t="n"/>
-      <c r="I131" s="117" t="n"/>
-      <c r="J131" s="117" t="n"/>
+      <c r="E131" s="7" t="n"/>
+      <c r="F131" s="138" t="n"/>
+      <c r="G131" s="101" t="n"/>
+      <c r="H131" s="102" t="n"/>
+      <c r="I131" s="102" t="n"/>
+      <c r="J131" s="102" t="n"/>
     </row>
     <row r="132">
-      <c r="A132" s="61" t="n"/>
-      <c r="B132" s="62" t="inlineStr">
+      <c r="A132" s="29" t="n"/>
+      <c r="B132" s="30" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C132" s="66" t="inlineStr">
+      <c r="C132" s="31" t="inlineStr">
         <is>
           <t>Villainous Reputation</t>
         </is>
       </c>
-      <c r="D132" s="95" t="inlineStr">
+      <c r="D132" s="91" t="inlineStr">
         <is>
           <t>Discard 1 whenever any Whistle triggers</t>
         </is>
       </c>
-      <c r="E132" s="68" t="n"/>
-      <c r="F132" s="140" t="n"/>
-      <c r="G132" s="126" t="inlineStr">
+      <c r="E132" s="7" t="n"/>
+      <c r="F132" s="138" t="n"/>
+      <c r="G132" s="101" t="inlineStr">
         <is>
           <t>Discarded during play, it attaches to a random player — possibly you again</t>
         </is>
       </c>
+      <c r="H132" s="102" t="n"/>
+      <c r="I132" s="102" t="n"/>
+      <c r="J132" s="102" t="n"/>
     </row>
     <row r="133">
-      <c r="A133" s="61" t="n"/>
-      <c r="B133" s="62" t="inlineStr">
+      <c r="A133" s="29" t="n"/>
+      <c r="B133" s="30" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C133" s="66" t="inlineStr">
+      <c r="C133" s="31" t="inlineStr">
         <is>
           <t>Free Agent</t>
         </is>
       </c>
-      <c r="D133" s="95" t="inlineStr">
+      <c r="D133" s="91" t="inlineStr">
         <is>
           <t>Discard your hand. Play a card at random from a player of your choosing (they keep it)</t>
         </is>
       </c>
-      <c r="E133" s="68" t="n"/>
-      <c r="F133" s="140" t="n"/>
-      <c r="G133" s="126" t="inlineStr">
+      <c r="E133" s="7" t="n"/>
+      <c r="F133" s="138" t="n"/>
+      <c r="G133" s="101" t="inlineStr">
         <is>
           <t>The discard waits for the draw chain to finish. Target is shuffled first and is affected by Floor General. Your own draws are kept. All-0 rebounds are yours; otherwise you cannot bid</t>
         </is>
       </c>
+      <c r="H133" s="102" t="n"/>
+      <c r="I133" s="102" t="n"/>
+      <c r="J133" s="102" t="n"/>
     </row>
     <row r="134">
-      <c r="A134" s="61" t="n"/>
-      <c r="B134" s="62" t="inlineStr">
+      <c r="A134" s="29" t="n"/>
+      <c r="B134" s="30" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C134" s="66" t="inlineStr">
+      <c r="C134" s="31" t="inlineStr">
         <is>
           <t>Franchise Player</t>
         </is>
       </c>
-      <c r="D134" s="95" t="inlineStr">
+      <c r="D134" s="91" t="inlineStr">
         <is>
           <t>When passing, choose 1 of the new player's Intangibles or a card in their hand for them to discard</t>
         </is>
       </c>
-      <c r="E134" s="68" t="n"/>
-      <c r="F134" s="140" t="n"/>
-      <c r="G134" s="126" t="n"/>
-      <c r="H134" s="117" t="n"/>
-      <c r="I134" s="117" t="n"/>
-      <c r="J134" s="117" t="n"/>
+      <c r="E134" s="7" t="n"/>
+      <c r="F134" s="138" t="n"/>
+      <c r="G134" s="101" t="n"/>
+      <c r="H134" s="102" t="n"/>
+      <c r="I134" s="102" t="n"/>
+      <c r="J134" s="102" t="n"/>
     </row>
     <row r="135">
-      <c r="A135" s="61" t="n"/>
-      <c r="B135" s="62" t="inlineStr">
+      <c r="A135" s="35" t="n"/>
+      <c r="B135" s="36" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C135" s="66" t="inlineStr">
+      <c r="C135" s="152" t="inlineStr">
         <is>
           <t>Fundamentalist</t>
         </is>
       </c>
-      <c r="D135" s="95" t="inlineStr">
+      <c r="D135" s="161" t="inlineStr">
         <is>
           <t>No Special Moves. Each Move once a turn. Swings, Skip Pass and Dribble are never spent</t>
         </is>
       </c>
-      <c r="E135" s="68" t="n"/>
-      <c r="F135" s="140" t="n"/>
-      <c r="G135" s="126" t="n"/>
-      <c r="H135" s="117" t="n"/>
-      <c r="I135" s="117" t="n"/>
-      <c r="J135" s="117" t="n"/>
+      <c r="E135" s="154" t="n"/>
+      <c r="F135" s="159" t="n"/>
+      <c r="G135" s="156" t="n"/>
+      <c r="H135" s="151" t="n"/>
+      <c r="I135" s="151" t="n"/>
+      <c r="J135" s="151" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="122">

</xml_diff>

<commit_message>
Competitive keeps the SHOT; Unguardable goes to the Zone
The Intangible is Competitive now — same card, same effect, and the name it was
using belongs to the Swissh-Up, which ignores clamps outright rather than only
their SHOT. Renamed in the game and on the sheet.

The name plate's numbers, read off its bench: plate three quarters of the trip
and hung a quarter off the leading edge, name at 32pt, squeezed to 0.750, three
tenths in.

**And its taper is back.** The mother shape's ramp had been cut to almost nothing
while the plate was being placed, which took the fade off the left of the card
altogether. With the plate hung off the edge the way it now is, that ramp lands
across the first eighth of the screen — which is the taper that went missing.
Both ends of it are on the bench.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -6173,7 +6173,7 @@
       </c>
       <c r="C128" s="31" t="inlineStr">
         <is>
-          <t>Unguardable</t>
+          <t>Competitive</t>
         </is>
       </c>
       <c r="D128" s="91" t="inlineStr">
@@ -6396,30 +6396,29 @@
   <mergeCells count="123">
     <mergeCell ref="G55:J55"/>
     <mergeCell ref="G4:J4"/>
+    <mergeCell ref="G135:J135"/>
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
-    <mergeCell ref="G135:J135"/>
+    <mergeCell ref="G119:J119"/>
     <mergeCell ref="G32:J32"/>
-    <mergeCell ref="G119:J119"/>
     <mergeCell ref="G46:J46"/>
     <mergeCell ref="G40:J40"/>
     <mergeCell ref="G111:J111"/>
     <mergeCell ref="G72:J72"/>
     <mergeCell ref="G81:J81"/>
     <mergeCell ref="G96:J96"/>
-    <mergeCell ref="G5:J5"/>
+    <mergeCell ref="G71:J71"/>
     <mergeCell ref="G136:J136"/>
-    <mergeCell ref="G71:J71"/>
     <mergeCell ref="G8:J8"/>
     <mergeCell ref="G82:J82"/>
     <mergeCell ref="G57:J57"/>
+    <mergeCell ref="G128:J128"/>
     <mergeCell ref="G10:J10"/>
     <mergeCell ref="G66:J66"/>
-    <mergeCell ref="G128:J128"/>
     <mergeCell ref="G18:J18"/>
     <mergeCell ref="G53:J53"/>
+    <mergeCell ref="G121:J121"/>
     <mergeCell ref="G34:J34"/>
-    <mergeCell ref="G121:J121"/>
     <mergeCell ref="G74:J74"/>
     <mergeCell ref="G68:J68"/>
     <mergeCell ref="G108:J108"/>
@@ -6447,9 +6446,9 @@
     <mergeCell ref="G48:J48"/>
     <mergeCell ref="G23:J23"/>
     <mergeCell ref="G97:J97"/>
+    <mergeCell ref="G125:J125"/>
     <mergeCell ref="G7:J7"/>
     <mergeCell ref="G38:J38"/>
-    <mergeCell ref="G125:J125"/>
     <mergeCell ref="G112:J112"/>
     <mergeCell ref="G45:J45"/>
     <mergeCell ref="G62:J62"/>
@@ -6469,16 +6468,15 @@
     <mergeCell ref="G60:J60"/>
     <mergeCell ref="G9:J9"/>
     <mergeCell ref="G131:J131"/>
-    <mergeCell ref="G124:J124"/>
+    <mergeCell ref="G59:J59"/>
     <mergeCell ref="G115:J115"/>
     <mergeCell ref="G130:J130"/>
-    <mergeCell ref="G59:J59"/>
     <mergeCell ref="G11:J11"/>
     <mergeCell ref="G117:J117"/>
     <mergeCell ref="G126:J126"/>
     <mergeCell ref="G132:J132"/>
+    <mergeCell ref="G39:J39"/>
     <mergeCell ref="G122:J122"/>
-    <mergeCell ref="G39:J39"/>
     <mergeCell ref="G101:J101"/>
     <mergeCell ref="G116:J116"/>
     <mergeCell ref="G103:J103"/>
@@ -6489,10 +6487,10 @@
     <mergeCell ref="G118:J118"/>
     <mergeCell ref="G87:J87"/>
     <mergeCell ref="G15:J15"/>
+    <mergeCell ref="G80:J80"/>
     <mergeCell ref="G95:J95"/>
-    <mergeCell ref="G80:J80"/>
+    <mergeCell ref="G64:J64"/>
     <mergeCell ref="G79:J79"/>
-    <mergeCell ref="G64:J64"/>
     <mergeCell ref="G73:J73"/>
     <mergeCell ref="G51:J51"/>
     <mergeCell ref="G54:J54"/>
@@ -6501,22 +6499,24 @@
     <mergeCell ref="G50:J50"/>
     <mergeCell ref="G106:J106"/>
     <mergeCell ref="G56:J56"/>
-    <mergeCell ref="G14:J14"/>
     <mergeCell ref="G105:J105"/>
     <mergeCell ref="G43:J43"/>
     <mergeCell ref="G52:J52"/>
     <mergeCell ref="G120:J120"/>
+    <mergeCell ref="G27:J27"/>
     <mergeCell ref="G98:J98"/>
-    <mergeCell ref="G107:J107"/>
-    <mergeCell ref="G27:J27"/>
     <mergeCell ref="G36:J36"/>
     <mergeCell ref="G42:J42"/>
+    <mergeCell ref="G107:J107"/>
     <mergeCell ref="G17:J17"/>
     <mergeCell ref="G19:J19"/>
     <mergeCell ref="G28:J28"/>
     <mergeCell ref="G6:J6"/>
     <mergeCell ref="G69:J69"/>
     <mergeCell ref="G83:J83"/>
+    <mergeCell ref="G124:J124"/>
+    <mergeCell ref="G5:J5"/>
+    <mergeCell ref="G14:J14"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
One place at a time, and a pile you can see
**The warp and the arrival were the same moment**, which is one man in two places
— the thing a teleport is meant to avoid. They take a turn each now: he comes
apart on the floor, and a warp later he assembles on the line; coming back he
leaves the line first and only then puts himself together where he stands. The
loop waits out both halves before the call, so nothing is announced over a man
who is still in pieces.

`Pacing.warp` owns the number, since the floor, the sideline and the loop all
have to agree on it.

The pile draws twice the slabs — the reading was set while a bug was making it
enormous, and once that was fixed it read as a handful of cards.

Hesi is a dribble, in the game and on the sheet.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -3455,7 +3455,11 @@
       <c r="F26" s="80" t="n">
         <v>15</v>
       </c>
-      <c r="G26" s="107" t="n"/>
+      <c r="G26" s="107" t="inlineStr">
+        <is>
+          <t>isDribble = true</t>
+        </is>
+      </c>
       <c r="H26" s="102" t="n"/>
       <c r="I26" s="102" t="n"/>
       <c r="J26" s="102" t="n"/>

</xml_diff>

<commit_message>
The floor and the ball are slots, and one SHOT = wins
Phase 0 and 1 of the Varena/Variaball queue.

- Varena and Variaball are card types, each with its own effect struct
- A game opens on Cardwood with a Regulation Ball: courtCard is never empty, ballCard nil
- Cardwood is in the library and the sheet, never dealt, and decodes off the wire
- Only one override applies to a shot: Intangible, then floor, then ball, then the card played
- Until they have faces of their own, both types print as the Game Breaks they replace

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -1876,7 +1876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="20" customHeight="1"/>
   <cols>
     <col width="26.5" customWidth="1" style="85" min="1" max="1"/>
@@ -2041,6 +2041,30 @@
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
       <c r="E11" s="7" t="n"/>
+    </row>
+    <row r="12" ht="32" customHeight="1" s="85">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>The floor. Persistent, global and replaceable: one is always out, Cardwood until somebody plays over it. One per player per possession</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1" s="85">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>The ball. An overlay on a Regulation Ball, which is no card at all. Persistent, global and replaceable, and never stacks. One per player per possession</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2065,7 +2089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J143"/>
+  <dimension ref="A1:J145"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="22.25" customHeight="1"/>
   <cols>
     <col width="15.5" customWidth="1" style="8" min="1" max="1"/>
@@ -2182,7 +2206,6 @@
         <v/>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="20.75" customHeight="1" s="85">
       <c r="A4" s="81" t="inlineStr">
         <is>
@@ -5907,7 +5930,7 @@
       <c r="I142" s="76" t="n"/>
       <c r="J142" s="76" t="n"/>
     </row>
-    <row r="143">
+    <row r="143" s="85">
       <c r="A143" s="27" t="n"/>
       <c r="B143" s="28" t="inlineStr">
         <is>
@@ -5931,8 +5954,55 @@
       <c r="G143" s="75" t="n"/>
       <c r="H143" s="76" t="n"/>
     </row>
+    <row r="144" ht="42" customHeight="1" s="85">
+      <c r="A144" s="52" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="B144" s="53">
+        <f>COUNTIF($B$145:$B$145,"Varena")</f>
+        <v/>
+      </c>
+      <c r="C144" s="54" t="n"/>
+      <c r="D144" s="54" t="n"/>
+      <c r="E144" s="54" t="n"/>
+      <c r="F144" s="55" t="n"/>
+      <c r="G144" s="66" t="n"/>
+      <c r="H144" s="67" t="n"/>
+      <c r="I144" s="67" t="n"/>
+      <c r="J144" s="67" t="n"/>
+    </row>
+    <row r="145" s="85">
+      <c r="A145" s="27" t="n"/>
+      <c r="B145" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C145" s="56" t="inlineStr">
+        <is>
+          <t>Cardwood</t>
+        </is>
+      </c>
+      <c r="D145" s="63" t="inlineStr">
+        <is>
+          <t>The default floor</t>
+        </is>
+      </c>
+      <c r="E145" s="58" t="n"/>
+      <c r="F145" s="61" t="n"/>
+      <c r="G145" s="75" t="inlineStr">
+        <is>
+          <t>Not in the deck. The floor every game opens on, and what the slot reads as when nobody has played a Varena over it</t>
+        </is>
+      </c>
+      <c r="H145" s="76" t="n"/>
+      <c r="I145" s="76" t="n"/>
+      <c r="J145" s="76" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="123">
+  <mergeCells count="124">
     <mergeCell ref="G55:J55"/>
     <mergeCell ref="G4:J4"/>
     <mergeCell ref="G135:J135"/>
@@ -5948,6 +6018,7 @@
     <mergeCell ref="G96:J96"/>
     <mergeCell ref="G71:J71"/>
     <mergeCell ref="G136:J136"/>
+    <mergeCell ref="G145:J145"/>
     <mergeCell ref="G8:J8"/>
     <mergeCell ref="G82:J82"/>
     <mergeCell ref="G57:J57"/>

</xml_diff>

<commit_message>
Ten Cardwoods go in the Standard deck
- Cardwood is dealt like any card, ten of them, and playing one changes the court back to basic
- Its card text, count and note match on the sheet
- The gallery has tabs for Varenas and Variaballs, shown once a type has cards
- The design doc counts 44 designed cards, 29 Varenas and 15 Variaballs, and records the 79-slot budget

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -5987,14 +5987,16 @@
       </c>
       <c r="D145" s="63" t="inlineStr">
         <is>
-          <t>The default floor</t>
+          <t>Changes the court back to basic</t>
         </is>
       </c>
       <c r="E145" s="58" t="n"/>
-      <c r="F145" s="61" t="n"/>
+      <c r="F145" s="61" t="n">
+        <v>10</v>
+      </c>
       <c r="G145" s="75" t="inlineStr">
         <is>
-          <t>Not in the deck. The floor every game opens on, and what the slot reads as when nobody has played a Varena over it</t>
+          <t>Also the floor every game opens on, before anybody plays a Varena over it</t>
         </is>
       </c>
       <c r="H145" s="76" t="n"/>

</xml_diff>

<commit_message>
The Game Breaks are out of the deck
- Only the Injuries are still dealt; the Standard deck is 431 cards
- The Break descriptors and the rules they lean on stay until each replacement is built
- The sheet marks the 30 as Retired Game Break at 0 copies, and the type table says so
- The gallery's Game Break tab, which only holds the Injuries now, is titled Injury

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -2005,7 +2005,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Play these immediately when dealt. One-off effects</t>
+          <t>Retired — out of the deck, replaced by Varenas and Variaballs. Only the Injuries below are still dealt</t>
         </is>
       </c>
       <c r="C9" s="7" t="n"/>
@@ -4298,11 +4298,11 @@
     <row r="79" ht="28" customHeight="1" s="85">
       <c r="A79" s="52" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Breaks</t>
         </is>
       </c>
       <c r="B79" s="53">
-        <f>COUNTIF($B$80:$B$143,"Game Break")</f>
+        <f>COUNTIF($B$80:$B$109,"Retired Game Break")</f>
         <v/>
       </c>
       <c r="C79" s="54" t="n"/>
@@ -4318,7 +4318,7 @@
       <c r="A80" s="21" t="n"/>
       <c r="B80" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C80" s="24" t="inlineStr">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="E80" s="26" t="n"/>
       <c r="F80" s="33" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G80" s="72" t="n"/>
       <c r="H80" s="71" t="n"/>
@@ -4344,7 +4344,7 @@
       <c r="A81" s="21" t="n"/>
       <c r="B81" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C81" s="23" t="inlineStr">
@@ -4359,7 +4359,7 @@
       </c>
       <c r="E81" s="7" t="n"/>
       <c r="F81" s="34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G81" s="74" t="inlineStr">
         <is>
@@ -4374,7 +4374,7 @@
       <c r="A82" s="21" t="n"/>
       <c r="B82" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C82" s="24" t="inlineStr">
@@ -4389,7 +4389,7 @@
       </c>
       <c r="E82" s="26" t="n"/>
       <c r="F82" s="33" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G82" s="72" t="n"/>
       <c r="H82" s="71" t="n"/>
@@ -4400,7 +4400,7 @@
       <c r="A83" s="21" t="n"/>
       <c r="B83" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C83" s="23" t="inlineStr">
@@ -4415,7 +4415,7 @@
       </c>
       <c r="E83" s="7" t="n"/>
       <c r="F83" s="34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G83" s="70" t="n"/>
       <c r="H83" s="71" t="n"/>
@@ -4426,7 +4426,7 @@
       <c r="A84" s="21" t="n"/>
       <c r="B84" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C84" s="37" t="inlineStr">
@@ -4441,7 +4441,7 @@
       </c>
       <c r="E84" s="26" t="n"/>
       <c r="F84" s="33" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G84" s="72" t="n"/>
       <c r="H84" s="71" t="n"/>
@@ -4452,7 +4452,7 @@
       <c r="A85" s="21" t="n"/>
       <c r="B85" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C85" s="23" t="inlineStr">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="E85" s="7" t="n"/>
       <c r="F85" s="34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G85" s="70" t="n"/>
       <c r="H85" s="71" t="n"/>
@@ -4478,7 +4478,7 @@
       <c r="A86" s="21" t="n"/>
       <c r="B86" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C86" s="24" t="inlineStr">
@@ -4493,7 +4493,7 @@
       </c>
       <c r="E86" s="26" t="n"/>
       <c r="F86" s="33" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G86" s="72" t="n"/>
       <c r="H86" s="71" t="n"/>
@@ -4504,7 +4504,7 @@
       <c r="A87" s="21" t="n"/>
       <c r="B87" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C87" s="23" t="inlineStr">
@@ -4523,7 +4523,7 @@
         </is>
       </c>
       <c r="F87" s="32" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G87" s="70" t="n"/>
       <c r="H87" s="71" t="n"/>
@@ -4534,7 +4534,7 @@
       <c r="A88" s="21" t="n"/>
       <c r="B88" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C88" s="24" t="inlineStr">
@@ -4553,7 +4553,7 @@
         </is>
       </c>
       <c r="F88" s="36" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G88" s="72" t="n"/>
       <c r="H88" s="71" t="n"/>
@@ -4564,7 +4564,7 @@
       <c r="A89" s="21" t="n"/>
       <c r="B89" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C89" s="23" t="inlineStr">
@@ -4579,7 +4579,7 @@
       </c>
       <c r="E89" s="7" t="n"/>
       <c r="F89" s="34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G89" s="74" t="n"/>
       <c r="H89" s="71" t="n"/>
@@ -4590,7 +4590,7 @@
       <c r="A90" s="21" t="n"/>
       <c r="B90" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C90" s="49" t="inlineStr">
@@ -4605,7 +4605,7 @@
       </c>
       <c r="E90" s="7" t="n"/>
       <c r="F90" s="34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G90" s="74" t="n"/>
       <c r="H90" s="71" t="n"/>
@@ -4616,7 +4616,7 @@
       <c r="A91" s="21" t="n"/>
       <c r="B91" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C91" s="49" t="inlineStr">
@@ -4631,7 +4631,7 @@
       </c>
       <c r="E91" s="7" t="n"/>
       <c r="F91" s="34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G91" s="74" t="inlineStr">
         <is>
@@ -4646,7 +4646,7 @@
       <c r="A92" s="21" t="n"/>
       <c r="B92" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C92" s="49" t="inlineStr">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="E92" s="7" t="n"/>
       <c r="F92" s="34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G92" s="74" t="n"/>
       <c r="H92" s="71" t="n"/>
@@ -4672,7 +4672,7 @@
       <c r="A93" s="21" t="n"/>
       <c r="B93" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C93" s="49" t="inlineStr">
@@ -4687,7 +4687,7 @@
       </c>
       <c r="E93" s="7" t="n"/>
       <c r="F93" s="34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G93" s="74" t="inlineStr">
         <is>
@@ -4702,7 +4702,7 @@
       <c r="A94" s="21" t="n"/>
       <c r="B94" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C94" s="49" t="inlineStr">
@@ -4717,7 +4717,7 @@
       </c>
       <c r="E94" s="7" t="n"/>
       <c r="F94" s="34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G94" s="74" t="n"/>
       <c r="H94" s="71" t="n"/>
@@ -4728,7 +4728,7 @@
       <c r="A95" s="21" t="n"/>
       <c r="B95" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C95" s="49" t="inlineStr">
@@ -4743,7 +4743,7 @@
       </c>
       <c r="E95" s="7" t="n"/>
       <c r="F95" s="34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G95" s="74" t="inlineStr">
         <is>
@@ -4758,7 +4758,7 @@
       <c r="A96" s="21" t="n"/>
       <c r="B96" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C96" s="49" t="inlineStr">
@@ -4773,7 +4773,7 @@
       </c>
       <c r="E96" s="7" t="n"/>
       <c r="F96" s="34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G96" s="74" t="inlineStr">
         <is>
@@ -4788,7 +4788,7 @@
       <c r="A97" s="21" t="n"/>
       <c r="B97" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C97" s="49" t="inlineStr">
@@ -4803,7 +4803,7 @@
       </c>
       <c r="E97" s="7" t="n"/>
       <c r="F97" s="34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G97" s="74" t="inlineStr">
         <is>
@@ -4818,7 +4818,7 @@
       <c r="A98" s="21" t="n"/>
       <c r="B98" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C98" s="49" t="inlineStr">
@@ -4833,7 +4833,7 @@
       </c>
       <c r="E98" s="7" t="n"/>
       <c r="F98" s="34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G98" s="74" t="n"/>
       <c r="H98" s="71" t="n"/>
@@ -4844,7 +4844,7 @@
       <c r="A99" s="21" t="n"/>
       <c r="B99" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C99" s="49" t="inlineStr">
@@ -4859,7 +4859,7 @@
       </c>
       <c r="E99" s="7" t="n"/>
       <c r="F99" s="34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G99" s="74" t="n"/>
       <c r="H99" s="71" t="n"/>
@@ -4870,7 +4870,7 @@
       <c r="A100" s="21" t="n"/>
       <c r="B100" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C100" s="49" t="inlineStr">
@@ -4885,7 +4885,7 @@
       </c>
       <c r="E100" s="7" t="n"/>
       <c r="F100" s="34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G100" s="74" t="n"/>
       <c r="H100" s="71" t="n"/>
@@ -4896,7 +4896,7 @@
       <c r="A101" s="21" t="n"/>
       <c r="B101" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C101" s="49" t="inlineStr">
@@ -4911,7 +4911,7 @@
       </c>
       <c r="E101" s="7" t="n"/>
       <c r="F101" s="34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G101" s="74" t="n"/>
       <c r="H101" s="71" t="n"/>
@@ -4922,7 +4922,7 @@
       <c r="A102" s="21" t="n"/>
       <c r="B102" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C102" s="49" t="inlineStr">
@@ -4937,7 +4937,7 @@
       </c>
       <c r="E102" s="7" t="n"/>
       <c r="F102" s="34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G102" s="74" t="n"/>
       <c r="H102" s="71" t="n"/>
@@ -4948,7 +4948,7 @@
       <c r="A103" s="21" t="n"/>
       <c r="B103" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C103" s="49" t="inlineStr">
@@ -4963,7 +4963,7 @@
       </c>
       <c r="E103" s="7" t="n"/>
       <c r="F103" s="34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G103" s="74" t="n"/>
       <c r="H103" s="71" t="n"/>
@@ -4974,7 +4974,7 @@
       <c r="A104" s="21" t="n"/>
       <c r="B104" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C104" s="49" t="inlineStr">
@@ -4989,7 +4989,7 @@
       </c>
       <c r="E104" s="7" t="n"/>
       <c r="F104" s="34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G104" s="74" t="n"/>
       <c r="H104" s="71" t="n"/>
@@ -5000,7 +5000,7 @@
       <c r="A105" s="21" t="n"/>
       <c r="B105" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C105" s="49" t="inlineStr">
@@ -5015,7 +5015,7 @@
       </c>
       <c r="E105" s="7" t="n"/>
       <c r="F105" s="34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G105" s="74" t="inlineStr">
         <is>
@@ -5030,7 +5030,7 @@
       <c r="A106" s="21" t="n"/>
       <c r="B106" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C106" s="49" t="inlineStr">
@@ -5045,7 +5045,7 @@
       </c>
       <c r="E106" s="7" t="n"/>
       <c r="F106" s="34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G106" s="74" t="n"/>
       <c r="H106" s="71" t="n"/>
@@ -5056,7 +5056,7 @@
       <c r="A107" s="21" t="n"/>
       <c r="B107" s="22" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C107" s="49" t="inlineStr">
@@ -5071,7 +5071,7 @@
       </c>
       <c r="E107" s="7" t="n"/>
       <c r="F107" s="34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G107" s="74" t="n"/>
       <c r="H107" s="71" t="n"/>
@@ -5082,7 +5082,7 @@
       <c r="A108" s="27" t="n"/>
       <c r="B108" s="28" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C108" s="62" t="inlineStr">
@@ -5097,7 +5097,7 @@
       </c>
       <c r="E108" s="58" t="n"/>
       <c r="F108" s="59" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G108" s="79" t="n"/>
       <c r="H108" s="76" t="n"/>
@@ -5108,7 +5108,7 @@
       <c r="A109" s="27" t="n"/>
       <c r="B109" s="28" t="inlineStr">
         <is>
-          <t>Game Break</t>
+          <t>Retired Game Break</t>
         </is>
       </c>
       <c r="C109" s="62" t="inlineStr">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="E109" s="58" t="n"/>
       <c r="F109" s="59" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G109" s="79" t="n"/>
       <c r="H109" s="76" t="n"/>

</xml_diff>

<commit_message>
Injury is its own card type, and Devastating Injury its sub-type
- Injuries carry their own effect: how long they last, Bone Bruise's discard, Torn Achilles' held hand
- They land through their own path, so Play-On, the answer to a Game Break, no longer waves one off
- Cleared to Play and Great Conditioning answer them as before
- Their own reveal, log line and call: "Injury!", in grey
- The gallery gives them their own tab; Downloaded still passes over them
- The sheet's Injury GB and Devastating Injury GB are Injury and Devastating Injury, and the Game Break total no longer counts them

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -2005,7 +2005,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Retired — out of the deck, replaced by Varenas and Variaballs. Only the Injuries below are still dealt</t>
+          <t>Retired — out of the deck, replaced by Varenas and Variaballs</t>
         </is>
       </c>
       <c r="C9" s="7" t="n"/>
@@ -2015,7 +2015,7 @@
     <row r="10" ht="32" customHeight="1" s="85">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Injury Game Break</t>
+          <t>Injury</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -2030,12 +2030,12 @@
     <row r="11" ht="32" customHeight="1" s="85">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Devastating Injury Game Break</t>
+          <t>Devastating Injury</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Same as above but also have effects that linger through the rounds </t>
+          <t>A sub-type of Injury. Same as above but also have effects that linger through the rounds</t>
         </is>
       </c>
       <c r="C11" s="7" t="n"/>
@@ -2144,12 +2144,12 @@
       </c>
       <c r="G1" s="11" t="inlineStr">
         <is>
-          <t>Injury GB</t>
+          <t>Injury</t>
         </is>
       </c>
       <c r="H1" s="11" t="inlineStr">
         <is>
-          <t>Devastating Injury GB</t>
+          <t>Devastating Injury</t>
         </is>
       </c>
       <c r="I1" s="11" t="inlineStr">
@@ -2186,15 +2186,15 @@
         <v/>
       </c>
       <c r="F2" s="16">
-        <f>COUNTIF($B$5:$B$140,"Game Break")&amp;" ("&amp;(COUNTIF($B$5:$B$140,"Game Break")+G2+H2)&amp;")"</f>
+        <f>COUNTIF($B$5:$B$140,"Game Break")</f>
         <v/>
       </c>
       <c r="G2" s="18">
-        <f>COUNTIF($B$5:$B$140,"Injury GB")</f>
+        <f>COUNTIF($B$5:$B$140,"Injury")</f>
         <v/>
       </c>
       <c r="H2" s="19">
-        <f>COUNTIF($B$5:$B$140,"Devastating Injury GB")</f>
+        <f>COUNTIF($B$5:$B$140,"Devastating Injury")</f>
         <v/>
       </c>
       <c r="I2" s="17">
@@ -5133,11 +5133,11 @@
     <row r="110" ht="56" customHeight="1" s="85">
       <c r="A110" s="52" t="inlineStr">
         <is>
-          <t>Injury GB</t>
+          <t>Injury</t>
         </is>
       </c>
       <c r="B110" s="53">
-        <f>COUNTIF($B$111:$B$143,"Injury GB")</f>
+        <f>COUNTIF($B$111:$B$143,"Injury")</f>
         <v/>
       </c>
       <c r="C110" s="54" t="n"/>
@@ -5153,7 +5153,7 @@
       <c r="A111" s="27" t="n"/>
       <c r="B111" s="28" t="inlineStr">
         <is>
-          <t>Injury GB</t>
+          <t>Injury</t>
         </is>
       </c>
       <c r="C111" s="56" t="inlineStr">
@@ -5178,11 +5178,11 @@
     <row r="112" ht="20" customHeight="1" s="85">
       <c r="A112" s="52" t="inlineStr">
         <is>
-          <t>Devastating Injury GB</t>
+          <t>Devastating Injury</t>
         </is>
       </c>
       <c r="B112" s="53">
-        <f>COUNTIF($B$113:$B$143,"Devastating Injury GB")</f>
+        <f>COUNTIF($B$113:$B$143,"Devastating Injury")</f>
         <v/>
       </c>
       <c r="C112" s="54" t="n"/>
@@ -5198,7 +5198,7 @@
       <c r="A113" s="27" t="n"/>
       <c r="B113" s="28" t="inlineStr">
         <is>
-          <t>Devastating Injury GB</t>
+          <t>Devastating Injury</t>
         </is>
       </c>
       <c r="C113" s="64" t="inlineStr">

</xml_diff>

<commit_message>
The rest of the deck is recounted from playtesting
- Passes 110, Moves 100, Special Moves 86, Clamps 30, Injuries 6: 380 without Varenas and Variaballs
- Swings to 20 each, Skip Pass to 10, and the other passes to 5
- Dribble and Drive at 15; Triple Threat, Pump Fake and Stepback at 10; the rest of the Moves at 5
- Every Special Move under 5 goes to 5, except Turnaround Three
- Every Clamp under 5 goes to 5, and Bone Bruise to 5
- The same counts on the sheet

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -2336,7 +2336,7 @@
       </c>
       <c r="E8" s="26" t="n"/>
       <c r="F8" s="33" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G8" s="72" t="n"/>
       <c r="H8" s="71" t="n"/>
@@ -2362,7 +2362,7 @@
       </c>
       <c r="E9" s="7" t="n"/>
       <c r="F9" s="34" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G9" s="70" t="n"/>
       <c r="H9" s="71" t="n"/>
@@ -2388,7 +2388,7 @@
       </c>
       <c r="E10" s="26" t="n"/>
       <c r="F10" s="33" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="G10" s="72" t="n"/>
       <c r="H10" s="71" t="n"/>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="E11" s="7" t="n"/>
       <c r="F11" s="34" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G11" s="70" t="n"/>
       <c r="H11" s="71" t="n"/>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="E12" s="26" t="n"/>
       <c r="F12" s="33" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G12" s="72" t="n"/>
       <c r="H12" s="71" t="n"/>
@@ -2466,7 +2466,7 @@
       </c>
       <c r="E13" s="7" t="n"/>
       <c r="F13" s="34" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G13" s="70" t="n"/>
       <c r="H13" s="71" t="n"/>
@@ -2496,7 +2496,7 @@
         </is>
       </c>
       <c r="F14" s="36" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G14" s="72" t="n"/>
       <c r="H14" s="71" t="n"/>
@@ -2556,7 +2556,7 @@
         </is>
       </c>
       <c r="F16" s="36" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G16" s="72" t="inlineStr">
         <is>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="E17" s="25" t="n"/>
       <c r="F17" s="36" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G17" s="72" t="inlineStr">
         <is>
@@ -2620,7 +2620,7 @@
         </is>
       </c>
       <c r="F18" s="36" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G18" s="72" t="inlineStr">
         <is>
@@ -2650,7 +2650,7 @@
       </c>
       <c r="E19" s="25" t="n"/>
       <c r="F19" s="36" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G19" s="72" t="inlineStr">
         <is>
@@ -2725,7 +2725,7 @@
       </c>
       <c r="E22" s="26" t="n"/>
       <c r="F22" s="33" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G22" s="72" t="n"/>
       <c r="H22" s="71" t="n"/>
@@ -2755,7 +2755,7 @@
         </is>
       </c>
       <c r="F23" s="32" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G23" s="70" t="n"/>
       <c r="H23" s="71" t="n"/>
@@ -2781,7 +2781,7 @@
       </c>
       <c r="E24" s="26" t="n"/>
       <c r="F24" s="33" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G24" s="72" t="n"/>
       <c r="H24" s="71" t="n"/>
@@ -2841,7 +2841,7 @@
         </is>
       </c>
       <c r="F26" s="36" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G26" s="72" t="inlineStr">
         <is>
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="F27" s="32" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G27" s="70" t="n"/>
       <c r="H27" s="71" t="n"/>
@@ -2953,7 +2953,7 @@
       </c>
       <c r="E30" s="26" t="n"/>
       <c r="F30" s="33" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G30" s="77" t="inlineStr">
         <is>
@@ -3017,7 +3017,7 @@
         </is>
       </c>
       <c r="F32" s="32" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G32" s="70" t="inlineStr">
         <is>
@@ -3054,7 +3054,7 @@
         </is>
       </c>
       <c r="F33" s="36" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G33" s="72" t="inlineStr">
         <is>
@@ -3084,7 +3084,7 @@
       </c>
       <c r="E34" s="30" t="n"/>
       <c r="F34" s="35" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G34" s="78" t="inlineStr">
         <is>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="F36" s="36" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G36" s="72" t="n"/>
       <c r="H36" s="71" t="n"/>
@@ -3169,7 +3169,7 @@
         </is>
       </c>
       <c r="F37" s="32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G37" s="74" t="inlineStr">
         <is>
@@ -3203,7 +3203,7 @@
         </is>
       </c>
       <c r="F38" s="36" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G38" s="72" t="n"/>
       <c r="H38" s="71" t="n"/>
@@ -3263,7 +3263,7 @@
         </is>
       </c>
       <c r="F40" s="36" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G40" s="72" t="n"/>
       <c r="H40" s="71" t="n"/>
@@ -3293,7 +3293,7 @@
         </is>
       </c>
       <c r="F41" s="32" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G41" s="70" t="n"/>
       <c r="H41" s="71" t="n"/>
@@ -3323,7 +3323,7 @@
         </is>
       </c>
       <c r="F42" s="36" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G42" s="72" t="n"/>
       <c r="H42" s="71" t="n"/>
@@ -3353,7 +3353,7 @@
         </is>
       </c>
       <c r="F43" s="32" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G43" s="70" t="n"/>
       <c r="H43" s="71" t="n"/>
@@ -3383,7 +3383,7 @@
         </is>
       </c>
       <c r="F44" s="36" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G44" s="72" t="n"/>
       <c r="H44" s="71" t="n"/>
@@ -3413,7 +3413,7 @@
         </is>
       </c>
       <c r="F45" s="32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G45" s="70" t="n"/>
       <c r="H45" s="71" t="n"/>
@@ -3503,7 +3503,7 @@
         </is>
       </c>
       <c r="F48" s="59" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G48" s="75" t="inlineStr">
         <is>
@@ -3657,7 +3657,7 @@
       </c>
       <c r="E54" s="26" t="n"/>
       <c r="F54" s="33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G54" s="77" t="inlineStr">
         <is>
@@ -3687,7 +3687,7 @@
       </c>
       <c r="E55" s="7" t="n"/>
       <c r="F55" s="34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G55" s="80" t="inlineStr">
         <is>
@@ -3747,7 +3747,7 @@
       </c>
       <c r="E57" s="58" t="n"/>
       <c r="F57" s="59" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G57" s="83" t="inlineStr">
         <is>
@@ -5168,7 +5168,7 @@
       </c>
       <c r="E111" s="58" t="n"/>
       <c r="F111" s="59" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G111" s="75" t="n"/>
       <c r="H111" s="76" t="n"/>

</xml_diff>

<commit_message>
Three-Ball, Man-To-Man and a new Kick-Out; the threes stop printing their extra point
- Three-Ball (5): SHOT -10%, shoot, a three
- Man-To-Man (5): the guarded player's SHOT drops 10% for every card played
- Kick-Out: SHOT +10%, draw 2, the passer's Clamps go to the receiver, who shoots a three after drawing
- From the Hash, From the Logo and Full-Court Heave drop to 3
- No three says +1 point in its text; the icon says it
- On the sheet as well, with Close-Out and Zone marked not in the game until their rules are settled
- Monster Ball and its rebound scene are in the design doc; nudging the three mark is on the todo

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -2089,7 +2089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J145"/>
+  <dimension ref="A1:J149"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="22.25" customHeight="1"/>
   <cols>
     <col width="15.5" customWidth="1" style="8" min="1" max="1"/>
@@ -2170,42 +2170,43 @@
         </is>
       </c>
       <c r="B2" s="12">
-        <f>COUNTIF($B$5:$B$140,"Pass")</f>
+        <f>COUNTIF($B$5:$B$144,"Pass")</f>
         <v/>
       </c>
       <c r="C2" s="13">
-        <f>COUNTIF($B$5:$B$140,"Move")+COUNTIF($B$5:$B$140,"Special Move")</f>
+        <f>COUNTIF($B$5:$B$144,"Move")+COUNTIF($B$5:$B$144,"Special Move")</f>
         <v/>
       </c>
       <c r="D2" s="14">
-        <f>COUNTIF($B$5:$B$140,"Clamp")</f>
+        <f>COUNTIF($B$5:$B$144,"Clamp")</f>
         <v/>
       </c>
       <c r="E2" s="15">
-        <f>COUNTIF($B$5:$B$140,"Whistle")</f>
+        <f>COUNTIF($B$5:$B$144,"Whistle")</f>
         <v/>
       </c>
       <c r="F2" s="16">
-        <f>COUNTIF($B$5:$B$140,"Game Break")</f>
+        <f>COUNTIF($B$5:$B$144,"Game Break")</f>
         <v/>
       </c>
       <c r="G2" s="18">
-        <f>COUNTIF($B$5:$B$140,"Injury")</f>
+        <f>COUNTIF($B$5:$B$144,"Injury")</f>
         <v/>
       </c>
       <c r="H2" s="19">
-        <f>COUNTIF($B$5:$B$140,"Devastating Injury")</f>
+        <f>COUNTIF($B$5:$B$144,"Devastating Injury")</f>
         <v/>
       </c>
       <c r="I2" s="17">
-        <f>COUNTIF($B$5:$B$140,"Intangible")</f>
+        <f>COUNTIF($B$5:$B$144,"Intangible")</f>
         <v/>
       </c>
       <c r="J2" s="87">
-        <f>SUM(B2:E2)+COUNTIF($B$5:$B$140,"Game Break")+SUM(G2:I2)</f>
+        <f>SUM(B2:E2)+COUNTIF($B$5:$B$144,"Game Break")+SUM(G2:I2)</f>
         <v/>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="20.75" customHeight="1" s="85">
       <c r="A4" s="81" t="inlineStr">
         <is>
@@ -2249,7 +2250,7 @@
         </is>
       </c>
       <c r="B5" s="53">
-        <f>COUNTIF($B$6:$B$143,"Pass")</f>
+        <f>COUNTIF($B$6:$B$147,"Pass")</f>
         <v/>
       </c>
       <c r="C5" s="54" t="n"/>
@@ -2611,20 +2612,16 @@
       </c>
       <c r="D18" s="25" t="inlineStr">
         <is>
-          <t>SHOT +20%. Upgraded to 3pt. Pass to player of choice</t>
-        </is>
-      </c>
-      <c r="E18" s="25" t="inlineStr">
-        <is>
-          <t>Following Drive: draw 1. Following a Dribble Drive: gain 1 AST also</t>
-        </is>
-      </c>
+          <t>SHOT +10%. Draw 2 Cards. Move all your Clamps to Receiver, and they immediately attempt a three</t>
+        </is>
+      </c>
+      <c r="E18" s="25" t="n"/>
       <c r="F18" s="36" t="n">
         <v>5</v>
       </c>
       <c r="G18" s="72" t="inlineStr">
         <is>
-          <t>The most it grants is a draw and 1 AST</t>
+          <t>They attempt the three after their draw</t>
         </is>
       </c>
       <c r="H18" s="71" t="n"/>
@@ -2694,7 +2691,7 @@
         </is>
       </c>
       <c r="B21" s="53">
-        <f>COUNTIF($B$22:$B$143,"Move")+COUNTIF($B$22:$B$143,"Special Move")</f>
+        <f>COUNTIF($B$22:$B$147,"Move")+COUNTIF($B$22:$B$147,"Special Move")</f>
         <v/>
       </c>
       <c r="C21" s="54" t="n"/>
@@ -3102,7 +3099,7 @@
         </is>
       </c>
       <c r="B35" s="53">
-        <f>COUNTIF($B$36:$B$143,"Special Move")</f>
+        <f>COUNTIF($B$36:$B$147,"Special Move")</f>
         <v/>
       </c>
       <c r="C35" s="54" t="n"/>
@@ -3199,7 +3196,7 @@
       </c>
       <c r="E38" s="25" t="inlineStr">
         <is>
-          <t>Shoot the ball. +1 Point on make</t>
+          <t>Shoot the ball</t>
         </is>
       </c>
       <c r="F38" s="36" t="n">
@@ -3259,11 +3256,11 @@
       </c>
       <c r="E40" s="25" t="inlineStr">
         <is>
-          <t>Shoot the ball. +1 Point on make</t>
+          <t>Shoot the ball</t>
         </is>
       </c>
       <c r="F40" s="36" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G40" s="72" t="n"/>
       <c r="H40" s="71" t="n"/>
@@ -3289,11 +3286,11 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>Shoot the ball. +1 Point on make</t>
+          <t>Shoot the ball</t>
         </is>
       </c>
       <c r="F41" s="32" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G41" s="70" t="n"/>
       <c r="H41" s="71" t="n"/>
@@ -3319,11 +3316,11 @@
       </c>
       <c r="E42" s="25" t="inlineStr">
         <is>
-          <t>Shoot the ball. +1 Point on make</t>
+          <t>Shoot the ball</t>
         </is>
       </c>
       <c r="F42" s="36" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G42" s="72" t="n"/>
       <c r="H42" s="71" t="n"/>
@@ -3439,7 +3436,7 @@
       </c>
       <c r="E46" s="25" t="inlineStr">
         <is>
-          <t>Shoot the ball. +1 Point on make</t>
+          <t>Shoot the ball</t>
         </is>
       </c>
       <c r="F46" s="36" t="n">
@@ -3499,7 +3496,7 @@
       </c>
       <c r="E48" s="58" t="inlineStr">
         <is>
-          <t>Shoot the ball. +1 Point on make. Selected players receive +1 AST on a make</t>
+          <t>Shoot the ball. Selected players receive +1 AST on a make</t>
         </is>
       </c>
       <c r="F48" s="59" t="n">
@@ -3589,54 +3586,50 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="54" customHeight="1" s="85">
-      <c r="A52" s="52" t="inlineStr">
+    <row r="52" ht="47" customHeight="1" s="85">
+      <c r="B52" s="0" t="inlineStr">
+        <is>
+          <t>Special Move</t>
+        </is>
+      </c>
+      <c r="C52" s="0" t="inlineStr">
+        <is>
+          <t>Three-Ball</t>
+        </is>
+      </c>
+      <c r="D52" s="0" t="inlineStr">
+        <is>
+          <t>SHOT -10%</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Shoot the ball</t>
+        </is>
+      </c>
+      <c r="F52" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="G52" s="0" t="n"/>
+    </row>
+    <row r="53" ht="54" customHeight="1" s="85">
+      <c r="A53" s="52" t="inlineStr">
         <is>
           <t>Clamp</t>
         </is>
       </c>
-      <c r="B52" s="53">
-        <f>COUNTIF($B$53:$B$143,"Clamp")</f>
+      <c r="B53" s="53">
+        <f>COUNTIF($B$54:$B$147,"Clamp")</f>
         <v/>
       </c>
-      <c r="C52" s="54" t="n"/>
-      <c r="D52" s="54" t="n"/>
-      <c r="E52" s="54" t="n"/>
-      <c r="F52" s="55" t="n"/>
-      <c r="G52" s="66" t="n"/>
-      <c r="H52" s="67" t="n"/>
-      <c r="I52" s="67" t="n"/>
-      <c r="J52" s="67" t="n"/>
-    </row>
-    <row r="53" ht="28" customHeight="1" s="85">
-      <c r="A53" s="21" t="n"/>
-      <c r="B53" s="22" t="inlineStr">
-        <is>
-          <t>Clamp</t>
-        </is>
-      </c>
-      <c r="C53" s="23" t="inlineStr">
-        <is>
-          <t>Contest</t>
-        </is>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>Next player SHOT -25% if they shoot</t>
-        </is>
-      </c>
-      <c r="E53" s="7" t="n"/>
-      <c r="F53" s="34" t="n">
-        <v>10</v>
-      </c>
-      <c r="G53" s="80" t="inlineStr">
-        <is>
-          <t>1 def</t>
-        </is>
-      </c>
-      <c r="H53" s="71" t="n"/>
-      <c r="I53" s="71" t="n"/>
-      <c r="J53" s="71" t="n"/>
+      <c r="C53" s="54" t="n"/>
+      <c r="D53" s="54" t="n"/>
+      <c r="E53" s="54" t="n"/>
+      <c r="F53" s="55" t="n"/>
+      <c r="G53" s="66" t="n"/>
+      <c r="H53" s="67" t="n"/>
+      <c r="I53" s="67" t="n"/>
+      <c r="J53" s="67" t="n"/>
     </row>
     <row r="54" ht="28" customHeight="1" s="85">
       <c r="A54" s="21" t="n"/>
@@ -3645,23 +3638,23 @@
           <t>Clamp</t>
         </is>
       </c>
-      <c r="C54" s="24" t="inlineStr">
-        <is>
-          <t>Double-Team</t>
-        </is>
-      </c>
-      <c r="D54" s="25" t="inlineStr">
-        <is>
-          <t>Next Player cannot play 2 random cards from hand.</t>
-        </is>
-      </c>
-      <c r="E54" s="26" t="n"/>
-      <c r="F54" s="33" t="n">
-        <v>5</v>
-      </c>
-      <c r="G54" s="77" t="inlineStr">
-        <is>
-          <t>2 def</t>
+      <c r="C54" s="23" t="inlineStr">
+        <is>
+          <t>Contest</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>Next player SHOT -25% if they shoot</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="n"/>
+      <c r="F54" s="34" t="n">
+        <v>10</v>
+      </c>
+      <c r="G54" s="80" t="inlineStr">
+        <is>
+          <t>1 def</t>
         </is>
       </c>
       <c r="H54" s="71" t="n"/>
@@ -3675,236 +3668,252 @@
           <t>Clamp</t>
         </is>
       </c>
-      <c r="C55" s="23" t="inlineStr">
-        <is>
-          <t>Full-Court Press</t>
-        </is>
-      </c>
-      <c r="D55" s="6" t="inlineStr">
-        <is>
-          <t>Next player discards 2 cards at the start of their turn</t>
-        </is>
-      </c>
-      <c r="E55" s="7" t="n"/>
-      <c r="F55" s="34" t="n">
+      <c r="C55" s="24" t="inlineStr">
+        <is>
+          <t>Double-Team</t>
+        </is>
+      </c>
+      <c r="D55" s="25" t="inlineStr">
+        <is>
+          <t>Next Player cannot play 2 random cards from hand.</t>
+        </is>
+      </c>
+      <c r="E55" s="26" t="n"/>
+      <c r="F55" s="33" t="n">
         <v>5</v>
       </c>
-      <c r="G55" s="80" t="inlineStr">
-        <is>
-          <t>1 def</t>
+      <c r="G55" s="77" t="inlineStr">
+        <is>
+          <t>2 def</t>
         </is>
       </c>
       <c r="H55" s="71" t="n"/>
       <c r="I55" s="71" t="n"/>
       <c r="J55" s="71" t="n"/>
     </row>
-    <row r="56" ht="42" customHeight="1" s="85">
+    <row r="56" ht="28" customHeight="1" s="85">
       <c r="A56" s="21" t="n"/>
       <c r="B56" s="22" t="inlineStr">
         <is>
           <t>Clamp</t>
         </is>
       </c>
-      <c r="C56" s="24" t="inlineStr">
-        <is>
-          <t>Trap</t>
-        </is>
-      </c>
-      <c r="D56" s="41" t="inlineStr">
-        <is>
-          <t>Next player can only play Pass cards during their turn</t>
-        </is>
-      </c>
-      <c r="E56" s="26" t="n"/>
-      <c r="F56" s="33" t="n">
+      <c r="C56" s="23" t="inlineStr">
+        <is>
+          <t>Full-Court Press</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>Next player discards 2 cards at the start of their turn</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="n"/>
+      <c r="F56" s="34" t="n">
         <v>5</v>
       </c>
-      <c r="G56" s="77" t="inlineStr">
-        <is>
-          <t>They can still shoot as another option; 3 def</t>
+      <c r="G56" s="80" t="inlineStr">
+        <is>
+          <t>1 def</t>
         </is>
       </c>
       <c r="H56" s="71" t="n"/>
       <c r="I56" s="71" t="n"/>
       <c r="J56" s="71" t="n"/>
     </row>
-    <row r="57" ht="40" customHeight="1" s="85">
-      <c r="A57" s="27" t="n"/>
-      <c r="B57" s="28" t="inlineStr">
+    <row r="57" ht="42" customHeight="1" s="85">
+      <c r="A57" s="21" t="n"/>
+      <c r="B57" s="22" t="inlineStr">
         <is>
           <t>Clamp</t>
         </is>
       </c>
-      <c r="C57" s="56" t="inlineStr">
+      <c r="C57" s="24" t="inlineStr">
+        <is>
+          <t>Trap</t>
+        </is>
+      </c>
+      <c r="D57" s="41" t="inlineStr">
+        <is>
+          <t>Next player can only play Pass cards during their turn</t>
+        </is>
+      </c>
+      <c r="E57" s="26" t="n"/>
+      <c r="F57" s="33" t="n">
+        <v>5</v>
+      </c>
+      <c r="G57" s="77" t="inlineStr">
+        <is>
+          <t>They can still shoot as another option; 3 def</t>
+        </is>
+      </c>
+      <c r="H57" s="71" t="n"/>
+      <c r="I57" s="71" t="n"/>
+      <c r="J57" s="71" t="n"/>
+    </row>
+    <row r="58" ht="40" customHeight="1" s="85">
+      <c r="A58" s="27" t="n"/>
+      <c r="B58" s="28" t="inlineStr">
+        <is>
+          <t>Clamp</t>
+        </is>
+      </c>
+      <c r="C58" s="56" t="inlineStr">
         <is>
           <t>Triple-Team</t>
         </is>
       </c>
-      <c r="D57" s="57" t="inlineStr">
+      <c r="D58" s="57" t="inlineStr">
         <is>
           <t>Next player cannot play 3 random cards from hand.</t>
         </is>
       </c>
-      <c r="E57" s="58" t="n"/>
-      <c r="F57" s="59" t="n">
+      <c r="E58" s="58" t="n"/>
+      <c r="F58" s="59" t="n">
         <v>5</v>
       </c>
-      <c r="G57" s="83" t="inlineStr">
+      <c r="G58" s="83" t="inlineStr">
         <is>
           <t>3 def</t>
         </is>
       </c>
-      <c r="H57" s="76" t="n"/>
-      <c r="I57" s="76" t="n"/>
-      <c r="J57" s="76" t="n"/>
-    </row>
-    <row r="58" ht="30" customHeight="1" s="85">
-      <c r="A58" s="52" t="inlineStr">
+      <c r="H58" s="76" t="n"/>
+      <c r="I58" s="76" t="n"/>
+      <c r="J58" s="76" t="n"/>
+    </row>
+    <row r="59" ht="40" customHeight="1" s="85">
+      <c r="A59" s="27" t="n"/>
+      <c r="B59" s="28" t="inlineStr">
+        <is>
+          <t>Clamp</t>
+        </is>
+      </c>
+      <c r="C59" s="56" t="inlineStr">
+        <is>
+          <t>Close-Out</t>
+        </is>
+      </c>
+      <c r="D59" s="57" t="inlineStr">
+        <is>
+          <t>Player cannot attempt a three-pointer</t>
+        </is>
+      </c>
+      <c r="E59" s="58" t="n"/>
+      <c r="F59" s="59" t="n">
+        <v>5</v>
+      </c>
+      <c r="G59" s="83" t="inlineStr">
+        <is>
+          <t>[NOT IN THE GAME YET]</t>
+        </is>
+      </c>
+      <c r="H59" s="76" t="n"/>
+      <c r="I59" s="76" t="n"/>
+      <c r="J59" s="76" t="n"/>
+    </row>
+    <row r="60" ht="40" customHeight="1" s="85">
+      <c r="A60" s="27" t="n"/>
+      <c r="B60" s="28" t="inlineStr">
+        <is>
+          <t>Clamp</t>
+        </is>
+      </c>
+      <c r="C60" s="56" t="inlineStr">
+        <is>
+          <t>Zone</t>
+        </is>
+      </c>
+      <c r="D60" s="57" t="inlineStr">
+        <is>
+          <t>Cannot Shoot. If player has no playable Pass cards, TOV +1; Round ends</t>
+        </is>
+      </c>
+      <c r="E60" s="58" t="n"/>
+      <c r="F60" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" s="83" t="inlineStr">
+        <is>
+          <t>[NOT IN THE GAME YET]</t>
+        </is>
+      </c>
+      <c r="H60" s="76" t="n"/>
+      <c r="I60" s="76" t="n"/>
+      <c r="J60" s="76" t="n"/>
+    </row>
+    <row r="61" ht="40" customHeight="1" s="85">
+      <c r="A61" s="27" t="n"/>
+      <c r="B61" s="28" t="inlineStr">
+        <is>
+          <t>Clamp</t>
+        </is>
+      </c>
+      <c r="C61" s="56" t="inlineStr">
+        <is>
+          <t>Man-To-Man</t>
+        </is>
+      </c>
+      <c r="D61" s="57" t="inlineStr">
+        <is>
+          <t>SHOT - 10% each time a card is played</t>
+        </is>
+      </c>
+      <c r="E61" s="58" t="n"/>
+      <c r="F61" s="59" t="n">
+        <v>5</v>
+      </c>
+      <c r="G61" s="83" t="n"/>
+      <c r="H61" s="76" t="n"/>
+      <c r="I61" s="76" t="n"/>
+      <c r="J61" s="76" t="n"/>
+    </row>
+    <row r="62" ht="30" customHeight="1" s="85">
+      <c r="A62" s="52" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="B58" s="53">
-        <f>COUNTIF($B$59:$B$143,"Whistle")</f>
+      <c r="B62" s="53">
+        <f>COUNTIF($B$63:$B$147,"Whistle")</f>
         <v/>
       </c>
-      <c r="C58" s="54" t="n"/>
-      <c r="D58" s="54" t="n"/>
-      <c r="E58" s="54" t="n"/>
-      <c r="F58" s="55" t="n"/>
-      <c r="G58" s="66" t="n"/>
-      <c r="H58" s="67" t="n"/>
-      <c r="I58" s="67" t="n"/>
-      <c r="J58" s="67" t="n"/>
-    </row>
-    <row r="59" ht="56" customHeight="1" s="85">
-      <c r="A59" s="21" t="inlineStr">
+      <c r="C62" s="54" t="n"/>
+      <c r="D62" s="54" t="n"/>
+      <c r="E62" s="54" t="n"/>
+      <c r="F62" s="55" t="n"/>
+      <c r="G62" s="66" t="n"/>
+      <c r="H62" s="67" t="n"/>
+      <c r="I62" s="67" t="n"/>
+      <c r="J62" s="67" t="n"/>
+    </row>
+    <row r="63" ht="56" customHeight="1" s="85">
+      <c r="A63" s="21" t="inlineStr">
         <is>
           <t>All whistles are limited to 1</t>
         </is>
       </c>
-      <c r="B59" s="22" t="inlineStr">
+      <c r="B63" s="22" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C59" s="23" t="inlineStr">
+      <c r="C63" s="23" t="inlineStr">
         <is>
           <t>Back Court Violation</t>
         </is>
       </c>
-      <c r="D59" s="6" t="inlineStr">
+      <c r="D63" s="6" t="inlineStr">
         <is>
           <t>Pass Card Played: Cancel that card. That player TOV +1. Move ball to player of choice</t>
         </is>
       </c>
-      <c r="E59" s="7" t="n"/>
-      <c r="F59" s="50" t="n"/>
-      <c r="G59" s="70" t="inlineStr">
+      <c r="E63" s="7" t="n"/>
+      <c r="F63" s="50" t="n"/>
+      <c r="G63" s="70" t="inlineStr">
         <is>
           <t>The player who played this whistle chooses, excluding the player who played the pass but including themselves.</t>
         </is>
       </c>
-      <c r="H59" s="71" t="n"/>
-      <c r="I59" s="71" t="n"/>
-      <c r="J59" s="71" t="n"/>
-    </row>
-    <row r="60" ht="42" customHeight="1" s="85">
-      <c r="A60" s="21" t="n"/>
-      <c r="B60" s="22" t="inlineStr">
-        <is>
-          <t>Whistle</t>
-        </is>
-      </c>
-      <c r="C60" s="37" t="inlineStr">
-        <is>
-          <t>Blocking Foul</t>
-        </is>
-      </c>
-      <c r="D60" s="40" t="inlineStr">
-        <is>
-          <t>Clamp Card Played: Cancel card. Clamped player +1 FT</t>
-        </is>
-      </c>
-      <c r="E60" s="26" t="n"/>
-      <c r="F60" s="50" t="n"/>
-      <c r="G60" s="72" t="n"/>
-      <c r="H60" s="71" t="n"/>
-      <c r="I60" s="71" t="n"/>
-      <c r="J60" s="71" t="n"/>
-    </row>
-    <row r="61" ht="42" customHeight="1" s="85">
-      <c r="A61" s="21" t="n"/>
-      <c r="B61" s="22" t="inlineStr">
-        <is>
-          <t>Whistle</t>
-        </is>
-      </c>
-      <c r="C61" s="23" t="inlineStr">
-        <is>
-          <t>Charge</t>
-        </is>
-      </c>
-      <c r="D61" s="39" t="inlineStr">
-        <is>
-          <t>Shot Attempt: Cancel. Shooter Inbounds</t>
-        </is>
-      </c>
-      <c r="E61" s="7" t="n"/>
-      <c r="F61" s="50" t="n"/>
-      <c r="G61" s="70" t="n"/>
-      <c r="H61" s="71" t="n"/>
-      <c r="I61" s="71" t="n"/>
-      <c r="J61" s="71" t="n"/>
-    </row>
-    <row r="62" ht="42" customHeight="1" s="85">
-      <c r="A62" s="21" t="n"/>
-      <c r="B62" s="22" t="inlineStr">
-        <is>
-          <t>Whistle</t>
-        </is>
-      </c>
-      <c r="C62" s="24" t="inlineStr">
-        <is>
-          <t>Cleared to Play</t>
-        </is>
-      </c>
-      <c r="D62" s="25" t="inlineStr">
-        <is>
-          <t>Injury Card Played: Cancel card.</t>
-        </is>
-      </c>
-      <c r="E62" s="26" t="n"/>
-      <c r="F62" s="50" t="n"/>
-      <c r="G62" s="72" t="n"/>
-      <c r="H62" s="71" t="n"/>
-      <c r="I62" s="71" t="n"/>
-      <c r="J62" s="71" t="n"/>
-    </row>
-    <row r="63" ht="28" customHeight="1" s="85">
-      <c r="A63" s="21" t="n"/>
-      <c r="B63" s="22" t="inlineStr">
-        <is>
-          <t>Whistle</t>
-        </is>
-      </c>
-      <c r="C63" s="23" t="inlineStr">
-        <is>
-          <t>Coach’s Challenge</t>
-        </is>
-      </c>
-      <c r="D63" s="6" t="inlineStr">
-        <is>
-          <t>Any Whistle Card Played: Cancel card.</t>
-        </is>
-      </c>
-      <c r="E63" s="7" t="inlineStr">
-        <is>
-          <t>Pull a Timeout from the discards, if one is there, and take it</t>
-        </is>
-      </c>
-      <c r="F63" s="50" t="n"/>
-      <c r="G63" s="70" t="n"/>
       <c r="H63" s="71" t="n"/>
       <c r="I63" s="71" t="n"/>
       <c r="J63" s="71" t="n"/>
@@ -3918,30 +3927,22 @@
       </c>
       <c r="C64" s="37" t="inlineStr">
         <is>
-          <t>Delay-of-Game Warning</t>
-        </is>
-      </c>
-      <c r="D64" s="41" t="inlineStr">
-        <is>
-          <t>Lower Shot Clock with a card: Cancel that card's effects</t>
-        </is>
-      </c>
-      <c r="E64" s="25" t="inlineStr">
-        <is>
-          <t>If 2nd time activated this round: Whistle player takes 1 FT in addition</t>
-        </is>
-      </c>
-      <c r="F64" s="51" t="n"/>
-      <c r="G64" s="73" t="inlineStr">
-        <is>
-          <t>The Shot Clock reduction still applies. Game Breaks do not count — those are game events, not cards the player activates.</t>
-        </is>
-      </c>
+          <t>Blocking Foul</t>
+        </is>
+      </c>
+      <c r="D64" s="40" t="inlineStr">
+        <is>
+          <t>Clamp Card Played: Cancel card. Clamped player +1 FT</t>
+        </is>
+      </c>
+      <c r="E64" s="26" t="n"/>
+      <c r="F64" s="50" t="n"/>
+      <c r="G64" s="72" t="n"/>
       <c r="H64" s="71" t="n"/>
       <c r="I64" s="71" t="n"/>
       <c r="J64" s="71" t="n"/>
     </row>
-    <row r="65" ht="29" customHeight="1" s="85">
+    <row r="65" ht="42" customHeight="1" s="85">
       <c r="A65" s="21" t="n"/>
       <c r="B65" s="22" t="inlineStr">
         <is>
@@ -3950,40 +3951,36 @@
       </c>
       <c r="C65" s="23" t="inlineStr">
         <is>
-          <t>Double Dribble</t>
-        </is>
-      </c>
-      <c r="D65" s="6" t="inlineStr">
-        <is>
-          <t>Dribble Move Card Played (Dribble, Rhythm Dribble, etc.): Cancel card. Discard 1 card. TOV +1</t>
+          <t>Charge</t>
+        </is>
+      </c>
+      <c r="D65" s="39" t="inlineStr">
+        <is>
+          <t>Shot Attempt: Cancel. Shooter Inbounds</t>
         </is>
       </c>
       <c r="E65" s="7" t="n"/>
       <c r="F65" s="50" t="n"/>
-      <c r="G65" s="70" t="inlineStr">
-        <is>
-          <t>The dribbling player inbounds. The round is NOT incremented.</t>
-        </is>
-      </c>
+      <c r="G65" s="70" t="n"/>
       <c r="H65" s="71" t="n"/>
       <c r="I65" s="71" t="n"/>
       <c r="J65" s="71" t="n"/>
     </row>
-    <row r="66" ht="20" customHeight="1" s="85">
+    <row r="66" ht="42" customHeight="1" s="85">
       <c r="A66" s="21" t="n"/>
       <c r="B66" s="22" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C66" s="37" t="inlineStr">
-        <is>
-          <t>Flagrant Foul</t>
-        </is>
-      </c>
-      <c r="D66" s="41" t="inlineStr">
-        <is>
-          <t>Clamp Card Played: Cancel card. Clamper discard 1. Clamped player +1 FT then gets ball</t>
+      <c r="C66" s="24" t="inlineStr">
+        <is>
+          <t>Cleared to Play</t>
+        </is>
+      </c>
+      <c r="D66" s="25" t="inlineStr">
+        <is>
+          <t>Injury Card Played: Cancel card.</t>
         </is>
       </c>
       <c r="E66" s="26" t="n"/>
@@ -4000,48 +3997,60 @@
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C67" s="37" t="inlineStr">
-        <is>
-          <t>Flagrant Foul II</t>
-        </is>
-      </c>
-      <c r="D67" s="38" t="inlineStr">
-        <is>
-          <t>Clamp Card Played: Cancel card. Clamper discards Bag. Clamped player +1 FT then gets ball</t>
-        </is>
-      </c>
-      <c r="E67" s="7" t="n"/>
+      <c r="C67" s="23" t="inlineStr">
+        <is>
+          <t>Coach’s Challenge</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>Any Whistle Card Played: Cancel card.</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>Pull a Timeout from the discards, if one is there, and take it</t>
+        </is>
+      </c>
       <c r="F67" s="50" t="n"/>
       <c r="G67" s="70" t="n"/>
       <c r="H67" s="71" t="n"/>
       <c r="I67" s="71" t="n"/>
       <c r="J67" s="71" t="n"/>
     </row>
-    <row r="68" ht="28" customHeight="1" s="85">
+    <row r="68" ht="42" customHeight="1" s="85">
       <c r="A68" s="21" t="n"/>
       <c r="B68" s="22" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C68" s="24" t="inlineStr">
-        <is>
-          <t>Goaltending</t>
-        </is>
-      </c>
-      <c r="D68" s="25" t="inlineStr">
-        <is>
-          <t>Clamp Card Played: Cancel card. Clamped player +2 points. End round.</t>
-        </is>
-      </c>
-      <c r="E68" s="26" t="n"/>
-      <c r="F68" s="50" t="n"/>
-      <c r="G68" s="72" t="n"/>
+      <c r="C68" s="37" t="inlineStr">
+        <is>
+          <t>Delay-of-Game Warning</t>
+        </is>
+      </c>
+      <c r="D68" s="41" t="inlineStr">
+        <is>
+          <t>Lower Shot Clock with a card: Cancel that card's effects</t>
+        </is>
+      </c>
+      <c r="E68" s="25" t="inlineStr">
+        <is>
+          <t>If 2nd time activated this round: Whistle player takes 1 FT in addition</t>
+        </is>
+      </c>
+      <c r="F68" s="51" t="n"/>
+      <c r="G68" s="73" t="inlineStr">
+        <is>
+          <t>The Shot Clock reduction still applies. Game Breaks do not count — those are game events, not cards the player activates.</t>
+        </is>
+      </c>
       <c r="H68" s="71" t="n"/>
       <c r="I68" s="71" t="n"/>
       <c r="J68" s="71" t="n"/>
     </row>
-    <row r="69" ht="14" customHeight="1" s="85">
+    <row r="69" ht="29" customHeight="1" s="85">
       <c r="A69" s="21" t="n"/>
       <c r="B69" s="22" t="inlineStr">
         <is>
@@ -4050,36 +4059,40 @@
       </c>
       <c r="C69" s="23" t="inlineStr">
         <is>
-          <t>Inadvertent Whistle</t>
-        </is>
-      </c>
-      <c r="D69" s="38" t="inlineStr">
-        <is>
-          <t>Any other whistle triggers: Cancel that card. Turn player draws 1 card.</t>
+          <t>Double Dribble</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>Dribble Move Card Played (Dribble, Rhythm Dribble, etc.): Cancel card. Discard 1 card. TOV +1</t>
         </is>
       </c>
       <c r="E69" s="7" t="n"/>
       <c r="F69" s="50" t="n"/>
-      <c r="G69" s="70" t="n"/>
+      <c r="G69" s="70" t="inlineStr">
+        <is>
+          <t>The dribbling player inbounds. The round is NOT incremented.</t>
+        </is>
+      </c>
       <c r="H69" s="71" t="n"/>
       <c r="I69" s="71" t="n"/>
       <c r="J69" s="71" t="n"/>
     </row>
-    <row r="70" ht="14" customHeight="1" s="85">
+    <row r="70" ht="20" customHeight="1" s="85">
       <c r="A70" s="21" t="n"/>
       <c r="B70" s="22" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C70" s="24" t="inlineStr">
-        <is>
-          <t>Official Review</t>
+      <c r="C70" s="37" t="inlineStr">
+        <is>
+          <t>Flagrant Foul</t>
         </is>
       </c>
       <c r="D70" s="41" t="inlineStr">
         <is>
-          <t>Intangible Played: Discard all Intangibles from player.</t>
+          <t>Clamp Card Played: Cancel card. Clamper discard 1. Clamped player +1 FT then gets ball</t>
         </is>
       </c>
       <c r="E70" s="26" t="n"/>
@@ -4089,30 +4102,26 @@
       <c r="I70" s="71" t="n"/>
       <c r="J70" s="71" t="n"/>
     </row>
-    <row r="71" ht="14" customHeight="1" s="85">
+    <row r="71" ht="28" customHeight="1" s="85">
       <c r="A71" s="21" t="n"/>
       <c r="B71" s="22" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C71" s="23" t="inlineStr">
-        <is>
-          <t>Shot Clock Violation</t>
+      <c r="C71" s="37" t="inlineStr">
+        <is>
+          <t>Flagrant Foul II</t>
         </is>
       </c>
       <c r="D71" s="38" t="inlineStr">
         <is>
-          <t>Shot Clock is changed: TOV +1. Ball OOB</t>
+          <t>Clamp Card Played: Cancel card. Clamper discards Bag. Clamped player +1 FT then gets ball</t>
         </is>
       </c>
       <c r="E71" s="7" t="n"/>
       <c r="F71" s="50" t="n"/>
-      <c r="G71" s="70" t="inlineStr">
-        <is>
-          <t>This inbound does NOT increment the round.</t>
-        </is>
-      </c>
+      <c r="G71" s="70" t="n"/>
       <c r="H71" s="71" t="n"/>
       <c r="I71" s="71" t="n"/>
       <c r="J71" s="71" t="n"/>
@@ -4126,12 +4135,12 @@
       </c>
       <c r="C72" s="24" t="inlineStr">
         <is>
-          <t>Technical Foul</t>
-        </is>
-      </c>
-      <c r="D72" s="41" t="inlineStr">
-        <is>
-          <t>Any Non-Whistle Card Played: Cancel card. Take 1 FT</t>
+          <t>Goaltending</t>
+        </is>
+      </c>
+      <c r="D72" s="25" t="inlineStr">
+        <is>
+          <t>Clamp Card Played: Cancel card. Clamped player +2 points. End round.</t>
         </is>
       </c>
       <c r="E72" s="26" t="n"/>
@@ -4141,7 +4150,7 @@
       <c r="I72" s="71" t="n"/>
       <c r="J72" s="71" t="n"/>
     </row>
-    <row r="73" ht="28" customHeight="1" s="85">
+    <row r="73" ht="14" customHeight="1" s="85">
       <c r="A73" s="21" t="n"/>
       <c r="B73" s="22" t="inlineStr">
         <is>
@@ -4150,12 +4159,12 @@
       </c>
       <c r="C73" s="23" t="inlineStr">
         <is>
-          <t>Timeout</t>
+          <t>Inadvertent Whistle</t>
         </is>
       </c>
       <c r="D73" s="38" t="inlineStr">
         <is>
-          <t>Immediate: Reset Shot Clock. You inbound. All players draw 1 card</t>
+          <t>Any other whistle triggers: Cancel that card. Turn player draws 1 card.</t>
         </is>
       </c>
       <c r="E73" s="7" t="n"/>
@@ -4165,7 +4174,7 @@
       <c r="I73" s="71" t="n"/>
       <c r="J73" s="71" t="n"/>
     </row>
-    <row r="74" ht="28" customHeight="1" s="85">
+    <row r="74" ht="14" customHeight="1" s="85">
       <c r="A74" s="21" t="n"/>
       <c r="B74" s="22" t="inlineStr">
         <is>
@@ -4174,12 +4183,12 @@
       </c>
       <c r="C74" s="24" t="inlineStr">
         <is>
-          <t>Travel</t>
-        </is>
-      </c>
-      <c r="D74" s="25" t="inlineStr">
-        <is>
-          <t>Move card played: Cancel card. TOV +1</t>
+          <t>Official Review</t>
+        </is>
+      </c>
+      <c r="D74" s="41" t="inlineStr">
+        <is>
+          <t>Intangible Played: Discard all Intangibles from player.</t>
         </is>
       </c>
       <c r="E74" s="26" t="n"/>
@@ -4189,28 +4198,28 @@
       <c r="I74" s="71" t="n"/>
       <c r="J74" s="71" t="n"/>
     </row>
-    <row r="75" ht="28" customHeight="1" s="85">
+    <row r="75" ht="14" customHeight="1" s="85">
       <c r="A75" s="21" t="n"/>
       <c r="B75" s="22" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C75" s="24" t="inlineStr">
-        <is>
-          <t>Clear Path Foul</t>
-        </is>
-      </c>
-      <c r="D75" s="25" t="inlineStr">
-        <is>
-          <t>On Shot, when Clamped by SHOT-reducing Clamps: Cancel those Clamps. Award the points the shot was worth. Take 1 FT</t>
-        </is>
-      </c>
-      <c r="E75" s="26" t="n"/>
+      <c r="C75" s="23" t="inlineStr">
+        <is>
+          <t>Shot Clock Violation</t>
+        </is>
+      </c>
+      <c r="D75" s="38" t="inlineStr">
+        <is>
+          <t>Shot Clock is changed: TOV +1. Ball OOB</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="n"/>
       <c r="F75" s="50" t="n"/>
-      <c r="G75" s="72" t="inlineStr">
-        <is>
-          <t>Fires as the shot starts, before the cutscene. This DOES count as a completed round.</t>
+      <c r="G75" s="70" t="inlineStr">
+        <is>
+          <t>This inbound does NOT increment the round.</t>
         </is>
       </c>
       <c r="H75" s="71" t="n"/>
@@ -4226,217 +4235,209 @@
       </c>
       <c r="C76" s="24" t="inlineStr">
         <is>
-          <t>Play-On</t>
-        </is>
-      </c>
-      <c r="D76" s="25" t="inlineStr">
-        <is>
-          <t>Discard each Game Break drawn and draw again, until a card is not one</t>
+          <t>Technical Foul</t>
+        </is>
+      </c>
+      <c r="D76" s="41" t="inlineStr">
+        <is>
+          <t>Any Non-Whistle Card Played: Cancel card. Take 1 FT</t>
         </is>
       </c>
       <c r="E76" s="26" t="n"/>
       <c r="F76" s="50" t="n"/>
-      <c r="G76" s="72" t="inlineStr">
-        <is>
-          <t>Raised where the Break lands, like Cleared to Play — nobody plays a Break</t>
-        </is>
-      </c>
+      <c r="G76" s="72" t="n"/>
       <c r="H76" s="71" t="n"/>
       <c r="I76" s="71" t="n"/>
       <c r="J76" s="71" t="n"/>
     </row>
-    <row r="77" ht="42" customHeight="1" s="85">
-      <c r="A77" s="27" t="n"/>
-      <c r="B77" s="28" t="inlineStr">
+    <row r="77" ht="28" customHeight="1" s="85">
+      <c r="A77" s="21" t="n"/>
+      <c r="B77" s="22" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C77" s="29" t="inlineStr">
-        <is>
-          <t>Crew Chief Review</t>
-        </is>
-      </c>
-      <c r="D77" s="30" t="inlineStr">
-        <is>
-          <t>Cancel a pass. The ball comes to you</t>
-        </is>
-      </c>
-      <c r="E77" s="60" t="n"/>
-      <c r="F77" s="61" t="n"/>
-      <c r="G77" s="78" t="n"/>
-      <c r="H77" s="76" t="n"/>
-      <c r="I77" s="76" t="n"/>
-      <c r="J77" s="76" t="n"/>
+      <c r="C77" s="23" t="inlineStr">
+        <is>
+          <t>Timeout</t>
+        </is>
+      </c>
+      <c r="D77" s="38" t="inlineStr">
+        <is>
+          <t>Immediate: Reset Shot Clock. You inbound. All players draw 1 card</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="n"/>
+      <c r="F77" s="50" t="n"/>
+      <c r="G77" s="70" t="n"/>
+      <c r="H77" s="71" t="n"/>
+      <c r="I77" s="71" t="n"/>
+      <c r="J77" s="71" t="n"/>
     </row>
     <row r="78" ht="28" customHeight="1" s="85">
-      <c r="A78" s="27" t="n"/>
-      <c r="B78" s="28" t="inlineStr">
+      <c r="A78" s="21" t="n"/>
+      <c r="B78" s="22" t="inlineStr">
         <is>
           <t>Whistle</t>
         </is>
       </c>
-      <c r="C78" s="29" t="inlineStr">
-        <is>
-          <t>Discontinued Dribble</t>
-        </is>
-      </c>
-      <c r="D78" s="30" t="inlineStr">
-        <is>
-          <t>Card Drawn: That player's possession ends immediately. They inbound</t>
-        </is>
-      </c>
-      <c r="E78" s="60" t="n"/>
-      <c r="F78" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="G78" s="78" t="n"/>
-      <c r="H78" s="76" t="n"/>
-      <c r="I78" s="76" t="n"/>
-      <c r="J78" s="76" t="n"/>
+      <c r="C78" s="24" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="D78" s="25" t="inlineStr">
+        <is>
+          <t>Move card played: Cancel card. TOV +1</t>
+        </is>
+      </c>
+      <c r="E78" s="26" t="n"/>
+      <c r="F78" s="50" t="n"/>
+      <c r="G78" s="72" t="n"/>
+      <c r="H78" s="71" t="n"/>
+      <c r="I78" s="71" t="n"/>
+      <c r="J78" s="71" t="n"/>
     </row>
     <row r="79" ht="28" customHeight="1" s="85">
-      <c r="A79" s="52" t="inlineStr">
-        <is>
-          <t>Retired Game Breaks</t>
-        </is>
-      </c>
-      <c r="B79" s="53">
-        <f>COUNTIF($B$80:$B$109,"Retired Game Break")</f>
-        <v/>
-      </c>
-      <c r="C79" s="54" t="n"/>
-      <c r="D79" s="54" t="n"/>
-      <c r="E79" s="54" t="n"/>
-      <c r="F79" s="55" t="n"/>
-      <c r="G79" s="66" t="n"/>
-      <c r="H79" s="67" t="n"/>
-      <c r="I79" s="67" t="n"/>
-      <c r="J79" s="67" t="n"/>
-    </row>
-    <row r="80" ht="20" customHeight="1" s="85">
+      <c r="A79" s="21" t="n"/>
+      <c r="B79" s="22" t="inlineStr">
+        <is>
+          <t>Whistle</t>
+        </is>
+      </c>
+      <c r="C79" s="24" t="inlineStr">
+        <is>
+          <t>Clear Path Foul</t>
+        </is>
+      </c>
+      <c r="D79" s="25" t="inlineStr">
+        <is>
+          <t>On Shot, when Clamped by SHOT-reducing Clamps: Cancel those Clamps. Award the points the shot was worth. Take 1 FT</t>
+        </is>
+      </c>
+      <c r="E79" s="26" t="n"/>
+      <c r="F79" s="50" t="n"/>
+      <c r="G79" s="72" t="inlineStr">
+        <is>
+          <t>Fires as the shot starts, before the cutscene. This DOES count as a completed round.</t>
+        </is>
+      </c>
+      <c r="H79" s="71" t="n"/>
+      <c r="I79" s="71" t="n"/>
+      <c r="J79" s="71" t="n"/>
+    </row>
+    <row r="80" ht="28" customHeight="1" s="85">
       <c r="A80" s="21" t="n"/>
       <c r="B80" s="22" t="inlineStr">
         <is>
-          <t>Retired Game Break</t>
+          <t>Whistle</t>
         </is>
       </c>
       <c r="C80" s="24" t="inlineStr">
         <is>
-          <t>2-Minute Warning</t>
+          <t>Play-On</t>
         </is>
       </c>
       <c r="D80" s="25" t="inlineStr">
         <is>
-          <t>All players discard down to 2 or fewer cards</t>
+          <t>Discard each Game Break drawn and draw again, until a card is not one</t>
         </is>
       </c>
       <c r="E80" s="26" t="n"/>
-      <c r="F80" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G80" s="72" t="n"/>
+      <c r="F80" s="50" t="n"/>
+      <c r="G80" s="72" t="inlineStr">
+        <is>
+          <t>Raised where the Break lands, like Cleared to Play — nobody plays a Break</t>
+        </is>
+      </c>
       <c r="H80" s="71" t="n"/>
       <c r="I80" s="71" t="n"/>
       <c r="J80" s="71" t="n"/>
     </row>
-    <row r="81" ht="28" customHeight="1" s="85">
-      <c r="A81" s="21" t="n"/>
-      <c r="B81" s="22" t="inlineStr">
-        <is>
-          <t>Retired Game Break</t>
-        </is>
-      </c>
-      <c r="C81" s="23" t="inlineStr">
-        <is>
-          <t>Benched</t>
-        </is>
-      </c>
-      <c r="D81" s="6" t="inlineStr">
-        <is>
-          <t>Immediately give ball to any other player.</t>
-        </is>
-      </c>
-      <c r="E81" s="7" t="n"/>
-      <c r="F81" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="G81" s="74" t="inlineStr">
-        <is>
-          <t>This is not a pass</t>
-        </is>
-      </c>
-      <c r="H81" s="71" t="n"/>
-      <c r="I81" s="71" t="n"/>
-      <c r="J81" s="71" t="n"/>
-    </row>
-    <row r="82" ht="20" customHeight="1" s="85">
-      <c r="A82" s="21" t="n"/>
-      <c r="B82" s="22" t="inlineStr">
-        <is>
-          <t>Retired Game Break</t>
-        </is>
-      </c>
-      <c r="C82" s="24" t="inlineStr">
-        <is>
-          <t>Crowd Noise</t>
-        </is>
-      </c>
-      <c r="D82" s="25" t="inlineStr">
-        <is>
-          <t>Discard 1 card.</t>
-        </is>
-      </c>
-      <c r="E82" s="26" t="n"/>
-      <c r="F82" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G82" s="72" t="n"/>
-      <c r="H82" s="71" t="n"/>
-      <c r="I82" s="71" t="n"/>
-      <c r="J82" s="71" t="n"/>
-    </row>
-    <row r="83" ht="42" customHeight="1" s="85">
-      <c r="A83" s="21" t="n"/>
-      <c r="B83" s="22" t="inlineStr">
-        <is>
-          <t>Retired Game Break</t>
-        </is>
-      </c>
-      <c r="C83" s="23" t="inlineStr">
-        <is>
-          <t>Designed Play</t>
-        </is>
-      </c>
-      <c r="D83" s="6" t="inlineStr">
-        <is>
-          <t>Draw up to a hand of 5</t>
-        </is>
-      </c>
-      <c r="E83" s="7" t="n"/>
-      <c r="F83" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="G83" s="70" t="n"/>
-      <c r="H83" s="71" t="n"/>
-      <c r="I83" s="71" t="n"/>
-      <c r="J83" s="71" t="n"/>
-    </row>
-    <row r="84" ht="28" customHeight="1" s="85">
+    <row r="81" ht="42" customHeight="1" s="85">
+      <c r="A81" s="27" t="n"/>
+      <c r="B81" s="28" t="inlineStr">
+        <is>
+          <t>Whistle</t>
+        </is>
+      </c>
+      <c r="C81" s="29" t="inlineStr">
+        <is>
+          <t>Crew Chief Review</t>
+        </is>
+      </c>
+      <c r="D81" s="30" t="inlineStr">
+        <is>
+          <t>Cancel a pass. The ball comes to you</t>
+        </is>
+      </c>
+      <c r="E81" s="60" t="n"/>
+      <c r="F81" s="61" t="n"/>
+      <c r="G81" s="78" t="n"/>
+      <c r="H81" s="76" t="n"/>
+      <c r="I81" s="76" t="n"/>
+      <c r="J81" s="76" t="n"/>
+    </row>
+    <row r="82" ht="28" customHeight="1" s="85">
+      <c r="A82" s="27" t="n"/>
+      <c r="B82" s="28" t="inlineStr">
+        <is>
+          <t>Whistle</t>
+        </is>
+      </c>
+      <c r="C82" s="29" t="inlineStr">
+        <is>
+          <t>Discontinued Dribble</t>
+        </is>
+      </c>
+      <c r="D82" s="30" t="inlineStr">
+        <is>
+          <t>Card Drawn: That player's possession ends immediately. They inbound</t>
+        </is>
+      </c>
+      <c r="E82" s="60" t="n"/>
+      <c r="F82" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G82" s="78" t="n"/>
+      <c r="H82" s="76" t="n"/>
+      <c r="I82" s="76" t="n"/>
+      <c r="J82" s="76" t="n"/>
+    </row>
+    <row r="83" ht="28" customHeight="1" s="85">
+      <c r="A83" s="52" t="inlineStr">
+        <is>
+          <t>Retired Game Breaks</t>
+        </is>
+      </c>
+      <c r="B83" s="53">
+        <f>COUNTIF($B$84:$B$113,"Retired Game Break")</f>
+        <v/>
+      </c>
+      <c r="C83" s="54" t="n"/>
+      <c r="D83" s="54" t="n"/>
+      <c r="E83" s="54" t="n"/>
+      <c r="F83" s="55" t="n"/>
+      <c r="G83" s="66" t="n"/>
+      <c r="H83" s="67" t="n"/>
+      <c r="I83" s="67" t="n"/>
+      <c r="J83" s="67" t="n"/>
+    </row>
+    <row r="84" ht="20" customHeight="1" s="85">
       <c r="A84" s="21" t="n"/>
       <c r="B84" s="22" t="inlineStr">
         <is>
           <t>Retired Game Break</t>
         </is>
       </c>
-      <c r="C84" s="37" t="inlineStr">
-        <is>
-          <t>Foul</t>
+      <c r="C84" s="24" t="inlineStr">
+        <is>
+          <t>2-Minute Warning</t>
         </is>
       </c>
       <c r="D84" s="25" t="inlineStr">
         <is>
-          <t>Take 1 FT</t>
+          <t>All players discard down to 2 or fewer cards</t>
         </is>
       </c>
       <c r="E84" s="26" t="n"/>
@@ -4448,7 +4449,7 @@
       <c r="I84" s="71" t="n"/>
       <c r="J84" s="71" t="n"/>
     </row>
-    <row r="85" ht="56" customHeight="1" s="85">
+    <row r="85" ht="28" customHeight="1" s="85">
       <c r="A85" s="21" t="n"/>
       <c r="B85" s="22" t="inlineStr">
         <is>
@@ -4457,24 +4458,28 @@
       </c>
       <c r="C85" s="23" t="inlineStr">
         <is>
-          <t>MVP Vote</t>
+          <t>Benched</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>Draw 3 cards up to a hand of 7</t>
+          <t>Immediately give ball to any other player.</t>
         </is>
       </c>
       <c r="E85" s="7" t="n"/>
       <c r="F85" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G85" s="70" t="n"/>
+      <c r="G85" s="74" t="inlineStr">
+        <is>
+          <t>This is not a pass</t>
+        </is>
+      </c>
       <c r="H85" s="71" t="n"/>
       <c r="I85" s="71" t="n"/>
       <c r="J85" s="71" t="n"/>
     </row>
-    <row r="86" ht="42" customHeight="1" s="85">
+    <row r="86" ht="20" customHeight="1" s="85">
       <c r="A86" s="21" t="n"/>
       <c r="B86" s="22" t="inlineStr">
         <is>
@@ -4483,12 +4488,12 @@
       </c>
       <c r="C86" s="24" t="inlineStr">
         <is>
-          <t>Off Night</t>
+          <t>Crowd Noise</t>
         </is>
       </c>
       <c r="D86" s="25" t="inlineStr">
         <is>
-          <t>SHOT -20% this possession</t>
+          <t>Discard 1 card.</t>
         </is>
       </c>
       <c r="E86" s="26" t="n"/>
@@ -4509,20 +4514,16 @@
       </c>
       <c r="C87" s="23" t="inlineStr">
         <is>
-          <t>Swallowed Whistle</t>
+          <t>Designed Play</t>
         </is>
       </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>Whistle cards cannot activate this turn.</t>
-        </is>
-      </c>
-      <c r="E87" s="6" t="inlineStr">
-        <is>
-          <t>Remains for remainder of round</t>
-        </is>
-      </c>
-      <c r="F87" s="32" t="n">
+          <t>Draw up to a hand of 5</t>
+        </is>
+      </c>
+      <c r="E87" s="7" t="n"/>
+      <c r="F87" s="34" t="n">
         <v>0</v>
       </c>
       <c r="G87" s="70" t="n"/>
@@ -4537,22 +4538,18 @@
           <t>Retired Game Break</t>
         </is>
       </c>
-      <c r="C88" s="24" t="inlineStr">
-        <is>
-          <t>Rock Fight</t>
+      <c r="C88" s="37" t="inlineStr">
+        <is>
+          <t>Foul</t>
         </is>
       </c>
       <c r="D88" s="25" t="inlineStr">
         <is>
-          <t>Players cannot shoot when SHOT is above 50%</t>
-        </is>
-      </c>
-      <c r="E88" s="25" t="inlineStr">
-        <is>
-          <t>Remains for remainder of round</t>
-        </is>
-      </c>
-      <c r="F88" s="36" t="n">
+          <t>Take 1 FT</t>
+        </is>
+      </c>
+      <c r="E88" s="26" t="n"/>
+      <c r="F88" s="33" t="n">
         <v>0</v>
       </c>
       <c r="G88" s="72" t="n"/>
@@ -4560,7 +4557,7 @@
       <c r="I88" s="71" t="n"/>
       <c r="J88" s="71" t="n"/>
     </row>
-    <row r="89" ht="28" customHeight="1" s="85">
+    <row r="89" ht="56" customHeight="1" s="85">
       <c r="A89" s="21" t="n"/>
       <c r="B89" s="22" t="inlineStr">
         <is>
@@ -4569,75 +4566,75 @@
       </c>
       <c r="C89" s="23" t="inlineStr">
         <is>
-          <t>Traded Mid-Game</t>
+          <t>MVP Vote</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>Swap hands with a random other player</t>
+          <t>Draw 3 cards up to a hand of 7</t>
         </is>
       </c>
       <c r="E89" s="7" t="n"/>
       <c r="F89" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G89" s="74" t="n"/>
+      <c r="G89" s="70" t="n"/>
       <c r="H89" s="71" t="n"/>
       <c r="I89" s="71" t="n"/>
       <c r="J89" s="71" t="n"/>
     </row>
-    <row r="90" ht="56" customHeight="1" s="85">
+    <row r="90" ht="42" customHeight="1" s="85">
       <c r="A90" s="21" t="n"/>
       <c r="B90" s="22" t="inlineStr">
         <is>
           <t>Retired Game Break</t>
         </is>
       </c>
-      <c r="C90" s="49" t="inlineStr">
-        <is>
-          <t>Salary Cap Increase</t>
-        </is>
-      </c>
-      <c r="D90" s="38" t="inlineStr">
-        <is>
-          <t>All players draw 2 cards</t>
-        </is>
-      </c>
-      <c r="E90" s="7" t="n"/>
-      <c r="F90" s="34" t="n">
+      <c r="C90" s="24" t="inlineStr">
+        <is>
+          <t>Off Night</t>
+        </is>
+      </c>
+      <c r="D90" s="25" t="inlineStr">
+        <is>
+          <t>SHOT -20% this possession</t>
+        </is>
+      </c>
+      <c r="E90" s="26" t="n"/>
+      <c r="F90" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="G90" s="74" t="n"/>
+      <c r="G90" s="72" t="n"/>
       <c r="H90" s="71" t="n"/>
       <c r="I90" s="71" t="n"/>
       <c r="J90" s="71" t="n"/>
     </row>
-    <row r="91" ht="56" customHeight="1" s="85">
+    <row r="91" ht="42" customHeight="1" s="85">
       <c r="A91" s="21" t="n"/>
       <c r="B91" s="22" t="inlineStr">
         <is>
           <t>Retired Game Break</t>
         </is>
       </c>
-      <c r="C91" s="49" t="inlineStr">
-        <is>
-          <t>All-Swissh Selection</t>
-        </is>
-      </c>
-      <c r="D91" s="38" t="inlineStr">
-        <is>
-          <t>Draw 3 cards after your next make</t>
-        </is>
-      </c>
-      <c r="E91" s="7" t="n"/>
-      <c r="F91" s="34" t="n">
+      <c r="C91" s="23" t="inlineStr">
+        <is>
+          <t>Swallowed Whistle</t>
+        </is>
+      </c>
+      <c r="D91" s="6" t="inlineStr">
+        <is>
+          <t>Whistle cards cannot activate this turn.</t>
+        </is>
+      </c>
+      <c r="E91" s="6" t="inlineStr">
+        <is>
+          <t>Remains for remainder of round</t>
+        </is>
+      </c>
+      <c r="F91" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="G91" s="74" t="inlineStr">
-        <is>
-          <t>Arms an icon in the HUD tracking the pending draws</t>
-        </is>
-      </c>
+      <c r="G91" s="70" t="n"/>
       <c r="H91" s="71" t="n"/>
       <c r="I91" s="71" t="n"/>
       <c r="J91" s="71" t="n"/>
@@ -4649,56 +4646,56 @@
           <t>Retired Game Break</t>
         </is>
       </c>
-      <c r="C92" s="49" t="inlineStr">
-        <is>
-          <t>All Star Selection</t>
-        </is>
-      </c>
-      <c r="D92" s="38" t="inlineStr">
-        <is>
-          <t>Draw 2 cards</t>
-        </is>
-      </c>
-      <c r="E92" s="7" t="n"/>
-      <c r="F92" s="34" t="n">
+      <c r="C92" s="24" t="inlineStr">
+        <is>
+          <t>Rock Fight</t>
+        </is>
+      </c>
+      <c r="D92" s="25" t="inlineStr">
+        <is>
+          <t>Players cannot shoot when SHOT is above 50%</t>
+        </is>
+      </c>
+      <c r="E92" s="25" t="inlineStr">
+        <is>
+          <t>Remains for remainder of round</t>
+        </is>
+      </c>
+      <c r="F92" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="G92" s="74" t="n"/>
+      <c r="G92" s="72" t="n"/>
       <c r="H92" s="71" t="n"/>
       <c r="I92" s="71" t="n"/>
       <c r="J92" s="71" t="n"/>
     </row>
-    <row r="93" ht="42" customHeight="1" s="85">
+    <row r="93" ht="28" customHeight="1" s="85">
       <c r="A93" s="21" t="n"/>
       <c r="B93" s="22" t="inlineStr">
         <is>
           <t>Retired Game Break</t>
         </is>
       </c>
-      <c r="C93" s="49" t="inlineStr">
-        <is>
-          <t>Hit the Bike</t>
-        </is>
-      </c>
-      <c r="D93" s="38" t="inlineStr">
-        <is>
-          <t>Discard all Injuries. Draw 1 card. Give possession to another player</t>
+      <c r="C93" s="23" t="inlineStr">
+        <is>
+          <t>Traded Mid-Game</t>
+        </is>
+      </c>
+      <c r="D93" s="6" t="inlineStr">
+        <is>
+          <t>Swap hands with a random other player</t>
         </is>
       </c>
       <c r="E93" s="7" t="n"/>
       <c r="F93" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G93" s="74" t="inlineStr">
-        <is>
-          <t>This is not a pass</t>
-        </is>
-      </c>
+      <c r="G93" s="74" t="n"/>
       <c r="H93" s="71" t="n"/>
       <c r="I93" s="71" t="n"/>
       <c r="J93" s="71" t="n"/>
     </row>
-    <row r="94" ht="28" customHeight="1" s="85">
+    <row r="94" ht="56" customHeight="1" s="85">
       <c r="A94" s="21" t="n"/>
       <c r="B94" s="22" t="inlineStr">
         <is>
@@ -4707,12 +4704,12 @@
       </c>
       <c r="C94" s="49" t="inlineStr">
         <is>
-          <t>Ice Wrap</t>
+          <t>Salary Cap Increase</t>
         </is>
       </c>
       <c r="D94" s="38" t="inlineStr">
         <is>
-          <t>Draw 1 card. Discard all Injuries. If none, draw 1 additional card</t>
+          <t>All players draw 2 cards</t>
         </is>
       </c>
       <c r="E94" s="7" t="n"/>
@@ -4724,7 +4721,7 @@
       <c r="I94" s="71" t="n"/>
       <c r="J94" s="71" t="n"/>
     </row>
-    <row r="95" ht="42" customHeight="1" s="85">
+    <row r="95" ht="56" customHeight="1" s="85">
       <c r="A95" s="21" t="n"/>
       <c r="B95" s="22" t="inlineStr">
         <is>
@@ -4733,12 +4730,12 @@
       </c>
       <c r="C95" s="49" t="inlineStr">
         <is>
-          <t>Wet Spot</t>
+          <t>All-Swissh Selection</t>
         </is>
       </c>
       <c r="D95" s="38" t="inlineStr">
         <is>
-          <t>All Injuries in the discards and deck are displayed. Take one</t>
+          <t>Draw 3 cards after your next make</t>
         </is>
       </c>
       <c r="E95" s="7" t="n"/>
@@ -4747,14 +4744,14 @@
       </c>
       <c r="G95" s="74" t="inlineStr">
         <is>
-          <t>Deck ones are shown face down</t>
+          <t>Arms an icon in the HUD tracking the pending draws</t>
         </is>
       </c>
       <c r="H95" s="71" t="n"/>
       <c r="I95" s="71" t="n"/>
       <c r="J95" s="71" t="n"/>
     </row>
-    <row r="96" ht="14" customHeight="1" s="85">
+    <row r="96" ht="28" customHeight="1" s="85">
       <c r="A96" s="21" t="n"/>
       <c r="B96" s="22" t="inlineStr">
         <is>
@@ -4763,28 +4760,24 @@
       </c>
       <c r="C96" s="49" t="inlineStr">
         <is>
-          <t>Fresh Ball</t>
+          <t>All Star Selection</t>
         </is>
       </c>
       <c r="D96" s="38" t="inlineStr">
         <is>
-          <t>Next player does not draw at the start of their possession</t>
+          <t>Draw 2 cards</t>
         </is>
       </c>
       <c r="E96" s="7" t="n"/>
       <c r="F96" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G96" s="74" t="inlineStr">
-        <is>
-          <t>This is a bad thing in the NBA</t>
-        </is>
-      </c>
+      <c r="G96" s="74" t="n"/>
       <c r="H96" s="71" t="n"/>
       <c r="I96" s="71" t="n"/>
       <c r="J96" s="71" t="n"/>
     </row>
-    <row r="97" ht="14" customHeight="1" s="85">
+    <row r="97" ht="42" customHeight="1" s="85">
       <c r="A97" s="21" t="n"/>
       <c r="B97" s="22" t="inlineStr">
         <is>
@@ -4793,12 +4786,12 @@
       </c>
       <c r="C97" s="49" t="inlineStr">
         <is>
-          <t>Trade Deadline</t>
+          <t>Hit the Bike</t>
         </is>
       </c>
       <c r="D97" s="38" t="inlineStr">
         <is>
-          <t>Declare Left or Right: every player passes their hand that way. The ball goes with it</t>
+          <t>Discard all Injuries. Draw 1 card. Give possession to another player</t>
         </is>
       </c>
       <c r="E97" s="7" t="n"/>
@@ -4807,14 +4800,14 @@
       </c>
       <c r="G97" s="74" t="inlineStr">
         <is>
-          <t>The hex travels in the declared direction too</t>
+          <t>This is not a pass</t>
         </is>
       </c>
       <c r="H97" s="71" t="n"/>
       <c r="I97" s="71" t="n"/>
       <c r="J97" s="71" t="n"/>
     </row>
-    <row r="98" ht="14" customHeight="1" s="85">
+    <row r="98" ht="28" customHeight="1" s="85">
       <c r="A98" s="21" t="n"/>
       <c r="B98" s="22" t="inlineStr">
         <is>
@@ -4823,12 +4816,12 @@
       </c>
       <c r="C98" s="49" t="inlineStr">
         <is>
-          <t>Floor Cleanup</t>
+          <t>Ice Wrap</t>
         </is>
       </c>
       <c r="D98" s="38" t="inlineStr">
         <is>
-          <t>All players shuffle their hands into the deck and draw the same number of cards</t>
+          <t>Draw 1 card. Discard all Injuries. If none, draw 1 additional card</t>
         </is>
       </c>
       <c r="E98" s="7" t="n"/>
@@ -4840,7 +4833,7 @@
       <c r="I98" s="71" t="n"/>
       <c r="J98" s="71" t="n"/>
     </row>
-    <row r="99" ht="14" customHeight="1" s="85">
+    <row r="99" ht="42" customHeight="1" s="85">
       <c r="A99" s="21" t="n"/>
       <c r="B99" s="22" t="inlineStr">
         <is>
@@ -4849,19 +4842,23 @@
       </c>
       <c r="C99" s="49" t="inlineStr">
         <is>
-          <t>Official Timeout</t>
+          <t>Wet Spot</t>
         </is>
       </c>
       <c r="D99" s="38" t="inlineStr">
         <is>
-          <t>At least 1 referee must be armed: discard all Injuries on all players and clear all referees. If none, all players draw 1 card</t>
+          <t>All Injuries in the discards and deck are displayed. Take one</t>
         </is>
       </c>
       <c r="E99" s="7" t="n"/>
       <c r="F99" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G99" s="74" t="n"/>
+      <c r="G99" s="74" t="inlineStr">
+        <is>
+          <t>Deck ones are shown face down</t>
+        </is>
+      </c>
       <c r="H99" s="71" t="n"/>
       <c r="I99" s="71" t="n"/>
       <c r="J99" s="71" t="n"/>
@@ -4875,19 +4872,23 @@
       </c>
       <c r="C100" s="49" t="inlineStr">
         <is>
-          <t>Team Doctor</t>
+          <t>Fresh Ball</t>
         </is>
       </c>
       <c r="D100" s="38" t="inlineStr">
         <is>
-          <t>Discard 1 Injury from a player of choice. Draw 2 cards if not choosing yourself</t>
+          <t>Next player does not draw at the start of their possession</t>
         </is>
       </c>
       <c r="E100" s="7" t="n"/>
       <c r="F100" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G100" s="74" t="n"/>
+      <c r="G100" s="74" t="inlineStr">
+        <is>
+          <t>This is a bad thing in the NBA</t>
+        </is>
+      </c>
       <c r="H100" s="71" t="n"/>
       <c r="I100" s="71" t="n"/>
       <c r="J100" s="71" t="n"/>
@@ -4901,19 +4902,23 @@
       </c>
       <c r="C101" s="49" t="inlineStr">
         <is>
-          <t>Altercation</t>
+          <t>Trade Deadline</t>
         </is>
       </c>
       <c r="D101" s="38" t="inlineStr">
         <is>
-          <t>Select another player: you and that player each discard 1 card at random. Inbound the ball to a player other than that target</t>
+          <t>Declare Left or Right: every player passes their hand that way. The ball goes with it</t>
         </is>
       </c>
       <c r="E101" s="7" t="n"/>
       <c r="F101" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G101" s="74" t="n"/>
+      <c r="G101" s="74" t="inlineStr">
+        <is>
+          <t>The hex travels in the declared direction too</t>
+        </is>
+      </c>
       <c r="H101" s="71" t="n"/>
       <c r="I101" s="71" t="n"/>
       <c r="J101" s="71" t="n"/>
@@ -4927,12 +4932,12 @@
       </c>
       <c r="C102" s="49" t="inlineStr">
         <is>
-          <t>Huge Altercation</t>
+          <t>Floor Cleanup</t>
         </is>
       </c>
       <c r="D102" s="38" t="inlineStr">
         <is>
-          <t>All players discard their hands. If a ref is armed, all players receive 1 TOV. Inbound the ball</t>
+          <t>All players shuffle their hands into the deck and draw the same number of cards</t>
         </is>
       </c>
       <c r="E102" s="7" t="n"/>
@@ -4953,12 +4958,12 @@
       </c>
       <c r="C103" s="49" t="inlineStr">
         <is>
-          <t>Home Court Advantage</t>
+          <t>Official Timeout</t>
         </is>
       </c>
       <c r="D103" s="38" t="inlineStr">
         <is>
-          <t>SHOT + 25%</t>
+          <t>At least 1 referee must be armed: discard all Injuries on all players and clear all referees. If none, all players draw 1 card</t>
         </is>
       </c>
       <c r="E103" s="7" t="n"/>
@@ -4979,12 +4984,12 @@
       </c>
       <c r="C104" s="49" t="inlineStr">
         <is>
-          <t>Away Game</t>
+          <t>Team Doctor</t>
         </is>
       </c>
       <c r="D104" s="38" t="inlineStr">
         <is>
-          <t>SHOT - 10%</t>
+          <t>Discard 1 Injury from a player of choice. Draw 2 cards if not choosing yourself</t>
         </is>
       </c>
       <c r="E104" s="7" t="n"/>
@@ -4996,7 +5001,7 @@
       <c r="I104" s="71" t="n"/>
       <c r="J104" s="71" t="n"/>
     </row>
-    <row r="105" ht="28" customHeight="1" s="85">
+    <row r="105" ht="14" customHeight="1" s="85">
       <c r="A105" s="21" t="n"/>
       <c r="B105" s="22" t="inlineStr">
         <is>
@@ -5005,28 +5010,24 @@
       </c>
       <c r="C105" s="49" t="inlineStr">
         <is>
-          <t>Mic'd Up</t>
+          <t>Altercation</t>
         </is>
       </c>
       <c r="D105" s="38" t="inlineStr">
         <is>
-          <t>SHOT + 10% until passed or shot</t>
+          <t>Select another player: you and that player each discard 1 card at random. Inbound the ball to a player other than that target</t>
         </is>
       </c>
       <c r="E105" s="7" t="n"/>
       <c r="F105" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G105" s="74" t="inlineStr">
-        <is>
-          <t>The boost is the holder's alone and does not travel with a pass</t>
-        </is>
-      </c>
+      <c r="G105" s="74" t="n"/>
       <c r="H105" s="71" t="n"/>
       <c r="I105" s="71" t="n"/>
       <c r="J105" s="71" t="n"/>
     </row>
-    <row r="106" ht="28" customHeight="1" s="85">
+    <row r="106" ht="14" customHeight="1" s="85">
       <c r="A106" s="21" t="n"/>
       <c r="B106" s="22" t="inlineStr">
         <is>
@@ -5035,12 +5036,12 @@
       </c>
       <c r="C106" s="49" t="inlineStr">
         <is>
-          <t>In The Zone</t>
+          <t>Huge Altercation</t>
         </is>
       </c>
       <c r="D106" s="38" t="inlineStr">
         <is>
-          <t>Draw 1 card for each 10% SHOT the ball has, rounded down. Minimum 1</t>
+          <t>All players discard their hands. If a ref is armed, all players receive 1 TOV. Inbound the ball</t>
         </is>
       </c>
       <c r="E106" s="7" t="n"/>
@@ -5052,7 +5053,7 @@
       <c r="I106" s="71" t="n"/>
       <c r="J106" s="71" t="n"/>
     </row>
-    <row r="107" ht="28" customHeight="1" s="85">
+    <row r="107" ht="14" customHeight="1" s="85">
       <c r="A107" s="21" t="n"/>
       <c r="B107" s="22" t="inlineStr">
         <is>
@@ -5061,12 +5062,12 @@
       </c>
       <c r="C107" s="49" t="inlineStr">
         <is>
-          <t>Role Player</t>
+          <t>Home Court Advantage</t>
         </is>
       </c>
       <c r="D107" s="38" t="inlineStr">
         <is>
-          <t>All other players draw 1 card</t>
+          <t>SHOT + 25%</t>
         </is>
       </c>
       <c r="E107" s="7" t="n"/>
@@ -5078,154 +5079,174 @@
       <c r="I107" s="71" t="n"/>
       <c r="J107" s="71" t="n"/>
     </row>
-    <row r="108" ht="28" customHeight="1" s="85">
-      <c r="A108" s="27" t="n"/>
-      <c r="B108" s="28" t="inlineStr">
+    <row r="108" ht="14" customHeight="1" s="85">
+      <c r="A108" s="21" t="n"/>
+      <c r="B108" s="22" t="inlineStr">
         <is>
           <t>Retired Game Break</t>
         </is>
       </c>
-      <c r="C108" s="62" t="inlineStr">
+      <c r="C108" s="49" t="inlineStr">
+        <is>
+          <t>Away Game</t>
+        </is>
+      </c>
+      <c r="D108" s="38" t="inlineStr">
+        <is>
+          <t>SHOT - 10%</t>
+        </is>
+      </c>
+      <c r="E108" s="7" t="n"/>
+      <c r="F108" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G108" s="74" t="n"/>
+      <c r="H108" s="71" t="n"/>
+      <c r="I108" s="71" t="n"/>
+      <c r="J108" s="71" t="n"/>
+    </row>
+    <row r="109" ht="28" customHeight="1" s="85">
+      <c r="A109" s="21" t="n"/>
+      <c r="B109" s="22" t="inlineStr">
+        <is>
+          <t>Retired Game Break</t>
+        </is>
+      </c>
+      <c r="C109" s="49" t="inlineStr">
+        <is>
+          <t>Mic'd Up</t>
+        </is>
+      </c>
+      <c r="D109" s="38" t="inlineStr">
+        <is>
+          <t>SHOT + 10% until passed or shot</t>
+        </is>
+      </c>
+      <c r="E109" s="7" t="n"/>
+      <c r="F109" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G109" s="74" t="inlineStr">
+        <is>
+          <t>The boost is the holder's alone and does not travel with a pass</t>
+        </is>
+      </c>
+      <c r="H109" s="71" t="n"/>
+      <c r="I109" s="71" t="n"/>
+      <c r="J109" s="71" t="n"/>
+    </row>
+    <row r="110" ht="28" customHeight="1" s="85">
+      <c r="A110" s="21" t="n"/>
+      <c r="B110" s="22" t="inlineStr">
+        <is>
+          <t>Retired Game Break</t>
+        </is>
+      </c>
+      <c r="C110" s="49" t="inlineStr">
+        <is>
+          <t>In The Zone</t>
+        </is>
+      </c>
+      <c r="D110" s="38" t="inlineStr">
+        <is>
+          <t>Draw 1 card for each 10% SHOT the ball has, rounded down. Minimum 1</t>
+        </is>
+      </c>
+      <c r="E110" s="7" t="n"/>
+      <c r="F110" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G110" s="74" t="n"/>
+      <c r="H110" s="71" t="n"/>
+      <c r="I110" s="71" t="n"/>
+      <c r="J110" s="71" t="n"/>
+    </row>
+    <row r="111" ht="28" customHeight="1" s="85">
+      <c r="A111" s="21" t="n"/>
+      <c r="B111" s="22" t="inlineStr">
+        <is>
+          <t>Retired Game Break</t>
+        </is>
+      </c>
+      <c r="C111" s="49" t="inlineStr">
+        <is>
+          <t>Role Player</t>
+        </is>
+      </c>
+      <c r="D111" s="38" t="inlineStr">
+        <is>
+          <t>All other players draw 1 card</t>
+        </is>
+      </c>
+      <c r="E111" s="7" t="n"/>
+      <c r="F111" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G111" s="74" t="n"/>
+      <c r="H111" s="71" t="n"/>
+      <c r="I111" s="71" t="n"/>
+      <c r="J111" s="71" t="n"/>
+    </row>
+    <row r="112" ht="28" customHeight="1" s="85">
+      <c r="A112" s="27" t="n"/>
+      <c r="B112" s="28" t="inlineStr">
+        <is>
+          <t>Retired Game Break</t>
+        </is>
+      </c>
+      <c r="C112" s="62" t="inlineStr">
         <is>
           <t>Back-and-Forth Game</t>
         </is>
       </c>
-      <c r="D108" s="63" t="inlineStr">
+      <c r="D112" s="63" t="inlineStr">
         <is>
           <t>Discard the next 3 Game Breaks. Whoever draws one draws again</t>
         </is>
       </c>
-      <c r="E108" s="58" t="n"/>
-      <c r="F108" s="59" t="n">
+      <c r="E112" s="58" t="n"/>
+      <c r="F112" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="G108" s="79" t="n"/>
-      <c r="H108" s="76" t="n"/>
-      <c r="I108" s="76" t="n"/>
-      <c r="J108" s="76" t="n"/>
-    </row>
-    <row r="109" ht="42" customHeight="1" s="85">
-      <c r="A109" s="27" t="n"/>
-      <c r="B109" s="28" t="inlineStr">
-        <is>
-          <t>Retired Game Break</t>
-        </is>
-      </c>
-      <c r="C109" s="62" t="inlineStr">
-        <is>
-          <t>Off the Backboard</t>
-        </is>
-      </c>
-      <c r="D109" s="63" t="inlineStr">
-        <is>
-          <t>Your next missed shot rebounds itself</t>
-        </is>
-      </c>
-      <c r="E109" s="58" t="n"/>
-      <c r="F109" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="G109" s="79" t="n"/>
-      <c r="H109" s="76" t="n"/>
-      <c r="I109" s="76" t="n"/>
-      <c r="J109" s="76" t="n"/>
-    </row>
-    <row r="110" ht="56" customHeight="1" s="85">
-      <c r="A110" s="52" t="inlineStr">
-        <is>
-          <t>Injury</t>
-        </is>
-      </c>
-      <c r="B110" s="53">
-        <f>COUNTIF($B$111:$B$143,"Injury")</f>
-        <v/>
-      </c>
-      <c r="C110" s="54" t="n"/>
-      <c r="D110" s="54" t="n"/>
-      <c r="E110" s="54" t="n"/>
-      <c r="F110" s="55" t="n"/>
-      <c r="G110" s="66" t="n"/>
-      <c r="H110" s="67" t="n"/>
-      <c r="I110" s="67" t="n"/>
-      <c r="J110" s="67" t="n"/>
-    </row>
-    <row r="111" ht="57" customHeight="1" s="85">
-      <c r="A111" s="27" t="n"/>
-      <c r="B111" s="28" t="inlineStr">
-        <is>
-          <t>Injury</t>
-        </is>
-      </c>
-      <c r="C111" s="56" t="inlineStr">
-        <is>
-          <t>Bone Bruise</t>
-        </is>
-      </c>
-      <c r="D111" s="63" t="inlineStr">
-        <is>
-          <t>Discard 1 card at the start of each turn after drawing (your choice)</t>
-        </is>
-      </c>
-      <c r="E111" s="58" t="n"/>
-      <c r="F111" s="59" t="n">
-        <v>5</v>
-      </c>
-      <c r="G111" s="75" t="n"/>
-      <c r="H111" s="76" t="n"/>
-      <c r="I111" s="76" t="n"/>
-      <c r="J111" s="76" t="n"/>
-    </row>
-    <row r="112" ht="20" customHeight="1" s="85">
-      <c r="A112" s="52" t="inlineStr">
-        <is>
-          <t>Devastating Injury</t>
-        </is>
-      </c>
-      <c r="B112" s="53">
-        <f>COUNTIF($B$113:$B$143,"Devastating Injury")</f>
-        <v/>
-      </c>
-      <c r="C112" s="54" t="n"/>
-      <c r="D112" s="54" t="n"/>
-      <c r="E112" s="54" t="n"/>
-      <c r="F112" s="55" t="n"/>
-      <c r="G112" s="66" t="n"/>
-      <c r="H112" s="67" t="n"/>
-      <c r="I112" s="67" t="n"/>
-      <c r="J112" s="67" t="n"/>
-    </row>
-    <row r="113" ht="28" customHeight="1" s="85">
+      <c r="G112" s="79" t="n"/>
+      <c r="H112" s="76" t="n"/>
+      <c r="I112" s="76" t="n"/>
+      <c r="J112" s="76" t="n"/>
+    </row>
+    <row r="113" ht="42" customHeight="1" s="85">
       <c r="A113" s="27" t="n"/>
       <c r="B113" s="28" t="inlineStr">
         <is>
-          <t>Devastating Injury</t>
-        </is>
-      </c>
-      <c r="C113" s="64" t="inlineStr">
-        <is>
-          <t>Torn Achilles</t>
-        </is>
-      </c>
-      <c r="D113" s="65" t="inlineStr">
-        <is>
-          <t>Hand is locked every turn except 1 card (randomly)</t>
+          <t>Retired Game Break</t>
+        </is>
+      </c>
+      <c r="C113" s="62" t="inlineStr">
+        <is>
+          <t>Off the Backboard</t>
+        </is>
+      </c>
+      <c r="D113" s="63" t="inlineStr">
+        <is>
+          <t>Your next missed shot rebounds itself</t>
         </is>
       </c>
       <c r="E113" s="58" t="n"/>
-      <c r="F113" s="61" t="n"/>
-      <c r="G113" s="75" t="n"/>
+      <c r="F113" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="G113" s="79" t="n"/>
       <c r="H113" s="76" t="n"/>
       <c r="I113" s="76" t="n"/>
       <c r="J113" s="76" t="n"/>
     </row>
-    <row r="114" ht="42" customHeight="1" s="85">
+    <row r="114" ht="56" customHeight="1" s="85">
       <c r="A114" s="52" t="inlineStr">
         <is>
-          <t>Intangible</t>
+          <t>Injury</t>
         </is>
       </c>
       <c r="B114" s="53">
-        <f>COUNTIF($B$115:$B$143,"Intangible")</f>
+        <f>COUNTIF($B$115:$B$147,"Injury")</f>
         <v/>
       </c>
       <c r="C114" s="54" t="n"/>
@@ -5237,119 +5258,118 @@
       <c r="I114" s="67" t="n"/>
       <c r="J114" s="67" t="n"/>
     </row>
-    <row r="115" ht="28" customHeight="1" s="85">
-      <c r="A115" s="42" t="inlineStr">
+    <row r="115" ht="57" customHeight="1" s="85">
+      <c r="A115" s="27" t="n"/>
+      <c r="B115" s="28" t="inlineStr">
+        <is>
+          <t>Injury</t>
+        </is>
+      </c>
+      <c r="C115" s="56" t="inlineStr">
+        <is>
+          <t>Bone Bruise</t>
+        </is>
+      </c>
+      <c r="D115" s="63" t="inlineStr">
+        <is>
+          <t>Discard 1 card at the start of each turn after drawing (your choice)</t>
+        </is>
+      </c>
+      <c r="E115" s="58" t="n"/>
+      <c r="F115" s="59" t="n">
+        <v>5</v>
+      </c>
+      <c r="G115" s="75" t="n"/>
+      <c r="H115" s="76" t="n"/>
+      <c r="I115" s="76" t="n"/>
+      <c r="J115" s="76" t="n"/>
+    </row>
+    <row r="116" ht="20" customHeight="1" s="85">
+      <c r="A116" s="52" t="inlineStr">
+        <is>
+          <t>Devastating Injury</t>
+        </is>
+      </c>
+      <c r="B116" s="53">
+        <f>COUNTIF($B$117:$B$147,"Devastating Injury")</f>
+        <v/>
+      </c>
+      <c r="C116" s="54" t="n"/>
+      <c r="D116" s="54" t="n"/>
+      <c r="E116" s="54" t="n"/>
+      <c r="F116" s="55" t="n"/>
+      <c r="G116" s="66" t="n"/>
+      <c r="H116" s="67" t="n"/>
+      <c r="I116" s="67" t="n"/>
+      <c r="J116" s="67" t="n"/>
+    </row>
+    <row r="117" ht="28" customHeight="1" s="85">
+      <c r="A117" s="27" t="n"/>
+      <c r="B117" s="28" t="inlineStr">
+        <is>
+          <t>Devastating Injury</t>
+        </is>
+      </c>
+      <c r="C117" s="64" t="inlineStr">
+        <is>
+          <t>Torn Achilles</t>
+        </is>
+      </c>
+      <c r="D117" s="65" t="inlineStr">
+        <is>
+          <t>Hand is locked every turn except 1 card (randomly)</t>
+        </is>
+      </c>
+      <c r="E117" s="58" t="n"/>
+      <c r="F117" s="61" t="n"/>
+      <c r="G117" s="75" t="n"/>
+      <c r="H117" s="76" t="n"/>
+      <c r="I117" s="76" t="n"/>
+      <c r="J117" s="76" t="n"/>
+    </row>
+    <row r="118" ht="42" customHeight="1" s="85">
+      <c r="A118" s="52" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="B118" s="53">
+        <f>COUNTIF($B$119:$B$147,"Intangible")</f>
+        <v/>
+      </c>
+      <c r="C118" s="54" t="n"/>
+      <c r="D118" s="54" t="n"/>
+      <c r="E118" s="54" t="n"/>
+      <c r="F118" s="55" t="n"/>
+      <c r="G118" s="66" t="n"/>
+      <c r="H118" s="67" t="n"/>
+      <c r="I118" s="67" t="n"/>
+      <c r="J118" s="67" t="n"/>
+    </row>
+    <row r="119" ht="28" customHeight="1" s="85">
+      <c r="A119" s="42" t="inlineStr">
         <is>
           <t>All intangibles are limited to 1</t>
         </is>
       </c>
-      <c r="B115" s="22" t="inlineStr">
+      <c r="B119" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C115" s="23" t="inlineStr">
+      <c r="C119" s="23" t="inlineStr">
         <is>
           <t>Board-Crasher</t>
         </is>
       </c>
-      <c r="D115" s="6" t="inlineStr">
+      <c r="D119" s="6" t="inlineStr">
         <is>
           <t>SHOT +10% upon Rebounding your own missed shot</t>
         </is>
       </c>
-      <c r="E115" s="7" t="n"/>
-      <c r="F115" s="50" t="n"/>
-      <c r="G115" s="70" t="n"/>
-      <c r="H115" s="71" t="n"/>
-      <c r="I115" s="71" t="n"/>
-      <c r="J115" s="71" t="n"/>
-    </row>
-    <row r="116" ht="28" customHeight="1" s="85">
-      <c r="A116" s="21" t="n"/>
-      <c r="B116" s="22" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C116" s="24" t="inlineStr">
-        <is>
-          <t>Catch &amp; Shoot Specialist</t>
-        </is>
-      </c>
-      <c r="D116" s="25" t="inlineStr">
-        <is>
-          <t>Additional SHOT +10% on all received passes</t>
-        </is>
-      </c>
-      <c r="E116" s="26" t="n"/>
-      <c r="F116" s="50" t="n"/>
-      <c r="G116" s="72" t="n"/>
-      <c r="H116" s="71" t="n"/>
-      <c r="I116" s="71" t="n"/>
-      <c r="J116" s="71" t="n"/>
-    </row>
-    <row r="117" ht="56" customHeight="1" s="85">
-      <c r="A117" s="21" t="n"/>
-      <c r="B117" s="22" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C117" s="23" t="inlineStr">
-        <is>
-          <t>Clutch Gene</t>
-        </is>
-      </c>
-      <c r="D117" s="6" t="inlineStr">
-        <is>
-          <t>SHOT x2 if attempting a shot with 1 or fewer cards in hand or Shot Clock 3 or less</t>
-        </is>
-      </c>
-      <c r="E117" s="7" t="n"/>
-      <c r="F117" s="50" t="n"/>
-      <c r="G117" s="70" t="n"/>
-      <c r="H117" s="71" t="n"/>
-      <c r="I117" s="71" t="n"/>
-      <c r="J117" s="71" t="n"/>
-    </row>
-    <row r="118" ht="56" customHeight="1" s="85">
-      <c r="B118" s="0" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C118" s="0" t="inlineStr">
-        <is>
-          <t>Roswell Reach</t>
-        </is>
-      </c>
-      <c r="D118" s="0" t="inlineStr">
-        <is>
-          <t>All your Rebound bids of 1 or more count as 1 higher</t>
-        </is>
-      </c>
-    </row>
-    <row r="119" ht="28" customHeight="1" s="85">
-      <c r="A119" s="21" t="n"/>
-      <c r="B119" s="22" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C119" s="24" t="inlineStr">
-        <is>
-          <t>Floor General</t>
-        </is>
-      </c>
-      <c r="D119" s="25" t="inlineStr">
-        <is>
-          <t>You choose all targets of all kinds — card declarations, non auto-pass targets, and the rest. Not choices about a player's own card: which effect of a multi-effect card, or whether to feed a shot an extra discard</t>
-        </is>
-      </c>
-      <c r="E119" s="26" t="n"/>
+      <c r="E119" s="7" t="n"/>
       <c r="F119" s="50" t="n"/>
-      <c r="G119" s="72" t="n"/>
+      <c r="G119" s="70" t="n"/>
       <c r="H119" s="71" t="n"/>
       <c r="I119" s="71" t="n"/>
       <c r="J119" s="71" t="n"/>
@@ -5361,76 +5381,65 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C120" s="23" t="inlineStr">
-        <is>
-          <t>Fox-Like First Step</t>
-        </is>
-      </c>
-      <c r="D120" s="6" t="inlineStr">
-        <is>
-          <t>All Move cards that reduce SHOT increase it by that amount instead.</t>
-        </is>
-      </c>
-      <c r="E120" s="6" t="inlineStr">
-        <is>
-          <t>Your Move cards are unaffected by opponents</t>
-        </is>
-      </c>
-      <c r="F120" s="51" t="n"/>
-      <c r="G120" s="70" t="n"/>
+      <c r="C120" s="24" t="inlineStr">
+        <is>
+          <t>Catch &amp; Shoot Specialist</t>
+        </is>
+      </c>
+      <c r="D120" s="25" t="inlineStr">
+        <is>
+          <t>Additional SHOT +10% on all received passes</t>
+        </is>
+      </c>
+      <c r="E120" s="26" t="n"/>
+      <c r="F120" s="50" t="n"/>
+      <c r="G120" s="72" t="n"/>
       <c r="H120" s="71" t="n"/>
       <c r="I120" s="71" t="n"/>
       <c r="J120" s="71" t="n"/>
     </row>
-    <row r="121" ht="28" customHeight="1" s="85">
+    <row r="121" ht="56" customHeight="1" s="85">
       <c r="A121" s="21" t="n"/>
       <c r="B121" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C121" s="37" t="inlineStr">
-        <is>
-          <t>Freethrow Merchant</t>
-        </is>
-      </c>
-      <c r="D121" s="41" t="inlineStr">
-        <is>
-          <t>All Clamps on you grant 1 FT instead</t>
-        </is>
-      </c>
-      <c r="E121" s="26" t="n"/>
+      <c r="C121" s="23" t="inlineStr">
+        <is>
+          <t>Clutch Gene</t>
+        </is>
+      </c>
+      <c r="D121" s="6" t="inlineStr">
+        <is>
+          <t>SHOT x2 if attempting a shot with 1 or fewer cards in hand or Shot Clock 3 or less</t>
+        </is>
+      </c>
+      <c r="E121" s="7" t="n"/>
       <c r="F121" s="50" t="n"/>
-      <c r="G121" s="77" t="n"/>
+      <c r="G121" s="70" t="n"/>
       <c r="H121" s="71" t="n"/>
       <c r="I121" s="71" t="n"/>
       <c r="J121" s="71" t="n"/>
     </row>
-    <row r="122" ht="28" customHeight="1" s="85">
-      <c r="A122" s="21" t="n"/>
-      <c r="B122" s="22" t="inlineStr">
+    <row r="122" ht="56" customHeight="1" s="85">
+      <c r="B122" s="0" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C122" s="37" t="inlineStr">
-        <is>
-          <t>Generational Whistle</t>
-        </is>
-      </c>
-      <c r="D122" s="38" t="inlineStr">
-        <is>
-          <t>Take 1 additional FT</t>
-        </is>
-      </c>
-      <c r="E122" s="7" t="n"/>
-      <c r="F122" s="50" t="n"/>
-      <c r="G122" s="70" t="n"/>
-      <c r="H122" s="71" t="n"/>
-      <c r="I122" s="71" t="n"/>
-      <c r="J122" s="71" t="n"/>
-    </row>
-    <row r="123" ht="14" customHeight="1" s="85">
+      <c r="C122" s="0" t="inlineStr">
+        <is>
+          <t>Roswell Reach</t>
+        </is>
+      </c>
+      <c r="D122" s="0" t="inlineStr">
+        <is>
+          <t>All your Rebound bids of 1 or more count as 1 higher</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="28" customHeight="1" s="85">
       <c r="A123" s="21" t="n"/>
       <c r="B123" s="22" t="inlineStr">
         <is>
@@ -5439,12 +5448,12 @@
       </c>
       <c r="C123" s="24" t="inlineStr">
         <is>
-          <t>Gravity</t>
+          <t>Floor General</t>
         </is>
       </c>
       <c r="D123" s="25" t="inlineStr">
         <is>
-          <t>All Clamps automatically apply to you. +1 AST whenever another player attempts a shot</t>
+          <t>You choose all targets of all kinds — card declarations, non auto-pass targets, and the rest. Not choices about a player's own card: which effect of a multi-effect card, or whether to feed a shot an extra discard</t>
         </is>
       </c>
       <c r="E123" s="26" t="n"/>
@@ -5463,16 +5472,20 @@
       </c>
       <c r="C124" s="23" t="inlineStr">
         <is>
-          <t>Great Conditioning</t>
+          <t>Fox-Like First Step</t>
         </is>
       </c>
       <c r="D124" s="6" t="inlineStr">
         <is>
-          <t>Immediately discard all Injury Game Breaks you draw and draw a new card for each</t>
-        </is>
-      </c>
-      <c r="E124" s="7" t="n"/>
-      <c r="F124" s="50" t="n"/>
+          <t>All Move cards that reduce SHOT increase it by that amount instead.</t>
+        </is>
+      </c>
+      <c r="E124" s="6" t="inlineStr">
+        <is>
+          <t>Your Move cards are unaffected by opponents</t>
+        </is>
+      </c>
+      <c r="F124" s="51" t="n"/>
       <c r="G124" s="70" t="n"/>
       <c r="H124" s="71" t="n"/>
       <c r="I124" s="71" t="n"/>
@@ -5485,19 +5498,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C125" s="24" t="inlineStr">
-        <is>
-          <t>Hot Hand</t>
-        </is>
-      </c>
-      <c r="D125" s="25" t="inlineStr">
-        <is>
-          <t>SHOT +25% if you scored last round.</t>
+      <c r="C125" s="37" t="inlineStr">
+        <is>
+          <t>Freethrow Merchant</t>
+        </is>
+      </c>
+      <c r="D125" s="41" t="inlineStr">
+        <is>
+          <t>All Clamps on you grant 1 FT instead</t>
         </is>
       </c>
       <c r="E125" s="26" t="n"/>
       <c r="F125" s="50" t="n"/>
-      <c r="G125" s="72" t="n"/>
+      <c r="G125" s="77" t="n"/>
       <c r="H125" s="71" t="n"/>
       <c r="I125" s="71" t="n"/>
       <c r="J125" s="71" t="n"/>
@@ -5509,14 +5522,14 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C126" s="23" t="inlineStr">
-        <is>
-          <t>Like That</t>
+      <c r="C126" s="37" t="inlineStr">
+        <is>
+          <t>Generational Whistle</t>
         </is>
       </c>
       <c r="D126" s="38" t="inlineStr">
         <is>
-          <t>Your SHOT % cannot be reduced</t>
+          <t>Take 1 additional FT</t>
         </is>
       </c>
       <c r="E126" s="7" t="n"/>
@@ -5526,7 +5539,7 @@
       <c r="I126" s="71" t="n"/>
       <c r="J126" s="71" t="n"/>
     </row>
-    <row r="127" ht="28" customHeight="1" s="85">
+    <row r="127" ht="14" customHeight="1" s="85">
       <c r="A127" s="21" t="n"/>
       <c r="B127" s="22" t="inlineStr">
         <is>
@@ -5535,21 +5548,17 @@
       </c>
       <c r="C127" s="24" t="inlineStr">
         <is>
-          <t>No Bag</t>
+          <t>Gravity</t>
         </is>
       </c>
       <c r="D127" s="25" t="inlineStr">
         <is>
-          <t>Cannot activate Move cards this round</t>
+          <t>All Clamps automatically apply to you. +1 AST whenever another player attempts a shot</t>
         </is>
       </c>
       <c r="E127" s="26" t="n"/>
       <c r="F127" s="50" t="n"/>
-      <c r="G127" s="73" t="inlineStr">
-        <is>
-          <t>Bad card to draw</t>
-        </is>
-      </c>
+      <c r="G127" s="72" t="n"/>
       <c r="H127" s="71" t="n"/>
       <c r="I127" s="71" t="n"/>
       <c r="J127" s="71" t="n"/>
@@ -5563,12 +5572,12 @@
       </c>
       <c r="C128" s="23" t="inlineStr">
         <is>
-          <t>Point God</t>
+          <t>Great Conditioning</t>
         </is>
       </c>
       <c r="D128" s="6" t="inlineStr">
         <is>
-          <t>Draw 1 card following each of your passes</t>
+          <t>Immediately discard all Injury Game Breaks you draw and draw a new card for each</t>
         </is>
       </c>
       <c r="E128" s="7" t="n"/>
@@ -5578,7 +5587,7 @@
       <c r="I128" s="71" t="n"/>
       <c r="J128" s="71" t="n"/>
     </row>
-    <row r="129" ht="56" customHeight="1" s="85">
+    <row r="129" ht="28" customHeight="1" s="85">
       <c r="A129" s="21" t="n"/>
       <c r="B129" s="22" t="inlineStr">
         <is>
@@ -5587,26 +5596,22 @@
       </c>
       <c r="C129" s="24" t="inlineStr">
         <is>
-          <t>Shooting Slump</t>
+          <t>Hot Hand</t>
         </is>
       </c>
       <c r="D129" s="25" t="inlineStr">
         <is>
-          <t>SHOT -20% this round</t>
+          <t>SHOT +25% if you scored last round.</t>
         </is>
       </c>
       <c r="E129" s="26" t="n"/>
       <c r="F129" s="50" t="n"/>
-      <c r="G129" s="73" t="inlineStr">
-        <is>
-          <t>Bad card to draw</t>
-        </is>
-      </c>
+      <c r="G129" s="72" t="n"/>
       <c r="H129" s="71" t="n"/>
       <c r="I129" s="71" t="n"/>
       <c r="J129" s="71" t="n"/>
     </row>
-    <row r="130" ht="56" customHeight="1" s="85">
+    <row r="130" ht="28" customHeight="1" s="85">
       <c r="A130" s="21" t="n"/>
       <c r="B130" s="22" t="inlineStr">
         <is>
@@ -5615,12 +5620,12 @@
       </c>
       <c r="C130" s="23" t="inlineStr">
         <is>
-          <t>Shot Creator</t>
-        </is>
-      </c>
-      <c r="D130" s="6" t="inlineStr">
-        <is>
-          <t>Draw 1 additional card after every draw effect</t>
+          <t>Like That</t>
+        </is>
+      </c>
+      <c r="D130" s="38" t="inlineStr">
+        <is>
+          <t>Your SHOT % cannot be reduced</t>
         </is>
       </c>
       <c r="E130" s="7" t="n"/>
@@ -5630,7 +5635,7 @@
       <c r="I130" s="71" t="n"/>
       <c r="J130" s="71" t="n"/>
     </row>
-    <row r="131" ht="56" customHeight="1" s="85">
+    <row r="131" ht="28" customHeight="1" s="85">
       <c r="A131" s="21" t="n"/>
       <c r="B131" s="22" t="inlineStr">
         <is>
@@ -5639,22 +5644,26 @@
       </c>
       <c r="C131" s="24" t="inlineStr">
         <is>
-          <t>Sixth Man</t>
+          <t>No Bag</t>
         </is>
       </c>
       <c r="D131" s="25" t="inlineStr">
         <is>
-          <t>SHOT +60% on any six: cards in hand, Shot Clock, shot of the round, or score</t>
+          <t>Cannot activate Move cards this round</t>
         </is>
       </c>
       <c r="E131" s="26" t="n"/>
       <c r="F131" s="50" t="n"/>
-      <c r="G131" s="72" t="n"/>
+      <c r="G131" s="73" t="inlineStr">
+        <is>
+          <t>Bad card to draw</t>
+        </is>
+      </c>
       <c r="H131" s="71" t="n"/>
       <c r="I131" s="71" t="n"/>
       <c r="J131" s="71" t="n"/>
     </row>
-    <row r="132" ht="56" customHeight="1" s="85">
+    <row r="132" ht="28" customHeight="1" s="85">
       <c r="A132" s="21" t="n"/>
       <c r="B132" s="22" t="inlineStr">
         <is>
@@ -5663,12 +5672,12 @@
       </c>
       <c r="C132" s="23" t="inlineStr">
         <is>
-          <t>Sniper</t>
+          <t>Point God</t>
         </is>
       </c>
       <c r="D132" s="6" t="inlineStr">
         <is>
-          <t>SHOT +25% on all Three-Point Line Shots</t>
+          <t>Draw 1 card following each of your passes</t>
         </is>
       </c>
       <c r="E132" s="7" t="n"/>
@@ -5687,22 +5696,26 @@
       </c>
       <c r="C133" s="24" t="inlineStr">
         <is>
-          <t>Splash Cousin</t>
+          <t>Shooting Slump</t>
         </is>
       </c>
       <c r="D133" s="25" t="inlineStr">
         <is>
-          <t>All Three-Point Line Shots: SHOT = 100%</t>
+          <t>SHOT -20% this round</t>
         </is>
       </c>
       <c r="E133" s="26" t="n"/>
       <c r="F133" s="50" t="n"/>
-      <c r="G133" s="72" t="n"/>
+      <c r="G133" s="73" t="inlineStr">
+        <is>
+          <t>Bad card to draw</t>
+        </is>
+      </c>
       <c r="H133" s="71" t="n"/>
       <c r="I133" s="71" t="n"/>
       <c r="J133" s="71" t="n"/>
     </row>
-    <row r="134" ht="126" customHeight="1" s="85">
+    <row r="134" ht="56" customHeight="1" s="85">
       <c r="A134" s="21" t="n"/>
       <c r="B134" s="22" t="inlineStr">
         <is>
@@ -5711,12 +5724,12 @@
       </c>
       <c r="C134" s="23" t="inlineStr">
         <is>
-          <t>Competitive</t>
-        </is>
-      </c>
-      <c r="D134" s="38" t="inlineStr">
-        <is>
-          <t>All Clamps on you have no effect on SHOT %</t>
+          <t>Shot Creator</t>
+        </is>
+      </c>
+      <c r="D134" s="6" t="inlineStr">
+        <is>
+          <t>Draw 1 additional card after every draw effect</t>
         </is>
       </c>
       <c r="E134" s="7" t="n"/>
@@ -5726,7 +5739,7 @@
       <c r="I134" s="71" t="n"/>
       <c r="J134" s="71" t="n"/>
     </row>
-    <row r="135" ht="70" customHeight="1" s="85">
+    <row r="135" ht="56" customHeight="1" s="85">
       <c r="A135" s="21" t="n"/>
       <c r="B135" s="22" t="inlineStr">
         <is>
@@ -5735,21 +5748,17 @@
       </c>
       <c r="C135" s="24" t="inlineStr">
         <is>
-          <t>Lethal Shooter</t>
+          <t>Sixth Man</t>
         </is>
       </c>
       <c r="D135" s="25" t="inlineStr">
         <is>
-          <t>SHOT = 100% on next shot attempt after rebounding your own miss.</t>
+          <t>SHOT +60% on any six: cards in hand, Shot Clock, shot of the round, or score</t>
         </is>
       </c>
       <c r="E135" s="26" t="n"/>
       <c r="F135" s="50" t="n"/>
-      <c r="G135" s="73" t="inlineStr">
-        <is>
-          <t>Special text: “I understand it now”</t>
-        </is>
-      </c>
+      <c r="G135" s="72" t="n"/>
       <c r="H135" s="71" t="n"/>
       <c r="I135" s="71" t="n"/>
       <c r="J135" s="71" t="n"/>
@@ -5763,12 +5772,12 @@
       </c>
       <c r="C136" s="23" t="inlineStr">
         <is>
-          <t>Ball Pounder</t>
-        </is>
-      </c>
-      <c r="D136" s="38" t="inlineStr">
-        <is>
-          <t>All Dribble cards you play draw an additional card but lower SHOT by an additional 10%</t>
+          <t>Sniper</t>
+        </is>
+      </c>
+      <c r="D136" s="6" t="inlineStr">
+        <is>
+          <t>SHOT +25% on all Three-Point Line Shots</t>
         </is>
       </c>
       <c r="E136" s="7" t="n"/>
@@ -5778,31 +5787,31 @@
       <c r="I136" s="71" t="n"/>
       <c r="J136" s="71" t="n"/>
     </row>
-    <row r="137">
+    <row r="137" ht="56" customHeight="1" s="85">
       <c r="A137" s="21" t="n"/>
       <c r="B137" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C137" s="23" t="inlineStr">
-        <is>
-          <t>Unselfish</t>
-        </is>
-      </c>
-      <c r="D137" s="38" t="inlineStr">
-        <is>
-          <t>Draw 1 card and increase next SHOT +5% whenever you positively affect another player</t>
-        </is>
-      </c>
-      <c r="E137" s="7" t="n"/>
+      <c r="C137" s="24" t="inlineStr">
+        <is>
+          <t>Splash Cousin</t>
+        </is>
+      </c>
+      <c r="D137" s="25" t="inlineStr">
+        <is>
+          <t>All Three-Point Line Shots: SHOT = 100%</t>
+        </is>
+      </c>
+      <c r="E137" s="26" t="n"/>
       <c r="F137" s="50" t="n"/>
-      <c r="G137" s="70" t="n"/>
+      <c r="G137" s="72" t="n"/>
       <c r="H137" s="71" t="n"/>
       <c r="I137" s="71" t="n"/>
       <c r="J137" s="71" t="n"/>
     </row>
-    <row r="138">
+    <row r="138" ht="126" customHeight="1" s="85">
       <c r="A138" s="21" t="n"/>
       <c r="B138" s="22" t="inlineStr">
         <is>
@@ -5811,12 +5820,12 @@
       </c>
       <c r="C138" s="23" t="inlineStr">
         <is>
-          <t>Dirty Player</t>
+          <t>Competitive</t>
         </is>
       </c>
       <c r="D138" s="38" t="inlineStr">
         <is>
-          <t>When sending Clamps, the clamped player discards 1 if they have any Injuries</t>
+          <t>All Clamps on you have no effect on SHOT %</t>
         </is>
       </c>
       <c r="E138" s="7" t="n"/>
@@ -5826,35 +5835,35 @@
       <c r="I138" s="71" t="n"/>
       <c r="J138" s="71" t="n"/>
     </row>
-    <row r="139">
+    <row r="139" ht="70" customHeight="1" s="85">
       <c r="A139" s="21" t="n"/>
       <c r="B139" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C139" s="23" t="inlineStr">
-        <is>
-          <t>Villainous Reputation</t>
-        </is>
-      </c>
-      <c r="D139" s="38" t="inlineStr">
-        <is>
-          <t>Discard 1 whenever any Whistle triggers</t>
-        </is>
-      </c>
-      <c r="E139" s="7" t="n"/>
+      <c r="C139" s="24" t="inlineStr">
+        <is>
+          <t>Lethal Shooter</t>
+        </is>
+      </c>
+      <c r="D139" s="25" t="inlineStr">
+        <is>
+          <t>SHOT = 100% on next shot attempt after rebounding your own miss.</t>
+        </is>
+      </c>
+      <c r="E139" s="26" t="n"/>
       <c r="F139" s="50" t="n"/>
-      <c r="G139" s="70" t="inlineStr">
-        <is>
-          <t>Discarded during play, it attaches to a random player — possibly you again</t>
+      <c r="G139" s="73" t="inlineStr">
+        <is>
+          <t>Special text: “I understand it now”</t>
         </is>
       </c>
       <c r="H139" s="71" t="n"/>
       <c r="I139" s="71" t="n"/>
       <c r="J139" s="71" t="n"/>
     </row>
-    <row r="140">
+    <row r="140" ht="56" customHeight="1" s="85">
       <c r="A140" s="21" t="n"/>
       <c r="B140" s="22" t="inlineStr">
         <is>
@@ -5863,26 +5872,22 @@
       </c>
       <c r="C140" s="23" t="inlineStr">
         <is>
-          <t>Free Agent</t>
+          <t>Ball Pounder</t>
         </is>
       </c>
       <c r="D140" s="38" t="inlineStr">
         <is>
-          <t>Discard your hand. Play a card at random from a player of your choosing (they keep it)</t>
+          <t>All Dribble cards you play draw an additional card but lower SHOT by an additional 10%</t>
         </is>
       </c>
       <c r="E140" s="7" t="n"/>
       <c r="F140" s="50" t="n"/>
-      <c r="G140" s="70" t="inlineStr">
-        <is>
-          <t>The discard waits for the draw chain to finish. Target is shuffled first and is affected by Floor General. Your own draws are kept. All-0 rebounds are yours; otherwise you cannot bid  [OUT OF THE DECK — the borrow button throws the answer away; back when it routes through Move.borrow]</t>
-        </is>
-      </c>
+      <c r="G140" s="70" t="n"/>
       <c r="H140" s="71" t="n"/>
       <c r="I140" s="71" t="n"/>
       <c r="J140" s="71" t="n"/>
     </row>
-    <row r="141">
+    <row r="141" s="85">
       <c r="A141" s="21" t="n"/>
       <c r="B141" s="22" t="inlineStr">
         <is>
@@ -5891,12 +5896,12 @@
       </c>
       <c r="C141" s="23" t="inlineStr">
         <is>
-          <t>Franchise Player</t>
+          <t>Unselfish</t>
         </is>
       </c>
       <c r="D141" s="38" t="inlineStr">
         <is>
-          <t>When passing, choose 1 of the new player's Intangibles or a card in their hand for them to discard</t>
+          <t>Draw 1 card and increase next SHOT +5% whenever you positively affect another player</t>
         </is>
       </c>
       <c r="E141" s="7" t="n"/>
@@ -5906,229 +5911,337 @@
       <c r="I141" s="71" t="n"/>
       <c r="J141" s="71" t="n"/>
     </row>
-    <row r="142">
-      <c r="A142" s="27" t="n"/>
-      <c r="B142" s="28" t="inlineStr">
+    <row r="142" s="85">
+      <c r="A142" s="21" t="n"/>
+      <c r="B142" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C142" s="56" t="inlineStr">
+      <c r="C142" s="23" t="inlineStr">
+        <is>
+          <t>Dirty Player</t>
+        </is>
+      </c>
+      <c r="D142" s="38" t="inlineStr">
+        <is>
+          <t>When sending Clamps, the clamped player discards 1 if they have any Injuries</t>
+        </is>
+      </c>
+      <c r="E142" s="7" t="n"/>
+      <c r="F142" s="50" t="n"/>
+      <c r="G142" s="70" t="n"/>
+      <c r="H142" s="71" t="n"/>
+      <c r="I142" s="71" t="n"/>
+      <c r="J142" s="71" t="n"/>
+    </row>
+    <row r="143" s="85">
+      <c r="A143" s="21" t="n"/>
+      <c r="B143" s="22" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C143" s="23" t="inlineStr">
+        <is>
+          <t>Villainous Reputation</t>
+        </is>
+      </c>
+      <c r="D143" s="38" t="inlineStr">
+        <is>
+          <t>Discard 1 whenever any Whistle triggers</t>
+        </is>
+      </c>
+      <c r="E143" s="7" t="n"/>
+      <c r="F143" s="50" t="n"/>
+      <c r="G143" s="70" t="inlineStr">
+        <is>
+          <t>Discarded during play, it attaches to a random player — possibly you again</t>
+        </is>
+      </c>
+      <c r="H143" s="71" t="n"/>
+      <c r="I143" s="71" t="n"/>
+      <c r="J143" s="71" t="n"/>
+    </row>
+    <row r="144" s="85">
+      <c r="A144" s="21" t="n"/>
+      <c r="B144" s="22" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C144" s="23" t="inlineStr">
+        <is>
+          <t>Free Agent</t>
+        </is>
+      </c>
+      <c r="D144" s="38" t="inlineStr">
+        <is>
+          <t>Discard your hand. Play a card at random from a player of your choosing (they keep it)</t>
+        </is>
+      </c>
+      <c r="E144" s="7" t="n"/>
+      <c r="F144" s="50" t="n"/>
+      <c r="G144" s="70" t="inlineStr">
+        <is>
+          <t>The discard waits for the draw chain to finish. Target is shuffled first and is affected by Floor General. Your own draws are kept. All-0 rebounds are yours; otherwise you cannot bid  [OUT OF THE DECK — the borrow button throws the answer away; back when it routes through Move.borrow]</t>
+        </is>
+      </c>
+      <c r="H144" s="71" t="n"/>
+      <c r="I144" s="71" t="n"/>
+      <c r="J144" s="71" t="n"/>
+    </row>
+    <row r="145" s="85">
+      <c r="A145" s="21" t="n"/>
+      <c r="B145" s="22" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C145" s="23" t="inlineStr">
+        <is>
+          <t>Franchise Player</t>
+        </is>
+      </c>
+      <c r="D145" s="38" t="inlineStr">
+        <is>
+          <t>When passing, choose 1 of the new player's Intangibles or a card in their hand for them to discard</t>
+        </is>
+      </c>
+      <c r="E145" s="7" t="n"/>
+      <c r="F145" s="50" t="n"/>
+      <c r="G145" s="70" t="n"/>
+      <c r="H145" s="71" t="n"/>
+      <c r="I145" s="71" t="n"/>
+      <c r="J145" s="71" t="n"/>
+    </row>
+    <row r="146" s="85">
+      <c r="A146" s="27" t="n"/>
+      <c r="B146" s="28" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C146" s="56" t="inlineStr">
         <is>
           <t>Fundamentalist</t>
         </is>
       </c>
-      <c r="D142" s="63" t="inlineStr">
+      <c r="D146" s="63" t="inlineStr">
         <is>
           <t>No Special Moves. Each Move once a turn. Swings, Skip Pass and Dribble are never spent</t>
         </is>
       </c>
-      <c r="E142" s="58" t="n"/>
-      <c r="F142" s="61" t="n"/>
-      <c r="G142" s="75" t="n"/>
-      <c r="H142" s="76" t="n"/>
-      <c r="I142" s="76" t="n"/>
-      <c r="J142" s="76" t="n"/>
-    </row>
-    <row r="143" s="85">
-      <c r="A143" s="27" t="n"/>
-      <c r="B143" s="28" t="inlineStr">
+      <c r="E146" s="58" t="n"/>
+      <c r="F146" s="61" t="n"/>
+      <c r="G146" s="75" t="n"/>
+      <c r="H146" s="76" t="n"/>
+      <c r="I146" s="76" t="n"/>
+      <c r="J146" s="76" t="n"/>
+    </row>
+    <row r="147" s="85">
+      <c r="A147" s="27" t="n"/>
+      <c r="B147" s="28" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C143" s="56" t="inlineStr">
+      <c r="C147" s="56" t="inlineStr">
         <is>
           <t>Moves At Own Pace</t>
         </is>
       </c>
-      <c r="D143" s="63" t="inlineStr">
+      <c r="D147" s="63" t="inlineStr">
         <is>
           <t>Cannot be called for Traveling or Shot Clock violations</t>
         </is>
       </c>
-      <c r="E143" s="58" t="n"/>
-      <c r="F143" s="61" t="n">
+      <c r="E147" s="58" t="n"/>
+      <c r="F147" s="61" t="n">
         <v>1</v>
       </c>
-      <c r="G143" s="75" t="n"/>
-      <c r="H143" s="76" t="n"/>
-    </row>
-    <row r="144" ht="42" customHeight="1" s="85">
-      <c r="A144" s="52" t="inlineStr">
+      <c r="G147" s="75" t="n"/>
+      <c r="H147" s="76" t="n"/>
+    </row>
+    <row r="148" ht="42" customHeight="1" s="85">
+      <c r="A148" s="52" t="inlineStr">
         <is>
           <t>Varena</t>
         </is>
       </c>
-      <c r="B144" s="53">
-        <f>COUNTIF($B$145:$B$145,"Varena")</f>
+      <c r="B148" s="53">
+        <f>COUNTIF($B$149:$B$149,"Varena")</f>
         <v/>
       </c>
-      <c r="C144" s="54" t="n"/>
-      <c r="D144" s="54" t="n"/>
-      <c r="E144" s="54" t="n"/>
-      <c r="F144" s="55" t="n"/>
-      <c r="G144" s="66" t="n"/>
-      <c r="H144" s="67" t="n"/>
-      <c r="I144" s="67" t="n"/>
-      <c r="J144" s="67" t="n"/>
-    </row>
-    <row r="145" s="85">
-      <c r="A145" s="27" t="n"/>
-      <c r="B145" s="28" t="inlineStr">
+      <c r="C148" s="54" t="n"/>
+      <c r="D148" s="54" t="n"/>
+      <c r="E148" s="54" t="n"/>
+      <c r="F148" s="55" t="n"/>
+      <c r="G148" s="66" t="n"/>
+      <c r="H148" s="67" t="n"/>
+      <c r="I148" s="67" t="n"/>
+      <c r="J148" s="67" t="n"/>
+    </row>
+    <row r="149" s="85">
+      <c r="A149" s="27" t="n"/>
+      <c r="B149" s="28" t="inlineStr">
         <is>
           <t>Varena</t>
         </is>
       </c>
-      <c r="C145" s="56" t="inlineStr">
+      <c r="C149" s="56" t="inlineStr">
         <is>
           <t>Cardwood</t>
         </is>
       </c>
-      <c r="D145" s="63" t="inlineStr">
+      <c r="D149" s="63" t="inlineStr">
         <is>
           <t>Changes the court back to basic</t>
         </is>
       </c>
-      <c r="E145" s="58" t="n"/>
-      <c r="F145" s="61" t="n">
+      <c r="E149" s="58" t="n"/>
+      <c r="F149" s="61" t="n">
         <v>5</v>
       </c>
-      <c r="G145" s="75" t="inlineStr">
+      <c r="G149" s="75" t="inlineStr">
         <is>
           <t>Also the floor every game opens on, before anybody plays a Varena over it</t>
         </is>
       </c>
-      <c r="H145" s="76" t="n"/>
-      <c r="I145" s="76" t="n"/>
-      <c r="J145" s="76" t="n"/>
+      <c r="H149" s="76" t="n"/>
+      <c r="I149" s="76" t="n"/>
+      <c r="J149" s="76" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="124">
+  <mergeCells count="128">
+    <mergeCell ref="G88:J88"/>
+    <mergeCell ref="G26:J26"/>
     <mergeCell ref="G55:J55"/>
+    <mergeCell ref="G35:J35"/>
     <mergeCell ref="G4:J4"/>
+    <mergeCell ref="G129:J129"/>
+    <mergeCell ref="G109:J109"/>
     <mergeCell ref="G135:J135"/>
-    <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
+    <mergeCell ref="G16:J16"/>
+    <mergeCell ref="G76:J76"/>
+    <mergeCell ref="G25:J25"/>
     <mergeCell ref="G119:J119"/>
     <mergeCell ref="G32:J32"/>
+    <mergeCell ref="G99:J99"/>
     <mergeCell ref="G46:J46"/>
+    <mergeCell ref="G60:J60"/>
     <mergeCell ref="G40:J40"/>
+    <mergeCell ref="G9:J9"/>
     <mergeCell ref="G111:J111"/>
+    <mergeCell ref="G131:J131"/>
+    <mergeCell ref="G140:J140"/>
     <mergeCell ref="G72:J72"/>
     <mergeCell ref="G81:J81"/>
-    <mergeCell ref="G96:J96"/>
+    <mergeCell ref="G59:J59"/>
+    <mergeCell ref="G115:J115"/>
+    <mergeCell ref="G130:J130"/>
+    <mergeCell ref="G11:J11"/>
     <mergeCell ref="G71:J71"/>
     <mergeCell ref="G136:J136"/>
-    <mergeCell ref="G145:J145"/>
+    <mergeCell ref="G117:J117"/>
+    <mergeCell ref="G126:J126"/>
+    <mergeCell ref="G132:J132"/>
     <mergeCell ref="G8:J8"/>
+    <mergeCell ref="G39:J39"/>
+    <mergeCell ref="G122:J122"/>
     <mergeCell ref="G82:J82"/>
-    <mergeCell ref="G57:J57"/>
+    <mergeCell ref="G101:J101"/>
+    <mergeCell ref="G116:J116"/>
+    <mergeCell ref="G103:J103"/>
+    <mergeCell ref="G37:J37"/>
     <mergeCell ref="G128:J128"/>
     <mergeCell ref="G10:J10"/>
     <mergeCell ref="G66:J66"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G57:J57"/>
+    <mergeCell ref="G13:J13"/>
     <mergeCell ref="G18:J18"/>
     <mergeCell ref="G53:J53"/>
+    <mergeCell ref="G78:J78"/>
+    <mergeCell ref="G118:J118"/>
+    <mergeCell ref="G87:J87"/>
     <mergeCell ref="G121:J121"/>
     <mergeCell ref="G34:J34"/>
     <mergeCell ref="G74:J74"/>
     <mergeCell ref="G68:J68"/>
+    <mergeCell ref="G139:J139"/>
+    <mergeCell ref="G15:J15"/>
     <mergeCell ref="G108:J108"/>
+    <mergeCell ref="G80:J80"/>
     <mergeCell ref="G58:J58"/>
     <mergeCell ref="G114:J114"/>
+    <mergeCell ref="G95:J95"/>
+    <mergeCell ref="G89:J89"/>
     <mergeCell ref="G123:J123"/>
     <mergeCell ref="G110:J110"/>
+    <mergeCell ref="G79:J79"/>
+    <mergeCell ref="G64:J64"/>
+    <mergeCell ref="G73:J73"/>
+    <mergeCell ref="G51:J51"/>
     <mergeCell ref="G20:J20"/>
     <mergeCell ref="G113:J113"/>
     <mergeCell ref="G91:J91"/>
     <mergeCell ref="G85:J85"/>
+    <mergeCell ref="G54:J54"/>
     <mergeCell ref="G100:J100"/>
-    <mergeCell ref="G94:J94"/>
+    <mergeCell ref="G63:J63"/>
+    <mergeCell ref="G41:J41"/>
+    <mergeCell ref="G134:J134"/>
+    <mergeCell ref="G50:J50"/>
+    <mergeCell ref="G106:J106"/>
     <mergeCell ref="G75:J75"/>
     <mergeCell ref="G44:J44"/>
     <mergeCell ref="G22:J22"/>
     <mergeCell ref="G84:J84"/>
+    <mergeCell ref="G149:J149"/>
+    <mergeCell ref="G56:J56"/>
     <mergeCell ref="G102:J102"/>
+    <mergeCell ref="G14:J14"/>
+    <mergeCell ref="G105:J105"/>
+    <mergeCell ref="G43:J43"/>
     <mergeCell ref="G12:J12"/>
     <mergeCell ref="G77:J77"/>
+    <mergeCell ref="G52:J52"/>
     <mergeCell ref="G21:J21"/>
+    <mergeCell ref="G86:J86"/>
+    <mergeCell ref="G120:J120"/>
+    <mergeCell ref="G27:J27"/>
+    <mergeCell ref="G98:J98"/>
     <mergeCell ref="G67:J67"/>
+    <mergeCell ref="G36:J36"/>
+    <mergeCell ref="G42:J42"/>
     <mergeCell ref="G61:J61"/>
+    <mergeCell ref="G107:J107"/>
     <mergeCell ref="G70:J70"/>
     <mergeCell ref="G48:J48"/>
     <mergeCell ref="G23:J23"/>
-    <mergeCell ref="G97:J97"/>
+    <mergeCell ref="G17:J17"/>
     <mergeCell ref="G125:J125"/>
+    <mergeCell ref="G38:J38"/>
     <mergeCell ref="G7:J7"/>
-    <mergeCell ref="G38:J38"/>
     <mergeCell ref="G112:J112"/>
-    <mergeCell ref="G45:J45"/>
+    <mergeCell ref="G19:J19"/>
+    <mergeCell ref="G28:J28"/>
     <mergeCell ref="G62:J62"/>
+    <mergeCell ref="G6:J6"/>
     <mergeCell ref="G127:J127"/>
+    <mergeCell ref="G69:J69"/>
     <mergeCell ref="G49:J49"/>
+    <mergeCell ref="G83:J83"/>
     <mergeCell ref="G24:J24"/>
     <mergeCell ref="G33:J33"/>
+    <mergeCell ref="G124:J124"/>
     <mergeCell ref="G104:J104"/>
+    <mergeCell ref="G5:J5"/>
+    <mergeCell ref="G133:J133"/>
     <mergeCell ref="G65:J65"/>
-    <mergeCell ref="G26:J26"/>
-    <mergeCell ref="G35:J35"/>
-    <mergeCell ref="G129:J129"/>
-    <mergeCell ref="G16:J16"/>
-    <mergeCell ref="G76:J76"/>
-    <mergeCell ref="G25:J25"/>
-    <mergeCell ref="G99:J99"/>
-    <mergeCell ref="G60:J60"/>
-    <mergeCell ref="G131:J131"/>
-    <mergeCell ref="G9:J9"/>
-    <mergeCell ref="G59:J59"/>
-    <mergeCell ref="G115:J115"/>
-    <mergeCell ref="G130:J130"/>
-    <mergeCell ref="G11:J11"/>
-    <mergeCell ref="G117:J117"/>
-    <mergeCell ref="G126:J126"/>
-    <mergeCell ref="G132:J132"/>
-    <mergeCell ref="G39:J39"/>
-    <mergeCell ref="G122:J122"/>
-    <mergeCell ref="G101:J101"/>
-    <mergeCell ref="G116:J116"/>
-    <mergeCell ref="G103:J103"/>
-    <mergeCell ref="G37:J37"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="G13:J13"/>
-    <mergeCell ref="G78:J78"/>
-    <mergeCell ref="G118:J118"/>
-    <mergeCell ref="G87:J87"/>
-    <mergeCell ref="G15:J15"/>
-    <mergeCell ref="G80:J80"/>
-    <mergeCell ref="G95:J95"/>
-    <mergeCell ref="G64:J64"/>
-    <mergeCell ref="G79:J79"/>
-    <mergeCell ref="G73:J73"/>
-    <mergeCell ref="G51:J51"/>
-    <mergeCell ref="G54:J54"/>
-    <mergeCell ref="G63:J63"/>
-    <mergeCell ref="G41:J41"/>
-    <mergeCell ref="G50:J50"/>
-    <mergeCell ref="G106:J106"/>
-    <mergeCell ref="G56:J56"/>
-    <mergeCell ref="G105:J105"/>
-    <mergeCell ref="G43:J43"/>
-    <mergeCell ref="G52:J52"/>
-    <mergeCell ref="G27:J27"/>
-    <mergeCell ref="G120:J120"/>
-    <mergeCell ref="G98:J98"/>
-    <mergeCell ref="G36:J36"/>
-    <mergeCell ref="G42:J42"/>
-    <mergeCell ref="G107:J107"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="G19:J19"/>
-    <mergeCell ref="G28:J28"/>
-    <mergeCell ref="G6:J6"/>
-    <mergeCell ref="G69:J69"/>
-    <mergeCell ref="G83:J83"/>
-    <mergeCell ref="G124:J124"/>
-    <mergeCell ref="G5:J5"/>
-    <mergeCell ref="G14:J14"/>
+    <mergeCell ref="G45:J45"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
Add Close-Out and Zone clamps
Close-Out bars threes; a Kick-Out to a Closed-Out player stays a normal pass.
Zone bars shooting, and a Zoned player left with no playable Pass at any point
in the possession turns it over and the round ends.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -3602,7 +3602,7 @@
           <t>SHOT -10%</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E52" s="0" t="inlineStr">
         <is>
           <t>Shoot the ball</t>
         </is>
@@ -3804,7 +3804,7 @@
       </c>
       <c r="G59" s="83" t="inlineStr">
         <is>
-          <t>[NOT IN THE GAME YET]</t>
+          <t>A Kick-Out to them is not shot — it becomes a normal pass</t>
         </is>
       </c>
       <c r="H59" s="76" t="n"/>
@@ -3834,7 +3834,7 @@
       </c>
       <c r="G60" s="83" t="inlineStr">
         <is>
-          <t>[NOT IN THE GAME YET]</t>
+          <t>Checked any time during the possession</t>
         </is>
       </c>
       <c r="H60" s="76" t="n"/>
@@ -6114,133 +6114,133 @@
     </row>
   </sheetData>
   <mergeCells count="128">
-    <mergeCell ref="G88:J88"/>
-    <mergeCell ref="G26:J26"/>
     <mergeCell ref="G55:J55"/>
-    <mergeCell ref="G35:J35"/>
     <mergeCell ref="G4:J4"/>
-    <mergeCell ref="G129:J129"/>
+    <mergeCell ref="G135:J135"/>
     <mergeCell ref="G109:J109"/>
-    <mergeCell ref="G135:J135"/>
     <mergeCell ref="G47:J47"/>
-    <mergeCell ref="G16:J16"/>
-    <mergeCell ref="G76:J76"/>
-    <mergeCell ref="G25:J25"/>
     <mergeCell ref="G119:J119"/>
     <mergeCell ref="G32:J32"/>
-    <mergeCell ref="G99:J99"/>
     <mergeCell ref="G46:J46"/>
-    <mergeCell ref="G60:J60"/>
     <mergeCell ref="G40:J40"/>
-    <mergeCell ref="G9:J9"/>
     <mergeCell ref="G111:J111"/>
-    <mergeCell ref="G131:J131"/>
-    <mergeCell ref="G140:J140"/>
     <mergeCell ref="G72:J72"/>
     <mergeCell ref="G81:J81"/>
-    <mergeCell ref="G59:J59"/>
-    <mergeCell ref="G115:J115"/>
-    <mergeCell ref="G130:J130"/>
-    <mergeCell ref="G11:J11"/>
     <mergeCell ref="G71:J71"/>
     <mergeCell ref="G136:J136"/>
-    <mergeCell ref="G117:J117"/>
-    <mergeCell ref="G126:J126"/>
-    <mergeCell ref="G132:J132"/>
     <mergeCell ref="G8:J8"/>
-    <mergeCell ref="G39:J39"/>
-    <mergeCell ref="G122:J122"/>
     <mergeCell ref="G82:J82"/>
-    <mergeCell ref="G101:J101"/>
-    <mergeCell ref="G116:J116"/>
-    <mergeCell ref="G103:J103"/>
-    <mergeCell ref="G37:J37"/>
+    <mergeCell ref="G57:J57"/>
     <mergeCell ref="G128:J128"/>
     <mergeCell ref="G10:J10"/>
     <mergeCell ref="G66:J66"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="G57:J57"/>
-    <mergeCell ref="G13:J13"/>
     <mergeCell ref="G18:J18"/>
     <mergeCell ref="G53:J53"/>
-    <mergeCell ref="G78:J78"/>
-    <mergeCell ref="G118:J118"/>
-    <mergeCell ref="G87:J87"/>
     <mergeCell ref="G121:J121"/>
     <mergeCell ref="G34:J34"/>
     <mergeCell ref="G74:J74"/>
     <mergeCell ref="G68:J68"/>
     <mergeCell ref="G139:J139"/>
-    <mergeCell ref="G15:J15"/>
     <mergeCell ref="G108:J108"/>
-    <mergeCell ref="G80:J80"/>
     <mergeCell ref="G58:J58"/>
     <mergeCell ref="G114:J114"/>
-    <mergeCell ref="G95:J95"/>
-    <mergeCell ref="G89:J89"/>
     <mergeCell ref="G123:J123"/>
     <mergeCell ref="G110:J110"/>
-    <mergeCell ref="G79:J79"/>
-    <mergeCell ref="G64:J64"/>
-    <mergeCell ref="G73:J73"/>
-    <mergeCell ref="G51:J51"/>
     <mergeCell ref="G20:J20"/>
     <mergeCell ref="G113:J113"/>
     <mergeCell ref="G91:J91"/>
     <mergeCell ref="G85:J85"/>
+    <mergeCell ref="G100:J100"/>
+    <mergeCell ref="G75:J75"/>
+    <mergeCell ref="G44:J44"/>
+    <mergeCell ref="G22:J22"/>
+    <mergeCell ref="G84:J84"/>
+    <mergeCell ref="G149:J149"/>
+    <mergeCell ref="G102:J102"/>
+    <mergeCell ref="G12:J12"/>
+    <mergeCell ref="G77:J77"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="G86:J86"/>
+    <mergeCell ref="G67:J67"/>
+    <mergeCell ref="G61:J61"/>
+    <mergeCell ref="G70:J70"/>
+    <mergeCell ref="G48:J48"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="G125:J125"/>
+    <mergeCell ref="G38:J38"/>
+    <mergeCell ref="G7:J7"/>
+    <mergeCell ref="G112:J112"/>
+    <mergeCell ref="G62:J62"/>
+    <mergeCell ref="G127:J127"/>
+    <mergeCell ref="G49:J49"/>
+    <mergeCell ref="G24:J24"/>
+    <mergeCell ref="G33:J33"/>
+    <mergeCell ref="G104:J104"/>
+    <mergeCell ref="G65:J65"/>
+    <mergeCell ref="G88:J88"/>
+    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="G35:J35"/>
+    <mergeCell ref="G129:J129"/>
+    <mergeCell ref="G16:J16"/>
+    <mergeCell ref="G76:J76"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="G99:J99"/>
+    <mergeCell ref="G60:J60"/>
+    <mergeCell ref="G9:J9"/>
+    <mergeCell ref="G131:J131"/>
+    <mergeCell ref="G140:J140"/>
+    <mergeCell ref="G59:J59"/>
+    <mergeCell ref="G115:J115"/>
+    <mergeCell ref="G130:J130"/>
+    <mergeCell ref="G11:J11"/>
+    <mergeCell ref="G117:J117"/>
+    <mergeCell ref="G126:J126"/>
+    <mergeCell ref="G132:J132"/>
+    <mergeCell ref="G39:J39"/>
+    <mergeCell ref="G122:J122"/>
+    <mergeCell ref="G101:J101"/>
+    <mergeCell ref="G116:J116"/>
+    <mergeCell ref="G103:J103"/>
+    <mergeCell ref="G37:J37"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G13:J13"/>
+    <mergeCell ref="G78:J78"/>
+    <mergeCell ref="G118:J118"/>
+    <mergeCell ref="G87:J87"/>
+    <mergeCell ref="G15:J15"/>
+    <mergeCell ref="G80:J80"/>
+    <mergeCell ref="G95:J95"/>
+    <mergeCell ref="G89:J89"/>
+    <mergeCell ref="G64:J64"/>
+    <mergeCell ref="G79:J79"/>
+    <mergeCell ref="G73:J73"/>
+    <mergeCell ref="G51:J51"/>
     <mergeCell ref="G54:J54"/>
-    <mergeCell ref="G100:J100"/>
     <mergeCell ref="G63:J63"/>
     <mergeCell ref="G41:J41"/>
     <mergeCell ref="G134:J134"/>
     <mergeCell ref="G50:J50"/>
     <mergeCell ref="G106:J106"/>
-    <mergeCell ref="G75:J75"/>
-    <mergeCell ref="G44:J44"/>
-    <mergeCell ref="G22:J22"/>
-    <mergeCell ref="G84:J84"/>
-    <mergeCell ref="G149:J149"/>
     <mergeCell ref="G56:J56"/>
-    <mergeCell ref="G102:J102"/>
     <mergeCell ref="G14:J14"/>
     <mergeCell ref="G105:J105"/>
     <mergeCell ref="G43:J43"/>
-    <mergeCell ref="G12:J12"/>
-    <mergeCell ref="G77:J77"/>
     <mergeCell ref="G52:J52"/>
-    <mergeCell ref="G21:J21"/>
-    <mergeCell ref="G86:J86"/>
     <mergeCell ref="G120:J120"/>
     <mergeCell ref="G27:J27"/>
     <mergeCell ref="G98:J98"/>
-    <mergeCell ref="G67:J67"/>
     <mergeCell ref="G36:J36"/>
     <mergeCell ref="G42:J42"/>
-    <mergeCell ref="G61:J61"/>
     <mergeCell ref="G107:J107"/>
-    <mergeCell ref="G70:J70"/>
-    <mergeCell ref="G48:J48"/>
-    <mergeCell ref="G23:J23"/>
     <mergeCell ref="G17:J17"/>
-    <mergeCell ref="G125:J125"/>
-    <mergeCell ref="G38:J38"/>
-    <mergeCell ref="G7:J7"/>
-    <mergeCell ref="G112:J112"/>
     <mergeCell ref="G19:J19"/>
     <mergeCell ref="G28:J28"/>
-    <mergeCell ref="G62:J62"/>
     <mergeCell ref="G6:J6"/>
-    <mergeCell ref="G127:J127"/>
     <mergeCell ref="G69:J69"/>
-    <mergeCell ref="G49:J49"/>
     <mergeCell ref="G83:J83"/>
-    <mergeCell ref="G24:J24"/>
-    <mergeCell ref="G33:J33"/>
     <mergeCell ref="G124:J124"/>
-    <mergeCell ref="G104:J104"/>
     <mergeCell ref="G5:J5"/>
     <mergeCell ref="G133:J133"/>
-    <mergeCell ref="G65:J65"/>
     <mergeCell ref="G45:J45"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>

</xml_diff>

<commit_message>
COMBO and BONUS buttons, the ball re-imported, Variaball art, Unselfish plumbing out
A raised card with a combo or a bonus gets capsule buttons under its words. COMBO opens a
scene over a dim: the card, dotted chevrons, and what it pairs with, fanned when there are
several routes. Routes not done yet are locked grey cards with a question mark on the
Variaball plate, and a combo with none done has no name. Combos done are recorded per
route, passes included. BONUS opens a popover with the card's conditional half and, on
every shooting card, Shoot the ball.

The ball is re-imported trimmed and on the palette, and the Variaball type icon is framed
from its plate and subject. Rules.credit and the owed shot bonus are gone with Unselfish.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -2206,7 +2206,6 @@
         <v/>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="20.75" customHeight="1" s="85">
       <c r="A4" s="81" t="inlineStr">
         <is>
@@ -2672,10 +2671,14 @@
       </c>
       <c r="D20" s="30" t="inlineStr">
         <is>
-          <t>SHOT +20%. Pass to player of choice. If played as first action, draw 2 cards</t>
-        </is>
-      </c>
-      <c r="E20" s="30" t="n"/>
+          <t>SHOT +20%. Pass to player of choice</t>
+        </is>
+      </c>
+      <c r="E20" s="30" t="inlineStr">
+        <is>
+          <t>If played as first action, draw 2 cards</t>
+        </is>
+      </c>
       <c r="F20" s="35" t="n">
         <v>5</v>
       </c>
@@ -2945,10 +2948,14 @@
       </c>
       <c r="D30" s="41" t="inlineStr">
         <is>
-          <t>SHOT + 10%. If being Clamped, discard all Clamps and gain additional SHOT +20% for each</t>
-        </is>
-      </c>
-      <c r="E30" s="26" t="n"/>
+          <t>SHOT + 10%</t>
+        </is>
+      </c>
+      <c r="E30" s="26" t="inlineStr">
+        <is>
+          <t>If being Clamped, discard all Clamps and gain additional SHOT +20% for each</t>
+        </is>
+      </c>
       <c r="F30" s="33" t="n">
         <v>5</v>
       </c>
@@ -2975,10 +2982,14 @@
       </c>
       <c r="D31" s="41" t="inlineStr">
         <is>
-          <t>Draw 1 Card. SHOT +20%. If being Clamped, discard all clamps and Draw 1 card and Clamp-sender discards 1card for each</t>
-        </is>
-      </c>
-      <c r="E31" s="26" t="n"/>
+          <t>Draw 1 Card. SHOT +20%</t>
+        </is>
+      </c>
+      <c r="E31" s="26" t="inlineStr">
+        <is>
+          <t>If being Clamped, discard all clamps and Draw 1 card and Clamp-sender discards 1card for each</t>
+        </is>
+      </c>
       <c r="F31" s="33" t="n">
         <v>5</v>
       </c>
@@ -3401,12 +3412,12 @@
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>SHOT +20%. SHOT = 100% if SHOT &gt;= 75%</t>
+          <t>SHOT +20%</t>
         </is>
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>Shoot the ball</t>
+          <t>Shoot the ball. SHOT = 100% if SHOT &gt;= 75%</t>
         </is>
       </c>
       <c r="F45" s="32" t="n">
@@ -3524,7 +3535,12 @@
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>SHOT +20%. Shoot the ball. Another +10% straight off your own board</t>
+          <t>SHOT +20%</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Shoot the ball. Another +10% straight off your own board</t>
         </is>
       </c>
       <c r="F49" s="0" t="n">
@@ -3549,7 +3565,12 @@
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>Clean look only — no Clamps on you and nothing has gone off this possession. SHOT +30%. Shoot the ball</t>
+          <t>Clean look only — no Clamps on you and nothing has gone off this possession. SHOT +30%</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Shoot the ball</t>
         </is>
       </c>
       <c r="F50" s="0" t="n">
@@ -3574,7 +3595,12 @@
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>SHOT +15% at 50% or better, −15% under it. Shoot the ball</t>
+          <t>SHOT +15% at 50% or better, −15% under it</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Shoot the ball</t>
         </is>
       </c>
       <c r="F51" s="0" t="n">
@@ -6154,12 +6180,12 @@
   <mergeCells count="128">
     <mergeCell ref="G55:J55"/>
     <mergeCell ref="G4:J4"/>
+    <mergeCell ref="G135:J135"/>
     <mergeCell ref="G109:J109"/>
-    <mergeCell ref="G135:J135"/>
     <mergeCell ref="G47:J47"/>
-    <mergeCell ref="G32:J32"/>
     <mergeCell ref="G119:J119"/>
     <mergeCell ref="G150:J150"/>
+    <mergeCell ref="G32:J32"/>
     <mergeCell ref="G46:J46"/>
     <mergeCell ref="G40:J40"/>
     <mergeCell ref="G111:J111"/>
@@ -6170,13 +6196,13 @@
     <mergeCell ref="G8:J8"/>
     <mergeCell ref="G82:J82"/>
     <mergeCell ref="G57:J57"/>
+    <mergeCell ref="G128:J128"/>
     <mergeCell ref="G10:J10"/>
     <mergeCell ref="G66:J66"/>
-    <mergeCell ref="G128:J128"/>
     <mergeCell ref="G18:J18"/>
     <mergeCell ref="G53:J53"/>
+    <mergeCell ref="G121:J121"/>
     <mergeCell ref="G34:J34"/>
-    <mergeCell ref="G121:J121"/>
     <mergeCell ref="G74:J74"/>
     <mergeCell ref="G68:J68"/>
     <mergeCell ref="G139:J139"/>
@@ -6204,9 +6230,9 @@
     <mergeCell ref="G70:J70"/>
     <mergeCell ref="G48:J48"/>
     <mergeCell ref="G23:J23"/>
+    <mergeCell ref="G125:J125"/>
     <mergeCell ref="G38:J38"/>
     <mergeCell ref="G7:J7"/>
-    <mergeCell ref="G125:J125"/>
     <mergeCell ref="G112:J112"/>
     <mergeCell ref="G62:J62"/>
     <mergeCell ref="G127:J127"/>
@@ -6226,17 +6252,16 @@
     <mergeCell ref="G60:J60"/>
     <mergeCell ref="G9:J9"/>
     <mergeCell ref="G131:J131"/>
-    <mergeCell ref="G124:J124"/>
     <mergeCell ref="G140:J140"/>
     <mergeCell ref="G59:J59"/>
     <mergeCell ref="G115:J115"/>
     <mergeCell ref="G130:J130"/>
     <mergeCell ref="G11:J11"/>
     <mergeCell ref="G117:J117"/>
+    <mergeCell ref="G126:J126"/>
     <mergeCell ref="G39:J39"/>
-    <mergeCell ref="G126:J126"/>
+    <mergeCell ref="G132:J132"/>
     <mergeCell ref="G122:J122"/>
-    <mergeCell ref="G132:J132"/>
     <mergeCell ref="G101:J101"/>
     <mergeCell ref="G116:J116"/>
     <mergeCell ref="G103:J103"/>
@@ -6246,7 +6271,6 @@
     <mergeCell ref="G78:J78"/>
     <mergeCell ref="G118:J118"/>
     <mergeCell ref="G87:J87"/>
-    <mergeCell ref="G133:J133"/>
     <mergeCell ref="G15:J15"/>
     <mergeCell ref="G80:J80"/>
     <mergeCell ref="G95:J95"/>
@@ -6267,8 +6291,8 @@
     <mergeCell ref="G43:J43"/>
     <mergeCell ref="G52:J52"/>
     <mergeCell ref="G27:J27"/>
+    <mergeCell ref="G120:J120"/>
     <mergeCell ref="G98:J98"/>
-    <mergeCell ref="G120:J120"/>
     <mergeCell ref="G36:J36"/>
     <mergeCell ref="G42:J42"/>
     <mergeCell ref="G107:J107"/>
@@ -6278,7 +6302,9 @@
     <mergeCell ref="G6:J6"/>
     <mergeCell ref="G69:J69"/>
     <mergeCell ref="G83:J83"/>
+    <mergeCell ref="G124:J124"/>
     <mergeCell ref="G5:J5"/>
+    <mergeCell ref="G133:J133"/>
     <mergeCell ref="G45:J45"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>

</xml_diff>

<commit_message>
Every Varena and Variaball in the deck
All 28 new Varenas and 16 Variaballs, Tile Tampering, Over-Varing Evidence, and the three
Intangibles that read the slots (Varsitile, Brawl Handler, Baller). The deck is 498.

One owner each for changing the floor and the ball, with every arrival effect; possession-
opening effects, shot-time effects, Monster Ball's Intangible boards through the rebound
bid, Policeum's referees, Tick-Tock and Frostbite's owed costs. New moves for Traderous
Tarmac hand-offs, Varsitile exchanges and S.O.S twos, with sheets for each. The floor and
ball in play sit top-left of the court; Dim Dome hides SHOT on the badge, in the log and on
the wire. The AI plays slot cards, hands off Clamps and takes S.O.S twos when they pay.

46 new tests in Tools/slottests.swift, and ./Tools/sim --slots reads out how often the house
plays each card. The master sheet and design docs carry every card and ruling.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -2089,7 +2089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J150"/>
+  <dimension ref="A1:J197"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="22.25" customHeight="1"/>
   <cols>
     <col width="15.5" customWidth="1" style="8" min="1" max="1"/>
@@ -2170,42 +2170,43 @@
         </is>
       </c>
       <c r="B2" s="12">
-        <f>COUNTIF($B$5:$B$144,"Pass")</f>
+        <f>COUNTIF($B$5:$B$146,"Pass")</f>
         <v/>
       </c>
       <c r="C2" s="13">
-        <f>COUNTIF($B$5:$B$144,"Move")+COUNTIF($B$5:$B$144,"Special Move")</f>
+        <f>COUNTIF($B$5:$B$146,"Move")+COUNTIF($B$5:$B$146,"Special Move")</f>
         <v/>
       </c>
       <c r="D2" s="14">
-        <f>COUNTIF($B$5:$B$144,"Clamp")</f>
+        <f>COUNTIF($B$5:$B$146,"Clamp")</f>
         <v/>
       </c>
       <c r="E2" s="15">
-        <f>COUNTIF($B$5:$B$144,"Whistle")</f>
+        <f>COUNTIF($B$5:$B$146,"Whistle")</f>
         <v/>
       </c>
       <c r="F2" s="16">
-        <f>COUNTIF($B$5:$B$144,"Game Break")</f>
+        <f>COUNTIF($B$5:$B$146,"Game Break")</f>
         <v/>
       </c>
       <c r="G2" s="18">
-        <f>COUNTIF($B$5:$B$144,"Injury")</f>
+        <f>COUNTIF($B$5:$B$146,"Injury")</f>
         <v/>
       </c>
       <c r="H2" s="19">
-        <f>COUNTIF($B$5:$B$144,"Devastating Injury")</f>
+        <f>COUNTIF($B$5:$B$146,"Devastating Injury")</f>
         <v/>
       </c>
       <c r="I2" s="17">
-        <f>COUNTIF($B$5:$B$144,"Intangible")</f>
+        <f>COUNTIF($B$5:$B$146,"Intangible")</f>
         <v/>
       </c>
       <c r="J2" s="87">
-        <f>SUM(B2:E2)+COUNTIF($B$5:$B$144,"Game Break")+SUM(G2:I2)</f>
+        <f>SUM(B2:E2)+COUNTIF($B$5:$B$146,"Game Break")+SUM(G2:I2)</f>
         <v/>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="20.75" customHeight="1" s="85">
       <c r="A4" s="81" t="inlineStr">
         <is>
@@ -2249,7 +2250,7 @@
         </is>
       </c>
       <c r="B5" s="53">
-        <f>COUNTIF($B$6:$B$148,"Pass")</f>
+        <f>COUNTIF($B$6:$B$150,"Pass")</f>
         <v/>
       </c>
       <c r="C5" s="54" t="n"/>
@@ -2694,7 +2695,7 @@
         </is>
       </c>
       <c r="B21" s="53">
-        <f>COUNTIF($B$22:$B$148,"Move")+COUNTIF($B$22:$B$148,"Special Move")</f>
+        <f>COUNTIF($B$22:$B$150,"Move")+COUNTIF($B$22:$B$150,"Special Move")</f>
         <v/>
       </c>
       <c r="C21" s="54" t="n"/>
@@ -3110,7 +3111,7 @@
         </is>
       </c>
       <c r="B35" s="53">
-        <f>COUNTIF($B$36:$B$148,"Special Move")</f>
+        <f>COUNTIF($B$36:$B$150,"Special Move")</f>
         <v/>
       </c>
       <c r="C35" s="54" t="n"/>
@@ -3538,7 +3539,7 @@
           <t>SHOT +20%</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E49" s="0" t="inlineStr">
         <is>
           <t>Shoot the ball. Another +10% straight off your own board</t>
         </is>
@@ -3568,7 +3569,7 @@
           <t>Clean look only — no Clamps on you and nothing has gone off this possession. SHOT +30%</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E50" s="0" t="inlineStr">
         <is>
           <t>Shoot the ball</t>
         </is>
@@ -3598,7 +3599,7 @@
           <t>SHOT +15% at 50% or better, −15% under it</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E51" s="0" t="inlineStr">
         <is>
           <t>Shoot the ball</t>
         </is>
@@ -3645,7 +3646,7 @@
         </is>
       </c>
       <c r="B53" s="53">
-        <f>COUNTIF($B$54:$B$148,"Clamp")</f>
+        <f>COUNTIF($B$54:$B$150,"Clamp")</f>
         <v/>
       </c>
       <c r="C53" s="54" t="n"/>
@@ -3900,7 +3901,7 @@
         </is>
       </c>
       <c r="B62" s="53">
-        <f>COUNTIF($B$63:$B$148,"Whistle")</f>
+        <f>COUNTIF($B$63:$B$150,"Whistle")</f>
         <v/>
       </c>
       <c r="C62" s="54" t="n"/>
@@ -4431,79 +4432,79 @@
       <c r="J82" s="76" t="n"/>
     </row>
     <row r="83" ht="28" customHeight="1" s="85">
-      <c r="A83" s="52" t="inlineStr">
+      <c r="A83" s="27" t="n"/>
+      <c r="B83" s="28" t="inlineStr">
+        <is>
+          <t>Whistle</t>
+        </is>
+      </c>
+      <c r="C83" s="29" t="inlineStr">
+        <is>
+          <t>Tile Tampering</t>
+        </is>
+      </c>
+      <c r="D83" s="30" t="inlineStr">
+        <is>
+          <t>Varena Played: Cancel card. TOV +1</t>
+        </is>
+      </c>
+      <c r="E83" s="60" t="n"/>
+      <c r="F83" s="61" t="n"/>
+      <c r="G83" s="78" t="inlineStr">
+        <is>
+          <t>The Varena's player inbounds (side-out)</t>
+        </is>
+      </c>
+      <c r="H83" s="76" t="n"/>
+      <c r="I83" s="76" t="n"/>
+      <c r="J83" s="76" t="n"/>
+    </row>
+    <row r="84" ht="28" customHeight="1" s="85">
+      <c r="A84" s="27" t="n"/>
+      <c r="B84" s="28" t="inlineStr">
+        <is>
+          <t>Whistle</t>
+        </is>
+      </c>
+      <c r="C84" s="29" t="inlineStr">
+        <is>
+          <t>Over-Varing Evidence</t>
+        </is>
+      </c>
+      <c r="D84" s="30" t="inlineStr">
+        <is>
+          <t>Variaball Played: Cancel card. TOV +1</t>
+        </is>
+      </c>
+      <c r="E84" s="60" t="n"/>
+      <c r="F84" s="61" t="n"/>
+      <c r="G84" s="78" t="inlineStr">
+        <is>
+          <t>The Variaball's player inbounds (side-out)</t>
+        </is>
+      </c>
+      <c r="H84" s="76" t="n"/>
+      <c r="I84" s="76" t="n"/>
+      <c r="J84" s="76" t="n"/>
+    </row>
+    <row r="85" ht="28" customHeight="1" s="85">
+      <c r="A85" s="52" t="inlineStr">
         <is>
           <t>Retired Game Breaks</t>
         </is>
       </c>
-      <c r="B83" s="53">
-        <f>COUNTIF($B$84:$B$113,"Retired Game Break")</f>
+      <c r="B85" s="53">
+        <f>COUNTIF($B$86:$B$115,"Retired Game Break")</f>
         <v/>
       </c>
-      <c r="C83" s="54" t="n"/>
-      <c r="D83" s="54" t="n"/>
-      <c r="E83" s="54" t="n"/>
-      <c r="F83" s="55" t="n"/>
-      <c r="G83" s="66" t="n"/>
-      <c r="H83" s="67" t="n"/>
-      <c r="I83" s="67" t="n"/>
-      <c r="J83" s="67" t="n"/>
-    </row>
-    <row r="84" ht="20" customHeight="1" s="85">
-      <c r="A84" s="21" t="n"/>
-      <c r="B84" s="22" t="inlineStr">
-        <is>
-          <t>Retired Game Break</t>
-        </is>
-      </c>
-      <c r="C84" s="24" t="inlineStr">
-        <is>
-          <t>2-Minute Warning</t>
-        </is>
-      </c>
-      <c r="D84" s="25" t="inlineStr">
-        <is>
-          <t>All players discard down to 2 or fewer cards</t>
-        </is>
-      </c>
-      <c r="E84" s="26" t="n"/>
-      <c r="F84" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G84" s="72" t="n"/>
-      <c r="H84" s="71" t="n"/>
-      <c r="I84" s="71" t="n"/>
-      <c r="J84" s="71" t="n"/>
-    </row>
-    <row r="85" ht="28" customHeight="1" s="85">
-      <c r="A85" s="21" t="n"/>
-      <c r="B85" s="22" t="inlineStr">
-        <is>
-          <t>Retired Game Break</t>
-        </is>
-      </c>
-      <c r="C85" s="23" t="inlineStr">
-        <is>
-          <t>Benched</t>
-        </is>
-      </c>
-      <c r="D85" s="6" t="inlineStr">
-        <is>
-          <t>Immediately give ball to any other player.</t>
-        </is>
-      </c>
-      <c r="E85" s="7" t="n"/>
-      <c r="F85" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="G85" s="74" t="inlineStr">
-        <is>
-          <t>This is not a pass</t>
-        </is>
-      </c>
-      <c r="H85" s="71" t="n"/>
-      <c r="I85" s="71" t="n"/>
-      <c r="J85" s="71" t="n"/>
+      <c r="C85" s="54" t="n"/>
+      <c r="D85" s="54" t="n"/>
+      <c r="E85" s="54" t="n"/>
+      <c r="F85" s="55" t="n"/>
+      <c r="G85" s="66" t="n"/>
+      <c r="H85" s="67" t="n"/>
+      <c r="I85" s="67" t="n"/>
+      <c r="J85" s="67" t="n"/>
     </row>
     <row r="86" ht="20" customHeight="1" s="85">
       <c r="A86" s="21" t="n"/>
@@ -4514,12 +4515,12 @@
       </c>
       <c r="C86" s="24" t="inlineStr">
         <is>
-          <t>Crowd Noise</t>
+          <t>2-Minute Warning</t>
         </is>
       </c>
       <c r="D86" s="25" t="inlineStr">
         <is>
-          <t>Discard 1 card.</t>
+          <t>All players discard down to 2 or fewer cards</t>
         </is>
       </c>
       <c r="E86" s="26" t="n"/>
@@ -4531,7 +4532,7 @@
       <c r="I86" s="71" t="n"/>
       <c r="J86" s="71" t="n"/>
     </row>
-    <row r="87" ht="42" customHeight="1" s="85">
+    <row r="87" ht="28" customHeight="1" s="85">
       <c r="A87" s="21" t="n"/>
       <c r="B87" s="22" t="inlineStr">
         <is>
@@ -4540,38 +4541,42 @@
       </c>
       <c r="C87" s="23" t="inlineStr">
         <is>
-          <t>Designed Play</t>
+          <t>Benched</t>
         </is>
       </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>Draw up to a hand of 5</t>
+          <t>Immediately give ball to any other player.</t>
         </is>
       </c>
       <c r="E87" s="7" t="n"/>
       <c r="F87" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G87" s="70" t="n"/>
+      <c r="G87" s="74" t="inlineStr">
+        <is>
+          <t>This is not a pass</t>
+        </is>
+      </c>
       <c r="H87" s="71" t="n"/>
       <c r="I87" s="71" t="n"/>
       <c r="J87" s="71" t="n"/>
     </row>
-    <row r="88" ht="28" customHeight="1" s="85">
+    <row r="88" ht="20" customHeight="1" s="85">
       <c r="A88" s="21" t="n"/>
       <c r="B88" s="22" t="inlineStr">
         <is>
           <t>Retired Game Break</t>
         </is>
       </c>
-      <c r="C88" s="37" t="inlineStr">
-        <is>
-          <t>Foul</t>
+      <c r="C88" s="24" t="inlineStr">
+        <is>
+          <t>Crowd Noise</t>
         </is>
       </c>
       <c r="D88" s="25" t="inlineStr">
         <is>
-          <t>Take 1 FT</t>
+          <t>Discard 1 card.</t>
         </is>
       </c>
       <c r="E88" s="26" t="n"/>
@@ -4583,7 +4588,7 @@
       <c r="I88" s="71" t="n"/>
       <c r="J88" s="71" t="n"/>
     </row>
-    <row r="89" ht="56" customHeight="1" s="85">
+    <row r="89" ht="42" customHeight="1" s="85">
       <c r="A89" s="21" t="n"/>
       <c r="B89" s="22" t="inlineStr">
         <is>
@@ -4592,12 +4597,12 @@
       </c>
       <c r="C89" s="23" t="inlineStr">
         <is>
-          <t>MVP Vote</t>
+          <t>Designed Play</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>Draw 3 cards up to a hand of 7</t>
+          <t>Draw up to a hand of 5</t>
         </is>
       </c>
       <c r="E89" s="7" t="n"/>
@@ -4609,21 +4614,21 @@
       <c r="I89" s="71" t="n"/>
       <c r="J89" s="71" t="n"/>
     </row>
-    <row r="90" ht="42" customHeight="1" s="85">
+    <row r="90" ht="28" customHeight="1" s="85">
       <c r="A90" s="21" t="n"/>
       <c r="B90" s="22" t="inlineStr">
         <is>
           <t>Retired Game Break</t>
         </is>
       </c>
-      <c r="C90" s="24" t="inlineStr">
-        <is>
-          <t>Off Night</t>
+      <c r="C90" s="37" t="inlineStr">
+        <is>
+          <t>Foul</t>
         </is>
       </c>
       <c r="D90" s="25" t="inlineStr">
         <is>
-          <t>SHOT -20% this possession</t>
+          <t>Take 1 FT</t>
         </is>
       </c>
       <c r="E90" s="26" t="n"/>
@@ -4635,7 +4640,7 @@
       <c r="I90" s="71" t="n"/>
       <c r="J90" s="71" t="n"/>
     </row>
-    <row r="91" ht="42" customHeight="1" s="85">
+    <row r="91" ht="56" customHeight="1" s="85">
       <c r="A91" s="21" t="n"/>
       <c r="B91" s="22" t="inlineStr">
         <is>
@@ -4644,20 +4649,16 @@
       </c>
       <c r="C91" s="23" t="inlineStr">
         <is>
-          <t>Swallowed Whistle</t>
+          <t>MVP Vote</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>Whistle cards cannot activate this turn.</t>
-        </is>
-      </c>
-      <c r="E91" s="6" t="inlineStr">
-        <is>
-          <t>Remains for remainder of round</t>
-        </is>
-      </c>
-      <c r="F91" s="32" t="n">
+          <t>Draw 3 cards up to a hand of 7</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="n"/>
+      <c r="F91" s="34" t="n">
         <v>0</v>
       </c>
       <c r="G91" s="70" t="n"/>
@@ -4665,7 +4666,7 @@
       <c r="I91" s="71" t="n"/>
       <c r="J91" s="71" t="n"/>
     </row>
-    <row r="92" ht="28" customHeight="1" s="85">
+    <row r="92" ht="42" customHeight="1" s="85">
       <c r="A92" s="21" t="n"/>
       <c r="B92" s="22" t="inlineStr">
         <is>
@@ -4674,20 +4675,16 @@
       </c>
       <c r="C92" s="24" t="inlineStr">
         <is>
-          <t>Rock Fight</t>
+          <t>Off Night</t>
         </is>
       </c>
       <c r="D92" s="25" t="inlineStr">
         <is>
-          <t>Players cannot shoot when SHOT is above 50%</t>
-        </is>
-      </c>
-      <c r="E92" s="25" t="inlineStr">
-        <is>
-          <t>Remains for remainder of round</t>
-        </is>
-      </c>
-      <c r="F92" s="36" t="n">
+          <t>SHOT -20% this possession</t>
+        </is>
+      </c>
+      <c r="E92" s="26" t="n"/>
+      <c r="F92" s="33" t="n">
         <v>0</v>
       </c>
       <c r="G92" s="72" t="n"/>
@@ -4695,7 +4692,7 @@
       <c r="I92" s="71" t="n"/>
       <c r="J92" s="71" t="n"/>
     </row>
-    <row r="93" ht="28" customHeight="1" s="85">
+    <row r="93" ht="42" customHeight="1" s="85">
       <c r="A93" s="21" t="n"/>
       <c r="B93" s="22" t="inlineStr">
         <is>
@@ -4704,80 +4701,84 @@
       </c>
       <c r="C93" s="23" t="inlineStr">
         <is>
-          <t>Traded Mid-Game</t>
+          <t>Swallowed Whistle</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>Swap hands with a random other player</t>
-        </is>
-      </c>
-      <c r="E93" s="7" t="n"/>
-      <c r="F93" s="34" t="n">
+          <t>Whistle cards cannot activate this turn.</t>
+        </is>
+      </c>
+      <c r="E93" s="6" t="inlineStr">
+        <is>
+          <t>Remains for remainder of round</t>
+        </is>
+      </c>
+      <c r="F93" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="G93" s="74" t="n"/>
+      <c r="G93" s="70" t="n"/>
       <c r="H93" s="71" t="n"/>
       <c r="I93" s="71" t="n"/>
       <c r="J93" s="71" t="n"/>
     </row>
-    <row r="94" ht="56" customHeight="1" s="85">
+    <row r="94" ht="28" customHeight="1" s="85">
       <c r="A94" s="21" t="n"/>
       <c r="B94" s="22" t="inlineStr">
         <is>
           <t>Retired Game Break</t>
         </is>
       </c>
-      <c r="C94" s="49" t="inlineStr">
-        <is>
-          <t>Salary Cap Increase</t>
-        </is>
-      </c>
-      <c r="D94" s="38" t="inlineStr">
-        <is>
-          <t>All players draw 2 cards</t>
-        </is>
-      </c>
-      <c r="E94" s="7" t="n"/>
-      <c r="F94" s="34" t="n">
+      <c r="C94" s="24" t="inlineStr">
+        <is>
+          <t>Rock Fight</t>
+        </is>
+      </c>
+      <c r="D94" s="25" t="inlineStr">
+        <is>
+          <t>Players cannot shoot when SHOT is above 50%</t>
+        </is>
+      </c>
+      <c r="E94" s="25" t="inlineStr">
+        <is>
+          <t>Remains for remainder of round</t>
+        </is>
+      </c>
+      <c r="F94" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="G94" s="74" t="n"/>
+      <c r="G94" s="72" t="n"/>
       <c r="H94" s="71" t="n"/>
       <c r="I94" s="71" t="n"/>
       <c r="J94" s="71" t="n"/>
     </row>
-    <row r="95" ht="56" customHeight="1" s="85">
+    <row r="95" ht="28" customHeight="1" s="85">
       <c r="A95" s="21" t="n"/>
       <c r="B95" s="22" t="inlineStr">
         <is>
           <t>Retired Game Break</t>
         </is>
       </c>
-      <c r="C95" s="49" t="inlineStr">
-        <is>
-          <t>All-Swissh Selection</t>
-        </is>
-      </c>
-      <c r="D95" s="38" t="inlineStr">
-        <is>
-          <t>Draw 3 cards after your next make</t>
+      <c r="C95" s="23" t="inlineStr">
+        <is>
+          <t>Traded Mid-Game</t>
+        </is>
+      </c>
+      <c r="D95" s="6" t="inlineStr">
+        <is>
+          <t>Swap hands with a random other player</t>
         </is>
       </c>
       <c r="E95" s="7" t="n"/>
       <c r="F95" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G95" s="74" t="inlineStr">
-        <is>
-          <t>Arms an icon in the HUD tracking the pending draws</t>
-        </is>
-      </c>
+      <c r="G95" s="74" t="n"/>
       <c r="H95" s="71" t="n"/>
       <c r="I95" s="71" t="n"/>
       <c r="J95" s="71" t="n"/>
     </row>
-    <row r="96" ht="28" customHeight="1" s="85">
+    <row r="96" ht="56" customHeight="1" s="85">
       <c r="A96" s="21" t="n"/>
       <c r="B96" s="22" t="inlineStr">
         <is>
@@ -4786,12 +4787,12 @@
       </c>
       <c r="C96" s="49" t="inlineStr">
         <is>
-          <t>All Star Selection</t>
+          <t>Salary Cap Increase</t>
         </is>
       </c>
       <c r="D96" s="38" t="inlineStr">
         <is>
-          <t>Draw 2 cards</t>
+          <t>All players draw 2 cards</t>
         </is>
       </c>
       <c r="E96" s="7" t="n"/>
@@ -4803,7 +4804,7 @@
       <c r="I96" s="71" t="n"/>
       <c r="J96" s="71" t="n"/>
     </row>
-    <row r="97" ht="42" customHeight="1" s="85">
+    <row r="97" ht="56" customHeight="1" s="85">
       <c r="A97" s="21" t="n"/>
       <c r="B97" s="22" t="inlineStr">
         <is>
@@ -4812,12 +4813,12 @@
       </c>
       <c r="C97" s="49" t="inlineStr">
         <is>
-          <t>Hit the Bike</t>
+          <t>All-Swissh Selection</t>
         </is>
       </c>
       <c r="D97" s="38" t="inlineStr">
         <is>
-          <t>Discard all Injuries. Draw 1 card. Give possession to another player</t>
+          <t>Draw 3 cards after your next make</t>
         </is>
       </c>
       <c r="E97" s="7" t="n"/>
@@ -4826,7 +4827,7 @@
       </c>
       <c r="G97" s="74" t="inlineStr">
         <is>
-          <t>This is not a pass</t>
+          <t>Arms an icon in the HUD tracking the pending draws</t>
         </is>
       </c>
       <c r="H97" s="71" t="n"/>
@@ -4842,12 +4843,12 @@
       </c>
       <c r="C98" s="49" t="inlineStr">
         <is>
-          <t>Ice Wrap</t>
+          <t>All Star Selection</t>
         </is>
       </c>
       <c r="D98" s="38" t="inlineStr">
         <is>
-          <t>Draw 1 card. Discard all Injuries. If none, draw 1 additional card</t>
+          <t>Draw 2 cards</t>
         </is>
       </c>
       <c r="E98" s="7" t="n"/>
@@ -4868,12 +4869,12 @@
       </c>
       <c r="C99" s="49" t="inlineStr">
         <is>
-          <t>Wet Spot</t>
+          <t>Hit the Bike</t>
         </is>
       </c>
       <c r="D99" s="38" t="inlineStr">
         <is>
-          <t>All Injuries in the discards and deck are displayed. Take one</t>
+          <t>Discard all Injuries. Draw 1 card. Give possession to another player</t>
         </is>
       </c>
       <c r="E99" s="7" t="n"/>
@@ -4882,14 +4883,14 @@
       </c>
       <c r="G99" s="74" t="inlineStr">
         <is>
-          <t>Deck ones are shown face down</t>
+          <t>This is not a pass</t>
         </is>
       </c>
       <c r="H99" s="71" t="n"/>
       <c r="I99" s="71" t="n"/>
       <c r="J99" s="71" t="n"/>
     </row>
-    <row r="100" ht="14" customHeight="1" s="85">
+    <row r="100" ht="28" customHeight="1" s="85">
       <c r="A100" s="21" t="n"/>
       <c r="B100" s="22" t="inlineStr">
         <is>
@@ -4898,28 +4899,24 @@
       </c>
       <c r="C100" s="49" t="inlineStr">
         <is>
-          <t>Fresh Ball</t>
+          <t>Ice Wrap</t>
         </is>
       </c>
       <c r="D100" s="38" t="inlineStr">
         <is>
-          <t>Next player does not draw at the start of their possession</t>
+          <t>Draw 1 card. Discard all Injuries. If none, draw 1 additional card</t>
         </is>
       </c>
       <c r="E100" s="7" t="n"/>
       <c r="F100" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G100" s="74" t="inlineStr">
-        <is>
-          <t>This is a bad thing in the NBA</t>
-        </is>
-      </c>
+      <c r="G100" s="74" t="n"/>
       <c r="H100" s="71" t="n"/>
       <c r="I100" s="71" t="n"/>
       <c r="J100" s="71" t="n"/>
     </row>
-    <row r="101" ht="14" customHeight="1" s="85">
+    <row r="101" ht="42" customHeight="1" s="85">
       <c r="A101" s="21" t="n"/>
       <c r="B101" s="22" t="inlineStr">
         <is>
@@ -4928,12 +4925,12 @@
       </c>
       <c r="C101" s="49" t="inlineStr">
         <is>
-          <t>Trade Deadline</t>
+          <t>Wet Spot</t>
         </is>
       </c>
       <c r="D101" s="38" t="inlineStr">
         <is>
-          <t>Declare Left or Right: every player passes their hand that way. The ball goes with it</t>
+          <t>All Injuries in the discards and deck are displayed. Take one</t>
         </is>
       </c>
       <c r="E101" s="7" t="n"/>
@@ -4942,7 +4939,7 @@
       </c>
       <c r="G101" s="74" t="inlineStr">
         <is>
-          <t>The hex travels in the declared direction too</t>
+          <t>Deck ones are shown face down</t>
         </is>
       </c>
       <c r="H101" s="71" t="n"/>
@@ -4958,19 +4955,23 @@
       </c>
       <c r="C102" s="49" t="inlineStr">
         <is>
-          <t>Floor Cleanup</t>
+          <t>Fresh Ball</t>
         </is>
       </c>
       <c r="D102" s="38" t="inlineStr">
         <is>
-          <t>All players shuffle their hands into the deck and draw the same number of cards</t>
+          <t>Next player does not draw at the start of their possession</t>
         </is>
       </c>
       <c r="E102" s="7" t="n"/>
       <c r="F102" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G102" s="74" t="n"/>
+      <c r="G102" s="74" t="inlineStr">
+        <is>
+          <t>This is a bad thing in the NBA</t>
+        </is>
+      </c>
       <c r="H102" s="71" t="n"/>
       <c r="I102" s="71" t="n"/>
       <c r="J102" s="71" t="n"/>
@@ -4984,19 +4985,23 @@
       </c>
       <c r="C103" s="49" t="inlineStr">
         <is>
-          <t>Official Timeout</t>
+          <t>Trade Deadline</t>
         </is>
       </c>
       <c r="D103" s="38" t="inlineStr">
         <is>
-          <t>At least 1 referee must be armed: discard all Injuries on all players and clear all referees. If none, all players draw 1 card</t>
+          <t>Declare Left or Right: every player passes their hand that way. The ball goes with it</t>
         </is>
       </c>
       <c r="E103" s="7" t="n"/>
       <c r="F103" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G103" s="74" t="n"/>
+      <c r="G103" s="74" t="inlineStr">
+        <is>
+          <t>The hex travels in the declared direction too</t>
+        </is>
+      </c>
       <c r="H103" s="71" t="n"/>
       <c r="I103" s="71" t="n"/>
       <c r="J103" s="71" t="n"/>
@@ -5010,12 +5015,12 @@
       </c>
       <c r="C104" s="49" t="inlineStr">
         <is>
-          <t>Team Doctor</t>
+          <t>Floor Cleanup</t>
         </is>
       </c>
       <c r="D104" s="38" t="inlineStr">
         <is>
-          <t>Discard 1 Injury from a player of choice. Draw 2 cards if not choosing yourself</t>
+          <t>All players shuffle their hands into the deck and draw the same number of cards</t>
         </is>
       </c>
       <c r="E104" s="7" t="n"/>
@@ -5036,12 +5041,12 @@
       </c>
       <c r="C105" s="49" t="inlineStr">
         <is>
-          <t>Altercation</t>
+          <t>Official Timeout</t>
         </is>
       </c>
       <c r="D105" s="38" t="inlineStr">
         <is>
-          <t>Select another player: you and that player each discard 1 card at random. Inbound the ball to a player other than that target</t>
+          <t>At least 1 referee must be armed: discard all Injuries on all players and clear all referees. If none, all players draw 1 card</t>
         </is>
       </c>
       <c r="E105" s="7" t="n"/>
@@ -5062,12 +5067,12 @@
       </c>
       <c r="C106" s="49" t="inlineStr">
         <is>
-          <t>Huge Altercation</t>
+          <t>Team Doctor</t>
         </is>
       </c>
       <c r="D106" s="38" t="inlineStr">
         <is>
-          <t>All players discard their hands. If a ref is armed, all players receive 1 TOV. Inbound the ball</t>
+          <t>Discard 1 Injury from a player of choice. Draw 2 cards if not choosing yourself</t>
         </is>
       </c>
       <c r="E106" s="7" t="n"/>
@@ -5088,12 +5093,12 @@
       </c>
       <c r="C107" s="49" t="inlineStr">
         <is>
-          <t>Home Court Advantage</t>
+          <t>Altercation</t>
         </is>
       </c>
       <c r="D107" s="38" t="inlineStr">
         <is>
-          <t>SHOT + 25%</t>
+          <t>Select another player: you and that player each discard 1 card at random. Inbound the ball to a player other than that target</t>
         </is>
       </c>
       <c r="E107" s="7" t="n"/>
@@ -5114,12 +5119,12 @@
       </c>
       <c r="C108" s="49" t="inlineStr">
         <is>
-          <t>Away Game</t>
+          <t>Huge Altercation</t>
         </is>
       </c>
       <c r="D108" s="38" t="inlineStr">
         <is>
-          <t>SHOT - 10%</t>
+          <t>All players discard their hands. If a ref is armed, all players receive 1 TOV. Inbound the ball</t>
         </is>
       </c>
       <c r="E108" s="7" t="n"/>
@@ -5131,7 +5136,7 @@
       <c r="I108" s="71" t="n"/>
       <c r="J108" s="71" t="n"/>
     </row>
-    <row r="109" ht="28" customHeight="1" s="85">
+    <row r="109" ht="14" customHeight="1" s="85">
       <c r="A109" s="21" t="n"/>
       <c r="B109" s="22" t="inlineStr">
         <is>
@@ -5140,28 +5145,24 @@
       </c>
       <c r="C109" s="49" t="inlineStr">
         <is>
-          <t>Mic'd Up</t>
+          <t>Home Court Advantage</t>
         </is>
       </c>
       <c r="D109" s="38" t="inlineStr">
         <is>
-          <t>SHOT + 10% until passed or shot</t>
+          <t>SHOT + 25%</t>
         </is>
       </c>
       <c r="E109" s="7" t="n"/>
       <c r="F109" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G109" s="74" t="inlineStr">
-        <is>
-          <t>The boost is the holder's alone and does not travel with a pass</t>
-        </is>
-      </c>
+      <c r="G109" s="74" t="n"/>
       <c r="H109" s="71" t="n"/>
       <c r="I109" s="71" t="n"/>
       <c r="J109" s="71" t="n"/>
     </row>
-    <row r="110" ht="28" customHeight="1" s="85">
+    <row r="110" ht="14" customHeight="1" s="85">
       <c r="A110" s="21" t="n"/>
       <c r="B110" s="22" t="inlineStr">
         <is>
@@ -5170,12 +5171,12 @@
       </c>
       <c r="C110" s="49" t="inlineStr">
         <is>
-          <t>In The Zone</t>
+          <t>Away Game</t>
         </is>
       </c>
       <c r="D110" s="38" t="inlineStr">
         <is>
-          <t>Draw 1 card for each 10% SHOT the ball has, rounded down. Minimum 1</t>
+          <t>SHOT - 10%</t>
         </is>
       </c>
       <c r="E110" s="7" t="n"/>
@@ -5196,128 +5197,139 @@
       </c>
       <c r="C111" s="49" t="inlineStr">
         <is>
-          <t>Role Player</t>
+          <t>Mic'd Up</t>
         </is>
       </c>
       <c r="D111" s="38" t="inlineStr">
         <is>
-          <t>All other players draw 1 card</t>
+          <t>SHOT + 10% until passed or shot</t>
         </is>
       </c>
       <c r="E111" s="7" t="n"/>
       <c r="F111" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="G111" s="74" t="n"/>
+      <c r="G111" s="74" t="inlineStr">
+        <is>
+          <t>The boost is the holder's alone and does not travel with a pass</t>
+        </is>
+      </c>
       <c r="H111" s="71" t="n"/>
       <c r="I111" s="71" t="n"/>
       <c r="J111" s="71" t="n"/>
     </row>
     <row r="112" ht="28" customHeight="1" s="85">
-      <c r="A112" s="27" t="n"/>
-      <c r="B112" s="28" t="inlineStr">
+      <c r="A112" s="21" t="n"/>
+      <c r="B112" s="22" t="inlineStr">
         <is>
           <t>Retired Game Break</t>
         </is>
       </c>
-      <c r="C112" s="62" t="inlineStr">
+      <c r="C112" s="49" t="inlineStr">
+        <is>
+          <t>In The Zone</t>
+        </is>
+      </c>
+      <c r="D112" s="38" t="inlineStr">
+        <is>
+          <t>Draw 1 card for each 10% SHOT the ball has, rounded down. Minimum 1</t>
+        </is>
+      </c>
+      <c r="E112" s="7" t="n"/>
+      <c r="F112" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G112" s="74" t="n"/>
+      <c r="H112" s="71" t="n"/>
+      <c r="I112" s="71" t="n"/>
+      <c r="J112" s="71" t="n"/>
+    </row>
+    <row r="113" ht="28" customHeight="1" s="85">
+      <c r="A113" s="21" t="n"/>
+      <c r="B113" s="22" t="inlineStr">
+        <is>
+          <t>Retired Game Break</t>
+        </is>
+      </c>
+      <c r="C113" s="49" t="inlineStr">
+        <is>
+          <t>Role Player</t>
+        </is>
+      </c>
+      <c r="D113" s="38" t="inlineStr">
+        <is>
+          <t>All other players draw 1 card</t>
+        </is>
+      </c>
+      <c r="E113" s="7" t="n"/>
+      <c r="F113" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G113" s="74" t="n"/>
+      <c r="H113" s="71" t="n"/>
+      <c r="I113" s="71" t="n"/>
+      <c r="J113" s="71" t="n"/>
+    </row>
+    <row r="114" ht="28" customHeight="1" s="85">
+      <c r="A114" s="27" t="n"/>
+      <c r="B114" s="28" t="inlineStr">
+        <is>
+          <t>Retired Game Break</t>
+        </is>
+      </c>
+      <c r="C114" s="62" t="inlineStr">
         <is>
           <t>Back-and-Forth Game</t>
         </is>
       </c>
-      <c r="D112" s="63" t="inlineStr">
+      <c r="D114" s="63" t="inlineStr">
         <is>
           <t>Discard the next 3 Game Breaks. Whoever draws one draws again</t>
         </is>
       </c>
-      <c r="E112" s="58" t="n"/>
-      <c r="F112" s="59" t="n">
+      <c r="E114" s="58" t="n"/>
+      <c r="F114" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="G112" s="79" t="n"/>
-      <c r="H112" s="76" t="n"/>
-      <c r="I112" s="76" t="n"/>
-      <c r="J112" s="76" t="n"/>
-    </row>
-    <row r="113" ht="42" customHeight="1" s="85">
-      <c r="A113" s="27" t="n"/>
-      <c r="B113" s="28" t="inlineStr">
-        <is>
-          <t>Retired Game Break</t>
-        </is>
-      </c>
-      <c r="C113" s="62" t="inlineStr">
-        <is>
-          <t>Off the Backboard</t>
-        </is>
-      </c>
-      <c r="D113" s="63" t="inlineStr">
-        <is>
-          <t>Your next missed shot rebounds itself</t>
-        </is>
-      </c>
-      <c r="E113" s="58" t="n"/>
-      <c r="F113" s="59" t="n">
-        <v>0</v>
-      </c>
-      <c r="G113" s="79" t="n"/>
-      <c r="H113" s="76" t="n"/>
-      <c r="I113" s="76" t="n"/>
-      <c r="J113" s="76" t="n"/>
-    </row>
-    <row r="114" ht="56" customHeight="1" s="85">
-      <c r="A114" s="52" t="inlineStr">
-        <is>
-          <t>Injury</t>
-        </is>
-      </c>
-      <c r="B114" s="53">
-        <f>COUNTIF($B$115:$B$148,"Injury")</f>
-        <v/>
-      </c>
-      <c r="C114" s="54" t="n"/>
-      <c r="D114" s="54" t="n"/>
-      <c r="E114" s="54" t="n"/>
-      <c r="F114" s="55" t="n"/>
-      <c r="G114" s="66" t="n"/>
-      <c r="H114" s="67" t="n"/>
-      <c r="I114" s="67" t="n"/>
-      <c r="J114" s="67" t="n"/>
-    </row>
-    <row r="115" ht="57" customHeight="1" s="85">
+      <c r="G114" s="79" t="n"/>
+      <c r="H114" s="76" t="n"/>
+      <c r="I114" s="76" t="n"/>
+      <c r="J114" s="76" t="n"/>
+    </row>
+    <row r="115" ht="42" customHeight="1" s="85">
       <c r="A115" s="27" t="n"/>
       <c r="B115" s="28" t="inlineStr">
         <is>
-          <t>Injury</t>
-        </is>
-      </c>
-      <c r="C115" s="56" t="inlineStr">
-        <is>
-          <t>Bone Bruise</t>
+          <t>Retired Game Break</t>
+        </is>
+      </c>
+      <c r="C115" s="62" t="inlineStr">
+        <is>
+          <t>Off the Backboard</t>
         </is>
       </c>
       <c r="D115" s="63" t="inlineStr">
         <is>
-          <t>Discard 1 card at the start of each turn after drawing (your choice)</t>
+          <t>Your next missed shot rebounds itself</t>
         </is>
       </c>
       <c r="E115" s="58" t="n"/>
       <c r="F115" s="59" t="n">
-        <v>5</v>
-      </c>
-      <c r="G115" s="75" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G115" s="79" t="n"/>
       <c r="H115" s="76" t="n"/>
       <c r="I115" s="76" t="n"/>
       <c r="J115" s="76" t="n"/>
     </row>
-    <row r="116" ht="20" customHeight="1" s="85">
+    <row r="116" ht="56" customHeight="1" s="85">
       <c r="A116" s="52" t="inlineStr">
         <is>
-          <t>Devastating Injury</t>
+          <t>Injury</t>
         </is>
       </c>
       <c r="B116" s="53">
-        <f>COUNTIF($B$117:$B$148,"Devastating Injury")</f>
+        <f>COUNTIF($B$117:$B$150,"Injury")</f>
         <v/>
       </c>
       <c r="C116" s="54" t="n"/>
@@ -5329,38 +5341,40 @@
       <c r="I116" s="67" t="n"/>
       <c r="J116" s="67" t="n"/>
     </row>
-    <row r="117" ht="28" customHeight="1" s="85">
+    <row r="117" ht="57" customHeight="1" s="85">
       <c r="A117" s="27" t="n"/>
       <c r="B117" s="28" t="inlineStr">
         <is>
-          <t>Devastating Injury</t>
-        </is>
-      </c>
-      <c r="C117" s="64" t="inlineStr">
-        <is>
-          <t>Torn Achilles</t>
-        </is>
-      </c>
-      <c r="D117" s="65" t="inlineStr">
-        <is>
-          <t>Hand is locked every turn except 1 card (randomly)</t>
+          <t>Injury</t>
+        </is>
+      </c>
+      <c r="C117" s="56" t="inlineStr">
+        <is>
+          <t>Bone Bruise</t>
+        </is>
+      </c>
+      <c r="D117" s="63" t="inlineStr">
+        <is>
+          <t>Discard 1 card at the start of each turn after drawing (your choice)</t>
         </is>
       </c>
       <c r="E117" s="58" t="n"/>
-      <c r="F117" s="61" t="n"/>
+      <c r="F117" s="59" t="n">
+        <v>5</v>
+      </c>
       <c r="G117" s="75" t="n"/>
       <c r="H117" s="76" t="n"/>
       <c r="I117" s="76" t="n"/>
       <c r="J117" s="76" t="n"/>
     </row>
-    <row r="118" ht="42" customHeight="1" s="85">
+    <row r="118" ht="20" customHeight="1" s="85">
       <c r="A118" s="52" t="inlineStr">
         <is>
-          <t>Intangible</t>
+          <t>Devastating Injury</t>
         </is>
       </c>
       <c r="B118" s="53">
-        <f>COUNTIF($B$119:$B$148,"Intangible")</f>
+        <f>COUNTIF($B$119:$B$150,"Devastating Injury")</f>
         <v/>
       </c>
       <c r="C118" s="54" t="n"/>
@@ -5373,72 +5387,67 @@
       <c r="J118" s="67" t="n"/>
     </row>
     <row r="119" ht="28" customHeight="1" s="85">
-      <c r="A119" s="42" t="inlineStr">
+      <c r="A119" s="27" t="n"/>
+      <c r="B119" s="28" t="inlineStr">
+        <is>
+          <t>Devastating Injury</t>
+        </is>
+      </c>
+      <c r="C119" s="64" t="inlineStr">
+        <is>
+          <t>Torn Achilles</t>
+        </is>
+      </c>
+      <c r="D119" s="65" t="inlineStr">
+        <is>
+          <t>Hand is locked every turn except 1 card (randomly)</t>
+        </is>
+      </c>
+      <c r="E119" s="58" t="n"/>
+      <c r="F119" s="61" t="n"/>
+      <c r="G119" s="75" t="n"/>
+      <c r="H119" s="76" t="n"/>
+      <c r="I119" s="76" t="n"/>
+      <c r="J119" s="76" t="n"/>
+    </row>
+    <row r="120" ht="42" customHeight="1" s="85">
+      <c r="A120" s="52" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="B120" s="53">
+        <f>COUNTIF($B$121:$B$150,"Intangible")</f>
+        <v/>
+      </c>
+      <c r="C120" s="54" t="n"/>
+      <c r="D120" s="54" t="n"/>
+      <c r="E120" s="54" t="n"/>
+      <c r="F120" s="55" t="n"/>
+      <c r="G120" s="66" t="n"/>
+      <c r="H120" s="67" t="n"/>
+      <c r="I120" s="67" t="n"/>
+      <c r="J120" s="67" t="n"/>
+    </row>
+    <row r="121" ht="28" customHeight="1" s="85">
+      <c r="A121" s="42" t="inlineStr">
         <is>
           <t>All intangibles are limited to 1</t>
         </is>
       </c>
-      <c r="B119" s="22" t="inlineStr">
+      <c r="B121" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C119" s="23" t="inlineStr">
+      <c r="C121" s="23" t="inlineStr">
         <is>
           <t>Board-Crasher</t>
         </is>
       </c>
-      <c r="D119" s="6" t="inlineStr">
+      <c r="D121" s="6" t="inlineStr">
         <is>
           <t>SHOT +10% upon Rebounding your own missed shot</t>
-        </is>
-      </c>
-      <c r="E119" s="7" t="n"/>
-      <c r="F119" s="50" t="n"/>
-      <c r="G119" s="70" t="n"/>
-      <c r="H119" s="71" t="n"/>
-      <c r="I119" s="71" t="n"/>
-      <c r="J119" s="71" t="n"/>
-    </row>
-    <row r="120" ht="28" customHeight="1" s="85">
-      <c r="A120" s="21" t="n"/>
-      <c r="B120" s="22" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C120" s="24" t="inlineStr">
-        <is>
-          <t>Catch &amp; Shoot Specialist</t>
-        </is>
-      </c>
-      <c r="D120" s="25" t="inlineStr">
-        <is>
-          <t>SHOT +25% on received passes, if shooting is your first action</t>
-        </is>
-      </c>
-      <c r="E120" s="26" t="n"/>
-      <c r="F120" s="50" t="n"/>
-      <c r="G120" s="72" t="n"/>
-      <c r="H120" s="71" t="n"/>
-      <c r="I120" s="71" t="n"/>
-      <c r="J120" s="71" t="n"/>
-    </row>
-    <row r="121" ht="56" customHeight="1" s="85">
-      <c r="A121" s="21" t="n"/>
-      <c r="B121" s="22" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C121" s="23" t="inlineStr">
-        <is>
-          <t>Clutch Gene</t>
-        </is>
-      </c>
-      <c r="D121" s="6" t="inlineStr">
-        <is>
-          <t>SHOT x2 if attempting a shot with 1 or fewer cards in hand or Shot Clock 3 or less</t>
         </is>
       </c>
       <c r="E121" s="7" t="n"/>
@@ -5448,70 +5457,70 @@
       <c r="I121" s="71" t="n"/>
       <c r="J121" s="71" t="n"/>
     </row>
-    <row r="122" ht="56" customHeight="1" s="85">
-      <c r="B122" s="0" t="inlineStr">
+    <row r="122" ht="28" customHeight="1" s="85">
+      <c r="A122" s="21" t="n"/>
+      <c r="B122" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C122" s="0" t="inlineStr">
-        <is>
-          <t>Roswell Reach</t>
-        </is>
-      </c>
-      <c r="D122" s="0" t="inlineStr">
-        <is>
-          <t>All your Rebound bids of 1 or more count as 1 higher</t>
-        </is>
-      </c>
-    </row>
-    <row r="123" ht="28" customHeight="1" s="85">
+      <c r="C122" s="24" t="inlineStr">
+        <is>
+          <t>Catch &amp; Shoot Specialist</t>
+        </is>
+      </c>
+      <c r="D122" s="25" t="inlineStr">
+        <is>
+          <t>SHOT +25% on received passes, if shooting is your first action</t>
+        </is>
+      </c>
+      <c r="E122" s="26" t="n"/>
+      <c r="F122" s="50" t="n"/>
+      <c r="G122" s="72" t="n"/>
+      <c r="H122" s="71" t="n"/>
+      <c r="I122" s="71" t="n"/>
+      <c r="J122" s="71" t="n"/>
+    </row>
+    <row r="123" ht="56" customHeight="1" s="85">
       <c r="A123" s="21" t="n"/>
       <c r="B123" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C123" s="24" t="inlineStr">
-        <is>
-          <t>Floor General</t>
-        </is>
-      </c>
-      <c r="D123" s="25" t="inlineStr">
-        <is>
-          <t>You choose all targets of all kinds — card declarations, non auto-pass targets, and the rest. Not choices about a player's own card: which effect of a multi-effect card, or whether to feed a shot an extra discard</t>
-        </is>
-      </c>
-      <c r="E123" s="26" t="n"/>
+      <c r="C123" s="23" t="inlineStr">
+        <is>
+          <t>Clutch Gene</t>
+        </is>
+      </c>
+      <c r="D123" s="6" t="inlineStr">
+        <is>
+          <t>SHOT x2 if attempting a shot with 1 or fewer cards in hand or Shot Clock 3 or less</t>
+        </is>
+      </c>
+      <c r="E123" s="7" t="n"/>
       <c r="F123" s="50" t="n"/>
-      <c r="G123" s="72" t="n"/>
+      <c r="G123" s="70" t="n"/>
       <c r="H123" s="71" t="n"/>
       <c r="I123" s="71" t="n"/>
       <c r="J123" s="71" t="n"/>
     </row>
-    <row r="124" ht="28" customHeight="1" s="85">
-      <c r="A124" s="21" t="n"/>
-      <c r="B124" s="22" t="inlineStr">
+    <row r="124" ht="56" customHeight="1" s="85">
+      <c r="B124" s="0" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C124" s="23" t="inlineStr">
-        <is>
-          <t>Southpaw Shooter</t>
-        </is>
-      </c>
-      <c r="D124" s="6" t="inlineStr">
-        <is>
-          <t>SHOT gains and losses are reversed</t>
-        </is>
-      </c>
-      <c r="E124" s="6" t="n"/>
-      <c r="F124" s="51" t="n"/>
-      <c r="G124" s="70" t="n"/>
-      <c r="H124" s="71" t="n"/>
-      <c r="I124" s="71" t="n"/>
-      <c r="J124" s="71" t="n"/>
+      <c r="C124" s="0" t="inlineStr">
+        <is>
+          <t>Roswell Reach</t>
+        </is>
+      </c>
+      <c r="D124" s="0" t="inlineStr">
+        <is>
+          <t>All your Rebound bids of 1 or more count as 1 higher</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="28" customHeight="1" s="85">
       <c r="A125" s="21" t="n"/>
@@ -5520,19 +5529,19 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C125" s="37" t="inlineStr">
-        <is>
-          <t>Freethrow Merchant</t>
-        </is>
-      </c>
-      <c r="D125" s="41" t="inlineStr">
-        <is>
-          <t>All Clamps on you grant 1 FT instead</t>
+      <c r="C125" s="24" t="inlineStr">
+        <is>
+          <t>Floor General</t>
+        </is>
+      </c>
+      <c r="D125" s="25" t="inlineStr">
+        <is>
+          <t>You choose all targets of all kinds — card declarations, non auto-pass targets, and the rest. Not choices about a player's own card: which effect of a multi-effect card, or whether to feed a shot an extra discard</t>
         </is>
       </c>
       <c r="E125" s="26" t="n"/>
       <c r="F125" s="50" t="n"/>
-      <c r="G125" s="77" t="n"/>
+      <c r="G125" s="72" t="n"/>
       <c r="H125" s="71" t="n"/>
       <c r="I125" s="71" t="n"/>
       <c r="J125" s="71" t="n"/>
@@ -5544,43 +5553,43 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C126" s="37" t="inlineStr">
-        <is>
-          <t>Generational Whistle</t>
-        </is>
-      </c>
-      <c r="D126" s="38" t="inlineStr">
-        <is>
-          <t>Take 1 additional FT</t>
-        </is>
-      </c>
-      <c r="E126" s="7" t="n"/>
-      <c r="F126" s="50" t="n"/>
+      <c r="C126" s="23" t="inlineStr">
+        <is>
+          <t>Southpaw Shooter</t>
+        </is>
+      </c>
+      <c r="D126" s="6" t="inlineStr">
+        <is>
+          <t>SHOT gains and losses are reversed</t>
+        </is>
+      </c>
+      <c r="E126" s="6" t="n"/>
+      <c r="F126" s="51" t="n"/>
       <c r="G126" s="70" t="n"/>
       <c r="H126" s="71" t="n"/>
       <c r="I126" s="71" t="n"/>
       <c r="J126" s="71" t="n"/>
     </row>
-    <row r="127" ht="14" customHeight="1" s="85">
+    <row r="127" ht="28" customHeight="1" s="85">
       <c r="A127" s="21" t="n"/>
       <c r="B127" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C127" s="24" t="inlineStr">
-        <is>
-          <t>Gravity</t>
-        </is>
-      </c>
-      <c r="D127" s="25" t="inlineStr">
-        <is>
-          <t>All Clamps automatically apply to you. +1 AST whenever another player attempts a shot</t>
+      <c r="C127" s="37" t="inlineStr">
+        <is>
+          <t>Freethrow Merchant</t>
+        </is>
+      </c>
+      <c r="D127" s="41" t="inlineStr">
+        <is>
+          <t>All Clamps on you grant 1 FT instead</t>
         </is>
       </c>
       <c r="E127" s="26" t="n"/>
       <c r="F127" s="50" t="n"/>
-      <c r="G127" s="72" t="n"/>
+      <c r="G127" s="77" t="n"/>
       <c r="H127" s="71" t="n"/>
       <c r="I127" s="71" t="n"/>
       <c r="J127" s="71" t="n"/>
@@ -5592,28 +5601,24 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C128" s="23" t="inlineStr">
-        <is>
-          <t>Great Conditioning</t>
-        </is>
-      </c>
-      <c r="D128" s="6" t="inlineStr">
-        <is>
-          <t>Immediately discard all Injuries you draw and draw a new card for each</t>
+      <c r="C128" s="37" t="inlineStr">
+        <is>
+          <t>Generational Whistle</t>
+        </is>
+      </c>
+      <c r="D128" s="38" t="inlineStr">
+        <is>
+          <t>Take 1 additional FT</t>
         </is>
       </c>
       <c r="E128" s="7" t="n"/>
       <c r="F128" s="50" t="n"/>
-      <c r="G128" s="70" t="inlineStr">
-        <is>
-          <t>Also discards any Injuries you already have (not on the card)</t>
-        </is>
-      </c>
+      <c r="G128" s="70" t="n"/>
       <c r="H128" s="71" t="n"/>
       <c r="I128" s="71" t="n"/>
       <c r="J128" s="71" t="n"/>
     </row>
-    <row r="129" ht="28" customHeight="1" s="85">
+    <row r="129" ht="14" customHeight="1" s="85">
       <c r="A129" s="21" t="n"/>
       <c r="B129" s="22" t="inlineStr">
         <is>
@@ -5622,12 +5627,12 @@
       </c>
       <c r="C129" s="24" t="inlineStr">
         <is>
-          <t>Hot Hand</t>
+          <t>Gravity</t>
         </is>
       </c>
       <c r="D129" s="25" t="inlineStr">
         <is>
-          <t>SHOT +25% if you scored last round.</t>
+          <t>All Clamps automatically apply to you. +1 AST whenever another player attempts a shot</t>
         </is>
       </c>
       <c r="E129" s="26" t="n"/>
@@ -5646,19 +5651,19 @@
       </c>
       <c r="C130" s="23" t="inlineStr">
         <is>
-          <t>Like That</t>
-        </is>
-      </c>
-      <c r="D130" s="38" t="inlineStr">
-        <is>
-          <t>Your SHOT % cannot be reduced</t>
+          <t>Great Conditioning</t>
+        </is>
+      </c>
+      <c r="D130" s="6" t="inlineStr">
+        <is>
+          <t>Immediately discard all Injuries you draw and draw a new card for each</t>
         </is>
       </c>
       <c r="E130" s="7" t="n"/>
       <c r="F130" s="50" t="n"/>
       <c r="G130" s="70" t="inlineStr">
         <is>
-          <t>Variaball effects still lower SHOT: the ball is altered, not the player (not on the card)</t>
+          <t>Also discards any Injuries you already have (not on the card)</t>
         </is>
       </c>
       <c r="H130" s="71" t="n"/>
@@ -5674,17 +5679,17 @@
       </c>
       <c r="C131" s="24" t="inlineStr">
         <is>
-          <t>Park Shark</t>
+          <t>Hot Hand</t>
         </is>
       </c>
       <c r="D131" s="25" t="inlineStr">
         <is>
-          <t>SHOT +25% on every shot. Cannot use Move or Special Move cards, or shoot threes</t>
+          <t>SHOT +25% if you scored last round.</t>
         </is>
       </c>
       <c r="E131" s="26" t="n"/>
       <c r="F131" s="50" t="n"/>
-      <c r="G131" s="73" t="n"/>
+      <c r="G131" s="72" t="n"/>
       <c r="H131" s="71" t="n"/>
       <c r="I131" s="71" t="n"/>
       <c r="J131" s="71" t="n"/>
@@ -5698,22 +5703,26 @@
       </c>
       <c r="C132" s="23" t="inlineStr">
         <is>
-          <t>Point God</t>
-        </is>
-      </c>
-      <c r="D132" s="6" t="inlineStr">
-        <is>
-          <t>Draw 1 card following each of your passes</t>
+          <t>Like That</t>
+        </is>
+      </c>
+      <c r="D132" s="38" t="inlineStr">
+        <is>
+          <t>Your SHOT % cannot be reduced</t>
         </is>
       </c>
       <c r="E132" s="7" t="n"/>
       <c r="F132" s="50" t="n"/>
-      <c r="G132" s="70" t="n"/>
+      <c r="G132" s="70" t="inlineStr">
+        <is>
+          <t>Variaball effects still lower SHOT: the ball is altered, not the player (not on the card)</t>
+        </is>
+      </c>
       <c r="H132" s="71" t="n"/>
       <c r="I132" s="71" t="n"/>
       <c r="J132" s="71" t="n"/>
     </row>
-    <row r="133" ht="56" customHeight="1" s="85">
+    <row r="133" ht="28" customHeight="1" s="85">
       <c r="A133" s="21" t="n"/>
       <c r="B133" s="22" t="inlineStr">
         <is>
@@ -5722,26 +5731,22 @@
       </c>
       <c r="C133" s="24" t="inlineStr">
         <is>
-          <t>Shot Creator</t>
+          <t>Park Shark</t>
         </is>
       </c>
       <c r="D133" s="25" t="inlineStr">
         <is>
-          <t>Draw 1 additional card after every draw effect</t>
+          <t>SHOT +25% on every shot. Cannot use Move or Special Move cards, or shoot threes</t>
         </is>
       </c>
       <c r="E133" s="26" t="n"/>
       <c r="F133" s="50" t="n"/>
-      <c r="G133" s="73" t="inlineStr">
-        <is>
-          <t>Triggers once per act of drawing: a Draw 2 still gives only 1 extra</t>
-        </is>
-      </c>
+      <c r="G133" s="73" t="n"/>
       <c r="H133" s="71" t="n"/>
       <c r="I133" s="71" t="n"/>
       <c r="J133" s="71" t="n"/>
     </row>
-    <row r="134" ht="56" customHeight="1" s="85">
+    <row r="134" ht="28" customHeight="1" s="85">
       <c r="A134" s="21" t="n"/>
       <c r="B134" s="22" t="inlineStr">
         <is>
@@ -5750,21 +5755,17 @@
       </c>
       <c r="C134" s="23" t="inlineStr">
         <is>
-          <t>Sixth Man</t>
+          <t>Point God</t>
         </is>
       </c>
       <c r="D134" s="6" t="inlineStr">
         <is>
-          <t>SHOT = 60% on any six: cards in hand, Shot Clock, shot of the round, or score</t>
+          <t>Draw 1 card following each of your passes</t>
         </is>
       </c>
       <c r="E134" s="7" t="n"/>
       <c r="F134" s="50" t="n"/>
-      <c r="G134" s="70" t="inlineStr">
-        <is>
-          <t>A second SHOOT (60%) button beside Shoot, shown only on a six. Ignore it when SHOT is already higher</t>
-        </is>
-      </c>
+      <c r="G134" s="70" t="n"/>
       <c r="H134" s="71" t="n"/>
       <c r="I134" s="71" t="n"/>
       <c r="J134" s="71" t="n"/>
@@ -5778,17 +5779,21 @@
       </c>
       <c r="C135" s="24" t="inlineStr">
         <is>
-          <t>Sniper</t>
+          <t>Shot Creator</t>
         </is>
       </c>
       <c r="D135" s="25" t="inlineStr">
         <is>
-          <t>SHOT +25% on all Three-Point Line Shots</t>
+          <t>Draw 1 additional card after every draw effect</t>
         </is>
       </c>
       <c r="E135" s="26" t="n"/>
       <c r="F135" s="50" t="n"/>
-      <c r="G135" s="72" t="n"/>
+      <c r="G135" s="73" t="inlineStr">
+        <is>
+          <t>Triggers once per act of drawing: a Draw 2 still gives only 1 extra</t>
+        </is>
+      </c>
       <c r="H135" s="71" t="n"/>
       <c r="I135" s="71" t="n"/>
       <c r="J135" s="71" t="n"/>
@@ -5802,17 +5807,21 @@
       </c>
       <c r="C136" s="23" t="inlineStr">
         <is>
-          <t>Splash Cousin</t>
+          <t>Sixth Man</t>
         </is>
       </c>
       <c r="D136" s="6" t="inlineStr">
         <is>
-          <t>All Three-Point Line Shots: SHOT = 100%</t>
+          <t>SHOT = 60% on any six: cards in hand, Shot Clock, shot of the round, or score</t>
         </is>
       </c>
       <c r="E136" s="7" t="n"/>
       <c r="F136" s="50" t="n"/>
-      <c r="G136" s="70" t="n"/>
+      <c r="G136" s="70" t="inlineStr">
+        <is>
+          <t>A second SHOOT (60%) button beside Shoot, shown only on a six. Ignore it when SHOT is already higher</t>
+        </is>
+      </c>
       <c r="H136" s="71" t="n"/>
       <c r="I136" s="71" t="n"/>
       <c r="J136" s="71" t="n"/>
@@ -5826,12 +5835,12 @@
       </c>
       <c r="C137" s="24" t="inlineStr">
         <is>
-          <t>Competitive</t>
+          <t>Sniper</t>
         </is>
       </c>
       <c r="D137" s="25" t="inlineStr">
         <is>
-          <t>All Clamps on you have no effect on SHOT %</t>
+          <t>SHOT +25% on all Three-Point Line Shots</t>
         </is>
       </c>
       <c r="E137" s="26" t="n"/>
@@ -5841,7 +5850,7 @@
       <c r="I137" s="71" t="n"/>
       <c r="J137" s="71" t="n"/>
     </row>
-    <row r="138" ht="126" customHeight="1" s="85">
+    <row r="138" ht="56" customHeight="1" s="85">
       <c r="A138" s="21" t="n"/>
       <c r="B138" s="22" t="inlineStr">
         <is>
@@ -5850,26 +5859,22 @@
       </c>
       <c r="C138" s="23" t="inlineStr">
         <is>
-          <t>Lethal Shooter</t>
-        </is>
-      </c>
-      <c r="D138" s="38" t="inlineStr">
-        <is>
-          <t>SHOT = 100% on next shot attempt after rebounding your own miss.</t>
+          <t>Splash Cousin</t>
+        </is>
+      </c>
+      <c r="D138" s="6" t="inlineStr">
+        <is>
+          <t>All Three-Point Line Shots: SHOT = 100%</t>
         </is>
       </c>
       <c r="E138" s="7" t="n"/>
       <c r="F138" s="50" t="n"/>
-      <c r="G138" s="70" t="inlineStr">
-        <is>
-          <t>Special text: “I understand it now”</t>
-        </is>
-      </c>
+      <c r="G138" s="70" t="n"/>
       <c r="H138" s="71" t="n"/>
       <c r="I138" s="71" t="n"/>
       <c r="J138" s="71" t="n"/>
     </row>
-    <row r="139" ht="70" customHeight="1" s="85">
+    <row r="139" ht="56" customHeight="1" s="85">
       <c r="A139" s="21" t="n"/>
       <c r="B139" s="22" t="inlineStr">
         <is>
@@ -5878,22 +5883,22 @@
       </c>
       <c r="C139" s="24" t="inlineStr">
         <is>
-          <t>Ball Pounder</t>
+          <t>Competitive</t>
         </is>
       </c>
       <c r="D139" s="25" t="inlineStr">
         <is>
-          <t>Every Dribble draws 1 card but gives SHOT -10% and Shot Clock - 01</t>
+          <t>All Clamps on you have no effect on SHOT %</t>
         </is>
       </c>
       <c r="E139" s="26" t="n"/>
       <c r="F139" s="50" t="n"/>
-      <c r="G139" s="73" t="n"/>
+      <c r="G139" s="72" t="n"/>
       <c r="H139" s="71" t="n"/>
       <c r="I139" s="71" t="n"/>
       <c r="J139" s="71" t="n"/>
     </row>
-    <row r="140" ht="56" customHeight="1" s="85">
+    <row r="140" ht="126" customHeight="1" s="85">
       <c r="A140" s="21" t="n"/>
       <c r="B140" s="22" t="inlineStr">
         <is>
@@ -5902,50 +5907,50 @@
       </c>
       <c r="C140" s="23" t="inlineStr">
         <is>
-          <t>Dirty Player</t>
+          <t>Lethal Shooter</t>
         </is>
       </c>
       <c r="D140" s="38" t="inlineStr">
         <is>
-          <t>When sending Clamps, the clamped player discards 1 for each of your Clamps if they have any Injuries. Discard 1 whenever a Whistle triggers</t>
+          <t>SHOT = 100% on next shot attempt after rebounding your own miss.</t>
         </is>
       </c>
       <c r="E140" s="7" t="n"/>
       <c r="F140" s="50" t="n"/>
-      <c r="G140" s="70" t="n"/>
+      <c r="G140" s="70" t="inlineStr">
+        <is>
+          <t>Special text: “I understand it now”</t>
+        </is>
+      </c>
       <c r="H140" s="71" t="n"/>
       <c r="I140" s="71" t="n"/>
       <c r="J140" s="71" t="n"/>
     </row>
-    <row r="141" s="85">
+    <row r="141" ht="70" customHeight="1" s="85">
       <c r="A141" s="21" t="n"/>
       <c r="B141" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C141" s="23" t="inlineStr">
-        <is>
-          <t>Free Agent</t>
-        </is>
-      </c>
-      <c r="D141" s="38" t="inlineStr">
-        <is>
-          <t>Discard your hand. Play a card at random from a player of your choosing (they keep it)</t>
-        </is>
-      </c>
-      <c r="E141" s="7" t="n"/>
+      <c r="C141" s="24" t="inlineStr">
+        <is>
+          <t>Ball Pounder</t>
+        </is>
+      </c>
+      <c r="D141" s="25" t="inlineStr">
+        <is>
+          <t>Every Dribble draws 1 card but gives SHOT -10% and Shot Clock - 01</t>
+        </is>
+      </c>
+      <c r="E141" s="26" t="n"/>
       <c r="F141" s="50" t="n"/>
-      <c r="G141" s="70" t="inlineStr">
-        <is>
-          <t>Low priority to bring back. The discard waits for the draw chain to finish. Target is shuffled first and is affected by Floor General. Your own draws are kept. All-0 rebounds are yours; otherwise you cannot bid  [OUT OF THE DECK — the borrow button throws the answer away; back when it routes through Move.borrow]</t>
-        </is>
-      </c>
+      <c r="G141" s="73" t="n"/>
       <c r="H141" s="71" t="n"/>
       <c r="I141" s="71" t="n"/>
       <c r="J141" s="71" t="n"/>
     </row>
-    <row r="142" s="85">
+    <row r="142" ht="56" customHeight="1" s="85">
       <c r="A142" s="21" t="n"/>
       <c r="B142" s="22" t="inlineStr">
         <is>
@@ -5954,12 +5959,12 @@
       </c>
       <c r="C142" s="23" t="inlineStr">
         <is>
-          <t>Franchise Player</t>
+          <t>Dirty Player</t>
         </is>
       </c>
       <c r="D142" s="38" t="inlineStr">
         <is>
-          <t>When passing, choose 1 of the new player's Intangibles or a card in their hand for them to discard</t>
+          <t>When sending Clamps, the clamped player discards 1 for each of your Clamps if they have any Injuries. Discard 1 whenever a Whistle triggers</t>
         </is>
       </c>
       <c r="E142" s="7" t="n"/>
@@ -5978,19 +5983,19 @@
       </c>
       <c r="C143" s="23" t="inlineStr">
         <is>
-          <t>Fundamentalist</t>
+          <t>Free Agent</t>
         </is>
       </c>
       <c r="D143" s="38" t="inlineStr">
         <is>
-          <t>No Special Moves. Each Move once a turn. Swings, Skip Pass and Dribble are never spent. Discards the current ball</t>
+          <t>Discard your hand. Play a card at random from a player of your choosing (they keep it)</t>
         </is>
       </c>
       <c r="E143" s="7" t="n"/>
       <c r="F143" s="50" t="n"/>
       <c r="G143" s="70" t="inlineStr">
         <is>
-          <t>The ball is discarded once, on activation</t>
+          <t>Low priority to bring back. The discard waits for the draw chain to finish. Target is shuffled first and is affected by Floor General. Your own draws are kept. All-0 rebounds are yours; otherwise you cannot bid  [OUT OF THE DECK — the borrow button throws the answer away; back when it routes through Move.borrow]</t>
         </is>
       </c>
       <c r="H143" s="71" t="n"/>
@@ -6006,18 +6011,16 @@
       </c>
       <c r="C144" s="23" t="inlineStr">
         <is>
-          <t>Moves At Own Pace</t>
+          <t>Franchise Player</t>
         </is>
       </c>
       <c r="D144" s="38" t="inlineStr">
         <is>
-          <t>Cannot be called for Traveling or Shot Clock violations</t>
+          <t>When passing, choose 1 of the new player's Intangibles or a card in their hand for them to discard</t>
         </is>
       </c>
       <c r="E144" s="7" t="n"/>
-      <c r="F144" s="50" t="n">
-        <v>1</v>
-      </c>
+      <c r="F144" s="50" t="n"/>
       <c r="G144" s="70" t="n"/>
       <c r="H144" s="71" t="n"/>
       <c r="I144" s="71" t="n"/>
@@ -6032,74 +6035,74 @@
       </c>
       <c r="C145" s="23" t="inlineStr">
         <is>
-          <t>Equalizer</t>
+          <t>Fundamentalist</t>
         </is>
       </c>
       <c r="D145" s="38" t="inlineStr">
         <is>
-          <t>Any 'SHOT =' shot you take becomes 100%</t>
+          <t>No Special Moves. Each Move once a turn. Swings, Skip Pass and Dribble are never spent. Discards the current ball</t>
         </is>
       </c>
       <c r="E145" s="7" t="n"/>
       <c r="F145" s="50" t="n"/>
-      <c r="G145" s="70" t="n"/>
+      <c r="G145" s="70" t="inlineStr">
+        <is>
+          <t>The ball is discarded once, on activation</t>
+        </is>
+      </c>
       <c r="H145" s="71" t="n"/>
       <c r="I145" s="71" t="n"/>
       <c r="J145" s="71" t="n"/>
     </row>
     <row r="146" s="85">
-      <c r="A146" s="27" t="n"/>
-      <c r="B146" s="28" t="inlineStr">
+      <c r="A146" s="21" t="n"/>
+      <c r="B146" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C146" s="56" t="inlineStr">
-        <is>
-          <t>Varsitile</t>
-        </is>
-      </c>
-      <c r="D146" s="63" t="inlineStr">
-        <is>
-          <t>You can play more than 1 Varena and Variaball per turn. Once per possession, you can exchange the Varena and/or ball for one in the Discards</t>
-        </is>
-      </c>
-      <c r="E146" s="58" t="n"/>
-      <c r="F146" s="61" t="n"/>
-      <c r="G146" s="75" t="inlineStr">
-        <is>
-          <t>One use can exchange both. Not in the deck until Variaballs are</t>
-        </is>
-      </c>
-      <c r="H146" s="76" t="n"/>
-      <c r="I146" s="76" t="n"/>
-      <c r="J146" s="76" t="n"/>
+      <c r="C146" s="23" t="inlineStr">
+        <is>
+          <t>Moves At Own Pace</t>
+        </is>
+      </c>
+      <c r="D146" s="38" t="inlineStr">
+        <is>
+          <t>Cannot be called for Traveling or Shot Clock violations</t>
+        </is>
+      </c>
+      <c r="E146" s="7" t="n"/>
+      <c r="F146" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G146" s="70" t="n"/>
+      <c r="H146" s="71" t="n"/>
+      <c r="I146" s="71" t="n"/>
+      <c r="J146" s="71" t="n"/>
     </row>
     <row r="147" s="85">
-      <c r="A147" s="27" t="n"/>
-      <c r="B147" s="28" t="inlineStr">
+      <c r="A147" s="21" t="n"/>
+      <c r="B147" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C147" s="56" t="inlineStr">
-        <is>
-          <t>Brawl Handler</t>
-        </is>
-      </c>
-      <c r="D147" s="63" t="inlineStr">
-        <is>
-          <t>Remove all your Clamps when you change the ball</t>
-        </is>
-      </c>
-      <c r="E147" s="58" t="n"/>
-      <c r="F147" s="61" t="n"/>
-      <c r="G147" s="75" t="inlineStr">
-        <is>
-          <t>Not in the deck until Variaballs are</t>
-        </is>
-      </c>
-      <c r="H147" s="76" t="n"/>
+      <c r="C147" s="23" t="inlineStr">
+        <is>
+          <t>Equalizer</t>
+        </is>
+      </c>
+      <c r="D147" s="38" t="inlineStr">
+        <is>
+          <t>Any 'SHOT =' shot you take becomes 100%</t>
+        </is>
+      </c>
+      <c r="E147" s="7" t="n"/>
+      <c r="F147" s="50" t="n"/>
+      <c r="G147" s="70" t="n"/>
+      <c r="H147" s="71" t="n"/>
+      <c r="I147" s="71" t="n"/>
+      <c r="J147" s="71" t="n"/>
     </row>
     <row r="148" s="85">
       <c r="A148" s="27" t="n"/>
@@ -6110,202 +6113,1582 @@
       </c>
       <c r="C148" s="56" t="inlineStr">
         <is>
-          <t>Baller</t>
+          <t>Varsitile</t>
         </is>
       </c>
       <c r="D148" s="63" t="inlineStr">
         <is>
-          <t>Draw 1 card each time you change the ball</t>
+          <t>You can play more than 1 Varena and Variaball per turn. Once per possession, you can exchange the Varena and/or ball for one in the Discards</t>
         </is>
       </c>
       <c r="E148" s="58" t="n"/>
       <c r="F148" s="61" t="n"/>
       <c r="G148" s="75" t="inlineStr">
         <is>
-          <t>Not in the deck until Variaballs are</t>
+          <t>One use can exchange both</t>
         </is>
       </c>
       <c r="H148" s="76" t="n"/>
-    </row>
-    <row r="149" ht="42" customHeight="1" s="85">
-      <c r="A149" s="52" t="inlineStr">
-        <is>
-          <t>Varena</t>
-        </is>
-      </c>
-      <c r="B149" s="53">
-        <f>COUNTIF($B$150:$B$150,"Varena")</f>
-        <v/>
-      </c>
-      <c r="C149" s="54" t="n"/>
-      <c r="D149" s="54" t="n"/>
-      <c r="E149" s="54" t="n"/>
-      <c r="F149" s="55" t="n"/>
-      <c r="G149" s="66" t="n"/>
-      <c r="H149" s="67" t="n"/>
-      <c r="I149" s="67" t="n"/>
-      <c r="J149" s="67" t="n"/>
+      <c r="I148" s="76" t="n"/>
+      <c r="J148" s="76" t="n"/>
+    </row>
+    <row r="149" s="85">
+      <c r="A149" s="27" t="n"/>
+      <c r="B149" s="28" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C149" s="56" t="inlineStr">
+        <is>
+          <t>Brawl Handler</t>
+        </is>
+      </c>
+      <c r="D149" s="63" t="inlineStr">
+        <is>
+          <t>Remove all your Clamps when you change the ball</t>
+        </is>
+      </c>
+      <c r="E149" s="58" t="n"/>
+      <c r="F149" s="61" t="n"/>
+      <c r="G149" s="75" t="n"/>
+      <c r="H149" s="76" t="n"/>
     </row>
     <row r="150" s="85">
       <c r="A150" s="27" t="n"/>
       <c r="B150" s="28" t="inlineStr">
         <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C150" s="56" t="inlineStr">
+        <is>
+          <t>Baller</t>
+        </is>
+      </c>
+      <c r="D150" s="63" t="inlineStr">
+        <is>
+          <t>Draw 1 card each time you change the ball</t>
+        </is>
+      </c>
+      <c r="E150" s="58" t="n"/>
+      <c r="F150" s="61" t="n"/>
+      <c r="G150" s="75" t="n"/>
+      <c r="H150" s="76" t="n"/>
+    </row>
+    <row r="151" ht="42" customHeight="1" s="85">
+      <c r="A151" s="52" t="inlineStr">
+        <is>
           <t>Varena</t>
         </is>
       </c>
-      <c r="C150" s="56" t="inlineStr">
+      <c r="B151" s="53">
+        <f>COUNTIF($B$152:$B$180,"Varena")</f>
+        <v/>
+      </c>
+      <c r="C151" s="54" t="n"/>
+      <c r="D151" s="54" t="n"/>
+      <c r="E151" s="54" t="n"/>
+      <c r="F151" s="55" t="n"/>
+      <c r="G151" s="66" t="n"/>
+      <c r="H151" s="67" t="n"/>
+      <c r="I151" s="67" t="n"/>
+      <c r="J151" s="67" t="n"/>
+    </row>
+    <row r="152" s="85">
+      <c r="A152" s="27" t="n"/>
+      <c r="B152" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C152" s="56" t="inlineStr">
         <is>
           <t>Cardwood</t>
         </is>
       </c>
-      <c r="D150" s="63" t="inlineStr">
+      <c r="D152" s="63" t="inlineStr">
         <is>
           <t>Changes the court back to basic</t>
         </is>
       </c>
-      <c r="E150" s="58" t="n"/>
-      <c r="F150" s="61" t="n">
+      <c r="E152" s="58" t="n"/>
+      <c r="F152" s="61" t="n">
         <v>5</v>
       </c>
-      <c r="G150" s="75" t="inlineStr">
+      <c r="G152" s="75" t="inlineStr">
         <is>
           <t>Also the floor every game opens on, before anybody plays a Varena over it</t>
         </is>
       </c>
-      <c r="H150" s="76" t="n"/>
-      <c r="I150" s="76" t="n"/>
-      <c r="J150" s="76" t="n"/>
+      <c r="H152" s="76" t="n"/>
+      <c r="I152" s="76" t="n"/>
+      <c r="J152" s="76" t="n"/>
+    </row>
+    <row r="153" s="85">
+      <c r="A153" s="27" t="n"/>
+      <c r="B153" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C153" s="56" t="inlineStr">
+        <is>
+          <t>Prime Parquet</t>
+        </is>
+      </c>
+      <c r="D153" s="63" t="inlineStr">
+        <is>
+          <t>SHOT +10% on every shot</t>
+        </is>
+      </c>
+      <c r="E153" s="58" t="n"/>
+      <c r="F153" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G153" s="75" t="n"/>
+      <c r="H153" s="76" t="n"/>
+      <c r="I153" s="76" t="n"/>
+      <c r="J153" s="76" t="n"/>
+    </row>
+    <row r="154" s="85">
+      <c r="A154" s="27" t="n"/>
+      <c r="B154" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C154" s="56" t="inlineStr">
+        <is>
+          <t>Lacktop</t>
+        </is>
+      </c>
+      <c r="D154" s="63" t="inlineStr">
+        <is>
+          <t>SHOT -10% on every shot</t>
+        </is>
+      </c>
+      <c r="E154" s="58" t="n"/>
+      <c r="F154" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G154" s="75" t="n"/>
+      <c r="H154" s="76" t="n"/>
+      <c r="I154" s="76" t="n"/>
+      <c r="J154" s="76" t="n"/>
+    </row>
+    <row r="155" s="85">
+      <c r="A155" s="27" t="n"/>
+      <c r="B155" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C155" s="56" t="inlineStr">
+        <is>
+          <t>Smacktop</t>
+        </is>
+      </c>
+      <c r="D155" s="63" t="inlineStr">
+        <is>
+          <t>Clear All Whistles. Whistles Cannot Be Played. All Clamps are enhanced</t>
+        </is>
+      </c>
+      <c r="E155" s="58" t="n"/>
+      <c r="F155" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G155" s="75" t="inlineStr">
+        <is>
+          <t>Enhanced: +10% more reduction, one more card discarded, one more card locked</t>
+        </is>
+      </c>
+      <c r="H155" s="76" t="n"/>
+      <c r="I155" s="76" t="n"/>
+      <c r="J155" s="76" t="n"/>
+    </row>
+    <row r="156" s="85">
+      <c r="A156" s="27" t="n"/>
+      <c r="B156" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C156" s="56" t="inlineStr">
+        <is>
+          <t>Boarder Court</t>
+        </is>
+      </c>
+      <c r="D156" s="63" t="inlineStr">
+        <is>
+          <t>Off your own miss, your Rebound bid counts as one card more</t>
+        </is>
+      </c>
+      <c r="E156" s="58" t="n"/>
+      <c r="F156" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G156" s="75" t="inlineStr">
+        <is>
+          <t>Still needs a bid of at least one</t>
+        </is>
+      </c>
+      <c r="H156" s="76" t="n"/>
+      <c r="I156" s="76" t="n"/>
+      <c r="J156" s="76" t="n"/>
+    </row>
+    <row r="157" s="85">
+      <c r="A157" s="27" t="n"/>
+      <c r="B157" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C157" s="56" t="inlineStr">
+        <is>
+          <t>Dim Dome</t>
+        </is>
+      </c>
+      <c r="D157" s="63" t="inlineStr">
+        <is>
+          <t>SHOT is hidden from everyone but the ball holder</t>
+        </is>
+      </c>
+      <c r="E157" s="58" t="n"/>
+      <c r="F157" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G157" s="75" t="inlineStr">
+        <is>
+          <t>On a table, flip the % device face down</t>
+        </is>
+      </c>
+      <c r="H157" s="76" t="n"/>
+      <c r="I157" s="76" t="n"/>
+      <c r="J157" s="76" t="n"/>
+    </row>
+    <row r="158" s="85">
+      <c r="A158" s="27" t="n"/>
+      <c r="B158" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C158" s="56" t="inlineStr">
+        <is>
+          <t>Tri-hard Tiling</t>
+        </is>
+      </c>
+      <c r="D158" s="63" t="inlineStr">
+        <is>
+          <t>Hand limit 3</t>
+        </is>
+      </c>
+      <c r="E158" s="58" t="n"/>
+      <c r="F158" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G158" s="75" t="inlineStr">
+        <is>
+          <t>Hands over 3 are cut to 3 when it lands (owner picks). A draw into a hand of 3 is discarded</t>
+        </is>
+      </c>
+      <c r="H158" s="76" t="n"/>
+      <c r="I158" s="76" t="n"/>
+      <c r="J158" s="76" t="n"/>
+    </row>
+    <row r="159" s="85">
+      <c r="A159" s="27" t="n"/>
+      <c r="B159" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C159" s="56" t="inlineStr">
+        <is>
+          <t>Policeum</t>
+        </is>
+      </c>
+      <c r="D159" s="63" t="inlineStr">
+        <is>
+          <t>Referees do not leave once triggered</t>
+        </is>
+      </c>
+      <c r="E159" s="58" t="n"/>
+      <c r="F159" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G159" s="75" t="inlineStr">
+        <is>
+          <t>A called referee stays until the floor changes. The 3-ref cap bounds it</t>
+        </is>
+      </c>
+      <c r="H159" s="76" t="n"/>
+      <c r="I159" s="76" t="n"/>
+      <c r="J159" s="76" t="n"/>
+    </row>
+    <row r="160" s="85">
+      <c r="A160" s="27" t="n"/>
+      <c r="B160" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C160" s="56" t="inlineStr">
+        <is>
+          <t>Kiddie Court</t>
+        </is>
+      </c>
+      <c r="D160" s="63" t="inlineStr">
+        <is>
+          <t>No threes. Every make counts 2. SHOT +10%, and dunks +10% more</t>
+        </is>
+      </c>
+      <c r="E160" s="58" t="n"/>
+      <c r="F160" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G160" s="75" t="inlineStr">
+        <is>
+          <t>Shuts off every card that makes a three (Kick-Out)</t>
+        </is>
+      </c>
+      <c r="H160" s="76" t="n"/>
+      <c r="I160" s="76" t="n"/>
+      <c r="J160" s="76" t="n"/>
+    </row>
+    <row r="161" s="85">
+      <c r="A161" s="27" t="n"/>
+      <c r="B161" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C161" s="56" t="inlineStr">
+        <is>
+          <t>Recharging Resin</t>
+        </is>
+      </c>
+      <c r="D161" s="63" t="inlineStr">
+        <is>
+          <t>Everyone refills to a hand of 5 at the start of their possession</t>
+        </is>
+      </c>
+      <c r="E161" s="58" t="n"/>
+      <c r="F161" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G161" s="75" t="inlineStr">
+        <is>
+          <t>After the draw for turn</t>
+        </is>
+      </c>
+      <c r="H161" s="76" t="n"/>
+      <c r="I161" s="76" t="n"/>
+      <c r="J161" s="76" t="n"/>
+    </row>
+    <row r="162" s="85">
+      <c r="A162" s="27" t="n"/>
+      <c r="B162" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C162" s="56" t="inlineStr">
+        <is>
+          <t>Contact Court</t>
+        </is>
+      </c>
+      <c r="D162" s="63" t="inlineStr">
+        <is>
+          <t>Being clamped: take 1 FT. The Clamp still lands</t>
+        </is>
+      </c>
+      <c r="E162" s="58" t="n"/>
+      <c r="F162" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G162" s="75" t="inlineStr">
+        <is>
+          <t>One free throw however many Clamps land</t>
+        </is>
+      </c>
+      <c r="H162" s="76" t="n"/>
+      <c r="I162" s="76" t="n"/>
+      <c r="J162" s="76" t="n"/>
+    </row>
+    <row r="163" s="85">
+      <c r="A163" s="27" t="n"/>
+      <c r="B163" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C163" s="56" t="inlineStr">
+        <is>
+          <t>MVPiquia</t>
+        </is>
+      </c>
+      <c r="D163" s="63" t="inlineStr">
+        <is>
+          <t>The highest scorer refills to 5 at the start of their possession</t>
+        </is>
+      </c>
+      <c r="E163" s="58" t="n"/>
+      <c r="F163" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G163" s="75" t="inlineStr">
+        <is>
+          <t>A tie for the lead counts</t>
+        </is>
+      </c>
+      <c r="H163" s="76" t="n"/>
+      <c r="I163" s="76" t="n"/>
+      <c r="J163" s="76" t="n"/>
+    </row>
+    <row r="164" s="85">
+      <c r="A164" s="27" t="n"/>
+      <c r="B164" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C164" s="56" t="inlineStr">
+        <is>
+          <t>Polypaypylene</t>
+        </is>
+      </c>
+      <c r="D164" s="63" t="inlineStr">
+        <is>
+          <t>Making a shot: Draw 3</t>
+        </is>
+      </c>
+      <c r="E164" s="58" t="n"/>
+      <c r="F164" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G164" s="75" t="n"/>
+      <c r="H164" s="76" t="n"/>
+      <c r="I164" s="76" t="n"/>
+      <c r="J164" s="76" t="n"/>
+    </row>
+    <row r="165" s="85">
+      <c r="A165" s="27" t="n"/>
+      <c r="B165" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C165" s="56" t="inlineStr">
+        <is>
+          <t>Recoverena</t>
+        </is>
+      </c>
+      <c r="D165" s="63" t="inlineStr">
+        <is>
+          <t>Discard all Injuries. A new Injury is discarded, and that player draws 1</t>
+        </is>
+      </c>
+      <c r="E165" s="58" t="n"/>
+      <c r="F165" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G165" s="75" t="inlineStr">
+        <is>
+          <t>Every player's Injuries go when it lands</t>
+        </is>
+      </c>
+      <c r="H165" s="76" t="n"/>
+      <c r="I165" s="76" t="n"/>
+      <c r="J165" s="76" t="n"/>
+    </row>
+    <row r="166" s="85">
+      <c r="A166" s="27" t="n"/>
+      <c r="B166" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C166" s="56" t="inlineStr">
+        <is>
+          <t>Carousel Court</t>
+        </is>
+      </c>
+      <c r="D166" s="63" t="inlineStr">
+        <is>
+          <t>Declare left or right. Every possession, hands move one seat that way</t>
+        </is>
+      </c>
+      <c r="E166" s="58" t="n"/>
+      <c r="F166" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G166" s="75" t="inlineStr">
+        <is>
+          <t>Declared by whoever plays it</t>
+        </is>
+      </c>
+      <c r="H166" s="76" t="n"/>
+      <c r="I166" s="76" t="n"/>
+      <c r="J166" s="76" t="n"/>
+    </row>
+    <row r="167" s="85">
+      <c r="A167" s="27" t="n"/>
+      <c r="B167" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C167" s="56" t="inlineStr">
+        <is>
+          <t>Traderous Tarmac</t>
+        </is>
+      </c>
+      <c r="D167" s="63" t="inlineStr">
+        <is>
+          <t>During your turn, hand off any number of the Clamps on you to other players</t>
+        </is>
+      </c>
+      <c r="E167" s="58" t="n"/>
+      <c r="F167" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G167" s="75" t="inlineStr">
+        <is>
+          <t>The player assigns each Clamp: all to one player, one each, or any split</t>
+        </is>
+      </c>
+      <c r="H167" s="76" t="n"/>
+      <c r="I167" s="76" t="n"/>
+      <c r="J167" s="76" t="n"/>
+    </row>
+    <row r="168" s="85">
+      <c r="A168" s="27" t="n"/>
+      <c r="B168" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C168" s="56" t="inlineStr">
+        <is>
+          <t>Clearcoat Court</t>
+        </is>
+      </c>
+      <c r="D168" s="63" t="inlineStr">
+        <is>
+          <t>Every possession: clear all referees, Clamps, Injuries and Intangibles</t>
+        </is>
+      </c>
+      <c r="E168" s="58" t="n"/>
+      <c r="F168" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G168" s="75" t="inlineStr">
+        <is>
+          <t>Standing Clamps only; Clamps still in the air land after the wipe</t>
+        </is>
+      </c>
+      <c r="H168" s="76" t="n"/>
+      <c r="I168" s="76" t="n"/>
+      <c r="J168" s="76" t="n"/>
+    </row>
+    <row r="169" s="85">
+      <c r="A169" s="27" t="n"/>
+      <c r="B169" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C169" s="56" t="inlineStr">
+        <is>
+          <t>Malice Palace</t>
+        </is>
+      </c>
+      <c r="D169" s="63" t="inlineStr">
+        <is>
+          <t>At the start of your possession, before your draw: discard your hand</t>
+        </is>
+      </c>
+      <c r="E169" s="58" t="n"/>
+      <c r="F169" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G169" s="75" t="n"/>
+      <c r="H169" s="76" t="n"/>
+      <c r="I169" s="76" t="n"/>
+      <c r="J169" s="76" t="n"/>
+    </row>
+    <row r="170" s="85">
+      <c r="A170" s="27" t="n"/>
+      <c r="B170" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C170" s="56" t="inlineStr">
+        <is>
+          <t>Turnstile Tile</t>
+        </is>
+      </c>
+      <c r="D170" s="63" t="inlineStr">
+        <is>
+          <t>SHOT +25% and -25%, alternating each possession</t>
+        </is>
+      </c>
+      <c r="E170" s="58" t="n"/>
+      <c r="F170" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G170" s="75" t="inlineStr">
+        <is>
+          <t>+25% the possession it lands</t>
+        </is>
+      </c>
+      <c r="H170" s="76" t="n"/>
+      <c r="I170" s="76" t="n"/>
+      <c r="J170" s="76" t="n"/>
+    </row>
+    <row r="171" s="85">
+      <c r="A171" s="27" t="n"/>
+      <c r="B171" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C171" s="56" t="inlineStr">
+        <is>
+          <t>Roleplayer Polymer</t>
+        </is>
+      </c>
+      <c r="D171" s="63" t="inlineStr">
+        <is>
+          <t>Every possession, everyone but the turn player draws 1</t>
+        </is>
+      </c>
+      <c r="E171" s="58" t="n"/>
+      <c r="F171" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="G171" s="75" t="n"/>
+      <c r="H171" s="76" t="n"/>
+      <c r="I171" s="76" t="n"/>
+      <c r="J171" s="76" t="n"/>
+    </row>
+    <row r="172" s="85">
+      <c r="A172" s="27" t="n"/>
+      <c r="B172" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C172" s="56" t="inlineStr">
+        <is>
+          <t>Variaball Vinyl</t>
+        </is>
+      </c>
+      <c r="D172" s="63" t="inlineStr">
+        <is>
+          <t>The draw for turn goes to a random player each possession</t>
+        </is>
+      </c>
+      <c r="E172" s="58" t="n"/>
+      <c r="F172" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G172" s="75" t="inlineStr">
+        <is>
+          <t>Can be the turn player</t>
+        </is>
+      </c>
+      <c r="H172" s="76" t="n"/>
+      <c r="I172" s="76" t="n"/>
+      <c r="J172" s="76" t="n"/>
+    </row>
+    <row r="173" s="85">
+      <c r="A173" s="27" t="n"/>
+      <c r="B173" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C173" s="56" t="inlineStr">
+        <is>
+          <t>Gravi-Gym</t>
+        </is>
+      </c>
+      <c r="D173" s="63" t="inlineStr">
+        <is>
+          <t>SHOT -10%. No dunks</t>
+        </is>
+      </c>
+      <c r="E173" s="58" t="n"/>
+      <c r="F173" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G173" s="75" t="inlineStr">
+        <is>
+          <t>Cards that dunk cannot be played</t>
+        </is>
+      </c>
+      <c r="H173" s="76" t="n"/>
+      <c r="I173" s="76" t="n"/>
+      <c r="J173" s="76" t="n"/>
+    </row>
+    <row r="174" s="85">
+      <c r="A174" s="27" t="n"/>
+      <c r="B174" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C174" s="56" t="inlineStr">
+        <is>
+          <t>Vintage Varnish</t>
+        </is>
+      </c>
+      <c r="D174" s="63" t="inlineStr">
+        <is>
+          <t>Shot Clock 14. No threes. No Variaballs. 1 Intangible per player</t>
+        </is>
+      </c>
+      <c r="E174" s="58" t="n"/>
+      <c r="F174" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G174" s="75" t="inlineStr">
+        <is>
+          <t>Discards the ball in play when it lands</t>
+        </is>
+      </c>
+      <c r="H174" s="76" t="n"/>
+      <c r="I174" s="76" t="n"/>
+      <c r="J174" s="76" t="n"/>
+    </row>
+    <row r="175" s="85">
+      <c r="A175" s="27" t="n"/>
+      <c r="B175" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C175" s="56" t="inlineStr">
+        <is>
+          <t>S.O.S — Sell-Out Stadium</t>
+        </is>
+      </c>
+      <c r="D175" s="63" t="inlineStr">
+        <is>
+          <t>A three can be shot as a two at double SHOT</t>
+        </is>
+      </c>
+      <c r="E175" s="58" t="n"/>
+      <c r="F175" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G175" s="75" t="inlineStr">
+        <is>
+          <t>Keeps every other printed effect</t>
+        </is>
+      </c>
+      <c r="H175" s="76" t="n"/>
+      <c r="I175" s="76" t="n"/>
+      <c r="J175" s="76" t="n"/>
+    </row>
+    <row r="176" s="85">
+      <c r="A176" s="27" t="n"/>
+      <c r="B176" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C176" s="56" t="inlineStr">
+        <is>
+          <t>Grayvstone</t>
+        </is>
+      </c>
+      <c r="D176" s="63" t="inlineStr">
+        <is>
+          <t>Each possession, the ball becomes the last Variaball in the discards</t>
+        </is>
+      </c>
+      <c r="E176" s="58" t="n"/>
+      <c r="F176" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G176" s="75" t="inlineStr">
+        <is>
+          <t>With none there, nothing happens</t>
+        </is>
+      </c>
+      <c r="H176" s="76" t="n"/>
+      <c r="I176" s="76" t="n"/>
+      <c r="J176" s="76" t="n"/>
+    </row>
+    <row r="177" s="85">
+      <c r="A177" s="27" t="n"/>
+      <c r="B177" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C177" s="56" t="inlineStr">
+        <is>
+          <t>Con-crete</t>
+        </is>
+      </c>
+      <c r="D177" s="63" t="inlineStr">
+        <is>
+          <t>Move cards: SHOT -10%</t>
+        </is>
+      </c>
+      <c r="E177" s="58" t="n"/>
+      <c r="F177" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G177" s="75" t="n"/>
+      <c r="H177" s="76" t="n"/>
+      <c r="I177" s="76" t="n"/>
+      <c r="J177" s="76" t="n"/>
+    </row>
+    <row r="178" s="85">
+      <c r="A178" s="27" t="n"/>
+      <c r="B178" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C178" s="56" t="inlineStr">
+        <is>
+          <t>Spazzphalt</t>
+        </is>
+      </c>
+      <c r="D178" s="63" t="inlineStr">
+        <is>
+          <t>SHOT = a random 0–100%, in steps of 5</t>
+        </is>
+      </c>
+      <c r="E178" s="58" t="n"/>
+      <c r="F178" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G178" s="75" t="inlineStr">
+        <is>
+          <t>Rolled fresh for every shot</t>
+        </is>
+      </c>
+      <c r="H178" s="76" t="n"/>
+      <c r="I178" s="76" t="n"/>
+      <c r="J178" s="76" t="n"/>
+    </row>
+    <row r="179" s="85">
+      <c r="A179" s="27" t="n"/>
+      <c r="B179" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C179" s="56" t="inlineStr">
+        <is>
+          <t>Frostbite Finish</t>
+        </is>
+      </c>
+      <c r="D179" s="63" t="inlineStr">
+        <is>
+          <t>Playing a Move costs discarding 1 other card</t>
+        </is>
+      </c>
+      <c r="E179" s="58" t="n"/>
+      <c r="F179" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="G179" s="75" t="inlineStr">
+        <is>
+          <t>The owner picks the card. A Move that is your whole hand can't be played</t>
+        </is>
+      </c>
+      <c r="H179" s="76" t="n"/>
+      <c r="I179" s="76" t="n"/>
+      <c r="J179" s="76" t="n"/>
+    </row>
+    <row r="180" s="85">
+      <c r="A180" s="27" t="n"/>
+      <c r="B180" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C180" s="56" t="inlineStr">
+        <is>
+          <t>Tick-Tock Tile</t>
+        </is>
+      </c>
+      <c r="D180" s="63" t="inlineStr">
+        <is>
+          <t>Playing any card also ticks the Shot Clock</t>
+        </is>
+      </c>
+      <c r="E180" s="58" t="n"/>
+      <c r="F180" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G180" s="75" t="inlineStr">
+        <is>
+          <t>The tick is paid after the card resolves, so a shot at 01 still goes up</t>
+        </is>
+      </c>
+      <c r="H180" s="76" t="n"/>
+      <c r="I180" s="76" t="n"/>
+      <c r="J180" s="76" t="n"/>
+    </row>
+    <row r="181" ht="42" customHeight="1" s="85">
+      <c r="A181" s="52" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="B181" s="53">
+        <f>COUNTIF($B$182:$B$197,"Variaball")</f>
+        <v/>
+      </c>
+      <c r="C181" s="54" t="n"/>
+      <c r="D181" s="54" t="n"/>
+      <c r="E181" s="54" t="n"/>
+      <c r="F181" s="55" t="n"/>
+      <c r="G181" s="66" t="n"/>
+      <c r="H181" s="67" t="n"/>
+      <c r="I181" s="67" t="n"/>
+      <c r="J181" s="67" t="n"/>
+    </row>
+    <row r="182" s="85">
+      <c r="A182" s="27" t="n"/>
+      <c r="B182" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C182" s="56" t="inlineStr">
+        <is>
+          <t>Med Ball</t>
+        </is>
+      </c>
+      <c r="D182" s="63" t="inlineStr">
+        <is>
+          <t>SHOT cannot exceed 50%</t>
+        </is>
+      </c>
+      <c r="E182" s="58" t="n"/>
+      <c r="F182" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="G182" s="75" t="inlineStr">
+        <is>
+          <t>An Intangible's or a Varena's SHOT = is not held to it</t>
+        </is>
+      </c>
+      <c r="H182" s="76" t="n"/>
+      <c r="I182" s="76" t="n"/>
+      <c r="J182" s="76" t="n"/>
+    </row>
+    <row r="183" s="85">
+      <c r="A183" s="27" t="n"/>
+      <c r="B183" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C183" s="56" t="inlineStr">
+        <is>
+          <t>Dishcount Ball</t>
+        </is>
+      </c>
+      <c r="D183" s="63" t="inlineStr">
+        <is>
+          <t>Discard one fewer for card costs and Clamps</t>
+        </is>
+      </c>
+      <c r="E183" s="58" t="n"/>
+      <c r="F183" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="G183" s="75" t="inlineStr">
+        <is>
+          <t>Counts: Clamps, Pound Dribble, Frostbite Finish, Stepback, Turnaround Three</t>
+        </is>
+      </c>
+      <c r="H183" s="76" t="n"/>
+      <c r="I183" s="76" t="n"/>
+      <c r="J183" s="76" t="n"/>
+    </row>
+    <row r="184" s="85">
+      <c r="A184" s="27" t="n"/>
+      <c r="B184" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C184" s="56" t="inlineStr">
+        <is>
+          <t>Blight Ball</t>
+        </is>
+      </c>
+      <c r="D184" s="63" t="inlineStr">
+        <is>
+          <t>Injuries travel with the ball, and new ones join the pile. Discarding the ball takes the pile with it</t>
+        </is>
+      </c>
+      <c r="E184" s="58" t="n"/>
+      <c r="F184" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G184" s="75" t="inlineStr">
+        <is>
+          <t>Moves on any change of hands</t>
+        </is>
+      </c>
+      <c r="H184" s="76" t="n"/>
+      <c r="I184" s="76" t="n"/>
+      <c r="J184" s="76" t="n"/>
+    </row>
+    <row r="185" s="85">
+      <c r="A185" s="27" t="n"/>
+      <c r="B185" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C185" s="56" t="inlineStr">
+        <is>
+          <t>Bench Ball</t>
+        </is>
+      </c>
+      <c r="D185" s="63" t="inlineStr">
+        <is>
+          <t>Receiving it by Pass: no draw, no turn. You inbound</t>
+        </is>
+      </c>
+      <c r="E185" s="58" t="n"/>
+      <c r="F185" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G185" s="75" t="n"/>
+      <c r="H185" s="76" t="n"/>
+      <c r="I185" s="76" t="n"/>
+      <c r="J185" s="76" t="n"/>
+    </row>
+    <row r="186" s="85">
+      <c r="A186" s="27" t="n"/>
+      <c r="B186" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C186" s="56" t="inlineStr">
+        <is>
+          <t>Dishtracting Ball</t>
+        </is>
+      </c>
+      <c r="D186" s="63" t="inlineStr">
+        <is>
+          <t>Receiving it: discard 1, after the draw for turn</t>
+        </is>
+      </c>
+      <c r="E186" s="58" t="n"/>
+      <c r="F186" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="G186" s="75" t="inlineStr">
+        <is>
+          <t>Any change of hands</t>
+        </is>
+      </c>
+      <c r="H186" s="76" t="n"/>
+      <c r="I186" s="76" t="n"/>
+      <c r="J186" s="76" t="n"/>
+    </row>
+    <row r="187" s="85">
+      <c r="A187" s="27" t="n"/>
+      <c r="B187" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C187" s="56" t="inlineStr">
+        <is>
+          <t>Hand Ball</t>
+        </is>
+      </c>
+      <c r="D187" s="63" t="inlineStr">
+        <is>
+          <t>A Pass swaps hands: yours goes with the ball, theirs comes back</t>
+        </is>
+      </c>
+      <c r="E187" s="58" t="n"/>
+      <c r="F187" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G187" s="75" t="n"/>
+      <c r="H187" s="76" t="n"/>
+      <c r="I187" s="76" t="n"/>
+      <c r="J187" s="76" t="n"/>
+    </row>
+    <row r="188" s="85">
+      <c r="A188" s="27" t="n"/>
+      <c r="B188" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C188" s="56" t="inlineStr">
+        <is>
+          <t>Foot Ball</t>
+        </is>
+      </c>
+      <c r="D188" s="63" t="inlineStr">
+        <is>
+          <t>Moves and Passes are not spent. They lock until your possession ends</t>
+        </is>
+      </c>
+      <c r="E188" s="58" t="n"/>
+      <c r="F188" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G188" s="75" t="n"/>
+      <c r="H188" s="76" t="n"/>
+      <c r="I188" s="76" t="n"/>
+      <c r="J188" s="76" t="n"/>
+    </row>
+    <row r="189" s="85">
+      <c r="A189" s="27" t="n"/>
+      <c r="B189" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C189" s="56" t="inlineStr">
+        <is>
+          <t>Recharge Rock</t>
+        </is>
+      </c>
+      <c r="D189" s="63" t="inlineStr">
+        <is>
+          <t>Double your draw for turn</t>
+        </is>
+      </c>
+      <c r="E189" s="58" t="n"/>
+      <c r="F189" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="G189" s="75" t="n"/>
+      <c r="H189" s="76" t="n"/>
+      <c r="I189" s="76" t="n"/>
+      <c r="J189" s="76" t="n"/>
+    </row>
+    <row r="190" s="85">
+      <c r="A190" s="27" t="n"/>
+      <c r="B190" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C190" s="56" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="D190" s="63" t="inlineStr">
+        <is>
+          <t>A random Variaball from the discards goes into play. Then discard this</t>
+        </is>
+      </c>
+      <c r="E190" s="58" t="n"/>
+      <c r="F190" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G190" s="75" t="inlineStr">
+        <is>
+          <t>From the deck if the discards have none; never the ball already in play</t>
+        </is>
+      </c>
+      <c r="H190" s="76" t="n"/>
+      <c r="I190" s="76" t="n"/>
+      <c r="J190" s="76" t="n"/>
+    </row>
+    <row r="191" s="85">
+      <c r="A191" s="27" t="n"/>
+      <c r="B191" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C191" s="56" t="inlineStr">
+        <is>
+          <t>Shufflebag Ball</t>
+        </is>
+      </c>
+      <c r="D191" s="63" t="inlineStr">
+        <is>
+          <t>Every possession, the turn player shuffles their hand into the deck and draws the same number, then draws for turn</t>
+        </is>
+      </c>
+      <c r="E191" s="58" t="n"/>
+      <c r="F191" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G191" s="75" t="n"/>
+      <c r="H191" s="76" t="n"/>
+      <c r="I191" s="76" t="n"/>
+      <c r="J191" s="76" t="n"/>
+    </row>
+    <row r="192" s="85">
+      <c r="A192" s="27" t="n"/>
+      <c r="B192" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C192" s="56" t="inlineStr">
+        <is>
+          <t>Bag'n Ball</t>
+        </is>
+      </c>
+      <c r="D192" s="63" t="inlineStr">
+        <is>
+          <t>Draw 1 on activation. SHOT = 10% for each card in your hand</t>
+        </is>
+      </c>
+      <c r="E192" s="58" t="n"/>
+      <c r="F192" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G192" s="75" t="n"/>
+      <c r="H192" s="76" t="n"/>
+      <c r="I192" s="76" t="n"/>
+      <c r="J192" s="76" t="n"/>
+    </row>
+    <row r="193" s="85">
+      <c r="A193" s="27" t="n"/>
+      <c r="B193" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C193" s="56" t="inlineStr">
+        <is>
+          <t>Blaze Ball</t>
+        </is>
+      </c>
+      <c r="D193" s="63" t="inlineStr">
+        <is>
+          <t>SHOT +10% each time it's passed</t>
+        </is>
+      </c>
+      <c r="E193" s="58" t="n"/>
+      <c r="F193" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="G193" s="75" t="inlineStr">
+        <is>
+          <t>Ignores every other pass modifier</t>
+        </is>
+      </c>
+      <c r="H193" s="76" t="n"/>
+      <c r="I193" s="76" t="n"/>
+      <c r="J193" s="76" t="n"/>
+    </row>
+    <row r="194" s="85">
+      <c r="A194" s="27" t="n"/>
+      <c r="B194" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C194" s="56" t="inlineStr">
+        <is>
+          <t>Snow Ball It</t>
+        </is>
+      </c>
+      <c r="D194" s="63" t="inlineStr">
+        <is>
+          <t>SHOT -10% each time it's passed</t>
+        </is>
+      </c>
+      <c r="E194" s="58" t="n"/>
+      <c r="F194" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="G194" s="75" t="inlineStr">
+        <is>
+          <t>Ignores every other pass modifier</t>
+        </is>
+      </c>
+      <c r="H194" s="76" t="n"/>
+      <c r="I194" s="76" t="n"/>
+      <c r="J194" s="76" t="n"/>
+    </row>
+    <row r="195" s="85">
+      <c r="A195" s="27" t="n"/>
+      <c r="B195" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C195" s="56" t="inlineStr">
+        <is>
+          <t>Brick Ball</t>
+        </is>
+      </c>
+      <c r="D195" s="63" t="inlineStr">
+        <is>
+          <t>SHOT = 25%</t>
+        </is>
+      </c>
+      <c r="E195" s="58" t="n"/>
+      <c r="F195" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="G195" s="75" t="n"/>
+      <c r="H195" s="76" t="n"/>
+      <c r="I195" s="76" t="n"/>
+      <c r="J195" s="76" t="n"/>
+    </row>
+    <row r="196" s="85">
+      <c r="A196" s="27" t="n"/>
+      <c r="B196" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C196" s="56" t="inlineStr">
+        <is>
+          <t>Monster Ball</t>
+        </is>
+      </c>
+      <c r="D196" s="63" t="inlineStr">
+        <is>
+          <t>Intangibles are absorbed into the ball. When it's discarded, players rebound for them one at a time</t>
+        </is>
+      </c>
+      <c r="E196" s="58" t="n"/>
+      <c r="F196" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G196" s="75" t="inlineStr">
+        <is>
+          <t>Swallows every Intangible already out and every one drawn while it's in play</t>
+        </is>
+      </c>
+      <c r="H196" s="76" t="n"/>
+      <c r="I196" s="76" t="n"/>
+      <c r="J196" s="76" t="n"/>
+    </row>
+    <row r="197" s="85">
+      <c r="A197" s="27" t="n"/>
+      <c r="B197" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C197" s="56" t="inlineStr">
+        <is>
+          <t>Brand New Ball</t>
+        </is>
+      </c>
+      <c r="D197" s="63" t="inlineStr">
+        <is>
+          <t>25% chance a shot attempt is a turnover instead</t>
+        </is>
+      </c>
+      <c r="E197" s="58" t="n"/>
+      <c r="F197" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G197" s="75" t="inlineStr">
+        <is>
+          <t>The round ends</t>
+        </is>
+      </c>
+      <c r="H197" s="76" t="n"/>
+      <c r="I197" s="76" t="n"/>
+      <c r="J197" s="76" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="128">
+  <mergeCells count="175">
     <mergeCell ref="G55:J55"/>
     <mergeCell ref="G4:J4"/>
-    <mergeCell ref="G135:J135"/>
+    <mergeCell ref="G182:J182"/>
+    <mergeCell ref="G188:J188"/>
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
-    <mergeCell ref="G119:J119"/>
-    <mergeCell ref="G150:J150"/>
+    <mergeCell ref="G135:J135"/>
     <mergeCell ref="G32:J32"/>
     <mergeCell ref="G46:J46"/>
+    <mergeCell ref="G119:J119"/>
     <mergeCell ref="G40:J40"/>
     <mergeCell ref="G111:J111"/>
+    <mergeCell ref="G159:J159"/>
+    <mergeCell ref="G193:J193"/>
     <mergeCell ref="G72:J72"/>
     <mergeCell ref="G81:J81"/>
+    <mergeCell ref="G161:J161"/>
+    <mergeCell ref="G5:J5"/>
     <mergeCell ref="G71:J71"/>
     <mergeCell ref="G136:J136"/>
+    <mergeCell ref="G194:J194"/>
+    <mergeCell ref="G181:J181"/>
     <mergeCell ref="G8:J8"/>
+    <mergeCell ref="G160:J160"/>
     <mergeCell ref="G82:J82"/>
+    <mergeCell ref="G174:J174"/>
+    <mergeCell ref="G156:J156"/>
     <mergeCell ref="G57:J57"/>
+    <mergeCell ref="G10:J10"/>
+    <mergeCell ref="G137:J137"/>
+    <mergeCell ref="G66:J66"/>
     <mergeCell ref="G128:J128"/>
-    <mergeCell ref="G10:J10"/>
-    <mergeCell ref="G66:J66"/>
     <mergeCell ref="G18:J18"/>
     <mergeCell ref="G53:J53"/>
+    <mergeCell ref="G171:J171"/>
+    <mergeCell ref="G189:J189"/>
     <mergeCell ref="G121:J121"/>
     <mergeCell ref="G34:J34"/>
     <mergeCell ref="G74:J74"/>
     <mergeCell ref="G68:J68"/>
-    <mergeCell ref="G139:J139"/>
     <mergeCell ref="G108:J108"/>
     <mergeCell ref="G58:J58"/>
     <mergeCell ref="G114:J114"/>
     <mergeCell ref="G123:J123"/>
+    <mergeCell ref="G163:J163"/>
     <mergeCell ref="G110:J110"/>
+    <mergeCell ref="G168:J168"/>
+    <mergeCell ref="G113:J113"/>
     <mergeCell ref="G20:J20"/>
-    <mergeCell ref="G113:J113"/>
     <mergeCell ref="G91:J91"/>
+    <mergeCell ref="G100:J100"/>
     <mergeCell ref="G85:J85"/>
-    <mergeCell ref="G100:J100"/>
+    <mergeCell ref="G183:J183"/>
+    <mergeCell ref="G165:J165"/>
     <mergeCell ref="G75:J75"/>
     <mergeCell ref="G44:J44"/>
     <mergeCell ref="G22:J22"/>
     <mergeCell ref="G84:J84"/>
     <mergeCell ref="G102:J102"/>
+    <mergeCell ref="G158:J158"/>
+    <mergeCell ref="G185:J185"/>
     <mergeCell ref="G12:J12"/>
     <mergeCell ref="G77:J77"/>
+    <mergeCell ref="G86:J86"/>
     <mergeCell ref="G21:J21"/>
-    <mergeCell ref="G86:J86"/>
+    <mergeCell ref="G178:J178"/>
     <mergeCell ref="G67:J67"/>
     <mergeCell ref="G61:J61"/>
     <mergeCell ref="G70:J70"/>
     <mergeCell ref="G48:J48"/>
     <mergeCell ref="G23:J23"/>
+    <mergeCell ref="G176:J176"/>
+    <mergeCell ref="G97:J97"/>
     <mergeCell ref="G125:J125"/>
     <mergeCell ref="G38:J38"/>
     <mergeCell ref="G7:J7"/>
     <mergeCell ref="G112:J112"/>
+    <mergeCell ref="G184:J184"/>
+    <mergeCell ref="G45:J45"/>
+    <mergeCell ref="G191:J191"/>
     <mergeCell ref="G62:J62"/>
+    <mergeCell ref="G175:J175"/>
     <mergeCell ref="G127:J127"/>
+    <mergeCell ref="G162:J162"/>
     <mergeCell ref="G49:J49"/>
     <mergeCell ref="G24:J24"/>
+    <mergeCell ref="G177:J177"/>
+    <mergeCell ref="G195:J195"/>
     <mergeCell ref="G33:J33"/>
     <mergeCell ref="G104:J104"/>
     <mergeCell ref="G65:J65"/>
     <mergeCell ref="G88:J88"/>
     <mergeCell ref="G26:J26"/>
+    <mergeCell ref="G154:J154"/>
+    <mergeCell ref="G197:J197"/>
     <mergeCell ref="G35:J35"/>
     <mergeCell ref="G129:J129"/>
+    <mergeCell ref="G138:J138"/>
     <mergeCell ref="G16:J16"/>
+    <mergeCell ref="G90:J90"/>
     <mergeCell ref="G76:J76"/>
     <mergeCell ref="G25:J25"/>
-    <mergeCell ref="G99:J99"/>
     <mergeCell ref="G60:J60"/>
+    <mergeCell ref="G131:J131"/>
     <mergeCell ref="G9:J9"/>
-    <mergeCell ref="G131:J131"/>
-    <mergeCell ref="G140:J140"/>
+    <mergeCell ref="G124:J124"/>
+    <mergeCell ref="G130:J130"/>
+    <mergeCell ref="G115:J115"/>
     <mergeCell ref="G59:J59"/>
-    <mergeCell ref="G115:J115"/>
-    <mergeCell ref="G130:J130"/>
     <mergeCell ref="G11:J11"/>
     <mergeCell ref="G117:J117"/>
+    <mergeCell ref="G169:J169"/>
+    <mergeCell ref="G179:J179"/>
+    <mergeCell ref="G132:J132"/>
+    <mergeCell ref="G39:J39"/>
+    <mergeCell ref="G122:J122"/>
     <mergeCell ref="G126:J126"/>
-    <mergeCell ref="G39:J39"/>
-    <mergeCell ref="G132:J132"/>
-    <mergeCell ref="G122:J122"/>
+    <mergeCell ref="G166:J166"/>
+    <mergeCell ref="G116:J116"/>
     <mergeCell ref="G101:J101"/>
-    <mergeCell ref="G116:J116"/>
     <mergeCell ref="G103:J103"/>
     <mergeCell ref="G37:J37"/>
+    <mergeCell ref="G186:J186"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G13:J13"/>
     <mergeCell ref="G78:J78"/>
     <mergeCell ref="G118:J118"/>
+    <mergeCell ref="G152:J152"/>
     <mergeCell ref="G87:J87"/>
+    <mergeCell ref="G133:J133"/>
+    <mergeCell ref="G167:J167"/>
     <mergeCell ref="G15:J15"/>
+    <mergeCell ref="G142:J142"/>
     <mergeCell ref="G80:J80"/>
-    <mergeCell ref="G95:J95"/>
     <mergeCell ref="G89:J89"/>
     <mergeCell ref="G64:J64"/>
     <mergeCell ref="G79:J79"/>
     <mergeCell ref="G73:J73"/>
     <mergeCell ref="G51:J51"/>
+    <mergeCell ref="G192:J192"/>
+    <mergeCell ref="G153:J153"/>
     <mergeCell ref="G54:J54"/>
     <mergeCell ref="G63:J63"/>
+    <mergeCell ref="G134:J134"/>
     <mergeCell ref="G41:J41"/>
-    <mergeCell ref="G134:J134"/>
+    <mergeCell ref="G106:J106"/>
     <mergeCell ref="G50:J50"/>
-    <mergeCell ref="G106:J106"/>
+    <mergeCell ref="G164:J164"/>
+    <mergeCell ref="G173:J173"/>
     <mergeCell ref="G56:J56"/>
+    <mergeCell ref="G105:J105"/>
     <mergeCell ref="G14:J14"/>
-    <mergeCell ref="G105:J105"/>
     <mergeCell ref="G43:J43"/>
     <mergeCell ref="G52:J52"/>
+    <mergeCell ref="G155:J155"/>
+    <mergeCell ref="G120:J120"/>
+    <mergeCell ref="G107:J107"/>
     <mergeCell ref="G27:J27"/>
-    <mergeCell ref="G120:J120"/>
-    <mergeCell ref="G98:J98"/>
     <mergeCell ref="G36:J36"/>
     <mergeCell ref="G42:J42"/>
-    <mergeCell ref="G107:J107"/>
     <mergeCell ref="G17:J17"/>
+    <mergeCell ref="G170:J170"/>
+    <mergeCell ref="G157:J157"/>
+    <mergeCell ref="G141:J141"/>
     <mergeCell ref="G19:J19"/>
+    <mergeCell ref="G172:J172"/>
+    <mergeCell ref="G93:J93"/>
     <mergeCell ref="G28:J28"/>
     <mergeCell ref="G6:J6"/>
+    <mergeCell ref="G190:J190"/>
+    <mergeCell ref="G187:J187"/>
     <mergeCell ref="G69:J69"/>
     <mergeCell ref="G83:J83"/>
-    <mergeCell ref="G124:J124"/>
-    <mergeCell ref="G5:J5"/>
-    <mergeCell ref="G133:J133"/>
-    <mergeCell ref="G45:J45"/>
+    <mergeCell ref="G196:J196"/>
+    <mergeCell ref="G180:J180"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
Hand Ball and Foot Ball art; icon tool reads Affinity's export scale; sheet catches up
- Hand Ball and Foot Ball use their drawings on the Variaball plate.
- The icon tool reads the DPI wrapper Affinity sometimes puts round a drawing instead of a
  hand-kept table: a ball, or a subject against its plate, takes the shared box at its own
  export scale. Snow Ball It now frames at the exact 300 DPI factor.
- Sheet: Alley-Oop is a Retired Pass at 0 with the combo note, Lob notes the Alley-Oop, and
  "Shoot the ball" is out of all 16 bonus cells.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -2339,7 +2339,11 @@
       <c r="F8" s="33" t="n">
         <v>5</v>
       </c>
-      <c r="G8" s="72" t="n"/>
+      <c r="G8" s="72" t="inlineStr">
+        <is>
+          <t>Dunked as the receiver's first action, it's the Alley-Oop combo: SHOT +10%. A receiver holding a dunk card is asked "Dunk It?"</t>
+        </is>
+      </c>
       <c r="H8" s="71" t="n"/>
       <c r="I8" s="71" t="n"/>
       <c r="J8" s="71" t="n"/>
@@ -2508,7 +2512,7 @@
       <c r="A15" s="21" t="n"/>
       <c r="B15" s="22" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Retired Pass</t>
         </is>
       </c>
       <c r="C15" s="24" t="inlineStr">
@@ -2527,9 +2531,13 @@
         </is>
       </c>
       <c r="F15" s="36" t="n">
-        <v>5</v>
-      </c>
-      <c r="G15" s="72" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G15" s="72" t="inlineStr">
+        <is>
+          <t>Retired: now the Alley-Oop combo — a Lob, then any dunk card as the first action, SHOT +10%</t>
+        </is>
+      </c>
       <c r="H15" s="71" t="n"/>
       <c r="I15" s="71" t="n"/>
       <c r="J15" s="71" t="n"/>
@@ -3142,11 +3150,7 @@
 Tails: SHOT -10%</t>
         </is>
       </c>
-      <c r="E36" s="25" t="inlineStr">
-        <is>
-          <t>Shoot the ball</t>
-        </is>
-      </c>
+      <c r="E36" s="25" t="n"/>
       <c r="F36" s="36" t="n">
         <v>5</v>
       </c>
@@ -3172,11 +3176,7 @@
           <t>SHOT = 100%</t>
         </is>
       </c>
-      <c r="E37" s="6" t="inlineStr">
-        <is>
-          <t>Shoot the ball</t>
-        </is>
-      </c>
+      <c r="E37" s="6" t="n"/>
       <c r="F37" s="32" t="n">
         <v>5</v>
       </c>
@@ -3206,11 +3206,7 @@
           <t>[SHOT + 30% at 01 Shot Clock, +20% at 02, +10% at 03, +0% at 04, -10% at 05, etc.]</t>
         </is>
       </c>
-      <c r="E38" s="25" t="inlineStr">
-        <is>
-          <t>Shoot the ball</t>
-        </is>
-      </c>
+      <c r="E38" s="25" t="n"/>
       <c r="F38" s="36" t="n">
         <v>5</v>
       </c>
@@ -3236,11 +3232,7 @@
           <t>SHOT -10%. Draw 1 card</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
-        <is>
-          <t>Shoot the ball.</t>
-        </is>
-      </c>
+      <c r="E39" s="6" t="n"/>
       <c r="F39" s="32" t="n">
         <v>10</v>
       </c>
@@ -3266,11 +3258,7 @@
           <t>SHOT -20%</t>
         </is>
       </c>
-      <c r="E40" s="25" t="inlineStr">
-        <is>
-          <t>Shoot the ball</t>
-        </is>
-      </c>
+      <c r="E40" s="25" t="n"/>
       <c r="F40" s="36" t="n">
         <v>3</v>
       </c>
@@ -3296,11 +3284,7 @@
           <t>SHOT -30%</t>
         </is>
       </c>
-      <c r="E41" s="6" t="inlineStr">
-        <is>
-          <t>Shoot the ball</t>
-        </is>
-      </c>
+      <c r="E41" s="6" t="n"/>
       <c r="F41" s="32" t="n">
         <v>3</v>
       </c>
@@ -3326,11 +3310,7 @@
           <t>SHOT = 25%</t>
         </is>
       </c>
-      <c r="E42" s="25" t="inlineStr">
-        <is>
-          <t>Shoot the ball</t>
-        </is>
-      </c>
+      <c r="E42" s="25" t="n"/>
       <c r="F42" s="36" t="n">
         <v>3</v>
       </c>
@@ -3358,7 +3338,7 @@
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>Shoot the ball. After a missed shot: SHOT = 100%</t>
+          <t>After a missed shot: SHOT = 100%</t>
         </is>
       </c>
       <c r="F43" s="32" t="n">
@@ -3388,7 +3368,7 @@
       </c>
       <c r="E44" s="41" t="inlineStr">
         <is>
-          <t>Shoot the ball. Shot is unaffected by Clamps</t>
+          <t>Shot is unaffected by Clamps</t>
         </is>
       </c>
       <c r="F44" s="36" t="n">
@@ -3418,7 +3398,7 @@
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>Shoot the ball. SHOT = 100% if SHOT &gt;= 75%</t>
+          <t>SHOT = 100% if SHOT &gt;= 75%</t>
         </is>
       </c>
       <c r="F45" s="32" t="n">
@@ -3446,11 +3426,7 @@
           <t>Discard any number of cards. SHOT +10% for each</t>
         </is>
       </c>
-      <c r="E46" s="25" t="inlineStr">
-        <is>
-          <t>Shoot the ball</t>
-        </is>
-      </c>
+      <c r="E46" s="25" t="n"/>
       <c r="F46" s="36" t="n">
         <v>1</v>
       </c>
@@ -3508,7 +3484,7 @@
       </c>
       <c r="E48" s="58" t="inlineStr">
         <is>
-          <t>Shoot the ball. Selected players receive +1 AST on a make</t>
+          <t>Selected players receive +1 AST on a make</t>
         </is>
       </c>
       <c r="F48" s="59" t="n">
@@ -3541,7 +3517,7 @@
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
-          <t>Shoot the ball. Another +10% straight off your own board</t>
+          <t>Another +10% straight off your own board</t>
         </is>
       </c>
       <c r="F49" s="0" t="n">
@@ -3569,11 +3545,7 @@
           <t>Clean look only — no Clamps on you and nothing has gone off this possession. SHOT +30%</t>
         </is>
       </c>
-      <c r="E50" s="0" t="inlineStr">
-        <is>
-          <t>Shoot the ball</t>
-        </is>
-      </c>
+      <c r="E50" s="0" t="n"/>
       <c r="F50" s="0" t="n">
         <v>5</v>
       </c>
@@ -3599,11 +3571,7 @@
           <t>SHOT +15% at 50% or better, −15% under it</t>
         </is>
       </c>
-      <c r="E51" s="0" t="inlineStr">
-        <is>
-          <t>Shoot the ball</t>
-        </is>
-      </c>
+      <c r="E51" s="0" t="n"/>
       <c r="F51" s="0" t="n">
         <v>5</v>
       </c>
@@ -3629,11 +3597,7 @@
           <t>SHOT -10%</t>
         </is>
       </c>
-      <c r="E52" s="0" t="inlineStr">
-        <is>
-          <t>Shoot the ball</t>
-        </is>
-      </c>
+      <c r="E52" s="0" t="n"/>
       <c r="F52" s="0" t="n">
         <v>5</v>
       </c>
@@ -7515,23 +7479,21 @@
   </sheetData>
   <mergeCells count="175">
     <mergeCell ref="G55:J55"/>
+    <mergeCell ref="G188:J188"/>
     <mergeCell ref="G4:J4"/>
     <mergeCell ref="G182:J182"/>
-    <mergeCell ref="G188:J188"/>
+    <mergeCell ref="G135:J135"/>
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
-    <mergeCell ref="G135:J135"/>
+    <mergeCell ref="G119:J119"/>
     <mergeCell ref="G32:J32"/>
     <mergeCell ref="G46:J46"/>
-    <mergeCell ref="G119:J119"/>
+    <mergeCell ref="G159:J159"/>
     <mergeCell ref="G40:J40"/>
     <mergeCell ref="G111:J111"/>
-    <mergeCell ref="G159:J159"/>
-    <mergeCell ref="G193:J193"/>
     <mergeCell ref="G72:J72"/>
     <mergeCell ref="G81:J81"/>
     <mergeCell ref="G161:J161"/>
-    <mergeCell ref="G5:J5"/>
     <mergeCell ref="G71:J71"/>
     <mergeCell ref="G136:J136"/>
     <mergeCell ref="G194:J194"/>
@@ -7542,10 +7504,11 @@
     <mergeCell ref="G174:J174"/>
     <mergeCell ref="G156:J156"/>
     <mergeCell ref="G57:J57"/>
+    <mergeCell ref="G128:J128"/>
     <mergeCell ref="G10:J10"/>
+    <mergeCell ref="G66:J66"/>
+    <mergeCell ref="G184:J184"/>
     <mergeCell ref="G137:J137"/>
-    <mergeCell ref="G66:J66"/>
-    <mergeCell ref="G128:J128"/>
     <mergeCell ref="G18:J18"/>
     <mergeCell ref="G53:J53"/>
     <mergeCell ref="G171:J171"/>
@@ -7564,12 +7527,13 @@
     <mergeCell ref="G113:J113"/>
     <mergeCell ref="G20:J20"/>
     <mergeCell ref="G91:J91"/>
+    <mergeCell ref="G85:J85"/>
     <mergeCell ref="G100:J100"/>
-    <mergeCell ref="G85:J85"/>
     <mergeCell ref="G183:J183"/>
     <mergeCell ref="G165:J165"/>
     <mergeCell ref="G75:J75"/>
     <mergeCell ref="G44:J44"/>
+    <mergeCell ref="G193:J193"/>
     <mergeCell ref="G22:J22"/>
     <mergeCell ref="G84:J84"/>
     <mergeCell ref="G102:J102"/>
@@ -7577,8 +7541,8 @@
     <mergeCell ref="G185:J185"/>
     <mergeCell ref="G12:J12"/>
     <mergeCell ref="G77:J77"/>
+    <mergeCell ref="G21:J21"/>
     <mergeCell ref="G86:J86"/>
-    <mergeCell ref="G21:J21"/>
     <mergeCell ref="G178:J178"/>
     <mergeCell ref="G67:J67"/>
     <mergeCell ref="G61:J61"/>
@@ -7590,18 +7554,17 @@
     <mergeCell ref="G125:J125"/>
     <mergeCell ref="G38:J38"/>
     <mergeCell ref="G7:J7"/>
+    <mergeCell ref="G191:J191"/>
     <mergeCell ref="G112:J112"/>
-    <mergeCell ref="G184:J184"/>
     <mergeCell ref="G45:J45"/>
-    <mergeCell ref="G191:J191"/>
     <mergeCell ref="G62:J62"/>
     <mergeCell ref="G175:J175"/>
     <mergeCell ref="G127:J127"/>
     <mergeCell ref="G162:J162"/>
     <mergeCell ref="G49:J49"/>
     <mergeCell ref="G24:J24"/>
+    <mergeCell ref="G195:J195"/>
     <mergeCell ref="G177:J177"/>
-    <mergeCell ref="G195:J195"/>
     <mergeCell ref="G33:J33"/>
     <mergeCell ref="G104:J104"/>
     <mergeCell ref="G65:J65"/>
@@ -7613,27 +7576,26 @@
     <mergeCell ref="G129:J129"/>
     <mergeCell ref="G138:J138"/>
     <mergeCell ref="G16:J16"/>
-    <mergeCell ref="G90:J90"/>
     <mergeCell ref="G76:J76"/>
     <mergeCell ref="G25:J25"/>
+    <mergeCell ref="G90:J90"/>
     <mergeCell ref="G60:J60"/>
     <mergeCell ref="G131:J131"/>
     <mergeCell ref="G9:J9"/>
-    <mergeCell ref="G124:J124"/>
+    <mergeCell ref="G59:J59"/>
+    <mergeCell ref="G115:J115"/>
     <mergeCell ref="G130:J130"/>
-    <mergeCell ref="G115:J115"/>
-    <mergeCell ref="G59:J59"/>
     <mergeCell ref="G11:J11"/>
     <mergeCell ref="G117:J117"/>
     <mergeCell ref="G169:J169"/>
     <mergeCell ref="G179:J179"/>
+    <mergeCell ref="G126:J126"/>
     <mergeCell ref="G132:J132"/>
     <mergeCell ref="G39:J39"/>
     <mergeCell ref="G122:J122"/>
-    <mergeCell ref="G126:J126"/>
     <mergeCell ref="G166:J166"/>
+    <mergeCell ref="G101:J101"/>
     <mergeCell ref="G116:J116"/>
-    <mergeCell ref="G101:J101"/>
     <mergeCell ref="G103:J103"/>
     <mergeCell ref="G37:J37"/>
     <mergeCell ref="G186:J186"/>
@@ -7641,9 +7603,8 @@
     <mergeCell ref="G13:J13"/>
     <mergeCell ref="G78:J78"/>
     <mergeCell ref="G118:J118"/>
+    <mergeCell ref="G87:J87"/>
     <mergeCell ref="G152:J152"/>
-    <mergeCell ref="G87:J87"/>
-    <mergeCell ref="G133:J133"/>
     <mergeCell ref="G167:J167"/>
     <mergeCell ref="G15:J15"/>
     <mergeCell ref="G142:J142"/>
@@ -7651,44 +7612,47 @@
     <mergeCell ref="G89:J89"/>
     <mergeCell ref="G64:J64"/>
     <mergeCell ref="G79:J79"/>
+    <mergeCell ref="G192:J192"/>
     <mergeCell ref="G73:J73"/>
     <mergeCell ref="G51:J51"/>
-    <mergeCell ref="G192:J192"/>
     <mergeCell ref="G153:J153"/>
     <mergeCell ref="G54:J54"/>
     <mergeCell ref="G63:J63"/>
     <mergeCell ref="G134:J134"/>
     <mergeCell ref="G41:J41"/>
+    <mergeCell ref="G50:J50"/>
     <mergeCell ref="G106:J106"/>
-    <mergeCell ref="G50:J50"/>
     <mergeCell ref="G164:J164"/>
     <mergeCell ref="G173:J173"/>
     <mergeCell ref="G56:J56"/>
     <mergeCell ref="G105:J105"/>
-    <mergeCell ref="G14:J14"/>
     <mergeCell ref="G43:J43"/>
     <mergeCell ref="G52:J52"/>
+    <mergeCell ref="G120:J120"/>
     <mergeCell ref="G155:J155"/>
-    <mergeCell ref="G120:J120"/>
-    <mergeCell ref="G107:J107"/>
     <mergeCell ref="G27:J27"/>
     <mergeCell ref="G36:J36"/>
     <mergeCell ref="G42:J42"/>
+    <mergeCell ref="G107:J107"/>
     <mergeCell ref="G17:J17"/>
     <mergeCell ref="G170:J170"/>
     <mergeCell ref="G157:J157"/>
     <mergeCell ref="G141:J141"/>
     <mergeCell ref="G19:J19"/>
     <mergeCell ref="G172:J172"/>
+    <mergeCell ref="G190:J190"/>
+    <mergeCell ref="G28:J28"/>
     <mergeCell ref="G93:J93"/>
-    <mergeCell ref="G28:J28"/>
     <mergeCell ref="G6:J6"/>
-    <mergeCell ref="G190:J190"/>
     <mergeCell ref="G187:J187"/>
     <mergeCell ref="G69:J69"/>
     <mergeCell ref="G83:J83"/>
     <mergeCell ref="G196:J196"/>
+    <mergeCell ref="G124:J124"/>
     <mergeCell ref="G180:J180"/>
+    <mergeCell ref="G5:J5"/>
+    <mergeCell ref="G133:J133"/>
+    <mergeCell ref="G14:J14"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
SHOT audit, stage 2: every "You may", The Future, Equalizer
- One yes-or-no prompt for a card's "You may": Lob takes the Ball out of play into your hand,
  No-Look flips for a card, Kick-Out's Clamps are yours to Assign, Outlet Pass offers a Shot Clock
  Reset as your next possession opens, Turnaround Three can dump a hand of three or more for
  SHOT = 100%, and the Ankle Breaker combo takes a card out of a target player's hand.
- Bullet Pass has the passer pick the discard, face down.
- Rhythm Dribble puts +10% extra on the very next action if that is a shot.
- Equalizer is a second Shoot button at 100%: it is discarded taking it, and a make levels every
  player's points to the shooter's.
- The Future (Varena, 1): Moves pay +10% and a card, passes cost 10%, and a three can be bought up
  to four points with one card at SHOT -10%. In the game and on the sheet.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -2089,7 +2089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J197"/>
+  <dimension ref="A1:J198"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="22.25" customHeight="1"/>
   <cols>
     <col width="15.5" customWidth="1" style="8" min="1" max="1"/>
@@ -6163,7 +6163,7 @@
         </is>
       </c>
       <c r="B151" s="53">
-        <f>COUNTIF($B$152:$B$180,"Varena")</f>
+        <f>COUNTIF($B$152:$B$181,"Varena")</f>
         <v/>
       </c>
       <c r="C151" s="54" t="n"/>
@@ -7006,75 +7006,80 @@
       </c>
       <c r="C180" s="56" t="inlineStr">
         <is>
-          <t>Tick-Tock Tile</t>
+          <t>The Future</t>
         </is>
       </c>
       <c r="D180" s="63" t="inlineStr">
         <is>
-          <t>Playing any card also ticks the Shot Clock</t>
-        </is>
-      </c>
-      <c r="E180" s="58" t="n"/>
+          <t>SHOT +10% and Draw 1 card when playing a Move card.
+SHOT -10% while Passing.</t>
+        </is>
+      </c>
+      <c r="E180" s="58" t="inlineStr">
+        <is>
+          <t>You may Discard 1 card during a three attempt to make it worth four pts (at SHOT-10%)</t>
+        </is>
+      </c>
       <c r="F180" s="61" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G180" s="75" t="inlineStr">
         <is>
-          <t>The tick is paid after the card resolves, so a shot at 01 still goes up</t>
+          <t>New in the SHOT audit (2026-09-14). Special Moves count as Moves</t>
         </is>
       </c>
       <c r="H180" s="76" t="n"/>
       <c r="I180" s="76" t="n"/>
       <c r="J180" s="76" t="n"/>
     </row>
-    <row r="181" ht="42" customHeight="1" s="85">
-      <c r="A181" s="52" t="inlineStr">
+    <row r="181" s="85">
+      <c r="A181" s="27" t="n"/>
+      <c r="B181" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C181" s="56" t="inlineStr">
+        <is>
+          <t>Tick-Tock Tile</t>
+        </is>
+      </c>
+      <c r="D181" s="63" t="inlineStr">
+        <is>
+          <t>Playing any card also ticks the Shot Clock</t>
+        </is>
+      </c>
+      <c r="E181" s="58" t="n"/>
+      <c r="F181" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G181" s="75" t="inlineStr">
+        <is>
+          <t>The tick is paid after the card resolves, so a shot at 01 still goes up</t>
+        </is>
+      </c>
+      <c r="H181" s="76" t="n"/>
+      <c r="I181" s="76" t="n"/>
+      <c r="J181" s="76" t="n"/>
+    </row>
+    <row r="182" ht="42" customHeight="1" s="85">
+      <c r="A182" s="52" t="inlineStr">
         <is>
           <t>Variaball</t>
         </is>
       </c>
-      <c r="B181" s="53">
-        <f>COUNTIF($B$182:$B$197,"Variaball")</f>
+      <c r="B182" s="53">
+        <f>COUNTIF($B$183:$B$198,"Variaball")</f>
         <v/>
       </c>
-      <c r="C181" s="54" t="n"/>
-      <c r="D181" s="54" t="n"/>
-      <c r="E181" s="54" t="n"/>
-      <c r="F181" s="55" t="n"/>
-      <c r="G181" s="66" t="n"/>
-      <c r="H181" s="67" t="n"/>
-      <c r="I181" s="67" t="n"/>
-      <c r="J181" s="67" t="n"/>
-    </row>
-    <row r="182" s="85">
-      <c r="A182" s="27" t="n"/>
-      <c r="B182" s="28" t="inlineStr">
-        <is>
-          <t>Variaball</t>
-        </is>
-      </c>
-      <c r="C182" s="56" t="inlineStr">
-        <is>
-          <t>Med Ball</t>
-        </is>
-      </c>
-      <c r="D182" s="63" t="inlineStr">
-        <is>
-          <t>SHOT cannot exceed 50%</t>
-        </is>
-      </c>
-      <c r="E182" s="58" t="n"/>
-      <c r="F182" s="61" t="n">
-        <v>2</v>
-      </c>
-      <c r="G182" s="75" t="inlineStr">
-        <is>
-          <t>An Intangible's or a Varena's SHOT = is not held to it</t>
-        </is>
-      </c>
-      <c r="H182" s="76" t="n"/>
-      <c r="I182" s="76" t="n"/>
-      <c r="J182" s="76" t="n"/>
+      <c r="C182" s="54" t="n"/>
+      <c r="D182" s="54" t="n"/>
+      <c r="E182" s="54" t="n"/>
+      <c r="F182" s="55" t="n"/>
+      <c r="G182" s="66" t="n"/>
+      <c r="H182" s="67" t="n"/>
+      <c r="I182" s="67" t="n"/>
+      <c r="J182" s="67" t="n"/>
     </row>
     <row r="183" s="85">
       <c r="A183" s="27" t="n"/>
@@ -7085,12 +7090,12 @@
       </c>
       <c r="C183" s="56" t="inlineStr">
         <is>
-          <t>Dishcount Ball</t>
+          <t>Med Ball</t>
         </is>
       </c>
       <c r="D183" s="63" t="inlineStr">
         <is>
-          <t>Discard one fewer for card costs and Clamps</t>
+          <t>SHOT cannot exceed 50%</t>
         </is>
       </c>
       <c r="E183" s="58" t="n"/>
@@ -7099,7 +7104,7 @@
       </c>
       <c r="G183" s="75" t="inlineStr">
         <is>
-          <t>Counts: Clamps, Pound Dribble, Frostbite Finish, Stepback, Turnaround Three</t>
+          <t>An Intangible's or a Varena's SHOT = is not held to it</t>
         </is>
       </c>
       <c r="H183" s="76" t="n"/>
@@ -7115,21 +7120,21 @@
       </c>
       <c r="C184" s="56" t="inlineStr">
         <is>
-          <t>Blight Ball</t>
+          <t>Dishcount Ball</t>
         </is>
       </c>
       <c r="D184" s="63" t="inlineStr">
         <is>
-          <t>Injuries travel with the ball, and new ones join the pile. Discarding the ball takes the pile with it</t>
+          <t>Discard one fewer for card costs and Clamps</t>
         </is>
       </c>
       <c r="E184" s="58" t="n"/>
       <c r="F184" s="61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G184" s="75" t="inlineStr">
         <is>
-          <t>Moves on any change of hands</t>
+          <t>Counts: Clamps, Pound Dribble, Frostbite Finish, Stepback, Turnaround Three</t>
         </is>
       </c>
       <c r="H184" s="76" t="n"/>
@@ -7145,19 +7150,23 @@
       </c>
       <c r="C185" s="56" t="inlineStr">
         <is>
-          <t>Bench Ball</t>
+          <t>Blight Ball</t>
         </is>
       </c>
       <c r="D185" s="63" t="inlineStr">
         <is>
-          <t>Receiving it by Pass: no draw, no turn. You inbound</t>
+          <t>Injuries travel with the ball, and new ones join the pile. Discarding the ball takes the pile with it</t>
         </is>
       </c>
       <c r="E185" s="58" t="n"/>
       <c r="F185" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="G185" s="75" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="G185" s="75" t="inlineStr">
+        <is>
+          <t>Moves on any change of hands</t>
+        </is>
+      </c>
       <c r="H185" s="76" t="n"/>
       <c r="I185" s="76" t="n"/>
       <c r="J185" s="76" t="n"/>
@@ -7171,23 +7180,19 @@
       </c>
       <c r="C186" s="56" t="inlineStr">
         <is>
-          <t>Dishtracting Ball</t>
+          <t>Bench Ball</t>
         </is>
       </c>
       <c r="D186" s="63" t="inlineStr">
         <is>
-          <t>Receiving it: discard 1, after the draw for turn</t>
+          <t>Receiving it by Pass: no draw, no turn. You inbound</t>
         </is>
       </c>
       <c r="E186" s="58" t="n"/>
       <c r="F186" s="61" t="n">
-        <v>2</v>
-      </c>
-      <c r="G186" s="75" t="inlineStr">
-        <is>
-          <t>Any change of hands</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G186" s="75" t="n"/>
       <c r="H186" s="76" t="n"/>
       <c r="I186" s="76" t="n"/>
       <c r="J186" s="76" t="n"/>
@@ -7201,19 +7206,23 @@
       </c>
       <c r="C187" s="56" t="inlineStr">
         <is>
-          <t>Hand Ball</t>
+          <t>Dishtracting Ball</t>
         </is>
       </c>
       <c r="D187" s="63" t="inlineStr">
         <is>
-          <t>A Pass swaps hands: yours goes with the ball, theirs comes back</t>
+          <t>Receiving it: discard 1, after the draw for turn</t>
         </is>
       </c>
       <c r="E187" s="58" t="n"/>
       <c r="F187" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="G187" s="75" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="G187" s="75" t="inlineStr">
+        <is>
+          <t>Any change of hands</t>
+        </is>
+      </c>
       <c r="H187" s="76" t="n"/>
       <c r="I187" s="76" t="n"/>
       <c r="J187" s="76" t="n"/>
@@ -7227,12 +7236,12 @@
       </c>
       <c r="C188" s="56" t="inlineStr">
         <is>
-          <t>Foot Ball</t>
+          <t>Hand Ball</t>
         </is>
       </c>
       <c r="D188" s="63" t="inlineStr">
         <is>
-          <t>Moves and Passes are not spent. They lock until your possession ends</t>
+          <t>A Pass swaps hands: yours goes with the ball, theirs comes back</t>
         </is>
       </c>
       <c r="E188" s="58" t="n"/>
@@ -7253,17 +7262,17 @@
       </c>
       <c r="C189" s="56" t="inlineStr">
         <is>
-          <t>Recharge Rock</t>
+          <t>Foot Ball</t>
         </is>
       </c>
       <c r="D189" s="63" t="inlineStr">
         <is>
-          <t>Double your draw for turn</t>
+          <t>Moves and Passes are not spent. They lock until your possession ends</t>
         </is>
       </c>
       <c r="E189" s="58" t="n"/>
       <c r="F189" s="61" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G189" s="75" t="n"/>
       <c r="H189" s="76" t="n"/>
@@ -7279,23 +7288,19 @@
       </c>
       <c r="C190" s="56" t="inlineStr">
         <is>
-          <t>Variaball</t>
+          <t>Recharge Rock</t>
         </is>
       </c>
       <c r="D190" s="63" t="inlineStr">
         <is>
-          <t>A random Variaball from the discards goes into play. Then discard this</t>
+          <t>Double your draw for turn</t>
         </is>
       </c>
       <c r="E190" s="58" t="n"/>
       <c r="F190" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="G190" s="75" t="inlineStr">
-        <is>
-          <t>From the deck if the discards have none; never the ball already in play</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="G190" s="75" t="n"/>
       <c r="H190" s="76" t="n"/>
       <c r="I190" s="76" t="n"/>
       <c r="J190" s="76" t="n"/>
@@ -7309,19 +7314,23 @@
       </c>
       <c r="C191" s="56" t="inlineStr">
         <is>
-          <t>Shufflebag Ball</t>
+          <t>Variaball</t>
         </is>
       </c>
       <c r="D191" s="63" t="inlineStr">
         <is>
-          <t>Every possession, the turn player shuffles their hand into the deck and draws the same number, then draws for turn</t>
+          <t>A random Variaball from the discards goes into play. Then discard this</t>
         </is>
       </c>
       <c r="E191" s="58" t="n"/>
       <c r="F191" s="61" t="n">
         <v>1</v>
       </c>
-      <c r="G191" s="75" t="n"/>
+      <c r="G191" s="75" t="inlineStr">
+        <is>
+          <t>From the deck if the discards have none; never the ball already in play</t>
+        </is>
+      </c>
       <c r="H191" s="76" t="n"/>
       <c r="I191" s="76" t="n"/>
       <c r="J191" s="76" t="n"/>
@@ -7335,12 +7344,12 @@
       </c>
       <c r="C192" s="56" t="inlineStr">
         <is>
-          <t>Bag'n Ball</t>
+          <t>Shufflebag Ball</t>
         </is>
       </c>
       <c r="D192" s="63" t="inlineStr">
         <is>
-          <t>Draw 1 card when played. SHOT = 10% for each card in your hand</t>
+          <t>Every possession, the turn player shuffles their hand into the deck and draws the same number, then draws for turn</t>
         </is>
       </c>
       <c r="E192" s="58" t="n"/>
@@ -7361,23 +7370,19 @@
       </c>
       <c r="C193" s="56" t="inlineStr">
         <is>
-          <t>Blaze Ball</t>
+          <t>Bag'n Ball</t>
         </is>
       </c>
       <c r="D193" s="63" t="inlineStr">
         <is>
-          <t>SHOT +10% as this Ball is Passed</t>
+          <t>Draw 1 card when played. SHOT = 10% for each card in your hand</t>
         </is>
       </c>
       <c r="E193" s="58" t="n"/>
       <c r="F193" s="61" t="n">
-        <v>5</v>
-      </c>
-      <c r="G193" s="75" t="inlineStr">
-        <is>
-          <t>Ignores every other pass modifier</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G193" s="75" t="n"/>
       <c r="H193" s="76" t="n"/>
       <c r="I193" s="76" t="n"/>
       <c r="J193" s="76" t="n"/>
@@ -7391,12 +7396,12 @@
       </c>
       <c r="C194" s="56" t="inlineStr">
         <is>
-          <t>Snow Ball It</t>
+          <t>Blaze Ball</t>
         </is>
       </c>
       <c r="D194" s="63" t="inlineStr">
         <is>
-          <t>SHOT -10% as this Ball is Passed</t>
+          <t>SHOT +10% as this Ball is Passed</t>
         </is>
       </c>
       <c r="E194" s="58" t="n"/>
@@ -7405,7 +7410,7 @@
       </c>
       <c r="G194" s="75" t="inlineStr">
         <is>
-          <t>Blaze Ball's opposite</t>
+          <t>Ignores every other pass modifier</t>
         </is>
       </c>
       <c r="H194" s="76" t="n"/>
@@ -7421,19 +7426,23 @@
       </c>
       <c r="C195" s="56" t="inlineStr">
         <is>
-          <t>Brick Ball</t>
+          <t>Snow Ball It</t>
         </is>
       </c>
       <c r="D195" s="63" t="inlineStr">
         <is>
-          <t>SHOT = 25%</t>
+          <t>SHOT -10% as this Ball is Passed</t>
         </is>
       </c>
       <c r="E195" s="58" t="n"/>
       <c r="F195" s="61" t="n">
-        <v>2</v>
-      </c>
-      <c r="G195" s="75" t="n"/>
+        <v>5</v>
+      </c>
+      <c r="G195" s="75" t="inlineStr">
+        <is>
+          <t>Blaze Ball's opposite</t>
+        </is>
+      </c>
       <c r="H195" s="76" t="n"/>
       <c r="I195" s="76" t="n"/>
       <c r="J195" s="76" t="n"/>
@@ -7447,23 +7456,19 @@
       </c>
       <c r="C196" s="56" t="inlineStr">
         <is>
-          <t>Monster Ball</t>
+          <t>Brick Ball</t>
         </is>
       </c>
       <c r="D196" s="63" t="inlineStr">
         <is>
-          <t>Intangibles are absorbed into the ball. When it's discarded, players rebound for them one at a time</t>
+          <t>SHOT = 25%</t>
         </is>
       </c>
       <c r="E196" s="58" t="n"/>
       <c r="F196" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="G196" s="75" t="inlineStr">
-        <is>
-          <t>Swallows every Intangible already out and every one drawn while it's in play</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="G196" s="75" t="n"/>
       <c r="H196" s="76" t="n"/>
       <c r="I196" s="76" t="n"/>
       <c r="J196" s="76" t="n"/>
@@ -7477,33 +7482,63 @@
       </c>
       <c r="C197" s="56" t="inlineStr">
         <is>
-          <t>Brand New Ball</t>
+          <t>Monster Ball</t>
         </is>
       </c>
       <c r="D197" s="63" t="inlineStr">
         <is>
-          <t>25% chance a shot attempt is a turnover instead</t>
+          <t>Intangibles are absorbed into the ball. When it's discarded, players rebound for them one at a time</t>
         </is>
       </c>
       <c r="E197" s="58" t="n"/>
       <c r="F197" s="61" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G197" s="75" t="inlineStr">
         <is>
-          <t>The round ends</t>
+          <t>Swallows every Intangible already out and every one drawn while it's in play</t>
         </is>
       </c>
       <c r="H197" s="76" t="n"/>
       <c r="I197" s="76" t="n"/>
       <c r="J197" s="76" t="n"/>
     </row>
+    <row r="198" s="85">
+      <c r="A198" s="27" t="n"/>
+      <c r="B198" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C198" s="56" t="inlineStr">
+        <is>
+          <t>Brand New Ball</t>
+        </is>
+      </c>
+      <c r="D198" s="63" t="inlineStr">
+        <is>
+          <t>25% chance a shot attempt is a turnover instead</t>
+        </is>
+      </c>
+      <c r="E198" s="58" t="n"/>
+      <c r="F198" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G198" s="75" t="inlineStr">
+        <is>
+          <t>The round ends</t>
+        </is>
+      </c>
+      <c r="H198" s="76" t="n"/>
+      <c r="I198" s="76" t="n"/>
+      <c r="J198" s="76" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="175">
+  <mergeCells count="176">
     <mergeCell ref="G55:J55"/>
-    <mergeCell ref="G188:J188"/>
     <mergeCell ref="G4:J4"/>
     <mergeCell ref="G182:J182"/>
+    <mergeCell ref="G188:J188"/>
     <mergeCell ref="G135:J135"/>
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
@@ -7529,8 +7564,8 @@
     <mergeCell ref="G128:J128"/>
     <mergeCell ref="G10:J10"/>
     <mergeCell ref="G66:J66"/>
+    <mergeCell ref="G137:J137"/>
     <mergeCell ref="G184:J184"/>
-    <mergeCell ref="G137:J137"/>
     <mergeCell ref="G18:J18"/>
     <mergeCell ref="G53:J53"/>
     <mergeCell ref="G171:J171"/>
@@ -7555,9 +7590,9 @@
     <mergeCell ref="G165:J165"/>
     <mergeCell ref="G75:J75"/>
     <mergeCell ref="G44:J44"/>
-    <mergeCell ref="G193:J193"/>
     <mergeCell ref="G22:J22"/>
     <mergeCell ref="G84:J84"/>
+    <mergeCell ref="G193:J193"/>
     <mergeCell ref="G102:J102"/>
     <mergeCell ref="G158:J158"/>
     <mergeCell ref="G185:J185"/>
@@ -7585,8 +7620,8 @@
     <mergeCell ref="G162:J162"/>
     <mergeCell ref="G49:J49"/>
     <mergeCell ref="G24:J24"/>
+    <mergeCell ref="G177:J177"/>
     <mergeCell ref="G195:J195"/>
-    <mergeCell ref="G177:J177"/>
     <mergeCell ref="G33:J33"/>
     <mergeCell ref="G104:J104"/>
     <mergeCell ref="G65:J65"/>
@@ -7604,11 +7639,13 @@
     <mergeCell ref="G60:J60"/>
     <mergeCell ref="G131:J131"/>
     <mergeCell ref="G9:J9"/>
+    <mergeCell ref="G198:J198"/>
     <mergeCell ref="G59:J59"/>
     <mergeCell ref="G115:J115"/>
     <mergeCell ref="G130:J130"/>
     <mergeCell ref="G11:J11"/>
     <mergeCell ref="G117:J117"/>
+    <mergeCell ref="G180:J180"/>
     <mergeCell ref="G169:J169"/>
     <mergeCell ref="G179:J179"/>
     <mergeCell ref="G126:J126"/>
@@ -7662,16 +7699,15 @@
     <mergeCell ref="G141:J141"/>
     <mergeCell ref="G19:J19"/>
     <mergeCell ref="G172:J172"/>
-    <mergeCell ref="G190:J190"/>
     <mergeCell ref="G28:J28"/>
     <mergeCell ref="G93:J93"/>
     <mergeCell ref="G6:J6"/>
+    <mergeCell ref="G190:J190"/>
+    <mergeCell ref="G69:J69"/>
     <mergeCell ref="G187:J187"/>
-    <mergeCell ref="G69:J69"/>
     <mergeCell ref="G83:J83"/>
     <mergeCell ref="G196:J196"/>
     <mergeCell ref="G124:J124"/>
-    <mergeCell ref="G180:J180"/>
     <mergeCell ref="G5:J5"/>
     <mergeCell ref="G133:J133"/>
     <mergeCell ref="G14:J14"/>

</xml_diff>

<commit_message>
500 again, readable inks, and the sheet caught up
- One more basic Variaball (2) and one more Drive (16).
- Keywords, card names and named types that are lost on a body swap to their nearest palette
  neighbour that reads there (contrast 2.0), so recolouring a body keeps its words readable.
- "Possession" on Torn Achilles and Torn Meniscus; the style guide says Turn only means rotating a card.
- Sheet: Snow Ball, the injury rework with the Devastating rule, Make-or-Take and Hero Ball,
  Policeum retired, Cardwood 6, Drive 16, Variaball 2. It matches the game card for card.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -2089,7 +2089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J198"/>
+  <dimension ref="A1:J208"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="22.25" customHeight="1"/>
   <cols>
     <col width="15.5" customWidth="1" style="8" min="1" max="1"/>
@@ -2170,39 +2170,39 @@
         </is>
       </c>
       <c r="B2" s="12">
-        <f>COUNTIF($B$5:$B$146,"Pass")</f>
+        <f>COUNTIF($B$5:$B$154,"Pass")</f>
         <v/>
       </c>
       <c r="C2" s="13">
-        <f>COUNTIF($B$5:$B$146,"Move")+COUNTIF($B$5:$B$146,"Special Move")</f>
+        <f>COUNTIF($B$5:$B$154,"Move")+COUNTIF($B$5:$B$154,"Special Move")</f>
         <v/>
       </c>
       <c r="D2" s="14">
-        <f>COUNTIF($B$5:$B$146,"Clamp")</f>
+        <f>COUNTIF($B$5:$B$154,"Clamp")</f>
         <v/>
       </c>
       <c r="E2" s="15">
-        <f>COUNTIF($B$5:$B$146,"Whistle")</f>
+        <f>COUNTIF($B$5:$B$154,"Whistle")</f>
         <v/>
       </c>
       <c r="F2" s="16">
-        <f>COUNTIF($B$5:$B$146,"Game Break")</f>
+        <f>COUNTIF($B$5:$B$154,"Game Break")</f>
         <v/>
       </c>
       <c r="G2" s="18">
-        <f>COUNTIF($B$5:$B$146,"Injury")</f>
+        <f>COUNTIF($B$5:$B$154,"Injury")</f>
         <v/>
       </c>
       <c r="H2" s="19">
-        <f>COUNTIF($B$5:$B$146,"Devastating Injury")</f>
+        <f>COUNTIF($B$5:$B$154,"Devastating Injury")</f>
         <v/>
       </c>
       <c r="I2" s="17">
-        <f>COUNTIF($B$5:$B$146,"Intangible")</f>
+        <f>COUNTIF($B$5:$B$154,"Intangible")</f>
         <v/>
       </c>
       <c r="J2" s="87">
-        <f>SUM(B2:E2)+COUNTIF($B$5:$B$146,"Game Break")+SUM(G2:I2)</f>
+        <f>SUM(B2:E2)+COUNTIF($B$5:$B$154,"Game Break")+SUM(G2:I2)</f>
         <v/>
       </c>
     </row>
@@ -2250,7 +2250,7 @@
         </is>
       </c>
       <c r="B5" s="53">
-        <f>COUNTIF($B$6:$B$150,"Pass")</f>
+        <f>COUNTIF($B$6:$B$158,"Pass")</f>
         <v/>
       </c>
       <c r="C5" s="54" t="n"/>
@@ -2715,7 +2715,7 @@
         </is>
       </c>
       <c r="B21" s="53">
-        <f>COUNTIF($B$22:$B$150,"Move")+COUNTIF($B$22:$B$150,"Special Move")</f>
+        <f>COUNTIF($B$22:$B$158,"Move")+COUNTIF($B$22:$B$158,"Special Move")</f>
         <v/>
       </c>
       <c r="C21" s="54" t="n"/>
@@ -2772,7 +2772,7 @@
       </c>
       <c r="E23" s="6" t="n"/>
       <c r="F23" s="32" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G23" s="70" t="inlineStr">
         <is>
@@ -3124,7 +3124,7 @@
         </is>
       </c>
       <c r="B35" s="53">
-        <f>COUNTIF($B$36:$B$150,"Special Move")</f>
+        <f>COUNTIF($B$36:$B$158,"Special Move")</f>
         <v/>
       </c>
       <c r="C35" s="54" t="n"/>
@@ -3622,7 +3622,7 @@
         </is>
       </c>
       <c r="B53" s="53">
-        <f>COUNTIF($B$54:$B$150,"Clamp")</f>
+        <f>COUNTIF($B$54:$B$158,"Clamp")</f>
         <v/>
       </c>
       <c r="C53" s="54" t="n"/>
@@ -3877,7 +3877,7 @@
         </is>
       </c>
       <c r="B62" s="53">
-        <f>COUNTIF($B$63:$B$150,"Whistle")</f>
+        <f>COUNTIF($B$63:$B$158,"Whistle")</f>
         <v/>
       </c>
       <c r="C62" s="54" t="n"/>
@@ -5305,7 +5305,7 @@
         </is>
       </c>
       <c r="B116" s="53">
-        <f>COUNTIF($B$117:$B$150,"Injury")</f>
+        <f>COUNTIF($B$117:$B$158,"Injury")</f>
         <v/>
       </c>
       <c r="C116" s="54" t="n"/>
@@ -5331,289 +5331,310 @@
       </c>
       <c r="D117" s="63" t="inlineStr">
         <is>
-          <t>Discard 1 card at the start of each turn after drawing (your choice)</t>
+          <t>SHOT -10%</t>
         </is>
       </c>
       <c r="E117" s="58" t="n"/>
       <c r="F117" s="59" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G117" s="75" t="n"/>
       <c r="H117" s="76" t="n"/>
       <c r="I117" s="76" t="n"/>
       <c r="J117" s="76" t="n"/>
     </row>
-    <row r="118" ht="20" customHeight="1" s="85">
-      <c r="A118" s="52" t="inlineStr">
-        <is>
-          <t>Devastating Injury</t>
-        </is>
-      </c>
-      <c r="B118" s="53">
-        <f>COUNTIF($B$119:$B$150,"Devastating Injury")</f>
-        <v/>
-      </c>
-      <c r="C118" s="54" t="n"/>
-      <c r="D118" s="54" t="n"/>
-      <c r="E118" s="54" t="n"/>
-      <c r="F118" s="55" t="n"/>
-      <c r="G118" s="66" t="n"/>
-      <c r="H118" s="67" t="n"/>
-      <c r="I118" s="67" t="n"/>
-      <c r="J118" s="67" t="n"/>
-    </row>
-    <row r="119" ht="28" customHeight="1" s="85">
+    <row r="118" ht="57" customHeight="1" s="85">
+      <c r="A118" s="27" t="n"/>
+      <c r="B118" s="28" t="inlineStr">
+        <is>
+          <t>Injury</t>
+        </is>
+      </c>
+      <c r="C118" s="56" t="inlineStr">
+        <is>
+          <t>Rolled Ankle</t>
+        </is>
+      </c>
+      <c r="D118" s="63" t="inlineStr">
+        <is>
+          <t>Discard 1 card to play a Move card</t>
+        </is>
+      </c>
+      <c r="E118" s="58" t="n"/>
+      <c r="F118" s="59" t="n">
+        <v>2</v>
+      </c>
+      <c r="G118" s="75" t="n"/>
+      <c r="H118" s="76" t="n"/>
+      <c r="I118" s="76" t="n"/>
+      <c r="J118" s="76" t="n"/>
+    </row>
+    <row r="119" ht="57" customHeight="1" s="85">
       <c r="A119" s="27" t="n"/>
       <c r="B119" s="28" t="inlineStr">
         <is>
-          <t>Devastating Injury</t>
-        </is>
-      </c>
-      <c r="C119" s="64" t="inlineStr">
-        <is>
-          <t>Torn Achilles</t>
-        </is>
-      </c>
-      <c r="D119" s="65" t="inlineStr">
-        <is>
-          <t>Hand is locked every turn except 1 card (randomly)</t>
+          <t>Injury</t>
+        </is>
+      </c>
+      <c r="C119" s="56" t="inlineStr">
+        <is>
+          <t>Fractured Collarbone</t>
+        </is>
+      </c>
+      <c r="D119" s="63" t="inlineStr">
+        <is>
+          <t>Cannot attempt Three-point shots</t>
         </is>
       </c>
       <c r="E119" s="58" t="n"/>
-      <c r="F119" s="61" t="n"/>
+      <c r="F119" s="59" t="n">
+        <v>2</v>
+      </c>
       <c r="G119" s="75" t="n"/>
       <c r="H119" s="76" t="n"/>
       <c r="I119" s="76" t="n"/>
       <c r="J119" s="76" t="n"/>
     </row>
-    <row r="120" ht="42" customHeight="1" s="85">
-      <c r="A120" s="52" t="inlineStr">
+    <row r="120" ht="57" customHeight="1" s="85">
+      <c r="A120" s="27" t="n"/>
+      <c r="B120" s="28" t="inlineStr">
+        <is>
+          <t>Injury</t>
+        </is>
+      </c>
+      <c r="C120" s="56" t="inlineStr">
+        <is>
+          <t>Jammed Finger</t>
+        </is>
+      </c>
+      <c r="D120" s="63" t="inlineStr">
+        <is>
+          <t>Discard 1 card at random while receiving a Pass</t>
+        </is>
+      </c>
+      <c r="E120" s="58" t="n"/>
+      <c r="F120" s="59" t="n">
+        <v>2</v>
+      </c>
+      <c r="G120" s="75" t="n"/>
+      <c r="H120" s="76" t="n"/>
+      <c r="I120" s="76" t="n"/>
+      <c r="J120" s="76" t="n"/>
+    </row>
+    <row r="121" ht="57" customHeight="1" s="85">
+      <c r="A121" s="27" t="n"/>
+      <c r="B121" s="28" t="inlineStr">
+        <is>
+          <t>Injury</t>
+        </is>
+      </c>
+      <c r="C121" s="56" t="inlineStr">
+        <is>
+          <t>Sprained Hamstring</t>
+        </is>
+      </c>
+      <c r="D121" s="63" t="inlineStr">
+        <is>
+          <t>Your Rebound Bids are worth 1 less</t>
+        </is>
+      </c>
+      <c r="E121" s="58" t="n"/>
+      <c r="F121" s="59" t="n">
+        <v>2</v>
+      </c>
+      <c r="G121" s="75" t="n"/>
+      <c r="H121" s="76" t="n"/>
+      <c r="I121" s="76" t="n"/>
+      <c r="J121" s="76" t="n"/>
+    </row>
+    <row r="122" ht="57" customHeight="1" s="85">
+      <c r="A122" s="27" t="n"/>
+      <c r="B122" s="28" t="inlineStr">
+        <is>
+          <t>Injury</t>
+        </is>
+      </c>
+      <c r="C122" s="56" t="inlineStr">
+        <is>
+          <t>Hip Contusion</t>
+        </is>
+      </c>
+      <c r="D122" s="63" t="inlineStr">
+        <is>
+          <t>Discard 1 card at random when playing a Pass card</t>
+        </is>
+      </c>
+      <c r="E122" s="58" t="n"/>
+      <c r="F122" s="59" t="n">
+        <v>2</v>
+      </c>
+      <c r="G122" s="75" t="n"/>
+      <c r="H122" s="76" t="n"/>
+      <c r="I122" s="76" t="n"/>
+      <c r="J122" s="76" t="n"/>
+    </row>
+    <row r="123" ht="20" customHeight="1" s="85">
+      <c r="A123" s="52" t="inlineStr">
+        <is>
+          <t>Devastating Injury</t>
+        </is>
+      </c>
+      <c r="B123" s="53">
+        <f>COUNTIF($B$124:$B$158,"Devastating Injury")</f>
+        <v/>
+      </c>
+      <c r="C123" s="54" t="n"/>
+      <c r="D123" s="54" t="n"/>
+      <c r="E123" s="54" t="n"/>
+      <c r="F123" s="55" t="n"/>
+      <c r="G123" s="66" t="n"/>
+      <c r="H123" s="67" t="n"/>
+      <c r="I123" s="67" t="n"/>
+      <c r="J123" s="67" t="n"/>
+    </row>
+    <row r="124" ht="28" customHeight="1" s="85">
+      <c r="A124" s="27" t="n"/>
+      <c r="B124" s="28" t="inlineStr">
+        <is>
+          <t>Devastating Injury</t>
+        </is>
+      </c>
+      <c r="C124" s="64" t="inlineStr">
+        <is>
+          <t>Torn Achilles</t>
+        </is>
+      </c>
+      <c r="D124" s="65" t="inlineStr">
+        <is>
+          <t>Cannot Play Dunk Cards. Can only play 1 Move card per possession</t>
+        </is>
+      </c>
+      <c r="E124" s="58" t="n"/>
+      <c r="F124" s="61" t="n"/>
+      <c r="G124" s="75" t="inlineStr">
+        <is>
+          <t>Landing one discards every other Injury, and while one is on you a new Injury is discarded</t>
+        </is>
+      </c>
+      <c r="H124" s="76" t="n"/>
+      <c r="I124" s="76" t="n"/>
+      <c r="J124" s="76" t="n"/>
+    </row>
+    <row r="125" ht="28" customHeight="1" s="85">
+      <c r="A125" s="27" t="n"/>
+      <c r="B125" s="28" t="inlineStr">
+        <is>
+          <t>Devastating Injury</t>
+        </is>
+      </c>
+      <c r="C125" s="64" t="inlineStr">
+        <is>
+          <t>Torn ACL</t>
+        </is>
+      </c>
+      <c r="D125" s="65" t="inlineStr">
+        <is>
+          <t>Cannot Play Move Cards.</t>
+        </is>
+      </c>
+      <c r="E125" s="58" t="n"/>
+      <c r="F125" s="61" t="n"/>
+      <c r="G125" s="75" t="n"/>
+      <c r="H125" s="76" t="n"/>
+      <c r="I125" s="76" t="n"/>
+      <c r="J125" s="76" t="n"/>
+    </row>
+    <row r="126" ht="28" customHeight="1" s="85">
+      <c r="A126" s="27" t="n"/>
+      <c r="B126" s="28" t="inlineStr">
+        <is>
+          <t>Devastating Injury</t>
+        </is>
+      </c>
+      <c r="C126" s="64" t="inlineStr">
+        <is>
+          <t>Torn Meniscus</t>
+        </is>
+      </c>
+      <c r="D126" s="65" t="inlineStr">
+        <is>
+          <t>Randomly Lock all but 1 Card Each Possession</t>
+        </is>
+      </c>
+      <c r="E126" s="58" t="n"/>
+      <c r="F126" s="61" t="n"/>
+      <c r="G126" s="75" t="n"/>
+      <c r="H126" s="76" t="n"/>
+      <c r="I126" s="76" t="n"/>
+      <c r="J126" s="76" t="n"/>
+    </row>
+    <row r="127" ht="28" customHeight="1" s="85">
+      <c r="A127" s="27" t="n"/>
+      <c r="B127" s="28" t="inlineStr">
+        <is>
+          <t>Devastating Injury</t>
+        </is>
+      </c>
+      <c r="C127" s="64" t="inlineStr">
+        <is>
+          <t>Patellar Tendon Tear</t>
+        </is>
+      </c>
+      <c r="D127" s="65" t="inlineStr">
+        <is>
+          <t>Cannot Draw Cards except at the start of your possession</t>
+        </is>
+      </c>
+      <c r="E127" s="58" t="n"/>
+      <c r="F127" s="61" t="n"/>
+      <c r="G127" s="75" t="n"/>
+      <c r="H127" s="76" t="n"/>
+      <c r="I127" s="76" t="n"/>
+      <c r="J127" s="76" t="n"/>
+    </row>
+    <row r="128" ht="42" customHeight="1" s="85">
+      <c r="A128" s="52" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="B120" s="53">
-        <f>COUNTIF($B$121:$B$150,"Intangible")</f>
+      <c r="B128" s="53">
+        <f>COUNTIF($B$129:$B$158,"Intangible")</f>
         <v/>
       </c>
-      <c r="C120" s="54" t="n"/>
-      <c r="D120" s="54" t="n"/>
-      <c r="E120" s="54" t="n"/>
-      <c r="F120" s="55" t="n"/>
-      <c r="G120" s="66" t="n"/>
-      <c r="H120" s="67" t="n"/>
-      <c r="I120" s="67" t="n"/>
-      <c r="J120" s="67" t="n"/>
-    </row>
-    <row r="121" ht="28" customHeight="1" s="85">
-      <c r="A121" s="42" t="inlineStr">
+      <c r="C128" s="54" t="n"/>
+      <c r="D128" s="54" t="n"/>
+      <c r="E128" s="54" t="n"/>
+      <c r="F128" s="55" t="n"/>
+      <c r="G128" s="66" t="n"/>
+      <c r="H128" s="67" t="n"/>
+      <c r="I128" s="67" t="n"/>
+      <c r="J128" s="67" t="n"/>
+    </row>
+    <row r="129" ht="28" customHeight="1" s="85">
+      <c r="A129" s="42" t="inlineStr">
         <is>
           <t>All intangibles are limited to 1</t>
         </is>
       </c>
-      <c r="B121" s="22" t="inlineStr">
+      <c r="B129" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C121" s="23" t="inlineStr">
+      <c r="C129" s="23" t="inlineStr">
         <is>
           <t>Board-Crasher</t>
         </is>
       </c>
-      <c r="D121" s="6" t="inlineStr">
+      <c r="D129" s="6" t="inlineStr">
         <is>
           <t>SHOT +25% when shooting as your first action after a Rebound of your own miss.</t>
         </is>
       </c>
-      <c r="E121" s="7" t="n"/>
-      <c r="F121" s="50" t="n"/>
-      <c r="G121" s="70" t="n"/>
-      <c r="H121" s="71" t="n"/>
-      <c r="I121" s="71" t="n"/>
-      <c r="J121" s="71" t="n"/>
-    </row>
-    <row r="122" ht="28" customHeight="1" s="85">
-      <c r="A122" s="21" t="n"/>
-      <c r="B122" s="22" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C122" s="24" t="inlineStr">
-        <is>
-          <t>Catch &amp; Shoot Specialist</t>
-        </is>
-      </c>
-      <c r="D122" s="25" t="inlineStr">
-        <is>
-          <t>SHOT +25% when shooting as your first action after a Pass</t>
-        </is>
-      </c>
-      <c r="E122" s="26" t="n"/>
-      <c r="F122" s="50" t="n"/>
-      <c r="G122" s="72" t="n"/>
-      <c r="H122" s="71" t="n"/>
-      <c r="I122" s="71" t="n"/>
-      <c r="J122" s="71" t="n"/>
-    </row>
-    <row r="123" ht="56" customHeight="1" s="85">
-      <c r="A123" s="21" t="n"/>
-      <c r="B123" s="22" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C123" s="23" t="inlineStr">
-        <is>
-          <t>Clutch Gene</t>
-        </is>
-      </c>
-      <c r="D123" s="6" t="inlineStr">
-        <is>
-          <t>SHOT = 2X if you have 1 card or fewer in hand, or the Shot Clock is 03 or less</t>
-        </is>
-      </c>
-      <c r="E123" s="7" t="n"/>
-      <c r="F123" s="50" t="n"/>
-      <c r="G123" s="70" t="n"/>
-      <c r="H123" s="71" t="n"/>
-      <c r="I123" s="71" t="n"/>
-      <c r="J123" s="71" t="n"/>
-    </row>
-    <row r="124" ht="56" customHeight="1" s="85">
-      <c r="B124" s="0" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C124" s="0" t="inlineStr">
-        <is>
-          <t>Roswell Reach</t>
-        </is>
-      </c>
-      <c r="D124" s="0" t="inlineStr">
-        <is>
-          <t>All your Rebound bids of 1 or more count as 1 higher</t>
-        </is>
-      </c>
-    </row>
-    <row r="125" ht="28" customHeight="1" s="85">
-      <c r="A125" s="21" t="n"/>
-      <c r="B125" s="22" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C125" s="24" t="inlineStr">
-        <is>
-          <t>Floor General</t>
-        </is>
-      </c>
-      <c r="D125" s="25" t="inlineStr">
-        <is>
-          <t>You choose all targets of all kinds — card declarations, non auto-pass targets, and the rest. Not choices about a player's own card: which effect of a multi-effect card, or whether to feed a shot an extra discard</t>
-        </is>
-      </c>
-      <c r="E125" s="26" t="n"/>
-      <c r="F125" s="50" t="n"/>
-      <c r="G125" s="72" t="n"/>
-      <c r="H125" s="71" t="n"/>
-      <c r="I125" s="71" t="n"/>
-      <c r="J125" s="71" t="n"/>
-    </row>
-    <row r="126" ht="28" customHeight="1" s="85">
-      <c r="A126" s="21" t="n"/>
-      <c r="B126" s="22" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C126" s="23" t="inlineStr">
-        <is>
-          <t>Southpaw Shooter</t>
-        </is>
-      </c>
-      <c r="D126" s="6" t="inlineStr">
-        <is>
-          <t>SHOT gains and losses are reversed</t>
-        </is>
-      </c>
-      <c r="E126" s="6" t="n"/>
-      <c r="F126" s="51" t="n"/>
-      <c r="G126" s="70" t="n"/>
-      <c r="H126" s="71" t="n"/>
-      <c r="I126" s="71" t="n"/>
-      <c r="J126" s="71" t="n"/>
-    </row>
-    <row r="127" ht="28" customHeight="1" s="85">
-      <c r="A127" s="21" t="n"/>
-      <c r="B127" s="22" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C127" s="37" t="inlineStr">
-        <is>
-          <t>Freethrow Merchant</t>
-        </is>
-      </c>
-      <c r="D127" s="41" t="inlineStr">
-        <is>
-          <t>All Clamps on you grant 1 FT instead</t>
-        </is>
-      </c>
-      <c r="E127" s="26" t="n"/>
-      <c r="F127" s="50" t="n"/>
-      <c r="G127" s="77" t="n"/>
-      <c r="H127" s="71" t="n"/>
-      <c r="I127" s="71" t="n"/>
-      <c r="J127" s="71" t="n"/>
-    </row>
-    <row r="128" ht="28" customHeight="1" s="85">
-      <c r="A128" s="21" t="n"/>
-      <c r="B128" s="22" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C128" s="37" t="inlineStr">
-        <is>
-          <t>Generational Whistle</t>
-        </is>
-      </c>
-      <c r="D128" s="38" t="inlineStr">
-        <is>
-          <t>Take 1 additional FT</t>
-        </is>
-      </c>
-      <c r="E128" s="7" t="n"/>
-      <c r="F128" s="50" t="n"/>
-      <c r="G128" s="70" t="n"/>
-      <c r="H128" s="71" t="n"/>
-      <c r="I128" s="71" t="n"/>
-      <c r="J128" s="71" t="n"/>
-    </row>
-    <row r="129" ht="14" customHeight="1" s="85">
-      <c r="A129" s="21" t="n"/>
-      <c r="B129" s="22" t="inlineStr">
-        <is>
-          <t>Intangible</t>
-        </is>
-      </c>
-      <c r="C129" s="24" t="inlineStr">
-        <is>
-          <t>Gravity</t>
-        </is>
-      </c>
-      <c r="D129" s="25" t="inlineStr">
-        <is>
-          <t>All Clamps automatically apply to you. +1 AST whenever another player attempts a shot</t>
-        </is>
-      </c>
-      <c r="E129" s="26" t="n"/>
+      <c r="E129" s="7" t="n"/>
       <c r="F129" s="50" t="n"/>
-      <c r="G129" s="72" t="n"/>
+      <c r="G129" s="70" t="n"/>
       <c r="H129" s="71" t="n"/>
       <c r="I129" s="71" t="n"/>
       <c r="J129" s="71" t="n"/>
@@ -5625,78 +5646,63 @@
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C130" s="23" t="inlineStr">
-        <is>
-          <t>Great Conditioning</t>
-        </is>
-      </c>
-      <c r="D130" s="6" t="inlineStr">
-        <is>
-          <t>Immediately discard all Injuries you draw and draw a new card for each</t>
-        </is>
-      </c>
-      <c r="E130" s="7" t="n"/>
+      <c r="C130" s="24" t="inlineStr">
+        <is>
+          <t>Catch &amp; Shoot Specialist</t>
+        </is>
+      </c>
+      <c r="D130" s="25" t="inlineStr">
+        <is>
+          <t>SHOT +25% when shooting as your first action after a Pass</t>
+        </is>
+      </c>
+      <c r="E130" s="26" t="n"/>
       <c r="F130" s="50" t="n"/>
-      <c r="G130" s="70" t="inlineStr">
-        <is>
-          <t>Also discards any Injuries you already have (not on the card)</t>
-        </is>
-      </c>
+      <c r="G130" s="72" t="n"/>
       <c r="H130" s="71" t="n"/>
       <c r="I130" s="71" t="n"/>
       <c r="J130" s="71" t="n"/>
     </row>
-    <row r="131" ht="28" customHeight="1" s="85">
+    <row r="131" ht="56" customHeight="1" s="85">
       <c r="A131" s="21" t="n"/>
       <c r="B131" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C131" s="24" t="inlineStr">
-        <is>
-          <t>Hot Hand</t>
-        </is>
-      </c>
-      <c r="D131" s="25" t="inlineStr">
-        <is>
-          <t>SHOT +25% if you scored last round.</t>
-        </is>
-      </c>
-      <c r="E131" s="26" t="n"/>
+      <c r="C131" s="23" t="inlineStr">
+        <is>
+          <t>Clutch Gene</t>
+        </is>
+      </c>
+      <c r="D131" s="6" t="inlineStr">
+        <is>
+          <t>SHOT = 2X if you have 1 card or fewer in hand, or the Shot Clock is 03 or less</t>
+        </is>
+      </c>
+      <c r="E131" s="7" t="n"/>
       <c r="F131" s="50" t="n"/>
-      <c r="G131" s="72" t="n"/>
+      <c r="G131" s="70" t="n"/>
       <c r="H131" s="71" t="n"/>
       <c r="I131" s="71" t="n"/>
       <c r="J131" s="71" t="n"/>
     </row>
-    <row r="132" ht="28" customHeight="1" s="85">
-      <c r="A132" s="21" t="n"/>
-      <c r="B132" s="22" t="inlineStr">
+    <row r="132" ht="56" customHeight="1" s="85">
+      <c r="B132" s="0" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C132" s="23" t="inlineStr">
-        <is>
-          <t>Like That</t>
-        </is>
-      </c>
-      <c r="D132" s="38" t="inlineStr">
-        <is>
-          <t>Your SHOT % cannot be reduced</t>
-        </is>
-      </c>
-      <c r="E132" s="7" t="n"/>
-      <c r="F132" s="50" t="n"/>
-      <c r="G132" s="70" t="inlineStr">
-        <is>
-          <t>Variaball effects still lower SHOT: the ball is altered, not the player (not on the card)</t>
-        </is>
-      </c>
-      <c r="H132" s="71" t="n"/>
-      <c r="I132" s="71" t="n"/>
-      <c r="J132" s="71" t="n"/>
+      <c r="C132" s="0" t="inlineStr">
+        <is>
+          <t>Roswell Reach</t>
+        </is>
+      </c>
+      <c r="D132" s="0" t="inlineStr">
+        <is>
+          <t>All your Rebound bids of 1 or more count as 1 higher</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="28" customHeight="1" s="85">
       <c r="A133" s="21" t="n"/>
@@ -5707,17 +5713,17 @@
       </c>
       <c r="C133" s="24" t="inlineStr">
         <is>
-          <t>Park Shark</t>
+          <t>Floor General</t>
         </is>
       </c>
       <c r="D133" s="25" t="inlineStr">
         <is>
-          <t>SHOT +25%. Cannot play Move cards or shoot Threes</t>
+          <t>You choose all targets of all kinds — card declarations, non auto-pass targets, and the rest. Not choices about a player's own card: which effect of a multi-effect card, or whether to feed a shot an extra discard</t>
         </is>
       </c>
       <c r="E133" s="26" t="n"/>
       <c r="F133" s="50" t="n"/>
-      <c r="G133" s="73" t="n"/>
+      <c r="G133" s="72" t="n"/>
       <c r="H133" s="71" t="n"/>
       <c r="I133" s="71" t="n"/>
       <c r="J133" s="71" t="n"/>
@@ -5731,78 +5737,70 @@
       </c>
       <c r="C134" s="23" t="inlineStr">
         <is>
-          <t>Point God</t>
+          <t>Southpaw Shooter</t>
         </is>
       </c>
       <c r="D134" s="6" t="inlineStr">
         <is>
-          <t>Draw 1 card following each of your passes</t>
-        </is>
-      </c>
-      <c r="E134" s="7" t="n"/>
-      <c r="F134" s="50" t="n"/>
+          <t>SHOT gains and losses are reversed</t>
+        </is>
+      </c>
+      <c r="E134" s="6" t="n"/>
+      <c r="F134" s="51" t="n"/>
       <c r="G134" s="70" t="n"/>
       <c r="H134" s="71" t="n"/>
       <c r="I134" s="71" t="n"/>
       <c r="J134" s="71" t="n"/>
     </row>
-    <row r="135" ht="56" customHeight="1" s="85">
+    <row r="135" ht="28" customHeight="1" s="85">
       <c r="A135" s="21" t="n"/>
       <c r="B135" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C135" s="24" t="inlineStr">
-        <is>
-          <t>Shot Creator</t>
-        </is>
-      </c>
-      <c r="D135" s="25" t="inlineStr">
-        <is>
-          <t>Draw 1 additional card after every draw effect</t>
+      <c r="C135" s="37" t="inlineStr">
+        <is>
+          <t>Freethrow Merchant</t>
+        </is>
+      </c>
+      <c r="D135" s="41" t="inlineStr">
+        <is>
+          <t>All Clamps on you grant 1 FT instead</t>
         </is>
       </c>
       <c r="E135" s="26" t="n"/>
       <c r="F135" s="50" t="n"/>
-      <c r="G135" s="73" t="inlineStr">
-        <is>
-          <t>Triggers once per act of drawing: a Draw 2 still gives only 1 extra</t>
-        </is>
-      </c>
+      <c r="G135" s="77" t="n"/>
       <c r="H135" s="71" t="n"/>
       <c r="I135" s="71" t="n"/>
       <c r="J135" s="71" t="n"/>
     </row>
-    <row r="136" ht="56" customHeight="1" s="85">
+    <row r="136" ht="28" customHeight="1" s="85">
       <c r="A136" s="21" t="n"/>
       <c r="B136" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C136" s="23" t="inlineStr">
-        <is>
-          <t>Sixth Man</t>
-        </is>
-      </c>
-      <c r="D136" s="6" t="inlineStr">
-        <is>
-          <t>SHOT = 60% on any six: cards in hand, Shot Clock, shot of the round, or Score</t>
+      <c r="C136" s="37" t="inlineStr">
+        <is>
+          <t>Generational Whistle</t>
+        </is>
+      </c>
+      <c r="D136" s="38" t="inlineStr">
+        <is>
+          <t>Take 1 additional FT</t>
         </is>
       </c>
       <c r="E136" s="7" t="n"/>
       <c r="F136" s="50" t="n"/>
-      <c r="G136" s="70" t="inlineStr">
-        <is>
-          <t>A second SHOOT (60%) button beside Shoot, shown only on a six. Ignore it when SHOT is already higher</t>
-        </is>
-      </c>
+      <c r="G136" s="70" t="n"/>
       <c r="H136" s="71" t="n"/>
       <c r="I136" s="71" t="n"/>
       <c r="J136" s="71" t="n"/>
     </row>
-    <row r="137" ht="56" customHeight="1" s="85">
+    <row r="137" ht="14" customHeight="1" s="85">
       <c r="A137" s="21" t="n"/>
       <c r="B137" s="22" t="inlineStr">
         <is>
@@ -5811,12 +5809,12 @@
       </c>
       <c r="C137" s="24" t="inlineStr">
         <is>
-          <t>Sniper</t>
+          <t>Gravity</t>
         </is>
       </c>
       <c r="D137" s="25" t="inlineStr">
         <is>
-          <t>SHOT +25% when attempting a Three</t>
+          <t>All Clamps automatically apply to you. +1 AST whenever another player attempts a shot</t>
         </is>
       </c>
       <c r="E137" s="26" t="n"/>
@@ -5826,7 +5824,7 @@
       <c r="I137" s="71" t="n"/>
       <c r="J137" s="71" t="n"/>
     </row>
-    <row r="138" ht="56" customHeight="1" s="85">
+    <row r="138" ht="28" customHeight="1" s="85">
       <c r="A138" s="21" t="n"/>
       <c r="B138" s="22" t="inlineStr">
         <is>
@@ -5835,22 +5833,26 @@
       </c>
       <c r="C138" s="23" t="inlineStr">
         <is>
-          <t>Splash Cousin</t>
+          <t>Great Conditioning</t>
         </is>
       </c>
       <c r="D138" s="6" t="inlineStr">
         <is>
-          <t>SHOT = 100% when attempting a Three</t>
+          <t>Immediately discard all Injuries you draw and draw a new card for each</t>
         </is>
       </c>
       <c r="E138" s="7" t="n"/>
       <c r="F138" s="50" t="n"/>
-      <c r="G138" s="70" t="n"/>
+      <c r="G138" s="70" t="inlineStr">
+        <is>
+          <t>Also discards any Injuries you already have (not on the card)</t>
+        </is>
+      </c>
       <c r="H138" s="71" t="n"/>
       <c r="I138" s="71" t="n"/>
       <c r="J138" s="71" t="n"/>
     </row>
-    <row r="139" ht="56" customHeight="1" s="85">
+    <row r="139" ht="28" customHeight="1" s="85">
       <c r="A139" s="21" t="n"/>
       <c r="B139" s="22" t="inlineStr">
         <is>
@@ -5859,12 +5861,12 @@
       </c>
       <c r="C139" s="24" t="inlineStr">
         <is>
-          <t>Competitive</t>
+          <t>Hot Hand</t>
         </is>
       </c>
       <c r="D139" s="25" t="inlineStr">
         <is>
-          <t>All Clamps on you have no effect on SHOT %</t>
+          <t>SHOT +25% if you scored last round.</t>
         </is>
       </c>
       <c r="E139" s="26" t="n"/>
@@ -5874,7 +5876,7 @@
       <c r="I139" s="71" t="n"/>
       <c r="J139" s="71" t="n"/>
     </row>
-    <row r="140" ht="126" customHeight="1" s="85">
+    <row r="140" ht="28" customHeight="1" s="85">
       <c r="A140" s="21" t="n"/>
       <c r="B140" s="22" t="inlineStr">
         <is>
@@ -5883,26 +5885,26 @@
       </c>
       <c r="C140" s="23" t="inlineStr">
         <is>
-          <t>Lethal Shooter</t>
+          <t>Like That</t>
         </is>
       </c>
       <c r="D140" s="38" t="inlineStr">
         <is>
-          <t>SHOT = 100% when shooting as your first action after a Rebound of your own miss</t>
+          <t>Your SHOT % cannot be reduced</t>
         </is>
       </c>
       <c r="E140" s="7" t="n"/>
       <c r="F140" s="50" t="n"/>
       <c r="G140" s="70" t="inlineStr">
         <is>
-          <t>Special text: “I understand it now”</t>
+          <t>Variaball effects still lower SHOT: the ball is altered, not the player (not on the card)</t>
         </is>
       </c>
       <c r="H140" s="71" t="n"/>
       <c r="I140" s="71" t="n"/>
       <c r="J140" s="71" t="n"/>
     </row>
-    <row r="141" ht="70" customHeight="1" s="85">
+    <row r="141" ht="28" customHeight="1" s="85">
       <c r="A141" s="21" t="n"/>
       <c r="B141" s="22" t="inlineStr">
         <is>
@@ -5911,12 +5913,12 @@
       </c>
       <c r="C141" s="24" t="inlineStr">
         <is>
-          <t>Ball Pounder</t>
+          <t>Park Shark</t>
         </is>
       </c>
       <c r="D141" s="25" t="inlineStr">
         <is>
-          <t>Every Dribble draws 1 card but gives SHOT -10% and Shot Clock - 01</t>
+          <t>SHOT +25%. Cannot play Move cards or shoot Threes</t>
         </is>
       </c>
       <c r="E141" s="26" t="n"/>
@@ -5926,7 +5928,7 @@
       <c r="I141" s="71" t="n"/>
       <c r="J141" s="71" t="n"/>
     </row>
-    <row r="142" ht="56" customHeight="1" s="85">
+    <row r="142" ht="28" customHeight="1" s="85">
       <c r="A142" s="21" t="n"/>
       <c r="B142" s="22" t="inlineStr">
         <is>
@@ -5935,12 +5937,12 @@
       </c>
       <c r="C142" s="23" t="inlineStr">
         <is>
-          <t>Dirty Player</t>
-        </is>
-      </c>
-      <c r="D142" s="38" t="inlineStr">
-        <is>
-          <t>When sending Clamps, the clamped player discards 1 for each of your Clamps if they have any Injuries. Discard 1 whenever a Whistle triggers</t>
+          <t>Point God</t>
+        </is>
+      </c>
+      <c r="D142" s="6" t="inlineStr">
+        <is>
+          <t>Draw 1 card following each of your passes</t>
         </is>
       </c>
       <c r="E142" s="7" t="n"/>
@@ -5950,35 +5952,35 @@
       <c r="I142" s="71" t="n"/>
       <c r="J142" s="71" t="n"/>
     </row>
-    <row r="143" s="85">
+    <row r="143" ht="56" customHeight="1" s="85">
       <c r="A143" s="21" t="n"/>
       <c r="B143" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C143" s="23" t="inlineStr">
-        <is>
-          <t>Free Agent</t>
-        </is>
-      </c>
-      <c r="D143" s="38" t="inlineStr">
-        <is>
-          <t>Discard your hand. Play a card at random from a player of your choosing (they keep it)</t>
-        </is>
-      </c>
-      <c r="E143" s="7" t="n"/>
+      <c r="C143" s="24" t="inlineStr">
+        <is>
+          <t>Shot Creator</t>
+        </is>
+      </c>
+      <c r="D143" s="25" t="inlineStr">
+        <is>
+          <t>Draw 1 additional card after every draw effect</t>
+        </is>
+      </c>
+      <c r="E143" s="26" t="n"/>
       <c r="F143" s="50" t="n"/>
-      <c r="G143" s="70" t="inlineStr">
-        <is>
-          <t>Low priority to bring back. The discard waits for the draw chain to finish. Target is shuffled first and is affected by Floor General. Your own draws are kept. All-0 rebounds are yours; otherwise you cannot bid  [OUT OF THE DECK — the borrow button throws the answer away; back when it routes through Move.borrow]</t>
+      <c r="G143" s="73" t="inlineStr">
+        <is>
+          <t>Triggers once per act of drawing: a Draw 2 still gives only 1 extra</t>
         </is>
       </c>
       <c r="H143" s="71" t="n"/>
       <c r="I143" s="71" t="n"/>
       <c r="J143" s="71" t="n"/>
     </row>
-    <row r="144" s="85">
+    <row r="144" ht="56" customHeight="1" s="85">
       <c r="A144" s="21" t="n"/>
       <c r="B144" s="22" t="inlineStr">
         <is>
@@ -5987,50 +5989,50 @@
       </c>
       <c r="C144" s="23" t="inlineStr">
         <is>
-          <t>Franchise Player</t>
-        </is>
-      </c>
-      <c r="D144" s="38" t="inlineStr">
-        <is>
-          <t>When passing, choose 1 of the new player's Intangibles or a card in their hand for them to discard</t>
+          <t>Sixth Man</t>
+        </is>
+      </c>
+      <c r="D144" s="6" t="inlineStr">
+        <is>
+          <t>SHOT = 60% on any six: cards in hand, Shot Clock, shot of the round, or Score</t>
         </is>
       </c>
       <c r="E144" s="7" t="n"/>
       <c r="F144" s="50" t="n"/>
-      <c r="G144" s="70" t="n"/>
+      <c r="G144" s="70" t="inlineStr">
+        <is>
+          <t>A second SHOOT (60%) button beside Shoot, shown only on a six. Ignore it when SHOT is already higher</t>
+        </is>
+      </c>
       <c r="H144" s="71" t="n"/>
       <c r="I144" s="71" t="n"/>
       <c r="J144" s="71" t="n"/>
     </row>
-    <row r="145" s="85">
+    <row r="145" ht="56" customHeight="1" s="85">
       <c r="A145" s="21" t="n"/>
       <c r="B145" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C145" s="23" t="inlineStr">
-        <is>
-          <t>Fundamentalist</t>
-        </is>
-      </c>
-      <c r="D145" s="38" t="inlineStr">
-        <is>
-          <t>No Special Moves. Each Move once a turn. Swings, Skip Pass and Dribble are never spent. Discards the current ball</t>
-        </is>
-      </c>
-      <c r="E145" s="7" t="n"/>
+      <c r="C145" s="24" t="inlineStr">
+        <is>
+          <t>Sniper</t>
+        </is>
+      </c>
+      <c r="D145" s="25" t="inlineStr">
+        <is>
+          <t>SHOT +25% when attempting a Three</t>
+        </is>
+      </c>
+      <c r="E145" s="26" t="n"/>
       <c r="F145" s="50" t="n"/>
-      <c r="G145" s="70" t="inlineStr">
-        <is>
-          <t>The ball is discarded once, on activation</t>
-        </is>
-      </c>
+      <c r="G145" s="72" t="n"/>
       <c r="H145" s="71" t="n"/>
       <c r="I145" s="71" t="n"/>
       <c r="J145" s="71" t="n"/>
     </row>
-    <row r="146" s="85">
+    <row r="146" ht="56" customHeight="1" s="85">
       <c r="A146" s="21" t="n"/>
       <c r="B146" s="22" t="inlineStr">
         <is>
@@ -6039,282 +6041,277 @@
       </c>
       <c r="C146" s="23" t="inlineStr">
         <is>
-          <t>Moves At Own Pace</t>
-        </is>
-      </c>
-      <c r="D146" s="38" t="inlineStr">
-        <is>
-          <t>Cannot be called for Traveling or Shot Clock violations</t>
+          <t>Splash Cousin</t>
+        </is>
+      </c>
+      <c r="D146" s="6" t="inlineStr">
+        <is>
+          <t>SHOT = 100% when attempting a Three</t>
         </is>
       </c>
       <c r="E146" s="7" t="n"/>
-      <c r="F146" s="50" t="n">
-        <v>1</v>
-      </c>
+      <c r="F146" s="50" t="n"/>
       <c r="G146" s="70" t="n"/>
       <c r="H146" s="71" t="n"/>
       <c r="I146" s="71" t="n"/>
       <c r="J146" s="71" t="n"/>
     </row>
-    <row r="147" s="85">
+    <row r="147" ht="56" customHeight="1" s="85">
       <c r="A147" s="21" t="n"/>
       <c r="B147" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C147" s="23" t="inlineStr">
-        <is>
-          <t>Equalizer</t>
-        </is>
-      </c>
-      <c r="D147" s="38" t="inlineStr">
-        <is>
-          <t>You may Discard this card when shooting: SHOT = 100%. All players' pts become your new total pts.</t>
-        </is>
-      </c>
-      <c r="E147" s="7" t="n"/>
+      <c r="C147" s="24" t="inlineStr">
+        <is>
+          <t>Competitive</t>
+        </is>
+      </c>
+      <c r="D147" s="25" t="inlineStr">
+        <is>
+          <t>All Clamps on you have no effect on SHOT %</t>
+        </is>
+      </c>
+      <c r="E147" s="26" t="n"/>
       <c r="F147" s="50" t="n"/>
-      <c r="G147" s="70" t="inlineStr">
-        <is>
-          <t>The points change comes after the make</t>
-        </is>
-      </c>
+      <c r="G147" s="72" t="n"/>
       <c r="H147" s="71" t="n"/>
       <c r="I147" s="71" t="n"/>
       <c r="J147" s="71" t="n"/>
     </row>
-    <row r="148" s="85">
-      <c r="A148" s="27" t="n"/>
-      <c r="B148" s="28" t="inlineStr">
+    <row r="148" ht="126" customHeight="1" s="85">
+      <c r="A148" s="21" t="n"/>
+      <c r="B148" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C148" s="56" t="inlineStr">
-        <is>
-          <t>Varsitile</t>
-        </is>
-      </c>
-      <c r="D148" s="63" t="inlineStr">
-        <is>
-          <t>You can play more than 1 Varena and Variaball per turn. Once per possession, you can exchange the Varena and/or ball for one in the Discards</t>
-        </is>
-      </c>
-      <c r="E148" s="58" t="n"/>
-      <c r="F148" s="61" t="n"/>
-      <c r="G148" s="75" t="inlineStr">
-        <is>
-          <t>One use can exchange both</t>
-        </is>
-      </c>
-      <c r="H148" s="76" t="n"/>
-      <c r="I148" s="76" t="n"/>
-      <c r="J148" s="76" t="n"/>
-    </row>
-    <row r="149" s="85">
-      <c r="A149" s="27" t="n"/>
-      <c r="B149" s="28" t="inlineStr">
+      <c r="C148" s="23" t="inlineStr">
+        <is>
+          <t>Lethal Shooter</t>
+        </is>
+      </c>
+      <c r="D148" s="38" t="inlineStr">
+        <is>
+          <t>SHOT = 100% when shooting as your first action after a Rebound of your own miss</t>
+        </is>
+      </c>
+      <c r="E148" s="7" t="n"/>
+      <c r="F148" s="50" t="n"/>
+      <c r="G148" s="70" t="inlineStr">
+        <is>
+          <t>Special text: “I understand it now”</t>
+        </is>
+      </c>
+      <c r="H148" s="71" t="n"/>
+      <c r="I148" s="71" t="n"/>
+      <c r="J148" s="71" t="n"/>
+    </row>
+    <row r="149" ht="70" customHeight="1" s="85">
+      <c r="A149" s="21" t="n"/>
+      <c r="B149" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C149" s="56" t="inlineStr">
-        <is>
-          <t>Brawl Handler</t>
-        </is>
-      </c>
-      <c r="D149" s="63" t="inlineStr">
-        <is>
-          <t>Remove all your Clamps when you change the ball</t>
-        </is>
-      </c>
-      <c r="E149" s="58" t="n"/>
-      <c r="F149" s="61" t="n"/>
-      <c r="G149" s="75" t="n"/>
-      <c r="H149" s="76" t="n"/>
-    </row>
-    <row r="150" s="85">
-      <c r="A150" s="27" t="n"/>
-      <c r="B150" s="28" t="inlineStr">
+      <c r="C149" s="24" t="inlineStr">
+        <is>
+          <t>Ball Pounder</t>
+        </is>
+      </c>
+      <c r="D149" s="25" t="inlineStr">
+        <is>
+          <t>Every Dribble draws 1 card but gives SHOT -10% and Shot Clock - 01</t>
+        </is>
+      </c>
+      <c r="E149" s="26" t="n"/>
+      <c r="F149" s="50" t="n"/>
+      <c r="G149" s="73" t="n"/>
+      <c r="H149" s="71" t="n"/>
+      <c r="I149" s="71" t="n"/>
+      <c r="J149" s="71" t="n"/>
+    </row>
+    <row r="150" ht="56" customHeight="1" s="85">
+      <c r="A150" s="21" t="n"/>
+      <c r="B150" s="22" t="inlineStr">
         <is>
           <t>Intangible</t>
         </is>
       </c>
-      <c r="C150" s="56" t="inlineStr">
-        <is>
-          <t>Baller</t>
-        </is>
-      </c>
-      <c r="D150" s="63" t="inlineStr">
-        <is>
-          <t>Draw 1 card each time you change the ball</t>
-        </is>
-      </c>
-      <c r="E150" s="58" t="n"/>
-      <c r="F150" s="61" t="n"/>
-      <c r="G150" s="75" t="n"/>
-      <c r="H150" s="76" t="n"/>
-    </row>
-    <row r="151" ht="42" customHeight="1" s="85">
-      <c r="A151" s="52" t="inlineStr">
-        <is>
-          <t>Varena</t>
-        </is>
-      </c>
-      <c r="B151" s="53">
-        <f>COUNTIF($B$152:$B$181,"Varena")</f>
-        <v/>
-      </c>
-      <c r="C151" s="54" t="n"/>
-      <c r="D151" s="54" t="n"/>
-      <c r="E151" s="54" t="n"/>
-      <c r="F151" s="55" t="n"/>
-      <c r="G151" s="66" t="n"/>
-      <c r="H151" s="67" t="n"/>
-      <c r="I151" s="67" t="n"/>
-      <c r="J151" s="67" t="n"/>
+      <c r="C150" s="23" t="inlineStr">
+        <is>
+          <t>Dirty Player</t>
+        </is>
+      </c>
+      <c r="D150" s="38" t="inlineStr">
+        <is>
+          <t>When sending Clamps, the clamped player discards 1 for each of your Clamps if they have any Injuries. Discard 1 whenever a Whistle triggers</t>
+        </is>
+      </c>
+      <c r="E150" s="7" t="n"/>
+      <c r="F150" s="50" t="n"/>
+      <c r="G150" s="70" t="n"/>
+      <c r="H150" s="71" t="n"/>
+      <c r="I150" s="71" t="n"/>
+      <c r="J150" s="71" t="n"/>
+    </row>
+    <row r="151" s="85">
+      <c r="A151" s="21" t="n"/>
+      <c r="B151" s="22" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C151" s="23" t="inlineStr">
+        <is>
+          <t>Free Agent</t>
+        </is>
+      </c>
+      <c r="D151" s="38" t="inlineStr">
+        <is>
+          <t>Discard your hand. Play a card at random from a player of your choosing (they keep it)</t>
+        </is>
+      </c>
+      <c r="E151" s="7" t="n"/>
+      <c r="F151" s="50" t="n"/>
+      <c r="G151" s="70" t="inlineStr">
+        <is>
+          <t>Low priority to bring back. The discard waits for the draw chain to finish. Target is shuffled first and is affected by Floor General. Your own draws are kept. All-0 rebounds are yours; otherwise you cannot bid  [OUT OF THE DECK — the borrow button throws the answer away; back when it routes through Move.borrow]</t>
+        </is>
+      </c>
+      <c r="H151" s="71" t="n"/>
+      <c r="I151" s="71" t="n"/>
+      <c r="J151" s="71" t="n"/>
     </row>
     <row r="152" s="85">
-      <c r="A152" s="27" t="n"/>
-      <c r="B152" s="28" t="inlineStr">
-        <is>
-          <t>Varena</t>
-        </is>
-      </c>
-      <c r="C152" s="56" t="inlineStr">
-        <is>
-          <t>Cardwood</t>
-        </is>
-      </c>
-      <c r="D152" s="63" t="inlineStr">
-        <is>
-          <t>Changes the court back to basic</t>
-        </is>
-      </c>
-      <c r="E152" s="58" t="n"/>
-      <c r="F152" s="61" t="n">
-        <v>5</v>
-      </c>
-      <c r="G152" s="75" t="inlineStr">
-        <is>
-          <t>Also the floor every game opens on, before anybody plays a Varena over it</t>
-        </is>
-      </c>
-      <c r="H152" s="76" t="n"/>
-      <c r="I152" s="76" t="n"/>
-      <c r="J152" s="76" t="n"/>
+      <c r="A152" s="21" t="n"/>
+      <c r="B152" s="22" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C152" s="23" t="inlineStr">
+        <is>
+          <t>Franchise Player</t>
+        </is>
+      </c>
+      <c r="D152" s="38" t="inlineStr">
+        <is>
+          <t>When passing, choose 1 of the new player's Intangibles or a card in their hand for them to discard</t>
+        </is>
+      </c>
+      <c r="E152" s="7" t="n"/>
+      <c r="F152" s="50" t="n"/>
+      <c r="G152" s="70" t="n"/>
+      <c r="H152" s="71" t="n"/>
+      <c r="I152" s="71" t="n"/>
+      <c r="J152" s="71" t="n"/>
     </row>
     <row r="153" s="85">
-      <c r="A153" s="27" t="n"/>
-      <c r="B153" s="28" t="inlineStr">
-        <is>
-          <t>Varena</t>
-        </is>
-      </c>
-      <c r="C153" s="56" t="inlineStr">
-        <is>
-          <t>Prime Parquet</t>
-        </is>
-      </c>
-      <c r="D153" s="63" t="inlineStr">
-        <is>
-          <t>SHOT +20%</t>
-        </is>
-      </c>
-      <c r="E153" s="58" t="n"/>
-      <c r="F153" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="G153" s="75" t="n"/>
-      <c r="H153" s="76" t="n"/>
-      <c r="I153" s="76" t="n"/>
-      <c r="J153" s="76" t="n"/>
+      <c r="A153" s="21" t="n"/>
+      <c r="B153" s="22" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C153" s="23" t="inlineStr">
+        <is>
+          <t>Fundamentalist</t>
+        </is>
+      </c>
+      <c r="D153" s="38" t="inlineStr">
+        <is>
+          <t>No Special Moves. Each Move once a turn. Swings, Skip Pass and Dribble are never spent. Discards the current ball</t>
+        </is>
+      </c>
+      <c r="E153" s="7" t="n"/>
+      <c r="F153" s="50" t="n"/>
+      <c r="G153" s="70" t="inlineStr">
+        <is>
+          <t>The ball is discarded once, on activation</t>
+        </is>
+      </c>
+      <c r="H153" s="71" t="n"/>
+      <c r="I153" s="71" t="n"/>
+      <c r="J153" s="71" t="n"/>
     </row>
     <row r="154" s="85">
-      <c r="A154" s="27" t="n"/>
-      <c r="B154" s="28" t="inlineStr">
-        <is>
-          <t>Varena</t>
-        </is>
-      </c>
-      <c r="C154" s="56" t="inlineStr">
-        <is>
-          <t>Lacktop</t>
-        </is>
-      </c>
-      <c r="D154" s="63" t="inlineStr">
-        <is>
-          <t>SHOT -20%</t>
-        </is>
-      </c>
-      <c r="E154" s="58" t="n"/>
-      <c r="F154" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="G154" s="75" t="inlineStr">
-        <is>
-          <t>Always Prime Parquet's opposite</t>
-        </is>
-      </c>
-      <c r="H154" s="76" t="n"/>
-      <c r="I154" s="76" t="n"/>
-      <c r="J154" s="76" t="n"/>
+      <c r="A154" s="21" t="n"/>
+      <c r="B154" s="22" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C154" s="23" t="inlineStr">
+        <is>
+          <t>Moves At Own Pace</t>
+        </is>
+      </c>
+      <c r="D154" s="38" t="inlineStr">
+        <is>
+          <t>Cannot be called for Traveling or Shot Clock violations</t>
+        </is>
+      </c>
+      <c r="E154" s="7" t="n"/>
+      <c r="F154" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G154" s="70" t="n"/>
+      <c r="H154" s="71" t="n"/>
+      <c r="I154" s="71" t="n"/>
+      <c r="J154" s="71" t="n"/>
     </row>
     <row r="155" s="85">
-      <c r="A155" s="27" t="n"/>
-      <c r="B155" s="28" t="inlineStr">
-        <is>
-          <t>Varena</t>
-        </is>
-      </c>
-      <c r="C155" s="56" t="inlineStr">
-        <is>
-          <t>Smacktop</t>
-        </is>
-      </c>
-      <c r="D155" s="63" t="inlineStr">
-        <is>
-          <t>Clear All Whistles. Whistles Cannot Be Played. All Clamps are enhanced</t>
-        </is>
-      </c>
-      <c r="E155" s="58" t="n"/>
-      <c r="F155" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="G155" s="75" t="inlineStr">
-        <is>
-          <t>Enhanced: +10% more reduction, one more card discarded, one more card locked</t>
-        </is>
-      </c>
-      <c r="H155" s="76" t="n"/>
-      <c r="I155" s="76" t="n"/>
-      <c r="J155" s="76" t="n"/>
+      <c r="A155" s="21" t="n"/>
+      <c r="B155" s="22" t="inlineStr">
+        <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C155" s="23" t="inlineStr">
+        <is>
+          <t>Equalizer</t>
+        </is>
+      </c>
+      <c r="D155" s="38" t="inlineStr">
+        <is>
+          <t>You may Discard this card when shooting: SHOT = 100%. All players' pts become your new total pts.</t>
+        </is>
+      </c>
+      <c r="E155" s="7" t="n"/>
+      <c r="F155" s="50" t="n"/>
+      <c r="G155" s="70" t="inlineStr">
+        <is>
+          <t>The points change comes after the make</t>
+        </is>
+      </c>
+      <c r="H155" s="71" t="n"/>
+      <c r="I155" s="71" t="n"/>
+      <c r="J155" s="71" t="n"/>
     </row>
     <row r="156" s="85">
       <c r="A156" s="27" t="n"/>
       <c r="B156" s="28" t="inlineStr">
         <is>
-          <t>Varena</t>
+          <t>Intangible</t>
         </is>
       </c>
       <c r="C156" s="56" t="inlineStr">
         <is>
-          <t>Boarder Court</t>
+          <t>Varsitile</t>
         </is>
       </c>
       <c r="D156" s="63" t="inlineStr">
         <is>
-          <t>Off your own miss, your Rebound bid counts as one card more</t>
+          <t>You can play more than 1 Varena and Variaball per turn. Once per possession, you can exchange the Varena and/or ball for one in the Discards</t>
         </is>
       </c>
       <c r="E156" s="58" t="n"/>
-      <c r="F156" s="61" t="n">
-        <v>1</v>
-      </c>
+      <c r="F156" s="61" t="n"/>
       <c r="G156" s="75" t="inlineStr">
         <is>
-          <t>Still needs a bid of at least one</t>
+          <t>One use can exchange both</t>
         </is>
       </c>
       <c r="H156" s="76" t="n"/>
@@ -6325,91 +6322,64 @@
       <c r="A157" s="27" t="n"/>
       <c r="B157" s="28" t="inlineStr">
         <is>
-          <t>Varena</t>
+          <t>Intangible</t>
         </is>
       </c>
       <c r="C157" s="56" t="inlineStr">
         <is>
-          <t>Dim Dome</t>
+          <t>Brawl Handler</t>
         </is>
       </c>
       <c r="D157" s="63" t="inlineStr">
         <is>
-          <t>SHOT is hidden from everyone but the ball holder</t>
+          <t>Remove all your Clamps when you change the ball</t>
         </is>
       </c>
       <c r="E157" s="58" t="n"/>
-      <c r="F157" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="G157" s="75" t="inlineStr">
-        <is>
-          <t>On a table, flip the % device face down</t>
-        </is>
-      </c>
+      <c r="F157" s="61" t="n"/>
+      <c r="G157" s="75" t="n"/>
       <c r="H157" s="76" t="n"/>
-      <c r="I157" s="76" t="n"/>
-      <c r="J157" s="76" t="n"/>
     </row>
     <row r="158" s="85">
       <c r="A158" s="27" t="n"/>
       <c r="B158" s="28" t="inlineStr">
         <is>
+          <t>Intangible</t>
+        </is>
+      </c>
+      <c r="C158" s="56" t="inlineStr">
+        <is>
+          <t>Baller</t>
+        </is>
+      </c>
+      <c r="D158" s="63" t="inlineStr">
+        <is>
+          <t>Draw 1 card each time you change the ball</t>
+        </is>
+      </c>
+      <c r="E158" s="58" t="n"/>
+      <c r="F158" s="61" t="n"/>
+      <c r="G158" s="75" t="n"/>
+      <c r="H158" s="76" t="n"/>
+    </row>
+    <row r="159" ht="42" customHeight="1" s="85">
+      <c r="A159" s="52" t="inlineStr">
+        <is>
           <t>Varena</t>
         </is>
       </c>
-      <c r="C158" s="56" t="inlineStr">
-        <is>
-          <t>Tri-hard Tiling</t>
-        </is>
-      </c>
-      <c r="D158" s="63" t="inlineStr">
-        <is>
-          <t>Hand limit 3</t>
-        </is>
-      </c>
-      <c r="E158" s="58" t="n"/>
-      <c r="F158" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="G158" s="75" t="inlineStr">
-        <is>
-          <t>Hands over 3 are cut to 3 when it lands (owner picks). A draw into a hand of 3 is discarded</t>
-        </is>
-      </c>
-      <c r="H158" s="76" t="n"/>
-      <c r="I158" s="76" t="n"/>
-      <c r="J158" s="76" t="n"/>
-    </row>
-    <row r="159" s="85">
-      <c r="A159" s="27" t="n"/>
-      <c r="B159" s="28" t="inlineStr">
-        <is>
-          <t>Varena</t>
-        </is>
-      </c>
-      <c r="C159" s="56" t="inlineStr">
-        <is>
-          <t>Policeum</t>
-        </is>
-      </c>
-      <c r="D159" s="63" t="inlineStr">
-        <is>
-          <t>Referees do not leave once triggered</t>
-        </is>
-      </c>
-      <c r="E159" s="58" t="n"/>
-      <c r="F159" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="G159" s="75" t="inlineStr">
-        <is>
-          <t>A called referee stays until the floor changes. The 3-ref cap bounds it</t>
-        </is>
-      </c>
-      <c r="H159" s="76" t="n"/>
-      <c r="I159" s="76" t="n"/>
-      <c r="J159" s="76" t="n"/>
+      <c r="B159" s="53">
+        <f>COUNTIF($B$160:$B$189,"Varena")</f>
+        <v/>
+      </c>
+      <c r="C159" s="54" t="n"/>
+      <c r="D159" s="54" t="n"/>
+      <c r="E159" s="54" t="n"/>
+      <c r="F159" s="55" t="n"/>
+      <c r="G159" s="66" t="n"/>
+      <c r="H159" s="67" t="n"/>
+      <c r="I159" s="67" t="n"/>
+      <c r="J159" s="67" t="n"/>
     </row>
     <row r="160" s="85">
       <c r="A160" s="27" t="n"/>
@@ -6420,21 +6390,21 @@
       </c>
       <c r="C160" s="56" t="inlineStr">
         <is>
-          <t>Kiddie Court</t>
+          <t>Cardwood</t>
         </is>
       </c>
       <c r="D160" s="63" t="inlineStr">
         <is>
-          <t>SHOT +10%. Dunks +10%. Three-point shots cannot be attempted.</t>
+          <t>Changes the court back to basic</t>
         </is>
       </c>
       <c r="E160" s="58" t="n"/>
       <c r="F160" s="61" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G160" s="75" t="inlineStr">
         <is>
-          <t>Shuts off every card that makes a three (Kick-Out)</t>
+          <t>Also the floor every game opens on, before anybody plays a Varena over it</t>
         </is>
       </c>
       <c r="H160" s="76" t="n"/>
@@ -6450,23 +6420,19 @@
       </c>
       <c r="C161" s="56" t="inlineStr">
         <is>
-          <t>Recharging Resin</t>
+          <t>Prime Parquet</t>
         </is>
       </c>
       <c r="D161" s="63" t="inlineStr">
         <is>
-          <t>Everyone refills to a hand of 5 at the start of their possession</t>
+          <t>SHOT +20%</t>
         </is>
       </c>
       <c r="E161" s="58" t="n"/>
       <c r="F161" s="61" t="n">
         <v>3</v>
       </c>
-      <c r="G161" s="75" t="inlineStr">
-        <is>
-          <t>After the draw for turn</t>
-        </is>
-      </c>
+      <c r="G161" s="75" t="n"/>
       <c r="H161" s="76" t="n"/>
       <c r="I161" s="76" t="n"/>
       <c r="J161" s="76" t="n"/>
@@ -6480,12 +6446,12 @@
       </c>
       <c r="C162" s="56" t="inlineStr">
         <is>
-          <t>Contact Court</t>
+          <t>Lacktop</t>
         </is>
       </c>
       <c r="D162" s="63" t="inlineStr">
         <is>
-          <t>Being clamped: take 1 FT. The Clamp still lands</t>
+          <t>SHOT -20%</t>
         </is>
       </c>
       <c r="E162" s="58" t="n"/>
@@ -6494,7 +6460,7 @@
       </c>
       <c r="G162" s="75" t="inlineStr">
         <is>
-          <t>One free throw however many Clamps land</t>
+          <t>Always Prime Parquet's opposite</t>
         </is>
       </c>
       <c r="H162" s="76" t="n"/>
@@ -6510,21 +6476,21 @@
       </c>
       <c r="C163" s="56" t="inlineStr">
         <is>
-          <t>MVPiquia</t>
+          <t>Smacktop</t>
         </is>
       </c>
       <c r="D163" s="63" t="inlineStr">
         <is>
-          <t>The highest scorer refills to 5 at the start of their possession</t>
+          <t>Clear All Whistles. Whistles Cannot Be Played. All Clamps are enhanced</t>
         </is>
       </c>
       <c r="E163" s="58" t="n"/>
       <c r="F163" s="61" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G163" s="75" t="inlineStr">
         <is>
-          <t>A tie for the lead counts</t>
+          <t>Enhanced: +10% more reduction, one more card discarded, one more card locked</t>
         </is>
       </c>
       <c r="H163" s="76" t="n"/>
@@ -6540,19 +6506,23 @@
       </c>
       <c r="C164" s="56" t="inlineStr">
         <is>
-          <t>Polypaypylene</t>
+          <t>Boarder Court</t>
         </is>
       </c>
       <c r="D164" s="63" t="inlineStr">
         <is>
-          <t>Making a shot: Draw 3</t>
+          <t>Off your own miss, your Rebound bid counts as one card more</t>
         </is>
       </c>
       <c r="E164" s="58" t="n"/>
       <c r="F164" s="61" t="n">
         <v>1</v>
       </c>
-      <c r="G164" s="75" t="n"/>
+      <c r="G164" s="75" t="inlineStr">
+        <is>
+          <t>Still needs a bid of at least one</t>
+        </is>
+      </c>
       <c r="H164" s="76" t="n"/>
       <c r="I164" s="76" t="n"/>
       <c r="J164" s="76" t="n"/>
@@ -6566,21 +6536,21 @@
       </c>
       <c r="C165" s="56" t="inlineStr">
         <is>
-          <t>Recoverena</t>
+          <t>Dim Dome</t>
         </is>
       </c>
       <c r="D165" s="63" t="inlineStr">
         <is>
-          <t>Discard all Injuries. A new Injury is discarded, and that player draws 1</t>
+          <t>SHOT is hidden from everyone but the ball holder</t>
         </is>
       </c>
       <c r="E165" s="58" t="n"/>
       <c r="F165" s="61" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G165" s="75" t="inlineStr">
         <is>
-          <t>Every player's Injuries go when it lands</t>
+          <t>On a table, flip the % device face down</t>
         </is>
       </c>
       <c r="H165" s="76" t="n"/>
@@ -6596,21 +6566,21 @@
       </c>
       <c r="C166" s="56" t="inlineStr">
         <is>
-          <t>Carousel Court</t>
+          <t>Tri-hard Tiling</t>
         </is>
       </c>
       <c r="D166" s="63" t="inlineStr">
         <is>
-          <t>Declare left or right. Every possession, hands move one seat that way</t>
+          <t>Hand limit 3</t>
         </is>
       </c>
       <c r="E166" s="58" t="n"/>
       <c r="F166" s="61" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G166" s="75" t="inlineStr">
         <is>
-          <t>Declared by whoever plays it</t>
+          <t>Hands over 3 are cut to 3 when it lands (owner picks). A draw into a hand of 3 is discarded</t>
         </is>
       </c>
       <c r="H166" s="76" t="n"/>
@@ -6621,26 +6591,26 @@
       <c r="A167" s="27" t="n"/>
       <c r="B167" s="28" t="inlineStr">
         <is>
-          <t>Varena</t>
+          <t>Retired Varena</t>
         </is>
       </c>
       <c r="C167" s="56" t="inlineStr">
         <is>
-          <t>Traderous Tarmac</t>
+          <t>Policeum</t>
         </is>
       </c>
       <c r="D167" s="63" t="inlineStr">
         <is>
-          <t>During your turn, hand off any number of the Clamps on you to other players</t>
+          <t>Referees do not leave once triggered</t>
         </is>
       </c>
       <c r="E167" s="58" t="n"/>
       <c r="F167" s="61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G167" s="75" t="inlineStr">
         <is>
-          <t>The player assigns each Clamp: all to one player, one each, or any split</t>
+          <t>Out of the deck (2026-09-15): its referees could lock a game into a loop</t>
         </is>
       </c>
       <c r="H167" s="76" t="n"/>
@@ -6656,12 +6626,12 @@
       </c>
       <c r="C168" s="56" t="inlineStr">
         <is>
-          <t>Clearcoat Court</t>
+          <t>Kiddie Court</t>
         </is>
       </c>
       <c r="D168" s="63" t="inlineStr">
         <is>
-          <t>Every possession: clear all referees, Clamps, Injuries and Intangibles</t>
+          <t>SHOT +10%. Dunks +10%. Three-point shots cannot be attempted.</t>
         </is>
       </c>
       <c r="E168" s="58" t="n"/>
@@ -6670,7 +6640,7 @@
       </c>
       <c r="G168" s="75" t="inlineStr">
         <is>
-          <t>Standing Clamps only; Clamps still in the air land after the wipe</t>
+          <t>Shuts off every card that makes a three (Kick-Out)</t>
         </is>
       </c>
       <c r="H168" s="76" t="n"/>
@@ -6686,19 +6656,23 @@
       </c>
       <c r="C169" s="56" t="inlineStr">
         <is>
-          <t>Malice Palace</t>
+          <t>Recharging Resin</t>
         </is>
       </c>
       <c r="D169" s="63" t="inlineStr">
         <is>
-          <t>At the start of your possession, before your draw: discard your hand</t>
+          <t>Everyone refills to a hand of 5 at the start of their possession</t>
         </is>
       </c>
       <c r="E169" s="58" t="n"/>
       <c r="F169" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="G169" s="75" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="G169" s="75" t="inlineStr">
+        <is>
+          <t>After the draw for turn</t>
+        </is>
+      </c>
       <c r="H169" s="76" t="n"/>
       <c r="I169" s="76" t="n"/>
       <c r="J169" s="76" t="n"/>
@@ -6712,14 +6686,12 @@
       </c>
       <c r="C170" s="56" t="inlineStr">
         <is>
-          <t>Turnstile Tile</t>
+          <t>Contact Court</t>
         </is>
       </c>
       <c r="D170" s="63" t="inlineStr">
         <is>
-          <t>Upright: SHOT +25%
-Reversed: SHOT -25%
-Turn this card at the start of each possession</t>
+          <t>Being clamped: take 1 FT. The Clamp still lands</t>
         </is>
       </c>
       <c r="E170" s="58" t="n"/>
@@ -6728,7 +6700,7 @@
       </c>
       <c r="G170" s="75" t="inlineStr">
         <is>
-          <t>+25% the possession it lands</t>
+          <t>One free throw however many Clamps land</t>
         </is>
       </c>
       <c r="H170" s="76" t="n"/>
@@ -6744,19 +6716,23 @@
       </c>
       <c r="C171" s="56" t="inlineStr">
         <is>
-          <t>Roleplayer Polymer</t>
+          <t>MVPiquia</t>
         </is>
       </c>
       <c r="D171" s="63" t="inlineStr">
         <is>
-          <t>Every possession, everyone but the turn player draws 1</t>
+          <t>The highest scorer refills to 5 at the start of their possession</t>
         </is>
       </c>
       <c r="E171" s="58" t="n"/>
       <c r="F171" s="61" t="n">
-        <v>2</v>
-      </c>
-      <c r="G171" s="75" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="G171" s="75" t="inlineStr">
+        <is>
+          <t>A tie for the lead counts</t>
+        </is>
+      </c>
       <c r="H171" s="76" t="n"/>
       <c r="I171" s="76" t="n"/>
       <c r="J171" s="76" t="n"/>
@@ -6770,23 +6746,19 @@
       </c>
       <c r="C172" s="56" t="inlineStr">
         <is>
-          <t>Variaball Vinyl</t>
+          <t>Polypaypylene</t>
         </is>
       </c>
       <c r="D172" s="63" t="inlineStr">
         <is>
-          <t>The draw for turn goes to a random player each possession</t>
+          <t>Making a shot: Draw 3</t>
         </is>
       </c>
       <c r="E172" s="58" t="n"/>
       <c r="F172" s="61" t="n">
         <v>1</v>
       </c>
-      <c r="G172" s="75" t="inlineStr">
-        <is>
-          <t>Can be the turn player</t>
-        </is>
-      </c>
+      <c r="G172" s="75" t="n"/>
       <c r="H172" s="76" t="n"/>
       <c r="I172" s="76" t="n"/>
       <c r="J172" s="76" t="n"/>
@@ -6800,12 +6772,12 @@
       </c>
       <c r="C173" s="56" t="inlineStr">
         <is>
-          <t>Gravi-Gym</t>
+          <t>Recoverena</t>
         </is>
       </c>
       <c r="D173" s="63" t="inlineStr">
         <is>
-          <t>SHOT -10%. No dunks</t>
+          <t>Discard all Injuries. A new Injury is discarded, and that player draws 1</t>
         </is>
       </c>
       <c r="E173" s="58" t="n"/>
@@ -6814,7 +6786,7 @@
       </c>
       <c r="G173" s="75" t="inlineStr">
         <is>
-          <t>Cards that dunk cannot be played</t>
+          <t>Every player's Injuries go when it lands</t>
         </is>
       </c>
       <c r="H173" s="76" t="n"/>
@@ -6830,21 +6802,21 @@
       </c>
       <c r="C174" s="56" t="inlineStr">
         <is>
-          <t>Vintage Varnish</t>
+          <t>Carousel Court</t>
         </is>
       </c>
       <c r="D174" s="63" t="inlineStr">
         <is>
-          <t>Shot Clock 14. No threes. No Variaballs. 1 Intangible per player</t>
+          <t>Declare left or right. Every possession, hands move one seat that way</t>
         </is>
       </c>
       <c r="E174" s="58" t="n"/>
       <c r="F174" s="61" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G174" s="75" t="inlineStr">
         <is>
-          <t>Discards the ball in play when it lands</t>
+          <t>Declared by whoever plays it</t>
         </is>
       </c>
       <c r="H174" s="76" t="n"/>
@@ -6860,21 +6832,21 @@
       </c>
       <c r="C175" s="56" t="inlineStr">
         <is>
-          <t>S.O.S — Sell-Out Stadium</t>
+          <t>Traderous Tarmac</t>
         </is>
       </c>
       <c r="D175" s="63" t="inlineStr">
         <is>
-          <t>A Three may be attempted as a two at 2X SHOT</t>
+          <t>During your turn, hand off any number of the Clamps on you to other players</t>
         </is>
       </c>
       <c r="E175" s="58" t="n"/>
       <c r="F175" s="61" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G175" s="75" t="inlineStr">
         <is>
-          <t>Keeps every other printed effect</t>
+          <t>The player assigns each Clamp: all to one player, one each, or any split</t>
         </is>
       </c>
       <c r="H175" s="76" t="n"/>
@@ -6890,21 +6862,21 @@
       </c>
       <c r="C176" s="56" t="inlineStr">
         <is>
-          <t>Grayvstone</t>
+          <t>Clearcoat Court</t>
         </is>
       </c>
       <c r="D176" s="63" t="inlineStr">
         <is>
-          <t>Each possession, the ball becomes the last Variaball in the discards</t>
+          <t>Every possession: clear all referees, Clamps, Injuries and Intangibles</t>
         </is>
       </c>
       <c r="E176" s="58" t="n"/>
       <c r="F176" s="61" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G176" s="75" t="inlineStr">
         <is>
-          <t>With none there, nothing happens</t>
+          <t>Standing Clamps only; Clamps still in the air land after the wipe</t>
         </is>
       </c>
       <c r="H176" s="76" t="n"/>
@@ -6920,17 +6892,17 @@
       </c>
       <c r="C177" s="56" t="inlineStr">
         <is>
-          <t>Con-crete</t>
+          <t>Malice Palace</t>
         </is>
       </c>
       <c r="D177" s="63" t="inlineStr">
         <is>
-          <t>Move cards: SHOT -10%</t>
+          <t>At the start of your possession, before your draw: discard your hand</t>
         </is>
       </c>
       <c r="E177" s="58" t="n"/>
       <c r="F177" s="61" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G177" s="75" t="n"/>
       <c r="H177" s="76" t="n"/>
@@ -6946,12 +6918,14 @@
       </c>
       <c r="C178" s="56" t="inlineStr">
         <is>
-          <t>Spazzphalt</t>
+          <t>Turnstile Tile</t>
         </is>
       </c>
       <c r="D178" s="63" t="inlineStr">
         <is>
-          <t>SHOT = ?</t>
+          <t>Upright: SHOT +25%
+Reversed: SHOT -25%
+Turn this card at the start of each possession</t>
         </is>
       </c>
       <c r="E178" s="58" t="n"/>
@@ -6960,7 +6934,7 @@
       </c>
       <c r="G178" s="75" t="inlineStr">
         <is>
-          <t>A random 0–100%, in steps of 5</t>
+          <t>+25% the possession it lands</t>
         </is>
       </c>
       <c r="H178" s="76" t="n"/>
@@ -6976,23 +6950,19 @@
       </c>
       <c r="C179" s="56" t="inlineStr">
         <is>
-          <t>Frostbite Finish</t>
+          <t>Roleplayer Polymer</t>
         </is>
       </c>
       <c r="D179" s="63" t="inlineStr">
         <is>
-          <t>Playing a Move costs discarding 1 other card</t>
+          <t>Every possession, everyone but the turn player draws 1</t>
         </is>
       </c>
       <c r="E179" s="58" t="n"/>
       <c r="F179" s="61" t="n">
         <v>2</v>
       </c>
-      <c r="G179" s="75" t="inlineStr">
-        <is>
-          <t>The owner picks the card. A Move that is your whole hand can't be played</t>
-        </is>
-      </c>
+      <c r="G179" s="75" t="n"/>
       <c r="H179" s="76" t="n"/>
       <c r="I179" s="76" t="n"/>
       <c r="J179" s="76" t="n"/>
@@ -7006,26 +6976,21 @@
       </c>
       <c r="C180" s="56" t="inlineStr">
         <is>
-          <t>The Future</t>
+          <t>Variaball Vinyl</t>
         </is>
       </c>
       <c r="D180" s="63" t="inlineStr">
         <is>
-          <t>SHOT +10% and Draw 1 card when playing a Move card.
-SHOT -10% while Passing.</t>
-        </is>
-      </c>
-      <c r="E180" s="58" t="inlineStr">
-        <is>
-          <t>You may Discard 1 card during a three attempt to make it worth four pts (at SHOT-10%)</t>
-        </is>
-      </c>
+          <t>The draw for turn goes to a random player each possession</t>
+        </is>
+      </c>
+      <c r="E180" s="58" t="n"/>
       <c r="F180" s="61" t="n">
         <v>1</v>
       </c>
       <c r="G180" s="75" t="inlineStr">
         <is>
-          <t>New in the SHOT audit (2026-09-14). Special Moves count as Moves</t>
+          <t>Can be the turn player</t>
         </is>
       </c>
       <c r="H180" s="76" t="n"/>
@@ -7041,12 +7006,12 @@
       </c>
       <c r="C181" s="56" t="inlineStr">
         <is>
-          <t>Tick-Tock Tile</t>
+          <t>Gravi-Gym</t>
         </is>
       </c>
       <c r="D181" s="63" t="inlineStr">
         <is>
-          <t>Playing any card also ticks the Shot Clock</t>
+          <t>SHOT -10%. No dunks</t>
         </is>
       </c>
       <c r="E181" s="58" t="n"/>
@@ -7055,56 +7020,67 @@
       </c>
       <c r="G181" s="75" t="inlineStr">
         <is>
-          <t>The tick is paid after the card resolves, so a shot at 01 still goes up</t>
+          <t>Cards that dunk cannot be played</t>
         </is>
       </c>
       <c r="H181" s="76" t="n"/>
       <c r="I181" s="76" t="n"/>
       <c r="J181" s="76" t="n"/>
     </row>
-    <row r="182" ht="42" customHeight="1" s="85">
-      <c r="A182" s="52" t="inlineStr">
-        <is>
-          <t>Variaball</t>
-        </is>
-      </c>
-      <c r="B182" s="53">
-        <f>COUNTIF($B$183:$B$198,"Variaball")</f>
-        <v/>
-      </c>
-      <c r="C182" s="54" t="n"/>
-      <c r="D182" s="54" t="n"/>
-      <c r="E182" s="54" t="n"/>
-      <c r="F182" s="55" t="n"/>
-      <c r="G182" s="66" t="n"/>
-      <c r="H182" s="67" t="n"/>
-      <c r="I182" s="67" t="n"/>
-      <c r="J182" s="67" t="n"/>
+    <row r="182" s="85">
+      <c r="A182" s="27" t="n"/>
+      <c r="B182" s="28" t="inlineStr">
+        <is>
+          <t>Varena</t>
+        </is>
+      </c>
+      <c r="C182" s="56" t="inlineStr">
+        <is>
+          <t>Vintage Varnish</t>
+        </is>
+      </c>
+      <c r="D182" s="63" t="inlineStr">
+        <is>
+          <t>Shot Clock 14. No threes. No Variaballs. 1 Intangible per player</t>
+        </is>
+      </c>
+      <c r="E182" s="58" t="n"/>
+      <c r="F182" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G182" s="75" t="inlineStr">
+        <is>
+          <t>Discards the ball in play when it lands</t>
+        </is>
+      </c>
+      <c r="H182" s="76" t="n"/>
+      <c r="I182" s="76" t="n"/>
+      <c r="J182" s="76" t="n"/>
     </row>
     <row r="183" s="85">
       <c r="A183" s="27" t="n"/>
       <c r="B183" s="28" t="inlineStr">
         <is>
-          <t>Variaball</t>
+          <t>Varena</t>
         </is>
       </c>
       <c r="C183" s="56" t="inlineStr">
         <is>
-          <t>Med Ball</t>
+          <t>S.O.S — Sell-Out Stadium</t>
         </is>
       </c>
       <c r="D183" s="63" t="inlineStr">
         <is>
-          <t>SHOT cannot exceed 50%</t>
+          <t>A Three may be attempted as a two at 2X SHOT</t>
         </is>
       </c>
       <c r="E183" s="58" t="n"/>
       <c r="F183" s="61" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G183" s="75" t="inlineStr">
         <is>
-          <t>An Intangible's or a Varena's SHOT = is not held to it</t>
+          <t>Keeps every other printed effect</t>
         </is>
       </c>
       <c r="H183" s="76" t="n"/>
@@ -7115,26 +7091,26 @@
       <c r="A184" s="27" t="n"/>
       <c r="B184" s="28" t="inlineStr">
         <is>
-          <t>Variaball</t>
+          <t>Varena</t>
         </is>
       </c>
       <c r="C184" s="56" t="inlineStr">
         <is>
-          <t>Dishcount Ball</t>
+          <t>Grayvstone</t>
         </is>
       </c>
       <c r="D184" s="63" t="inlineStr">
         <is>
-          <t>Discard one fewer for card costs and Clamps</t>
+          <t>Each possession, the ball becomes the last Variaball in the discards</t>
         </is>
       </c>
       <c r="E184" s="58" t="n"/>
       <c r="F184" s="61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G184" s="75" t="inlineStr">
         <is>
-          <t>Counts: Clamps, Pound Dribble, Frostbite Finish, Stepback, Turnaround Three</t>
+          <t>With none there, nothing happens</t>
         </is>
       </c>
       <c r="H184" s="76" t="n"/>
@@ -7145,28 +7121,24 @@
       <c r="A185" s="27" t="n"/>
       <c r="B185" s="28" t="inlineStr">
         <is>
-          <t>Variaball</t>
+          <t>Varena</t>
         </is>
       </c>
       <c r="C185" s="56" t="inlineStr">
         <is>
-          <t>Blight Ball</t>
+          <t>Con-crete</t>
         </is>
       </c>
       <c r="D185" s="63" t="inlineStr">
         <is>
-          <t>Injuries travel with the ball, and new ones join the pile. Discarding the ball takes the pile with it</t>
+          <t>Move cards: SHOT -10%</t>
         </is>
       </c>
       <c r="E185" s="58" t="n"/>
       <c r="F185" s="61" t="n">
         <v>3</v>
       </c>
-      <c r="G185" s="75" t="inlineStr">
-        <is>
-          <t>Moves on any change of hands</t>
-        </is>
-      </c>
+      <c r="G185" s="75" t="n"/>
       <c r="H185" s="76" t="n"/>
       <c r="I185" s="76" t="n"/>
       <c r="J185" s="76" t="n"/>
@@ -7175,24 +7147,28 @@
       <c r="A186" s="27" t="n"/>
       <c r="B186" s="28" t="inlineStr">
         <is>
-          <t>Variaball</t>
+          <t>Varena</t>
         </is>
       </c>
       <c r="C186" s="56" t="inlineStr">
         <is>
-          <t>Bench Ball</t>
+          <t>Spazzphalt</t>
         </is>
       </c>
       <c r="D186" s="63" t="inlineStr">
         <is>
-          <t>Receiving it by Pass: no draw, no turn. You inbound</t>
+          <t>SHOT = ?</t>
         </is>
       </c>
       <c r="E186" s="58" t="n"/>
       <c r="F186" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="G186" s="75" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="G186" s="75" t="inlineStr">
+        <is>
+          <t>A random 0–100%, in steps of 5</t>
+        </is>
+      </c>
       <c r="H186" s="76" t="n"/>
       <c r="I186" s="76" t="n"/>
       <c r="J186" s="76" t="n"/>
@@ -7201,17 +7177,17 @@
       <c r="A187" s="27" t="n"/>
       <c r="B187" s="28" t="inlineStr">
         <is>
-          <t>Variaball</t>
+          <t>Varena</t>
         </is>
       </c>
       <c r="C187" s="56" t="inlineStr">
         <is>
-          <t>Dishtracting Ball</t>
+          <t>Frostbite Finish</t>
         </is>
       </c>
       <c r="D187" s="63" t="inlineStr">
         <is>
-          <t>Receiving it: discard 1, after the draw for turn</t>
+          <t>Playing a Move costs discarding 1 other card</t>
         </is>
       </c>
       <c r="E187" s="58" t="n"/>
@@ -7220,7 +7196,7 @@
       </c>
       <c r="G187" s="75" t="inlineStr">
         <is>
-          <t>Any change of hands</t>
+          <t>The owner picks the card. A Move that is your whole hand can't be played</t>
         </is>
       </c>
       <c r="H187" s="76" t="n"/>
@@ -7231,24 +7207,33 @@
       <c r="A188" s="27" t="n"/>
       <c r="B188" s="28" t="inlineStr">
         <is>
-          <t>Variaball</t>
+          <t>Varena</t>
         </is>
       </c>
       <c r="C188" s="56" t="inlineStr">
         <is>
-          <t>Hand Ball</t>
+          <t>The Future</t>
         </is>
       </c>
       <c r="D188" s="63" t="inlineStr">
         <is>
-          <t>A Pass swaps hands: yours goes with the ball, theirs comes back</t>
-        </is>
-      </c>
-      <c r="E188" s="58" t="n"/>
+          <t>SHOT +10% and Draw 1 card when playing a Move card.
+SHOT -10% while Passing.</t>
+        </is>
+      </c>
+      <c r="E188" s="58" t="inlineStr">
+        <is>
+          <t>You may Discard 1 card during a three attempt to make it worth four pts (at SHOT-10%)</t>
+        </is>
+      </c>
       <c r="F188" s="61" t="n">
         <v>1</v>
       </c>
-      <c r="G188" s="75" t="n"/>
+      <c r="G188" s="75" t="inlineStr">
+        <is>
+          <t>New in the SHOT audit (2026-09-14). Special Moves count as Moves</t>
+        </is>
+      </c>
       <c r="H188" s="76" t="n"/>
       <c r="I188" s="76" t="n"/>
       <c r="J188" s="76" t="n"/>
@@ -7257,53 +7242,50 @@
       <c r="A189" s="27" t="n"/>
       <c r="B189" s="28" t="inlineStr">
         <is>
-          <t>Variaball</t>
+          <t>Varena</t>
         </is>
       </c>
       <c r="C189" s="56" t="inlineStr">
         <is>
-          <t>Foot Ball</t>
+          <t>Tick-Tock Tile</t>
         </is>
       </c>
       <c r="D189" s="63" t="inlineStr">
         <is>
-          <t>Moves and Passes are not spent. They lock until your possession ends</t>
+          <t>Playing any card also ticks the Shot Clock</t>
         </is>
       </c>
       <c r="E189" s="58" t="n"/>
       <c r="F189" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="G189" s="75" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="G189" s="75" t="inlineStr">
+        <is>
+          <t>The tick is paid after the card resolves, so a shot at 01 still goes up</t>
+        </is>
+      </c>
       <c r="H189" s="76" t="n"/>
       <c r="I189" s="76" t="n"/>
       <c r="J189" s="76" t="n"/>
     </row>
-    <row r="190" s="85">
-      <c r="A190" s="27" t="n"/>
-      <c r="B190" s="28" t="inlineStr">
+    <row r="190" ht="42" customHeight="1" s="85">
+      <c r="A190" s="52" t="inlineStr">
         <is>
           <t>Variaball</t>
         </is>
       </c>
-      <c r="C190" s="56" t="inlineStr">
-        <is>
-          <t>Recharge Rock</t>
-        </is>
-      </c>
-      <c r="D190" s="63" t="inlineStr">
-        <is>
-          <t>Double your draw for turn</t>
-        </is>
-      </c>
-      <c r="E190" s="58" t="n"/>
-      <c r="F190" s="61" t="n">
-        <v>5</v>
-      </c>
-      <c r="G190" s="75" t="n"/>
-      <c r="H190" s="76" t="n"/>
-      <c r="I190" s="76" t="n"/>
-      <c r="J190" s="76" t="n"/>
+      <c r="B190" s="53">
+        <f>COUNTIF($B$191:$B$208,"Variaball")</f>
+        <v/>
+      </c>
+      <c r="C190" s="54" t="n"/>
+      <c r="D190" s="54" t="n"/>
+      <c r="E190" s="54" t="n"/>
+      <c r="F190" s="55" t="n"/>
+      <c r="G190" s="66" t="n"/>
+      <c r="H190" s="67" t="n"/>
+      <c r="I190" s="67" t="n"/>
+      <c r="J190" s="67" t="n"/>
     </row>
     <row r="191" s="85">
       <c r="A191" s="27" t="n"/>
@@ -7314,21 +7296,21 @@
       </c>
       <c r="C191" s="56" t="inlineStr">
         <is>
-          <t>Variaball</t>
+          <t>Med Ball</t>
         </is>
       </c>
       <c r="D191" s="63" t="inlineStr">
         <is>
-          <t>A random Variaball from the discards goes into play. Then discard this</t>
+          <t>SHOT cannot exceed 50%</t>
         </is>
       </c>
       <c r="E191" s="58" t="n"/>
       <c r="F191" s="61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G191" s="75" t="inlineStr">
         <is>
-          <t>From the deck if the discards have none; never the ball already in play</t>
+          <t>An Intangible's or a Varena's SHOT = is not held to it</t>
         </is>
       </c>
       <c r="H191" s="76" t="n"/>
@@ -7344,19 +7326,23 @@
       </c>
       <c r="C192" s="56" t="inlineStr">
         <is>
-          <t>Shufflebag Ball</t>
+          <t>Dishcount Ball</t>
         </is>
       </c>
       <c r="D192" s="63" t="inlineStr">
         <is>
-          <t>Every possession, the turn player shuffles their hand into the deck and draws the same number, then draws for turn</t>
+          <t>Discard one fewer for card costs and Clamps</t>
         </is>
       </c>
       <c r="E192" s="58" t="n"/>
       <c r="F192" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="G192" s="75" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="G192" s="75" t="inlineStr">
+        <is>
+          <t>Counts: Clamps, Pound Dribble, Frostbite Finish, Stepback, Turnaround Three</t>
+        </is>
+      </c>
       <c r="H192" s="76" t="n"/>
       <c r="I192" s="76" t="n"/>
       <c r="J192" s="76" t="n"/>
@@ -7370,19 +7356,23 @@
       </c>
       <c r="C193" s="56" t="inlineStr">
         <is>
-          <t>Bag'n Ball</t>
+          <t>Blight Ball</t>
         </is>
       </c>
       <c r="D193" s="63" t="inlineStr">
         <is>
-          <t>Draw 1 card when played. SHOT = 10% for each card in your hand</t>
+          <t>Injuries travel with the ball, and new ones join the pile. Discarding the ball takes the pile with it</t>
         </is>
       </c>
       <c r="E193" s="58" t="n"/>
       <c r="F193" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="G193" s="75" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="G193" s="75" t="inlineStr">
+        <is>
+          <t>Moves on any change of hands</t>
+        </is>
+      </c>
       <c r="H193" s="76" t="n"/>
       <c r="I193" s="76" t="n"/>
       <c r="J193" s="76" t="n"/>
@@ -7396,23 +7386,19 @@
       </c>
       <c r="C194" s="56" t="inlineStr">
         <is>
-          <t>Blaze Ball</t>
+          <t>Bench Ball</t>
         </is>
       </c>
       <c r="D194" s="63" t="inlineStr">
         <is>
-          <t>SHOT +10% as this Ball is Passed</t>
+          <t>Receiving it by Pass: no draw, no turn. You inbound</t>
         </is>
       </c>
       <c r="E194" s="58" t="n"/>
       <c r="F194" s="61" t="n">
-        <v>5</v>
-      </c>
-      <c r="G194" s="75" t="inlineStr">
-        <is>
-          <t>Ignores every other pass modifier</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G194" s="75" t="n"/>
       <c r="H194" s="76" t="n"/>
       <c r="I194" s="76" t="n"/>
       <c r="J194" s="76" t="n"/>
@@ -7426,21 +7412,21 @@
       </c>
       <c r="C195" s="56" t="inlineStr">
         <is>
-          <t>Snow Ball It</t>
+          <t>Dishtracting Ball</t>
         </is>
       </c>
       <c r="D195" s="63" t="inlineStr">
         <is>
-          <t>SHOT -10% as this Ball is Passed</t>
+          <t>Receiving it: discard 1, after the draw for turn</t>
         </is>
       </c>
       <c r="E195" s="58" t="n"/>
       <c r="F195" s="61" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G195" s="75" t="inlineStr">
         <is>
-          <t>Blaze Ball's opposite</t>
+          <t>Any change of hands</t>
         </is>
       </c>
       <c r="H195" s="76" t="n"/>
@@ -7456,17 +7442,17 @@
       </c>
       <c r="C196" s="56" t="inlineStr">
         <is>
-          <t>Brick Ball</t>
+          <t>Hand Ball</t>
         </is>
       </c>
       <c r="D196" s="63" t="inlineStr">
         <is>
-          <t>SHOT = 25%</t>
+          <t>A Pass swaps hands: yours goes with the ball, theirs comes back</t>
         </is>
       </c>
       <c r="E196" s="58" t="n"/>
       <c r="F196" s="61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G196" s="75" t="n"/>
       <c r="H196" s="76" t="n"/>
@@ -7482,23 +7468,19 @@
       </c>
       <c r="C197" s="56" t="inlineStr">
         <is>
-          <t>Monster Ball</t>
+          <t>Foot Ball</t>
         </is>
       </c>
       <c r="D197" s="63" t="inlineStr">
         <is>
-          <t>Intangibles are absorbed into the ball. When it's discarded, players rebound for them one at a time</t>
+          <t>Moves and Passes are not spent. They lock until your possession ends</t>
         </is>
       </c>
       <c r="E197" s="58" t="n"/>
       <c r="F197" s="61" t="n">
         <v>1</v>
       </c>
-      <c r="G197" s="75" t="inlineStr">
-        <is>
-          <t>Swallows every Intangible already out and every one drawn while it's in play</t>
-        </is>
-      </c>
+      <c r="G197" s="75" t="n"/>
       <c r="H197" s="76" t="n"/>
       <c r="I197" s="76" t="n"/>
       <c r="J197" s="76" t="n"/>
@@ -7512,75 +7494,414 @@
       </c>
       <c r="C198" s="56" t="inlineStr">
         <is>
-          <t>Brand New Ball</t>
+          <t>Recharge Rock</t>
         </is>
       </c>
       <c r="D198" s="63" t="inlineStr">
         <is>
-          <t>25% chance a shot attempt is a turnover instead</t>
+          <t>Double your draw for turn</t>
         </is>
       </c>
       <c r="E198" s="58" t="n"/>
       <c r="F198" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="G198" s="75" t="inlineStr">
-        <is>
-          <t>The round ends</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="G198" s="75" t="n"/>
       <c r="H198" s="76" t="n"/>
       <c r="I198" s="76" t="n"/>
       <c r="J198" s="76" t="n"/>
     </row>
+    <row r="199" s="85">
+      <c r="A199" s="27" t="n"/>
+      <c r="B199" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C199" s="56" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="D199" s="63" t="inlineStr">
+        <is>
+          <t>A random Variaball from the discards goes into play. Then discard this</t>
+        </is>
+      </c>
+      <c r="E199" s="58" t="n"/>
+      <c r="F199" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="G199" s="75" t="inlineStr">
+        <is>
+          <t>From the deck if the discards have none; never the ball already in play</t>
+        </is>
+      </c>
+      <c r="H199" s="76" t="n"/>
+      <c r="I199" s="76" t="n"/>
+      <c r="J199" s="76" t="n"/>
+    </row>
+    <row r="200" s="85">
+      <c r="A200" s="27" t="n"/>
+      <c r="B200" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C200" s="56" t="inlineStr">
+        <is>
+          <t>Shufflebag Ball</t>
+        </is>
+      </c>
+      <c r="D200" s="63" t="inlineStr">
+        <is>
+          <t>Every possession, the turn player shuffles their hand into the deck and draws the same number, then draws for turn</t>
+        </is>
+      </c>
+      <c r="E200" s="58" t="n"/>
+      <c r="F200" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G200" s="75" t="n"/>
+      <c r="H200" s="76" t="n"/>
+      <c r="I200" s="76" t="n"/>
+      <c r="J200" s="76" t="n"/>
+    </row>
+    <row r="201" s="85">
+      <c r="A201" s="27" t="n"/>
+      <c r="B201" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C201" s="56" t="inlineStr">
+        <is>
+          <t>Bag'n Ball</t>
+        </is>
+      </c>
+      <c r="D201" s="63" t="inlineStr">
+        <is>
+          <t>Draw 1 card when played. SHOT = 10% for each card in your hand</t>
+        </is>
+      </c>
+      <c r="E201" s="58" t="n"/>
+      <c r="F201" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G201" s="75" t="n"/>
+      <c r="H201" s="76" t="n"/>
+      <c r="I201" s="76" t="n"/>
+      <c r="J201" s="76" t="n"/>
+    </row>
+    <row r="202" s="85">
+      <c r="A202" s="27" t="n"/>
+      <c r="B202" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C202" s="56" t="inlineStr">
+        <is>
+          <t>Blaze Ball</t>
+        </is>
+      </c>
+      <c r="D202" s="63" t="inlineStr">
+        <is>
+          <t>SHOT +10% as this Ball is Passed</t>
+        </is>
+      </c>
+      <c r="E202" s="58" t="n"/>
+      <c r="F202" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="G202" s="75" t="inlineStr">
+        <is>
+          <t>Ignores every other pass modifier</t>
+        </is>
+      </c>
+      <c r="H202" s="76" t="n"/>
+      <c r="I202" s="76" t="n"/>
+      <c r="J202" s="76" t="n"/>
+    </row>
+    <row r="203" s="85">
+      <c r="A203" s="27" t="n"/>
+      <c r="B203" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C203" s="56" t="inlineStr">
+        <is>
+          <t>Snow Ball</t>
+        </is>
+      </c>
+      <c r="D203" s="63" t="inlineStr">
+        <is>
+          <t>SHOT -10% as this Ball is Passed</t>
+        </is>
+      </c>
+      <c r="E203" s="58" t="n"/>
+      <c r="F203" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="G203" s="75" t="inlineStr">
+        <is>
+          <t>Blaze Ball's opposite</t>
+        </is>
+      </c>
+      <c r="H203" s="76" t="n"/>
+      <c r="I203" s="76" t="n"/>
+      <c r="J203" s="76" t="n"/>
+    </row>
+    <row r="204" s="85">
+      <c r="A204" s="27" t="n"/>
+      <c r="B204" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C204" s="56" t="inlineStr">
+        <is>
+          <t>Brick Ball</t>
+        </is>
+      </c>
+      <c r="D204" s="63" t="inlineStr">
+        <is>
+          <t>SHOT = 25%</t>
+        </is>
+      </c>
+      <c r="E204" s="58" t="n"/>
+      <c r="F204" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="G204" s="75" t="n"/>
+      <c r="H204" s="76" t="n"/>
+      <c r="I204" s="76" t="n"/>
+      <c r="J204" s="76" t="n"/>
+    </row>
+    <row r="205" s="85">
+      <c r="A205" s="27" t="n"/>
+      <c r="B205" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C205" s="56" t="inlineStr">
+        <is>
+          <t>Monster Ball</t>
+        </is>
+      </c>
+      <c r="D205" s="63" t="inlineStr">
+        <is>
+          <t>Intangibles are absorbed into the ball. When it's discarded, players rebound for them one at a time</t>
+        </is>
+      </c>
+      <c r="E205" s="58" t="n"/>
+      <c r="F205" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G205" s="75" t="inlineStr">
+        <is>
+          <t>Swallows every Intangible already out and every one drawn while it's in play</t>
+        </is>
+      </c>
+      <c r="H205" s="76" t="n"/>
+      <c r="I205" s="76" t="n"/>
+      <c r="J205" s="76" t="n"/>
+    </row>
+    <row r="206" s="85">
+      <c r="A206" s="27" t="n"/>
+      <c r="B206" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C206" s="56" t="inlineStr">
+        <is>
+          <t>Brand New Ball</t>
+        </is>
+      </c>
+      <c r="D206" s="63" t="inlineStr">
+        <is>
+          <t>25% chance a shot attempt is a turnover instead</t>
+        </is>
+      </c>
+      <c r="E206" s="58" t="n"/>
+      <c r="F206" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G206" s="75" t="inlineStr">
+        <is>
+          <t>The round ends</t>
+        </is>
+      </c>
+      <c r="H206" s="76" t="n"/>
+      <c r="I206" s="76" t="n"/>
+      <c r="J206" s="76" t="n"/>
+    </row>
+    <row r="207" s="85">
+      <c r="A207" s="27" t="n"/>
+      <c r="B207" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C207" s="56" t="inlineStr">
+        <is>
+          <t>Make-or-Take Ball</t>
+        </is>
+      </c>
+      <c r="D207" s="63" t="inlineStr">
+        <is>
+          <t>Take 1 FT after missing a shot attempt.</t>
+        </is>
+      </c>
+      <c r="E207" s="58" t="n"/>
+      <c r="F207" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G207" s="75" t="n"/>
+      <c r="H207" s="76" t="n"/>
+      <c r="I207" s="76" t="n"/>
+      <c r="J207" s="76" t="n"/>
+    </row>
+    <row r="208" s="85">
+      <c r="A208" s="27" t="n"/>
+      <c r="B208" s="28" t="inlineStr">
+        <is>
+          <t>Variaball</t>
+        </is>
+      </c>
+      <c r="C208" s="56" t="inlineStr">
+        <is>
+          <t>Hero Ball</t>
+        </is>
+      </c>
+      <c r="D208" s="63" t="inlineStr">
+        <is>
+          <t>Cannot play Pass cards. Made shots grant no AST</t>
+        </is>
+      </c>
+      <c r="E208" s="58" t="n"/>
+      <c r="F208" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G208" s="75" t="n"/>
+      <c r="H208" s="76" t="n"/>
+      <c r="I208" s="76" t="n"/>
+      <c r="J208" s="76" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="176">
+  <mergeCells count="186">
     <mergeCell ref="G55:J55"/>
+    <mergeCell ref="G188:J188"/>
     <mergeCell ref="G4:J4"/>
     <mergeCell ref="G182:J182"/>
-    <mergeCell ref="G188:J188"/>
+    <mergeCell ref="G200:J200"/>
     <mergeCell ref="G135:J135"/>
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
     <mergeCell ref="G119:J119"/>
-    <mergeCell ref="G32:J32"/>
+    <mergeCell ref="G202:J202"/>
     <mergeCell ref="G46:J46"/>
-    <mergeCell ref="G159:J159"/>
     <mergeCell ref="G40:J40"/>
     <mergeCell ref="G111:J111"/>
-    <mergeCell ref="G72:J72"/>
-    <mergeCell ref="G81:J81"/>
-    <mergeCell ref="G161:J161"/>
     <mergeCell ref="G71:J71"/>
-    <mergeCell ref="G136:J136"/>
-    <mergeCell ref="G194:J194"/>
-    <mergeCell ref="G181:J181"/>
     <mergeCell ref="G8:J8"/>
-    <mergeCell ref="G160:J160"/>
     <mergeCell ref="G82:J82"/>
-    <mergeCell ref="G174:J174"/>
-    <mergeCell ref="G156:J156"/>
     <mergeCell ref="G57:J57"/>
     <mergeCell ref="G128:J128"/>
     <mergeCell ref="G10:J10"/>
     <mergeCell ref="G66:J66"/>
+    <mergeCell ref="G184:J184"/>
     <mergeCell ref="G137:J137"/>
-    <mergeCell ref="G184:J184"/>
-    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="G171:J171"/>
     <mergeCell ref="G53:J53"/>
-    <mergeCell ref="G171:J171"/>
-    <mergeCell ref="G189:J189"/>
+    <mergeCell ref="G146:J146"/>
     <mergeCell ref="G121:J121"/>
-    <mergeCell ref="G34:J34"/>
     <mergeCell ref="G74:J74"/>
     <mergeCell ref="G68:J68"/>
-    <mergeCell ref="G108:J108"/>
+    <mergeCell ref="G139:J139"/>
     <mergeCell ref="G58:J58"/>
     <mergeCell ref="G114:J114"/>
     <mergeCell ref="G123:J123"/>
-    <mergeCell ref="G163:J163"/>
     <mergeCell ref="G110:J110"/>
     <mergeCell ref="G168:J168"/>
+    <mergeCell ref="G143:J143"/>
+    <mergeCell ref="G75:J75"/>
+    <mergeCell ref="G12:J12"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="G67:J67"/>
+    <mergeCell ref="G61:J61"/>
+    <mergeCell ref="G70:J70"/>
+    <mergeCell ref="G48:J48"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="G125:J125"/>
+    <mergeCell ref="G7:J7"/>
+    <mergeCell ref="G112:J112"/>
+    <mergeCell ref="G62:J62"/>
+    <mergeCell ref="G127:J127"/>
+    <mergeCell ref="G65:J65"/>
+    <mergeCell ref="G201:J201"/>
+    <mergeCell ref="G129:J129"/>
+    <mergeCell ref="G16:J16"/>
+    <mergeCell ref="G138:J138"/>
+    <mergeCell ref="G76:J76"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="G203:J203"/>
+    <mergeCell ref="G60:J60"/>
+    <mergeCell ref="G9:J9"/>
+    <mergeCell ref="G131:J131"/>
+    <mergeCell ref="G140:J140"/>
+    <mergeCell ref="G198:J198"/>
+    <mergeCell ref="G11:J11"/>
+    <mergeCell ref="G169:J169"/>
+    <mergeCell ref="G126:J126"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G13:J13"/>
+    <mergeCell ref="G78:J78"/>
+    <mergeCell ref="G87:J87"/>
+    <mergeCell ref="G15:J15"/>
+    <mergeCell ref="G142:J142"/>
+    <mergeCell ref="G80:J80"/>
+    <mergeCell ref="G89:J89"/>
+    <mergeCell ref="G64:J64"/>
+    <mergeCell ref="G79:J79"/>
+    <mergeCell ref="G73:J73"/>
+    <mergeCell ref="G51:J51"/>
+    <mergeCell ref="G144:J144"/>
+    <mergeCell ref="G164:J164"/>
+    <mergeCell ref="G173:J173"/>
+    <mergeCell ref="G42:J42"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="G170:J170"/>
+    <mergeCell ref="G141:J141"/>
+    <mergeCell ref="G19:J19"/>
+    <mergeCell ref="G172:J172"/>
+    <mergeCell ref="G190:J190"/>
+    <mergeCell ref="G28:J28"/>
+    <mergeCell ref="G6:J6"/>
+    <mergeCell ref="G83:J83"/>
+    <mergeCell ref="G5:J5"/>
+    <mergeCell ref="G14:J14"/>
+    <mergeCell ref="G150:J150"/>
+    <mergeCell ref="G32:J32"/>
+    <mergeCell ref="G72:J72"/>
+    <mergeCell ref="G81:J81"/>
+    <mergeCell ref="G208:J208"/>
+    <mergeCell ref="G161:J161"/>
+    <mergeCell ref="G136:J136"/>
+    <mergeCell ref="G194:J194"/>
+    <mergeCell ref="G145:J145"/>
+    <mergeCell ref="G181:J181"/>
+    <mergeCell ref="G160:J160"/>
+    <mergeCell ref="G174:J174"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="G189:J189"/>
+    <mergeCell ref="G34:J34"/>
+    <mergeCell ref="G108:J108"/>
+    <mergeCell ref="G207:J207"/>
+    <mergeCell ref="G163:J163"/>
     <mergeCell ref="G113:J113"/>
     <mergeCell ref="G20:J20"/>
     <mergeCell ref="G91:J91"/>
@@ -7588,129 +7909,76 @@
     <mergeCell ref="G100:J100"/>
     <mergeCell ref="G183:J183"/>
     <mergeCell ref="G165:J165"/>
-    <mergeCell ref="G75:J75"/>
     <mergeCell ref="G44:J44"/>
+    <mergeCell ref="G84:J84"/>
     <mergeCell ref="G22:J22"/>
-    <mergeCell ref="G84:J84"/>
     <mergeCell ref="G193:J193"/>
+    <mergeCell ref="G149:J149"/>
     <mergeCell ref="G102:J102"/>
-    <mergeCell ref="G158:J158"/>
     <mergeCell ref="G185:J185"/>
-    <mergeCell ref="G12:J12"/>
     <mergeCell ref="G77:J77"/>
-    <mergeCell ref="G21:J21"/>
     <mergeCell ref="G86:J86"/>
     <mergeCell ref="G178:J178"/>
-    <mergeCell ref="G67:J67"/>
-    <mergeCell ref="G61:J61"/>
-    <mergeCell ref="G70:J70"/>
-    <mergeCell ref="G48:J48"/>
-    <mergeCell ref="G23:J23"/>
     <mergeCell ref="G176:J176"/>
     <mergeCell ref="G97:J97"/>
-    <mergeCell ref="G125:J125"/>
     <mergeCell ref="G38:J38"/>
-    <mergeCell ref="G7:J7"/>
     <mergeCell ref="G191:J191"/>
-    <mergeCell ref="G112:J112"/>
-    <mergeCell ref="G45:J45"/>
-    <mergeCell ref="G62:J62"/>
     <mergeCell ref="G175:J175"/>
-    <mergeCell ref="G127:J127"/>
     <mergeCell ref="G162:J162"/>
     <mergeCell ref="G49:J49"/>
     <mergeCell ref="G24:J24"/>
+    <mergeCell ref="G195:J195"/>
     <mergeCell ref="G177:J177"/>
-    <mergeCell ref="G195:J195"/>
     <mergeCell ref="G33:J33"/>
+    <mergeCell ref="G204:J204"/>
     <mergeCell ref="G104:J104"/>
-    <mergeCell ref="G65:J65"/>
     <mergeCell ref="G88:J88"/>
     <mergeCell ref="G26:J26"/>
-    <mergeCell ref="G154:J154"/>
     <mergeCell ref="G197:J197"/>
     <mergeCell ref="G35:J35"/>
-    <mergeCell ref="G129:J129"/>
-    <mergeCell ref="G138:J138"/>
-    <mergeCell ref="G16:J16"/>
-    <mergeCell ref="G76:J76"/>
-    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="G206:J206"/>
     <mergeCell ref="G90:J90"/>
-    <mergeCell ref="G60:J60"/>
-    <mergeCell ref="G131:J131"/>
-    <mergeCell ref="G9:J9"/>
-    <mergeCell ref="G198:J198"/>
     <mergeCell ref="G59:J59"/>
     <mergeCell ref="G115:J115"/>
     <mergeCell ref="G130:J130"/>
-    <mergeCell ref="G11:J11"/>
     <mergeCell ref="G117:J117"/>
-    <mergeCell ref="G180:J180"/>
-    <mergeCell ref="G169:J169"/>
     <mergeCell ref="G179:J179"/>
-    <mergeCell ref="G126:J126"/>
+    <mergeCell ref="G39:J39"/>
     <mergeCell ref="G132:J132"/>
-    <mergeCell ref="G39:J39"/>
     <mergeCell ref="G122:J122"/>
     <mergeCell ref="G166:J166"/>
     <mergeCell ref="G101:J101"/>
     <mergeCell ref="G116:J116"/>
+    <mergeCell ref="G199:J199"/>
     <mergeCell ref="G103:J103"/>
     <mergeCell ref="G37:J37"/>
     <mergeCell ref="G186:J186"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="G13:J13"/>
-    <mergeCell ref="G78:J78"/>
     <mergeCell ref="G118:J118"/>
-    <mergeCell ref="G87:J87"/>
-    <mergeCell ref="G152:J152"/>
     <mergeCell ref="G167:J167"/>
-    <mergeCell ref="G15:J15"/>
-    <mergeCell ref="G142:J142"/>
-    <mergeCell ref="G80:J80"/>
-    <mergeCell ref="G89:J89"/>
-    <mergeCell ref="G64:J64"/>
-    <mergeCell ref="G79:J79"/>
     <mergeCell ref="G192:J192"/>
-    <mergeCell ref="G73:J73"/>
-    <mergeCell ref="G51:J51"/>
-    <mergeCell ref="G153:J153"/>
     <mergeCell ref="G54:J54"/>
     <mergeCell ref="G63:J63"/>
+    <mergeCell ref="G41:J41"/>
     <mergeCell ref="G134:J134"/>
-    <mergeCell ref="G41:J41"/>
     <mergeCell ref="G50:J50"/>
     <mergeCell ref="G106:J106"/>
-    <mergeCell ref="G164:J164"/>
-    <mergeCell ref="G173:J173"/>
     <mergeCell ref="G56:J56"/>
     <mergeCell ref="G105:J105"/>
     <mergeCell ref="G43:J43"/>
     <mergeCell ref="G52:J52"/>
+    <mergeCell ref="G27:J27"/>
     <mergeCell ref="G120:J120"/>
-    <mergeCell ref="G155:J155"/>
-    <mergeCell ref="G27:J27"/>
     <mergeCell ref="G36:J36"/>
-    <mergeCell ref="G42:J42"/>
     <mergeCell ref="G107:J107"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="G170:J170"/>
-    <mergeCell ref="G157:J157"/>
-    <mergeCell ref="G141:J141"/>
-    <mergeCell ref="G19:J19"/>
-    <mergeCell ref="G172:J172"/>
-    <mergeCell ref="G28:J28"/>
     <mergeCell ref="G93:J93"/>
-    <mergeCell ref="G6:J6"/>
-    <mergeCell ref="G190:J190"/>
+    <mergeCell ref="G187:J187"/>
     <mergeCell ref="G69:J69"/>
-    <mergeCell ref="G187:J187"/>
-    <mergeCell ref="G83:J83"/>
     <mergeCell ref="G196:J196"/>
+    <mergeCell ref="G205:J205"/>
     <mergeCell ref="G124:J124"/>
-    <mergeCell ref="G5:J5"/>
+    <mergeCell ref="G180:J180"/>
     <mergeCell ref="G133:J133"/>
-    <mergeCell ref="G14:J14"/>
+    <mergeCell ref="G45:J45"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
Wide-Open Three: 100% once everyone else has had the ball; Hero Ball to 1
- Wide-Open Three: "If all other players have had possession of the Ball this round:
  SHOT = 100%". The game remembers who has had the ball each round.
- Hero Ball down to 1: it was stopping the game's pace.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -3498,7 +3498,7 @@
       </c>
       <c r="D48" s="57" t="inlineStr">
         <is>
-          <t>SHOT = 100%. (Must be played as your first action and have no Clamps, Injuries, or active Whistles)</t>
+          <t>If all other players have had possession of the Ball this round: SHOT = 100%</t>
         </is>
       </c>
       <c r="E48" s="58" t="n"/>
@@ -7784,7 +7784,7 @@
       </c>
       <c r="E208" s="58" t="n"/>
       <c r="F208" s="61" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G208" s="75" t="n"/>
       <c r="H208" s="76" t="n"/>
@@ -7794,21 +7794,33 @@
   </sheetData>
   <mergeCells count="186">
     <mergeCell ref="G55:J55"/>
+    <mergeCell ref="G200:J200"/>
     <mergeCell ref="G188:J188"/>
     <mergeCell ref="G4:J4"/>
     <mergeCell ref="G182:J182"/>
-    <mergeCell ref="G200:J200"/>
     <mergeCell ref="G135:J135"/>
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
     <mergeCell ref="G119:J119"/>
+    <mergeCell ref="G32:J32"/>
+    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G202:J202"/>
     <mergeCell ref="G46:J46"/>
     <mergeCell ref="G40:J40"/>
     <mergeCell ref="G111:J111"/>
+    <mergeCell ref="G72:J72"/>
+    <mergeCell ref="G81:J81"/>
+    <mergeCell ref="G208:J208"/>
+    <mergeCell ref="G161:J161"/>
     <mergeCell ref="G71:J71"/>
+    <mergeCell ref="G136:J136"/>
+    <mergeCell ref="G194:J194"/>
+    <mergeCell ref="G145:J145"/>
+    <mergeCell ref="G181:J181"/>
     <mergeCell ref="G8:J8"/>
+    <mergeCell ref="G160:J160"/>
     <mergeCell ref="G82:J82"/>
+    <mergeCell ref="G174:J174"/>
     <mergeCell ref="G57:J57"/>
     <mergeCell ref="G128:J128"/>
     <mergeCell ref="G10:J10"/>
@@ -7818,97 +7830,30 @@
     <mergeCell ref="G171:J171"/>
     <mergeCell ref="G53:J53"/>
     <mergeCell ref="G146:J146"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="G189:J189"/>
     <mergeCell ref="G121:J121"/>
+    <mergeCell ref="G34:J34"/>
     <mergeCell ref="G74:J74"/>
     <mergeCell ref="G68:J68"/>
     <mergeCell ref="G139:J139"/>
+    <mergeCell ref="G108:J108"/>
     <mergeCell ref="G58:J58"/>
     <mergeCell ref="G114:J114"/>
     <mergeCell ref="G123:J123"/>
+    <mergeCell ref="G207:J207"/>
+    <mergeCell ref="G163:J163"/>
     <mergeCell ref="G110:J110"/>
     <mergeCell ref="G168:J168"/>
-    <mergeCell ref="G143:J143"/>
-    <mergeCell ref="G75:J75"/>
-    <mergeCell ref="G12:J12"/>
-    <mergeCell ref="G21:J21"/>
-    <mergeCell ref="G67:J67"/>
-    <mergeCell ref="G61:J61"/>
-    <mergeCell ref="G70:J70"/>
-    <mergeCell ref="G48:J48"/>
-    <mergeCell ref="G23:J23"/>
-    <mergeCell ref="G125:J125"/>
-    <mergeCell ref="G7:J7"/>
-    <mergeCell ref="G112:J112"/>
-    <mergeCell ref="G62:J62"/>
-    <mergeCell ref="G127:J127"/>
-    <mergeCell ref="G65:J65"/>
-    <mergeCell ref="G201:J201"/>
-    <mergeCell ref="G129:J129"/>
-    <mergeCell ref="G16:J16"/>
-    <mergeCell ref="G138:J138"/>
-    <mergeCell ref="G76:J76"/>
-    <mergeCell ref="G25:J25"/>
-    <mergeCell ref="G203:J203"/>
-    <mergeCell ref="G60:J60"/>
-    <mergeCell ref="G9:J9"/>
-    <mergeCell ref="G131:J131"/>
-    <mergeCell ref="G140:J140"/>
-    <mergeCell ref="G198:J198"/>
-    <mergeCell ref="G11:J11"/>
-    <mergeCell ref="G169:J169"/>
-    <mergeCell ref="G126:J126"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="G13:J13"/>
-    <mergeCell ref="G78:J78"/>
-    <mergeCell ref="G87:J87"/>
-    <mergeCell ref="G15:J15"/>
-    <mergeCell ref="G142:J142"/>
-    <mergeCell ref="G80:J80"/>
-    <mergeCell ref="G89:J89"/>
-    <mergeCell ref="G64:J64"/>
-    <mergeCell ref="G79:J79"/>
-    <mergeCell ref="G73:J73"/>
-    <mergeCell ref="G51:J51"/>
-    <mergeCell ref="G144:J144"/>
-    <mergeCell ref="G164:J164"/>
-    <mergeCell ref="G173:J173"/>
-    <mergeCell ref="G42:J42"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="G170:J170"/>
-    <mergeCell ref="G141:J141"/>
-    <mergeCell ref="G19:J19"/>
-    <mergeCell ref="G172:J172"/>
-    <mergeCell ref="G190:J190"/>
-    <mergeCell ref="G28:J28"/>
-    <mergeCell ref="G6:J6"/>
-    <mergeCell ref="G83:J83"/>
-    <mergeCell ref="G5:J5"/>
-    <mergeCell ref="G14:J14"/>
-    <mergeCell ref="G150:J150"/>
-    <mergeCell ref="G32:J32"/>
-    <mergeCell ref="G72:J72"/>
-    <mergeCell ref="G81:J81"/>
-    <mergeCell ref="G208:J208"/>
-    <mergeCell ref="G161:J161"/>
-    <mergeCell ref="G136:J136"/>
-    <mergeCell ref="G194:J194"/>
-    <mergeCell ref="G145:J145"/>
-    <mergeCell ref="G181:J181"/>
-    <mergeCell ref="G160:J160"/>
-    <mergeCell ref="G174:J174"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="G189:J189"/>
-    <mergeCell ref="G34:J34"/>
-    <mergeCell ref="G108:J108"/>
-    <mergeCell ref="G207:J207"/>
-    <mergeCell ref="G163:J163"/>
     <mergeCell ref="G113:J113"/>
     <mergeCell ref="G20:J20"/>
     <mergeCell ref="G91:J91"/>
+    <mergeCell ref="G143:J143"/>
     <mergeCell ref="G85:J85"/>
     <mergeCell ref="G100:J100"/>
     <mergeCell ref="G183:J183"/>
     <mergeCell ref="G165:J165"/>
+    <mergeCell ref="G75:J75"/>
     <mergeCell ref="G44:J44"/>
     <mergeCell ref="G84:J84"/>
     <mergeCell ref="G22:J22"/>
@@ -7916,14 +7861,26 @@
     <mergeCell ref="G149:J149"/>
     <mergeCell ref="G102:J102"/>
     <mergeCell ref="G185:J185"/>
+    <mergeCell ref="G12:J12"/>
     <mergeCell ref="G77:J77"/>
+    <mergeCell ref="G21:J21"/>
     <mergeCell ref="G86:J86"/>
     <mergeCell ref="G178:J178"/>
+    <mergeCell ref="G67:J67"/>
+    <mergeCell ref="G61:J61"/>
+    <mergeCell ref="G70:J70"/>
+    <mergeCell ref="G48:J48"/>
+    <mergeCell ref="G23:J23"/>
     <mergeCell ref="G176:J176"/>
     <mergeCell ref="G97:J97"/>
+    <mergeCell ref="G125:J125"/>
+    <mergeCell ref="G7:J7"/>
     <mergeCell ref="G38:J38"/>
     <mergeCell ref="G191:J191"/>
+    <mergeCell ref="G112:J112"/>
+    <mergeCell ref="G62:J62"/>
     <mergeCell ref="G175:J175"/>
+    <mergeCell ref="G127:J127"/>
     <mergeCell ref="G162:J162"/>
     <mergeCell ref="G49:J49"/>
     <mergeCell ref="G24:J24"/>
@@ -7932,17 +7889,33 @@
     <mergeCell ref="G33:J33"/>
     <mergeCell ref="G204:J204"/>
     <mergeCell ref="G104:J104"/>
+    <mergeCell ref="G65:J65"/>
+    <mergeCell ref="G201:J201"/>
     <mergeCell ref="G88:J88"/>
     <mergeCell ref="G26:J26"/>
     <mergeCell ref="G197:J197"/>
     <mergeCell ref="G35:J35"/>
     <mergeCell ref="G206:J206"/>
+    <mergeCell ref="G129:J129"/>
+    <mergeCell ref="G16:J16"/>
+    <mergeCell ref="G138:J138"/>
+    <mergeCell ref="G76:J76"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="G203:J203"/>
     <mergeCell ref="G90:J90"/>
+    <mergeCell ref="G60:J60"/>
+    <mergeCell ref="G9:J9"/>
+    <mergeCell ref="G131:J131"/>
+    <mergeCell ref="G140:J140"/>
+    <mergeCell ref="G198:J198"/>
     <mergeCell ref="G59:J59"/>
     <mergeCell ref="G115:J115"/>
     <mergeCell ref="G130:J130"/>
+    <mergeCell ref="G11:J11"/>
     <mergeCell ref="G117:J117"/>
+    <mergeCell ref="G169:J169"/>
     <mergeCell ref="G179:J179"/>
+    <mergeCell ref="G126:J126"/>
     <mergeCell ref="G39:J39"/>
     <mergeCell ref="G132:J132"/>
     <mergeCell ref="G122:J122"/>
@@ -7953,30 +7926,57 @@
     <mergeCell ref="G103:J103"/>
     <mergeCell ref="G37:J37"/>
     <mergeCell ref="G186:J186"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G13:J13"/>
+    <mergeCell ref="G78:J78"/>
     <mergeCell ref="G118:J118"/>
+    <mergeCell ref="G87:J87"/>
     <mergeCell ref="G167:J167"/>
+    <mergeCell ref="G15:J15"/>
+    <mergeCell ref="G142:J142"/>
+    <mergeCell ref="G80:J80"/>
+    <mergeCell ref="G89:J89"/>
+    <mergeCell ref="G64:J64"/>
+    <mergeCell ref="G79:J79"/>
     <mergeCell ref="G192:J192"/>
+    <mergeCell ref="G73:J73"/>
+    <mergeCell ref="G51:J51"/>
+    <mergeCell ref="G144:J144"/>
     <mergeCell ref="G54:J54"/>
     <mergeCell ref="G63:J63"/>
     <mergeCell ref="G41:J41"/>
     <mergeCell ref="G134:J134"/>
     <mergeCell ref="G50:J50"/>
+    <mergeCell ref="G164:J164"/>
     <mergeCell ref="G106:J106"/>
+    <mergeCell ref="G173:J173"/>
     <mergeCell ref="G56:J56"/>
+    <mergeCell ref="G14:J14"/>
     <mergeCell ref="G105:J105"/>
     <mergeCell ref="G43:J43"/>
     <mergeCell ref="G52:J52"/>
     <mergeCell ref="G27:J27"/>
     <mergeCell ref="G120:J120"/>
     <mergeCell ref="G36:J36"/>
+    <mergeCell ref="G42:J42"/>
     <mergeCell ref="G107:J107"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="G170:J170"/>
+    <mergeCell ref="G141:J141"/>
+    <mergeCell ref="G19:J19"/>
+    <mergeCell ref="G172:J172"/>
+    <mergeCell ref="G190:J190"/>
+    <mergeCell ref="G28:J28"/>
     <mergeCell ref="G93:J93"/>
+    <mergeCell ref="G6:J6"/>
     <mergeCell ref="G187:J187"/>
     <mergeCell ref="G69:J69"/>
+    <mergeCell ref="G83:J83"/>
     <mergeCell ref="G196:J196"/>
     <mergeCell ref="G205:J205"/>
     <mergeCell ref="G124:J124"/>
     <mergeCell ref="G180:J180"/>
+    <mergeCell ref="G5:J5"/>
     <mergeCell ref="G133:J133"/>
     <mergeCell ref="G45:J45"/>
   </mergeCells>

</xml_diff>

<commit_message>
The camera, the separated balls, directional passes, and the measurements
Pass sprites for all four directions, the court camera that zooms the scene
without the HUD, the in-play ball art split out of each Variaball's SVG and
palette-swapped onto the sprite, the referee on shot scenes, and the ball bench
for colour-correcting them.

Snow Ball now overrides the pass gain instead of cancelling it, Hero Ball shoots
at +25% and draws on its own rebound, Recharging Resin and MVPiquia read the
match's bag size, halftime no longer reshuffles, Play-On retires into Extravagant
Mechanics, and every Dribble draws one more.

Also the headless measurements this design work was argued from: discards,
bricks, shots, tempo, variety and density, plus what-makes-it-fun.md and the
rework doc they produced.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -2206,7 +2206,6 @@
         <v/>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="20.75" customHeight="1" s="85">
       <c r="A4" s="81" t="inlineStr">
         <is>
@@ -4338,21 +4337,17 @@
       </c>
       <c r="C80" s="24" t="inlineStr">
         <is>
-          <t>Play-On</t>
+          <t>Extravagant Mechanics</t>
         </is>
       </c>
       <c r="D80" s="25" t="inlineStr">
         <is>
-          <t>Discard each Game Break drawn and draw again, until a card is not one</t>
+          <t>Intangible, Varena, Variaball or Special Move Played: Cancel card.</t>
         </is>
       </c>
       <c r="E80" s="26" t="n"/>
       <c r="F80" s="50" t="n"/>
-      <c r="G80" s="72" t="inlineStr">
-        <is>
-          <t>Raised where the Break lands, like Cleared to Play — nobody plays a Break</t>
-        </is>
-      </c>
+      <c r="G80" s="72" t="n"/>
       <c r="H80" s="71" t="n"/>
       <c r="I80" s="71" t="n"/>
       <c r="J80" s="71" t="n"/>
@@ -6661,7 +6656,7 @@
       </c>
       <c r="D169" s="63" t="inlineStr">
         <is>
-          <t>Everyone refills to a hand of 5 at the start of their possession</t>
+          <t>Everyone refills their hand at the start of their possession</t>
         </is>
       </c>
       <c r="E169" s="58" t="n"/>
@@ -6721,7 +6716,7 @@
       </c>
       <c r="D171" s="63" t="inlineStr">
         <is>
-          <t>The highest scorer refills to 5 at the start of their possession</t>
+          <t>The highest scorer refills their hand at the start of their possession</t>
         </is>
       </c>
       <c r="E171" s="58" t="n"/>
@@ -7779,7 +7774,7 @@
       </c>
       <c r="D208" s="63" t="inlineStr">
         <is>
-          <t>Cannot play Pass cards. Made shots grant no AST</t>
+          <t>Cannot play Pass cards. Made shots grant no AST. SHOT +25% while shooting. Draw 1 extra when this Ball is rebounded</t>
         </is>
       </c>
       <c r="E208" s="58" t="n"/>
@@ -7801,9 +7796,9 @@
     <mergeCell ref="G135:J135"/>
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
+    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G119:J119"/>
     <mergeCell ref="G32:J32"/>
-    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G202:J202"/>
     <mergeCell ref="G46:J46"/>
     <mergeCell ref="G40:J40"/>

</xml_diff>

<commit_message>
Dishtracting Ball costs a card to shoot, not to catch
A toll every player paid the moment the ball reached them taxed the whole table
on every change of possession — and with three officials out and re-inbounds up,
it was the ball in play in all four games the soak could not finish. Paid by the
man who decided to put it up, it is a price against a decision instead.

The attempt is owed while he is being asked, so answering is what makes it go up
and nothing about the shot is lost in between. Soak is clean.

Shooting: Discard 1 card.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -3889,6 +3889,9 @@
           <t>Pace defender: only bites at 2 cards or fewer. Beaten by drawing back up</t>
         </is>
       </c>
+      <c r="H62" s="76" t="n"/>
+      <c r="I62" s="76" t="n"/>
+      <c r="J62" s="76" t="n"/>
     </row>
     <row r="63" ht="56" customHeight="1" s="85">
       <c r="B63" s="28" t="inlineStr">
@@ -3915,6 +3918,9 @@
           <t>Pace defender: only bites at 4 cards or more. Beaten by spending down</t>
         </is>
       </c>
+      <c r="H63" s="76" t="n"/>
+      <c r="I63" s="76" t="n"/>
+      <c r="J63" s="76" t="n"/>
     </row>
     <row r="64" ht="42" customHeight="1" s="85">
       <c r="B64" s="28" t="inlineStr">
@@ -3941,6 +3947,9 @@
           <t>Only bites late on the Shot Clock. Beaten by Resetting it</t>
         </is>
       </c>
+      <c r="H64" s="76" t="n"/>
+      <c r="I64" s="76" t="n"/>
+      <c r="J64" s="76" t="n"/>
     </row>
     <row r="65" ht="42" customHeight="1" s="85">
       <c r="B65" s="28" t="inlineStr">
@@ -3967,6 +3976,9 @@
           <t>Always bites. Beaten off the dribble</t>
         </is>
       </c>
+      <c r="H65" s="76" t="n"/>
+      <c r="I65" s="76" t="n"/>
+      <c r="J65" s="76" t="n"/>
     </row>
     <row r="66" ht="42" customHeight="1" s="85">
       <c r="B66" s="28" t="inlineStr">
@@ -3993,6 +4005,9 @@
           <t>Forcer: walks the player into a Layup, which Offensive Foul is watching</t>
         </is>
       </c>
+      <c r="H66" s="76" t="n"/>
+      <c r="I66" s="76" t="n"/>
+      <c r="J66" s="76" t="n"/>
     </row>
     <row r="67" ht="28" customHeight="1" s="85">
       <c r="B67" s="28" t="inlineStr">
@@ -4019,6 +4034,9 @@
           <t>Forcer: walks the player into a Three, which Foot On The Line is watching</t>
         </is>
       </c>
+      <c r="H67" s="76" t="n"/>
+      <c r="I67" s="76" t="n"/>
+      <c r="J67" s="76" t="n"/>
     </row>
     <row r="68" ht="42" customHeight="1" s="85">
       <c r="B68" s="28" t="inlineStr">
@@ -4045,6 +4063,9 @@
           <t>Forcer: walks the player into a Dunk, which Charge is watching</t>
         </is>
       </c>
+      <c r="H68" s="76" t="n"/>
+      <c r="I68" s="76" t="n"/>
+      <c r="J68" s="76" t="n"/>
     </row>
     <row r="69" ht="29" customHeight="1" s="85">
       <c r="A69" s="52" t="inlineStr">
@@ -4718,6 +4739,9 @@
           <t>Crew: watches the Layup</t>
         </is>
       </c>
+      <c r="H93" s="76" t="n"/>
+      <c r="I93" s="76" t="n"/>
+      <c r="J93" s="76" t="n"/>
     </row>
     <row r="94" ht="28" customHeight="1" s="85">
       <c r="A94" s="52" t="inlineStr">
@@ -5592,9 +5616,13 @@
       </c>
       <c r="E126" s="58" t="n"/>
       <c r="F126" s="59" t="n">
-        <v>2</v>
-      </c>
-      <c r="G126" s="75" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G126" s="75" t="inlineStr">
+        <is>
+          <t>Parked while the knocks are redesigned</t>
+        </is>
+      </c>
       <c r="H126" s="76" t="n"/>
       <c r="I126" s="76" t="n"/>
       <c r="J126" s="76" t="n"/>
@@ -5618,9 +5646,13 @@
       </c>
       <c r="E127" s="58" t="n"/>
       <c r="F127" s="59" t="n">
-        <v>2</v>
-      </c>
-      <c r="G127" s="75" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G127" s="75" t="inlineStr">
+        <is>
+          <t>Parked while the knocks are redesigned</t>
+        </is>
+      </c>
       <c r="H127" s="76" t="n"/>
       <c r="I127" s="76" t="n"/>
       <c r="J127" s="76" t="n"/>
@@ -5644,9 +5676,13 @@
       </c>
       <c r="E128" s="58" t="n"/>
       <c r="F128" s="59" t="n">
-        <v>2</v>
-      </c>
-      <c r="G128" s="75" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G128" s="75" t="inlineStr">
+        <is>
+          <t>Parked while the knocks are redesigned</t>
+        </is>
+      </c>
       <c r="H128" s="76" t="n"/>
       <c r="I128" s="76" t="n"/>
       <c r="J128" s="76" t="n"/>
@@ -5670,9 +5706,13 @@
       </c>
       <c r="E129" s="58" t="n"/>
       <c r="F129" s="59" t="n">
-        <v>2</v>
-      </c>
-      <c r="G129" s="75" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G129" s="75" t="inlineStr">
+        <is>
+          <t>Parked while the knocks are redesigned</t>
+        </is>
+      </c>
       <c r="H129" s="76" t="n"/>
       <c r="I129" s="76" t="n"/>
       <c r="J129" s="76" t="n"/>
@@ -5696,9 +5736,13 @@
       </c>
       <c r="E130" s="58" t="n"/>
       <c r="F130" s="59" t="n">
-        <v>2</v>
-      </c>
-      <c r="G130" s="75" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G130" s="75" t="inlineStr">
+        <is>
+          <t>Parked while the knocks are redesigned</t>
+        </is>
+      </c>
       <c r="H130" s="76" t="n"/>
       <c r="I130" s="76" t="n"/>
       <c r="J130" s="76" t="n"/>
@@ -5722,9 +5766,13 @@
       </c>
       <c r="E131" s="58" t="n"/>
       <c r="F131" s="59" t="n">
-        <v>2</v>
-      </c>
-      <c r="G131" s="75" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G131" s="75" t="inlineStr">
+        <is>
+          <t>Parked while the knocks are redesigned</t>
+        </is>
+      </c>
       <c r="H131" s="76" t="n"/>
       <c r="I131" s="76" t="n"/>
       <c r="J131" s="76" t="n"/>
@@ -5767,11 +5815,11 @@
       </c>
       <c r="E133" s="58" t="n"/>
       <c r="F133" s="61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G133" s="75" t="inlineStr">
         <is>
-          <t>Landing one discards every other Injury, and while one is on you a new Injury is discarded</t>
+          <t>Landing one discards every other Injury, and while one is on you a new Injury is discarded · Parked while the knocks are redesigned</t>
         </is>
       </c>
       <c r="H133" s="76" t="n"/>
@@ -5797,9 +5845,13 @@
       </c>
       <c r="E134" s="58" t="n"/>
       <c r="F134" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="G134" s="75" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G134" s="75" t="inlineStr">
+        <is>
+          <t>Parked while the knocks are redesigned</t>
+        </is>
+      </c>
       <c r="H134" s="76" t="n"/>
       <c r="I134" s="76" t="n"/>
       <c r="J134" s="76" t="n"/>
@@ -5823,9 +5875,13 @@
       </c>
       <c r="E135" s="58" t="n"/>
       <c r="F135" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="G135" s="75" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G135" s="75" t="inlineStr">
+        <is>
+          <t>Parked while the knocks are redesigned</t>
+        </is>
+      </c>
       <c r="H135" s="76" t="n"/>
       <c r="I135" s="76" t="n"/>
       <c r="J135" s="76" t="n"/>
@@ -5849,9 +5905,13 @@
       </c>
       <c r="E136" s="58" t="n"/>
       <c r="F136" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="G136" s="75" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G136" s="75" t="inlineStr">
+        <is>
+          <t>Parked while the knocks are redesigned</t>
+        </is>
+      </c>
       <c r="H136" s="76" t="n"/>
       <c r="I136" s="76" t="n"/>
       <c r="J136" s="76" t="n"/>
@@ -6658,6 +6718,8 @@
       </c>
       <c r="G166" s="75" t="n"/>
       <c r="H166" s="76" t="n"/>
+      <c r="I166" s="76" t="n"/>
+      <c r="J166" s="76" t="n"/>
     </row>
     <row r="167" s="85">
       <c r="A167" s="27" t="n"/>
@@ -6682,6 +6744,8 @@
       </c>
       <c r="G167" s="75" t="n"/>
       <c r="H167" s="76" t="n"/>
+      <c r="I167" s="76" t="n"/>
+      <c r="J167" s="76" t="n"/>
     </row>
     <row r="168" s="85">
       <c r="A168" s="52" t="inlineStr">
@@ -7758,7 +7822,7 @@
       </c>
       <c r="D204" s="63" t="inlineStr">
         <is>
-          <t>Receiving it: Discard 1, after the draw for turn</t>
+          <t>Shooting: Discard 1 card</t>
         </is>
       </c>
       <c r="E204" s="58" t="n"/>
@@ -8142,8 +8206,8 @@
     <mergeCell ref="G135:J135"/>
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
+    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G119:J119"/>
-    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G32:J32"/>
     <mergeCell ref="G202:J202"/>
     <mergeCell ref="G46:J46"/>

</xml_diff>

<commit_message>
Med Ball runs all day
A ball whose only word was a ceiling is a card you are sorry to be handed. The
other half makes picking it up a decision: you cannot get a good look with it,
but the man carrying it is never called for Traveling, so the speed limit the
crew works to simply does not apply to him.

SHOT cannot exceed 50%. Move cards never Travel.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -7706,7 +7706,7 @@
       </c>
       <c r="D200" s="63" t="inlineStr">
         <is>
-          <t>SHOT cannot exceed 50%</t>
+          <t>SHOT cannot exceed 50%. Move cards never Travel</t>
         </is>
       </c>
       <c r="E200" s="58" t="n"/>
@@ -8206,9 +8206,9 @@
     <mergeCell ref="G135:J135"/>
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
-    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G119:J119"/>
     <mergeCell ref="G32:J32"/>
+    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G202:J202"/>
     <mergeCell ref="G46:J46"/>
     <mergeCell ref="G40:J40"/>

</xml_diff>

<commit_message>
Blight Ball carries the TOV stat; player-facing hand → Bag, turn → possession
Receiving Blight Ball adds the last holder's TOV to yours and zeroes theirs,
with no prompt. Retiring it leaves the pile with whoever last had it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -1960,7 +1960,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>The most plentiful card type. Usually changes possession of the ball while increasing Shot %. If a player scores following a turn you gave them possession, you gain +1 AST</t>
+          <t>The most plentiful card type. Usually changes possession of the ball while increasing Shot %. If a player scores following a possession you gave them, you gain +1 AST</t>
         </is>
       </c>
       <c r="C6" s="7" t="n"/>
@@ -2089,7 +2089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J259"/>
+  <dimension ref="A1:J224"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="22.25" customHeight="1"/>
   <cols>
     <col width="15.5" customWidth="1" style="8" min="1" max="1"/>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="E8" s="26" t="inlineStr">
         <is>
-          <t>You may add current Ball to hand while passing.</t>
+          <t>You may add current Ball to your Bag while passing.</t>
         </is>
       </c>
       <c r="F8" s="33" t="n">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="D14" s="25" t="inlineStr">
         <is>
-          <t>SHOT +10%. Pass to target player. Retire 1 card from their hand while passing</t>
+          <t>SHOT +10%. Pass to target player. Retire 1 card from their Bag while passing</t>
         </is>
       </c>
       <c r="E14" s="25" t="n"/>
@@ -2542,7 +2542,7 @@
       </c>
       <c r="E15" s="25" t="inlineStr">
         <is>
-          <t>Receiving player shoots immediately after drawing for turn</t>
+          <t>Receiving player shoots immediately after drawing for possession</t>
         </is>
       </c>
       <c r="F15" s="36" t="n">
@@ -3446,7 +3446,7 @@
       </c>
       <c r="E46" s="25" t="inlineStr">
         <is>
-          <t>If you have 3 or more cards in hand, you may Retire them: SHOT = 100%</t>
+          <t>If you have 3 or more cards in your Bag, you may Retire them: SHOT = 100%</t>
         </is>
       </c>
       <c r="F46" s="36" t="n">
@@ -3680,7 +3680,7 @@
       </c>
       <c r="D55" s="25" t="inlineStr">
         <is>
-          <t>Target player Lock|2 Clear: 2 cards or fewer in hand</t>
+          <t>Target player Lock|2 Clear: 2 cards or fewer in Bag</t>
         </is>
       </c>
       <c r="E55" s="26" t="n"/>
@@ -3770,7 +3770,7 @@
       </c>
       <c r="D58" s="57" t="inlineStr">
         <is>
-          <t>Target player Lock|3 Clear: 1 card or fewer in hand</t>
+          <t>Target player Lock|3 Clear: 1 card or fewer in Bag</t>
         </is>
       </c>
       <c r="E58" s="58" t="n"/>
@@ -3885,7 +3885,7 @@
       </c>
       <c r="D62" s="57" t="inlineStr">
         <is>
-          <t>Target player with 2 cards or fewer in hand: SHOT -30% Clear: 4 cards or more in hand</t>
+          <t>Target player with 2 cards or fewer in Bag: SHOT -30% Clear: 4 cards or more in Bag</t>
         </is>
       </c>
       <c r="E62" s="58" t="n"/>
@@ -3914,7 +3914,7 @@
       </c>
       <c r="D63" s="57" t="inlineStr">
         <is>
-          <t>Target player with 4 cards or more in hand: SHOT -30% Clear: 2 cards or fewer in hand</t>
+          <t>Target player with 4 cards or more in Bag: SHOT -30% Clear: 2 cards or fewer in Bag</t>
         </is>
       </c>
       <c r="E63" s="58" t="n"/>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="D66" s="57" t="inlineStr">
         <is>
-          <t>Target player can only shoot a Layup Clear: 5 cards in hand</t>
+          <t>Target player can only shoot a Layup Clear: 5 cards in Bag</t>
         </is>
       </c>
       <c r="E66" s="58" t="n"/>
@@ -4030,7 +4030,7 @@
       </c>
       <c r="D67" s="57" t="inlineStr">
         <is>
-          <t>Target player can only shoot a Three Clear: 2 cards or fewer in hand</t>
+          <t>Target player can only shoot a Three Clear: 2 cards or fewer in Bag</t>
         </is>
       </c>
       <c r="E67" s="58" t="n"/>
@@ -4390,7 +4390,7 @@
       </c>
       <c r="D80" s="38" t="inlineStr">
         <is>
-          <t>Any other whistle triggers: Cancel that card. Turn player draws 1 card.</t>
+          <t>Any other whistle triggers: Cancel that card. Player in possession draws 1 card.</t>
         </is>
       </c>
       <c r="E80" s="7" t="n"/>
@@ -4866,7 +4866,7 @@
       </c>
       <c r="D98" s="6" t="inlineStr">
         <is>
-          <t>Draw up to a hand of 5</t>
+          <t>Draw up to a Bag of 5</t>
         </is>
       </c>
       <c r="E98" s="7" t="n"/>
@@ -4918,7 +4918,7 @@
       </c>
       <c r="D100" s="6" t="inlineStr">
         <is>
-          <t>Draw 3 cards up to a hand of 7</t>
+          <t>Draw 3 cards up to a Bag of 7</t>
         </is>
       </c>
       <c r="E100" s="7" t="n"/>
@@ -4970,7 +4970,7 @@
       </c>
       <c r="D102" s="6" t="inlineStr">
         <is>
-          <t>Whistle cards cannot activate this turn.</t>
+          <t>Whistle cards cannot activate this possession.</t>
         </is>
       </c>
       <c r="E102" s="6" t="inlineStr">
@@ -5030,7 +5030,7 @@
       </c>
       <c r="D104" s="6" t="inlineStr">
         <is>
-          <t>Swap hands with a random other player</t>
+          <t>Swap Bags with a random other player</t>
         </is>
       </c>
       <c r="E104" s="7" t="n"/>
@@ -5254,7 +5254,7 @@
       </c>
       <c r="D112" s="38" t="inlineStr">
         <is>
-          <t>Declare Left or Right: every player passes their hand that way. The ball goes with it</t>
+          <t>Declare Left or Right: every player passes their Bag that way. The ball goes with it</t>
         </is>
       </c>
       <c r="E112" s="7" t="n"/>
@@ -5284,7 +5284,7 @@
       </c>
       <c r="D113" s="38" t="inlineStr">
         <is>
-          <t>All players shuffle their hands into the deck and draw the same number of cards</t>
+          <t>All players shuffle their Bags into the deck and draw the same number of cards</t>
         </is>
       </c>
       <c r="E113" s="7" t="n"/>
@@ -5388,7 +5388,7 @@
       </c>
       <c r="D117" s="38" t="inlineStr">
         <is>
-          <t>All players discard their hands. If a ref is armed, all players receive 1 TOV. Inbound the ball</t>
+          <t>All players discard their Bags. If a ref is armed, all players receive 1 TOV. Inbound the ball</t>
         </is>
       </c>
       <c r="E117" s="7" t="n"/>
@@ -6013,7 +6013,7 @@
       </c>
       <c r="D140" s="6" t="inlineStr">
         <is>
-          <t>SHOT = 2X if you have 1 card or fewer in hand, or the Shot Clock is 03 or less</t>
+          <t>SHOT = 2X if you have 1 card or fewer in your Bag, or the Shot Clock is 03 or less</t>
         </is>
       </c>
       <c r="E140" s="7" t="n"/>
@@ -6547,7 +6547,7 @@
       </c>
       <c r="D160" s="38" t="inlineStr">
         <is>
-          <t>Discard your hand. Play a card at random from a player of your choosing (they keep it)</t>
+          <t>Discard your Bag. Play a card at random from a player of your choosing (they keep it)</t>
         </is>
       </c>
       <c r="E160" s="7" t="n"/>
@@ -6657,7 +6657,7 @@
       </c>
       <c r="D164" s="38" t="inlineStr">
         <is>
-          <t>A player may Retire this card and their hand: SHOT = 100%. All players' PTS become your new total PTS. (This card does not shuffle back into the deck once Retired and cannot be retrieved from Retirement)</t>
+          <t>A player may Retire this card and their Bag: SHOT = 100%. All players' PTS become your new total PTS. (This card does not shuffle back into the deck once Retired and cannot be retrieved from Retirement)</t>
         </is>
       </c>
       <c r="E164" s="7" t="n"/>
@@ -6968,7 +6968,7 @@
       </c>
       <c r="D175" s="63" t="inlineStr">
         <is>
-          <t>Hand limit 3</t>
+          <t>Max Bag size 3</t>
         </is>
       </c>
       <c r="E175" s="58" t="n"/>
@@ -7058,7 +7058,7 @@
       </c>
       <c r="D178" s="63" t="inlineStr">
         <is>
-          <t>Everyone refills their hand at the start of their possession</t>
+          <t>Everyone refills their Bag at the start of their possession</t>
         </is>
       </c>
       <c r="E178" s="58" t="n"/>
@@ -7118,7 +7118,7 @@
       </c>
       <c r="D180" s="63" t="inlineStr">
         <is>
-          <t>The highest scorer refills their hand at the start of their possession</t>
+          <t>The highest scorer refills their Bag at the start of their possession</t>
         </is>
       </c>
       <c r="E180" s="58" t="n"/>
@@ -7208,7 +7208,7 @@
       </c>
       <c r="D183" s="63" t="inlineStr">
         <is>
-          <t>Declare left or right. Every possession, hands move one seat that way</t>
+          <t>Declare left or right. Every possession, Bags move one seat that way</t>
         </is>
       </c>
       <c r="E183" s="58" t="n"/>
@@ -7238,7 +7238,7 @@
       </c>
       <c r="D184" s="63" t="inlineStr">
         <is>
-          <t>During your turn, hand off any number of the Clamps on you to other players</t>
+          <t>During your possession, hand off any number of the Clamps on you to other players</t>
         </is>
       </c>
       <c r="E184" s="58" t="n"/>
@@ -7298,7 +7298,7 @@
       </c>
       <c r="D186" s="63" t="inlineStr">
         <is>
-          <t>At the start of your possession, before your draw: discard your hand</t>
+          <t>At the start of your possession, before your draw: discard your Bag</t>
         </is>
       </c>
       <c r="E186" s="58" t="n"/>
@@ -7360,7 +7360,7 @@
       </c>
       <c r="D188" s="63" t="inlineStr">
         <is>
-          <t>Every possession, everyone but the turn player draws 1</t>
+          <t>Every possession, everyone but the player in possession draws 1</t>
         </is>
       </c>
       <c r="E188" s="58" t="n"/>
@@ -7390,7 +7390,7 @@
       </c>
       <c r="D189" s="63" t="inlineStr">
         <is>
-          <t>The draw for turn goes to a random player each possession</t>
+          <t>The draw for possession goes to a random player each possession</t>
         </is>
       </c>
       <c r="E189" s="58" t="n"/>
@@ -7774,7 +7774,7 @@
       </c>
       <c r="D202" s="63" t="inlineStr">
         <is>
-          <t>Injuries travel with the ball, and new ones join the pile. Discarding the ball takes the pile with it</t>
+          <t>TOV travels with the ball: whoever receives it takes on the last holder's TOV</t>
         </is>
       </c>
       <c r="E202" s="58" t="n"/>
@@ -7783,7 +7783,7 @@
       </c>
       <c r="G202" s="75" t="inlineStr">
         <is>
-          <t>Moves on any change of hands</t>
+          <t>Moves on any change of hands; last holder keeps it once Retired</t>
         </is>
       </c>
       <c r="H202" s="76" t="n"/>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="D205" s="63" t="inlineStr">
         <is>
-          <t>A Pass swaps hands: yours goes with the ball, theirs comes back</t>
+          <t>A Pass swaps Bags: yours goes with the ball, theirs comes back</t>
         </is>
       </c>
       <c r="E205" s="58" t="n"/>
@@ -7912,7 +7912,7 @@
       </c>
       <c r="D207" s="63" t="inlineStr">
         <is>
-          <t>Double your draw for turn</t>
+          <t>Double your draw for possession</t>
         </is>
       </c>
       <c r="E207" s="58" t="n"/>
@@ -7968,7 +7968,7 @@
       </c>
       <c r="D209" s="63" t="inlineStr">
         <is>
-          <t>Every possession, the turn player shuffles their hand into the deck and Draws the same number, then draws for turn</t>
+          <t>Every possession, the player in possession shuffles their Bag into the deck and Draws the same number, then draws for possession</t>
         </is>
       </c>
       <c r="E209" s="58" t="n"/>
@@ -7994,7 +7994,7 @@
       </c>
       <c r="D210" s="63" t="inlineStr">
         <is>
-          <t>Draw 1 card when played. SHOT = 10% for each card in your hand</t>
+          <t>Draw 1 card when played. SHOT = 10% for each card in your Bag</t>
         </is>
       </c>
       <c r="E210" s="58" t="n"/>
@@ -8414,41 +8414,6 @@
       <c r="I224" s="71" t="n"/>
       <c r="J224" s="71" t="n"/>
     </row>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
   </sheetData>
   <mergeCells count="186">
     <mergeCell ref="G55:J55"/>

</xml_diff>

<commit_message>
Blight Ball text: TOVs travel with the ball.
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -7774,7 +7774,7 @@
       </c>
       <c r="D202" s="63" t="inlineStr">
         <is>
-          <t>TOV travels with the ball: whoever receives it takes on the last holder's TOV</t>
+          <t>TOVs travel with the ball.</t>
         </is>
       </c>
       <c r="E202" s="58" t="n"/>
@@ -8424,8 +8424,8 @@
     <mergeCell ref="G135:J135"/>
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
+    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G119:J119"/>
-    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G32:J32"/>
     <mergeCell ref="G202:J202"/>
     <mergeCell ref="G46:J46"/>

</xml_diff>

<commit_message>
Clamp audit: new Clears, shot bans, trims to 50; Clamp reward removed
- Target player dropped from Clamp text; Open keyword (no Clamps on them)
- Clears on events: Attempt a Shot, Pass the ball, Pass to an Open player,
  Play an Intangible or change the ball, Any stoppage of play
- Crushing Center no Dunk; Pressing Point and Rim Runner no Layup
- Full-Court Press Moves only; Baseline Denial shoot only; Waiting Wing (was Lurking)
- Meeting a Clear retires the Clamp; the payoff choice is gone

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -2206,6 +2206,7 @@
         <v/>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="20.75" customHeight="1" s="85">
       <c r="A4" s="81" t="inlineStr">
         <is>
@@ -3650,12 +3651,12 @@
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>Target player: SHOT -25% Clear: SHOT 60% or more</t>
+          <t>SHOT -25% when shooting Clear: SHOT above 50%</t>
         </is>
       </c>
       <c r="E54" s="7" t="n"/>
       <c r="F54" s="34" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G54" s="80" t="inlineStr">
         <is>
@@ -3680,7 +3681,7 @@
       </c>
       <c r="D55" s="25" t="inlineStr">
         <is>
-          <t>Target player Lock|2 Clear: 2 cards or fewer in Bag</t>
+          <t>Lock 2 cards Clear: 2 cards or fewer in Bag</t>
         </is>
       </c>
       <c r="E55" s="26" t="n"/>
@@ -3710,12 +3711,12 @@
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
-          <t>Target player Retire|2</t>
+          <t>Can only play Move cards Clear: Play 3 Move cards in a possession</t>
         </is>
       </c>
       <c r="E56" s="7" t="n"/>
       <c r="F56" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G56" s="80" t="inlineStr">
         <is>
@@ -3740,12 +3741,12 @@
       </c>
       <c r="D57" s="41" t="inlineStr">
         <is>
-          <t>Target player can only Pass or Shoot Clear: Give up the ball</t>
+          <t>Can only Pass or Shoot Clear: Pass to an Open player</t>
         </is>
       </c>
       <c r="E57" s="26" t="n"/>
       <c r="F57" s="33" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G57" s="77" t="inlineStr">
         <is>
@@ -3770,7 +3771,7 @@
       </c>
       <c r="D58" s="57" t="inlineStr">
         <is>
-          <t>Target player Lock|3 Clear: 1 card or fewer in Bag</t>
+          <t>Lock 3 cards Clear: Pass the ball</t>
         </is>
       </c>
       <c r="E58" s="58" t="n"/>
@@ -3800,12 +3801,12 @@
       </c>
       <c r="D59" s="57" t="inlineStr">
         <is>
-          <t>Target player cannot attempt a Three Clear: Shot Clock 03 or less</t>
+          <t>Cannot attempt a Three Clear: Attempt a Shot</t>
         </is>
       </c>
       <c r="E59" s="58" t="n"/>
       <c r="F59" s="59" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G59" s="83" t="inlineStr">
         <is>
@@ -3830,7 +3831,7 @@
       </c>
       <c r="D60" s="57" t="inlineStr">
         <is>
-          <t>Target player cannot Shoot. With no playable Pass cards, TOV +1 and the round ends Clear: Give up the ball</t>
+          <t>Cannot Shoot. With no playable Pass cards, TOV +1 and the round ends Clear: Pass the ball</t>
         </is>
       </c>
       <c r="E60" s="58" t="n"/>
@@ -3860,12 +3861,12 @@
       </c>
       <c r="D61" s="57" t="inlineStr">
         <is>
-          <t>Target player: SHOT -10% each time a card is played Clear: 3 Move cards this possession</t>
+          <t>SHOT -10% each time a card is played Clear: 3 Move cards this possession</t>
         </is>
       </c>
       <c r="E61" s="58" t="n"/>
       <c r="F61" s="59" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G61" s="83" t="n"/>
       <c r="H61" s="76" t="n"/>
@@ -3885,12 +3886,12 @@
       </c>
       <c r="D62" s="57" t="inlineStr">
         <is>
-          <t>Target player with 2 cards or fewer in Bag: SHOT -30% Clear: 4 cards or more in Bag</t>
+          <t>2 cards or fewer in Bag: SHOT -30% Cannot Dunk Clear: 4 cards or more in Bag</t>
         </is>
       </c>
       <c r="E62" s="58" t="n"/>
       <c r="F62" s="59" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G62" s="83" t="inlineStr">
         <is>
@@ -3914,12 +3915,12 @@
       </c>
       <c r="D63" s="57" t="inlineStr">
         <is>
-          <t>Target player with 4 cards or more in Bag: SHOT -30% Clear: 2 cards or fewer in Bag</t>
+          <t>4 cards or more in Bag: SHOT -30% Cannot shoot Layups Clear: 2 cards or fewer in Bag</t>
         </is>
       </c>
       <c r="E63" s="58" t="n"/>
       <c r="F63" s="59" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G63" s="83" t="inlineStr">
         <is>
@@ -3938,17 +3939,17 @@
       </c>
       <c r="C64" s="56" t="inlineStr">
         <is>
-          <t>Lurking Wing</t>
+          <t>Waiting Wing</t>
         </is>
       </c>
       <c r="D64" s="57" t="inlineStr">
         <is>
-          <t>Target player at Shot Clock 05 or less: SHOT -25% Clear: Shot Clock 06 or more</t>
+          <t>2 to 4 cards in Bag: SHOT -30% Clear: 1 card or fewer, or 5 cards or more in Bag</t>
         </is>
       </c>
       <c r="E64" s="58" t="n"/>
       <c r="F64" s="59" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G64" s="83" t="inlineStr">
         <is>
@@ -3972,12 +3973,12 @@
       </c>
       <c r="D65" s="57" t="inlineStr">
         <is>
-          <t>Target player: SHOT -15% Clear: 2 Move cards this possession</t>
+          <t>SHOT -15% Clear: Play an Intangible or change the Ball</t>
         </is>
       </c>
       <c r="E65" s="58" t="n"/>
       <c r="F65" s="59" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G65" s="83" t="inlineStr">
         <is>
@@ -4001,12 +4002,12 @@
       </c>
       <c r="D66" s="57" t="inlineStr">
         <is>
-          <t>Target player can only shoot a Layup Clear: 5 cards in Bag</t>
+          <t>Can only Shoot Clear: Any stoppage of play</t>
         </is>
       </c>
       <c r="E66" s="58" t="n"/>
       <c r="F66" s="59" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G66" s="83" t="inlineStr">
         <is>
@@ -4030,12 +4031,12 @@
       </c>
       <c r="D67" s="57" t="inlineStr">
         <is>
-          <t>Target player can only shoot a Three Clear: 2 cards or fewer in Bag</t>
+          <t>When shooting: can only shoot a Three Clear: Pass the ball</t>
         </is>
       </c>
       <c r="E67" s="58" t="n"/>
       <c r="F67" s="59" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G67" s="83" t="inlineStr">
         <is>
@@ -4059,12 +4060,12 @@
       </c>
       <c r="D68" s="57" t="inlineStr">
         <is>
-          <t>Target player can only shoot a Dunk Clear: SHOT 40% or less</t>
+          <t>Cannot shoot Layups Clear: SHOT 40% or less</t>
         </is>
       </c>
       <c r="E68" s="58" t="n"/>
       <c r="F68" s="59" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G68" s="83" t="inlineStr">
         <is>
@@ -8424,9 +8425,9 @@
     <mergeCell ref="G135:J135"/>
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
-    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G119:J119"/>
     <mergeCell ref="G32:J32"/>
+    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G202:J202"/>
     <mergeCell ref="G46:J46"/>
     <mergeCell ref="G40:J40"/>

</xml_diff>

<commit_message>
Cuts: passing the ball without a Pass card; four harness stalls fixed
- Backdoor, Flare, Flash, Curl Cut (x3) and L-Cut, V-Cut (x1): only while
  Clamped, Clamps travel with the ball, receiver's forced first action
- Spin Move and Crossover to 3; deck back to 300
- Card shots set their shot type before the crew reads it, and Foot On The
  Line only takes the point; Skyhook never pulls itself from Retirement
- Force picks, declined Challenges and Pump Fake naming now check for a
  dead possession

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -2089,7 +2089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J224"/>
+  <dimension ref="A1:J230"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="22.25" customHeight="1"/>
   <cols>
     <col width="15.5" customWidth="1" style="8" min="1" max="1"/>
@@ -2986,7 +2986,7 @@
         </is>
       </c>
       <c r="F30" s="33" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G30" s="77" t="inlineStr">
         <is>
@@ -3020,7 +3020,7 @@
         </is>
       </c>
       <c r="F31" s="33" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G31" s="77" t="inlineStr">
         <is>
@@ -8414,6 +8414,156 @@
       <c r="H224" s="71" t="n"/>
       <c r="I224" s="71" t="n"/>
       <c r="J224" s="71" t="n"/>
+    </row>
+    <row r="225">
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Move</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Backdoor Cut</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>If Clamped: Draw 1 card. Pass your Clamps and the ball to target player. They must Pass as their first action. (If they cannot, TOV +1)</t>
+        </is>
+      </c>
+      <c r="F225" t="n">
+        <v>3</v>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>Cut: passes the ball without a Pass card; only playable while Clamped</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Move</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Flare Cut</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>If Clamped: Draw 1 card. Pass your Clamps and the ball to target player. They must Shoot as their first action. (If they cannot, TOV +1)</t>
+        </is>
+      </c>
+      <c r="F226" t="n">
+        <v>3</v>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>Cut: passes the ball without a Pass card; only playable while Clamped</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Move</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Flash Cut</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>If Clamped: Draw 1 card. Pass your Clamps and the ball to target player. They must play a Move card as their first action. (If they cannot, TOV +1)</t>
+        </is>
+      </c>
+      <c r="F227" t="n">
+        <v>3</v>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>Cut: passes the ball without a Pass card; only playable while Clamped</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Move</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Curl Cut</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>If Clamped: Draw 1 card. Pass your Clamps and the ball to target player. Force 1 random card from their Bag to yours</t>
+        </is>
+      </c>
+      <c r="F228" t="n">
+        <v>3</v>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>Cut: passes the ball without a Pass card; only playable while Clamped</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Special Move</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>L-Cut</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>If Clamped: Draw 2 cards. Pass your Clamps and the ball to target player. You may Retire target Ref, Intangible, or the Ball</t>
+        </is>
+      </c>
+      <c r="F229" t="n">
+        <v>1</v>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>Cut: passes the ball without a Pass card; only playable while Clamped</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Special Move</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>V-Cut</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>If Clamped: Draw 2 cards. Pass your Clamps and the ball to target player, who passes it back immediately. SHOT +30% if your first action is a Three</t>
+        </is>
+      </c>
+      <c r="F230" t="n">
+        <v>1</v>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>Cut: passes the ball without a Pass card; only playable while Clamped</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="186">
@@ -8426,8 +8576,8 @@
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
     <mergeCell ref="G119:J119"/>
+    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G32:J32"/>
-    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G202:J202"/>
     <mergeCell ref="G46:J46"/>
     <mergeCell ref="G40:J40"/>

</xml_diff>

<commit_message>
Retirement picker, Ref deck rule, Flagrant Foul on any Clamp
- Skyhook chooses a card from Retirement (never another Skyhook) before shooting
- Varsitile exchanges the Ball or an Intangible for one in Retirement, via the
  same picker; old floor-and-ball exchange removed
- Tapping Retirement opens it: the whole pile footprint is the target
- Retired Refs go to the bottom of the Ref deck, which shuffles every round;
  The Equalizer leaves the game when Retired
- Flagrant Foul fires on any Clamp assignment

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -4313,7 +4313,7 @@
       </c>
       <c r="D77" s="41" t="inlineStr">
         <is>
-          <t>Clamp that Retires cards: no effect. Clamper Retires 1. Target player +1 FT and keeps the ball</t>
+          <t>Clamp assigned: no effect. Clamper Retires 1. Target player +1 FT and keeps the ball</t>
         </is>
       </c>
       <c r="E77" s="26" t="n"/>
@@ -8416,150 +8416,150 @@
       <c r="J224" s="71" t="n"/>
     </row>
     <row r="225">
-      <c r="B225" t="inlineStr">
+      <c r="B225" s="0" t="inlineStr">
         <is>
           <t>Move</t>
         </is>
       </c>
-      <c r="C225" t="inlineStr">
+      <c r="C225" s="0" t="inlineStr">
         <is>
           <t>Backdoor Cut</t>
         </is>
       </c>
-      <c r="D225" t="inlineStr">
+      <c r="D225" s="0" t="inlineStr">
         <is>
           <t>If Clamped: Draw 1 card. Pass your Clamps and the ball to target player. They must Pass as their first action. (If they cannot, TOV +1)</t>
         </is>
       </c>
-      <c r="F225" t="n">
+      <c r="F225" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="G225" t="inlineStr">
+      <c r="G225" s="0" t="inlineStr">
         <is>
           <t>Cut: passes the ball without a Pass card; only playable while Clamped</t>
         </is>
       </c>
     </row>
     <row r="226">
-      <c r="B226" t="inlineStr">
+      <c r="B226" s="0" t="inlineStr">
         <is>
           <t>Move</t>
         </is>
       </c>
-      <c r="C226" t="inlineStr">
+      <c r="C226" s="0" t="inlineStr">
         <is>
           <t>Flare Cut</t>
         </is>
       </c>
-      <c r="D226" t="inlineStr">
+      <c r="D226" s="0" t="inlineStr">
         <is>
           <t>If Clamped: Draw 1 card. Pass your Clamps and the ball to target player. They must Shoot as their first action. (If they cannot, TOV +1)</t>
         </is>
       </c>
-      <c r="F226" t="n">
+      <c r="F226" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="G226" t="inlineStr">
+      <c r="G226" s="0" t="inlineStr">
         <is>
           <t>Cut: passes the ball without a Pass card; only playable while Clamped</t>
         </is>
       </c>
     </row>
     <row r="227">
-      <c r="B227" t="inlineStr">
+      <c r="B227" s="0" t="inlineStr">
         <is>
           <t>Move</t>
         </is>
       </c>
-      <c r="C227" t="inlineStr">
+      <c r="C227" s="0" t="inlineStr">
         <is>
           <t>Flash Cut</t>
         </is>
       </c>
-      <c r="D227" t="inlineStr">
+      <c r="D227" s="0" t="inlineStr">
         <is>
           <t>If Clamped: Draw 1 card. Pass your Clamps and the ball to target player. They must play a Move card as their first action. (If they cannot, TOV +1)</t>
         </is>
       </c>
-      <c r="F227" t="n">
+      <c r="F227" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="G227" t="inlineStr">
+      <c r="G227" s="0" t="inlineStr">
         <is>
           <t>Cut: passes the ball without a Pass card; only playable while Clamped</t>
         </is>
       </c>
     </row>
     <row r="228">
-      <c r="B228" t="inlineStr">
+      <c r="B228" s="0" t="inlineStr">
         <is>
           <t>Move</t>
         </is>
       </c>
-      <c r="C228" t="inlineStr">
+      <c r="C228" s="0" t="inlineStr">
         <is>
           <t>Curl Cut</t>
         </is>
       </c>
-      <c r="D228" t="inlineStr">
+      <c r="D228" s="0" t="inlineStr">
         <is>
           <t>If Clamped: Draw 1 card. Pass your Clamps and the ball to target player. Force 1 random card from their Bag to yours</t>
         </is>
       </c>
-      <c r="F228" t="n">
+      <c r="F228" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="G228" t="inlineStr">
+      <c r="G228" s="0" t="inlineStr">
         <is>
           <t>Cut: passes the ball without a Pass card; only playable while Clamped</t>
         </is>
       </c>
     </row>
     <row r="229">
-      <c r="B229" t="inlineStr">
+      <c r="B229" s="0" t="inlineStr">
         <is>
           <t>Special Move</t>
         </is>
       </c>
-      <c r="C229" t="inlineStr">
+      <c r="C229" s="0" t="inlineStr">
         <is>
           <t>L-Cut</t>
         </is>
       </c>
-      <c r="D229" t="inlineStr">
+      <c r="D229" s="0" t="inlineStr">
         <is>
           <t>If Clamped: Draw 2 cards. Pass your Clamps and the ball to target player. You may Retire target Ref, Intangible, or the Ball</t>
         </is>
       </c>
-      <c r="F229" t="n">
+      <c r="F229" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G229" t="inlineStr">
+      <c r="G229" s="0" t="inlineStr">
         <is>
           <t>Cut: passes the ball without a Pass card; only playable while Clamped</t>
         </is>
       </c>
     </row>
     <row r="230">
-      <c r="B230" t="inlineStr">
+      <c r="B230" s="0" t="inlineStr">
         <is>
           <t>Special Move</t>
         </is>
       </c>
-      <c r="C230" t="inlineStr">
+      <c r="C230" s="0" t="inlineStr">
         <is>
           <t>V-Cut</t>
         </is>
       </c>
-      <c r="D230" t="inlineStr">
+      <c r="D230" s="0" t="inlineStr">
         <is>
           <t>If Clamped: Draw 2 cards. Pass your Clamps and the ball to target player, who passes it back immediately. SHOT +30% if your first action is a Three</t>
         </is>
       </c>
-      <c r="F230" t="n">
+      <c r="F230" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G230" t="inlineStr">
+      <c r="G230" s="0" t="inlineStr">
         <is>
           <t>Cut: passes the ball without a Pass card; only playable while Clamped</t>
         </is>
@@ -8575,8 +8575,8 @@
     <mergeCell ref="G135:J135"/>
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
+    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G119:J119"/>
-    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G32:J32"/>
     <mergeCell ref="G202:J202"/>
     <mergeCell ref="G46:J46"/>

</xml_diff>

<commit_message>
Refs everywhere, and a catch that plays every time
The rename had landed in the game — the type prints as Ref — but the sheet was
still typed Whistle throughout, formulas included, and three card texts still
said it. Both done: 31 type cells, 2 COUNTIFs, and the four effect lines that
name the type.

The catch was owned by two tasks. The throw-in stamped the landing and the
pass task cleared it on its way past, so the animation played on some balls
and not others; the stamp is only ever moved forward now and the figure picks
itself out of it. The throw-in's own flight time joins the bench's pass door.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -1970,7 +1970,7 @@
     <row r="7" ht="32" customHeight="1" s="85">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="E1" s="11" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="F1" s="11" t="inlineStr">
@@ -2182,7 +2182,7 @@
         <v/>
       </c>
       <c r="E2" s="15">
-        <f>COUNTIF($B$5:$B$154,"Whistle")</f>
+        <f>COUNTIF($B$5:$B$154,"Ref")</f>
         <v/>
       </c>
       <c r="F2" s="16">
@@ -2206,6 +2206,7 @@
         <v/>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="20.75" customHeight="1" s="85">
       <c r="A4" s="81" t="inlineStr">
         <is>
@@ -4082,11 +4083,11 @@
     <row r="69" ht="29" customHeight="1" s="85">
       <c r="A69" s="52" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="B69" s="53">
-        <f>COUNTIF($B$63:$B$158,"Whistle")</f>
+        <f>COUNTIF($B$63:$B$158,"Ref")</f>
         <v/>
       </c>
       <c r="C69" s="54" t="n"/>
@@ -4106,7 +4107,7 @@
       </c>
       <c r="B70" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C70" s="23" t="inlineStr">
@@ -4136,7 +4137,7 @@
       <c r="A71" s="21" t="n"/>
       <c r="B71" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C71" s="37" t="inlineStr">
@@ -4162,7 +4163,7 @@
       <c r="A72" s="21" t="n"/>
       <c r="B72" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C72" s="23" t="inlineStr">
@@ -4188,7 +4189,7 @@
       <c r="A73" s="21" t="n"/>
       <c r="B73" s="22" t="inlineStr">
         <is>
-          <t>Retired Whistle</t>
+          <t>Retired Ref</t>
         </is>
       </c>
       <c r="C73" s="24" t="inlineStr">
@@ -4214,7 +4215,7 @@
       <c r="A74" s="21" t="n"/>
       <c r="B74" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C74" s="23" t="inlineStr">
@@ -4224,7 +4225,7 @@
       </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
-          <t>Any Whistle Card Played: Cancel card.</t>
+          <t>Any Ref Card Played: Cancel card.</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
@@ -4242,7 +4243,7 @@
       <c r="A75" s="21" t="n"/>
       <c r="B75" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C75" s="37" t="inlineStr">
@@ -4276,7 +4277,7 @@
       <c r="A76" s="21" t="n"/>
       <c r="B76" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C76" s="23" t="inlineStr">
@@ -4306,7 +4307,7 @@
       <c r="A77" s="21" t="n"/>
       <c r="B77" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C77" s="37" t="inlineStr">
@@ -4332,7 +4333,7 @@
       <c r="A78" s="21" t="n"/>
       <c r="B78" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C78" s="37" t="inlineStr">
@@ -4358,7 +4359,7 @@
       <c r="A79" s="21" t="n"/>
       <c r="B79" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C79" s="24" t="inlineStr">
@@ -4384,7 +4385,7 @@
       <c r="A80" s="21" t="n"/>
       <c r="B80" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C80" s="23" t="inlineStr">
@@ -4394,7 +4395,7 @@
       </c>
       <c r="D80" s="38" t="inlineStr">
         <is>
-          <t>Any other whistle triggers: Cancel that card. Player in possession draws 1 card.</t>
+          <t>Any other Ref triggers: Cancel that card. Player in possession draws 1 card.</t>
         </is>
       </c>
       <c r="E80" s="7" t="n"/>
@@ -4408,7 +4409,7 @@
       <c r="A81" s="21" t="n"/>
       <c r="B81" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C81" s="24" t="inlineStr">
@@ -4434,7 +4435,7 @@
       <c r="A82" s="21" t="n"/>
       <c r="B82" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C82" s="23" t="inlineStr">
@@ -4464,7 +4465,7 @@
       <c r="A83" s="21" t="n"/>
       <c r="B83" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C83" s="24" t="inlineStr">
@@ -4490,7 +4491,7 @@
       <c r="A84" s="21" t="n"/>
       <c r="B84" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C84" s="23" t="inlineStr">
@@ -4514,7 +4515,7 @@
       <c r="A85" s="21" t="n"/>
       <c r="B85" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C85" s="24" t="inlineStr">
@@ -4540,7 +4541,7 @@
       <c r="A86" s="21" t="n"/>
       <c r="B86" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C86" s="24" t="inlineStr">
@@ -4570,7 +4571,7 @@
       <c r="A87" s="21" t="n"/>
       <c r="B87" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C87" s="24" t="inlineStr">
@@ -4596,7 +4597,7 @@
       <c r="A88" s="27" t="n"/>
       <c r="B88" s="28" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C88" s="29" t="inlineStr">
@@ -4620,7 +4621,7 @@
       <c r="A89" s="27" t="n"/>
       <c r="B89" s="28" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C89" s="29" t="inlineStr">
@@ -4646,7 +4647,7 @@
       <c r="A90" s="27" t="n"/>
       <c r="B90" s="28" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C90" s="29" t="inlineStr">
@@ -4674,7 +4675,7 @@
       <c r="A91" s="27" t="n"/>
       <c r="B91" s="28" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C91" s="29" t="inlineStr">
@@ -4703,7 +4704,7 @@
     <row r="92" ht="42" customHeight="1" s="85">
       <c r="B92" s="28" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C92" s="29" t="inlineStr">
@@ -4729,7 +4730,7 @@
     <row r="93" ht="42" customHeight="1" s="85">
       <c r="B93" s="28" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C93" s="29" t="inlineStr">
@@ -4974,7 +4975,7 @@
       </c>
       <c r="D102" s="6" t="inlineStr">
         <is>
-          <t>Whistle cards cannot activate this possession.</t>
+          <t>Ref cards cannot activate this possession.</t>
         </is>
       </c>
       <c r="E102" s="6" t="inlineStr">
@@ -6651,7 +6652,7 @@
       <c r="A164" s="21" t="n"/>
       <c r="B164" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C164" s="23" t="inlineStr">
@@ -6882,7 +6883,7 @@
       </c>
       <c r="D172" s="63" t="inlineStr">
         <is>
-          <t>Clear All Whistles. Whistles Cannot Be Played. All Clamps are enhanced</t>
+          <t>Clear All Refs. Refs Cannot Be Played. All Clamps are enhanced</t>
         </is>
       </c>
       <c r="E172" s="58" t="n"/>
@@ -8272,7 +8273,7 @@
       <c r="A220" s="21" t="n"/>
       <c r="B220" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C220" s="23" t="inlineStr">
@@ -8302,7 +8303,7 @@
       <c r="A221" s="21" t="n"/>
       <c r="B221" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C221" s="23" t="inlineStr">
@@ -8332,7 +8333,7 @@
       <c r="A222" s="21" t="n"/>
       <c r="B222" s="22" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Ref</t>
         </is>
       </c>
       <c r="C222" s="23" t="inlineStr">
@@ -8578,9 +8579,9 @@
     <mergeCell ref="G135:J135"/>
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
-    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G119:J119"/>
     <mergeCell ref="G32:J32"/>
+    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G202:J202"/>
     <mergeCell ref="G46:J46"/>
     <mergeCell ref="G40:J40"/>

</xml_diff>

<commit_message>
Four cards, and the man holding it when the clock dies
Floater gives half what it did — it was paying more than the Skyhook for a
layup. One Clamp a player means one word for ignoring it, so it ignores Clamps
rather than a target one. Flagrant Foul II loses the clause about clamping a
clamped man, which cannot happen any more. Foot Ball keeps its hands off
Special Moves: a finish is a shot going up, and keeping one in the hand is
keeping the shot.

And nought on the clock is still a violation on whoever is holding the ball.
The period ends either way — that is the clock on the wall — but somebody was
standing there with it when it went.

A puff clears now. Pausing a timeline freezes its date at the last tick and
that tick is inside the sheet, so the smoke held its final cell for the rest
of the game.

A Pass held up lights the men it could reach: the floor dims a man at a time
for one instead of putting a sheet over the arrows.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -2206,7 +2206,6 @@
         <v/>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="20.75" customHeight="1" s="85">
       <c r="A4" s="81" t="inlineStr">
         <is>
@@ -4343,7 +4342,7 @@
       </c>
       <c r="D78" s="38" t="inlineStr">
         <is>
-          <t>Clamp on a clamped player: Clamper Retires 2. Target player +1 FT</t>
+          <t>Clamp played: Clamper Retires 2. Target player +1 FT</t>
         </is>
       </c>
       <c r="E78" s="7" t="n"/>
@@ -7891,7 +7890,7 @@
       </c>
       <c r="D206" s="63" t="inlineStr">
         <is>
-          <t>Moves and Passes are not spent. They lock until your possession ends</t>
+          <t>Moves and Passes are not spent, except Special Moves. They lock until your possession ends</t>
         </is>
       </c>
       <c r="E206" s="58" t="n"/>
@@ -8373,7 +8372,7 @@
       </c>
       <c r="D223" s="38" t="inlineStr">
         <is>
-          <t>Draw 1 card. SHOT +30% Ignore target Clamp</t>
+          <t>Draw 1 card. SHOT +15% Ignores Clamps</t>
         </is>
       </c>
       <c r="E223" s="7" t="n"/>
@@ -8580,8 +8579,8 @@
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
     <mergeCell ref="G119:J119"/>
+    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G32:J32"/>
-    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G202:J202"/>
     <mergeCell ref="G46:J46"/>
     <mergeCell ref="G40:J40"/>

</xml_diff>

<commit_message>
A dunk starts behind the wall, and a Review shuts the slot
He was being pushed back by the trip instead of starting there, so a miss —
which never reaches the ring — never got the moment that would have moved him,
and he rose in front of the men he was supposed to be climbing past. He starts
behind now and comes forward when he is over the ring, which a failed dunk
never is.

Official Review stops a new Intangible going down rather than trimming the
slots to one. Whatever is already standing there stays: he is reviewing the
call, not clearing the table.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -4418,7 +4418,7 @@
       </c>
       <c r="D81" s="41" t="inlineStr">
         <is>
-          <t>Intangible slots: 1</t>
+          <t>Cannot place a new Intangible</t>
         </is>
       </c>
       <c r="E81" s="26" t="n"/>
@@ -8578,8 +8578,8 @@
     <mergeCell ref="G135:J135"/>
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
+    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G119:J119"/>
-    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G32:J32"/>
     <mergeCell ref="G202:J202"/>
     <mergeCell ref="G46:J46"/>

</xml_diff>

<commit_message>
Clutch Gene is back to 03
Game and sheet.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -6017,7 +6017,7 @@
       </c>
       <c r="D140" s="6" t="inlineStr">
         <is>
-          <t>SHOT = 2X if you have 1 card or fewer in your Bag, or the Shot Clock is 05 or less</t>
+          <t>SHOT = 2X if you have 1 card or fewer in your Bag, or the Shot Clock is 03 or less</t>
         </is>
       </c>
       <c r="E140" s="7" t="n"/>
@@ -8578,9 +8578,9 @@
     <mergeCell ref="G135:J135"/>
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
-    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G119:J119"/>
     <mergeCell ref="G32:J32"/>
+    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G202:J202"/>
     <mergeCell ref="G46:J46"/>
     <mergeCell ref="G40:J40"/>

</xml_diff>

<commit_message>
Shot Clock Violation resets the clock to 14
"If it is higher" was a clause that could never fire once a quarter started at
fourteen. It resets the clock to 14 whatever it read. The rest of the card is
as it was. Game and sheet.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -4444,7 +4444,7 @@
       </c>
       <c r="D82" s="38" t="inlineStr">
         <is>
-          <t>Shot Clock changes: TOV +1. Side-out. Shot Clock resets to 14 if it is higher.</t>
+          <t>Shot Clock changes: TOV +1. Side-out. Resets the Shot Clock to 14.</t>
         </is>
       </c>
       <c r="E82" s="7" t="n"/>
@@ -8579,8 +8579,8 @@
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
     <mergeCell ref="G119:J119"/>
+    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G32:J32"/>
-    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G202:J202"/>
     <mergeCell ref="G46:J46"/>
     <mergeCell ref="G40:J40"/>

</xml_diff>

<commit_message>
Flop says it has to go first
It was enforced and never printed: a hand that held one went grey apart from
it, with nothing on the card to say why, which reads as the game being broken.
"Must be your first action while it is in your Bag", on its own line since it
is a rule rather than a clarification. Game and sheet.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -2834,7 +2834,7 @@
       </c>
       <c r="D25" s="38" t="inlineStr">
         <is>
-          <t>Draw 1 card. Clear all Clamps. Take 1 FT for each. If no Clamps, TOV +1</t>
+          <t>Draw 1 card. Clear all Clamps. Take 1 FT for each. If no Clamps, TOV +1. Must be your first action while it is in your Bag</t>
         </is>
       </c>
       <c r="E25" s="7" t="n"/>
@@ -8578,8 +8578,8 @@
     <mergeCell ref="G135:J135"/>
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
+    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G119:J119"/>
-    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G32:J32"/>
     <mergeCell ref="G202:J202"/>
     <mergeCell ref="G46:J46"/>

</xml_diff>

<commit_message>
Flagrant Foul II sends somebody to the line
Its free throw was read in exactly one place — where a *voided* Clamp is
resolved, which is Flagrant I's road. Flagrant II lets the Clamp stand, so it
never went that way: it took the clamper's two cards and nobody went to the
line. The man the Clamp was put on goes now, and the Clamp still lands.

And Flop reads "if it is in your Bag".

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project CardCourt_CardDB.xlsx
+++ b/Project CardCourt_CardDB.xlsx
@@ -2834,7 +2834,7 @@
       </c>
       <c r="D25" s="38" t="inlineStr">
         <is>
-          <t>Draw 1 card. Clear all Clamps. Take 1 FT for each. If no Clamps, TOV +1. Must be your first action while it is in your Bag</t>
+          <t>Draw 1 card. Clear all Clamps. Take 1 FT for each. If no Clamps, TOV +1. Must be your first action if it is in your Bag</t>
         </is>
       </c>
       <c r="E25" s="7" t="n"/>
@@ -8578,9 +8578,9 @@
     <mergeCell ref="G135:J135"/>
     <mergeCell ref="G109:J109"/>
     <mergeCell ref="G47:J47"/>
-    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G119:J119"/>
     <mergeCell ref="G32:J32"/>
+    <mergeCell ref="G150:J150"/>
     <mergeCell ref="G202:J202"/>
     <mergeCell ref="G46:J46"/>
     <mergeCell ref="G40:J40"/>

</xml_diff>